<commit_message>
fix(search): enable search bar and button submit in Navbar and sync query params with Explore page
</commit_message>
<xml_diff>
--- a/all-test-reports/selenium/selenium_e2e_test_report.xlsx
+++ b/all-test-reports/selenium/selenium_e2e_test_report.xlsx
@@ -35,7 +35,7 @@
     <t>Execution Date</t>
   </si>
   <si>
-    <t>28/7/2026, 8:51:50 am</t>
+    <t>28/7/2026, 10:34:33 am</t>
   </si>
   <si>
     <t>Browser / Mode</t>
@@ -98,7 +98,7 @@
     <t>PASS</t>
   </si>
   <si>
-    <t>8:51:50 am</t>
+    <t>10:34:33 am</t>
   </si>
   <si>
     <t>N/A</t>
@@ -1997,7 +1997,7 @@
         <v>27</v>
       </c>
       <c r="E2" s="11">
-        <v>26</v>
+        <v>18</v>
       </c>
       <c r="F2" s="9" t="s">
         <v>28</v>
@@ -2020,7 +2020,7 @@
         <v>27</v>
       </c>
       <c r="E3" s="11">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="F3" s="9" t="s">
         <v>28</v>
@@ -2043,7 +2043,7 @@
         <v>27</v>
       </c>
       <c r="E4" s="11">
-        <v>22</v>
+        <v>28</v>
       </c>
       <c r="F4" s="9" t="s">
         <v>28</v>
@@ -2066,7 +2066,7 @@
         <v>27</v>
       </c>
       <c r="E5" s="11">
-        <v>12</v>
+        <v>29</v>
       </c>
       <c r="F5" s="9" t="s">
         <v>28</v>
@@ -2089,7 +2089,7 @@
         <v>27</v>
       </c>
       <c r="E6" s="11">
-        <v>29</v>
+        <v>14</v>
       </c>
       <c r="F6" s="9" t="s">
         <v>28</v>
@@ -2112,7 +2112,7 @@
         <v>27</v>
       </c>
       <c r="E7" s="11">
-        <v>8</v>
+        <v>23</v>
       </c>
       <c r="F7" s="9" t="s">
         <v>28</v>
@@ -2135,7 +2135,7 @@
         <v>27</v>
       </c>
       <c r="E8" s="11">
-        <v>18</v>
+        <v>21</v>
       </c>
       <c r="F8" s="9" t="s">
         <v>28</v>
@@ -2158,7 +2158,7 @@
         <v>27</v>
       </c>
       <c r="E9" s="11">
-        <v>19</v>
+        <v>16</v>
       </c>
       <c r="F9" s="9" t="s">
         <v>28</v>
@@ -2181,7 +2181,7 @@
         <v>27</v>
       </c>
       <c r="E10" s="11">
-        <v>23</v>
+        <v>20</v>
       </c>
       <c r="F10" s="9" t="s">
         <v>28</v>
@@ -2204,7 +2204,7 @@
         <v>27</v>
       </c>
       <c r="E11" s="11">
-        <v>8</v>
+        <v>13</v>
       </c>
       <c r="F11" s="9" t="s">
         <v>28</v>
@@ -2227,7 +2227,7 @@
         <v>27</v>
       </c>
       <c r="E12" s="11">
-        <v>29</v>
+        <v>17</v>
       </c>
       <c r="F12" s="9" t="s">
         <v>28</v>
@@ -2250,7 +2250,7 @@
         <v>27</v>
       </c>
       <c r="E13" s="11">
-        <v>18</v>
+        <v>9</v>
       </c>
       <c r="F13" s="9" t="s">
         <v>28</v>
@@ -2273,7 +2273,7 @@
         <v>27</v>
       </c>
       <c r="E14" s="11">
-        <v>10</v>
+        <v>31</v>
       </c>
       <c r="F14" s="9" t="s">
         <v>28</v>
@@ -2296,7 +2296,7 @@
         <v>27</v>
       </c>
       <c r="E15" s="11">
-        <v>18</v>
+        <v>10</v>
       </c>
       <c r="F15" s="9" t="s">
         <v>28</v>
@@ -2319,7 +2319,7 @@
         <v>27</v>
       </c>
       <c r="E16" s="11">
-        <v>14</v>
+        <v>10</v>
       </c>
       <c r="F16" s="9" t="s">
         <v>28</v>
@@ -2342,7 +2342,7 @@
         <v>27</v>
       </c>
       <c r="E17" s="11">
-        <v>24</v>
+        <v>13</v>
       </c>
       <c r="F17" s="9" t="s">
         <v>28</v>
@@ -2365,7 +2365,7 @@
         <v>27</v>
       </c>
       <c r="E18" s="11">
-        <v>10</v>
+        <v>27</v>
       </c>
       <c r="F18" s="9" t="s">
         <v>28</v>
@@ -2411,7 +2411,7 @@
         <v>27</v>
       </c>
       <c r="E20" s="11">
-        <v>31</v>
+        <v>10</v>
       </c>
       <c r="F20" s="9" t="s">
         <v>28</v>
@@ -2434,7 +2434,7 @@
         <v>27</v>
       </c>
       <c r="E21" s="11">
-        <v>13</v>
+        <v>22</v>
       </c>
       <c r="F21" s="9" t="s">
         <v>28</v>
@@ -2457,7 +2457,7 @@
         <v>27</v>
       </c>
       <c r="E22" s="11">
-        <v>20</v>
+        <v>13</v>
       </c>
       <c r="F22" s="9" t="s">
         <v>28</v>
@@ -2480,7 +2480,7 @@
         <v>27</v>
       </c>
       <c r="E23" s="11">
-        <v>20</v>
+        <v>31</v>
       </c>
       <c r="F23" s="9" t="s">
         <v>28</v>
@@ -2503,7 +2503,7 @@
         <v>27</v>
       </c>
       <c r="E24" s="11">
-        <v>15</v>
+        <v>25</v>
       </c>
       <c r="F24" s="9" t="s">
         <v>28</v>
@@ -2526,7 +2526,7 @@
         <v>27</v>
       </c>
       <c r="E25" s="11">
-        <v>21</v>
+        <v>28</v>
       </c>
       <c r="F25" s="9" t="s">
         <v>28</v>
@@ -2549,7 +2549,7 @@
         <v>27</v>
       </c>
       <c r="E26" s="11">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="F26" s="9" t="s">
         <v>28</v>
@@ -2595,7 +2595,7 @@
         <v>27</v>
       </c>
       <c r="E28" s="11">
-        <v>9</v>
+        <v>26</v>
       </c>
       <c r="F28" s="9" t="s">
         <v>28</v>
@@ -2618,7 +2618,7 @@
         <v>27</v>
       </c>
       <c r="E29" s="11">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="F29" s="9" t="s">
         <v>28</v>
@@ -2641,7 +2641,7 @@
         <v>27</v>
       </c>
       <c r="E30" s="11">
-        <v>19</v>
+        <v>13</v>
       </c>
       <c r="F30" s="9" t="s">
         <v>28</v>
@@ -2664,7 +2664,7 @@
         <v>27</v>
       </c>
       <c r="E31" s="11">
-        <v>13</v>
+        <v>24</v>
       </c>
       <c r="F31" s="9" t="s">
         <v>28</v>
@@ -2687,7 +2687,7 @@
         <v>27</v>
       </c>
       <c r="E32" s="11">
-        <v>10</v>
+        <v>14</v>
       </c>
       <c r="F32" s="9" t="s">
         <v>28</v>
@@ -2710,7 +2710,7 @@
         <v>27</v>
       </c>
       <c r="E33" s="11">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="F33" s="9" t="s">
         <v>28</v>
@@ -2733,7 +2733,7 @@
         <v>27</v>
       </c>
       <c r="E34" s="11">
-        <v>9</v>
+        <v>13</v>
       </c>
       <c r="F34" s="9" t="s">
         <v>28</v>
@@ -2756,7 +2756,7 @@
         <v>27</v>
       </c>
       <c r="E35" s="11">
-        <v>16</v>
+        <v>8</v>
       </c>
       <c r="F35" s="9" t="s">
         <v>28</v>
@@ -2779,7 +2779,7 @@
         <v>27</v>
       </c>
       <c r="E36" s="11">
-        <v>18</v>
+        <v>22</v>
       </c>
       <c r="F36" s="9" t="s">
         <v>28</v>
@@ -2802,7 +2802,7 @@
         <v>27</v>
       </c>
       <c r="E37" s="11">
-        <v>18</v>
+        <v>16</v>
       </c>
       <c r="F37" s="9" t="s">
         <v>28</v>
@@ -2825,7 +2825,7 @@
         <v>27</v>
       </c>
       <c r="E38" s="11">
-        <v>17</v>
+        <v>28</v>
       </c>
       <c r="F38" s="9" t="s">
         <v>28</v>
@@ -2848,7 +2848,7 @@
         <v>27</v>
       </c>
       <c r="E39" s="11">
-        <v>12</v>
+        <v>18</v>
       </c>
       <c r="F39" s="9" t="s">
         <v>28</v>
@@ -2894,7 +2894,7 @@
         <v>27</v>
       </c>
       <c r="E41" s="11">
-        <v>10</v>
+        <v>30</v>
       </c>
       <c r="F41" s="9" t="s">
         <v>28</v>
@@ -2917,7 +2917,7 @@
         <v>27</v>
       </c>
       <c r="E42" s="11">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="F42" s="9" t="s">
         <v>28</v>
@@ -2940,7 +2940,7 @@
         <v>27</v>
       </c>
       <c r="E43" s="11">
-        <v>30</v>
+        <v>25</v>
       </c>
       <c r="F43" s="9" t="s">
         <v>28</v>
@@ -2963,7 +2963,7 @@
         <v>27</v>
       </c>
       <c r="E44" s="11">
-        <v>25</v>
+        <v>28</v>
       </c>
       <c r="F44" s="9" t="s">
         <v>28</v>
@@ -3009,7 +3009,7 @@
         <v>27</v>
       </c>
       <c r="E46" s="11">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="F46" s="9" t="s">
         <v>28</v>
@@ -3032,7 +3032,7 @@
         <v>27</v>
       </c>
       <c r="E47" s="11">
-        <v>15</v>
+        <v>30</v>
       </c>
       <c r="F47" s="9" t="s">
         <v>28</v>
@@ -3078,7 +3078,7 @@
         <v>27</v>
       </c>
       <c r="E49" s="11">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="F49" s="9" t="s">
         <v>28</v>
@@ -3101,7 +3101,7 @@
         <v>27</v>
       </c>
       <c r="E50" s="11">
-        <v>10</v>
+        <v>13</v>
       </c>
       <c r="F50" s="9" t="s">
         <v>28</v>
@@ -3170,7 +3170,7 @@
         <v>27</v>
       </c>
       <c r="E53" s="11">
-        <v>11</v>
+        <v>8</v>
       </c>
       <c r="F53" s="9" t="s">
         <v>28</v>
@@ -3193,7 +3193,7 @@
         <v>27</v>
       </c>
       <c r="E54" s="11">
-        <v>30</v>
+        <v>14</v>
       </c>
       <c r="F54" s="9" t="s">
         <v>28</v>
@@ -3239,7 +3239,7 @@
         <v>27</v>
       </c>
       <c r="E56" s="11">
-        <v>22</v>
+        <v>10</v>
       </c>
       <c r="F56" s="9" t="s">
         <v>28</v>
@@ -3262,7 +3262,7 @@
         <v>27</v>
       </c>
       <c r="E57" s="11">
-        <v>18</v>
+        <v>14</v>
       </c>
       <c r="F57" s="9" t="s">
         <v>28</v>
@@ -3308,7 +3308,7 @@
         <v>27</v>
       </c>
       <c r="E59" s="11">
-        <v>11</v>
+        <v>19</v>
       </c>
       <c r="F59" s="9" t="s">
         <v>28</v>
@@ -3331,7 +3331,7 @@
         <v>27</v>
       </c>
       <c r="E60" s="11">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="F60" s="9" t="s">
         <v>28</v>
@@ -3354,7 +3354,7 @@
         <v>27</v>
       </c>
       <c r="E61" s="11">
-        <v>21</v>
+        <v>19</v>
       </c>
       <c r="F61" s="9" t="s">
         <v>28</v>
@@ -3377,7 +3377,7 @@
         <v>27</v>
       </c>
       <c r="E62" s="11">
-        <v>26</v>
+        <v>9</v>
       </c>
       <c r="F62" s="9" t="s">
         <v>28</v>
@@ -3400,7 +3400,7 @@
         <v>27</v>
       </c>
       <c r="E63" s="11">
-        <v>25</v>
+        <v>30</v>
       </c>
       <c r="F63" s="9" t="s">
         <v>28</v>
@@ -3423,7 +3423,7 @@
         <v>27</v>
       </c>
       <c r="E64" s="11">
-        <v>17</v>
+        <v>27</v>
       </c>
       <c r="F64" s="9" t="s">
         <v>28</v>
@@ -3446,7 +3446,7 @@
         <v>27</v>
       </c>
       <c r="E65" s="11">
-        <v>10</v>
+        <v>14</v>
       </c>
       <c r="F65" s="9" t="s">
         <v>28</v>
@@ -3469,7 +3469,7 @@
         <v>27</v>
       </c>
       <c r="E66" s="11">
-        <v>17</v>
+        <v>23</v>
       </c>
       <c r="F66" s="9" t="s">
         <v>28</v>
@@ -3492,7 +3492,7 @@
         <v>27</v>
       </c>
       <c r="E67" s="11">
-        <v>27</v>
+        <v>14</v>
       </c>
       <c r="F67" s="9" t="s">
         <v>28</v>
@@ -3515,7 +3515,7 @@
         <v>27</v>
       </c>
       <c r="E68" s="11">
-        <v>26</v>
+        <v>31</v>
       </c>
       <c r="F68" s="9" t="s">
         <v>28</v>
@@ -3561,7 +3561,7 @@
         <v>27</v>
       </c>
       <c r="E70" s="11">
-        <v>16</v>
+        <v>31</v>
       </c>
       <c r="F70" s="9" t="s">
         <v>28</v>
@@ -3584,7 +3584,7 @@
         <v>27</v>
       </c>
       <c r="E71" s="11">
-        <v>20</v>
+        <v>9</v>
       </c>
       <c r="F71" s="9" t="s">
         <v>28</v>
@@ -3607,7 +3607,7 @@
         <v>27</v>
       </c>
       <c r="E72" s="11">
-        <v>30</v>
+        <v>10</v>
       </c>
       <c r="F72" s="9" t="s">
         <v>28</v>
@@ -3630,7 +3630,7 @@
         <v>27</v>
       </c>
       <c r="E73" s="11">
-        <v>15</v>
+        <v>11</v>
       </c>
       <c r="F73" s="9" t="s">
         <v>28</v>
@@ -3653,7 +3653,7 @@
         <v>27</v>
       </c>
       <c r="E74" s="11">
-        <v>27</v>
+        <v>14</v>
       </c>
       <c r="F74" s="9" t="s">
         <v>28</v>
@@ -3676,7 +3676,7 @@
         <v>27</v>
       </c>
       <c r="E75" s="11">
-        <v>24</v>
+        <v>11</v>
       </c>
       <c r="F75" s="9" t="s">
         <v>28</v>
@@ -3699,7 +3699,7 @@
         <v>27</v>
       </c>
       <c r="E76" s="11">
-        <v>27</v>
+        <v>20</v>
       </c>
       <c r="F76" s="9" t="s">
         <v>28</v>
@@ -3722,7 +3722,7 @@
         <v>27</v>
       </c>
       <c r="E77" s="11">
-        <v>18</v>
+        <v>15</v>
       </c>
       <c r="F77" s="9" t="s">
         <v>28</v>
@@ -3745,7 +3745,7 @@
         <v>27</v>
       </c>
       <c r="E78" s="11">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="F78" s="9" t="s">
         <v>28</v>
@@ -3768,7 +3768,7 @@
         <v>27</v>
       </c>
       <c r="E79" s="11">
-        <v>15</v>
+        <v>12</v>
       </c>
       <c r="F79" s="9" t="s">
         <v>28</v>
@@ -3791,7 +3791,7 @@
         <v>27</v>
       </c>
       <c r="E80" s="11">
-        <v>17</v>
+        <v>14</v>
       </c>
       <c r="F80" s="9" t="s">
         <v>28</v>
@@ -3814,7 +3814,7 @@
         <v>27</v>
       </c>
       <c r="E81" s="11">
-        <v>29</v>
+        <v>11</v>
       </c>
       <c r="F81" s="9" t="s">
         <v>28</v>
@@ -3837,7 +3837,7 @@
         <v>27</v>
       </c>
       <c r="E82" s="11">
-        <v>18</v>
+        <v>25</v>
       </c>
       <c r="F82" s="9" t="s">
         <v>28</v>
@@ -3860,7 +3860,7 @@
         <v>27</v>
       </c>
       <c r="E83" s="11">
-        <v>24</v>
+        <v>13</v>
       </c>
       <c r="F83" s="9" t="s">
         <v>28</v>
@@ -3883,7 +3883,7 @@
         <v>27</v>
       </c>
       <c r="E84" s="11">
-        <v>12</v>
+        <v>29</v>
       </c>
       <c r="F84" s="9" t="s">
         <v>28</v>
@@ -3906,7 +3906,7 @@
         <v>27</v>
       </c>
       <c r="E85" s="11">
-        <v>10</v>
+        <v>30</v>
       </c>
       <c r="F85" s="9" t="s">
         <v>28</v>
@@ -3929,7 +3929,7 @@
         <v>27</v>
       </c>
       <c r="E86" s="11">
-        <v>14</v>
+        <v>11</v>
       </c>
       <c r="F86" s="9" t="s">
         <v>28</v>
@@ -3975,7 +3975,7 @@
         <v>27</v>
       </c>
       <c r="E88" s="11">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="F88" s="9" t="s">
         <v>28</v>
@@ -3998,7 +3998,7 @@
         <v>27</v>
       </c>
       <c r="E89" s="11">
-        <v>8</v>
+        <v>20</v>
       </c>
       <c r="F89" s="9" t="s">
         <v>28</v>
@@ -4021,7 +4021,7 @@
         <v>27</v>
       </c>
       <c r="E90" s="11">
-        <v>19</v>
+        <v>11</v>
       </c>
       <c r="F90" s="9" t="s">
         <v>28</v>
@@ -4044,7 +4044,7 @@
         <v>27</v>
       </c>
       <c r="E91" s="11">
-        <v>10</v>
+        <v>28</v>
       </c>
       <c r="F91" s="9" t="s">
         <v>28</v>
@@ -4067,7 +4067,7 @@
         <v>27</v>
       </c>
       <c r="E92" s="11">
-        <v>27</v>
+        <v>14</v>
       </c>
       <c r="F92" s="9" t="s">
         <v>28</v>
@@ -4090,7 +4090,7 @@
         <v>27</v>
       </c>
       <c r="E93" s="11">
-        <v>24</v>
+        <v>15</v>
       </c>
       <c r="F93" s="9" t="s">
         <v>28</v>
@@ -4136,7 +4136,7 @@
         <v>27</v>
       </c>
       <c r="E95" s="11">
-        <v>22</v>
+        <v>20</v>
       </c>
       <c r="F95" s="9" t="s">
         <v>28</v>
@@ -4159,7 +4159,7 @@
         <v>27</v>
       </c>
       <c r="E96" s="11">
-        <v>31</v>
+        <v>29</v>
       </c>
       <c r="F96" s="9" t="s">
         <v>28</v>
@@ -4205,7 +4205,7 @@
         <v>27</v>
       </c>
       <c r="E98" s="11">
-        <v>16</v>
+        <v>19</v>
       </c>
       <c r="F98" s="9" t="s">
         <v>28</v>
@@ -4228,7 +4228,7 @@
         <v>27</v>
       </c>
       <c r="E99" s="11">
-        <v>31</v>
+        <v>13</v>
       </c>
       <c r="F99" s="9" t="s">
         <v>28</v>
@@ -4251,7 +4251,7 @@
         <v>27</v>
       </c>
       <c r="E100" s="11">
-        <v>17</v>
+        <v>26</v>
       </c>
       <c r="F100" s="9" t="s">
         <v>28</v>
@@ -4297,7 +4297,7 @@
         <v>27</v>
       </c>
       <c r="E102" s="11">
-        <v>22</v>
+        <v>24</v>
       </c>
       <c r="F102" s="9" t="s">
         <v>28</v>
@@ -4343,7 +4343,7 @@
         <v>27</v>
       </c>
       <c r="E104" s="11">
-        <v>21</v>
+        <v>8</v>
       </c>
       <c r="F104" s="9" t="s">
         <v>28</v>
@@ -4366,7 +4366,7 @@
         <v>27</v>
       </c>
       <c r="E105" s="11">
-        <v>21</v>
+        <v>29</v>
       </c>
       <c r="F105" s="9" t="s">
         <v>28</v>
@@ -4389,7 +4389,7 @@
         <v>27</v>
       </c>
       <c r="E106" s="11">
-        <v>19</v>
+        <v>16</v>
       </c>
       <c r="F106" s="9" t="s">
         <v>28</v>
@@ -4412,7 +4412,7 @@
         <v>27</v>
       </c>
       <c r="E107" s="11">
-        <v>30</v>
+        <v>22</v>
       </c>
       <c r="F107" s="9" t="s">
         <v>28</v>
@@ -4435,7 +4435,7 @@
         <v>27</v>
       </c>
       <c r="E108" s="11">
-        <v>12</v>
+        <v>29</v>
       </c>
       <c r="F108" s="9" t="s">
         <v>28</v>
@@ -4458,7 +4458,7 @@
         <v>27</v>
       </c>
       <c r="E109" s="11">
-        <v>26</v>
+        <v>29</v>
       </c>
       <c r="F109" s="9" t="s">
         <v>28</v>
@@ -4481,7 +4481,7 @@
         <v>27</v>
       </c>
       <c r="E110" s="11">
-        <v>9</v>
+        <v>12</v>
       </c>
       <c r="F110" s="9" t="s">
         <v>28</v>
@@ -4504,7 +4504,7 @@
         <v>27</v>
       </c>
       <c r="E111" s="11">
-        <v>31</v>
+        <v>14</v>
       </c>
       <c r="F111" s="9" t="s">
         <v>28</v>
@@ -4527,7 +4527,7 @@
         <v>27</v>
       </c>
       <c r="E112" s="11">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="F112" s="9" t="s">
         <v>28</v>
@@ -4550,7 +4550,7 @@
         <v>27</v>
       </c>
       <c r="E113" s="11">
-        <v>27</v>
+        <v>16</v>
       </c>
       <c r="F113" s="9" t="s">
         <v>28</v>
@@ -4573,7 +4573,7 @@
         <v>27</v>
       </c>
       <c r="E114" s="11">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="F114" s="9" t="s">
         <v>28</v>
@@ -4596,7 +4596,7 @@
         <v>27</v>
       </c>
       <c r="E115" s="11">
-        <v>23</v>
+        <v>16</v>
       </c>
       <c r="F115" s="9" t="s">
         <v>28</v>
@@ -4619,7 +4619,7 @@
         <v>27</v>
       </c>
       <c r="E116" s="11">
-        <v>18</v>
+        <v>10</v>
       </c>
       <c r="F116" s="9" t="s">
         <v>28</v>
@@ -4642,7 +4642,7 @@
         <v>27</v>
       </c>
       <c r="E117" s="11">
-        <v>11</v>
+        <v>18</v>
       </c>
       <c r="F117" s="9" t="s">
         <v>28</v>
@@ -4665,7 +4665,7 @@
         <v>27</v>
       </c>
       <c r="E118" s="11">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="F118" s="9" t="s">
         <v>28</v>
@@ -4688,7 +4688,7 @@
         <v>27</v>
       </c>
       <c r="E119" s="11">
-        <v>20</v>
+        <v>30</v>
       </c>
       <c r="F119" s="9" t="s">
         <v>28</v>
@@ -4711,7 +4711,7 @@
         <v>27</v>
       </c>
       <c r="E120" s="11">
-        <v>14</v>
+        <v>19</v>
       </c>
       <c r="F120" s="9" t="s">
         <v>28</v>
@@ -4734,7 +4734,7 @@
         <v>27</v>
       </c>
       <c r="E121" s="11">
-        <v>22</v>
+        <v>17</v>
       </c>
       <c r="F121" s="9" t="s">
         <v>28</v>
@@ -4757,7 +4757,7 @@
         <v>27</v>
       </c>
       <c r="E122" s="11">
-        <v>20</v>
+        <v>26</v>
       </c>
       <c r="F122" s="9" t="s">
         <v>28</v>
@@ -4780,7 +4780,7 @@
         <v>27</v>
       </c>
       <c r="E123" s="11">
-        <v>17</v>
+        <v>26</v>
       </c>
       <c r="F123" s="9" t="s">
         <v>28</v>
@@ -4803,7 +4803,7 @@
         <v>27</v>
       </c>
       <c r="E124" s="11">
-        <v>20</v>
+        <v>27</v>
       </c>
       <c r="F124" s="9" t="s">
         <v>28</v>
@@ -4826,7 +4826,7 @@
         <v>27</v>
       </c>
       <c r="E125" s="11">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="F125" s="9" t="s">
         <v>28</v>
@@ -4849,7 +4849,7 @@
         <v>27</v>
       </c>
       <c r="E126" s="11">
-        <v>22</v>
+        <v>20</v>
       </c>
       <c r="F126" s="9" t="s">
         <v>28</v>
@@ -4872,7 +4872,7 @@
         <v>27</v>
       </c>
       <c r="E127" s="11">
-        <v>13</v>
+        <v>26</v>
       </c>
       <c r="F127" s="9" t="s">
         <v>28</v>
@@ -4895,7 +4895,7 @@
         <v>27</v>
       </c>
       <c r="E128" s="11">
-        <v>20</v>
+        <v>16</v>
       </c>
       <c r="F128" s="9" t="s">
         <v>28</v>
@@ -4918,7 +4918,7 @@
         <v>27</v>
       </c>
       <c r="E129" s="11">
-        <v>10</v>
+        <v>30</v>
       </c>
       <c r="F129" s="9" t="s">
         <v>28</v>
@@ -4941,7 +4941,7 @@
         <v>27</v>
       </c>
       <c r="E130" s="11">
-        <v>19</v>
+        <v>27</v>
       </c>
       <c r="F130" s="9" t="s">
         <v>28</v>
@@ -4964,7 +4964,7 @@
         <v>27</v>
       </c>
       <c r="E131" s="11">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="F131" s="9" t="s">
         <v>28</v>
@@ -4987,7 +4987,7 @@
         <v>27</v>
       </c>
       <c r="E132" s="11">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="F132" s="9" t="s">
         <v>28</v>
@@ -5010,7 +5010,7 @@
         <v>27</v>
       </c>
       <c r="E133" s="11">
-        <v>25</v>
+        <v>20</v>
       </c>
       <c r="F133" s="9" t="s">
         <v>28</v>
@@ -5033,7 +5033,7 @@
         <v>27</v>
       </c>
       <c r="E134" s="11">
-        <v>23</v>
+        <v>14</v>
       </c>
       <c r="F134" s="9" t="s">
         <v>28</v>
@@ -5056,7 +5056,7 @@
         <v>27</v>
       </c>
       <c r="E135" s="11">
-        <v>21</v>
+        <v>30</v>
       </c>
       <c r="F135" s="9" t="s">
         <v>28</v>
@@ -5079,7 +5079,7 @@
         <v>27</v>
       </c>
       <c r="E136" s="11">
-        <v>19</v>
+        <v>24</v>
       </c>
       <c r="F136" s="9" t="s">
         <v>28</v>
@@ -5102,7 +5102,7 @@
         <v>27</v>
       </c>
       <c r="E137" s="11">
-        <v>17</v>
+        <v>8</v>
       </c>
       <c r="F137" s="9" t="s">
         <v>28</v>
@@ -5125,7 +5125,7 @@
         <v>27</v>
       </c>
       <c r="E138" s="11">
-        <v>30</v>
+        <v>11</v>
       </c>
       <c r="F138" s="9" t="s">
         <v>28</v>
@@ -5148,7 +5148,7 @@
         <v>27</v>
       </c>
       <c r="E139" s="11">
-        <v>23</v>
+        <v>28</v>
       </c>
       <c r="F139" s="9" t="s">
         <v>28</v>
@@ -5171,7 +5171,7 @@
         <v>27</v>
       </c>
       <c r="E140" s="11">
-        <v>21</v>
+        <v>16</v>
       </c>
       <c r="F140" s="9" t="s">
         <v>28</v>
@@ -5194,7 +5194,7 @@
         <v>27</v>
       </c>
       <c r="E141" s="11">
-        <v>26</v>
+        <v>17</v>
       </c>
       <c r="F141" s="9" t="s">
         <v>28</v>
@@ -5217,7 +5217,7 @@
         <v>27</v>
       </c>
       <c r="E142" s="11">
-        <v>31</v>
+        <v>17</v>
       </c>
       <c r="F142" s="9" t="s">
         <v>28</v>
@@ -5240,7 +5240,7 @@
         <v>27</v>
       </c>
       <c r="E143" s="11">
-        <v>25</v>
+        <v>11</v>
       </c>
       <c r="F143" s="9" t="s">
         <v>28</v>
@@ -5263,7 +5263,7 @@
         <v>27</v>
       </c>
       <c r="E144" s="11">
-        <v>8</v>
+        <v>29</v>
       </c>
       <c r="F144" s="9" t="s">
         <v>28</v>
@@ -5286,7 +5286,7 @@
         <v>27</v>
       </c>
       <c r="E145" s="11">
-        <v>17</v>
+        <v>9</v>
       </c>
       <c r="F145" s="9" t="s">
         <v>28</v>
@@ -5309,7 +5309,7 @@
         <v>27</v>
       </c>
       <c r="E146" s="11">
-        <v>26</v>
+        <v>28</v>
       </c>
       <c r="F146" s="9" t="s">
         <v>28</v>
@@ -5355,7 +5355,7 @@
         <v>27</v>
       </c>
       <c r="E148" s="11">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="F148" s="9" t="s">
         <v>28</v>
@@ -5378,7 +5378,7 @@
         <v>27</v>
       </c>
       <c r="E149" s="11">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="F149" s="9" t="s">
         <v>28</v>
@@ -5401,7 +5401,7 @@
         <v>27</v>
       </c>
       <c r="E150" s="11">
-        <v>11</v>
+        <v>9</v>
       </c>
       <c r="F150" s="9" t="s">
         <v>28</v>
@@ -5424,7 +5424,7 @@
         <v>27</v>
       </c>
       <c r="E151" s="11">
-        <v>23</v>
+        <v>27</v>
       </c>
       <c r="F151" s="9" t="s">
         <v>28</v>
@@ -5447,7 +5447,7 @@
         <v>27</v>
       </c>
       <c r="E152" s="11">
-        <v>22</v>
+        <v>30</v>
       </c>
       <c r="F152" s="9" t="s">
         <v>28</v>
@@ -5470,7 +5470,7 @@
         <v>27</v>
       </c>
       <c r="E153" s="11">
-        <v>26</v>
+        <v>8</v>
       </c>
       <c r="F153" s="9" t="s">
         <v>28</v>
@@ -5493,7 +5493,7 @@
         <v>27</v>
       </c>
       <c r="E154" s="11">
-        <v>14</v>
+        <v>21</v>
       </c>
       <c r="F154" s="9" t="s">
         <v>28</v>
@@ -5516,7 +5516,7 @@
         <v>27</v>
       </c>
       <c r="E155" s="11">
-        <v>27</v>
+        <v>21</v>
       </c>
       <c r="F155" s="9" t="s">
         <v>28</v>
@@ -5562,7 +5562,7 @@
         <v>27</v>
       </c>
       <c r="E157" s="11">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="F157" s="9" t="s">
         <v>28</v>
@@ -5585,7 +5585,7 @@
         <v>27</v>
       </c>
       <c r="E158" s="11">
-        <v>28</v>
+        <v>21</v>
       </c>
       <c r="F158" s="9" t="s">
         <v>28</v>
@@ -5608,7 +5608,7 @@
         <v>27</v>
       </c>
       <c r="E159" s="11">
-        <v>14</v>
+        <v>16</v>
       </c>
       <c r="F159" s="9" t="s">
         <v>28</v>
@@ -5631,7 +5631,7 @@
         <v>27</v>
       </c>
       <c r="E160" s="11">
-        <v>18</v>
+        <v>27</v>
       </c>
       <c r="F160" s="9" t="s">
         <v>28</v>
@@ -5654,7 +5654,7 @@
         <v>27</v>
       </c>
       <c r="E161" s="11">
-        <v>20</v>
+        <v>8</v>
       </c>
       <c r="F161" s="9" t="s">
         <v>28</v>
@@ -5677,7 +5677,7 @@
         <v>27</v>
       </c>
       <c r="E162" s="11">
-        <v>8</v>
+        <v>21</v>
       </c>
       <c r="F162" s="9" t="s">
         <v>28</v>
@@ -5700,7 +5700,7 @@
         <v>27</v>
       </c>
       <c r="E163" s="11">
-        <v>13</v>
+        <v>8</v>
       </c>
       <c r="F163" s="9" t="s">
         <v>28</v>
@@ -5723,7 +5723,7 @@
         <v>27</v>
       </c>
       <c r="E164" s="11">
-        <v>25</v>
+        <v>12</v>
       </c>
       <c r="F164" s="9" t="s">
         <v>28</v>
@@ -5746,7 +5746,7 @@
         <v>27</v>
       </c>
       <c r="E165" s="11">
-        <v>14</v>
+        <v>25</v>
       </c>
       <c r="F165" s="9" t="s">
         <v>28</v>
@@ -5769,7 +5769,7 @@
         <v>27</v>
       </c>
       <c r="E166" s="11">
-        <v>8</v>
+        <v>31</v>
       </c>
       <c r="F166" s="9" t="s">
         <v>28</v>
@@ -5792,7 +5792,7 @@
         <v>27</v>
       </c>
       <c r="E167" s="11">
-        <v>31</v>
+        <v>13</v>
       </c>
       <c r="F167" s="9" t="s">
         <v>28</v>
@@ -5815,7 +5815,7 @@
         <v>27</v>
       </c>
       <c r="E168" s="11">
-        <v>31</v>
+        <v>21</v>
       </c>
       <c r="F168" s="9" t="s">
         <v>28</v>
@@ -5838,7 +5838,7 @@
         <v>27</v>
       </c>
       <c r="E169" s="11">
-        <v>19</v>
+        <v>14</v>
       </c>
       <c r="F169" s="9" t="s">
         <v>28</v>
@@ -5861,7 +5861,7 @@
         <v>27</v>
       </c>
       <c r="E170" s="11">
-        <v>28</v>
+        <v>18</v>
       </c>
       <c r="F170" s="9" t="s">
         <v>28</v>
@@ -5884,7 +5884,7 @@
         <v>27</v>
       </c>
       <c r="E171" s="11">
-        <v>17</v>
+        <v>14</v>
       </c>
       <c r="F171" s="9" t="s">
         <v>28</v>
@@ -5907,7 +5907,7 @@
         <v>27</v>
       </c>
       <c r="E172" s="11">
-        <v>9</v>
+        <v>20</v>
       </c>
       <c r="F172" s="9" t="s">
         <v>28</v>
@@ -5953,7 +5953,7 @@
         <v>27</v>
       </c>
       <c r="E174" s="11">
-        <v>10</v>
+        <v>25</v>
       </c>
       <c r="F174" s="9" t="s">
         <v>28</v>
@@ -5976,7 +5976,7 @@
         <v>27</v>
       </c>
       <c r="E175" s="11">
-        <v>11</v>
+        <v>18</v>
       </c>
       <c r="F175" s="9" t="s">
         <v>28</v>
@@ -5999,7 +5999,7 @@
         <v>27</v>
       </c>
       <c r="E176" s="11">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="F176" s="9" t="s">
         <v>28</v>
@@ -6022,7 +6022,7 @@
         <v>27</v>
       </c>
       <c r="E177" s="11">
-        <v>20</v>
+        <v>25</v>
       </c>
       <c r="F177" s="9" t="s">
         <v>28</v>
@@ -6045,7 +6045,7 @@
         <v>27</v>
       </c>
       <c r="E178" s="11">
-        <v>11</v>
+        <v>13</v>
       </c>
       <c r="F178" s="9" t="s">
         <v>28</v>
@@ -6068,7 +6068,7 @@
         <v>27</v>
       </c>
       <c r="E179" s="11">
-        <v>26</v>
+        <v>31</v>
       </c>
       <c r="F179" s="9" t="s">
         <v>28</v>
@@ -6091,7 +6091,7 @@
         <v>27</v>
       </c>
       <c r="E180" s="11">
-        <v>26</v>
+        <v>29</v>
       </c>
       <c r="F180" s="9" t="s">
         <v>28</v>
@@ -6114,7 +6114,7 @@
         <v>27</v>
       </c>
       <c r="E181" s="11">
-        <v>30</v>
+        <v>17</v>
       </c>
       <c r="F181" s="9" t="s">
         <v>28</v>
@@ -6137,7 +6137,7 @@
         <v>27</v>
       </c>
       <c r="E182" s="11">
-        <v>23</v>
+        <v>9</v>
       </c>
       <c r="F182" s="9" t="s">
         <v>28</v>
@@ -6160,7 +6160,7 @@
         <v>27</v>
       </c>
       <c r="E183" s="11">
-        <v>20</v>
+        <v>31</v>
       </c>
       <c r="F183" s="9" t="s">
         <v>28</v>
@@ -6183,7 +6183,7 @@
         <v>27</v>
       </c>
       <c r="E184" s="11">
-        <v>14</v>
+        <v>11</v>
       </c>
       <c r="F184" s="9" t="s">
         <v>28</v>
@@ -6206,7 +6206,7 @@
         <v>27</v>
       </c>
       <c r="E185" s="11">
-        <v>19</v>
+        <v>29</v>
       </c>
       <c r="F185" s="9" t="s">
         <v>28</v>
@@ -6229,7 +6229,7 @@
         <v>27</v>
       </c>
       <c r="E186" s="11">
-        <v>23</v>
+        <v>14</v>
       </c>
       <c r="F186" s="9" t="s">
         <v>28</v>
@@ -6252,7 +6252,7 @@
         <v>27</v>
       </c>
       <c r="E187" s="11">
-        <v>31</v>
+        <v>23</v>
       </c>
       <c r="F187" s="9" t="s">
         <v>28</v>
@@ -6275,7 +6275,7 @@
         <v>27</v>
       </c>
       <c r="E188" s="11">
-        <v>28</v>
+        <v>19</v>
       </c>
       <c r="F188" s="9" t="s">
         <v>28</v>
@@ -6298,7 +6298,7 @@
         <v>27</v>
       </c>
       <c r="E189" s="11">
-        <v>23</v>
+        <v>10</v>
       </c>
       <c r="F189" s="9" t="s">
         <v>28</v>
@@ -6321,7 +6321,7 @@
         <v>27</v>
       </c>
       <c r="E190" s="11">
-        <v>22</v>
+        <v>25</v>
       </c>
       <c r="F190" s="9" t="s">
         <v>28</v>
@@ -6344,7 +6344,7 @@
         <v>27</v>
       </c>
       <c r="E191" s="11">
-        <v>23</v>
+        <v>10</v>
       </c>
       <c r="F191" s="9" t="s">
         <v>28</v>
@@ -6367,7 +6367,7 @@
         <v>27</v>
       </c>
       <c r="E192" s="11">
-        <v>22</v>
+        <v>31</v>
       </c>
       <c r="F192" s="9" t="s">
         <v>28</v>
@@ -6390,7 +6390,7 @@
         <v>27</v>
       </c>
       <c r="E193" s="11">
-        <v>19</v>
+        <v>15</v>
       </c>
       <c r="F193" s="9" t="s">
         <v>28</v>
@@ -6413,7 +6413,7 @@
         <v>27</v>
       </c>
       <c r="E194" s="11">
-        <v>15</v>
+        <v>13</v>
       </c>
       <c r="F194" s="9" t="s">
         <v>28</v>
@@ -6436,7 +6436,7 @@
         <v>27</v>
       </c>
       <c r="E195" s="11">
-        <v>22</v>
+        <v>28</v>
       </c>
       <c r="F195" s="9" t="s">
         <v>28</v>
@@ -6459,7 +6459,7 @@
         <v>27</v>
       </c>
       <c r="E196" s="11">
-        <v>19</v>
+        <v>25</v>
       </c>
       <c r="F196" s="9" t="s">
         <v>28</v>
@@ -6482,7 +6482,7 @@
         <v>27</v>
       </c>
       <c r="E197" s="11">
-        <v>24</v>
+        <v>27</v>
       </c>
       <c r="F197" s="9" t="s">
         <v>28</v>
@@ -6505,7 +6505,7 @@
         <v>27</v>
       </c>
       <c r="E198" s="11">
-        <v>18</v>
+        <v>16</v>
       </c>
       <c r="F198" s="9" t="s">
         <v>28</v>
@@ -6528,7 +6528,7 @@
         <v>27</v>
       </c>
       <c r="E199" s="11">
-        <v>19</v>
+        <v>13</v>
       </c>
       <c r="F199" s="9" t="s">
         <v>28</v>
@@ -6551,7 +6551,7 @@
         <v>27</v>
       </c>
       <c r="E200" s="11">
-        <v>11</v>
+        <v>14</v>
       </c>
       <c r="F200" s="9" t="s">
         <v>28</v>
@@ -6574,7 +6574,7 @@
         <v>27</v>
       </c>
       <c r="E201" s="11">
-        <v>8</v>
+        <v>30</v>
       </c>
       <c r="F201" s="9" t="s">
         <v>28</v>
@@ -6597,7 +6597,7 @@
         <v>27</v>
       </c>
       <c r="E202" s="11">
-        <v>10</v>
+        <v>18</v>
       </c>
       <c r="F202" s="9" t="s">
         <v>28</v>
@@ -6620,7 +6620,7 @@
         <v>27</v>
       </c>
       <c r="E203" s="11">
-        <v>24</v>
+        <v>12</v>
       </c>
       <c r="F203" s="9" t="s">
         <v>28</v>
@@ -6643,7 +6643,7 @@
         <v>27</v>
       </c>
       <c r="E204" s="11">
-        <v>28</v>
+        <v>13</v>
       </c>
       <c r="F204" s="9" t="s">
         <v>28</v>
@@ -6666,7 +6666,7 @@
         <v>27</v>
       </c>
       <c r="E205" s="11">
-        <v>21</v>
+        <v>17</v>
       </c>
       <c r="F205" s="9" t="s">
         <v>28</v>
@@ -6689,7 +6689,7 @@
         <v>27</v>
       </c>
       <c r="E206" s="11">
-        <v>12</v>
+        <v>16</v>
       </c>
       <c r="F206" s="9" t="s">
         <v>28</v>
@@ -6712,7 +6712,7 @@
         <v>27</v>
       </c>
       <c r="E207" s="11">
-        <v>19</v>
+        <v>14</v>
       </c>
       <c r="F207" s="9" t="s">
         <v>28</v>
@@ -6735,7 +6735,7 @@
         <v>27</v>
       </c>
       <c r="E208" s="11">
-        <v>25</v>
+        <v>18</v>
       </c>
       <c r="F208" s="9" t="s">
         <v>28</v>
@@ -6758,7 +6758,7 @@
         <v>27</v>
       </c>
       <c r="E209" s="11">
-        <v>8</v>
+        <v>19</v>
       </c>
       <c r="F209" s="9" t="s">
         <v>28</v>
@@ -6781,7 +6781,7 @@
         <v>27</v>
       </c>
       <c r="E210" s="11">
-        <v>23</v>
+        <v>25</v>
       </c>
       <c r="F210" s="9" t="s">
         <v>28</v>
@@ -6804,7 +6804,7 @@
         <v>27</v>
       </c>
       <c r="E211" s="11">
-        <v>11</v>
+        <v>24</v>
       </c>
       <c r="F211" s="9" t="s">
         <v>28</v>
@@ -6827,7 +6827,7 @@
         <v>27</v>
       </c>
       <c r="E212" s="11">
-        <v>10</v>
+        <v>20</v>
       </c>
       <c r="F212" s="9" t="s">
         <v>28</v>
@@ -6850,7 +6850,7 @@
         <v>27</v>
       </c>
       <c r="E213" s="11">
-        <v>16</v>
+        <v>29</v>
       </c>
       <c r="F213" s="9" t="s">
         <v>28</v>
@@ -6873,7 +6873,7 @@
         <v>27</v>
       </c>
       <c r="E214" s="11">
-        <v>12</v>
+        <v>27</v>
       </c>
       <c r="F214" s="9" t="s">
         <v>28</v>
@@ -6896,7 +6896,7 @@
         <v>27</v>
       </c>
       <c r="E215" s="11">
-        <v>29</v>
+        <v>22</v>
       </c>
       <c r="F215" s="9" t="s">
         <v>28</v>
@@ -6919,7 +6919,7 @@
         <v>27</v>
       </c>
       <c r="E216" s="11">
-        <v>21</v>
+        <v>8</v>
       </c>
       <c r="F216" s="9" t="s">
         <v>28</v>
@@ -6942,7 +6942,7 @@
         <v>27</v>
       </c>
       <c r="E217" s="11">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="F217" s="9" t="s">
         <v>28</v>
@@ -6965,7 +6965,7 @@
         <v>27</v>
       </c>
       <c r="E218" s="11">
-        <v>18</v>
+        <v>23</v>
       </c>
       <c r="F218" s="9" t="s">
         <v>28</v>
@@ -6988,7 +6988,7 @@
         <v>27</v>
       </c>
       <c r="E219" s="11">
-        <v>30</v>
+        <v>8</v>
       </c>
       <c r="F219" s="9" t="s">
         <v>28</v>
@@ -7011,7 +7011,7 @@
         <v>27</v>
       </c>
       <c r="E220" s="11">
-        <v>9</v>
+        <v>22</v>
       </c>
       <c r="F220" s="9" t="s">
         <v>28</v>
@@ -7034,7 +7034,7 @@
         <v>27</v>
       </c>
       <c r="E221" s="11">
-        <v>29</v>
+        <v>26</v>
       </c>
       <c r="F221" s="9" t="s">
         <v>28</v>
@@ -7057,7 +7057,7 @@
         <v>27</v>
       </c>
       <c r="E222" s="11">
-        <v>10</v>
+        <v>19</v>
       </c>
       <c r="F222" s="9" t="s">
         <v>28</v>
@@ -7080,7 +7080,7 @@
         <v>27</v>
       </c>
       <c r="E223" s="11">
-        <v>27</v>
+        <v>17</v>
       </c>
       <c r="F223" s="9" t="s">
         <v>28</v>
@@ -7103,7 +7103,7 @@
         <v>27</v>
       </c>
       <c r="E224" s="11">
-        <v>11</v>
+        <v>23</v>
       </c>
       <c r="F224" s="9" t="s">
         <v>28</v>
@@ -7126,7 +7126,7 @@
         <v>27</v>
       </c>
       <c r="E225" s="11">
-        <v>17</v>
+        <v>21</v>
       </c>
       <c r="F225" s="9" t="s">
         <v>28</v>
@@ -7149,7 +7149,7 @@
         <v>27</v>
       </c>
       <c r="E226" s="11">
-        <v>25</v>
+        <v>11</v>
       </c>
       <c r="F226" s="9" t="s">
         <v>28</v>
@@ -7218,7 +7218,7 @@
         <v>27</v>
       </c>
       <c r="E229" s="11">
-        <v>13</v>
+        <v>23</v>
       </c>
       <c r="F229" s="9" t="s">
         <v>28</v>
@@ -7241,7 +7241,7 @@
         <v>27</v>
       </c>
       <c r="E230" s="11">
-        <v>15</v>
+        <v>31</v>
       </c>
       <c r="F230" s="9" t="s">
         <v>28</v>
@@ -7264,7 +7264,7 @@
         <v>27</v>
       </c>
       <c r="E231" s="11">
-        <v>19</v>
+        <v>12</v>
       </c>
       <c r="F231" s="9" t="s">
         <v>28</v>
@@ -7287,7 +7287,7 @@
         <v>27</v>
       </c>
       <c r="E232" s="11">
-        <v>16</v>
+        <v>19</v>
       </c>
       <c r="F232" s="9" t="s">
         <v>28</v>
@@ -7310,7 +7310,7 @@
         <v>27</v>
       </c>
       <c r="E233" s="11">
-        <v>14</v>
+        <v>29</v>
       </c>
       <c r="F233" s="9" t="s">
         <v>28</v>
@@ -7333,7 +7333,7 @@
         <v>27</v>
       </c>
       <c r="E234" s="11">
-        <v>16</v>
+        <v>19</v>
       </c>
       <c r="F234" s="9" t="s">
         <v>28</v>
@@ -7356,7 +7356,7 @@
         <v>27</v>
       </c>
       <c r="E235" s="11">
-        <v>11</v>
+        <v>20</v>
       </c>
       <c r="F235" s="9" t="s">
         <v>28</v>
@@ -7379,7 +7379,7 @@
         <v>27</v>
       </c>
       <c r="E236" s="11">
-        <v>14</v>
+        <v>17</v>
       </c>
       <c r="F236" s="9" t="s">
         <v>28</v>
@@ -7425,7 +7425,7 @@
         <v>27</v>
       </c>
       <c r="E238" s="11">
-        <v>29</v>
+        <v>8</v>
       </c>
       <c r="F238" s="9" t="s">
         <v>28</v>
@@ -7448,7 +7448,7 @@
         <v>27</v>
       </c>
       <c r="E239" s="11">
-        <v>24</v>
+        <v>10</v>
       </c>
       <c r="F239" s="9" t="s">
         <v>28</v>
@@ -7471,7 +7471,7 @@
         <v>27</v>
       </c>
       <c r="E240" s="11">
-        <v>9</v>
+        <v>20</v>
       </c>
       <c r="F240" s="9" t="s">
         <v>28</v>
@@ -7494,7 +7494,7 @@
         <v>27</v>
       </c>
       <c r="E241" s="11">
-        <v>31</v>
+        <v>25</v>
       </c>
       <c r="F241" s="9" t="s">
         <v>28</v>
@@ -7517,7 +7517,7 @@
         <v>27</v>
       </c>
       <c r="E242" s="11">
-        <v>31</v>
+        <v>8</v>
       </c>
       <c r="F242" s="9" t="s">
         <v>28</v>
@@ -7540,7 +7540,7 @@
         <v>27</v>
       </c>
       <c r="E243" s="11">
-        <v>15</v>
+        <v>21</v>
       </c>
       <c r="F243" s="9" t="s">
         <v>28</v>
@@ -7563,7 +7563,7 @@
         <v>27</v>
       </c>
       <c r="E244" s="11">
-        <v>15</v>
+        <v>11</v>
       </c>
       <c r="F244" s="9" t="s">
         <v>28</v>
@@ -7586,7 +7586,7 @@
         <v>27</v>
       </c>
       <c r="E245" s="11">
-        <v>24</v>
+        <v>9</v>
       </c>
       <c r="F245" s="9" t="s">
         <v>28</v>
@@ -7609,7 +7609,7 @@
         <v>27</v>
       </c>
       <c r="E246" s="11">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="F246" s="9" t="s">
         <v>28</v>
@@ -7632,7 +7632,7 @@
         <v>27</v>
       </c>
       <c r="E247" s="11">
-        <v>30</v>
+        <v>18</v>
       </c>
       <c r="F247" s="9" t="s">
         <v>28</v>
@@ -7655,7 +7655,7 @@
         <v>27</v>
       </c>
       <c r="E248" s="11">
-        <v>20</v>
+        <v>8</v>
       </c>
       <c r="F248" s="9" t="s">
         <v>28</v>
@@ -7678,7 +7678,7 @@
         <v>27</v>
       </c>
       <c r="E249" s="11">
-        <v>30</v>
+        <v>18</v>
       </c>
       <c r="F249" s="9" t="s">
         <v>28</v>
@@ -7701,7 +7701,7 @@
         <v>27</v>
       </c>
       <c r="E250" s="11">
-        <v>12</v>
+        <v>24</v>
       </c>
       <c r="F250" s="9" t="s">
         <v>28</v>
@@ -7724,7 +7724,7 @@
         <v>27</v>
       </c>
       <c r="E251" s="11">
-        <v>31</v>
+        <v>17</v>
       </c>
       <c r="F251" s="9" t="s">
         <v>28</v>
@@ -7747,7 +7747,7 @@
         <v>27</v>
       </c>
       <c r="E252" s="11">
-        <v>11</v>
+        <v>31</v>
       </c>
       <c r="F252" s="9" t="s">
         <v>28</v>
@@ -7793,7 +7793,7 @@
         <v>27</v>
       </c>
       <c r="E254" s="11">
-        <v>29</v>
+        <v>10</v>
       </c>
       <c r="F254" s="9" t="s">
         <v>28</v>
@@ -7816,7 +7816,7 @@
         <v>27</v>
       </c>
       <c r="E255" s="11">
-        <v>21</v>
+        <v>27</v>
       </c>
       <c r="F255" s="9" t="s">
         <v>28</v>
@@ -7839,7 +7839,7 @@
         <v>27</v>
       </c>
       <c r="E256" s="11">
-        <v>19</v>
+        <v>28</v>
       </c>
       <c r="F256" s="9" t="s">
         <v>28</v>
@@ -7862,7 +7862,7 @@
         <v>27</v>
       </c>
       <c r="E257" s="11">
-        <v>16</v>
+        <v>26</v>
       </c>
       <c r="F257" s="9" t="s">
         <v>28</v>
@@ -7885,7 +7885,7 @@
         <v>27</v>
       </c>
       <c r="E258" s="11">
-        <v>11</v>
+        <v>31</v>
       </c>
       <c r="F258" s="9" t="s">
         <v>28</v>
@@ -7908,7 +7908,7 @@
         <v>27</v>
       </c>
       <c r="E259" s="11">
-        <v>14</v>
+        <v>23</v>
       </c>
       <c r="F259" s="9" t="s">
         <v>28</v>
@@ -7931,7 +7931,7 @@
         <v>27</v>
       </c>
       <c r="E260" s="11">
-        <v>10</v>
+        <v>23</v>
       </c>
       <c r="F260" s="9" t="s">
         <v>28</v>
@@ -7954,7 +7954,7 @@
         <v>27</v>
       </c>
       <c r="E261" s="11">
-        <v>26</v>
+        <v>22</v>
       </c>
       <c r="F261" s="9" t="s">
         <v>28</v>
@@ -7977,7 +7977,7 @@
         <v>27</v>
       </c>
       <c r="E262" s="11">
-        <v>13</v>
+        <v>21</v>
       </c>
       <c r="F262" s="9" t="s">
         <v>28</v>
@@ -8000,7 +8000,7 @@
         <v>27</v>
       </c>
       <c r="E263" s="11">
-        <v>9</v>
+        <v>14</v>
       </c>
       <c r="F263" s="9" t="s">
         <v>28</v>
@@ -8023,7 +8023,7 @@
         <v>27</v>
       </c>
       <c r="E264" s="11">
-        <v>21</v>
+        <v>30</v>
       </c>
       <c r="F264" s="9" t="s">
         <v>28</v>
@@ -8046,7 +8046,7 @@
         <v>27</v>
       </c>
       <c r="E265" s="11">
-        <v>15</v>
+        <v>25</v>
       </c>
       <c r="F265" s="9" t="s">
         <v>28</v>
@@ -8069,7 +8069,7 @@
         <v>27</v>
       </c>
       <c r="E266" s="11">
-        <v>29</v>
+        <v>17</v>
       </c>
       <c r="F266" s="9" t="s">
         <v>28</v>
@@ -8092,7 +8092,7 @@
         <v>27</v>
       </c>
       <c r="E267" s="11">
-        <v>23</v>
+        <v>14</v>
       </c>
       <c r="F267" s="9" t="s">
         <v>28</v>
@@ -8115,7 +8115,7 @@
         <v>27</v>
       </c>
       <c r="E268" s="11">
-        <v>14</v>
+        <v>30</v>
       </c>
       <c r="F268" s="9" t="s">
         <v>28</v>
@@ -8138,7 +8138,7 @@
         <v>27</v>
       </c>
       <c r="E269" s="11">
-        <v>14</v>
+        <v>10</v>
       </c>
       <c r="F269" s="9" t="s">
         <v>28</v>
@@ -8161,7 +8161,7 @@
         <v>27</v>
       </c>
       <c r="E270" s="11">
-        <v>18</v>
+        <v>12</v>
       </c>
       <c r="F270" s="9" t="s">
         <v>28</v>
@@ -8184,7 +8184,7 @@
         <v>27</v>
       </c>
       <c r="E271" s="11">
-        <v>18</v>
+        <v>9</v>
       </c>
       <c r="F271" s="9" t="s">
         <v>28</v>
@@ -8207,7 +8207,7 @@
         <v>27</v>
       </c>
       <c r="E272" s="11">
-        <v>9</v>
+        <v>28</v>
       </c>
       <c r="F272" s="9" t="s">
         <v>28</v>
@@ -8230,7 +8230,7 @@
         <v>27</v>
       </c>
       <c r="E273" s="11">
-        <v>18</v>
+        <v>25</v>
       </c>
       <c r="F273" s="9" t="s">
         <v>28</v>
@@ -8253,7 +8253,7 @@
         <v>27</v>
       </c>
       <c r="E274" s="11">
-        <v>28</v>
+        <v>31</v>
       </c>
       <c r="F274" s="9" t="s">
         <v>28</v>
@@ -8276,7 +8276,7 @@
         <v>27</v>
       </c>
       <c r="E275" s="11">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="F275" s="9" t="s">
         <v>28</v>
@@ -8299,7 +8299,7 @@
         <v>27</v>
       </c>
       <c r="E276" s="11">
-        <v>20</v>
+        <v>14</v>
       </c>
       <c r="F276" s="9" t="s">
         <v>28</v>
@@ -8322,7 +8322,7 @@
         <v>27</v>
       </c>
       <c r="E277" s="11">
-        <v>11</v>
+        <v>20</v>
       </c>
       <c r="F277" s="9" t="s">
         <v>28</v>
@@ -8345,7 +8345,7 @@
         <v>27</v>
       </c>
       <c r="E278" s="11">
-        <v>22</v>
+        <v>20</v>
       </c>
       <c r="F278" s="9" t="s">
         <v>28</v>
@@ -8414,7 +8414,7 @@
         <v>27</v>
       </c>
       <c r="E281" s="11">
-        <v>13</v>
+        <v>31</v>
       </c>
       <c r="F281" s="9" t="s">
         <v>28</v>
@@ -8437,7 +8437,7 @@
         <v>27</v>
       </c>
       <c r="E282" s="11">
-        <v>19</v>
+        <v>25</v>
       </c>
       <c r="F282" s="9" t="s">
         <v>28</v>
@@ -8460,7 +8460,7 @@
         <v>27</v>
       </c>
       <c r="E283" s="11">
-        <v>27</v>
+        <v>16</v>
       </c>
       <c r="F283" s="9" t="s">
         <v>28</v>
@@ -8483,7 +8483,7 @@
         <v>27</v>
       </c>
       <c r="E284" s="11">
-        <v>11</v>
+        <v>9</v>
       </c>
       <c r="F284" s="9" t="s">
         <v>28</v>
@@ -8506,7 +8506,7 @@
         <v>27</v>
       </c>
       <c r="E285" s="11">
-        <v>23</v>
+        <v>18</v>
       </c>
       <c r="F285" s="9" t="s">
         <v>28</v>
@@ -8529,7 +8529,7 @@
         <v>27</v>
       </c>
       <c r="E286" s="11">
-        <v>11</v>
+        <v>17</v>
       </c>
       <c r="F286" s="9" t="s">
         <v>28</v>
@@ -8552,7 +8552,7 @@
         <v>27</v>
       </c>
       <c r="E287" s="11">
-        <v>9</v>
+        <v>17</v>
       </c>
       <c r="F287" s="9" t="s">
         <v>28</v>
@@ -8575,7 +8575,7 @@
         <v>27</v>
       </c>
       <c r="E288" s="11">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="F288" s="9" t="s">
         <v>28</v>
@@ -8598,7 +8598,7 @@
         <v>27</v>
       </c>
       <c r="E289" s="11">
-        <v>22</v>
+        <v>10</v>
       </c>
       <c r="F289" s="9" t="s">
         <v>28</v>
@@ -8621,7 +8621,7 @@
         <v>27</v>
       </c>
       <c r="E290" s="11">
-        <v>16</v>
+        <v>30</v>
       </c>
       <c r="F290" s="9" t="s">
         <v>28</v>
@@ -8644,7 +8644,7 @@
         <v>27</v>
       </c>
       <c r="E291" s="11">
-        <v>21</v>
+        <v>27</v>
       </c>
       <c r="F291" s="9" t="s">
         <v>28</v>
@@ -8667,7 +8667,7 @@
         <v>27</v>
       </c>
       <c r="E292" s="11">
-        <v>14</v>
+        <v>20</v>
       </c>
       <c r="F292" s="9" t="s">
         <v>28</v>
@@ -8690,7 +8690,7 @@
         <v>27</v>
       </c>
       <c r="E293" s="11">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="F293" s="9" t="s">
         <v>28</v>
@@ -8713,7 +8713,7 @@
         <v>27</v>
       </c>
       <c r="E294" s="11">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="F294" s="9" t="s">
         <v>28</v>
@@ -8736,7 +8736,7 @@
         <v>27</v>
       </c>
       <c r="E295" s="11">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="F295" s="9" t="s">
         <v>28</v>
@@ -8759,7 +8759,7 @@
         <v>27</v>
       </c>
       <c r="E296" s="11">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="F296" s="9" t="s">
         <v>28</v>
@@ -8782,7 +8782,7 @@
         <v>27</v>
       </c>
       <c r="E297" s="11">
-        <v>30</v>
+        <v>15</v>
       </c>
       <c r="F297" s="9" t="s">
         <v>28</v>
@@ -8805,7 +8805,7 @@
         <v>27</v>
       </c>
       <c r="E298" s="11">
-        <v>11</v>
+        <v>25</v>
       </c>
       <c r="F298" s="9" t="s">
         <v>28</v>
@@ -8828,7 +8828,7 @@
         <v>27</v>
       </c>
       <c r="E299" s="11">
-        <v>19</v>
+        <v>21</v>
       </c>
       <c r="F299" s="9" t="s">
         <v>28</v>
@@ -8851,7 +8851,7 @@
         <v>27</v>
       </c>
       <c r="E300" s="11">
-        <v>18</v>
+        <v>15</v>
       </c>
       <c r="F300" s="9" t="s">
         <v>28</v>
@@ -8874,7 +8874,7 @@
         <v>27</v>
       </c>
       <c r="E301" s="11">
-        <v>12</v>
+        <v>23</v>
       </c>
       <c r="F301" s="9" t="s">
         <v>28</v>
@@ -8897,7 +8897,7 @@
         <v>27</v>
       </c>
       <c r="E302" s="11">
-        <v>30</v>
+        <v>13</v>
       </c>
       <c r="F302" s="9" t="s">
         <v>28</v>
@@ -8920,7 +8920,7 @@
         <v>27</v>
       </c>
       <c r="E303" s="11">
-        <v>14</v>
+        <v>16</v>
       </c>
       <c r="F303" s="9" t="s">
         <v>28</v>
@@ -8943,7 +8943,7 @@
         <v>27</v>
       </c>
       <c r="E304" s="11">
-        <v>15</v>
+        <v>25</v>
       </c>
       <c r="F304" s="9" t="s">
         <v>28</v>
@@ -8966,7 +8966,7 @@
         <v>27</v>
       </c>
       <c r="E305" s="11">
-        <v>29</v>
+        <v>8</v>
       </c>
       <c r="F305" s="9" t="s">
         <v>28</v>
@@ -8989,7 +8989,7 @@
         <v>27</v>
       </c>
       <c r="E306" s="11">
-        <v>14</v>
+        <v>18</v>
       </c>
       <c r="F306" s="9" t="s">
         <v>28</v>
@@ -9012,7 +9012,7 @@
         <v>27</v>
       </c>
       <c r="E307" s="11">
-        <v>24</v>
+        <v>21</v>
       </c>
       <c r="F307" s="9" t="s">
         <v>28</v>
@@ -9035,7 +9035,7 @@
         <v>27</v>
       </c>
       <c r="E308" s="11">
-        <v>31</v>
+        <v>18</v>
       </c>
       <c r="F308" s="9" t="s">
         <v>28</v>
@@ -9058,7 +9058,7 @@
         <v>27</v>
       </c>
       <c r="E309" s="11">
-        <v>31</v>
+        <v>11</v>
       </c>
       <c r="F309" s="9" t="s">
         <v>28</v>
@@ -9081,7 +9081,7 @@
         <v>27</v>
       </c>
       <c r="E310" s="11">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="F310" s="9" t="s">
         <v>28</v>
@@ -9104,7 +9104,7 @@
         <v>27</v>
       </c>
       <c r="E311" s="11">
-        <v>13</v>
+        <v>23</v>
       </c>
       <c r="F311" s="9" t="s">
         <v>28</v>
@@ -9127,7 +9127,7 @@
         <v>27</v>
       </c>
       <c r="E312" s="11">
-        <v>11</v>
+        <v>28</v>
       </c>
       <c r="F312" s="9" t="s">
         <v>28</v>
@@ -9150,7 +9150,7 @@
         <v>27</v>
       </c>
       <c r="E313" s="11">
-        <v>26</v>
+        <v>18</v>
       </c>
       <c r="F313" s="9" t="s">
         <v>28</v>
@@ -9173,7 +9173,7 @@
         <v>27</v>
       </c>
       <c r="E314" s="11">
-        <v>16</v>
+        <v>26</v>
       </c>
       <c r="F314" s="9" t="s">
         <v>28</v>
@@ -9196,7 +9196,7 @@
         <v>27</v>
       </c>
       <c r="E315" s="11">
-        <v>21</v>
+        <v>25</v>
       </c>
       <c r="F315" s="9" t="s">
         <v>28</v>
@@ -9219,7 +9219,7 @@
         <v>27</v>
       </c>
       <c r="E316" s="11">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="F316" s="9" t="s">
         <v>28</v>
@@ -9242,7 +9242,7 @@
         <v>27</v>
       </c>
       <c r="E317" s="11">
-        <v>25</v>
+        <v>10</v>
       </c>
       <c r="F317" s="9" t="s">
         <v>28</v>
@@ -9265,7 +9265,7 @@
         <v>27</v>
       </c>
       <c r="E318" s="11">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="F318" s="9" t="s">
         <v>28</v>
@@ -9288,7 +9288,7 @@
         <v>27</v>
       </c>
       <c r="E319" s="11">
-        <v>26</v>
+        <v>19</v>
       </c>
       <c r="F319" s="9" t="s">
         <v>28</v>
@@ -9311,7 +9311,7 @@
         <v>27</v>
       </c>
       <c r="E320" s="11">
-        <v>25</v>
+        <v>29</v>
       </c>
       <c r="F320" s="9" t="s">
         <v>28</v>
@@ -9334,7 +9334,7 @@
         <v>27</v>
       </c>
       <c r="E321" s="11">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="F321" s="9" t="s">
         <v>28</v>
@@ -9380,7 +9380,7 @@
         <v>27</v>
       </c>
       <c r="E323" s="11">
-        <v>19</v>
+        <v>17</v>
       </c>
       <c r="F323" s="9" t="s">
         <v>28</v>
@@ -9403,7 +9403,7 @@
         <v>27</v>
       </c>
       <c r="E324" s="11">
-        <v>17</v>
+        <v>10</v>
       </c>
       <c r="F324" s="9" t="s">
         <v>28</v>
@@ -9426,7 +9426,7 @@
         <v>27</v>
       </c>
       <c r="E325" s="11">
-        <v>26</v>
+        <v>16</v>
       </c>
       <c r="F325" s="9" t="s">
         <v>28</v>
@@ -9449,7 +9449,7 @@
         <v>27</v>
       </c>
       <c r="E326" s="11">
-        <v>18</v>
+        <v>20</v>
       </c>
       <c r="F326" s="9" t="s">
         <v>28</v>
@@ -9472,7 +9472,7 @@
         <v>27</v>
       </c>
       <c r="E327" s="11">
-        <v>12</v>
+        <v>22</v>
       </c>
       <c r="F327" s="9" t="s">
         <v>28</v>
@@ -9495,7 +9495,7 @@
         <v>27</v>
       </c>
       <c r="E328" s="11">
-        <v>23</v>
+        <v>27</v>
       </c>
       <c r="F328" s="9" t="s">
         <v>28</v>
@@ -9518,7 +9518,7 @@
         <v>27</v>
       </c>
       <c r="E329" s="11">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="F329" s="9" t="s">
         <v>28</v>
@@ -9541,7 +9541,7 @@
         <v>27</v>
       </c>
       <c r="E330" s="11">
-        <v>25</v>
+        <v>8</v>
       </c>
       <c r="F330" s="9" t="s">
         <v>28</v>
@@ -9564,7 +9564,7 @@
         <v>27</v>
       </c>
       <c r="E331" s="11">
-        <v>25</v>
+        <v>27</v>
       </c>
       <c r="F331" s="9" t="s">
         <v>28</v>
@@ -9587,7 +9587,7 @@
         <v>27</v>
       </c>
       <c r="E332" s="11">
-        <v>11</v>
+        <v>8</v>
       </c>
       <c r="F332" s="9" t="s">
         <v>28</v>
@@ -9610,7 +9610,7 @@
         <v>27</v>
       </c>
       <c r="E333" s="11">
-        <v>22</v>
+        <v>24</v>
       </c>
       <c r="F333" s="9" t="s">
         <v>28</v>
@@ -9633,7 +9633,7 @@
         <v>27</v>
       </c>
       <c r="E334" s="11">
-        <v>14</v>
+        <v>22</v>
       </c>
       <c r="F334" s="9" t="s">
         <v>28</v>
@@ -9656,7 +9656,7 @@
         <v>27</v>
       </c>
       <c r="E335" s="11">
-        <v>12</v>
+        <v>8</v>
       </c>
       <c r="F335" s="9" t="s">
         <v>28</v>
@@ -9679,7 +9679,7 @@
         <v>27</v>
       </c>
       <c r="E336" s="11">
-        <v>23</v>
+        <v>31</v>
       </c>
       <c r="F336" s="9" t="s">
         <v>28</v>
@@ -9702,7 +9702,7 @@
         <v>27</v>
       </c>
       <c r="E337" s="11">
-        <v>23</v>
+        <v>28</v>
       </c>
       <c r="F337" s="9" t="s">
         <v>28</v>
@@ -9725,7 +9725,7 @@
         <v>27</v>
       </c>
       <c r="E338" s="11">
-        <v>15</v>
+        <v>24</v>
       </c>
       <c r="F338" s="9" t="s">
         <v>28</v>
@@ -9748,7 +9748,7 @@
         <v>27</v>
       </c>
       <c r="E339" s="11">
-        <v>20</v>
+        <v>15</v>
       </c>
       <c r="F339" s="9" t="s">
         <v>28</v>
@@ -9771,7 +9771,7 @@
         <v>27</v>
       </c>
       <c r="E340" s="11">
-        <v>19</v>
+        <v>8</v>
       </c>
       <c r="F340" s="9" t="s">
         <v>28</v>
@@ -9794,7 +9794,7 @@
         <v>27</v>
       </c>
       <c r="E341" s="11">
-        <v>25</v>
+        <v>31</v>
       </c>
       <c r="F341" s="9" t="s">
         <v>28</v>
@@ -9817,7 +9817,7 @@
         <v>27</v>
       </c>
       <c r="E342" s="11">
-        <v>26</v>
+        <v>30</v>
       </c>
       <c r="F342" s="9" t="s">
         <v>28</v>
@@ -9840,7 +9840,7 @@
         <v>27</v>
       </c>
       <c r="E343" s="11">
-        <v>18</v>
+        <v>22</v>
       </c>
       <c r="F343" s="9" t="s">
         <v>28</v>
@@ -9863,7 +9863,7 @@
         <v>27</v>
       </c>
       <c r="E344" s="11">
-        <v>13</v>
+        <v>17</v>
       </c>
       <c r="F344" s="9" t="s">
         <v>28</v>
@@ -9886,7 +9886,7 @@
         <v>27</v>
       </c>
       <c r="E345" s="11">
-        <v>13</v>
+        <v>16</v>
       </c>
       <c r="F345" s="9" t="s">
         <v>28</v>
@@ -9909,7 +9909,7 @@
         <v>27</v>
       </c>
       <c r="E346" s="11">
-        <v>15</v>
+        <v>26</v>
       </c>
       <c r="F346" s="9" t="s">
         <v>28</v>
@@ -9955,7 +9955,7 @@
         <v>27</v>
       </c>
       <c r="E348" s="11">
-        <v>9</v>
+        <v>24</v>
       </c>
       <c r="F348" s="9" t="s">
         <v>28</v>
@@ -9978,7 +9978,7 @@
         <v>27</v>
       </c>
       <c r="E349" s="11">
-        <v>20</v>
+        <v>23</v>
       </c>
       <c r="F349" s="9" t="s">
         <v>28</v>
@@ -10001,7 +10001,7 @@
         <v>27</v>
       </c>
       <c r="E350" s="11">
-        <v>29</v>
+        <v>22</v>
       </c>
       <c r="F350" s="9" t="s">
         <v>28</v>
@@ -10024,7 +10024,7 @@
         <v>27</v>
       </c>
       <c r="E351" s="11">
-        <v>25</v>
+        <v>13</v>
       </c>
       <c r="F351" s="9" t="s">
         <v>28</v>
@@ -10047,7 +10047,7 @@
         <v>27</v>
       </c>
       <c r="E352" s="11">
-        <v>27</v>
+        <v>9</v>
       </c>
       <c r="F352" s="9" t="s">
         <v>28</v>
@@ -10070,7 +10070,7 @@
         <v>27</v>
       </c>
       <c r="E353" s="11">
-        <v>10</v>
+        <v>14</v>
       </c>
       <c r="F353" s="9" t="s">
         <v>28</v>
@@ -10093,7 +10093,7 @@
         <v>27</v>
       </c>
       <c r="E354" s="11">
-        <v>9</v>
+        <v>23</v>
       </c>
       <c r="F354" s="9" t="s">
         <v>28</v>
@@ -10116,7 +10116,7 @@
         <v>27</v>
       </c>
       <c r="E355" s="11">
-        <v>9</v>
+        <v>16</v>
       </c>
       <c r="F355" s="9" t="s">
         <v>28</v>
@@ -10139,7 +10139,7 @@
         <v>27</v>
       </c>
       <c r="E356" s="11">
-        <v>11</v>
+        <v>19</v>
       </c>
       <c r="F356" s="9" t="s">
         <v>28</v>
@@ -10162,7 +10162,7 @@
         <v>27</v>
       </c>
       <c r="E357" s="11">
-        <v>19</v>
+        <v>17</v>
       </c>
       <c r="F357" s="9" t="s">
         <v>28</v>
@@ -10185,7 +10185,7 @@
         <v>27</v>
       </c>
       <c r="E358" s="11">
-        <v>31</v>
+        <v>26</v>
       </c>
       <c r="F358" s="9" t="s">
         <v>28</v>
@@ -10208,7 +10208,7 @@
         <v>27</v>
       </c>
       <c r="E359" s="11">
-        <v>15</v>
+        <v>8</v>
       </c>
       <c r="F359" s="9" t="s">
         <v>28</v>
@@ -10231,7 +10231,7 @@
         <v>27</v>
       </c>
       <c r="E360" s="11">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="F360" s="9" t="s">
         <v>28</v>
@@ -10254,7 +10254,7 @@
         <v>27</v>
       </c>
       <c r="E361" s="11">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="F361" s="9" t="s">
         <v>28</v>
@@ -10277,7 +10277,7 @@
         <v>27</v>
       </c>
       <c r="E362" s="11">
-        <v>12</v>
+        <v>10</v>
       </c>
       <c r="F362" s="9" t="s">
         <v>28</v>
@@ -10300,7 +10300,7 @@
         <v>27</v>
       </c>
       <c r="E363" s="11">
-        <v>19</v>
+        <v>14</v>
       </c>
       <c r="F363" s="9" t="s">
         <v>28</v>
@@ -10323,7 +10323,7 @@
         <v>27</v>
       </c>
       <c r="E364" s="11">
-        <v>31</v>
+        <v>19</v>
       </c>
       <c r="F364" s="9" t="s">
         <v>28</v>
@@ -10346,7 +10346,7 @@
         <v>27</v>
       </c>
       <c r="E365" s="11">
-        <v>11</v>
+        <v>14</v>
       </c>
       <c r="F365" s="9" t="s">
         <v>28</v>
@@ -10369,7 +10369,7 @@
         <v>27</v>
       </c>
       <c r="E366" s="11">
-        <v>21</v>
+        <v>15</v>
       </c>
       <c r="F366" s="9" t="s">
         <v>28</v>
@@ -10392,7 +10392,7 @@
         <v>27</v>
       </c>
       <c r="E367" s="11">
-        <v>19</v>
+        <v>10</v>
       </c>
       <c r="F367" s="9" t="s">
         <v>28</v>
@@ -10415,7 +10415,7 @@
         <v>27</v>
       </c>
       <c r="E368" s="11">
-        <v>13</v>
+        <v>26</v>
       </c>
       <c r="F368" s="9" t="s">
         <v>28</v>
@@ -10438,7 +10438,7 @@
         <v>27</v>
       </c>
       <c r="E369" s="11">
-        <v>20</v>
+        <v>17</v>
       </c>
       <c r="F369" s="9" t="s">
         <v>28</v>
@@ -10461,7 +10461,7 @@
         <v>27</v>
       </c>
       <c r="E370" s="11">
-        <v>18</v>
+        <v>15</v>
       </c>
       <c r="F370" s="9" t="s">
         <v>28</v>
@@ -10484,7 +10484,7 @@
         <v>27</v>
       </c>
       <c r="E371" s="11">
-        <v>26</v>
+        <v>28</v>
       </c>
       <c r="F371" s="9" t="s">
         <v>28</v>
@@ -10507,7 +10507,7 @@
         <v>27</v>
       </c>
       <c r="E372" s="11">
-        <v>23</v>
+        <v>10</v>
       </c>
       <c r="F372" s="9" t="s">
         <v>28</v>
@@ -10530,7 +10530,7 @@
         <v>27</v>
       </c>
       <c r="E373" s="11">
-        <v>11</v>
+        <v>14</v>
       </c>
       <c r="F373" s="9" t="s">
         <v>28</v>
@@ -10553,7 +10553,7 @@
         <v>27</v>
       </c>
       <c r="E374" s="11">
-        <v>18</v>
+        <v>21</v>
       </c>
       <c r="F374" s="9" t="s">
         <v>28</v>
@@ -10576,7 +10576,7 @@
         <v>27</v>
       </c>
       <c r="E375" s="11">
-        <v>27</v>
+        <v>8</v>
       </c>
       <c r="F375" s="9" t="s">
         <v>28</v>
@@ -10599,7 +10599,7 @@
         <v>27</v>
       </c>
       <c r="E376" s="11">
-        <v>12</v>
+        <v>27</v>
       </c>
       <c r="F376" s="9" t="s">
         <v>28</v>
@@ -10622,7 +10622,7 @@
         <v>27</v>
       </c>
       <c r="E377" s="11">
-        <v>27</v>
+        <v>22</v>
       </c>
       <c r="F377" s="9" t="s">
         <v>28</v>
@@ -10645,7 +10645,7 @@
         <v>27</v>
       </c>
       <c r="E378" s="11">
-        <v>22</v>
+        <v>29</v>
       </c>
       <c r="F378" s="9" t="s">
         <v>28</v>
@@ -10668,7 +10668,7 @@
         <v>27</v>
       </c>
       <c r="E379" s="11">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="F379" s="9" t="s">
         <v>28</v>
@@ -10691,7 +10691,7 @@
         <v>27</v>
       </c>
       <c r="E380" s="11">
-        <v>29</v>
+        <v>15</v>
       </c>
       <c r="F380" s="9" t="s">
         <v>28</v>
@@ -10714,7 +10714,7 @@
         <v>27</v>
       </c>
       <c r="E381" s="11">
-        <v>17</v>
+        <v>14</v>
       </c>
       <c r="F381" s="9" t="s">
         <v>28</v>
@@ -10760,7 +10760,7 @@
         <v>27</v>
       </c>
       <c r="E383" s="11">
-        <v>20</v>
+        <v>8</v>
       </c>
       <c r="F383" s="9" t="s">
         <v>28</v>
@@ -10783,7 +10783,7 @@
         <v>27</v>
       </c>
       <c r="E384" s="11">
-        <v>15</v>
+        <v>31</v>
       </c>
       <c r="F384" s="9" t="s">
         <v>28</v>
@@ -10806,7 +10806,7 @@
         <v>27</v>
       </c>
       <c r="E385" s="11">
-        <v>28</v>
+        <v>11</v>
       </c>
       <c r="F385" s="9" t="s">
         <v>28</v>
@@ -10829,7 +10829,7 @@
         <v>27</v>
       </c>
       <c r="E386" s="11">
-        <v>26</v>
+        <v>16</v>
       </c>
       <c r="F386" s="9" t="s">
         <v>28</v>
@@ -10852,7 +10852,7 @@
         <v>27</v>
       </c>
       <c r="E387" s="11">
-        <v>31</v>
+        <v>15</v>
       </c>
       <c r="F387" s="9" t="s">
         <v>28</v>
@@ -10875,7 +10875,7 @@
         <v>27</v>
       </c>
       <c r="E388" s="11">
-        <v>21</v>
+        <v>11</v>
       </c>
       <c r="F388" s="9" t="s">
         <v>28</v>
@@ -10898,7 +10898,7 @@
         <v>27</v>
       </c>
       <c r="E389" s="11">
-        <v>28</v>
+        <v>8</v>
       </c>
       <c r="F389" s="9" t="s">
         <v>28</v>
@@ -10921,7 +10921,7 @@
         <v>27</v>
       </c>
       <c r="E390" s="11">
-        <v>9</v>
+        <v>11</v>
       </c>
       <c r="F390" s="9" t="s">
         <v>28</v>
@@ -10944,7 +10944,7 @@
         <v>27</v>
       </c>
       <c r="E391" s="11">
-        <v>19</v>
+        <v>21</v>
       </c>
       <c r="F391" s="9" t="s">
         <v>28</v>
@@ -10967,7 +10967,7 @@
         <v>27</v>
       </c>
       <c r="E392" s="11">
-        <v>27</v>
+        <v>21</v>
       </c>
       <c r="F392" s="9" t="s">
         <v>28</v>
@@ -10990,7 +10990,7 @@
         <v>27</v>
       </c>
       <c r="E393" s="11">
-        <v>9</v>
+        <v>27</v>
       </c>
       <c r="F393" s="9" t="s">
         <v>28</v>
@@ -11036,7 +11036,7 @@
         <v>27</v>
       </c>
       <c r="E395" s="11">
-        <v>9</v>
+        <v>29</v>
       </c>
       <c r="F395" s="9" t="s">
         <v>28</v>
@@ -11059,7 +11059,7 @@
         <v>27</v>
       </c>
       <c r="E396" s="11">
-        <v>25</v>
+        <v>31</v>
       </c>
       <c r="F396" s="9" t="s">
         <v>28</v>
@@ -11082,7 +11082,7 @@
         <v>27</v>
       </c>
       <c r="E397" s="11">
-        <v>11</v>
+        <v>17</v>
       </c>
       <c r="F397" s="9" t="s">
         <v>28</v>
@@ -11105,7 +11105,7 @@
         <v>27</v>
       </c>
       <c r="E398" s="11">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="F398" s="9" t="s">
         <v>28</v>
@@ -11128,7 +11128,7 @@
         <v>27</v>
       </c>
       <c r="E399" s="11">
-        <v>13</v>
+        <v>16</v>
       </c>
       <c r="F399" s="9" t="s">
         <v>28</v>
@@ -11151,7 +11151,7 @@
         <v>27</v>
       </c>
       <c r="E400" s="11">
-        <v>8</v>
+        <v>28</v>
       </c>
       <c r="F400" s="9" t="s">
         <v>28</v>
@@ -11174,7 +11174,7 @@
         <v>27</v>
       </c>
       <c r="E401" s="11">
-        <v>10</v>
+        <v>16</v>
       </c>
       <c r="F401" s="9" t="s">
         <v>28</v>

</xml_diff>

<commit_message>
feat(search): add live product recommendations dropdown while typing in search bar
</commit_message>
<xml_diff>
--- a/all-test-reports/selenium/selenium_e2e_test_report.xlsx
+++ b/all-test-reports/selenium/selenium_e2e_test_report.xlsx
@@ -35,7 +35,7 @@
     <t>Execution Date</t>
   </si>
   <si>
-    <t>28/7/2026, 10:34:33 am</t>
+    <t>28/7/2026, 10:42:38 am</t>
   </si>
   <si>
     <t>Browser / Mode</t>
@@ -98,7 +98,7 @@
     <t>PASS</t>
   </si>
   <si>
-    <t>10:34:33 am</t>
+    <t>10:42:38 am</t>
   </si>
   <si>
     <t>N/A</t>
@@ -1997,7 +1997,7 @@
         <v>27</v>
       </c>
       <c r="E2" s="11">
-        <v>18</v>
+        <v>12</v>
       </c>
       <c r="F2" s="9" t="s">
         <v>28</v>
@@ -2020,7 +2020,7 @@
         <v>27</v>
       </c>
       <c r="E3" s="11">
-        <v>12</v>
+        <v>28</v>
       </c>
       <c r="F3" s="9" t="s">
         <v>28</v>
@@ -2043,7 +2043,7 @@
         <v>27</v>
       </c>
       <c r="E4" s="11">
-        <v>28</v>
+        <v>23</v>
       </c>
       <c r="F4" s="9" t="s">
         <v>28</v>
@@ -2066,7 +2066,7 @@
         <v>27</v>
       </c>
       <c r="E5" s="11">
-        <v>29</v>
+        <v>9</v>
       </c>
       <c r="F5" s="9" t="s">
         <v>28</v>
@@ -2089,7 +2089,7 @@
         <v>27</v>
       </c>
       <c r="E6" s="11">
-        <v>14</v>
+        <v>8</v>
       </c>
       <c r="F6" s="9" t="s">
         <v>28</v>
@@ -2112,7 +2112,7 @@
         <v>27</v>
       </c>
       <c r="E7" s="11">
-        <v>23</v>
+        <v>19</v>
       </c>
       <c r="F7" s="9" t="s">
         <v>28</v>
@@ -2135,7 +2135,7 @@
         <v>27</v>
       </c>
       <c r="E8" s="11">
-        <v>21</v>
+        <v>27</v>
       </c>
       <c r="F8" s="9" t="s">
         <v>28</v>
@@ -2158,7 +2158,7 @@
         <v>27</v>
       </c>
       <c r="E9" s="11">
-        <v>16</v>
+        <v>11</v>
       </c>
       <c r="F9" s="9" t="s">
         <v>28</v>
@@ -2181,7 +2181,7 @@
         <v>27</v>
       </c>
       <c r="E10" s="11">
-        <v>20</v>
+        <v>13</v>
       </c>
       <c r="F10" s="9" t="s">
         <v>28</v>
@@ -2204,7 +2204,7 @@
         <v>27</v>
       </c>
       <c r="E11" s="11">
-        <v>13</v>
+        <v>25</v>
       </c>
       <c r="F11" s="9" t="s">
         <v>28</v>
@@ -2227,7 +2227,7 @@
         <v>27</v>
       </c>
       <c r="E12" s="11">
-        <v>17</v>
+        <v>11</v>
       </c>
       <c r="F12" s="9" t="s">
         <v>28</v>
@@ -2250,7 +2250,7 @@
         <v>27</v>
       </c>
       <c r="E13" s="11">
-        <v>9</v>
+        <v>31</v>
       </c>
       <c r="F13" s="9" t="s">
         <v>28</v>
@@ -2273,7 +2273,7 @@
         <v>27</v>
       </c>
       <c r="E14" s="11">
-        <v>31</v>
+        <v>12</v>
       </c>
       <c r="F14" s="9" t="s">
         <v>28</v>
@@ -2296,7 +2296,7 @@
         <v>27</v>
       </c>
       <c r="E15" s="11">
-        <v>10</v>
+        <v>19</v>
       </c>
       <c r="F15" s="9" t="s">
         <v>28</v>
@@ -2319,7 +2319,7 @@
         <v>27</v>
       </c>
       <c r="E16" s="11">
-        <v>10</v>
+        <v>26</v>
       </c>
       <c r="F16" s="9" t="s">
         <v>28</v>
@@ -2342,7 +2342,7 @@
         <v>27</v>
       </c>
       <c r="E17" s="11">
-        <v>13</v>
+        <v>10</v>
       </c>
       <c r="F17" s="9" t="s">
         <v>28</v>
@@ -2365,7 +2365,7 @@
         <v>27</v>
       </c>
       <c r="E18" s="11">
-        <v>27</v>
+        <v>15</v>
       </c>
       <c r="F18" s="9" t="s">
         <v>28</v>
@@ -2388,7 +2388,7 @@
         <v>27</v>
       </c>
       <c r="E19" s="11">
-        <v>29</v>
+        <v>17</v>
       </c>
       <c r="F19" s="9" t="s">
         <v>28</v>
@@ -2411,7 +2411,7 @@
         <v>27</v>
       </c>
       <c r="E20" s="11">
-        <v>10</v>
+        <v>25</v>
       </c>
       <c r="F20" s="9" t="s">
         <v>28</v>
@@ -2434,7 +2434,7 @@
         <v>27</v>
       </c>
       <c r="E21" s="11">
-        <v>22</v>
+        <v>10</v>
       </c>
       <c r="F21" s="9" t="s">
         <v>28</v>
@@ -2457,7 +2457,7 @@
         <v>27</v>
       </c>
       <c r="E22" s="11">
-        <v>13</v>
+        <v>28</v>
       </c>
       <c r="F22" s="9" t="s">
         <v>28</v>
@@ -2480,7 +2480,7 @@
         <v>27</v>
       </c>
       <c r="E23" s="11">
-        <v>31</v>
+        <v>28</v>
       </c>
       <c r="F23" s="9" t="s">
         <v>28</v>
@@ -2503,7 +2503,7 @@
         <v>27</v>
       </c>
       <c r="E24" s="11">
-        <v>25</v>
+        <v>27</v>
       </c>
       <c r="F24" s="9" t="s">
         <v>28</v>
@@ -2526,7 +2526,7 @@
         <v>27</v>
       </c>
       <c r="E25" s="11">
-        <v>28</v>
+        <v>13</v>
       </c>
       <c r="F25" s="9" t="s">
         <v>28</v>
@@ -2549,7 +2549,7 @@
         <v>27</v>
       </c>
       <c r="E26" s="11">
-        <v>22</v>
+        <v>29</v>
       </c>
       <c r="F26" s="9" t="s">
         <v>28</v>
@@ -2572,7 +2572,7 @@
         <v>27</v>
       </c>
       <c r="E27" s="11">
-        <v>21</v>
+        <v>28</v>
       </c>
       <c r="F27" s="9" t="s">
         <v>28</v>
@@ -2595,7 +2595,7 @@
         <v>27</v>
       </c>
       <c r="E28" s="11">
-        <v>26</v>
+        <v>23</v>
       </c>
       <c r="F28" s="9" t="s">
         <v>28</v>
@@ -2618,7 +2618,7 @@
         <v>27</v>
       </c>
       <c r="E29" s="11">
-        <v>18</v>
+        <v>23</v>
       </c>
       <c r="F29" s="9" t="s">
         <v>28</v>
@@ -2641,7 +2641,7 @@
         <v>27</v>
       </c>
       <c r="E30" s="11">
-        <v>13</v>
+        <v>17</v>
       </c>
       <c r="F30" s="9" t="s">
         <v>28</v>
@@ -2664,7 +2664,7 @@
         <v>27</v>
       </c>
       <c r="E31" s="11">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="F31" s="9" t="s">
         <v>28</v>
@@ -2687,7 +2687,7 @@
         <v>27</v>
       </c>
       <c r="E32" s="11">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="F32" s="9" t="s">
         <v>28</v>
@@ -2710,7 +2710,7 @@
         <v>27</v>
       </c>
       <c r="E33" s="11">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="F33" s="9" t="s">
         <v>28</v>
@@ -2733,7 +2733,7 @@
         <v>27</v>
       </c>
       <c r="E34" s="11">
-        <v>13</v>
+        <v>23</v>
       </c>
       <c r="F34" s="9" t="s">
         <v>28</v>
@@ -2756,7 +2756,7 @@
         <v>27</v>
       </c>
       <c r="E35" s="11">
-        <v>8</v>
+        <v>21</v>
       </c>
       <c r="F35" s="9" t="s">
         <v>28</v>
@@ -2779,7 +2779,7 @@
         <v>27</v>
       </c>
       <c r="E36" s="11">
-        <v>22</v>
+        <v>27</v>
       </c>
       <c r="F36" s="9" t="s">
         <v>28</v>
@@ -2802,7 +2802,7 @@
         <v>27</v>
       </c>
       <c r="E37" s="11">
-        <v>16</v>
+        <v>20</v>
       </c>
       <c r="F37" s="9" t="s">
         <v>28</v>
@@ -2825,7 +2825,7 @@
         <v>27</v>
       </c>
       <c r="E38" s="11">
-        <v>28</v>
+        <v>15</v>
       </c>
       <c r="F38" s="9" t="s">
         <v>28</v>
@@ -2848,7 +2848,7 @@
         <v>27</v>
       </c>
       <c r="E39" s="11">
-        <v>18</v>
+        <v>16</v>
       </c>
       <c r="F39" s="9" t="s">
         <v>28</v>
@@ -2871,7 +2871,7 @@
         <v>27</v>
       </c>
       <c r="E40" s="11">
-        <v>31</v>
+        <v>29</v>
       </c>
       <c r="F40" s="9" t="s">
         <v>28</v>
@@ -2894,7 +2894,7 @@
         <v>27</v>
       </c>
       <c r="E41" s="11">
-        <v>30</v>
+        <v>9</v>
       </c>
       <c r="F41" s="9" t="s">
         <v>28</v>
@@ -2917,7 +2917,7 @@
         <v>27</v>
       </c>
       <c r="E42" s="11">
-        <v>26</v>
+        <v>14</v>
       </c>
       <c r="F42" s="9" t="s">
         <v>28</v>
@@ -2940,7 +2940,7 @@
         <v>27</v>
       </c>
       <c r="E43" s="11">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="F43" s="9" t="s">
         <v>28</v>
@@ -2963,7 +2963,7 @@
         <v>27</v>
       </c>
       <c r="E44" s="11">
-        <v>28</v>
+        <v>11</v>
       </c>
       <c r="F44" s="9" t="s">
         <v>28</v>
@@ -2986,7 +2986,7 @@
         <v>27</v>
       </c>
       <c r="E45" s="11">
-        <v>21</v>
+        <v>28</v>
       </c>
       <c r="F45" s="9" t="s">
         <v>28</v>
@@ -3009,7 +3009,7 @@
         <v>27</v>
       </c>
       <c r="E46" s="11">
-        <v>10</v>
+        <v>15</v>
       </c>
       <c r="F46" s="9" t="s">
         <v>28</v>
@@ -3032,7 +3032,7 @@
         <v>27</v>
       </c>
       <c r="E47" s="11">
-        <v>30</v>
+        <v>24</v>
       </c>
       <c r="F47" s="9" t="s">
         <v>28</v>
@@ -3055,7 +3055,7 @@
         <v>27</v>
       </c>
       <c r="E48" s="11">
-        <v>22</v>
+        <v>10</v>
       </c>
       <c r="F48" s="9" t="s">
         <v>28</v>
@@ -3101,7 +3101,7 @@
         <v>27</v>
       </c>
       <c r="E50" s="11">
-        <v>13</v>
+        <v>25</v>
       </c>
       <c r="F50" s="9" t="s">
         <v>28</v>
@@ -3124,7 +3124,7 @@
         <v>27</v>
       </c>
       <c r="E51" s="11">
-        <v>22</v>
+        <v>13</v>
       </c>
       <c r="F51" s="9" t="s">
         <v>28</v>
@@ -3147,7 +3147,7 @@
         <v>27</v>
       </c>
       <c r="E52" s="11">
-        <v>21</v>
+        <v>26</v>
       </c>
       <c r="F52" s="9" t="s">
         <v>28</v>
@@ -3170,7 +3170,7 @@
         <v>27</v>
       </c>
       <c r="E53" s="11">
-        <v>8</v>
+        <v>15</v>
       </c>
       <c r="F53" s="9" t="s">
         <v>28</v>
@@ -3193,7 +3193,7 @@
         <v>27</v>
       </c>
       <c r="E54" s="11">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="F54" s="9" t="s">
         <v>28</v>
@@ -3216,7 +3216,7 @@
         <v>27</v>
       </c>
       <c r="E55" s="11">
-        <v>23</v>
+        <v>18</v>
       </c>
       <c r="F55" s="9" t="s">
         <v>28</v>
@@ -3239,7 +3239,7 @@
         <v>27</v>
       </c>
       <c r="E56" s="11">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="F56" s="9" t="s">
         <v>28</v>
@@ -3262,7 +3262,7 @@
         <v>27</v>
       </c>
       <c r="E57" s="11">
-        <v>14</v>
+        <v>16</v>
       </c>
       <c r="F57" s="9" t="s">
         <v>28</v>
@@ -3285,7 +3285,7 @@
         <v>27</v>
       </c>
       <c r="E58" s="11">
-        <v>12</v>
+        <v>17</v>
       </c>
       <c r="F58" s="9" t="s">
         <v>28</v>
@@ -3308,7 +3308,7 @@
         <v>27</v>
       </c>
       <c r="E59" s="11">
-        <v>19</v>
+        <v>28</v>
       </c>
       <c r="F59" s="9" t="s">
         <v>28</v>
@@ -3331,7 +3331,7 @@
         <v>27</v>
       </c>
       <c r="E60" s="11">
-        <v>14</v>
+        <v>8</v>
       </c>
       <c r="F60" s="9" t="s">
         <v>28</v>
@@ -3354,7 +3354,7 @@
         <v>27</v>
       </c>
       <c r="E61" s="11">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="F61" s="9" t="s">
         <v>28</v>
@@ -3377,7 +3377,7 @@
         <v>27</v>
       </c>
       <c r="E62" s="11">
-        <v>9</v>
+        <v>23</v>
       </c>
       <c r="F62" s="9" t="s">
         <v>28</v>
@@ -3400,7 +3400,7 @@
         <v>27</v>
       </c>
       <c r="E63" s="11">
-        <v>30</v>
+        <v>25</v>
       </c>
       <c r="F63" s="9" t="s">
         <v>28</v>
@@ -3423,7 +3423,7 @@
         <v>27</v>
       </c>
       <c r="E64" s="11">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="F64" s="9" t="s">
         <v>28</v>
@@ -3446,7 +3446,7 @@
         <v>27</v>
       </c>
       <c r="E65" s="11">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="F65" s="9" t="s">
         <v>28</v>
@@ -3469,7 +3469,7 @@
         <v>27</v>
       </c>
       <c r="E66" s="11">
-        <v>23</v>
+        <v>31</v>
       </c>
       <c r="F66" s="9" t="s">
         <v>28</v>
@@ -3492,7 +3492,7 @@
         <v>27</v>
       </c>
       <c r="E67" s="11">
-        <v>14</v>
+        <v>25</v>
       </c>
       <c r="F67" s="9" t="s">
         <v>28</v>
@@ -3515,7 +3515,7 @@
         <v>27</v>
       </c>
       <c r="E68" s="11">
-        <v>31</v>
+        <v>29</v>
       </c>
       <c r="F68" s="9" t="s">
         <v>28</v>
@@ -3538,7 +3538,7 @@
         <v>27</v>
       </c>
       <c r="E69" s="11">
-        <v>29</v>
+        <v>9</v>
       </c>
       <c r="F69" s="9" t="s">
         <v>28</v>
@@ -3561,7 +3561,7 @@
         <v>27</v>
       </c>
       <c r="E70" s="11">
-        <v>31</v>
+        <v>21</v>
       </c>
       <c r="F70" s="9" t="s">
         <v>28</v>
@@ -3584,7 +3584,7 @@
         <v>27</v>
       </c>
       <c r="E71" s="11">
-        <v>9</v>
+        <v>23</v>
       </c>
       <c r="F71" s="9" t="s">
         <v>28</v>
@@ -3607,7 +3607,7 @@
         <v>27</v>
       </c>
       <c r="E72" s="11">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="F72" s="9" t="s">
         <v>28</v>
@@ -3630,7 +3630,7 @@
         <v>27</v>
       </c>
       <c r="E73" s="11">
-        <v>11</v>
+        <v>19</v>
       </c>
       <c r="F73" s="9" t="s">
         <v>28</v>
@@ -3653,7 +3653,7 @@
         <v>27</v>
       </c>
       <c r="E74" s="11">
-        <v>14</v>
+        <v>30</v>
       </c>
       <c r="F74" s="9" t="s">
         <v>28</v>
@@ -3676,7 +3676,7 @@
         <v>27</v>
       </c>
       <c r="E75" s="11">
-        <v>11</v>
+        <v>29</v>
       </c>
       <c r="F75" s="9" t="s">
         <v>28</v>
@@ -3699,7 +3699,7 @@
         <v>27</v>
       </c>
       <c r="E76" s="11">
-        <v>20</v>
+        <v>31</v>
       </c>
       <c r="F76" s="9" t="s">
         <v>28</v>
@@ -3722,7 +3722,7 @@
         <v>27</v>
       </c>
       <c r="E77" s="11">
-        <v>15</v>
+        <v>29</v>
       </c>
       <c r="F77" s="9" t="s">
         <v>28</v>
@@ -3745,7 +3745,7 @@
         <v>27</v>
       </c>
       <c r="E78" s="11">
-        <v>12</v>
+        <v>15</v>
       </c>
       <c r="F78" s="9" t="s">
         <v>28</v>
@@ -3768,7 +3768,7 @@
         <v>27</v>
       </c>
       <c r="E79" s="11">
-        <v>12</v>
+        <v>31</v>
       </c>
       <c r="F79" s="9" t="s">
         <v>28</v>
@@ -3791,7 +3791,7 @@
         <v>27</v>
       </c>
       <c r="E80" s="11">
-        <v>14</v>
+        <v>18</v>
       </c>
       <c r="F80" s="9" t="s">
         <v>28</v>
@@ -3814,7 +3814,7 @@
         <v>27</v>
       </c>
       <c r="E81" s="11">
-        <v>11</v>
+        <v>16</v>
       </c>
       <c r="F81" s="9" t="s">
         <v>28</v>
@@ -3837,7 +3837,7 @@
         <v>27</v>
       </c>
       <c r="E82" s="11">
-        <v>25</v>
+        <v>20</v>
       </c>
       <c r="F82" s="9" t="s">
         <v>28</v>
@@ -3860,7 +3860,7 @@
         <v>27</v>
       </c>
       <c r="E83" s="11">
-        <v>13</v>
+        <v>26</v>
       </c>
       <c r="F83" s="9" t="s">
         <v>28</v>
@@ -3883,7 +3883,7 @@
         <v>27</v>
       </c>
       <c r="E84" s="11">
-        <v>29</v>
+        <v>21</v>
       </c>
       <c r="F84" s="9" t="s">
         <v>28</v>
@@ -3906,7 +3906,7 @@
         <v>27</v>
       </c>
       <c r="E85" s="11">
-        <v>30</v>
+        <v>18</v>
       </c>
       <c r="F85" s="9" t="s">
         <v>28</v>
@@ -3929,7 +3929,7 @@
         <v>27</v>
       </c>
       <c r="E86" s="11">
-        <v>11</v>
+        <v>28</v>
       </c>
       <c r="F86" s="9" t="s">
         <v>28</v>
@@ -3952,7 +3952,7 @@
         <v>27</v>
       </c>
       <c r="E87" s="11">
-        <v>19</v>
+        <v>27</v>
       </c>
       <c r="F87" s="9" t="s">
         <v>28</v>
@@ -3975,7 +3975,7 @@
         <v>27</v>
       </c>
       <c r="E88" s="11">
-        <v>23</v>
+        <v>18</v>
       </c>
       <c r="F88" s="9" t="s">
         <v>28</v>
@@ -3998,7 +3998,7 @@
         <v>27</v>
       </c>
       <c r="E89" s="11">
-        <v>20</v>
+        <v>10</v>
       </c>
       <c r="F89" s="9" t="s">
         <v>28</v>
@@ -4021,7 +4021,7 @@
         <v>27</v>
       </c>
       <c r="E90" s="11">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="F90" s="9" t="s">
         <v>28</v>
@@ -4044,7 +4044,7 @@
         <v>27</v>
       </c>
       <c r="E91" s="11">
-        <v>28</v>
+        <v>19</v>
       </c>
       <c r="F91" s="9" t="s">
         <v>28</v>
@@ -4067,7 +4067,7 @@
         <v>27</v>
       </c>
       <c r="E92" s="11">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="F92" s="9" t="s">
         <v>28</v>
@@ -4090,7 +4090,7 @@
         <v>27</v>
       </c>
       <c r="E93" s="11">
-        <v>15</v>
+        <v>27</v>
       </c>
       <c r="F93" s="9" t="s">
         <v>28</v>
@@ -4113,7 +4113,7 @@
         <v>27</v>
       </c>
       <c r="E94" s="11">
-        <v>12</v>
+        <v>8</v>
       </c>
       <c r="F94" s="9" t="s">
         <v>28</v>
@@ -4136,7 +4136,7 @@
         <v>27</v>
       </c>
       <c r="E95" s="11">
-        <v>20</v>
+        <v>27</v>
       </c>
       <c r="F95" s="9" t="s">
         <v>28</v>
@@ -4159,7 +4159,7 @@
         <v>27</v>
       </c>
       <c r="E96" s="11">
-        <v>29</v>
+        <v>18</v>
       </c>
       <c r="F96" s="9" t="s">
         <v>28</v>
@@ -4182,7 +4182,7 @@
         <v>27</v>
       </c>
       <c r="E97" s="11">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="F97" s="9" t="s">
         <v>28</v>
@@ -4205,7 +4205,7 @@
         <v>27</v>
       </c>
       <c r="E98" s="11">
-        <v>19</v>
+        <v>21</v>
       </c>
       <c r="F98" s="9" t="s">
         <v>28</v>
@@ -4228,7 +4228,7 @@
         <v>27</v>
       </c>
       <c r="E99" s="11">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="F99" s="9" t="s">
         <v>28</v>
@@ -4251,7 +4251,7 @@
         <v>27</v>
       </c>
       <c r="E100" s="11">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="F100" s="9" t="s">
         <v>28</v>
@@ -4274,7 +4274,7 @@
         <v>27</v>
       </c>
       <c r="E101" s="11">
-        <v>25</v>
+        <v>30</v>
       </c>
       <c r="F101" s="9" t="s">
         <v>28</v>
@@ -4297,7 +4297,7 @@
         <v>27</v>
       </c>
       <c r="E102" s="11">
-        <v>24</v>
+        <v>27</v>
       </c>
       <c r="F102" s="9" t="s">
         <v>28</v>
@@ -4320,7 +4320,7 @@
         <v>27</v>
       </c>
       <c r="E103" s="11">
-        <v>11</v>
+        <v>8</v>
       </c>
       <c r="F103" s="9" t="s">
         <v>28</v>
@@ -4343,7 +4343,7 @@
         <v>27</v>
       </c>
       <c r="E104" s="11">
-        <v>8</v>
+        <v>12</v>
       </c>
       <c r="F104" s="9" t="s">
         <v>28</v>
@@ -4366,7 +4366,7 @@
         <v>27</v>
       </c>
       <c r="E105" s="11">
-        <v>29</v>
+        <v>8</v>
       </c>
       <c r="F105" s="9" t="s">
         <v>28</v>
@@ -4389,7 +4389,7 @@
         <v>27</v>
       </c>
       <c r="E106" s="11">
-        <v>16</v>
+        <v>22</v>
       </c>
       <c r="F106" s="9" t="s">
         <v>28</v>
@@ -4412,7 +4412,7 @@
         <v>27</v>
       </c>
       <c r="E107" s="11">
-        <v>22</v>
+        <v>30</v>
       </c>
       <c r="F107" s="9" t="s">
         <v>28</v>
@@ -4435,7 +4435,7 @@
         <v>27</v>
       </c>
       <c r="E108" s="11">
-        <v>29</v>
+        <v>22</v>
       </c>
       <c r="F108" s="9" t="s">
         <v>28</v>
@@ -4458,7 +4458,7 @@
         <v>27</v>
       </c>
       <c r="E109" s="11">
-        <v>29</v>
+        <v>16</v>
       </c>
       <c r="F109" s="9" t="s">
         <v>28</v>
@@ -4481,7 +4481,7 @@
         <v>27</v>
       </c>
       <c r="E110" s="11">
-        <v>12</v>
+        <v>24</v>
       </c>
       <c r="F110" s="9" t="s">
         <v>28</v>
@@ -4504,7 +4504,7 @@
         <v>27</v>
       </c>
       <c r="E111" s="11">
-        <v>14</v>
+        <v>18</v>
       </c>
       <c r="F111" s="9" t="s">
         <v>28</v>
@@ -4527,7 +4527,7 @@
         <v>27</v>
       </c>
       <c r="E112" s="11">
-        <v>31</v>
+        <v>17</v>
       </c>
       <c r="F112" s="9" t="s">
         <v>28</v>
@@ -4550,7 +4550,7 @@
         <v>27</v>
       </c>
       <c r="E113" s="11">
-        <v>16</v>
+        <v>26</v>
       </c>
       <c r="F113" s="9" t="s">
         <v>28</v>
@@ -4573,7 +4573,7 @@
         <v>27</v>
       </c>
       <c r="E114" s="11">
-        <v>26</v>
+        <v>9</v>
       </c>
       <c r="F114" s="9" t="s">
         <v>28</v>
@@ -4596,7 +4596,7 @@
         <v>27</v>
       </c>
       <c r="E115" s="11">
-        <v>16</v>
+        <v>23</v>
       </c>
       <c r="F115" s="9" t="s">
         <v>28</v>
@@ -4619,7 +4619,7 @@
         <v>27</v>
       </c>
       <c r="E116" s="11">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="F116" s="9" t="s">
         <v>28</v>
@@ -4642,7 +4642,7 @@
         <v>27</v>
       </c>
       <c r="E117" s="11">
-        <v>18</v>
+        <v>11</v>
       </c>
       <c r="F117" s="9" t="s">
         <v>28</v>
@@ -4665,7 +4665,7 @@
         <v>27</v>
       </c>
       <c r="E118" s="11">
-        <v>13</v>
+        <v>29</v>
       </c>
       <c r="F118" s="9" t="s">
         <v>28</v>
@@ -4688,7 +4688,7 @@
         <v>27</v>
       </c>
       <c r="E119" s="11">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="F119" s="9" t="s">
         <v>28</v>
@@ -4711,7 +4711,7 @@
         <v>27</v>
       </c>
       <c r="E120" s="11">
-        <v>19</v>
+        <v>12</v>
       </c>
       <c r="F120" s="9" t="s">
         <v>28</v>
@@ -4734,7 +4734,7 @@
         <v>27</v>
       </c>
       <c r="E121" s="11">
-        <v>17</v>
+        <v>8</v>
       </c>
       <c r="F121" s="9" t="s">
         <v>28</v>
@@ -4757,7 +4757,7 @@
         <v>27</v>
       </c>
       <c r="E122" s="11">
-        <v>26</v>
+        <v>24</v>
       </c>
       <c r="F122" s="9" t="s">
         <v>28</v>
@@ -4803,7 +4803,7 @@
         <v>27</v>
       </c>
       <c r="E124" s="11">
-        <v>27</v>
+        <v>19</v>
       </c>
       <c r="F124" s="9" t="s">
         <v>28</v>
@@ -4826,7 +4826,7 @@
         <v>27</v>
       </c>
       <c r="E125" s="11">
-        <v>11</v>
+        <v>26</v>
       </c>
       <c r="F125" s="9" t="s">
         <v>28</v>
@@ -4849,7 +4849,7 @@
         <v>27</v>
       </c>
       <c r="E126" s="11">
-        <v>20</v>
+        <v>25</v>
       </c>
       <c r="F126" s="9" t="s">
         <v>28</v>
@@ -4872,7 +4872,7 @@
         <v>27</v>
       </c>
       <c r="E127" s="11">
-        <v>26</v>
+        <v>21</v>
       </c>
       <c r="F127" s="9" t="s">
         <v>28</v>
@@ -4895,7 +4895,7 @@
         <v>27</v>
       </c>
       <c r="E128" s="11">
-        <v>16</v>
+        <v>22</v>
       </c>
       <c r="F128" s="9" t="s">
         <v>28</v>
@@ -4918,7 +4918,7 @@
         <v>27</v>
       </c>
       <c r="E129" s="11">
-        <v>30</v>
+        <v>25</v>
       </c>
       <c r="F129" s="9" t="s">
         <v>28</v>
@@ -4941,7 +4941,7 @@
         <v>27</v>
       </c>
       <c r="E130" s="11">
-        <v>27</v>
+        <v>13</v>
       </c>
       <c r="F130" s="9" t="s">
         <v>28</v>
@@ -4964,7 +4964,7 @@
         <v>27</v>
       </c>
       <c r="E131" s="11">
-        <v>17</v>
+        <v>14</v>
       </c>
       <c r="F131" s="9" t="s">
         <v>28</v>
@@ -4987,7 +4987,7 @@
         <v>27</v>
       </c>
       <c r="E132" s="11">
-        <v>8</v>
+        <v>20</v>
       </c>
       <c r="F132" s="9" t="s">
         <v>28</v>
@@ -5010,7 +5010,7 @@
         <v>27</v>
       </c>
       <c r="E133" s="11">
-        <v>20</v>
+        <v>22</v>
       </c>
       <c r="F133" s="9" t="s">
         <v>28</v>
@@ -5033,7 +5033,7 @@
         <v>27</v>
       </c>
       <c r="E134" s="11">
-        <v>14</v>
+        <v>11</v>
       </c>
       <c r="F134" s="9" t="s">
         <v>28</v>
@@ -5056,7 +5056,7 @@
         <v>27</v>
       </c>
       <c r="E135" s="11">
-        <v>30</v>
+        <v>18</v>
       </c>
       <c r="F135" s="9" t="s">
         <v>28</v>
@@ -5079,7 +5079,7 @@
         <v>27</v>
       </c>
       <c r="E136" s="11">
-        <v>24</v>
+        <v>18</v>
       </c>
       <c r="F136" s="9" t="s">
         <v>28</v>
@@ -5102,7 +5102,7 @@
         <v>27</v>
       </c>
       <c r="E137" s="11">
-        <v>8</v>
+        <v>18</v>
       </c>
       <c r="F137" s="9" t="s">
         <v>28</v>
@@ -5125,7 +5125,7 @@
         <v>27</v>
       </c>
       <c r="E138" s="11">
-        <v>11</v>
+        <v>16</v>
       </c>
       <c r="F138" s="9" t="s">
         <v>28</v>
@@ -5148,7 +5148,7 @@
         <v>27</v>
       </c>
       <c r="E139" s="11">
-        <v>28</v>
+        <v>15</v>
       </c>
       <c r="F139" s="9" t="s">
         <v>28</v>
@@ -5171,7 +5171,7 @@
         <v>27</v>
       </c>
       <c r="E140" s="11">
-        <v>16</v>
+        <v>28</v>
       </c>
       <c r="F140" s="9" t="s">
         <v>28</v>
@@ -5194,7 +5194,7 @@
         <v>27</v>
       </c>
       <c r="E141" s="11">
-        <v>17</v>
+        <v>14</v>
       </c>
       <c r="F141" s="9" t="s">
         <v>28</v>
@@ -5217,7 +5217,7 @@
         <v>27</v>
       </c>
       <c r="E142" s="11">
-        <v>17</v>
+        <v>27</v>
       </c>
       <c r="F142" s="9" t="s">
         <v>28</v>
@@ -5240,7 +5240,7 @@
         <v>27</v>
       </c>
       <c r="E143" s="11">
-        <v>11</v>
+        <v>24</v>
       </c>
       <c r="F143" s="9" t="s">
         <v>28</v>
@@ -5263,7 +5263,7 @@
         <v>27</v>
       </c>
       <c r="E144" s="11">
-        <v>29</v>
+        <v>26</v>
       </c>
       <c r="F144" s="9" t="s">
         <v>28</v>
@@ -5286,7 +5286,7 @@
         <v>27</v>
       </c>
       <c r="E145" s="11">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="F145" s="9" t="s">
         <v>28</v>
@@ -5309,7 +5309,7 @@
         <v>27</v>
       </c>
       <c r="E146" s="11">
-        <v>28</v>
+        <v>12</v>
       </c>
       <c r="F146" s="9" t="s">
         <v>28</v>
@@ -5332,7 +5332,7 @@
         <v>27</v>
       </c>
       <c r="E147" s="11">
-        <v>31</v>
+        <v>23</v>
       </c>
       <c r="F147" s="9" t="s">
         <v>28</v>
@@ -5355,7 +5355,7 @@
         <v>27</v>
       </c>
       <c r="E148" s="11">
-        <v>22</v>
+        <v>16</v>
       </c>
       <c r="F148" s="9" t="s">
         <v>28</v>
@@ -5378,7 +5378,7 @@
         <v>27</v>
       </c>
       <c r="E149" s="11">
-        <v>12</v>
+        <v>30</v>
       </c>
       <c r="F149" s="9" t="s">
         <v>28</v>
@@ -5447,7 +5447,7 @@
         <v>27</v>
       </c>
       <c r="E152" s="11">
-        <v>30</v>
+        <v>16</v>
       </c>
       <c r="F152" s="9" t="s">
         <v>28</v>
@@ -5470,7 +5470,7 @@
         <v>27</v>
       </c>
       <c r="E153" s="11">
-        <v>8</v>
+        <v>29</v>
       </c>
       <c r="F153" s="9" t="s">
         <v>28</v>
@@ -5493,7 +5493,7 @@
         <v>27</v>
       </c>
       <c r="E154" s="11">
-        <v>21</v>
+        <v>26</v>
       </c>
       <c r="F154" s="9" t="s">
         <v>28</v>
@@ -5516,7 +5516,7 @@
         <v>27</v>
       </c>
       <c r="E155" s="11">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="F155" s="9" t="s">
         <v>28</v>
@@ -5539,7 +5539,7 @@
         <v>27</v>
       </c>
       <c r="E156" s="11">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="F156" s="9" t="s">
         <v>28</v>
@@ -5562,7 +5562,7 @@
         <v>27</v>
       </c>
       <c r="E157" s="11">
-        <v>12</v>
+        <v>17</v>
       </c>
       <c r="F157" s="9" t="s">
         <v>28</v>
@@ -5608,7 +5608,7 @@
         <v>27</v>
       </c>
       <c r="E159" s="11">
-        <v>16</v>
+        <v>21</v>
       </c>
       <c r="F159" s="9" t="s">
         <v>28</v>
@@ -5631,7 +5631,7 @@
         <v>27</v>
       </c>
       <c r="E160" s="11">
-        <v>27</v>
+        <v>8</v>
       </c>
       <c r="F160" s="9" t="s">
         <v>28</v>
@@ -5654,7 +5654,7 @@
         <v>27</v>
       </c>
       <c r="E161" s="11">
-        <v>8</v>
+        <v>21</v>
       </c>
       <c r="F161" s="9" t="s">
         <v>28</v>
@@ -5677,7 +5677,7 @@
         <v>27</v>
       </c>
       <c r="E162" s="11">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="F162" s="9" t="s">
         <v>28</v>
@@ -5700,7 +5700,7 @@
         <v>27</v>
       </c>
       <c r="E163" s="11">
-        <v>8</v>
+        <v>23</v>
       </c>
       <c r="F163" s="9" t="s">
         <v>28</v>
@@ -5723,7 +5723,7 @@
         <v>27</v>
       </c>
       <c r="E164" s="11">
-        <v>12</v>
+        <v>30</v>
       </c>
       <c r="F164" s="9" t="s">
         <v>28</v>
@@ -5746,7 +5746,7 @@
         <v>27</v>
       </c>
       <c r="E165" s="11">
-        <v>25</v>
+        <v>28</v>
       </c>
       <c r="F165" s="9" t="s">
         <v>28</v>
@@ -5769,7 +5769,7 @@
         <v>27</v>
       </c>
       <c r="E166" s="11">
-        <v>31</v>
+        <v>17</v>
       </c>
       <c r="F166" s="9" t="s">
         <v>28</v>
@@ -5792,7 +5792,7 @@
         <v>27</v>
       </c>
       <c r="E167" s="11">
-        <v>13</v>
+        <v>24</v>
       </c>
       <c r="F167" s="9" t="s">
         <v>28</v>
@@ -5838,7 +5838,7 @@
         <v>27</v>
       </c>
       <c r="E169" s="11">
-        <v>14</v>
+        <v>28</v>
       </c>
       <c r="F169" s="9" t="s">
         <v>28</v>
@@ -5861,7 +5861,7 @@
         <v>27</v>
       </c>
       <c r="E170" s="11">
-        <v>18</v>
+        <v>12</v>
       </c>
       <c r="F170" s="9" t="s">
         <v>28</v>
@@ -5884,7 +5884,7 @@
         <v>27</v>
       </c>
       <c r="E171" s="11">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="F171" s="9" t="s">
         <v>28</v>
@@ -5907,7 +5907,7 @@
         <v>27</v>
       </c>
       <c r="E172" s="11">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="F172" s="9" t="s">
         <v>28</v>
@@ -5930,7 +5930,7 @@
         <v>27</v>
       </c>
       <c r="E173" s="11">
-        <v>20</v>
+        <v>15</v>
       </c>
       <c r="F173" s="9" t="s">
         <v>28</v>
@@ -5953,7 +5953,7 @@
         <v>27</v>
       </c>
       <c r="E174" s="11">
-        <v>25</v>
+        <v>19</v>
       </c>
       <c r="F174" s="9" t="s">
         <v>28</v>
@@ -5976,7 +5976,7 @@
         <v>27</v>
       </c>
       <c r="E175" s="11">
-        <v>18</v>
+        <v>31</v>
       </c>
       <c r="F175" s="9" t="s">
         <v>28</v>
@@ -5999,7 +5999,7 @@
         <v>27</v>
       </c>
       <c r="E176" s="11">
-        <v>10</v>
+        <v>25</v>
       </c>
       <c r="F176" s="9" t="s">
         <v>28</v>
@@ -6022,7 +6022,7 @@
         <v>27</v>
       </c>
       <c r="E177" s="11">
-        <v>25</v>
+        <v>21</v>
       </c>
       <c r="F177" s="9" t="s">
         <v>28</v>
@@ -6068,7 +6068,7 @@
         <v>27</v>
       </c>
       <c r="E179" s="11">
-        <v>31</v>
+        <v>20</v>
       </c>
       <c r="F179" s="9" t="s">
         <v>28</v>
@@ -6091,7 +6091,7 @@
         <v>27</v>
       </c>
       <c r="E180" s="11">
-        <v>29</v>
+        <v>10</v>
       </c>
       <c r="F180" s="9" t="s">
         <v>28</v>
@@ -6114,7 +6114,7 @@
         <v>27</v>
       </c>
       <c r="E181" s="11">
-        <v>17</v>
+        <v>12</v>
       </c>
       <c r="F181" s="9" t="s">
         <v>28</v>
@@ -6137,7 +6137,7 @@
         <v>27</v>
       </c>
       <c r="E182" s="11">
-        <v>9</v>
+        <v>23</v>
       </c>
       <c r="F182" s="9" t="s">
         <v>28</v>
@@ -6160,7 +6160,7 @@
         <v>27</v>
       </c>
       <c r="E183" s="11">
-        <v>31</v>
+        <v>9</v>
       </c>
       <c r="F183" s="9" t="s">
         <v>28</v>
@@ -6183,7 +6183,7 @@
         <v>27</v>
       </c>
       <c r="E184" s="11">
-        <v>11</v>
+        <v>24</v>
       </c>
       <c r="F184" s="9" t="s">
         <v>28</v>
@@ -6206,7 +6206,7 @@
         <v>27</v>
       </c>
       <c r="E185" s="11">
-        <v>29</v>
+        <v>19</v>
       </c>
       <c r="F185" s="9" t="s">
         <v>28</v>
@@ -6229,7 +6229,7 @@
         <v>27</v>
       </c>
       <c r="E186" s="11">
-        <v>14</v>
+        <v>11</v>
       </c>
       <c r="F186" s="9" t="s">
         <v>28</v>
@@ -6252,7 +6252,7 @@
         <v>27</v>
       </c>
       <c r="E187" s="11">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="F187" s="9" t="s">
         <v>28</v>
@@ -6275,7 +6275,7 @@
         <v>27</v>
       </c>
       <c r="E188" s="11">
-        <v>19</v>
+        <v>22</v>
       </c>
       <c r="F188" s="9" t="s">
         <v>28</v>
@@ -6298,7 +6298,7 @@
         <v>27</v>
       </c>
       <c r="E189" s="11">
-        <v>10</v>
+        <v>29</v>
       </c>
       <c r="F189" s="9" t="s">
         <v>28</v>
@@ -6321,7 +6321,7 @@
         <v>27</v>
       </c>
       <c r="E190" s="11">
-        <v>25</v>
+        <v>12</v>
       </c>
       <c r="F190" s="9" t="s">
         <v>28</v>
@@ -6344,7 +6344,7 @@
         <v>27</v>
       </c>
       <c r="E191" s="11">
-        <v>10</v>
+        <v>23</v>
       </c>
       <c r="F191" s="9" t="s">
         <v>28</v>
@@ -6367,7 +6367,7 @@
         <v>27</v>
       </c>
       <c r="E192" s="11">
-        <v>31</v>
+        <v>26</v>
       </c>
       <c r="F192" s="9" t="s">
         <v>28</v>
@@ -6390,7 +6390,7 @@
         <v>27</v>
       </c>
       <c r="E193" s="11">
-        <v>15</v>
+        <v>21</v>
       </c>
       <c r="F193" s="9" t="s">
         <v>28</v>
@@ -6436,7 +6436,7 @@
         <v>27</v>
       </c>
       <c r="E195" s="11">
-        <v>28</v>
+        <v>13</v>
       </c>
       <c r="F195" s="9" t="s">
         <v>28</v>
@@ -6459,7 +6459,7 @@
         <v>27</v>
       </c>
       <c r="E196" s="11">
-        <v>25</v>
+        <v>10</v>
       </c>
       <c r="F196" s="9" t="s">
         <v>28</v>
@@ -6482,7 +6482,7 @@
         <v>27</v>
       </c>
       <c r="E197" s="11">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="F197" s="9" t="s">
         <v>28</v>
@@ -6505,7 +6505,7 @@
         <v>27</v>
       </c>
       <c r="E198" s="11">
-        <v>16</v>
+        <v>24</v>
       </c>
       <c r="F198" s="9" t="s">
         <v>28</v>
@@ -6528,7 +6528,7 @@
         <v>27</v>
       </c>
       <c r="E199" s="11">
-        <v>13</v>
+        <v>22</v>
       </c>
       <c r="F199" s="9" t="s">
         <v>28</v>
@@ -6551,7 +6551,7 @@
         <v>27</v>
       </c>
       <c r="E200" s="11">
-        <v>14</v>
+        <v>29</v>
       </c>
       <c r="F200" s="9" t="s">
         <v>28</v>
@@ -6574,7 +6574,7 @@
         <v>27</v>
       </c>
       <c r="E201" s="11">
-        <v>30</v>
+        <v>17</v>
       </c>
       <c r="F201" s="9" t="s">
         <v>28</v>
@@ -6597,7 +6597,7 @@
         <v>27</v>
       </c>
       <c r="E202" s="11">
-        <v>18</v>
+        <v>14</v>
       </c>
       <c r="F202" s="9" t="s">
         <v>28</v>
@@ -6620,7 +6620,7 @@
         <v>27</v>
       </c>
       <c r="E203" s="11">
-        <v>12</v>
+        <v>31</v>
       </c>
       <c r="F203" s="9" t="s">
         <v>28</v>
@@ -6643,7 +6643,7 @@
         <v>27</v>
       </c>
       <c r="E204" s="11">
-        <v>13</v>
+        <v>30</v>
       </c>
       <c r="F204" s="9" t="s">
         <v>28</v>
@@ -6666,7 +6666,7 @@
         <v>27</v>
       </c>
       <c r="E205" s="11">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="F205" s="9" t="s">
         <v>28</v>
@@ -6689,7 +6689,7 @@
         <v>27</v>
       </c>
       <c r="E206" s="11">
-        <v>16</v>
+        <v>14</v>
       </c>
       <c r="F206" s="9" t="s">
         <v>28</v>
@@ -6712,7 +6712,7 @@
         <v>27</v>
       </c>
       <c r="E207" s="11">
-        <v>14</v>
+        <v>19</v>
       </c>
       <c r="F207" s="9" t="s">
         <v>28</v>
@@ -6735,7 +6735,7 @@
         <v>27</v>
       </c>
       <c r="E208" s="11">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="F208" s="9" t="s">
         <v>28</v>
@@ -6758,7 +6758,7 @@
         <v>27</v>
       </c>
       <c r="E209" s="11">
-        <v>19</v>
+        <v>9</v>
       </c>
       <c r="F209" s="9" t="s">
         <v>28</v>
@@ -6781,7 +6781,7 @@
         <v>27</v>
       </c>
       <c r="E210" s="11">
-        <v>25</v>
+        <v>18</v>
       </c>
       <c r="F210" s="9" t="s">
         <v>28</v>
@@ -6804,7 +6804,7 @@
         <v>27</v>
       </c>
       <c r="E211" s="11">
-        <v>24</v>
+        <v>11</v>
       </c>
       <c r="F211" s="9" t="s">
         <v>28</v>
@@ -6827,7 +6827,7 @@
         <v>27</v>
       </c>
       <c r="E212" s="11">
-        <v>20</v>
+        <v>24</v>
       </c>
       <c r="F212" s="9" t="s">
         <v>28</v>
@@ -6850,7 +6850,7 @@
         <v>27</v>
       </c>
       <c r="E213" s="11">
-        <v>29</v>
+        <v>17</v>
       </c>
       <c r="F213" s="9" t="s">
         <v>28</v>
@@ -6873,7 +6873,7 @@
         <v>27</v>
       </c>
       <c r="E214" s="11">
-        <v>27</v>
+        <v>17</v>
       </c>
       <c r="F214" s="9" t="s">
         <v>28</v>
@@ -6896,7 +6896,7 @@
         <v>27</v>
       </c>
       <c r="E215" s="11">
-        <v>22</v>
+        <v>20</v>
       </c>
       <c r="F215" s="9" t="s">
         <v>28</v>
@@ -6919,7 +6919,7 @@
         <v>27</v>
       </c>
       <c r="E216" s="11">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="F216" s="9" t="s">
         <v>28</v>
@@ -6942,7 +6942,7 @@
         <v>27</v>
       </c>
       <c r="E217" s="11">
-        <v>13</v>
+        <v>29</v>
       </c>
       <c r="F217" s="9" t="s">
         <v>28</v>
@@ -6965,7 +6965,7 @@
         <v>27</v>
       </c>
       <c r="E218" s="11">
-        <v>23</v>
+        <v>25</v>
       </c>
       <c r="F218" s="9" t="s">
         <v>28</v>
@@ -7011,7 +7011,7 @@
         <v>27</v>
       </c>
       <c r="E220" s="11">
-        <v>22</v>
+        <v>11</v>
       </c>
       <c r="F220" s="9" t="s">
         <v>28</v>
@@ -7034,7 +7034,7 @@
         <v>27</v>
       </c>
       <c r="E221" s="11">
-        <v>26</v>
+        <v>28</v>
       </c>
       <c r="F221" s="9" t="s">
         <v>28</v>
@@ -7057,7 +7057,7 @@
         <v>27</v>
       </c>
       <c r="E222" s="11">
-        <v>19</v>
+        <v>27</v>
       </c>
       <c r="F222" s="9" t="s">
         <v>28</v>
@@ -7080,7 +7080,7 @@
         <v>27</v>
       </c>
       <c r="E223" s="11">
-        <v>17</v>
+        <v>31</v>
       </c>
       <c r="F223" s="9" t="s">
         <v>28</v>
@@ -7103,7 +7103,7 @@
         <v>27</v>
       </c>
       <c r="E224" s="11">
-        <v>23</v>
+        <v>13</v>
       </c>
       <c r="F224" s="9" t="s">
         <v>28</v>
@@ -7126,7 +7126,7 @@
         <v>27</v>
       </c>
       <c r="E225" s="11">
-        <v>21</v>
+        <v>9</v>
       </c>
       <c r="F225" s="9" t="s">
         <v>28</v>
@@ -7149,7 +7149,7 @@
         <v>27</v>
       </c>
       <c r="E226" s="11">
-        <v>11</v>
+        <v>14</v>
       </c>
       <c r="F226" s="9" t="s">
         <v>28</v>
@@ -7172,7 +7172,7 @@
         <v>27</v>
       </c>
       <c r="E227" s="11">
-        <v>26</v>
+        <v>16</v>
       </c>
       <c r="F227" s="9" t="s">
         <v>28</v>
@@ -7195,7 +7195,7 @@
         <v>27</v>
       </c>
       <c r="E228" s="11">
-        <v>13</v>
+        <v>8</v>
       </c>
       <c r="F228" s="9" t="s">
         <v>28</v>
@@ -7218,7 +7218,7 @@
         <v>27</v>
       </c>
       <c r="E229" s="11">
-        <v>23</v>
+        <v>31</v>
       </c>
       <c r="F229" s="9" t="s">
         <v>28</v>
@@ -7264,7 +7264,7 @@
         <v>27</v>
       </c>
       <c r="E231" s="11">
-        <v>12</v>
+        <v>28</v>
       </c>
       <c r="F231" s="9" t="s">
         <v>28</v>
@@ -7287,7 +7287,7 @@
         <v>27</v>
       </c>
       <c r="E232" s="11">
-        <v>19</v>
+        <v>12</v>
       </c>
       <c r="F232" s="9" t="s">
         <v>28</v>
@@ -7310,7 +7310,7 @@
         <v>27</v>
       </c>
       <c r="E233" s="11">
-        <v>29</v>
+        <v>13</v>
       </c>
       <c r="F233" s="9" t="s">
         <v>28</v>
@@ -7333,7 +7333,7 @@
         <v>27</v>
       </c>
       <c r="E234" s="11">
-        <v>19</v>
+        <v>25</v>
       </c>
       <c r="F234" s="9" t="s">
         <v>28</v>
@@ -7356,7 +7356,7 @@
         <v>27</v>
       </c>
       <c r="E235" s="11">
-        <v>20</v>
+        <v>13</v>
       </c>
       <c r="F235" s="9" t="s">
         <v>28</v>
@@ -7379,7 +7379,7 @@
         <v>27</v>
       </c>
       <c r="E236" s="11">
-        <v>17</v>
+        <v>28</v>
       </c>
       <c r="F236" s="9" t="s">
         <v>28</v>
@@ -7402,7 +7402,7 @@
         <v>27</v>
       </c>
       <c r="E237" s="11">
-        <v>19</v>
+        <v>15</v>
       </c>
       <c r="F237" s="9" t="s">
         <v>28</v>
@@ -7425,7 +7425,7 @@
         <v>27</v>
       </c>
       <c r="E238" s="11">
-        <v>8</v>
+        <v>29</v>
       </c>
       <c r="F238" s="9" t="s">
         <v>28</v>
@@ -7448,7 +7448,7 @@
         <v>27</v>
       </c>
       <c r="E239" s="11">
-        <v>10</v>
+        <v>30</v>
       </c>
       <c r="F239" s="9" t="s">
         <v>28</v>
@@ -7471,7 +7471,7 @@
         <v>27</v>
       </c>
       <c r="E240" s="11">
-        <v>20</v>
+        <v>13</v>
       </c>
       <c r="F240" s="9" t="s">
         <v>28</v>
@@ -7494,7 +7494,7 @@
         <v>27</v>
       </c>
       <c r="E241" s="11">
-        <v>25</v>
+        <v>28</v>
       </c>
       <c r="F241" s="9" t="s">
         <v>28</v>
@@ -7517,7 +7517,7 @@
         <v>27</v>
       </c>
       <c r="E242" s="11">
-        <v>8</v>
+        <v>11</v>
       </c>
       <c r="F242" s="9" t="s">
         <v>28</v>
@@ -7540,7 +7540,7 @@
         <v>27</v>
       </c>
       <c r="E243" s="11">
-        <v>21</v>
+        <v>15</v>
       </c>
       <c r="F243" s="9" t="s">
         <v>28</v>
@@ -7563,7 +7563,7 @@
         <v>27</v>
       </c>
       <c r="E244" s="11">
-        <v>11</v>
+        <v>29</v>
       </c>
       <c r="F244" s="9" t="s">
         <v>28</v>
@@ -7586,7 +7586,7 @@
         <v>27</v>
       </c>
       <c r="E245" s="11">
-        <v>9</v>
+        <v>23</v>
       </c>
       <c r="F245" s="9" t="s">
         <v>28</v>
@@ -7609,7 +7609,7 @@
         <v>27</v>
       </c>
       <c r="E246" s="11">
-        <v>29</v>
+        <v>24</v>
       </c>
       <c r="F246" s="9" t="s">
         <v>28</v>
@@ -7632,7 +7632,7 @@
         <v>27</v>
       </c>
       <c r="E247" s="11">
-        <v>18</v>
+        <v>10</v>
       </c>
       <c r="F247" s="9" t="s">
         <v>28</v>
@@ -7655,7 +7655,7 @@
         <v>27</v>
       </c>
       <c r="E248" s="11">
-        <v>8</v>
+        <v>12</v>
       </c>
       <c r="F248" s="9" t="s">
         <v>28</v>
@@ -7678,7 +7678,7 @@
         <v>27</v>
       </c>
       <c r="E249" s="11">
-        <v>18</v>
+        <v>21</v>
       </c>
       <c r="F249" s="9" t="s">
         <v>28</v>
@@ -7701,7 +7701,7 @@
         <v>27</v>
       </c>
       <c r="E250" s="11">
-        <v>24</v>
+        <v>12</v>
       </c>
       <c r="F250" s="9" t="s">
         <v>28</v>
@@ -7747,7 +7747,7 @@
         <v>27</v>
       </c>
       <c r="E252" s="11">
-        <v>31</v>
+        <v>19</v>
       </c>
       <c r="F252" s="9" t="s">
         <v>28</v>
@@ -7770,7 +7770,7 @@
         <v>27</v>
       </c>
       <c r="E253" s="11">
-        <v>17</v>
+        <v>26</v>
       </c>
       <c r="F253" s="9" t="s">
         <v>28</v>
@@ -7793,7 +7793,7 @@
         <v>27</v>
       </c>
       <c r="E254" s="11">
-        <v>10</v>
+        <v>16</v>
       </c>
       <c r="F254" s="9" t="s">
         <v>28</v>
@@ -7816,7 +7816,7 @@
         <v>27</v>
       </c>
       <c r="E255" s="11">
-        <v>27</v>
+        <v>14</v>
       </c>
       <c r="F255" s="9" t="s">
         <v>28</v>
@@ -7839,7 +7839,7 @@
         <v>27</v>
       </c>
       <c r="E256" s="11">
-        <v>28</v>
+        <v>12</v>
       </c>
       <c r="F256" s="9" t="s">
         <v>28</v>
@@ -7862,7 +7862,7 @@
         <v>27</v>
       </c>
       <c r="E257" s="11">
-        <v>26</v>
+        <v>12</v>
       </c>
       <c r="F257" s="9" t="s">
         <v>28</v>
@@ -7885,7 +7885,7 @@
         <v>27</v>
       </c>
       <c r="E258" s="11">
-        <v>31</v>
+        <v>10</v>
       </c>
       <c r="F258" s="9" t="s">
         <v>28</v>
@@ -7908,7 +7908,7 @@
         <v>27</v>
       </c>
       <c r="E259" s="11">
-        <v>23</v>
+        <v>16</v>
       </c>
       <c r="F259" s="9" t="s">
         <v>28</v>
@@ -7931,7 +7931,7 @@
         <v>27</v>
       </c>
       <c r="E260" s="11">
-        <v>23</v>
+        <v>31</v>
       </c>
       <c r="F260" s="9" t="s">
         <v>28</v>
@@ -7954,7 +7954,7 @@
         <v>27</v>
       </c>
       <c r="E261" s="11">
-        <v>22</v>
+        <v>31</v>
       </c>
       <c r="F261" s="9" t="s">
         <v>28</v>
@@ -7977,7 +7977,7 @@
         <v>27</v>
       </c>
       <c r="E262" s="11">
-        <v>21</v>
+        <v>23</v>
       </c>
       <c r="F262" s="9" t="s">
         <v>28</v>
@@ -8000,7 +8000,7 @@
         <v>27</v>
       </c>
       <c r="E263" s="11">
-        <v>14</v>
+        <v>25</v>
       </c>
       <c r="F263" s="9" t="s">
         <v>28</v>
@@ -8023,7 +8023,7 @@
         <v>27</v>
       </c>
       <c r="E264" s="11">
-        <v>30</v>
+        <v>20</v>
       </c>
       <c r="F264" s="9" t="s">
         <v>28</v>
@@ -8046,7 +8046,7 @@
         <v>27</v>
       </c>
       <c r="E265" s="11">
-        <v>25</v>
+        <v>21</v>
       </c>
       <c r="F265" s="9" t="s">
         <v>28</v>
@@ -8069,7 +8069,7 @@
         <v>27</v>
       </c>
       <c r="E266" s="11">
-        <v>17</v>
+        <v>29</v>
       </c>
       <c r="F266" s="9" t="s">
         <v>28</v>
@@ -8092,7 +8092,7 @@
         <v>27</v>
       </c>
       <c r="E267" s="11">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="F267" s="9" t="s">
         <v>28</v>
@@ -8115,7 +8115,7 @@
         <v>27</v>
       </c>
       <c r="E268" s="11">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="F268" s="9" t="s">
         <v>28</v>
@@ -8138,7 +8138,7 @@
         <v>27</v>
       </c>
       <c r="E269" s="11">
-        <v>10</v>
+        <v>16</v>
       </c>
       <c r="F269" s="9" t="s">
         <v>28</v>
@@ -8161,7 +8161,7 @@
         <v>27</v>
       </c>
       <c r="E270" s="11">
-        <v>12</v>
+        <v>16</v>
       </c>
       <c r="F270" s="9" t="s">
         <v>28</v>
@@ -8184,7 +8184,7 @@
         <v>27</v>
       </c>
       <c r="E271" s="11">
-        <v>9</v>
+        <v>28</v>
       </c>
       <c r="F271" s="9" t="s">
         <v>28</v>
@@ -8207,7 +8207,7 @@
         <v>27</v>
       </c>
       <c r="E272" s="11">
-        <v>28</v>
+        <v>22</v>
       </c>
       <c r="F272" s="9" t="s">
         <v>28</v>
@@ -8230,7 +8230,7 @@
         <v>27</v>
       </c>
       <c r="E273" s="11">
-        <v>25</v>
+        <v>22</v>
       </c>
       <c r="F273" s="9" t="s">
         <v>28</v>
@@ -8253,7 +8253,7 @@
         <v>27</v>
       </c>
       <c r="E274" s="11">
-        <v>31</v>
+        <v>12</v>
       </c>
       <c r="F274" s="9" t="s">
         <v>28</v>
@@ -8276,7 +8276,7 @@
         <v>27</v>
       </c>
       <c r="E275" s="11">
-        <v>13</v>
+        <v>9</v>
       </c>
       <c r="F275" s="9" t="s">
         <v>28</v>
@@ -8299,7 +8299,7 @@
         <v>27</v>
       </c>
       <c r="E276" s="11">
-        <v>14</v>
+        <v>30</v>
       </c>
       <c r="F276" s="9" t="s">
         <v>28</v>
@@ -8322,7 +8322,7 @@
         <v>27</v>
       </c>
       <c r="E277" s="11">
-        <v>20</v>
+        <v>27</v>
       </c>
       <c r="F277" s="9" t="s">
         <v>28</v>
@@ -8345,7 +8345,7 @@
         <v>27</v>
       </c>
       <c r="E278" s="11">
-        <v>20</v>
+        <v>22</v>
       </c>
       <c r="F278" s="9" t="s">
         <v>28</v>
@@ -8368,7 +8368,7 @@
         <v>27</v>
       </c>
       <c r="E279" s="11">
-        <v>22</v>
+        <v>12</v>
       </c>
       <c r="F279" s="9" t="s">
         <v>28</v>
@@ -8414,7 +8414,7 @@
         <v>27</v>
       </c>
       <c r="E281" s="11">
-        <v>31</v>
+        <v>19</v>
       </c>
       <c r="F281" s="9" t="s">
         <v>28</v>
@@ -8437,7 +8437,7 @@
         <v>27</v>
       </c>
       <c r="E282" s="11">
-        <v>25</v>
+        <v>28</v>
       </c>
       <c r="F282" s="9" t="s">
         <v>28</v>
@@ -8460,7 +8460,7 @@
         <v>27</v>
       </c>
       <c r="E283" s="11">
-        <v>16</v>
+        <v>20</v>
       </c>
       <c r="F283" s="9" t="s">
         <v>28</v>
@@ -8483,7 +8483,7 @@
         <v>27</v>
       </c>
       <c r="E284" s="11">
-        <v>9</v>
+        <v>24</v>
       </c>
       <c r="F284" s="9" t="s">
         <v>28</v>
@@ -8506,7 +8506,7 @@
         <v>27</v>
       </c>
       <c r="E285" s="11">
-        <v>18</v>
+        <v>11</v>
       </c>
       <c r="F285" s="9" t="s">
         <v>28</v>
@@ -8529,7 +8529,7 @@
         <v>27</v>
       </c>
       <c r="E286" s="11">
-        <v>17</v>
+        <v>30</v>
       </c>
       <c r="F286" s="9" t="s">
         <v>28</v>
@@ -8552,7 +8552,7 @@
         <v>27</v>
       </c>
       <c r="E287" s="11">
-        <v>17</v>
+        <v>15</v>
       </c>
       <c r="F287" s="9" t="s">
         <v>28</v>
@@ -8575,7 +8575,7 @@
         <v>27</v>
       </c>
       <c r="E288" s="11">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="F288" s="9" t="s">
         <v>28</v>
@@ -8598,7 +8598,7 @@
         <v>27</v>
       </c>
       <c r="E289" s="11">
-        <v>10</v>
+        <v>18</v>
       </c>
       <c r="F289" s="9" t="s">
         <v>28</v>
@@ -8621,7 +8621,7 @@
         <v>27</v>
       </c>
       <c r="E290" s="11">
-        <v>30</v>
+        <v>8</v>
       </c>
       <c r="F290" s="9" t="s">
         <v>28</v>
@@ -8644,7 +8644,7 @@
         <v>27</v>
       </c>
       <c r="E291" s="11">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="F291" s="9" t="s">
         <v>28</v>
@@ -8667,7 +8667,7 @@
         <v>27</v>
       </c>
       <c r="E292" s="11">
-        <v>20</v>
+        <v>15</v>
       </c>
       <c r="F292" s="9" t="s">
         <v>28</v>
@@ -8690,7 +8690,7 @@
         <v>27</v>
       </c>
       <c r="E293" s="11">
-        <v>21</v>
+        <v>27</v>
       </c>
       <c r="F293" s="9" t="s">
         <v>28</v>
@@ -8713,7 +8713,7 @@
         <v>27</v>
       </c>
       <c r="E294" s="11">
-        <v>12</v>
+        <v>23</v>
       </c>
       <c r="F294" s="9" t="s">
         <v>28</v>
@@ -8736,7 +8736,7 @@
         <v>27</v>
       </c>
       <c r="E295" s="11">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="F295" s="9" t="s">
         <v>28</v>
@@ -8759,7 +8759,7 @@
         <v>27</v>
       </c>
       <c r="E296" s="11">
-        <v>8</v>
+        <v>16</v>
       </c>
       <c r="F296" s="9" t="s">
         <v>28</v>
@@ -8782,7 +8782,7 @@
         <v>27</v>
       </c>
       <c r="E297" s="11">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="F297" s="9" t="s">
         <v>28</v>
@@ -8805,7 +8805,7 @@
         <v>27</v>
       </c>
       <c r="E298" s="11">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="F298" s="9" t="s">
         <v>28</v>
@@ -8828,7 +8828,7 @@
         <v>27</v>
       </c>
       <c r="E299" s="11">
-        <v>21</v>
+        <v>25</v>
       </c>
       <c r="F299" s="9" t="s">
         <v>28</v>
@@ -8851,7 +8851,7 @@
         <v>27</v>
       </c>
       <c r="E300" s="11">
-        <v>15</v>
+        <v>21</v>
       </c>
       <c r="F300" s="9" t="s">
         <v>28</v>
@@ -8874,7 +8874,7 @@
         <v>27</v>
       </c>
       <c r="E301" s="11">
-        <v>23</v>
+        <v>15</v>
       </c>
       <c r="F301" s="9" t="s">
         <v>28</v>
@@ -8897,7 +8897,7 @@
         <v>27</v>
       </c>
       <c r="E302" s="11">
-        <v>13</v>
+        <v>16</v>
       </c>
       <c r="F302" s="9" t="s">
         <v>28</v>
@@ -8920,7 +8920,7 @@
         <v>27</v>
       </c>
       <c r="E303" s="11">
-        <v>16</v>
+        <v>22</v>
       </c>
       <c r="F303" s="9" t="s">
         <v>28</v>
@@ -8943,7 +8943,7 @@
         <v>27</v>
       </c>
       <c r="E304" s="11">
-        <v>25</v>
+        <v>18</v>
       </c>
       <c r="F304" s="9" t="s">
         <v>28</v>
@@ -8966,7 +8966,7 @@
         <v>27</v>
       </c>
       <c r="E305" s="11">
-        <v>8</v>
+        <v>30</v>
       </c>
       <c r="F305" s="9" t="s">
         <v>28</v>
@@ -8989,7 +8989,7 @@
         <v>27</v>
       </c>
       <c r="E306" s="11">
-        <v>18</v>
+        <v>24</v>
       </c>
       <c r="F306" s="9" t="s">
         <v>28</v>
@@ -9012,7 +9012,7 @@
         <v>27</v>
       </c>
       <c r="E307" s="11">
-        <v>21</v>
+        <v>11</v>
       </c>
       <c r="F307" s="9" t="s">
         <v>28</v>
@@ -9035,7 +9035,7 @@
         <v>27</v>
       </c>
       <c r="E308" s="11">
-        <v>18</v>
+        <v>10</v>
       </c>
       <c r="F308" s="9" t="s">
         <v>28</v>
@@ -9058,7 +9058,7 @@
         <v>27</v>
       </c>
       <c r="E309" s="11">
-        <v>11</v>
+        <v>14</v>
       </c>
       <c r="F309" s="9" t="s">
         <v>28</v>
@@ -9081,7 +9081,7 @@
         <v>27</v>
       </c>
       <c r="E310" s="11">
-        <v>20</v>
+        <v>24</v>
       </c>
       <c r="F310" s="9" t="s">
         <v>28</v>
@@ -9104,7 +9104,7 @@
         <v>27</v>
       </c>
       <c r="E311" s="11">
-        <v>23</v>
+        <v>13</v>
       </c>
       <c r="F311" s="9" t="s">
         <v>28</v>
@@ -9127,7 +9127,7 @@
         <v>27</v>
       </c>
       <c r="E312" s="11">
-        <v>28</v>
+        <v>24</v>
       </c>
       <c r="F312" s="9" t="s">
         <v>28</v>
@@ -9150,7 +9150,7 @@
         <v>27</v>
       </c>
       <c r="E313" s="11">
-        <v>18</v>
+        <v>27</v>
       </c>
       <c r="F313" s="9" t="s">
         <v>28</v>
@@ -9173,7 +9173,7 @@
         <v>27</v>
       </c>
       <c r="E314" s="11">
-        <v>26</v>
+        <v>8</v>
       </c>
       <c r="F314" s="9" t="s">
         <v>28</v>
@@ -9196,7 +9196,7 @@
         <v>27</v>
       </c>
       <c r="E315" s="11">
-        <v>25</v>
+        <v>23</v>
       </c>
       <c r="F315" s="9" t="s">
         <v>28</v>
@@ -9219,7 +9219,7 @@
         <v>27</v>
       </c>
       <c r="E316" s="11">
-        <v>12</v>
+        <v>8</v>
       </c>
       <c r="F316" s="9" t="s">
         <v>28</v>
@@ -9242,7 +9242,7 @@
         <v>27</v>
       </c>
       <c r="E317" s="11">
-        <v>10</v>
+        <v>17</v>
       </c>
       <c r="F317" s="9" t="s">
         <v>28</v>
@@ -9265,7 +9265,7 @@
         <v>27</v>
       </c>
       <c r="E318" s="11">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="F318" s="9" t="s">
         <v>28</v>
@@ -9288,7 +9288,7 @@
         <v>27</v>
       </c>
       <c r="E319" s="11">
-        <v>19</v>
+        <v>26</v>
       </c>
       <c r="F319" s="9" t="s">
         <v>28</v>
@@ -9311,7 +9311,7 @@
         <v>27</v>
       </c>
       <c r="E320" s="11">
-        <v>29</v>
+        <v>16</v>
       </c>
       <c r="F320" s="9" t="s">
         <v>28</v>
@@ -9334,7 +9334,7 @@
         <v>27</v>
       </c>
       <c r="E321" s="11">
-        <v>14</v>
+        <v>28</v>
       </c>
       <c r="F321" s="9" t="s">
         <v>28</v>
@@ -9357,7 +9357,7 @@
         <v>27</v>
       </c>
       <c r="E322" s="11">
-        <v>27</v>
+        <v>12</v>
       </c>
       <c r="F322" s="9" t="s">
         <v>28</v>
@@ -9380,7 +9380,7 @@
         <v>27</v>
       </c>
       <c r="E323" s="11">
-        <v>17</v>
+        <v>9</v>
       </c>
       <c r="F323" s="9" t="s">
         <v>28</v>
@@ -9403,7 +9403,7 @@
         <v>27</v>
       </c>
       <c r="E324" s="11">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="F324" s="9" t="s">
         <v>28</v>
@@ -9426,7 +9426,7 @@
         <v>27</v>
       </c>
       <c r="E325" s="11">
-        <v>16</v>
+        <v>18</v>
       </c>
       <c r="F325" s="9" t="s">
         <v>28</v>
@@ -9449,7 +9449,7 @@
         <v>27</v>
       </c>
       <c r="E326" s="11">
-        <v>20</v>
+        <v>30</v>
       </c>
       <c r="F326" s="9" t="s">
         <v>28</v>
@@ -9472,7 +9472,7 @@
         <v>27</v>
       </c>
       <c r="E327" s="11">
-        <v>22</v>
+        <v>30</v>
       </c>
       <c r="F327" s="9" t="s">
         <v>28</v>
@@ -9495,7 +9495,7 @@
         <v>27</v>
       </c>
       <c r="E328" s="11">
-        <v>27</v>
+        <v>29</v>
       </c>
       <c r="F328" s="9" t="s">
         <v>28</v>
@@ -9518,7 +9518,7 @@
         <v>27</v>
       </c>
       <c r="E329" s="11">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="F329" s="9" t="s">
         <v>28</v>
@@ -9541,7 +9541,7 @@
         <v>27</v>
       </c>
       <c r="E330" s="11">
-        <v>8</v>
+        <v>16</v>
       </c>
       <c r="F330" s="9" t="s">
         <v>28</v>
@@ -9564,7 +9564,7 @@
         <v>27</v>
       </c>
       <c r="E331" s="11">
-        <v>27</v>
+        <v>24</v>
       </c>
       <c r="F331" s="9" t="s">
         <v>28</v>
@@ -9587,7 +9587,7 @@
         <v>27</v>
       </c>
       <c r="E332" s="11">
-        <v>8</v>
+        <v>20</v>
       </c>
       <c r="F332" s="9" t="s">
         <v>28</v>
@@ -9610,7 +9610,7 @@
         <v>27</v>
       </c>
       <c r="E333" s="11">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="F333" s="9" t="s">
         <v>28</v>
@@ -9633,7 +9633,7 @@
         <v>27</v>
       </c>
       <c r="E334" s="11">
-        <v>22</v>
+        <v>16</v>
       </c>
       <c r="F334" s="9" t="s">
         <v>28</v>
@@ -9656,7 +9656,7 @@
         <v>27</v>
       </c>
       <c r="E335" s="11">
-        <v>8</v>
+        <v>13</v>
       </c>
       <c r="F335" s="9" t="s">
         <v>28</v>
@@ -9679,7 +9679,7 @@
         <v>27</v>
       </c>
       <c r="E336" s="11">
-        <v>31</v>
+        <v>18</v>
       </c>
       <c r="F336" s="9" t="s">
         <v>28</v>
@@ -9702,7 +9702,7 @@
         <v>27</v>
       </c>
       <c r="E337" s="11">
-        <v>28</v>
+        <v>26</v>
       </c>
       <c r="F337" s="9" t="s">
         <v>28</v>
@@ -9725,7 +9725,7 @@
         <v>27</v>
       </c>
       <c r="E338" s="11">
-        <v>24</v>
+        <v>18</v>
       </c>
       <c r="F338" s="9" t="s">
         <v>28</v>
@@ -9748,7 +9748,7 @@
         <v>27</v>
       </c>
       <c r="E339" s="11">
-        <v>15</v>
+        <v>9</v>
       </c>
       <c r="F339" s="9" t="s">
         <v>28</v>
@@ -9771,7 +9771,7 @@
         <v>27</v>
       </c>
       <c r="E340" s="11">
-        <v>8</v>
+        <v>26</v>
       </c>
       <c r="F340" s="9" t="s">
         <v>28</v>
@@ -9794,7 +9794,7 @@
         <v>27</v>
       </c>
       <c r="E341" s="11">
-        <v>31</v>
+        <v>12</v>
       </c>
       <c r="F341" s="9" t="s">
         <v>28</v>
@@ -9817,7 +9817,7 @@
         <v>27</v>
       </c>
       <c r="E342" s="11">
-        <v>30</v>
+        <v>28</v>
       </c>
       <c r="F342" s="9" t="s">
         <v>28</v>
@@ -9840,7 +9840,7 @@
         <v>27</v>
       </c>
       <c r="E343" s="11">
-        <v>22</v>
+        <v>13</v>
       </c>
       <c r="F343" s="9" t="s">
         <v>28</v>
@@ -9863,7 +9863,7 @@
         <v>27</v>
       </c>
       <c r="E344" s="11">
-        <v>17</v>
+        <v>12</v>
       </c>
       <c r="F344" s="9" t="s">
         <v>28</v>
@@ -9886,7 +9886,7 @@
         <v>27</v>
       </c>
       <c r="E345" s="11">
-        <v>16</v>
+        <v>10</v>
       </c>
       <c r="F345" s="9" t="s">
         <v>28</v>
@@ -9909,7 +9909,7 @@
         <v>27</v>
       </c>
       <c r="E346" s="11">
-        <v>26</v>
+        <v>10</v>
       </c>
       <c r="F346" s="9" t="s">
         <v>28</v>
@@ -9932,7 +9932,7 @@
         <v>27</v>
       </c>
       <c r="E347" s="11">
-        <v>11</v>
+        <v>17</v>
       </c>
       <c r="F347" s="9" t="s">
         <v>28</v>
@@ -9955,7 +9955,7 @@
         <v>27</v>
       </c>
       <c r="E348" s="11">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="F348" s="9" t="s">
         <v>28</v>
@@ -9978,7 +9978,7 @@
         <v>27</v>
       </c>
       <c r="E349" s="11">
-        <v>23</v>
+        <v>21</v>
       </c>
       <c r="F349" s="9" t="s">
         <v>28</v>
@@ -10001,7 +10001,7 @@
         <v>27</v>
       </c>
       <c r="E350" s="11">
-        <v>22</v>
+        <v>31</v>
       </c>
       <c r="F350" s="9" t="s">
         <v>28</v>
@@ -10024,7 +10024,7 @@
         <v>27</v>
       </c>
       <c r="E351" s="11">
-        <v>13</v>
+        <v>31</v>
       </c>
       <c r="F351" s="9" t="s">
         <v>28</v>
@@ -10047,7 +10047,7 @@
         <v>27</v>
       </c>
       <c r="E352" s="11">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="F352" s="9" t="s">
         <v>28</v>
@@ -10070,7 +10070,7 @@
         <v>27</v>
       </c>
       <c r="E353" s="11">
-        <v>14</v>
+        <v>29</v>
       </c>
       <c r="F353" s="9" t="s">
         <v>28</v>
@@ -10093,7 +10093,7 @@
         <v>27</v>
       </c>
       <c r="E354" s="11">
-        <v>23</v>
+        <v>20</v>
       </c>
       <c r="F354" s="9" t="s">
         <v>28</v>
@@ -10116,7 +10116,7 @@
         <v>27</v>
       </c>
       <c r="E355" s="11">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="F355" s="9" t="s">
         <v>28</v>
@@ -10139,7 +10139,7 @@
         <v>27</v>
       </c>
       <c r="E356" s="11">
-        <v>19</v>
+        <v>26</v>
       </c>
       <c r="F356" s="9" t="s">
         <v>28</v>
@@ -10162,7 +10162,7 @@
         <v>27</v>
       </c>
       <c r="E357" s="11">
-        <v>17</v>
+        <v>14</v>
       </c>
       <c r="F357" s="9" t="s">
         <v>28</v>
@@ -10185,7 +10185,7 @@
         <v>27</v>
       </c>
       <c r="E358" s="11">
-        <v>26</v>
+        <v>14</v>
       </c>
       <c r="F358" s="9" t="s">
         <v>28</v>
@@ -10208,7 +10208,7 @@
         <v>27</v>
       </c>
       <c r="E359" s="11">
-        <v>8</v>
+        <v>26</v>
       </c>
       <c r="F359" s="9" t="s">
         <v>28</v>
@@ -10231,7 +10231,7 @@
         <v>27</v>
       </c>
       <c r="E360" s="11">
-        <v>31</v>
+        <v>24</v>
       </c>
       <c r="F360" s="9" t="s">
         <v>28</v>
@@ -10254,7 +10254,7 @@
         <v>27</v>
       </c>
       <c r="E361" s="11">
-        <v>26</v>
+        <v>30</v>
       </c>
       <c r="F361" s="9" t="s">
         <v>28</v>
@@ -10300,7 +10300,7 @@
         <v>27</v>
       </c>
       <c r="E363" s="11">
-        <v>14</v>
+        <v>27</v>
       </c>
       <c r="F363" s="9" t="s">
         <v>28</v>
@@ -10323,7 +10323,7 @@
         <v>27</v>
       </c>
       <c r="E364" s="11">
-        <v>19</v>
+        <v>8</v>
       </c>
       <c r="F364" s="9" t="s">
         <v>28</v>
@@ -10346,7 +10346,7 @@
         <v>27</v>
       </c>
       <c r="E365" s="11">
-        <v>14</v>
+        <v>27</v>
       </c>
       <c r="F365" s="9" t="s">
         <v>28</v>
@@ -10369,7 +10369,7 @@
         <v>27</v>
       </c>
       <c r="E366" s="11">
-        <v>15</v>
+        <v>29</v>
       </c>
       <c r="F366" s="9" t="s">
         <v>28</v>
@@ -10392,7 +10392,7 @@
         <v>27</v>
       </c>
       <c r="E367" s="11">
-        <v>10</v>
+        <v>13</v>
       </c>
       <c r="F367" s="9" t="s">
         <v>28</v>
@@ -10415,7 +10415,7 @@
         <v>27</v>
       </c>
       <c r="E368" s="11">
-        <v>26</v>
+        <v>18</v>
       </c>
       <c r="F368" s="9" t="s">
         <v>28</v>
@@ -10438,7 +10438,7 @@
         <v>27</v>
       </c>
       <c r="E369" s="11">
-        <v>17</v>
+        <v>10</v>
       </c>
       <c r="F369" s="9" t="s">
         <v>28</v>
@@ -10461,7 +10461,7 @@
         <v>27</v>
       </c>
       <c r="E370" s="11">
-        <v>15</v>
+        <v>13</v>
       </c>
       <c r="F370" s="9" t="s">
         <v>28</v>
@@ -10484,7 +10484,7 @@
         <v>27</v>
       </c>
       <c r="E371" s="11">
-        <v>28</v>
+        <v>8</v>
       </c>
       <c r="F371" s="9" t="s">
         <v>28</v>
@@ -10507,7 +10507,7 @@
         <v>27</v>
       </c>
       <c r="E372" s="11">
-        <v>10</v>
+        <v>30</v>
       </c>
       <c r="F372" s="9" t="s">
         <v>28</v>
@@ -10530,7 +10530,7 @@
         <v>27</v>
       </c>
       <c r="E373" s="11">
-        <v>14</v>
+        <v>23</v>
       </c>
       <c r="F373" s="9" t="s">
         <v>28</v>
@@ -10553,7 +10553,7 @@
         <v>27</v>
       </c>
       <c r="E374" s="11">
-        <v>21</v>
+        <v>23</v>
       </c>
       <c r="F374" s="9" t="s">
         <v>28</v>
@@ -10599,7 +10599,7 @@
         <v>27</v>
       </c>
       <c r="E376" s="11">
-        <v>27</v>
+        <v>18</v>
       </c>
       <c r="F376" s="9" t="s">
         <v>28</v>
@@ -10622,7 +10622,7 @@
         <v>27</v>
       </c>
       <c r="E377" s="11">
-        <v>22</v>
+        <v>12</v>
       </c>
       <c r="F377" s="9" t="s">
         <v>28</v>
@@ -10645,7 +10645,7 @@
         <v>27</v>
       </c>
       <c r="E378" s="11">
-        <v>29</v>
+        <v>17</v>
       </c>
       <c r="F378" s="9" t="s">
         <v>28</v>
@@ -10668,7 +10668,7 @@
         <v>27</v>
       </c>
       <c r="E379" s="11">
-        <v>23</v>
+        <v>15</v>
       </c>
       <c r="F379" s="9" t="s">
         <v>28</v>
@@ -10691,7 +10691,7 @@
         <v>27</v>
       </c>
       <c r="E380" s="11">
-        <v>15</v>
+        <v>26</v>
       </c>
       <c r="F380" s="9" t="s">
         <v>28</v>
@@ -10714,7 +10714,7 @@
         <v>27</v>
       </c>
       <c r="E381" s="11">
-        <v>14</v>
+        <v>31</v>
       </c>
       <c r="F381" s="9" t="s">
         <v>28</v>
@@ -10737,7 +10737,7 @@
         <v>27</v>
       </c>
       <c r="E382" s="11">
-        <v>18</v>
+        <v>22</v>
       </c>
       <c r="F382" s="9" t="s">
         <v>28</v>
@@ -10760,7 +10760,7 @@
         <v>27</v>
       </c>
       <c r="E383" s="11">
-        <v>8</v>
+        <v>31</v>
       </c>
       <c r="F383" s="9" t="s">
         <v>28</v>
@@ -10783,7 +10783,7 @@
         <v>27</v>
       </c>
       <c r="E384" s="11">
-        <v>31</v>
+        <v>10</v>
       </c>
       <c r="F384" s="9" t="s">
         <v>28</v>
@@ -10806,7 +10806,7 @@
         <v>27</v>
       </c>
       <c r="E385" s="11">
-        <v>11</v>
+        <v>14</v>
       </c>
       <c r="F385" s="9" t="s">
         <v>28</v>
@@ -10829,7 +10829,7 @@
         <v>27</v>
       </c>
       <c r="E386" s="11">
-        <v>16</v>
+        <v>31</v>
       </c>
       <c r="F386" s="9" t="s">
         <v>28</v>
@@ -10852,7 +10852,7 @@
         <v>27</v>
       </c>
       <c r="E387" s="11">
-        <v>15</v>
+        <v>29</v>
       </c>
       <c r="F387" s="9" t="s">
         <v>28</v>
@@ -10875,7 +10875,7 @@
         <v>27</v>
       </c>
       <c r="E388" s="11">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="F388" s="9" t="s">
         <v>28</v>
@@ -10898,7 +10898,7 @@
         <v>27</v>
       </c>
       <c r="E389" s="11">
-        <v>8</v>
+        <v>28</v>
       </c>
       <c r="F389" s="9" t="s">
         <v>28</v>
@@ -10921,7 +10921,7 @@
         <v>27</v>
       </c>
       <c r="E390" s="11">
-        <v>11</v>
+        <v>14</v>
       </c>
       <c r="F390" s="9" t="s">
         <v>28</v>
@@ -10944,7 +10944,7 @@
         <v>27</v>
       </c>
       <c r="E391" s="11">
-        <v>21</v>
+        <v>18</v>
       </c>
       <c r="F391" s="9" t="s">
         <v>28</v>
@@ -10967,7 +10967,7 @@
         <v>27</v>
       </c>
       <c r="E392" s="11">
-        <v>21</v>
+        <v>11</v>
       </c>
       <c r="F392" s="9" t="s">
         <v>28</v>
@@ -10990,7 +10990,7 @@
         <v>27</v>
       </c>
       <c r="E393" s="11">
-        <v>27</v>
+        <v>19</v>
       </c>
       <c r="F393" s="9" t="s">
         <v>28</v>
@@ -11013,7 +11013,7 @@
         <v>27</v>
       </c>
       <c r="E394" s="11">
-        <v>31</v>
+        <v>28</v>
       </c>
       <c r="F394" s="9" t="s">
         <v>28</v>
@@ -11036,7 +11036,7 @@
         <v>27</v>
       </c>
       <c r="E395" s="11">
-        <v>29</v>
+        <v>27</v>
       </c>
       <c r="F395" s="9" t="s">
         <v>28</v>
@@ -11059,7 +11059,7 @@
         <v>27</v>
       </c>
       <c r="E396" s="11">
-        <v>31</v>
+        <v>18</v>
       </c>
       <c r="F396" s="9" t="s">
         <v>28</v>
@@ -11082,7 +11082,7 @@
         <v>27</v>
       </c>
       <c r="E397" s="11">
-        <v>17</v>
+        <v>19</v>
       </c>
       <c r="F397" s="9" t="s">
         <v>28</v>
@@ -11105,7 +11105,7 @@
         <v>27</v>
       </c>
       <c r="E398" s="11">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="F398" s="9" t="s">
         <v>28</v>
@@ -11128,7 +11128,7 @@
         <v>27</v>
       </c>
       <c r="E399" s="11">
-        <v>16</v>
+        <v>27</v>
       </c>
       <c r="F399" s="9" t="s">
         <v>28</v>
@@ -11151,7 +11151,7 @@
         <v>27</v>
       </c>
       <c r="E400" s="11">
-        <v>28</v>
+        <v>26</v>
       </c>
       <c r="F400" s="9" t="s">
         <v>28</v>
@@ -11174,7 +11174,7 @@
         <v>27</v>
       </c>
       <c r="E401" s="11">
-        <v>16</v>
+        <v>12</v>
       </c>
       <c r="F401" s="9" t="s">
         <v>28</v>

</xml_diff>

<commit_message>
refactor(catalog): remove all default mock items from home page and application data catalog
</commit_message>
<xml_diff>
--- a/all-test-reports/selenium/selenium_e2e_test_report.xlsx
+++ b/all-test-reports/selenium/selenium_e2e_test_report.xlsx
@@ -35,7 +35,7 @@
     <t>Execution Date</t>
   </si>
   <si>
-    <t>28/7/2026, 10:42:38 am</t>
+    <t>28/7/2026, 10:47:41 am</t>
   </si>
   <si>
     <t>Browser / Mode</t>
@@ -47,7 +47,7 @@
     <t>Total Duration</t>
   </si>
   <si>
-    <t>0.03 seconds</t>
+    <t>0.02 seconds</t>
   </si>
   <si>
     <t>Selenium Test Execution Summary Metrics</t>
@@ -98,7 +98,7 @@
     <t>PASS</t>
   </si>
   <si>
-    <t>10:42:38 am</t>
+    <t>10:47:41 am</t>
   </si>
   <si>
     <t>N/A</t>
@@ -1997,7 +1997,7 @@
         <v>27</v>
       </c>
       <c r="E2" s="11">
-        <v>12</v>
+        <v>21</v>
       </c>
       <c r="F2" s="9" t="s">
         <v>28</v>
@@ -2043,7 +2043,7 @@
         <v>27</v>
       </c>
       <c r="E4" s="11">
-        <v>23</v>
+        <v>18</v>
       </c>
       <c r="F4" s="9" t="s">
         <v>28</v>
@@ -2066,7 +2066,7 @@
         <v>27</v>
       </c>
       <c r="E5" s="11">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="F5" s="9" t="s">
         <v>28</v>
@@ -2089,7 +2089,7 @@
         <v>27</v>
       </c>
       <c r="E6" s="11">
-        <v>8</v>
+        <v>13</v>
       </c>
       <c r="F6" s="9" t="s">
         <v>28</v>
@@ -2112,7 +2112,7 @@
         <v>27</v>
       </c>
       <c r="E7" s="11">
-        <v>19</v>
+        <v>28</v>
       </c>
       <c r="F7" s="9" t="s">
         <v>28</v>
@@ -2135,7 +2135,7 @@
         <v>27</v>
       </c>
       <c r="E8" s="11">
-        <v>27</v>
+        <v>17</v>
       </c>
       <c r="F8" s="9" t="s">
         <v>28</v>
@@ -2158,7 +2158,7 @@
         <v>27</v>
       </c>
       <c r="E9" s="11">
-        <v>11</v>
+        <v>25</v>
       </c>
       <c r="F9" s="9" t="s">
         <v>28</v>
@@ -2181,7 +2181,7 @@
         <v>27</v>
       </c>
       <c r="E10" s="11">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="F10" s="9" t="s">
         <v>28</v>
@@ -2204,7 +2204,7 @@
         <v>27</v>
       </c>
       <c r="E11" s="11">
-        <v>25</v>
+        <v>16</v>
       </c>
       <c r="F11" s="9" t="s">
         <v>28</v>
@@ -2227,7 +2227,7 @@
         <v>27</v>
       </c>
       <c r="E12" s="11">
-        <v>11</v>
+        <v>26</v>
       </c>
       <c r="F12" s="9" t="s">
         <v>28</v>
@@ -2250,7 +2250,7 @@
         <v>27</v>
       </c>
       <c r="E13" s="11">
-        <v>31</v>
+        <v>22</v>
       </c>
       <c r="F13" s="9" t="s">
         <v>28</v>
@@ -2273,7 +2273,7 @@
         <v>27</v>
       </c>
       <c r="E14" s="11">
-        <v>12</v>
+        <v>20</v>
       </c>
       <c r="F14" s="9" t="s">
         <v>28</v>
@@ -2296,7 +2296,7 @@
         <v>27</v>
       </c>
       <c r="E15" s="11">
-        <v>19</v>
+        <v>26</v>
       </c>
       <c r="F15" s="9" t="s">
         <v>28</v>
@@ -2319,7 +2319,7 @@
         <v>27</v>
       </c>
       <c r="E16" s="11">
-        <v>26</v>
+        <v>10</v>
       </c>
       <c r="F16" s="9" t="s">
         <v>28</v>
@@ -2342,7 +2342,7 @@
         <v>27</v>
       </c>
       <c r="E17" s="11">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="F17" s="9" t="s">
         <v>28</v>
@@ -2365,7 +2365,7 @@
         <v>27</v>
       </c>
       <c r="E18" s="11">
-        <v>15</v>
+        <v>8</v>
       </c>
       <c r="F18" s="9" t="s">
         <v>28</v>
@@ -2388,7 +2388,7 @@
         <v>27</v>
       </c>
       <c r="E19" s="11">
-        <v>17</v>
+        <v>8</v>
       </c>
       <c r="F19" s="9" t="s">
         <v>28</v>
@@ -2411,7 +2411,7 @@
         <v>27</v>
       </c>
       <c r="E20" s="11">
-        <v>25</v>
+        <v>20</v>
       </c>
       <c r="F20" s="9" t="s">
         <v>28</v>
@@ -2434,7 +2434,7 @@
         <v>27</v>
       </c>
       <c r="E21" s="11">
-        <v>10</v>
+        <v>17</v>
       </c>
       <c r="F21" s="9" t="s">
         <v>28</v>
@@ -2457,7 +2457,7 @@
         <v>27</v>
       </c>
       <c r="E22" s="11">
-        <v>28</v>
+        <v>26</v>
       </c>
       <c r="F22" s="9" t="s">
         <v>28</v>
@@ -2480,7 +2480,7 @@
         <v>27</v>
       </c>
       <c r="E23" s="11">
-        <v>28</v>
+        <v>18</v>
       </c>
       <c r="F23" s="9" t="s">
         <v>28</v>
@@ -2503,7 +2503,7 @@
         <v>27</v>
       </c>
       <c r="E24" s="11">
-        <v>27</v>
+        <v>20</v>
       </c>
       <c r="F24" s="9" t="s">
         <v>28</v>
@@ -2526,7 +2526,7 @@
         <v>27</v>
       </c>
       <c r="E25" s="11">
-        <v>13</v>
+        <v>30</v>
       </c>
       <c r="F25" s="9" t="s">
         <v>28</v>
@@ -2549,7 +2549,7 @@
         <v>27</v>
       </c>
       <c r="E26" s="11">
-        <v>29</v>
+        <v>16</v>
       </c>
       <c r="F26" s="9" t="s">
         <v>28</v>
@@ -2572,7 +2572,7 @@
         <v>27</v>
       </c>
       <c r="E27" s="11">
-        <v>28</v>
+        <v>20</v>
       </c>
       <c r="F27" s="9" t="s">
         <v>28</v>
@@ -2595,7 +2595,7 @@
         <v>27</v>
       </c>
       <c r="E28" s="11">
-        <v>23</v>
+        <v>25</v>
       </c>
       <c r="F28" s="9" t="s">
         <v>28</v>
@@ -2618,7 +2618,7 @@
         <v>27</v>
       </c>
       <c r="E29" s="11">
-        <v>23</v>
+        <v>14</v>
       </c>
       <c r="F29" s="9" t="s">
         <v>28</v>
@@ -2641,7 +2641,7 @@
         <v>27</v>
       </c>
       <c r="E30" s="11">
-        <v>17</v>
+        <v>28</v>
       </c>
       <c r="F30" s="9" t="s">
         <v>28</v>
@@ -2664,7 +2664,7 @@
         <v>27</v>
       </c>
       <c r="E31" s="11">
-        <v>25</v>
+        <v>21</v>
       </c>
       <c r="F31" s="9" t="s">
         <v>28</v>
@@ -2687,7 +2687,7 @@
         <v>27</v>
       </c>
       <c r="E32" s="11">
-        <v>12</v>
+        <v>21</v>
       </c>
       <c r="F32" s="9" t="s">
         <v>28</v>
@@ -2710,7 +2710,7 @@
         <v>27</v>
       </c>
       <c r="E33" s="11">
-        <v>30</v>
+        <v>18</v>
       </c>
       <c r="F33" s="9" t="s">
         <v>28</v>
@@ -2733,7 +2733,7 @@
         <v>27</v>
       </c>
       <c r="E34" s="11">
-        <v>23</v>
+        <v>29</v>
       </c>
       <c r="F34" s="9" t="s">
         <v>28</v>
@@ -2756,7 +2756,7 @@
         <v>27</v>
       </c>
       <c r="E35" s="11">
-        <v>21</v>
+        <v>15</v>
       </c>
       <c r="F35" s="9" t="s">
         <v>28</v>
@@ -2779,7 +2779,7 @@
         <v>27</v>
       </c>
       <c r="E36" s="11">
-        <v>27</v>
+        <v>30</v>
       </c>
       <c r="F36" s="9" t="s">
         <v>28</v>
@@ -2802,7 +2802,7 @@
         <v>27</v>
       </c>
       <c r="E37" s="11">
-        <v>20</v>
+        <v>11</v>
       </c>
       <c r="F37" s="9" t="s">
         <v>28</v>
@@ -2825,7 +2825,7 @@
         <v>27</v>
       </c>
       <c r="E38" s="11">
-        <v>15</v>
+        <v>22</v>
       </c>
       <c r="F38" s="9" t="s">
         <v>28</v>
@@ -2871,7 +2871,7 @@
         <v>27</v>
       </c>
       <c r="E40" s="11">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="F40" s="9" t="s">
         <v>28</v>
@@ -2894,7 +2894,7 @@
         <v>27</v>
       </c>
       <c r="E41" s="11">
-        <v>9</v>
+        <v>30</v>
       </c>
       <c r="F41" s="9" t="s">
         <v>28</v>
@@ -2917,7 +2917,7 @@
         <v>27</v>
       </c>
       <c r="E42" s="11">
-        <v>14</v>
+        <v>30</v>
       </c>
       <c r="F42" s="9" t="s">
         <v>28</v>
@@ -2940,7 +2940,7 @@
         <v>27</v>
       </c>
       <c r="E43" s="11">
-        <v>26</v>
+        <v>13</v>
       </c>
       <c r="F43" s="9" t="s">
         <v>28</v>
@@ -2963,7 +2963,7 @@
         <v>27</v>
       </c>
       <c r="E44" s="11">
-        <v>11</v>
+        <v>22</v>
       </c>
       <c r="F44" s="9" t="s">
         <v>28</v>
@@ -2986,7 +2986,7 @@
         <v>27</v>
       </c>
       <c r="E45" s="11">
-        <v>28</v>
+        <v>14</v>
       </c>
       <c r="F45" s="9" t="s">
         <v>28</v>
@@ -3009,7 +3009,7 @@
         <v>27</v>
       </c>
       <c r="E46" s="11">
-        <v>15</v>
+        <v>24</v>
       </c>
       <c r="F46" s="9" t="s">
         <v>28</v>
@@ -3032,7 +3032,7 @@
         <v>27</v>
       </c>
       <c r="E47" s="11">
-        <v>24</v>
+        <v>11</v>
       </c>
       <c r="F47" s="9" t="s">
         <v>28</v>
@@ -3055,7 +3055,7 @@
         <v>27</v>
       </c>
       <c r="E48" s="11">
-        <v>10</v>
+        <v>30</v>
       </c>
       <c r="F48" s="9" t="s">
         <v>28</v>
@@ -3078,7 +3078,7 @@
         <v>27</v>
       </c>
       <c r="E49" s="11">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="F49" s="9" t="s">
         <v>28</v>
@@ -3101,7 +3101,7 @@
         <v>27</v>
       </c>
       <c r="E50" s="11">
-        <v>25</v>
+        <v>11</v>
       </c>
       <c r="F50" s="9" t="s">
         <v>28</v>
@@ -3124,7 +3124,7 @@
         <v>27</v>
       </c>
       <c r="E51" s="11">
-        <v>13</v>
+        <v>17</v>
       </c>
       <c r="F51" s="9" t="s">
         <v>28</v>
@@ -3147,7 +3147,7 @@
         <v>27</v>
       </c>
       <c r="E52" s="11">
-        <v>26</v>
+        <v>17</v>
       </c>
       <c r="F52" s="9" t="s">
         <v>28</v>
@@ -3170,7 +3170,7 @@
         <v>27</v>
       </c>
       <c r="E53" s="11">
-        <v>15</v>
+        <v>9</v>
       </c>
       <c r="F53" s="9" t="s">
         <v>28</v>
@@ -3193,7 +3193,7 @@
         <v>27</v>
       </c>
       <c r="E54" s="11">
-        <v>15</v>
+        <v>23</v>
       </c>
       <c r="F54" s="9" t="s">
         <v>28</v>
@@ -3216,7 +3216,7 @@
         <v>27</v>
       </c>
       <c r="E55" s="11">
-        <v>18</v>
+        <v>28</v>
       </c>
       <c r="F55" s="9" t="s">
         <v>28</v>
@@ -3239,7 +3239,7 @@
         <v>27</v>
       </c>
       <c r="E56" s="11">
-        <v>12</v>
+        <v>9</v>
       </c>
       <c r="F56" s="9" t="s">
         <v>28</v>
@@ -3262,7 +3262,7 @@
         <v>27</v>
       </c>
       <c r="E57" s="11">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="F57" s="9" t="s">
         <v>28</v>
@@ -3285,7 +3285,7 @@
         <v>27</v>
       </c>
       <c r="E58" s="11">
-        <v>17</v>
+        <v>24</v>
       </c>
       <c r="F58" s="9" t="s">
         <v>28</v>
@@ -3308,7 +3308,7 @@
         <v>27</v>
       </c>
       <c r="E59" s="11">
-        <v>28</v>
+        <v>10</v>
       </c>
       <c r="F59" s="9" t="s">
         <v>28</v>
@@ -3331,7 +3331,7 @@
         <v>27</v>
       </c>
       <c r="E60" s="11">
-        <v>8</v>
+        <v>24</v>
       </c>
       <c r="F60" s="9" t="s">
         <v>28</v>
@@ -3354,7 +3354,7 @@
         <v>27</v>
       </c>
       <c r="E61" s="11">
-        <v>18</v>
+        <v>25</v>
       </c>
       <c r="F61" s="9" t="s">
         <v>28</v>
@@ -3377,7 +3377,7 @@
         <v>27</v>
       </c>
       <c r="E62" s="11">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="F62" s="9" t="s">
         <v>28</v>
@@ -3400,7 +3400,7 @@
         <v>27</v>
       </c>
       <c r="E63" s="11">
-        <v>25</v>
+        <v>27</v>
       </c>
       <c r="F63" s="9" t="s">
         <v>28</v>
@@ -3423,7 +3423,7 @@
         <v>27</v>
       </c>
       <c r="E64" s="11">
-        <v>28</v>
+        <v>12</v>
       </c>
       <c r="F64" s="9" t="s">
         <v>28</v>
@@ -3446,7 +3446,7 @@
         <v>27</v>
       </c>
       <c r="E65" s="11">
-        <v>15</v>
+        <v>12</v>
       </c>
       <c r="F65" s="9" t="s">
         <v>28</v>
@@ -3469,7 +3469,7 @@
         <v>27</v>
       </c>
       <c r="E66" s="11">
-        <v>31</v>
+        <v>29</v>
       </c>
       <c r="F66" s="9" t="s">
         <v>28</v>
@@ -3492,7 +3492,7 @@
         <v>27</v>
       </c>
       <c r="E67" s="11">
-        <v>25</v>
+        <v>21</v>
       </c>
       <c r="F67" s="9" t="s">
         <v>28</v>
@@ -3515,7 +3515,7 @@
         <v>27</v>
       </c>
       <c r="E68" s="11">
-        <v>29</v>
+        <v>23</v>
       </c>
       <c r="F68" s="9" t="s">
         <v>28</v>
@@ -3538,7 +3538,7 @@
         <v>27</v>
       </c>
       <c r="E69" s="11">
-        <v>9</v>
+        <v>30</v>
       </c>
       <c r="F69" s="9" t="s">
         <v>28</v>
@@ -3561,7 +3561,7 @@
         <v>27</v>
       </c>
       <c r="E70" s="11">
-        <v>21</v>
+        <v>11</v>
       </c>
       <c r="F70" s="9" t="s">
         <v>28</v>
@@ -3584,7 +3584,7 @@
         <v>27</v>
       </c>
       <c r="E71" s="11">
-        <v>23</v>
+        <v>27</v>
       </c>
       <c r="F71" s="9" t="s">
         <v>28</v>
@@ -3630,7 +3630,7 @@
         <v>27</v>
       </c>
       <c r="E73" s="11">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="F73" s="9" t="s">
         <v>28</v>
@@ -3653,7 +3653,7 @@
         <v>27</v>
       </c>
       <c r="E74" s="11">
-        <v>30</v>
+        <v>18</v>
       </c>
       <c r="F74" s="9" t="s">
         <v>28</v>
@@ -3676,7 +3676,7 @@
         <v>27</v>
       </c>
       <c r="E75" s="11">
-        <v>29</v>
+        <v>25</v>
       </c>
       <c r="F75" s="9" t="s">
         <v>28</v>
@@ -3699,7 +3699,7 @@
         <v>27</v>
       </c>
       <c r="E76" s="11">
-        <v>31</v>
+        <v>28</v>
       </c>
       <c r="F76" s="9" t="s">
         <v>28</v>
@@ -3722,7 +3722,7 @@
         <v>27</v>
       </c>
       <c r="E77" s="11">
-        <v>29</v>
+        <v>23</v>
       </c>
       <c r="F77" s="9" t="s">
         <v>28</v>
@@ -3745,7 +3745,7 @@
         <v>27</v>
       </c>
       <c r="E78" s="11">
-        <v>15</v>
+        <v>19</v>
       </c>
       <c r="F78" s="9" t="s">
         <v>28</v>
@@ -3768,7 +3768,7 @@
         <v>27</v>
       </c>
       <c r="E79" s="11">
-        <v>31</v>
+        <v>21</v>
       </c>
       <c r="F79" s="9" t="s">
         <v>28</v>
@@ -3791,7 +3791,7 @@
         <v>27</v>
       </c>
       <c r="E80" s="11">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="F80" s="9" t="s">
         <v>28</v>
@@ -3814,7 +3814,7 @@
         <v>27</v>
       </c>
       <c r="E81" s="11">
-        <v>16</v>
+        <v>12</v>
       </c>
       <c r="F81" s="9" t="s">
         <v>28</v>
@@ -3837,7 +3837,7 @@
         <v>27</v>
       </c>
       <c r="E82" s="11">
-        <v>20</v>
+        <v>13</v>
       </c>
       <c r="F82" s="9" t="s">
         <v>28</v>
@@ -3860,7 +3860,7 @@
         <v>27</v>
       </c>
       <c r="E83" s="11">
-        <v>26</v>
+        <v>13</v>
       </c>
       <c r="F83" s="9" t="s">
         <v>28</v>
@@ -3883,7 +3883,7 @@
         <v>27</v>
       </c>
       <c r="E84" s="11">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="F84" s="9" t="s">
         <v>28</v>
@@ -3906,7 +3906,7 @@
         <v>27</v>
       </c>
       <c r="E85" s="11">
-        <v>18</v>
+        <v>31</v>
       </c>
       <c r="F85" s="9" t="s">
         <v>28</v>
@@ -3929,7 +3929,7 @@
         <v>27</v>
       </c>
       <c r="E86" s="11">
-        <v>28</v>
+        <v>24</v>
       </c>
       <c r="F86" s="9" t="s">
         <v>28</v>
@@ -3952,7 +3952,7 @@
         <v>27</v>
       </c>
       <c r="E87" s="11">
-        <v>27</v>
+        <v>25</v>
       </c>
       <c r="F87" s="9" t="s">
         <v>28</v>
@@ -3975,7 +3975,7 @@
         <v>27</v>
       </c>
       <c r="E88" s="11">
-        <v>18</v>
+        <v>28</v>
       </c>
       <c r="F88" s="9" t="s">
         <v>28</v>
@@ -3998,7 +3998,7 @@
         <v>27</v>
       </c>
       <c r="E89" s="11">
-        <v>10</v>
+        <v>21</v>
       </c>
       <c r="F89" s="9" t="s">
         <v>28</v>
@@ -4021,7 +4021,7 @@
         <v>27</v>
       </c>
       <c r="E90" s="11">
-        <v>10</v>
+        <v>18</v>
       </c>
       <c r="F90" s="9" t="s">
         <v>28</v>
@@ -4044,7 +4044,7 @@
         <v>27</v>
       </c>
       <c r="E91" s="11">
-        <v>19</v>
+        <v>27</v>
       </c>
       <c r="F91" s="9" t="s">
         <v>28</v>
@@ -4067,7 +4067,7 @@
         <v>27</v>
       </c>
       <c r="E92" s="11">
-        <v>13</v>
+        <v>21</v>
       </c>
       <c r="F92" s="9" t="s">
         <v>28</v>
@@ -4090,7 +4090,7 @@
         <v>27</v>
       </c>
       <c r="E93" s="11">
-        <v>27</v>
+        <v>29</v>
       </c>
       <c r="F93" s="9" t="s">
         <v>28</v>
@@ -4113,7 +4113,7 @@
         <v>27</v>
       </c>
       <c r="E94" s="11">
-        <v>8</v>
+        <v>18</v>
       </c>
       <c r="F94" s="9" t="s">
         <v>28</v>
@@ -4136,7 +4136,7 @@
         <v>27</v>
       </c>
       <c r="E95" s="11">
-        <v>27</v>
+        <v>25</v>
       </c>
       <c r="F95" s="9" t="s">
         <v>28</v>
@@ -4159,7 +4159,7 @@
         <v>27</v>
       </c>
       <c r="E96" s="11">
-        <v>18</v>
+        <v>23</v>
       </c>
       <c r="F96" s="9" t="s">
         <v>28</v>
@@ -4182,7 +4182,7 @@
         <v>27</v>
       </c>
       <c r="E97" s="11">
-        <v>30</v>
+        <v>27</v>
       </c>
       <c r="F97" s="9" t="s">
         <v>28</v>
@@ -4205,7 +4205,7 @@
         <v>27</v>
       </c>
       <c r="E98" s="11">
-        <v>21</v>
+        <v>8</v>
       </c>
       <c r="F98" s="9" t="s">
         <v>28</v>
@@ -4228,7 +4228,7 @@
         <v>27</v>
       </c>
       <c r="E99" s="11">
-        <v>12</v>
+        <v>22</v>
       </c>
       <c r="F99" s="9" t="s">
         <v>28</v>
@@ -4251,7 +4251,7 @@
         <v>27</v>
       </c>
       <c r="E100" s="11">
-        <v>27</v>
+        <v>16</v>
       </c>
       <c r="F100" s="9" t="s">
         <v>28</v>
@@ -4274,7 +4274,7 @@
         <v>27</v>
       </c>
       <c r="E101" s="11">
-        <v>30</v>
+        <v>11</v>
       </c>
       <c r="F101" s="9" t="s">
         <v>28</v>
@@ -4297,7 +4297,7 @@
         <v>27</v>
       </c>
       <c r="E102" s="11">
-        <v>27</v>
+        <v>10</v>
       </c>
       <c r="F102" s="9" t="s">
         <v>28</v>
@@ -4320,7 +4320,7 @@
         <v>27</v>
       </c>
       <c r="E103" s="11">
-        <v>8</v>
+        <v>12</v>
       </c>
       <c r="F103" s="9" t="s">
         <v>28</v>
@@ -4343,7 +4343,7 @@
         <v>27</v>
       </c>
       <c r="E104" s="11">
-        <v>12</v>
+        <v>24</v>
       </c>
       <c r="F104" s="9" t="s">
         <v>28</v>
@@ -4366,7 +4366,7 @@
         <v>27</v>
       </c>
       <c r="E105" s="11">
-        <v>8</v>
+        <v>24</v>
       </c>
       <c r="F105" s="9" t="s">
         <v>28</v>
@@ -4389,7 +4389,7 @@
         <v>27</v>
       </c>
       <c r="E106" s="11">
-        <v>22</v>
+        <v>24</v>
       </c>
       <c r="F106" s="9" t="s">
         <v>28</v>
@@ -4412,7 +4412,7 @@
         <v>27</v>
       </c>
       <c r="E107" s="11">
-        <v>30</v>
+        <v>18</v>
       </c>
       <c r="F107" s="9" t="s">
         <v>28</v>
@@ -4435,7 +4435,7 @@
         <v>27</v>
       </c>
       <c r="E108" s="11">
-        <v>22</v>
+        <v>8</v>
       </c>
       <c r="F108" s="9" t="s">
         <v>28</v>
@@ -4458,7 +4458,7 @@
         <v>27</v>
       </c>
       <c r="E109" s="11">
-        <v>16</v>
+        <v>18</v>
       </c>
       <c r="F109" s="9" t="s">
         <v>28</v>
@@ -4481,7 +4481,7 @@
         <v>27</v>
       </c>
       <c r="E110" s="11">
-        <v>24</v>
+        <v>16</v>
       </c>
       <c r="F110" s="9" t="s">
         <v>28</v>
@@ -4504,7 +4504,7 @@
         <v>27</v>
       </c>
       <c r="E111" s="11">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="F111" s="9" t="s">
         <v>28</v>
@@ -4527,7 +4527,7 @@
         <v>27</v>
       </c>
       <c r="E112" s="11">
-        <v>17</v>
+        <v>29</v>
       </c>
       <c r="F112" s="9" t="s">
         <v>28</v>
@@ -4550,7 +4550,7 @@
         <v>27</v>
       </c>
       <c r="E113" s="11">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="F113" s="9" t="s">
         <v>28</v>
@@ -4573,7 +4573,7 @@
         <v>27</v>
       </c>
       <c r="E114" s="11">
-        <v>9</v>
+        <v>19</v>
       </c>
       <c r="F114" s="9" t="s">
         <v>28</v>
@@ -4596,7 +4596,7 @@
         <v>27</v>
       </c>
       <c r="E115" s="11">
-        <v>23</v>
+        <v>15</v>
       </c>
       <c r="F115" s="9" t="s">
         <v>28</v>
@@ -4619,7 +4619,7 @@
         <v>27</v>
       </c>
       <c r="E116" s="11">
-        <v>11</v>
+        <v>8</v>
       </c>
       <c r="F116" s="9" t="s">
         <v>28</v>
@@ -4642,7 +4642,7 @@
         <v>27</v>
       </c>
       <c r="E117" s="11">
-        <v>11</v>
+        <v>9</v>
       </c>
       <c r="F117" s="9" t="s">
         <v>28</v>
@@ -4665,7 +4665,7 @@
         <v>27</v>
       </c>
       <c r="E118" s="11">
-        <v>29</v>
+        <v>12</v>
       </c>
       <c r="F118" s="9" t="s">
         <v>28</v>
@@ -4688,7 +4688,7 @@
         <v>27</v>
       </c>
       <c r="E119" s="11">
-        <v>29</v>
+        <v>27</v>
       </c>
       <c r="F119" s="9" t="s">
         <v>28</v>
@@ -4711,7 +4711,7 @@
         <v>27</v>
       </c>
       <c r="E120" s="11">
-        <v>12</v>
+        <v>26</v>
       </c>
       <c r="F120" s="9" t="s">
         <v>28</v>
@@ -4734,7 +4734,7 @@
         <v>27</v>
       </c>
       <c r="E121" s="11">
-        <v>8</v>
+        <v>13</v>
       </c>
       <c r="F121" s="9" t="s">
         <v>28</v>
@@ -4757,7 +4757,7 @@
         <v>27</v>
       </c>
       <c r="E122" s="11">
-        <v>24</v>
+        <v>21</v>
       </c>
       <c r="F122" s="9" t="s">
         <v>28</v>
@@ -4780,7 +4780,7 @@
         <v>27</v>
       </c>
       <c r="E123" s="11">
-        <v>26</v>
+        <v>31</v>
       </c>
       <c r="F123" s="9" t="s">
         <v>28</v>
@@ -4803,7 +4803,7 @@
         <v>27</v>
       </c>
       <c r="E124" s="11">
-        <v>19</v>
+        <v>24</v>
       </c>
       <c r="F124" s="9" t="s">
         <v>28</v>
@@ -4826,7 +4826,7 @@
         <v>27</v>
       </c>
       <c r="E125" s="11">
-        <v>26</v>
+        <v>13</v>
       </c>
       <c r="F125" s="9" t="s">
         <v>28</v>
@@ -4849,7 +4849,7 @@
         <v>27</v>
       </c>
       <c r="E126" s="11">
-        <v>25</v>
+        <v>19</v>
       </c>
       <c r="F126" s="9" t="s">
         <v>28</v>
@@ -4872,7 +4872,7 @@
         <v>27</v>
       </c>
       <c r="E127" s="11">
-        <v>21</v>
+        <v>16</v>
       </c>
       <c r="F127" s="9" t="s">
         <v>28</v>
@@ -4895,7 +4895,7 @@
         <v>27</v>
       </c>
       <c r="E128" s="11">
-        <v>22</v>
+        <v>8</v>
       </c>
       <c r="F128" s="9" t="s">
         <v>28</v>
@@ -4918,7 +4918,7 @@
         <v>27</v>
       </c>
       <c r="E129" s="11">
-        <v>25</v>
+        <v>20</v>
       </c>
       <c r="F129" s="9" t="s">
         <v>28</v>
@@ -4964,7 +4964,7 @@
         <v>27</v>
       </c>
       <c r="E131" s="11">
-        <v>14</v>
+        <v>30</v>
       </c>
       <c r="F131" s="9" t="s">
         <v>28</v>
@@ -4987,7 +4987,7 @@
         <v>27</v>
       </c>
       <c r="E132" s="11">
-        <v>20</v>
+        <v>24</v>
       </c>
       <c r="F132" s="9" t="s">
         <v>28</v>
@@ -5033,7 +5033,7 @@
         <v>27</v>
       </c>
       <c r="E134" s="11">
-        <v>11</v>
+        <v>23</v>
       </c>
       <c r="F134" s="9" t="s">
         <v>28</v>
@@ -5056,7 +5056,7 @@
         <v>27</v>
       </c>
       <c r="E135" s="11">
-        <v>18</v>
+        <v>24</v>
       </c>
       <c r="F135" s="9" t="s">
         <v>28</v>
@@ -5079,7 +5079,7 @@
         <v>27</v>
       </c>
       <c r="E136" s="11">
-        <v>18</v>
+        <v>29</v>
       </c>
       <c r="F136" s="9" t="s">
         <v>28</v>
@@ -5102,7 +5102,7 @@
         <v>27</v>
       </c>
       <c r="E137" s="11">
-        <v>18</v>
+        <v>26</v>
       </c>
       <c r="F137" s="9" t="s">
         <v>28</v>
@@ -5125,7 +5125,7 @@
         <v>27</v>
       </c>
       <c r="E138" s="11">
-        <v>16</v>
+        <v>31</v>
       </c>
       <c r="F138" s="9" t="s">
         <v>28</v>
@@ -5148,7 +5148,7 @@
         <v>27</v>
       </c>
       <c r="E139" s="11">
-        <v>15</v>
+        <v>13</v>
       </c>
       <c r="F139" s="9" t="s">
         <v>28</v>
@@ -5194,7 +5194,7 @@
         <v>27</v>
       </c>
       <c r="E141" s="11">
-        <v>14</v>
+        <v>30</v>
       </c>
       <c r="F141" s="9" t="s">
         <v>28</v>
@@ -5240,7 +5240,7 @@
         <v>27</v>
       </c>
       <c r="E143" s="11">
-        <v>24</v>
+        <v>27</v>
       </c>
       <c r="F143" s="9" t="s">
         <v>28</v>
@@ -5263,7 +5263,7 @@
         <v>27</v>
       </c>
       <c r="E144" s="11">
-        <v>26</v>
+        <v>9</v>
       </c>
       <c r="F144" s="9" t="s">
         <v>28</v>
@@ -5286,7 +5286,7 @@
         <v>27</v>
       </c>
       <c r="E145" s="11">
-        <v>10</v>
+        <v>27</v>
       </c>
       <c r="F145" s="9" t="s">
         <v>28</v>
@@ -5309,7 +5309,7 @@
         <v>27</v>
       </c>
       <c r="E146" s="11">
-        <v>12</v>
+        <v>24</v>
       </c>
       <c r="F146" s="9" t="s">
         <v>28</v>
@@ -5332,7 +5332,7 @@
         <v>27</v>
       </c>
       <c r="E147" s="11">
-        <v>23</v>
+        <v>28</v>
       </c>
       <c r="F147" s="9" t="s">
         <v>28</v>
@@ -5355,7 +5355,7 @@
         <v>27</v>
       </c>
       <c r="E148" s="11">
-        <v>16</v>
+        <v>8</v>
       </c>
       <c r="F148" s="9" t="s">
         <v>28</v>
@@ -5378,7 +5378,7 @@
         <v>27</v>
       </c>
       <c r="E149" s="11">
-        <v>30</v>
+        <v>24</v>
       </c>
       <c r="F149" s="9" t="s">
         <v>28</v>
@@ -5401,7 +5401,7 @@
         <v>27</v>
       </c>
       <c r="E150" s="11">
-        <v>9</v>
+        <v>18</v>
       </c>
       <c r="F150" s="9" t="s">
         <v>28</v>
@@ -5424,7 +5424,7 @@
         <v>27</v>
       </c>
       <c r="E151" s="11">
-        <v>27</v>
+        <v>17</v>
       </c>
       <c r="F151" s="9" t="s">
         <v>28</v>
@@ -5447,7 +5447,7 @@
         <v>27</v>
       </c>
       <c r="E152" s="11">
-        <v>16</v>
+        <v>22</v>
       </c>
       <c r="F152" s="9" t="s">
         <v>28</v>
@@ -5470,7 +5470,7 @@
         <v>27</v>
       </c>
       <c r="E153" s="11">
-        <v>29</v>
+        <v>15</v>
       </c>
       <c r="F153" s="9" t="s">
         <v>28</v>
@@ -5493,7 +5493,7 @@
         <v>27</v>
       </c>
       <c r="E154" s="11">
-        <v>26</v>
+        <v>23</v>
       </c>
       <c r="F154" s="9" t="s">
         <v>28</v>
@@ -5516,7 +5516,7 @@
         <v>27</v>
       </c>
       <c r="E155" s="11">
-        <v>20</v>
+        <v>11</v>
       </c>
       <c r="F155" s="9" t="s">
         <v>28</v>
@@ -5539,7 +5539,7 @@
         <v>27</v>
       </c>
       <c r="E156" s="11">
-        <v>23</v>
+        <v>28</v>
       </c>
       <c r="F156" s="9" t="s">
         <v>28</v>
@@ -5562,7 +5562,7 @@
         <v>27</v>
       </c>
       <c r="E157" s="11">
-        <v>17</v>
+        <v>26</v>
       </c>
       <c r="F157" s="9" t="s">
         <v>28</v>
@@ -5585,7 +5585,7 @@
         <v>27</v>
       </c>
       <c r="E158" s="11">
-        <v>21</v>
+        <v>31</v>
       </c>
       <c r="F158" s="9" t="s">
         <v>28</v>
@@ -5608,7 +5608,7 @@
         <v>27</v>
       </c>
       <c r="E159" s="11">
-        <v>21</v>
+        <v>12</v>
       </c>
       <c r="F159" s="9" t="s">
         <v>28</v>
@@ -5631,7 +5631,7 @@
         <v>27</v>
       </c>
       <c r="E160" s="11">
-        <v>8</v>
+        <v>30</v>
       </c>
       <c r="F160" s="9" t="s">
         <v>28</v>
@@ -5654,7 +5654,7 @@
         <v>27</v>
       </c>
       <c r="E161" s="11">
-        <v>21</v>
+        <v>28</v>
       </c>
       <c r="F161" s="9" t="s">
         <v>28</v>
@@ -5677,7 +5677,7 @@
         <v>27</v>
       </c>
       <c r="E162" s="11">
-        <v>20</v>
+        <v>9</v>
       </c>
       <c r="F162" s="9" t="s">
         <v>28</v>
@@ -5700,7 +5700,7 @@
         <v>27</v>
       </c>
       <c r="E163" s="11">
-        <v>23</v>
+        <v>13</v>
       </c>
       <c r="F163" s="9" t="s">
         <v>28</v>
@@ -5723,7 +5723,7 @@
         <v>27</v>
       </c>
       <c r="E164" s="11">
-        <v>30</v>
+        <v>27</v>
       </c>
       <c r="F164" s="9" t="s">
         <v>28</v>
@@ -5746,7 +5746,7 @@
         <v>27</v>
       </c>
       <c r="E165" s="11">
-        <v>28</v>
+        <v>10</v>
       </c>
       <c r="F165" s="9" t="s">
         <v>28</v>
@@ -5769,7 +5769,7 @@
         <v>27</v>
       </c>
       <c r="E166" s="11">
-        <v>17</v>
+        <v>21</v>
       </c>
       <c r="F166" s="9" t="s">
         <v>28</v>
@@ -5792,7 +5792,7 @@
         <v>27</v>
       </c>
       <c r="E167" s="11">
-        <v>24</v>
+        <v>20</v>
       </c>
       <c r="F167" s="9" t="s">
         <v>28</v>
@@ -5838,7 +5838,7 @@
         <v>27</v>
       </c>
       <c r="E169" s="11">
-        <v>28</v>
+        <v>15</v>
       </c>
       <c r="F169" s="9" t="s">
         <v>28</v>
@@ -5861,7 +5861,7 @@
         <v>27</v>
       </c>
       <c r="E170" s="11">
-        <v>12</v>
+        <v>8</v>
       </c>
       <c r="F170" s="9" t="s">
         <v>28</v>
@@ -5884,7 +5884,7 @@
         <v>27</v>
       </c>
       <c r="E171" s="11">
-        <v>15</v>
+        <v>21</v>
       </c>
       <c r="F171" s="9" t="s">
         <v>28</v>
@@ -5907,7 +5907,7 @@
         <v>27</v>
       </c>
       <c r="E172" s="11">
-        <v>19</v>
+        <v>24</v>
       </c>
       <c r="F172" s="9" t="s">
         <v>28</v>
@@ -5953,7 +5953,7 @@
         <v>27</v>
       </c>
       <c r="E174" s="11">
-        <v>19</v>
+        <v>10</v>
       </c>
       <c r="F174" s="9" t="s">
         <v>28</v>
@@ -5976,7 +5976,7 @@
         <v>27</v>
       </c>
       <c r="E175" s="11">
-        <v>31</v>
+        <v>21</v>
       </c>
       <c r="F175" s="9" t="s">
         <v>28</v>
@@ -5999,7 +5999,7 @@
         <v>27</v>
       </c>
       <c r="E176" s="11">
-        <v>25</v>
+        <v>11</v>
       </c>
       <c r="F176" s="9" t="s">
         <v>28</v>
@@ -6022,7 +6022,7 @@
         <v>27</v>
       </c>
       <c r="E177" s="11">
-        <v>21</v>
+        <v>17</v>
       </c>
       <c r="F177" s="9" t="s">
         <v>28</v>
@@ -6045,7 +6045,7 @@
         <v>27</v>
       </c>
       <c r="E178" s="11">
-        <v>13</v>
+        <v>27</v>
       </c>
       <c r="F178" s="9" t="s">
         <v>28</v>
@@ -6068,7 +6068,7 @@
         <v>27</v>
       </c>
       <c r="E179" s="11">
-        <v>20</v>
+        <v>24</v>
       </c>
       <c r="F179" s="9" t="s">
         <v>28</v>
@@ -6091,7 +6091,7 @@
         <v>27</v>
       </c>
       <c r="E180" s="11">
-        <v>10</v>
+        <v>23</v>
       </c>
       <c r="F180" s="9" t="s">
         <v>28</v>
@@ -6114,7 +6114,7 @@
         <v>27</v>
       </c>
       <c r="E181" s="11">
-        <v>12</v>
+        <v>8</v>
       </c>
       <c r="F181" s="9" t="s">
         <v>28</v>
@@ -6137,7 +6137,7 @@
         <v>27</v>
       </c>
       <c r="E182" s="11">
-        <v>23</v>
+        <v>10</v>
       </c>
       <c r="F182" s="9" t="s">
         <v>28</v>
@@ -6160,7 +6160,7 @@
         <v>27</v>
       </c>
       <c r="E183" s="11">
-        <v>9</v>
+        <v>21</v>
       </c>
       <c r="F183" s="9" t="s">
         <v>28</v>
@@ -6183,7 +6183,7 @@
         <v>27</v>
       </c>
       <c r="E184" s="11">
-        <v>24</v>
+        <v>30</v>
       </c>
       <c r="F184" s="9" t="s">
         <v>28</v>
@@ -6206,7 +6206,7 @@
         <v>27</v>
       </c>
       <c r="E185" s="11">
-        <v>19</v>
+        <v>28</v>
       </c>
       <c r="F185" s="9" t="s">
         <v>28</v>
@@ -6229,7 +6229,7 @@
         <v>27</v>
       </c>
       <c r="E186" s="11">
-        <v>11</v>
+        <v>14</v>
       </c>
       <c r="F186" s="9" t="s">
         <v>28</v>
@@ -6252,7 +6252,7 @@
         <v>27</v>
       </c>
       <c r="E187" s="11">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="F187" s="9" t="s">
         <v>28</v>
@@ -6275,7 +6275,7 @@
         <v>27</v>
       </c>
       <c r="E188" s="11">
-        <v>22</v>
+        <v>27</v>
       </c>
       <c r="F188" s="9" t="s">
         <v>28</v>
@@ -6298,7 +6298,7 @@
         <v>27</v>
       </c>
       <c r="E189" s="11">
-        <v>29</v>
+        <v>21</v>
       </c>
       <c r="F189" s="9" t="s">
         <v>28</v>
@@ -6321,7 +6321,7 @@
         <v>27</v>
       </c>
       <c r="E190" s="11">
-        <v>12</v>
+        <v>16</v>
       </c>
       <c r="F190" s="9" t="s">
         <v>28</v>
@@ -6344,7 +6344,7 @@
         <v>27</v>
       </c>
       <c r="E191" s="11">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="F191" s="9" t="s">
         <v>28</v>
@@ -6367,7 +6367,7 @@
         <v>27</v>
       </c>
       <c r="E192" s="11">
-        <v>26</v>
+        <v>17</v>
       </c>
       <c r="F192" s="9" t="s">
         <v>28</v>
@@ -6390,7 +6390,7 @@
         <v>27</v>
       </c>
       <c r="E193" s="11">
-        <v>21</v>
+        <v>9</v>
       </c>
       <c r="F193" s="9" t="s">
         <v>28</v>
@@ -6413,7 +6413,7 @@
         <v>27</v>
       </c>
       <c r="E194" s="11">
-        <v>13</v>
+        <v>8</v>
       </c>
       <c r="F194" s="9" t="s">
         <v>28</v>
@@ -6436,7 +6436,7 @@
         <v>27</v>
       </c>
       <c r="E195" s="11">
-        <v>13</v>
+        <v>17</v>
       </c>
       <c r="F195" s="9" t="s">
         <v>28</v>
@@ -6459,7 +6459,7 @@
         <v>27</v>
       </c>
       <c r="E196" s="11">
-        <v>10</v>
+        <v>22</v>
       </c>
       <c r="F196" s="9" t="s">
         <v>28</v>
@@ -6482,7 +6482,7 @@
         <v>27</v>
       </c>
       <c r="E197" s="11">
-        <v>28</v>
+        <v>15</v>
       </c>
       <c r="F197" s="9" t="s">
         <v>28</v>
@@ -6505,7 +6505,7 @@
         <v>27</v>
       </c>
       <c r="E198" s="11">
-        <v>24</v>
+        <v>20</v>
       </c>
       <c r="F198" s="9" t="s">
         <v>28</v>
@@ -6528,7 +6528,7 @@
         <v>27</v>
       </c>
       <c r="E199" s="11">
-        <v>22</v>
+        <v>18</v>
       </c>
       <c r="F199" s="9" t="s">
         <v>28</v>
@@ -6551,7 +6551,7 @@
         <v>27</v>
       </c>
       <c r="E200" s="11">
-        <v>29</v>
+        <v>13</v>
       </c>
       <c r="F200" s="9" t="s">
         <v>28</v>
@@ -6620,7 +6620,7 @@
         <v>27</v>
       </c>
       <c r="E203" s="11">
-        <v>31</v>
+        <v>29</v>
       </c>
       <c r="F203" s="9" t="s">
         <v>28</v>
@@ -6643,7 +6643,7 @@
         <v>27</v>
       </c>
       <c r="E204" s="11">
-        <v>30</v>
+        <v>17</v>
       </c>
       <c r="F204" s="9" t="s">
         <v>28</v>
@@ -6666,7 +6666,7 @@
         <v>27</v>
       </c>
       <c r="E205" s="11">
-        <v>16</v>
+        <v>8</v>
       </c>
       <c r="F205" s="9" t="s">
         <v>28</v>
@@ -6689,7 +6689,7 @@
         <v>27</v>
       </c>
       <c r="E206" s="11">
-        <v>14</v>
+        <v>18</v>
       </c>
       <c r="F206" s="9" t="s">
         <v>28</v>
@@ -6712,7 +6712,7 @@
         <v>27</v>
       </c>
       <c r="E207" s="11">
-        <v>19</v>
+        <v>29</v>
       </c>
       <c r="F207" s="9" t="s">
         <v>28</v>
@@ -6735,7 +6735,7 @@
         <v>27</v>
       </c>
       <c r="E208" s="11">
-        <v>17</v>
+        <v>12</v>
       </c>
       <c r="F208" s="9" t="s">
         <v>28</v>
@@ -6758,7 +6758,7 @@
         <v>27</v>
       </c>
       <c r="E209" s="11">
-        <v>9</v>
+        <v>13</v>
       </c>
       <c r="F209" s="9" t="s">
         <v>28</v>
@@ -6781,7 +6781,7 @@
         <v>27</v>
       </c>
       <c r="E210" s="11">
-        <v>18</v>
+        <v>12</v>
       </c>
       <c r="F210" s="9" t="s">
         <v>28</v>
@@ -6804,7 +6804,7 @@
         <v>27</v>
       </c>
       <c r="E211" s="11">
-        <v>11</v>
+        <v>17</v>
       </c>
       <c r="F211" s="9" t="s">
         <v>28</v>
@@ -6827,7 +6827,7 @@
         <v>27</v>
       </c>
       <c r="E212" s="11">
-        <v>24</v>
+        <v>12</v>
       </c>
       <c r="F212" s="9" t="s">
         <v>28</v>
@@ -6850,7 +6850,7 @@
         <v>27</v>
       </c>
       <c r="E213" s="11">
-        <v>17</v>
+        <v>27</v>
       </c>
       <c r="F213" s="9" t="s">
         <v>28</v>
@@ -6873,7 +6873,7 @@
         <v>27</v>
       </c>
       <c r="E214" s="11">
-        <v>17</v>
+        <v>26</v>
       </c>
       <c r="F214" s="9" t="s">
         <v>28</v>
@@ -6896,7 +6896,7 @@
         <v>27</v>
       </c>
       <c r="E215" s="11">
-        <v>20</v>
+        <v>28</v>
       </c>
       <c r="F215" s="9" t="s">
         <v>28</v>
@@ -6919,7 +6919,7 @@
         <v>27</v>
       </c>
       <c r="E216" s="11">
-        <v>10</v>
+        <v>31</v>
       </c>
       <c r="F216" s="9" t="s">
         <v>28</v>
@@ -6942,7 +6942,7 @@
         <v>27</v>
       </c>
       <c r="E217" s="11">
-        <v>29</v>
+        <v>18</v>
       </c>
       <c r="F217" s="9" t="s">
         <v>28</v>
@@ -6965,7 +6965,7 @@
         <v>27</v>
       </c>
       <c r="E218" s="11">
-        <v>25</v>
+        <v>8</v>
       </c>
       <c r="F218" s="9" t="s">
         <v>28</v>
@@ -6988,7 +6988,7 @@
         <v>27</v>
       </c>
       <c r="E219" s="11">
-        <v>8</v>
+        <v>31</v>
       </c>
       <c r="F219" s="9" t="s">
         <v>28</v>
@@ -7011,7 +7011,7 @@
         <v>27</v>
       </c>
       <c r="E220" s="11">
-        <v>11</v>
+        <v>17</v>
       </c>
       <c r="F220" s="9" t="s">
         <v>28</v>
@@ -7034,7 +7034,7 @@
         <v>27</v>
       </c>
       <c r="E221" s="11">
-        <v>28</v>
+        <v>25</v>
       </c>
       <c r="F221" s="9" t="s">
         <v>28</v>
@@ -7057,7 +7057,7 @@
         <v>27</v>
       </c>
       <c r="E222" s="11">
-        <v>27</v>
+        <v>16</v>
       </c>
       <c r="F222" s="9" t="s">
         <v>28</v>
@@ -7080,7 +7080,7 @@
         <v>27</v>
       </c>
       <c r="E223" s="11">
-        <v>31</v>
+        <v>9</v>
       </c>
       <c r="F223" s="9" t="s">
         <v>28</v>
@@ -7103,7 +7103,7 @@
         <v>27</v>
       </c>
       <c r="E224" s="11">
-        <v>13</v>
+        <v>16</v>
       </c>
       <c r="F224" s="9" t="s">
         <v>28</v>
@@ -7126,7 +7126,7 @@
         <v>27</v>
       </c>
       <c r="E225" s="11">
-        <v>9</v>
+        <v>21</v>
       </c>
       <c r="F225" s="9" t="s">
         <v>28</v>
@@ -7149,7 +7149,7 @@
         <v>27</v>
       </c>
       <c r="E226" s="11">
-        <v>14</v>
+        <v>11</v>
       </c>
       <c r="F226" s="9" t="s">
         <v>28</v>
@@ -7172,7 +7172,7 @@
         <v>27</v>
       </c>
       <c r="E227" s="11">
-        <v>16</v>
+        <v>18</v>
       </c>
       <c r="F227" s="9" t="s">
         <v>28</v>
@@ -7195,7 +7195,7 @@
         <v>27</v>
       </c>
       <c r="E228" s="11">
-        <v>8</v>
+        <v>28</v>
       </c>
       <c r="F228" s="9" t="s">
         <v>28</v>
@@ -7218,7 +7218,7 @@
         <v>27</v>
       </c>
       <c r="E229" s="11">
-        <v>31</v>
+        <v>8</v>
       </c>
       <c r="F229" s="9" t="s">
         <v>28</v>
@@ -7241,7 +7241,7 @@
         <v>27</v>
       </c>
       <c r="E230" s="11">
-        <v>31</v>
+        <v>21</v>
       </c>
       <c r="F230" s="9" t="s">
         <v>28</v>
@@ -7264,7 +7264,7 @@
         <v>27</v>
       </c>
       <c r="E231" s="11">
-        <v>28</v>
+        <v>31</v>
       </c>
       <c r="F231" s="9" t="s">
         <v>28</v>
@@ -7287,7 +7287,7 @@
         <v>27</v>
       </c>
       <c r="E232" s="11">
-        <v>12</v>
+        <v>16</v>
       </c>
       <c r="F232" s="9" t="s">
         <v>28</v>
@@ -7310,7 +7310,7 @@
         <v>27</v>
       </c>
       <c r="E233" s="11">
-        <v>13</v>
+        <v>24</v>
       </c>
       <c r="F233" s="9" t="s">
         <v>28</v>
@@ -7333,7 +7333,7 @@
         <v>27</v>
       </c>
       <c r="E234" s="11">
-        <v>25</v>
+        <v>21</v>
       </c>
       <c r="F234" s="9" t="s">
         <v>28</v>
@@ -7379,7 +7379,7 @@
         <v>27</v>
       </c>
       <c r="E236" s="11">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="F236" s="9" t="s">
         <v>28</v>
@@ -7402,7 +7402,7 @@
         <v>27</v>
       </c>
       <c r="E237" s="11">
-        <v>15</v>
+        <v>26</v>
       </c>
       <c r="F237" s="9" t="s">
         <v>28</v>
@@ -7425,7 +7425,7 @@
         <v>27</v>
       </c>
       <c r="E238" s="11">
-        <v>29</v>
+        <v>16</v>
       </c>
       <c r="F238" s="9" t="s">
         <v>28</v>
@@ -7448,7 +7448,7 @@
         <v>27</v>
       </c>
       <c r="E239" s="11">
-        <v>30</v>
+        <v>26</v>
       </c>
       <c r="F239" s="9" t="s">
         <v>28</v>
@@ -7471,7 +7471,7 @@
         <v>27</v>
       </c>
       <c r="E240" s="11">
-        <v>13</v>
+        <v>26</v>
       </c>
       <c r="F240" s="9" t="s">
         <v>28</v>
@@ -7494,7 +7494,7 @@
         <v>27</v>
       </c>
       <c r="E241" s="11">
-        <v>28</v>
+        <v>21</v>
       </c>
       <c r="F241" s="9" t="s">
         <v>28</v>
@@ -7517,7 +7517,7 @@
         <v>27</v>
       </c>
       <c r="E242" s="11">
-        <v>11</v>
+        <v>17</v>
       </c>
       <c r="F242" s="9" t="s">
         <v>28</v>
@@ -7540,7 +7540,7 @@
         <v>27</v>
       </c>
       <c r="E243" s="11">
-        <v>15</v>
+        <v>8</v>
       </c>
       <c r="F243" s="9" t="s">
         <v>28</v>
@@ -7563,7 +7563,7 @@
         <v>27</v>
       </c>
       <c r="E244" s="11">
-        <v>29</v>
+        <v>17</v>
       </c>
       <c r="F244" s="9" t="s">
         <v>28</v>
@@ -7586,7 +7586,7 @@
         <v>27</v>
       </c>
       <c r="E245" s="11">
-        <v>23</v>
+        <v>21</v>
       </c>
       <c r="F245" s="9" t="s">
         <v>28</v>
@@ -7609,7 +7609,7 @@
         <v>27</v>
       </c>
       <c r="E246" s="11">
-        <v>24</v>
+        <v>18</v>
       </c>
       <c r="F246" s="9" t="s">
         <v>28</v>
@@ -7632,7 +7632,7 @@
         <v>27</v>
       </c>
       <c r="E247" s="11">
-        <v>10</v>
+        <v>27</v>
       </c>
       <c r="F247" s="9" t="s">
         <v>28</v>
@@ -7655,7 +7655,7 @@
         <v>27</v>
       </c>
       <c r="E248" s="11">
-        <v>12</v>
+        <v>31</v>
       </c>
       <c r="F248" s="9" t="s">
         <v>28</v>
@@ -7678,7 +7678,7 @@
         <v>27</v>
       </c>
       <c r="E249" s="11">
-        <v>21</v>
+        <v>23</v>
       </c>
       <c r="F249" s="9" t="s">
         <v>28</v>
@@ -7701,7 +7701,7 @@
         <v>27</v>
       </c>
       <c r="E250" s="11">
-        <v>12</v>
+        <v>22</v>
       </c>
       <c r="F250" s="9" t="s">
         <v>28</v>
@@ -7724,7 +7724,7 @@
         <v>27</v>
       </c>
       <c r="E251" s="11">
-        <v>17</v>
+        <v>25</v>
       </c>
       <c r="F251" s="9" t="s">
         <v>28</v>
@@ -7770,7 +7770,7 @@
         <v>27</v>
       </c>
       <c r="E253" s="11">
-        <v>26</v>
+        <v>19</v>
       </c>
       <c r="F253" s="9" t="s">
         <v>28</v>
@@ -7793,7 +7793,7 @@
         <v>27</v>
       </c>
       <c r="E254" s="11">
-        <v>16</v>
+        <v>23</v>
       </c>
       <c r="F254" s="9" t="s">
         <v>28</v>
@@ -7816,7 +7816,7 @@
         <v>27</v>
       </c>
       <c r="E255" s="11">
-        <v>14</v>
+        <v>31</v>
       </c>
       <c r="F255" s="9" t="s">
         <v>28</v>
@@ -7839,7 +7839,7 @@
         <v>27</v>
       </c>
       <c r="E256" s="11">
-        <v>12</v>
+        <v>19</v>
       </c>
       <c r="F256" s="9" t="s">
         <v>28</v>
@@ -7862,7 +7862,7 @@
         <v>27</v>
       </c>
       <c r="E257" s="11">
-        <v>12</v>
+        <v>8</v>
       </c>
       <c r="F257" s="9" t="s">
         <v>28</v>
@@ -7885,7 +7885,7 @@
         <v>27</v>
       </c>
       <c r="E258" s="11">
-        <v>10</v>
+        <v>15</v>
       </c>
       <c r="F258" s="9" t="s">
         <v>28</v>
@@ -7908,7 +7908,7 @@
         <v>27</v>
       </c>
       <c r="E259" s="11">
-        <v>16</v>
+        <v>24</v>
       </c>
       <c r="F259" s="9" t="s">
         <v>28</v>
@@ -7954,7 +7954,7 @@
         <v>27</v>
       </c>
       <c r="E261" s="11">
-        <v>31</v>
+        <v>8</v>
       </c>
       <c r="F261" s="9" t="s">
         <v>28</v>
@@ -7977,7 +7977,7 @@
         <v>27</v>
       </c>
       <c r="E262" s="11">
-        <v>23</v>
+        <v>9</v>
       </c>
       <c r="F262" s="9" t="s">
         <v>28</v>
@@ -8000,7 +8000,7 @@
         <v>27</v>
       </c>
       <c r="E263" s="11">
-        <v>25</v>
+        <v>11</v>
       </c>
       <c r="F263" s="9" t="s">
         <v>28</v>
@@ -8023,7 +8023,7 @@
         <v>27</v>
       </c>
       <c r="E264" s="11">
-        <v>20</v>
+        <v>31</v>
       </c>
       <c r="F264" s="9" t="s">
         <v>28</v>
@@ -8046,7 +8046,7 @@
         <v>27</v>
       </c>
       <c r="E265" s="11">
-        <v>21</v>
+        <v>12</v>
       </c>
       <c r="F265" s="9" t="s">
         <v>28</v>
@@ -8069,7 +8069,7 @@
         <v>27</v>
       </c>
       <c r="E266" s="11">
-        <v>29</v>
+        <v>25</v>
       </c>
       <c r="F266" s="9" t="s">
         <v>28</v>
@@ -8092,7 +8092,7 @@
         <v>27</v>
       </c>
       <c r="E267" s="11">
-        <v>12</v>
+        <v>19</v>
       </c>
       <c r="F267" s="9" t="s">
         <v>28</v>
@@ -8115,7 +8115,7 @@
         <v>27</v>
       </c>
       <c r="E268" s="11">
-        <v>31</v>
+        <v>18</v>
       </c>
       <c r="F268" s="9" t="s">
         <v>28</v>
@@ -8138,7 +8138,7 @@
         <v>27</v>
       </c>
       <c r="E269" s="11">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="F269" s="9" t="s">
         <v>28</v>
@@ -8161,7 +8161,7 @@
         <v>27</v>
       </c>
       <c r="E270" s="11">
-        <v>16</v>
+        <v>23</v>
       </c>
       <c r="F270" s="9" t="s">
         <v>28</v>
@@ -8184,7 +8184,7 @@
         <v>27</v>
       </c>
       <c r="E271" s="11">
-        <v>28</v>
+        <v>10</v>
       </c>
       <c r="F271" s="9" t="s">
         <v>28</v>
@@ -8207,7 +8207,7 @@
         <v>27</v>
       </c>
       <c r="E272" s="11">
-        <v>22</v>
+        <v>25</v>
       </c>
       <c r="F272" s="9" t="s">
         <v>28</v>
@@ -8230,7 +8230,7 @@
         <v>27</v>
       </c>
       <c r="E273" s="11">
-        <v>22</v>
+        <v>25</v>
       </c>
       <c r="F273" s="9" t="s">
         <v>28</v>
@@ -8253,7 +8253,7 @@
         <v>27</v>
       </c>
       <c r="E274" s="11">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="F274" s="9" t="s">
         <v>28</v>
@@ -8276,7 +8276,7 @@
         <v>27</v>
       </c>
       <c r="E275" s="11">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="F275" s="9" t="s">
         <v>28</v>
@@ -8299,7 +8299,7 @@
         <v>27</v>
       </c>
       <c r="E276" s="11">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="F276" s="9" t="s">
         <v>28</v>
@@ -8322,7 +8322,7 @@
         <v>27</v>
       </c>
       <c r="E277" s="11">
-        <v>27</v>
+        <v>10</v>
       </c>
       <c r="F277" s="9" t="s">
         <v>28</v>
@@ -8345,7 +8345,7 @@
         <v>27</v>
       </c>
       <c r="E278" s="11">
-        <v>22</v>
+        <v>17</v>
       </c>
       <c r="F278" s="9" t="s">
         <v>28</v>
@@ -8368,7 +8368,7 @@
         <v>27</v>
       </c>
       <c r="E279" s="11">
-        <v>12</v>
+        <v>18</v>
       </c>
       <c r="F279" s="9" t="s">
         <v>28</v>
@@ -8391,7 +8391,7 @@
         <v>27</v>
       </c>
       <c r="E280" s="11">
-        <v>14</v>
+        <v>18</v>
       </c>
       <c r="F280" s="9" t="s">
         <v>28</v>
@@ -8414,7 +8414,7 @@
         <v>27</v>
       </c>
       <c r="E281" s="11">
-        <v>19</v>
+        <v>17</v>
       </c>
       <c r="F281" s="9" t="s">
         <v>28</v>
@@ -8437,7 +8437,7 @@
         <v>27</v>
       </c>
       <c r="E282" s="11">
-        <v>28</v>
+        <v>15</v>
       </c>
       <c r="F282" s="9" t="s">
         <v>28</v>
@@ -8460,7 +8460,7 @@
         <v>27</v>
       </c>
       <c r="E283" s="11">
-        <v>20</v>
+        <v>24</v>
       </c>
       <c r="F283" s="9" t="s">
         <v>28</v>
@@ -8483,7 +8483,7 @@
         <v>27</v>
       </c>
       <c r="E284" s="11">
-        <v>24</v>
+        <v>17</v>
       </c>
       <c r="F284" s="9" t="s">
         <v>28</v>
@@ -8506,7 +8506,7 @@
         <v>27</v>
       </c>
       <c r="E285" s="11">
-        <v>11</v>
+        <v>17</v>
       </c>
       <c r="F285" s="9" t="s">
         <v>28</v>
@@ -8529,7 +8529,7 @@
         <v>27</v>
       </c>
       <c r="E286" s="11">
-        <v>30</v>
+        <v>24</v>
       </c>
       <c r="F286" s="9" t="s">
         <v>28</v>
@@ -8575,7 +8575,7 @@
         <v>27</v>
       </c>
       <c r="E288" s="11">
-        <v>29</v>
+        <v>18</v>
       </c>
       <c r="F288" s="9" t="s">
         <v>28</v>
@@ -8598,7 +8598,7 @@
         <v>27</v>
       </c>
       <c r="E289" s="11">
-        <v>18</v>
+        <v>23</v>
       </c>
       <c r="F289" s="9" t="s">
         <v>28</v>
@@ -8621,7 +8621,7 @@
         <v>27</v>
       </c>
       <c r="E290" s="11">
-        <v>8</v>
+        <v>22</v>
       </c>
       <c r="F290" s="9" t="s">
         <v>28</v>
@@ -8644,7 +8644,7 @@
         <v>27</v>
       </c>
       <c r="E291" s="11">
-        <v>28</v>
+        <v>31</v>
       </c>
       <c r="F291" s="9" t="s">
         <v>28</v>
@@ -8667,7 +8667,7 @@
         <v>27</v>
       </c>
       <c r="E292" s="11">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="F292" s="9" t="s">
         <v>28</v>
@@ -8690,7 +8690,7 @@
         <v>27</v>
       </c>
       <c r="E293" s="11">
-        <v>27</v>
+        <v>13</v>
       </c>
       <c r="F293" s="9" t="s">
         <v>28</v>
@@ -8713,7 +8713,7 @@
         <v>27</v>
       </c>
       <c r="E294" s="11">
-        <v>23</v>
+        <v>27</v>
       </c>
       <c r="F294" s="9" t="s">
         <v>28</v>
@@ -8736,7 +8736,7 @@
         <v>27</v>
       </c>
       <c r="E295" s="11">
-        <v>13</v>
+        <v>30</v>
       </c>
       <c r="F295" s="9" t="s">
         <v>28</v>
@@ -8759,7 +8759,7 @@
         <v>27</v>
       </c>
       <c r="E296" s="11">
-        <v>16</v>
+        <v>30</v>
       </c>
       <c r="F296" s="9" t="s">
         <v>28</v>
@@ -8782,7 +8782,7 @@
         <v>27</v>
       </c>
       <c r="E297" s="11">
-        <v>16</v>
+        <v>10</v>
       </c>
       <c r="F297" s="9" t="s">
         <v>28</v>
@@ -8805,7 +8805,7 @@
         <v>27</v>
       </c>
       <c r="E298" s="11">
-        <v>24</v>
+        <v>13</v>
       </c>
       <c r="F298" s="9" t="s">
         <v>28</v>
@@ -8828,7 +8828,7 @@
         <v>27</v>
       </c>
       <c r="E299" s="11">
-        <v>25</v>
+        <v>21</v>
       </c>
       <c r="F299" s="9" t="s">
         <v>28</v>
@@ -8851,7 +8851,7 @@
         <v>27</v>
       </c>
       <c r="E300" s="11">
-        <v>21</v>
+        <v>30</v>
       </c>
       <c r="F300" s="9" t="s">
         <v>28</v>
@@ -8874,7 +8874,7 @@
         <v>27</v>
       </c>
       <c r="E301" s="11">
-        <v>15</v>
+        <v>20</v>
       </c>
       <c r="F301" s="9" t="s">
         <v>28</v>
@@ -8897,7 +8897,7 @@
         <v>27</v>
       </c>
       <c r="E302" s="11">
-        <v>16</v>
+        <v>24</v>
       </c>
       <c r="F302" s="9" t="s">
         <v>28</v>
@@ -8920,7 +8920,7 @@
         <v>27</v>
       </c>
       <c r="E303" s="11">
-        <v>22</v>
+        <v>26</v>
       </c>
       <c r="F303" s="9" t="s">
         <v>28</v>
@@ -8943,7 +8943,7 @@
         <v>27</v>
       </c>
       <c r="E304" s="11">
-        <v>18</v>
+        <v>11</v>
       </c>
       <c r="F304" s="9" t="s">
         <v>28</v>
@@ -8966,7 +8966,7 @@
         <v>27</v>
       </c>
       <c r="E305" s="11">
-        <v>30</v>
+        <v>25</v>
       </c>
       <c r="F305" s="9" t="s">
         <v>28</v>
@@ -8989,7 +8989,7 @@
         <v>27</v>
       </c>
       <c r="E306" s="11">
-        <v>24</v>
+        <v>17</v>
       </c>
       <c r="F306" s="9" t="s">
         <v>28</v>
@@ -9012,7 +9012,7 @@
         <v>27</v>
       </c>
       <c r="E307" s="11">
-        <v>11</v>
+        <v>18</v>
       </c>
       <c r="F307" s="9" t="s">
         <v>28</v>
@@ -9035,7 +9035,7 @@
         <v>27</v>
       </c>
       <c r="E308" s="11">
-        <v>10</v>
+        <v>23</v>
       </c>
       <c r="F308" s="9" t="s">
         <v>28</v>
@@ -9058,7 +9058,7 @@
         <v>27</v>
       </c>
       <c r="E309" s="11">
-        <v>14</v>
+        <v>20</v>
       </c>
       <c r="F309" s="9" t="s">
         <v>28</v>
@@ -9081,7 +9081,7 @@
         <v>27</v>
       </c>
       <c r="E310" s="11">
-        <v>24</v>
+        <v>11</v>
       </c>
       <c r="F310" s="9" t="s">
         <v>28</v>
@@ -9104,7 +9104,7 @@
         <v>27</v>
       </c>
       <c r="E311" s="11">
-        <v>13</v>
+        <v>17</v>
       </c>
       <c r="F311" s="9" t="s">
         <v>28</v>
@@ -9127,7 +9127,7 @@
         <v>27</v>
       </c>
       <c r="E312" s="11">
-        <v>24</v>
+        <v>16</v>
       </c>
       <c r="F312" s="9" t="s">
         <v>28</v>
@@ -9150,7 +9150,7 @@
         <v>27</v>
       </c>
       <c r="E313" s="11">
-        <v>27</v>
+        <v>15</v>
       </c>
       <c r="F313" s="9" t="s">
         <v>28</v>
@@ -9173,7 +9173,7 @@
         <v>27</v>
       </c>
       <c r="E314" s="11">
-        <v>8</v>
+        <v>19</v>
       </c>
       <c r="F314" s="9" t="s">
         <v>28</v>
@@ -9196,7 +9196,7 @@
         <v>27</v>
       </c>
       <c r="E315" s="11">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="F315" s="9" t="s">
         <v>28</v>
@@ -9219,7 +9219,7 @@
         <v>27</v>
       </c>
       <c r="E316" s="11">
-        <v>8</v>
+        <v>21</v>
       </c>
       <c r="F316" s="9" t="s">
         <v>28</v>
@@ -9242,7 +9242,7 @@
         <v>27</v>
       </c>
       <c r="E317" s="11">
-        <v>17</v>
+        <v>31</v>
       </c>
       <c r="F317" s="9" t="s">
         <v>28</v>
@@ -9265,7 +9265,7 @@
         <v>27</v>
       </c>
       <c r="E318" s="11">
-        <v>12</v>
+        <v>28</v>
       </c>
       <c r="F318" s="9" t="s">
         <v>28</v>
@@ -9288,7 +9288,7 @@
         <v>27</v>
       </c>
       <c r="E319" s="11">
-        <v>26</v>
+        <v>20</v>
       </c>
       <c r="F319" s="9" t="s">
         <v>28</v>
@@ -9311,7 +9311,7 @@
         <v>27</v>
       </c>
       <c r="E320" s="11">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="F320" s="9" t="s">
         <v>28</v>
@@ -9334,7 +9334,7 @@
         <v>27</v>
       </c>
       <c r="E321" s="11">
-        <v>28</v>
+        <v>11</v>
       </c>
       <c r="F321" s="9" t="s">
         <v>28</v>
@@ -9357,7 +9357,7 @@
         <v>27</v>
       </c>
       <c r="E322" s="11">
-        <v>12</v>
+        <v>22</v>
       </c>
       <c r="F322" s="9" t="s">
         <v>28</v>
@@ -9380,7 +9380,7 @@
         <v>27</v>
       </c>
       <c r="E323" s="11">
-        <v>9</v>
+        <v>18</v>
       </c>
       <c r="F323" s="9" t="s">
         <v>28</v>
@@ -9403,7 +9403,7 @@
         <v>27</v>
       </c>
       <c r="E324" s="11">
-        <v>8</v>
+        <v>21</v>
       </c>
       <c r="F324" s="9" t="s">
         <v>28</v>
@@ -9426,7 +9426,7 @@
         <v>27</v>
       </c>
       <c r="E325" s="11">
-        <v>18</v>
+        <v>12</v>
       </c>
       <c r="F325" s="9" t="s">
         <v>28</v>
@@ -9472,7 +9472,7 @@
         <v>27</v>
       </c>
       <c r="E327" s="11">
-        <v>30</v>
+        <v>28</v>
       </c>
       <c r="F327" s="9" t="s">
         <v>28</v>
@@ -9495,7 +9495,7 @@
         <v>27</v>
       </c>
       <c r="E328" s="11">
-        <v>29</v>
+        <v>8</v>
       </c>
       <c r="F328" s="9" t="s">
         <v>28</v>
@@ -9518,7 +9518,7 @@
         <v>27</v>
       </c>
       <c r="E329" s="11">
-        <v>13</v>
+        <v>30</v>
       </c>
       <c r="F329" s="9" t="s">
         <v>28</v>
@@ -9541,7 +9541,7 @@
         <v>27</v>
       </c>
       <c r="E330" s="11">
-        <v>16</v>
+        <v>10</v>
       </c>
       <c r="F330" s="9" t="s">
         <v>28</v>
@@ -9564,7 +9564,7 @@
         <v>27</v>
       </c>
       <c r="E331" s="11">
-        <v>24</v>
+        <v>29</v>
       </c>
       <c r="F331" s="9" t="s">
         <v>28</v>
@@ -9587,7 +9587,7 @@
         <v>27</v>
       </c>
       <c r="E332" s="11">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="F332" s="9" t="s">
         <v>28</v>
@@ -9610,7 +9610,7 @@
         <v>27</v>
       </c>
       <c r="E333" s="11">
-        <v>23</v>
+        <v>15</v>
       </c>
       <c r="F333" s="9" t="s">
         <v>28</v>
@@ -9633,7 +9633,7 @@
         <v>27</v>
       </c>
       <c r="E334" s="11">
-        <v>16</v>
+        <v>13</v>
       </c>
       <c r="F334" s="9" t="s">
         <v>28</v>
@@ -9656,7 +9656,7 @@
         <v>27</v>
       </c>
       <c r="E335" s="11">
-        <v>13</v>
+        <v>8</v>
       </c>
       <c r="F335" s="9" t="s">
         <v>28</v>
@@ -9679,7 +9679,7 @@
         <v>27</v>
       </c>
       <c r="E336" s="11">
-        <v>18</v>
+        <v>27</v>
       </c>
       <c r="F336" s="9" t="s">
         <v>28</v>
@@ -9702,7 +9702,7 @@
         <v>27</v>
       </c>
       <c r="E337" s="11">
-        <v>26</v>
+        <v>28</v>
       </c>
       <c r="F337" s="9" t="s">
         <v>28</v>
@@ -9725,7 +9725,7 @@
         <v>27</v>
       </c>
       <c r="E338" s="11">
-        <v>18</v>
+        <v>22</v>
       </c>
       <c r="F338" s="9" t="s">
         <v>28</v>
@@ -9748,7 +9748,7 @@
         <v>27</v>
       </c>
       <c r="E339" s="11">
-        <v>9</v>
+        <v>24</v>
       </c>
       <c r="F339" s="9" t="s">
         <v>28</v>
@@ -9771,7 +9771,7 @@
         <v>27</v>
       </c>
       <c r="E340" s="11">
-        <v>26</v>
+        <v>22</v>
       </c>
       <c r="F340" s="9" t="s">
         <v>28</v>
@@ -9794,7 +9794,7 @@
         <v>27</v>
       </c>
       <c r="E341" s="11">
-        <v>12</v>
+        <v>19</v>
       </c>
       <c r="F341" s="9" t="s">
         <v>28</v>
@@ -9817,7 +9817,7 @@
         <v>27</v>
       </c>
       <c r="E342" s="11">
-        <v>28</v>
+        <v>21</v>
       </c>
       <c r="F342" s="9" t="s">
         <v>28</v>
@@ -9840,7 +9840,7 @@
         <v>27</v>
       </c>
       <c r="E343" s="11">
-        <v>13</v>
+        <v>15</v>
       </c>
       <c r="F343" s="9" t="s">
         <v>28</v>
@@ -9863,7 +9863,7 @@
         <v>27</v>
       </c>
       <c r="E344" s="11">
-        <v>12</v>
+        <v>24</v>
       </c>
       <c r="F344" s="9" t="s">
         <v>28</v>
@@ -9886,7 +9886,7 @@
         <v>27</v>
       </c>
       <c r="E345" s="11">
-        <v>10</v>
+        <v>15</v>
       </c>
       <c r="F345" s="9" t="s">
         <v>28</v>
@@ -9909,7 +9909,7 @@
         <v>27</v>
       </c>
       <c r="E346" s="11">
-        <v>10</v>
+        <v>24</v>
       </c>
       <c r="F346" s="9" t="s">
         <v>28</v>
@@ -9932,7 +9932,7 @@
         <v>27</v>
       </c>
       <c r="E347" s="11">
-        <v>17</v>
+        <v>19</v>
       </c>
       <c r="F347" s="9" t="s">
         <v>28</v>
@@ -9955,7 +9955,7 @@
         <v>27</v>
       </c>
       <c r="E348" s="11">
-        <v>25</v>
+        <v>14</v>
       </c>
       <c r="F348" s="9" t="s">
         <v>28</v>
@@ -9978,7 +9978,7 @@
         <v>27</v>
       </c>
       <c r="E349" s="11">
-        <v>21</v>
+        <v>29</v>
       </c>
       <c r="F349" s="9" t="s">
         <v>28</v>
@@ -10001,7 +10001,7 @@
         <v>27</v>
       </c>
       <c r="E350" s="11">
-        <v>31</v>
+        <v>9</v>
       </c>
       <c r="F350" s="9" t="s">
         <v>28</v>
@@ -10024,7 +10024,7 @@
         <v>27</v>
       </c>
       <c r="E351" s="11">
-        <v>31</v>
+        <v>23</v>
       </c>
       <c r="F351" s="9" t="s">
         <v>28</v>
@@ -10047,7 +10047,7 @@
         <v>27</v>
       </c>
       <c r="E352" s="11">
-        <v>10</v>
+        <v>17</v>
       </c>
       <c r="F352" s="9" t="s">
         <v>28</v>
@@ -10070,7 +10070,7 @@
         <v>27</v>
       </c>
       <c r="E353" s="11">
-        <v>29</v>
+        <v>17</v>
       </c>
       <c r="F353" s="9" t="s">
         <v>28</v>
@@ -10093,7 +10093,7 @@
         <v>27</v>
       </c>
       <c r="E354" s="11">
-        <v>20</v>
+        <v>14</v>
       </c>
       <c r="F354" s="9" t="s">
         <v>28</v>
@@ -10116,7 +10116,7 @@
         <v>27</v>
       </c>
       <c r="E355" s="11">
-        <v>17</v>
+        <v>8</v>
       </c>
       <c r="F355" s="9" t="s">
         <v>28</v>
@@ -10139,7 +10139,7 @@
         <v>27</v>
       </c>
       <c r="E356" s="11">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="F356" s="9" t="s">
         <v>28</v>
@@ -10162,7 +10162,7 @@
         <v>27</v>
       </c>
       <c r="E357" s="11">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="F357" s="9" t="s">
         <v>28</v>
@@ -10185,7 +10185,7 @@
         <v>27</v>
       </c>
       <c r="E358" s="11">
-        <v>14</v>
+        <v>31</v>
       </c>
       <c r="F358" s="9" t="s">
         <v>28</v>
@@ -10208,7 +10208,7 @@
         <v>27</v>
       </c>
       <c r="E359" s="11">
-        <v>26</v>
+        <v>12</v>
       </c>
       <c r="F359" s="9" t="s">
         <v>28</v>
@@ -10231,7 +10231,7 @@
         <v>27</v>
       </c>
       <c r="E360" s="11">
-        <v>24</v>
+        <v>30</v>
       </c>
       <c r="F360" s="9" t="s">
         <v>28</v>
@@ -10254,7 +10254,7 @@
         <v>27</v>
       </c>
       <c r="E361" s="11">
-        <v>30</v>
+        <v>24</v>
       </c>
       <c r="F361" s="9" t="s">
         <v>28</v>
@@ -10277,7 +10277,7 @@
         <v>27</v>
       </c>
       <c r="E362" s="11">
-        <v>10</v>
+        <v>26</v>
       </c>
       <c r="F362" s="9" t="s">
         <v>28</v>
@@ -10300,7 +10300,7 @@
         <v>27</v>
       </c>
       <c r="E363" s="11">
-        <v>27</v>
+        <v>14</v>
       </c>
       <c r="F363" s="9" t="s">
         <v>28</v>
@@ -10323,7 +10323,7 @@
         <v>27</v>
       </c>
       <c r="E364" s="11">
-        <v>8</v>
+        <v>14</v>
       </c>
       <c r="F364" s="9" t="s">
         <v>28</v>
@@ -10346,7 +10346,7 @@
         <v>27</v>
       </c>
       <c r="E365" s="11">
-        <v>27</v>
+        <v>22</v>
       </c>
       <c r="F365" s="9" t="s">
         <v>28</v>
@@ -10369,7 +10369,7 @@
         <v>27</v>
       </c>
       <c r="E366" s="11">
-        <v>29</v>
+        <v>21</v>
       </c>
       <c r="F366" s="9" t="s">
         <v>28</v>
@@ -10392,7 +10392,7 @@
         <v>27</v>
       </c>
       <c r="E367" s="11">
-        <v>13</v>
+        <v>10</v>
       </c>
       <c r="F367" s="9" t="s">
         <v>28</v>
@@ -10415,7 +10415,7 @@
         <v>27</v>
       </c>
       <c r="E368" s="11">
-        <v>18</v>
+        <v>31</v>
       </c>
       <c r="F368" s="9" t="s">
         <v>28</v>
@@ -10438,7 +10438,7 @@
         <v>27</v>
       </c>
       <c r="E369" s="11">
-        <v>10</v>
+        <v>13</v>
       </c>
       <c r="F369" s="9" t="s">
         <v>28</v>
@@ -10461,7 +10461,7 @@
         <v>27</v>
       </c>
       <c r="E370" s="11">
-        <v>13</v>
+        <v>18</v>
       </c>
       <c r="F370" s="9" t="s">
         <v>28</v>
@@ -10484,7 +10484,7 @@
         <v>27</v>
       </c>
       <c r="E371" s="11">
-        <v>8</v>
+        <v>27</v>
       </c>
       <c r="F371" s="9" t="s">
         <v>28</v>
@@ -10507,7 +10507,7 @@
         <v>27</v>
       </c>
       <c r="E372" s="11">
-        <v>30</v>
+        <v>10</v>
       </c>
       <c r="F372" s="9" t="s">
         <v>28</v>
@@ -10530,7 +10530,7 @@
         <v>27</v>
       </c>
       <c r="E373" s="11">
-        <v>23</v>
+        <v>27</v>
       </c>
       <c r="F373" s="9" t="s">
         <v>28</v>
@@ -10553,7 +10553,7 @@
         <v>27</v>
       </c>
       <c r="E374" s="11">
-        <v>23</v>
+        <v>12</v>
       </c>
       <c r="F374" s="9" t="s">
         <v>28</v>
@@ -10576,7 +10576,7 @@
         <v>27</v>
       </c>
       <c r="E375" s="11">
-        <v>8</v>
+        <v>22</v>
       </c>
       <c r="F375" s="9" t="s">
         <v>28</v>
@@ -10599,7 +10599,7 @@
         <v>27</v>
       </c>
       <c r="E376" s="11">
-        <v>18</v>
+        <v>21</v>
       </c>
       <c r="F376" s="9" t="s">
         <v>28</v>
@@ -10622,7 +10622,7 @@
         <v>27</v>
       </c>
       <c r="E377" s="11">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="F377" s="9" t="s">
         <v>28</v>
@@ -10645,7 +10645,7 @@
         <v>27</v>
       </c>
       <c r="E378" s="11">
-        <v>17</v>
+        <v>22</v>
       </c>
       <c r="F378" s="9" t="s">
         <v>28</v>
@@ -10668,7 +10668,7 @@
         <v>27</v>
       </c>
       <c r="E379" s="11">
-        <v>15</v>
+        <v>17</v>
       </c>
       <c r="F379" s="9" t="s">
         <v>28</v>
@@ -10691,7 +10691,7 @@
         <v>27</v>
       </c>
       <c r="E380" s="11">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="F380" s="9" t="s">
         <v>28</v>
@@ -10714,7 +10714,7 @@
         <v>27</v>
       </c>
       <c r="E381" s="11">
-        <v>31</v>
+        <v>12</v>
       </c>
       <c r="F381" s="9" t="s">
         <v>28</v>
@@ -10737,7 +10737,7 @@
         <v>27</v>
       </c>
       <c r="E382" s="11">
-        <v>22</v>
+        <v>16</v>
       </c>
       <c r="F382" s="9" t="s">
         <v>28</v>
@@ -10760,7 +10760,7 @@
         <v>27</v>
       </c>
       <c r="E383" s="11">
-        <v>31</v>
+        <v>27</v>
       </c>
       <c r="F383" s="9" t="s">
         <v>28</v>
@@ -10783,7 +10783,7 @@
         <v>27</v>
       </c>
       <c r="E384" s="11">
-        <v>10</v>
+        <v>23</v>
       </c>
       <c r="F384" s="9" t="s">
         <v>28</v>
@@ -10806,7 +10806,7 @@
         <v>27</v>
       </c>
       <c r="E385" s="11">
-        <v>14</v>
+        <v>25</v>
       </c>
       <c r="F385" s="9" t="s">
         <v>28</v>
@@ -10829,7 +10829,7 @@
         <v>27</v>
       </c>
       <c r="E386" s="11">
-        <v>31</v>
+        <v>9</v>
       </c>
       <c r="F386" s="9" t="s">
         <v>28</v>
@@ -10852,7 +10852,7 @@
         <v>27</v>
       </c>
       <c r="E387" s="11">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="F387" s="9" t="s">
         <v>28</v>
@@ -10875,7 +10875,7 @@
         <v>27</v>
       </c>
       <c r="E388" s="11">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="F388" s="9" t="s">
         <v>28</v>
@@ -10898,7 +10898,7 @@
         <v>27</v>
       </c>
       <c r="E389" s="11">
-        <v>28</v>
+        <v>16</v>
       </c>
       <c r="F389" s="9" t="s">
         <v>28</v>
@@ -10921,7 +10921,7 @@
         <v>27</v>
       </c>
       <c r="E390" s="11">
-        <v>14</v>
+        <v>26</v>
       </c>
       <c r="F390" s="9" t="s">
         <v>28</v>
@@ -10944,7 +10944,7 @@
         <v>27</v>
       </c>
       <c r="E391" s="11">
-        <v>18</v>
+        <v>20</v>
       </c>
       <c r="F391" s="9" t="s">
         <v>28</v>
@@ -10967,7 +10967,7 @@
         <v>27</v>
       </c>
       <c r="E392" s="11">
-        <v>11</v>
+        <v>25</v>
       </c>
       <c r="F392" s="9" t="s">
         <v>28</v>
@@ -10990,7 +10990,7 @@
         <v>27</v>
       </c>
       <c r="E393" s="11">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="F393" s="9" t="s">
         <v>28</v>
@@ -11013,7 +11013,7 @@
         <v>27</v>
       </c>
       <c r="E394" s="11">
-        <v>28</v>
+        <v>13</v>
       </c>
       <c r="F394" s="9" t="s">
         <v>28</v>
@@ -11036,7 +11036,7 @@
         <v>27</v>
       </c>
       <c r="E395" s="11">
-        <v>27</v>
+        <v>24</v>
       </c>
       <c r="F395" s="9" t="s">
         <v>28</v>
@@ -11059,7 +11059,7 @@
         <v>27</v>
       </c>
       <c r="E396" s="11">
-        <v>18</v>
+        <v>26</v>
       </c>
       <c r="F396" s="9" t="s">
         <v>28</v>
@@ -11082,7 +11082,7 @@
         <v>27</v>
       </c>
       <c r="E397" s="11">
-        <v>19</v>
+        <v>25</v>
       </c>
       <c r="F397" s="9" t="s">
         <v>28</v>
@@ -11105,7 +11105,7 @@
         <v>27</v>
       </c>
       <c r="E398" s="11">
-        <v>10</v>
+        <v>17</v>
       </c>
       <c r="F398" s="9" t="s">
         <v>28</v>
@@ -11128,7 +11128,7 @@
         <v>27</v>
       </c>
       <c r="E399" s="11">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="F399" s="9" t="s">
         <v>28</v>
@@ -11151,7 +11151,7 @@
         <v>27</v>
       </c>
       <c r="E400" s="11">
-        <v>26</v>
+        <v>24</v>
       </c>
       <c r="F400" s="9" t="s">
         <v>28</v>
@@ -11174,7 +11174,7 @@
         <v>27</v>
       </c>
       <c r="E401" s="11">
-        <v>12</v>
+        <v>25</v>
       </c>
       <c r="F401" s="9" t="s">
         <v>28</v>

</xml_diff>

<commit_message>
feat(upload): add drag-and-drop & button photo rearrangement controls on Add Item page
</commit_message>
<xml_diff>
--- a/all-test-reports/selenium/selenium_e2e_test_report.xlsx
+++ b/all-test-reports/selenium/selenium_e2e_test_report.xlsx
@@ -35,7 +35,7 @@
     <t>Execution Date</t>
   </si>
   <si>
-    <t>28/7/2026, 10:47:41 am</t>
+    <t>28/7/2026, 10:59:38 am</t>
   </si>
   <si>
     <t>Browser / Mode</t>
@@ -47,7 +47,7 @@
     <t>Total Duration</t>
   </si>
   <si>
-    <t>0.02 seconds</t>
+    <t>0.01 seconds</t>
   </si>
   <si>
     <t>Selenium Test Execution Summary Metrics</t>
@@ -98,7 +98,7 @@
     <t>PASS</t>
   </si>
   <si>
-    <t>10:47:41 am</t>
+    <t>10:59:38 am</t>
   </si>
   <si>
     <t>N/A</t>
@@ -1997,7 +1997,7 @@
         <v>27</v>
       </c>
       <c r="E2" s="11">
-        <v>21</v>
+        <v>23</v>
       </c>
       <c r="F2" s="9" t="s">
         <v>28</v>
@@ -2020,7 +2020,7 @@
         <v>27</v>
       </c>
       <c r="E3" s="11">
-        <v>28</v>
+        <v>26</v>
       </c>
       <c r="F3" s="9" t="s">
         <v>28</v>
@@ -2043,7 +2043,7 @@
         <v>27</v>
       </c>
       <c r="E4" s="11">
-        <v>18</v>
+        <v>15</v>
       </c>
       <c r="F4" s="9" t="s">
         <v>28</v>
@@ -2066,7 +2066,7 @@
         <v>27</v>
       </c>
       <c r="E5" s="11">
-        <v>10</v>
+        <v>24</v>
       </c>
       <c r="F5" s="9" t="s">
         <v>28</v>
@@ -2089,7 +2089,7 @@
         <v>27</v>
       </c>
       <c r="E6" s="11">
-        <v>13</v>
+        <v>17</v>
       </c>
       <c r="F6" s="9" t="s">
         <v>28</v>
@@ -2112,7 +2112,7 @@
         <v>27</v>
       </c>
       <c r="E7" s="11">
-        <v>28</v>
+        <v>24</v>
       </c>
       <c r="F7" s="9" t="s">
         <v>28</v>
@@ -2135,7 +2135,7 @@
         <v>27</v>
       </c>
       <c r="E8" s="11">
-        <v>17</v>
+        <v>29</v>
       </c>
       <c r="F8" s="9" t="s">
         <v>28</v>
@@ -2158,7 +2158,7 @@
         <v>27</v>
       </c>
       <c r="E9" s="11">
-        <v>25</v>
+        <v>23</v>
       </c>
       <c r="F9" s="9" t="s">
         <v>28</v>
@@ -2181,7 +2181,7 @@
         <v>27</v>
       </c>
       <c r="E10" s="11">
-        <v>11</v>
+        <v>19</v>
       </c>
       <c r="F10" s="9" t="s">
         <v>28</v>
@@ -2204,7 +2204,7 @@
         <v>27</v>
       </c>
       <c r="E11" s="11">
-        <v>16</v>
+        <v>12</v>
       </c>
       <c r="F11" s="9" t="s">
         <v>28</v>
@@ -2227,7 +2227,7 @@
         <v>27</v>
       </c>
       <c r="E12" s="11">
-        <v>26</v>
+        <v>13</v>
       </c>
       <c r="F12" s="9" t="s">
         <v>28</v>
@@ -2250,7 +2250,7 @@
         <v>27</v>
       </c>
       <c r="E13" s="11">
-        <v>22</v>
+        <v>16</v>
       </c>
       <c r="F13" s="9" t="s">
         <v>28</v>
@@ -2273,7 +2273,7 @@
         <v>27</v>
       </c>
       <c r="E14" s="11">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="F14" s="9" t="s">
         <v>28</v>
@@ -2296,7 +2296,7 @@
         <v>27</v>
       </c>
       <c r="E15" s="11">
-        <v>26</v>
+        <v>28</v>
       </c>
       <c r="F15" s="9" t="s">
         <v>28</v>
@@ -2319,7 +2319,7 @@
         <v>27</v>
       </c>
       <c r="E16" s="11">
-        <v>10</v>
+        <v>24</v>
       </c>
       <c r="F16" s="9" t="s">
         <v>28</v>
@@ -2342,7 +2342,7 @@
         <v>27</v>
       </c>
       <c r="E17" s="11">
-        <v>12</v>
+        <v>22</v>
       </c>
       <c r="F17" s="9" t="s">
         <v>28</v>
@@ -2365,7 +2365,7 @@
         <v>27</v>
       </c>
       <c r="E18" s="11">
-        <v>8</v>
+        <v>28</v>
       </c>
       <c r="F18" s="9" t="s">
         <v>28</v>
@@ -2388,7 +2388,7 @@
         <v>27</v>
       </c>
       <c r="E19" s="11">
-        <v>8</v>
+        <v>15</v>
       </c>
       <c r="F19" s="9" t="s">
         <v>28</v>
@@ -2411,7 +2411,7 @@
         <v>27</v>
       </c>
       <c r="E20" s="11">
-        <v>20</v>
+        <v>18</v>
       </c>
       <c r="F20" s="9" t="s">
         <v>28</v>
@@ -2434,7 +2434,7 @@
         <v>27</v>
       </c>
       <c r="E21" s="11">
-        <v>17</v>
+        <v>12</v>
       </c>
       <c r="F21" s="9" t="s">
         <v>28</v>
@@ -2457,7 +2457,7 @@
         <v>27</v>
       </c>
       <c r="E22" s="11">
-        <v>26</v>
+        <v>10</v>
       </c>
       <c r="F22" s="9" t="s">
         <v>28</v>
@@ -2480,7 +2480,7 @@
         <v>27</v>
       </c>
       <c r="E23" s="11">
-        <v>18</v>
+        <v>24</v>
       </c>
       <c r="F23" s="9" t="s">
         <v>28</v>
@@ -2503,7 +2503,7 @@
         <v>27</v>
       </c>
       <c r="E24" s="11">
-        <v>20</v>
+        <v>27</v>
       </c>
       <c r="F24" s="9" t="s">
         <v>28</v>
@@ -2526,7 +2526,7 @@
         <v>27</v>
       </c>
       <c r="E25" s="11">
-        <v>30</v>
+        <v>11</v>
       </c>
       <c r="F25" s="9" t="s">
         <v>28</v>
@@ -2549,7 +2549,7 @@
         <v>27</v>
       </c>
       <c r="E26" s="11">
-        <v>16</v>
+        <v>21</v>
       </c>
       <c r="F26" s="9" t="s">
         <v>28</v>
@@ -2572,7 +2572,7 @@
         <v>27</v>
       </c>
       <c r="E27" s="11">
-        <v>20</v>
+        <v>16</v>
       </c>
       <c r="F27" s="9" t="s">
         <v>28</v>
@@ -2595,7 +2595,7 @@
         <v>27</v>
       </c>
       <c r="E28" s="11">
-        <v>25</v>
+        <v>31</v>
       </c>
       <c r="F28" s="9" t="s">
         <v>28</v>
@@ -2618,7 +2618,7 @@
         <v>27</v>
       </c>
       <c r="E29" s="11">
-        <v>14</v>
+        <v>24</v>
       </c>
       <c r="F29" s="9" t="s">
         <v>28</v>
@@ -2641,7 +2641,7 @@
         <v>27</v>
       </c>
       <c r="E30" s="11">
-        <v>28</v>
+        <v>15</v>
       </c>
       <c r="F30" s="9" t="s">
         <v>28</v>
@@ -2664,7 +2664,7 @@
         <v>27</v>
       </c>
       <c r="E31" s="11">
-        <v>21</v>
+        <v>18</v>
       </c>
       <c r="F31" s="9" t="s">
         <v>28</v>
@@ -2687,7 +2687,7 @@
         <v>27</v>
       </c>
       <c r="E32" s="11">
-        <v>21</v>
+        <v>24</v>
       </c>
       <c r="F32" s="9" t="s">
         <v>28</v>
@@ -2710,7 +2710,7 @@
         <v>27</v>
       </c>
       <c r="E33" s="11">
-        <v>18</v>
+        <v>22</v>
       </c>
       <c r="F33" s="9" t="s">
         <v>28</v>
@@ -2733,7 +2733,7 @@
         <v>27</v>
       </c>
       <c r="E34" s="11">
-        <v>29</v>
+        <v>21</v>
       </c>
       <c r="F34" s="9" t="s">
         <v>28</v>
@@ -2756,7 +2756,7 @@
         <v>27</v>
       </c>
       <c r="E35" s="11">
-        <v>15</v>
+        <v>30</v>
       </c>
       <c r="F35" s="9" t="s">
         <v>28</v>
@@ -2779,7 +2779,7 @@
         <v>27</v>
       </c>
       <c r="E36" s="11">
-        <v>30</v>
+        <v>15</v>
       </c>
       <c r="F36" s="9" t="s">
         <v>28</v>
@@ -2802,7 +2802,7 @@
         <v>27</v>
       </c>
       <c r="E37" s="11">
-        <v>11</v>
+        <v>27</v>
       </c>
       <c r="F37" s="9" t="s">
         <v>28</v>
@@ -2825,7 +2825,7 @@
         <v>27</v>
       </c>
       <c r="E38" s="11">
-        <v>22</v>
+        <v>8</v>
       </c>
       <c r="F38" s="9" t="s">
         <v>28</v>
@@ -2848,7 +2848,7 @@
         <v>27</v>
       </c>
       <c r="E39" s="11">
-        <v>16</v>
+        <v>10</v>
       </c>
       <c r="F39" s="9" t="s">
         <v>28</v>
@@ -2871,7 +2871,7 @@
         <v>27</v>
       </c>
       <c r="E40" s="11">
-        <v>30</v>
+        <v>12</v>
       </c>
       <c r="F40" s="9" t="s">
         <v>28</v>
@@ -2894,7 +2894,7 @@
         <v>27</v>
       </c>
       <c r="E41" s="11">
-        <v>30</v>
+        <v>23</v>
       </c>
       <c r="F41" s="9" t="s">
         <v>28</v>
@@ -2917,7 +2917,7 @@
         <v>27</v>
       </c>
       <c r="E42" s="11">
-        <v>30</v>
+        <v>23</v>
       </c>
       <c r="F42" s="9" t="s">
         <v>28</v>
@@ -2940,7 +2940,7 @@
         <v>27</v>
       </c>
       <c r="E43" s="11">
-        <v>13</v>
+        <v>19</v>
       </c>
       <c r="F43" s="9" t="s">
         <v>28</v>
@@ -2963,7 +2963,7 @@
         <v>27</v>
       </c>
       <c r="E44" s="11">
-        <v>22</v>
+        <v>29</v>
       </c>
       <c r="F44" s="9" t="s">
         <v>28</v>
@@ -2986,7 +2986,7 @@
         <v>27</v>
       </c>
       <c r="E45" s="11">
-        <v>14</v>
+        <v>20</v>
       </c>
       <c r="F45" s="9" t="s">
         <v>28</v>
@@ -3009,7 +3009,7 @@
         <v>27</v>
       </c>
       <c r="E46" s="11">
-        <v>24</v>
+        <v>31</v>
       </c>
       <c r="F46" s="9" t="s">
         <v>28</v>
@@ -3032,7 +3032,7 @@
         <v>27</v>
       </c>
       <c r="E47" s="11">
-        <v>11</v>
+        <v>28</v>
       </c>
       <c r="F47" s="9" t="s">
         <v>28</v>
@@ -3055,7 +3055,7 @@
         <v>27</v>
       </c>
       <c r="E48" s="11">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="F48" s="9" t="s">
         <v>28</v>
@@ -3078,7 +3078,7 @@
         <v>27</v>
       </c>
       <c r="E49" s="11">
-        <v>11</v>
+        <v>30</v>
       </c>
       <c r="F49" s="9" t="s">
         <v>28</v>
@@ -3101,7 +3101,7 @@
         <v>27</v>
       </c>
       <c r="E50" s="11">
-        <v>11</v>
+        <v>19</v>
       </c>
       <c r="F50" s="9" t="s">
         <v>28</v>
@@ -3124,7 +3124,7 @@
         <v>27</v>
       </c>
       <c r="E51" s="11">
-        <v>17</v>
+        <v>12</v>
       </c>
       <c r="F51" s="9" t="s">
         <v>28</v>
@@ -3147,7 +3147,7 @@
         <v>27</v>
       </c>
       <c r="E52" s="11">
-        <v>17</v>
+        <v>21</v>
       </c>
       <c r="F52" s="9" t="s">
         <v>28</v>
@@ -3170,7 +3170,7 @@
         <v>27</v>
       </c>
       <c r="E53" s="11">
-        <v>9</v>
+        <v>15</v>
       </c>
       <c r="F53" s="9" t="s">
         <v>28</v>
@@ -3193,7 +3193,7 @@
         <v>27</v>
       </c>
       <c r="E54" s="11">
-        <v>23</v>
+        <v>21</v>
       </c>
       <c r="F54" s="9" t="s">
         <v>28</v>
@@ -3216,7 +3216,7 @@
         <v>27</v>
       </c>
       <c r="E55" s="11">
-        <v>28</v>
+        <v>25</v>
       </c>
       <c r="F55" s="9" t="s">
         <v>28</v>
@@ -3239,7 +3239,7 @@
         <v>27</v>
       </c>
       <c r="E56" s="11">
-        <v>9</v>
+        <v>25</v>
       </c>
       <c r="F56" s="9" t="s">
         <v>28</v>
@@ -3262,7 +3262,7 @@
         <v>27</v>
       </c>
       <c r="E57" s="11">
-        <v>15</v>
+        <v>31</v>
       </c>
       <c r="F57" s="9" t="s">
         <v>28</v>
@@ -3285,7 +3285,7 @@
         <v>27</v>
       </c>
       <c r="E58" s="11">
-        <v>24</v>
+        <v>10</v>
       </c>
       <c r="F58" s="9" t="s">
         <v>28</v>
@@ -3308,7 +3308,7 @@
         <v>27</v>
       </c>
       <c r="E59" s="11">
-        <v>10</v>
+        <v>14</v>
       </c>
       <c r="F59" s="9" t="s">
         <v>28</v>
@@ -3331,7 +3331,7 @@
         <v>27</v>
       </c>
       <c r="E60" s="11">
-        <v>24</v>
+        <v>19</v>
       </c>
       <c r="F60" s="9" t="s">
         <v>28</v>
@@ -3377,7 +3377,7 @@
         <v>27</v>
       </c>
       <c r="E62" s="11">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="F62" s="9" t="s">
         <v>28</v>
@@ -3400,7 +3400,7 @@
         <v>27</v>
       </c>
       <c r="E63" s="11">
-        <v>27</v>
+        <v>13</v>
       </c>
       <c r="F63" s="9" t="s">
         <v>28</v>
@@ -3423,7 +3423,7 @@
         <v>27</v>
       </c>
       <c r="E64" s="11">
-        <v>12</v>
+        <v>24</v>
       </c>
       <c r="F64" s="9" t="s">
         <v>28</v>
@@ -3446,7 +3446,7 @@
         <v>27</v>
       </c>
       <c r="E65" s="11">
-        <v>12</v>
+        <v>19</v>
       </c>
       <c r="F65" s="9" t="s">
         <v>28</v>
@@ -3492,7 +3492,7 @@
         <v>27</v>
       </c>
       <c r="E67" s="11">
-        <v>21</v>
+        <v>14</v>
       </c>
       <c r="F67" s="9" t="s">
         <v>28</v>
@@ -3515,7 +3515,7 @@
         <v>27</v>
       </c>
       <c r="E68" s="11">
-        <v>23</v>
+        <v>16</v>
       </c>
       <c r="F68" s="9" t="s">
         <v>28</v>
@@ -3538,7 +3538,7 @@
         <v>27</v>
       </c>
       <c r="E69" s="11">
-        <v>30</v>
+        <v>13</v>
       </c>
       <c r="F69" s="9" t="s">
         <v>28</v>
@@ -3561,7 +3561,7 @@
         <v>27</v>
       </c>
       <c r="E70" s="11">
-        <v>11</v>
+        <v>18</v>
       </c>
       <c r="F70" s="9" t="s">
         <v>28</v>
@@ -3584,7 +3584,7 @@
         <v>27</v>
       </c>
       <c r="E71" s="11">
-        <v>27</v>
+        <v>16</v>
       </c>
       <c r="F71" s="9" t="s">
         <v>28</v>
@@ -3607,7 +3607,7 @@
         <v>27</v>
       </c>
       <c r="E72" s="11">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="F72" s="9" t="s">
         <v>28</v>
@@ -3630,7 +3630,7 @@
         <v>27</v>
       </c>
       <c r="E73" s="11">
-        <v>18</v>
+        <v>29</v>
       </c>
       <c r="F73" s="9" t="s">
         <v>28</v>
@@ -3653,7 +3653,7 @@
         <v>27</v>
       </c>
       <c r="E74" s="11">
-        <v>18</v>
+        <v>12</v>
       </c>
       <c r="F74" s="9" t="s">
         <v>28</v>
@@ -3676,7 +3676,7 @@
         <v>27</v>
       </c>
       <c r="E75" s="11">
-        <v>25</v>
+        <v>21</v>
       </c>
       <c r="F75" s="9" t="s">
         <v>28</v>
@@ -3699,7 +3699,7 @@
         <v>27</v>
       </c>
       <c r="E76" s="11">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="F76" s="9" t="s">
         <v>28</v>
@@ -3722,7 +3722,7 @@
         <v>27</v>
       </c>
       <c r="E77" s="11">
-        <v>23</v>
+        <v>15</v>
       </c>
       <c r="F77" s="9" t="s">
         <v>28</v>
@@ -3745,7 +3745,7 @@
         <v>27</v>
       </c>
       <c r="E78" s="11">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="F78" s="9" t="s">
         <v>28</v>
@@ -3768,7 +3768,7 @@
         <v>27</v>
       </c>
       <c r="E79" s="11">
-        <v>21</v>
+        <v>19</v>
       </c>
       <c r="F79" s="9" t="s">
         <v>28</v>
@@ -3791,7 +3791,7 @@
         <v>27</v>
       </c>
       <c r="E80" s="11">
-        <v>19</v>
+        <v>11</v>
       </c>
       <c r="F80" s="9" t="s">
         <v>28</v>
@@ -3814,7 +3814,7 @@
         <v>27</v>
       </c>
       <c r="E81" s="11">
-        <v>12</v>
+        <v>26</v>
       </c>
       <c r="F81" s="9" t="s">
         <v>28</v>
@@ -3837,7 +3837,7 @@
         <v>27</v>
       </c>
       <c r="E82" s="11">
-        <v>13</v>
+        <v>27</v>
       </c>
       <c r="F82" s="9" t="s">
         <v>28</v>
@@ -3860,7 +3860,7 @@
         <v>27</v>
       </c>
       <c r="E83" s="11">
-        <v>13</v>
+        <v>25</v>
       </c>
       <c r="F83" s="9" t="s">
         <v>28</v>
@@ -3883,7 +3883,7 @@
         <v>27</v>
       </c>
       <c r="E84" s="11">
-        <v>20</v>
+        <v>22</v>
       </c>
       <c r="F84" s="9" t="s">
         <v>28</v>
@@ -3906,7 +3906,7 @@
         <v>27</v>
       </c>
       <c r="E85" s="11">
-        <v>31</v>
+        <v>25</v>
       </c>
       <c r="F85" s="9" t="s">
         <v>28</v>
@@ -3929,7 +3929,7 @@
         <v>27</v>
       </c>
       <c r="E86" s="11">
-        <v>24</v>
+        <v>11</v>
       </c>
       <c r="F86" s="9" t="s">
         <v>28</v>
@@ -3952,7 +3952,7 @@
         <v>27</v>
       </c>
       <c r="E87" s="11">
-        <v>25</v>
+        <v>23</v>
       </c>
       <c r="F87" s="9" t="s">
         <v>28</v>
@@ -3975,7 +3975,7 @@
         <v>27</v>
       </c>
       <c r="E88" s="11">
-        <v>28</v>
+        <v>13</v>
       </c>
       <c r="F88" s="9" t="s">
         <v>28</v>
@@ -3998,7 +3998,7 @@
         <v>27</v>
       </c>
       <c r="E89" s="11">
-        <v>21</v>
+        <v>13</v>
       </c>
       <c r="F89" s="9" t="s">
         <v>28</v>
@@ -4021,7 +4021,7 @@
         <v>27</v>
       </c>
       <c r="E90" s="11">
-        <v>18</v>
+        <v>25</v>
       </c>
       <c r="F90" s="9" t="s">
         <v>28</v>
@@ -4044,7 +4044,7 @@
         <v>27</v>
       </c>
       <c r="E91" s="11">
-        <v>27</v>
+        <v>25</v>
       </c>
       <c r="F91" s="9" t="s">
         <v>28</v>
@@ -4067,7 +4067,7 @@
         <v>27</v>
       </c>
       <c r="E92" s="11">
-        <v>21</v>
+        <v>19</v>
       </c>
       <c r="F92" s="9" t="s">
         <v>28</v>
@@ -4090,7 +4090,7 @@
         <v>27</v>
       </c>
       <c r="E93" s="11">
-        <v>29</v>
+        <v>25</v>
       </c>
       <c r="F93" s="9" t="s">
         <v>28</v>
@@ -4113,7 +4113,7 @@
         <v>27</v>
       </c>
       <c r="E94" s="11">
-        <v>18</v>
+        <v>21</v>
       </c>
       <c r="F94" s="9" t="s">
         <v>28</v>
@@ -4136,7 +4136,7 @@
         <v>27</v>
       </c>
       <c r="E95" s="11">
-        <v>25</v>
+        <v>21</v>
       </c>
       <c r="F95" s="9" t="s">
         <v>28</v>
@@ -4159,7 +4159,7 @@
         <v>27</v>
       </c>
       <c r="E96" s="11">
-        <v>23</v>
+        <v>30</v>
       </c>
       <c r="F96" s="9" t="s">
         <v>28</v>
@@ -4182,7 +4182,7 @@
         <v>27</v>
       </c>
       <c r="E97" s="11">
-        <v>27</v>
+        <v>12</v>
       </c>
       <c r="F97" s="9" t="s">
         <v>28</v>
@@ -4205,7 +4205,7 @@
         <v>27</v>
       </c>
       <c r="E98" s="11">
-        <v>8</v>
+        <v>25</v>
       </c>
       <c r="F98" s="9" t="s">
         <v>28</v>
@@ -4228,7 +4228,7 @@
         <v>27</v>
       </c>
       <c r="E99" s="11">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="F99" s="9" t="s">
         <v>28</v>
@@ -4251,7 +4251,7 @@
         <v>27</v>
       </c>
       <c r="E100" s="11">
-        <v>16</v>
+        <v>8</v>
       </c>
       <c r="F100" s="9" t="s">
         <v>28</v>
@@ -4274,7 +4274,7 @@
         <v>27</v>
       </c>
       <c r="E101" s="11">
-        <v>11</v>
+        <v>24</v>
       </c>
       <c r="F101" s="9" t="s">
         <v>28</v>
@@ -4297,7 +4297,7 @@
         <v>27</v>
       </c>
       <c r="E102" s="11">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="F102" s="9" t="s">
         <v>28</v>
@@ -4320,7 +4320,7 @@
         <v>27</v>
       </c>
       <c r="E103" s="11">
-        <v>12</v>
+        <v>30</v>
       </c>
       <c r="F103" s="9" t="s">
         <v>28</v>
@@ -4343,7 +4343,7 @@
         <v>27</v>
       </c>
       <c r="E104" s="11">
-        <v>24</v>
+        <v>9</v>
       </c>
       <c r="F104" s="9" t="s">
         <v>28</v>
@@ -4366,7 +4366,7 @@
         <v>27</v>
       </c>
       <c r="E105" s="11">
-        <v>24</v>
+        <v>14</v>
       </c>
       <c r="F105" s="9" t="s">
         <v>28</v>
@@ -4389,7 +4389,7 @@
         <v>27</v>
       </c>
       <c r="E106" s="11">
-        <v>24</v>
+        <v>26</v>
       </c>
       <c r="F106" s="9" t="s">
         <v>28</v>
@@ -4412,7 +4412,7 @@
         <v>27</v>
       </c>
       <c r="E107" s="11">
-        <v>18</v>
+        <v>13</v>
       </c>
       <c r="F107" s="9" t="s">
         <v>28</v>
@@ -4435,7 +4435,7 @@
         <v>27</v>
       </c>
       <c r="E108" s="11">
-        <v>8</v>
+        <v>15</v>
       </c>
       <c r="F108" s="9" t="s">
         <v>28</v>
@@ -4481,7 +4481,7 @@
         <v>27</v>
       </c>
       <c r="E110" s="11">
-        <v>16</v>
+        <v>11</v>
       </c>
       <c r="F110" s="9" t="s">
         <v>28</v>
@@ -4504,7 +4504,7 @@
         <v>27</v>
       </c>
       <c r="E111" s="11">
-        <v>19</v>
+        <v>23</v>
       </c>
       <c r="F111" s="9" t="s">
         <v>28</v>
@@ -4527,7 +4527,7 @@
         <v>27</v>
       </c>
       <c r="E112" s="11">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="F112" s="9" t="s">
         <v>28</v>
@@ -4550,7 +4550,7 @@
         <v>27</v>
       </c>
       <c r="E113" s="11">
-        <v>27</v>
+        <v>23</v>
       </c>
       <c r="F113" s="9" t="s">
         <v>28</v>
@@ -4573,7 +4573,7 @@
         <v>27</v>
       </c>
       <c r="E114" s="11">
-        <v>19</v>
+        <v>13</v>
       </c>
       <c r="F114" s="9" t="s">
         <v>28</v>
@@ -4596,7 +4596,7 @@
         <v>27</v>
       </c>
       <c r="E115" s="11">
-        <v>15</v>
+        <v>30</v>
       </c>
       <c r="F115" s="9" t="s">
         <v>28</v>
@@ -4642,7 +4642,7 @@
         <v>27</v>
       </c>
       <c r="E117" s="11">
-        <v>9</v>
+        <v>28</v>
       </c>
       <c r="F117" s="9" t="s">
         <v>28</v>
@@ -4665,7 +4665,7 @@
         <v>27</v>
       </c>
       <c r="E118" s="11">
-        <v>12</v>
+        <v>9</v>
       </c>
       <c r="F118" s="9" t="s">
         <v>28</v>
@@ -4688,7 +4688,7 @@
         <v>27</v>
       </c>
       <c r="E119" s="11">
-        <v>27</v>
+        <v>14</v>
       </c>
       <c r="F119" s="9" t="s">
         <v>28</v>
@@ -4711,7 +4711,7 @@
         <v>27</v>
       </c>
       <c r="E120" s="11">
-        <v>26</v>
+        <v>20</v>
       </c>
       <c r="F120" s="9" t="s">
         <v>28</v>
@@ -4734,7 +4734,7 @@
         <v>27</v>
       </c>
       <c r="E121" s="11">
-        <v>13</v>
+        <v>20</v>
       </c>
       <c r="F121" s="9" t="s">
         <v>28</v>
@@ -4757,7 +4757,7 @@
         <v>27</v>
       </c>
       <c r="E122" s="11">
-        <v>21</v>
+        <v>8</v>
       </c>
       <c r="F122" s="9" t="s">
         <v>28</v>
@@ -4780,7 +4780,7 @@
         <v>27</v>
       </c>
       <c r="E123" s="11">
-        <v>31</v>
+        <v>19</v>
       </c>
       <c r="F123" s="9" t="s">
         <v>28</v>
@@ -4803,7 +4803,7 @@
         <v>27</v>
       </c>
       <c r="E124" s="11">
-        <v>24</v>
+        <v>26</v>
       </c>
       <c r="F124" s="9" t="s">
         <v>28</v>
@@ -4826,7 +4826,7 @@
         <v>27</v>
       </c>
       <c r="E125" s="11">
-        <v>13</v>
+        <v>27</v>
       </c>
       <c r="F125" s="9" t="s">
         <v>28</v>
@@ -4849,7 +4849,7 @@
         <v>27</v>
       </c>
       <c r="E126" s="11">
-        <v>19</v>
+        <v>25</v>
       </c>
       <c r="F126" s="9" t="s">
         <v>28</v>
@@ -4872,7 +4872,7 @@
         <v>27</v>
       </c>
       <c r="E127" s="11">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="F127" s="9" t="s">
         <v>28</v>
@@ -4895,7 +4895,7 @@
         <v>27</v>
       </c>
       <c r="E128" s="11">
-        <v>8</v>
+        <v>18</v>
       </c>
       <c r="F128" s="9" t="s">
         <v>28</v>
@@ -4918,7 +4918,7 @@
         <v>27</v>
       </c>
       <c r="E129" s="11">
-        <v>20</v>
+        <v>8</v>
       </c>
       <c r="F129" s="9" t="s">
         <v>28</v>
@@ -4941,7 +4941,7 @@
         <v>27</v>
       </c>
       <c r="E130" s="11">
-        <v>13</v>
+        <v>9</v>
       </c>
       <c r="F130" s="9" t="s">
         <v>28</v>
@@ -4964,7 +4964,7 @@
         <v>27</v>
       </c>
       <c r="E131" s="11">
-        <v>30</v>
+        <v>27</v>
       </c>
       <c r="F131" s="9" t="s">
         <v>28</v>
@@ -4987,7 +4987,7 @@
         <v>27</v>
       </c>
       <c r="E132" s="11">
-        <v>24</v>
+        <v>9</v>
       </c>
       <c r="F132" s="9" t="s">
         <v>28</v>
@@ -5010,7 +5010,7 @@
         <v>27</v>
       </c>
       <c r="E133" s="11">
-        <v>22</v>
+        <v>16</v>
       </c>
       <c r="F133" s="9" t="s">
         <v>28</v>
@@ -5033,7 +5033,7 @@
         <v>27</v>
       </c>
       <c r="E134" s="11">
-        <v>23</v>
+        <v>17</v>
       </c>
       <c r="F134" s="9" t="s">
         <v>28</v>
@@ -5056,7 +5056,7 @@
         <v>27</v>
       </c>
       <c r="E135" s="11">
-        <v>24</v>
+        <v>17</v>
       </c>
       <c r="F135" s="9" t="s">
         <v>28</v>
@@ -5079,7 +5079,7 @@
         <v>27</v>
       </c>
       <c r="E136" s="11">
-        <v>29</v>
+        <v>14</v>
       </c>
       <c r="F136" s="9" t="s">
         <v>28</v>
@@ -5102,7 +5102,7 @@
         <v>27</v>
       </c>
       <c r="E137" s="11">
-        <v>26</v>
+        <v>29</v>
       </c>
       <c r="F137" s="9" t="s">
         <v>28</v>
@@ -5148,7 +5148,7 @@
         <v>27</v>
       </c>
       <c r="E139" s="11">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="F139" s="9" t="s">
         <v>28</v>
@@ -5194,7 +5194,7 @@
         <v>27</v>
       </c>
       <c r="E141" s="11">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="F141" s="9" t="s">
         <v>28</v>
@@ -5240,7 +5240,7 @@
         <v>27</v>
       </c>
       <c r="E143" s="11">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="F143" s="9" t="s">
         <v>28</v>
@@ -5263,7 +5263,7 @@
         <v>27</v>
       </c>
       <c r="E144" s="11">
-        <v>9</v>
+        <v>16</v>
       </c>
       <c r="F144" s="9" t="s">
         <v>28</v>
@@ -5286,7 +5286,7 @@
         <v>27</v>
       </c>
       <c r="E145" s="11">
-        <v>27</v>
+        <v>22</v>
       </c>
       <c r="F145" s="9" t="s">
         <v>28</v>
@@ -5309,7 +5309,7 @@
         <v>27</v>
       </c>
       <c r="E146" s="11">
-        <v>24</v>
+        <v>27</v>
       </c>
       <c r="F146" s="9" t="s">
         <v>28</v>
@@ -5332,7 +5332,7 @@
         <v>27</v>
       </c>
       <c r="E147" s="11">
-        <v>28</v>
+        <v>16</v>
       </c>
       <c r="F147" s="9" t="s">
         <v>28</v>
@@ -5355,7 +5355,7 @@
         <v>27</v>
       </c>
       <c r="E148" s="11">
-        <v>8</v>
+        <v>31</v>
       </c>
       <c r="F148" s="9" t="s">
         <v>28</v>
@@ -5378,7 +5378,7 @@
         <v>27</v>
       </c>
       <c r="E149" s="11">
-        <v>24</v>
+        <v>8</v>
       </c>
       <c r="F149" s="9" t="s">
         <v>28</v>
@@ -5401,7 +5401,7 @@
         <v>27</v>
       </c>
       <c r="E150" s="11">
-        <v>18</v>
+        <v>22</v>
       </c>
       <c r="F150" s="9" t="s">
         <v>28</v>
@@ -5447,7 +5447,7 @@
         <v>27</v>
       </c>
       <c r="E152" s="11">
-        <v>22</v>
+        <v>18</v>
       </c>
       <c r="F152" s="9" t="s">
         <v>28</v>
@@ -5470,7 +5470,7 @@
         <v>27</v>
       </c>
       <c r="E153" s="11">
-        <v>15</v>
+        <v>23</v>
       </c>
       <c r="F153" s="9" t="s">
         <v>28</v>
@@ -5493,7 +5493,7 @@
         <v>27</v>
       </c>
       <c r="E154" s="11">
-        <v>23</v>
+        <v>19</v>
       </c>
       <c r="F154" s="9" t="s">
         <v>28</v>
@@ -5516,7 +5516,7 @@
         <v>27</v>
       </c>
       <c r="E155" s="11">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="F155" s="9" t="s">
         <v>28</v>
@@ -5539,7 +5539,7 @@
         <v>27</v>
       </c>
       <c r="E156" s="11">
-        <v>28</v>
+        <v>19</v>
       </c>
       <c r="F156" s="9" t="s">
         <v>28</v>
@@ -5562,7 +5562,7 @@
         <v>27</v>
       </c>
       <c r="E157" s="11">
-        <v>26</v>
+        <v>8</v>
       </c>
       <c r="F157" s="9" t="s">
         <v>28</v>
@@ -5585,7 +5585,7 @@
         <v>27</v>
       </c>
       <c r="E158" s="11">
-        <v>31</v>
+        <v>29</v>
       </c>
       <c r="F158" s="9" t="s">
         <v>28</v>
@@ -5608,7 +5608,7 @@
         <v>27</v>
       </c>
       <c r="E159" s="11">
-        <v>12</v>
+        <v>27</v>
       </c>
       <c r="F159" s="9" t="s">
         <v>28</v>
@@ -5631,7 +5631,7 @@
         <v>27</v>
       </c>
       <c r="E160" s="11">
-        <v>30</v>
+        <v>8</v>
       </c>
       <c r="F160" s="9" t="s">
         <v>28</v>
@@ -5654,7 +5654,7 @@
         <v>27</v>
       </c>
       <c r="E161" s="11">
-        <v>28</v>
+        <v>18</v>
       </c>
       <c r="F161" s="9" t="s">
         <v>28</v>
@@ -5677,7 +5677,7 @@
         <v>27</v>
       </c>
       <c r="E162" s="11">
-        <v>9</v>
+        <v>31</v>
       </c>
       <c r="F162" s="9" t="s">
         <v>28</v>
@@ -5700,7 +5700,7 @@
         <v>27</v>
       </c>
       <c r="E163" s="11">
-        <v>13</v>
+        <v>29</v>
       </c>
       <c r="F163" s="9" t="s">
         <v>28</v>
@@ -5723,7 +5723,7 @@
         <v>27</v>
       </c>
       <c r="E164" s="11">
-        <v>27</v>
+        <v>12</v>
       </c>
       <c r="F164" s="9" t="s">
         <v>28</v>
@@ -5746,7 +5746,7 @@
         <v>27</v>
       </c>
       <c r="E165" s="11">
-        <v>10</v>
+        <v>21</v>
       </c>
       <c r="F165" s="9" t="s">
         <v>28</v>
@@ -5769,7 +5769,7 @@
         <v>27</v>
       </c>
       <c r="E166" s="11">
-        <v>21</v>
+        <v>10</v>
       </c>
       <c r="F166" s="9" t="s">
         <v>28</v>
@@ -5792,7 +5792,7 @@
         <v>27</v>
       </c>
       <c r="E167" s="11">
-        <v>20</v>
+        <v>29</v>
       </c>
       <c r="F167" s="9" t="s">
         <v>28</v>
@@ -5815,7 +5815,7 @@
         <v>27</v>
       </c>
       <c r="E168" s="11">
-        <v>21</v>
+        <v>26</v>
       </c>
       <c r="F168" s="9" t="s">
         <v>28</v>
@@ -5838,7 +5838,7 @@
         <v>27</v>
       </c>
       <c r="E169" s="11">
-        <v>15</v>
+        <v>13</v>
       </c>
       <c r="F169" s="9" t="s">
         <v>28</v>
@@ -5861,7 +5861,7 @@
         <v>27</v>
       </c>
       <c r="E170" s="11">
-        <v>8</v>
+        <v>17</v>
       </c>
       <c r="F170" s="9" t="s">
         <v>28</v>
@@ -5884,7 +5884,7 @@
         <v>27</v>
       </c>
       <c r="E171" s="11">
-        <v>21</v>
+        <v>30</v>
       </c>
       <c r="F171" s="9" t="s">
         <v>28</v>
@@ -5907,7 +5907,7 @@
         <v>27</v>
       </c>
       <c r="E172" s="11">
-        <v>24</v>
+        <v>28</v>
       </c>
       <c r="F172" s="9" t="s">
         <v>28</v>
@@ -5930,7 +5930,7 @@
         <v>27</v>
       </c>
       <c r="E173" s="11">
-        <v>15</v>
+        <v>9</v>
       </c>
       <c r="F173" s="9" t="s">
         <v>28</v>
@@ -5953,7 +5953,7 @@
         <v>27</v>
       </c>
       <c r="E174" s="11">
-        <v>10</v>
+        <v>31</v>
       </c>
       <c r="F174" s="9" t="s">
         <v>28</v>
@@ -5976,7 +5976,7 @@
         <v>27</v>
       </c>
       <c r="E175" s="11">
-        <v>21</v>
+        <v>14</v>
       </c>
       <c r="F175" s="9" t="s">
         <v>28</v>
@@ -5999,7 +5999,7 @@
         <v>27</v>
       </c>
       <c r="E176" s="11">
-        <v>11</v>
+        <v>30</v>
       </c>
       <c r="F176" s="9" t="s">
         <v>28</v>
@@ -6022,7 +6022,7 @@
         <v>27</v>
       </c>
       <c r="E177" s="11">
-        <v>17</v>
+        <v>27</v>
       </c>
       <c r="F177" s="9" t="s">
         <v>28</v>
@@ -6045,7 +6045,7 @@
         <v>27</v>
       </c>
       <c r="E178" s="11">
-        <v>27</v>
+        <v>11</v>
       </c>
       <c r="F178" s="9" t="s">
         <v>28</v>
@@ -6068,7 +6068,7 @@
         <v>27</v>
       </c>
       <c r="E179" s="11">
-        <v>24</v>
+        <v>20</v>
       </c>
       <c r="F179" s="9" t="s">
         <v>28</v>
@@ -6091,7 +6091,7 @@
         <v>27</v>
       </c>
       <c r="E180" s="11">
-        <v>23</v>
+        <v>12</v>
       </c>
       <c r="F180" s="9" t="s">
         <v>28</v>
@@ -6114,7 +6114,7 @@
         <v>27</v>
       </c>
       <c r="E181" s="11">
-        <v>8</v>
+        <v>14</v>
       </c>
       <c r="F181" s="9" t="s">
         <v>28</v>
@@ -6137,7 +6137,7 @@
         <v>27</v>
       </c>
       <c r="E182" s="11">
-        <v>10</v>
+        <v>25</v>
       </c>
       <c r="F182" s="9" t="s">
         <v>28</v>
@@ -6160,7 +6160,7 @@
         <v>27</v>
       </c>
       <c r="E183" s="11">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="F183" s="9" t="s">
         <v>28</v>
@@ -6183,7 +6183,7 @@
         <v>27</v>
       </c>
       <c r="E184" s="11">
-        <v>30</v>
+        <v>28</v>
       </c>
       <c r="F184" s="9" t="s">
         <v>28</v>
@@ -6206,7 +6206,7 @@
         <v>27</v>
       </c>
       <c r="E185" s="11">
-        <v>28</v>
+        <v>11</v>
       </c>
       <c r="F185" s="9" t="s">
         <v>28</v>
@@ -6229,7 +6229,7 @@
         <v>27</v>
       </c>
       <c r="E186" s="11">
-        <v>14</v>
+        <v>27</v>
       </c>
       <c r="F186" s="9" t="s">
         <v>28</v>
@@ -6252,7 +6252,7 @@
         <v>27</v>
       </c>
       <c r="E187" s="11">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="F187" s="9" t="s">
         <v>28</v>
@@ -6275,7 +6275,7 @@
         <v>27</v>
       </c>
       <c r="E188" s="11">
-        <v>27</v>
+        <v>13</v>
       </c>
       <c r="F188" s="9" t="s">
         <v>28</v>
@@ -6298,7 +6298,7 @@
         <v>27</v>
       </c>
       <c r="E189" s="11">
-        <v>21</v>
+        <v>27</v>
       </c>
       <c r="F189" s="9" t="s">
         <v>28</v>
@@ -6321,7 +6321,7 @@
         <v>27</v>
       </c>
       <c r="E190" s="11">
-        <v>16</v>
+        <v>10</v>
       </c>
       <c r="F190" s="9" t="s">
         <v>28</v>
@@ -6344,7 +6344,7 @@
         <v>27</v>
       </c>
       <c r="E191" s="11">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="F191" s="9" t="s">
         <v>28</v>
@@ -6367,7 +6367,7 @@
         <v>27</v>
       </c>
       <c r="E192" s="11">
-        <v>17</v>
+        <v>25</v>
       </c>
       <c r="F192" s="9" t="s">
         <v>28</v>
@@ -6413,7 +6413,7 @@
         <v>27</v>
       </c>
       <c r="E194" s="11">
-        <v>8</v>
+        <v>24</v>
       </c>
       <c r="F194" s="9" t="s">
         <v>28</v>
@@ -6436,7 +6436,7 @@
         <v>27</v>
       </c>
       <c r="E195" s="11">
-        <v>17</v>
+        <v>21</v>
       </c>
       <c r="F195" s="9" t="s">
         <v>28</v>
@@ -6459,7 +6459,7 @@
         <v>27</v>
       </c>
       <c r="E196" s="11">
-        <v>22</v>
+        <v>30</v>
       </c>
       <c r="F196" s="9" t="s">
         <v>28</v>
@@ -6482,7 +6482,7 @@
         <v>27</v>
       </c>
       <c r="E197" s="11">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="F197" s="9" t="s">
         <v>28</v>
@@ -6505,7 +6505,7 @@
         <v>27</v>
       </c>
       <c r="E198" s="11">
-        <v>20</v>
+        <v>24</v>
       </c>
       <c r="F198" s="9" t="s">
         <v>28</v>
@@ -6528,7 +6528,7 @@
         <v>27</v>
       </c>
       <c r="E199" s="11">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="F199" s="9" t="s">
         <v>28</v>
@@ -6551,7 +6551,7 @@
         <v>27</v>
       </c>
       <c r="E200" s="11">
-        <v>13</v>
+        <v>15</v>
       </c>
       <c r="F200" s="9" t="s">
         <v>28</v>
@@ -6574,7 +6574,7 @@
         <v>27</v>
       </c>
       <c r="E201" s="11">
-        <v>17</v>
+        <v>12</v>
       </c>
       <c r="F201" s="9" t="s">
         <v>28</v>
@@ -6597,7 +6597,7 @@
         <v>27</v>
       </c>
       <c r="E202" s="11">
-        <v>14</v>
+        <v>9</v>
       </c>
       <c r="F202" s="9" t="s">
         <v>28</v>
@@ -6620,7 +6620,7 @@
         <v>27</v>
       </c>
       <c r="E203" s="11">
-        <v>29</v>
+        <v>27</v>
       </c>
       <c r="F203" s="9" t="s">
         <v>28</v>
@@ -6643,7 +6643,7 @@
         <v>27</v>
       </c>
       <c r="E204" s="11">
-        <v>17</v>
+        <v>15</v>
       </c>
       <c r="F204" s="9" t="s">
         <v>28</v>
@@ -6666,7 +6666,7 @@
         <v>27</v>
       </c>
       <c r="E205" s="11">
-        <v>8</v>
+        <v>14</v>
       </c>
       <c r="F205" s="9" t="s">
         <v>28</v>
@@ -6689,7 +6689,7 @@
         <v>27</v>
       </c>
       <c r="E206" s="11">
-        <v>18</v>
+        <v>10</v>
       </c>
       <c r="F206" s="9" t="s">
         <v>28</v>
@@ -6712,7 +6712,7 @@
         <v>27</v>
       </c>
       <c r="E207" s="11">
-        <v>29</v>
+        <v>19</v>
       </c>
       <c r="F207" s="9" t="s">
         <v>28</v>
@@ -6735,7 +6735,7 @@
         <v>27</v>
       </c>
       <c r="E208" s="11">
-        <v>12</v>
+        <v>10</v>
       </c>
       <c r="F208" s="9" t="s">
         <v>28</v>
@@ -6758,7 +6758,7 @@
         <v>27</v>
       </c>
       <c r="E209" s="11">
-        <v>13</v>
+        <v>21</v>
       </c>
       <c r="F209" s="9" t="s">
         <v>28</v>
@@ -6781,7 +6781,7 @@
         <v>27</v>
       </c>
       <c r="E210" s="11">
-        <v>12</v>
+        <v>27</v>
       </c>
       <c r="F210" s="9" t="s">
         <v>28</v>
@@ -6804,7 +6804,7 @@
         <v>27</v>
       </c>
       <c r="E211" s="11">
-        <v>17</v>
+        <v>20</v>
       </c>
       <c r="F211" s="9" t="s">
         <v>28</v>
@@ -6827,7 +6827,7 @@
         <v>27</v>
       </c>
       <c r="E212" s="11">
-        <v>12</v>
+        <v>27</v>
       </c>
       <c r="F212" s="9" t="s">
         <v>28</v>
@@ -6850,7 +6850,7 @@
         <v>27</v>
       </c>
       <c r="E213" s="11">
-        <v>27</v>
+        <v>23</v>
       </c>
       <c r="F213" s="9" t="s">
         <v>28</v>
@@ -6873,7 +6873,7 @@
         <v>27</v>
       </c>
       <c r="E214" s="11">
-        <v>26</v>
+        <v>10</v>
       </c>
       <c r="F214" s="9" t="s">
         <v>28</v>
@@ -6896,7 +6896,7 @@
         <v>27</v>
       </c>
       <c r="E215" s="11">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="F215" s="9" t="s">
         <v>28</v>
@@ -6919,7 +6919,7 @@
         <v>27</v>
       </c>
       <c r="E216" s="11">
-        <v>31</v>
+        <v>22</v>
       </c>
       <c r="F216" s="9" t="s">
         <v>28</v>
@@ -6942,7 +6942,7 @@
         <v>27</v>
       </c>
       <c r="E217" s="11">
-        <v>18</v>
+        <v>24</v>
       </c>
       <c r="F217" s="9" t="s">
         <v>28</v>
@@ -6965,7 +6965,7 @@
         <v>27</v>
       </c>
       <c r="E218" s="11">
-        <v>8</v>
+        <v>31</v>
       </c>
       <c r="F218" s="9" t="s">
         <v>28</v>
@@ -6988,7 +6988,7 @@
         <v>27</v>
       </c>
       <c r="E219" s="11">
-        <v>31</v>
+        <v>11</v>
       </c>
       <c r="F219" s="9" t="s">
         <v>28</v>
@@ -7011,7 +7011,7 @@
         <v>27</v>
       </c>
       <c r="E220" s="11">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="F220" s="9" t="s">
         <v>28</v>
@@ -7034,7 +7034,7 @@
         <v>27</v>
       </c>
       <c r="E221" s="11">
-        <v>25</v>
+        <v>10</v>
       </c>
       <c r="F221" s="9" t="s">
         <v>28</v>
@@ -7057,7 +7057,7 @@
         <v>27</v>
       </c>
       <c r="E222" s="11">
-        <v>16</v>
+        <v>24</v>
       </c>
       <c r="F222" s="9" t="s">
         <v>28</v>
@@ -7080,7 +7080,7 @@
         <v>27</v>
       </c>
       <c r="E223" s="11">
-        <v>9</v>
+        <v>22</v>
       </c>
       <c r="F223" s="9" t="s">
         <v>28</v>
@@ -7103,7 +7103,7 @@
         <v>27</v>
       </c>
       <c r="E224" s="11">
-        <v>16</v>
+        <v>20</v>
       </c>
       <c r="F224" s="9" t="s">
         <v>28</v>
@@ -7126,7 +7126,7 @@
         <v>27</v>
       </c>
       <c r="E225" s="11">
-        <v>21</v>
+        <v>11</v>
       </c>
       <c r="F225" s="9" t="s">
         <v>28</v>
@@ -7149,7 +7149,7 @@
         <v>27</v>
       </c>
       <c r="E226" s="11">
-        <v>11</v>
+        <v>17</v>
       </c>
       <c r="F226" s="9" t="s">
         <v>28</v>
@@ -7172,7 +7172,7 @@
         <v>27</v>
       </c>
       <c r="E227" s="11">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="F227" s="9" t="s">
         <v>28</v>
@@ -7195,7 +7195,7 @@
         <v>27</v>
       </c>
       <c r="E228" s="11">
-        <v>28</v>
+        <v>22</v>
       </c>
       <c r="F228" s="9" t="s">
         <v>28</v>
@@ -7218,7 +7218,7 @@
         <v>27</v>
       </c>
       <c r="E229" s="11">
-        <v>8</v>
+        <v>22</v>
       </c>
       <c r="F229" s="9" t="s">
         <v>28</v>
@@ -7241,7 +7241,7 @@
         <v>27</v>
       </c>
       <c r="E230" s="11">
-        <v>21</v>
+        <v>31</v>
       </c>
       <c r="F230" s="9" t="s">
         <v>28</v>
@@ -7264,7 +7264,7 @@
         <v>27</v>
       </c>
       <c r="E231" s="11">
-        <v>31</v>
+        <v>8</v>
       </c>
       <c r="F231" s="9" t="s">
         <v>28</v>
@@ -7287,7 +7287,7 @@
         <v>27</v>
       </c>
       <c r="E232" s="11">
-        <v>16</v>
+        <v>14</v>
       </c>
       <c r="F232" s="9" t="s">
         <v>28</v>
@@ -7310,7 +7310,7 @@
         <v>27</v>
       </c>
       <c r="E233" s="11">
-        <v>24</v>
+        <v>27</v>
       </c>
       <c r="F233" s="9" t="s">
         <v>28</v>
@@ -7333,7 +7333,7 @@
         <v>27</v>
       </c>
       <c r="E234" s="11">
-        <v>21</v>
+        <v>8</v>
       </c>
       <c r="F234" s="9" t="s">
         <v>28</v>
@@ -7356,7 +7356,7 @@
         <v>27</v>
       </c>
       <c r="E235" s="11">
-        <v>13</v>
+        <v>21</v>
       </c>
       <c r="F235" s="9" t="s">
         <v>28</v>
@@ -7379,7 +7379,7 @@
         <v>27</v>
       </c>
       <c r="E236" s="11">
-        <v>29</v>
+        <v>18</v>
       </c>
       <c r="F236" s="9" t="s">
         <v>28</v>
@@ -7402,7 +7402,7 @@
         <v>27</v>
       </c>
       <c r="E237" s="11">
-        <v>26</v>
+        <v>8</v>
       </c>
       <c r="F237" s="9" t="s">
         <v>28</v>
@@ -7425,7 +7425,7 @@
         <v>27</v>
       </c>
       <c r="E238" s="11">
-        <v>16</v>
+        <v>11</v>
       </c>
       <c r="F238" s="9" t="s">
         <v>28</v>
@@ -7448,7 +7448,7 @@
         <v>27</v>
       </c>
       <c r="E239" s="11">
-        <v>26</v>
+        <v>10</v>
       </c>
       <c r="F239" s="9" t="s">
         <v>28</v>
@@ -7471,7 +7471,7 @@
         <v>27</v>
       </c>
       <c r="E240" s="11">
-        <v>26</v>
+        <v>20</v>
       </c>
       <c r="F240" s="9" t="s">
         <v>28</v>
@@ -7494,7 +7494,7 @@
         <v>27</v>
       </c>
       <c r="E241" s="11">
-        <v>21</v>
+        <v>29</v>
       </c>
       <c r="F241" s="9" t="s">
         <v>28</v>
@@ -7517,7 +7517,7 @@
         <v>27</v>
       </c>
       <c r="E242" s="11">
-        <v>17</v>
+        <v>12</v>
       </c>
       <c r="F242" s="9" t="s">
         <v>28</v>
@@ -7540,7 +7540,7 @@
         <v>27</v>
       </c>
       <c r="E243" s="11">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="F243" s="9" t="s">
         <v>28</v>
@@ -7563,7 +7563,7 @@
         <v>27</v>
       </c>
       <c r="E244" s="11">
-        <v>17</v>
+        <v>9</v>
       </c>
       <c r="F244" s="9" t="s">
         <v>28</v>
@@ -7586,7 +7586,7 @@
         <v>27</v>
       </c>
       <c r="E245" s="11">
-        <v>21</v>
+        <v>25</v>
       </c>
       <c r="F245" s="9" t="s">
         <v>28</v>
@@ -7609,7 +7609,7 @@
         <v>27</v>
       </c>
       <c r="E246" s="11">
-        <v>18</v>
+        <v>14</v>
       </c>
       <c r="F246" s="9" t="s">
         <v>28</v>
@@ -7632,7 +7632,7 @@
         <v>27</v>
       </c>
       <c r="E247" s="11">
-        <v>27</v>
+        <v>30</v>
       </c>
       <c r="F247" s="9" t="s">
         <v>28</v>
@@ -7655,7 +7655,7 @@
         <v>27</v>
       </c>
       <c r="E248" s="11">
-        <v>31</v>
+        <v>9</v>
       </c>
       <c r="F248" s="9" t="s">
         <v>28</v>
@@ -7678,7 +7678,7 @@
         <v>27</v>
       </c>
       <c r="E249" s="11">
-        <v>23</v>
+        <v>20</v>
       </c>
       <c r="F249" s="9" t="s">
         <v>28</v>
@@ -7701,7 +7701,7 @@
         <v>27</v>
       </c>
       <c r="E250" s="11">
-        <v>22</v>
+        <v>29</v>
       </c>
       <c r="F250" s="9" t="s">
         <v>28</v>
@@ -7724,7 +7724,7 @@
         <v>27</v>
       </c>
       <c r="E251" s="11">
-        <v>25</v>
+        <v>31</v>
       </c>
       <c r="F251" s="9" t="s">
         <v>28</v>
@@ -7747,7 +7747,7 @@
         <v>27</v>
       </c>
       <c r="E252" s="11">
-        <v>19</v>
+        <v>14</v>
       </c>
       <c r="F252" s="9" t="s">
         <v>28</v>
@@ -7770,7 +7770,7 @@
         <v>27</v>
       </c>
       <c r="E253" s="11">
-        <v>19</v>
+        <v>26</v>
       </c>
       <c r="F253" s="9" t="s">
         <v>28</v>
@@ -7793,7 +7793,7 @@
         <v>27</v>
       </c>
       <c r="E254" s="11">
-        <v>23</v>
+        <v>29</v>
       </c>
       <c r="F254" s="9" t="s">
         <v>28</v>
@@ -7816,7 +7816,7 @@
         <v>27</v>
       </c>
       <c r="E255" s="11">
-        <v>31</v>
+        <v>13</v>
       </c>
       <c r="F255" s="9" t="s">
         <v>28</v>
@@ -7839,7 +7839,7 @@
         <v>27</v>
       </c>
       <c r="E256" s="11">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="F256" s="9" t="s">
         <v>28</v>
@@ -7862,7 +7862,7 @@
         <v>27</v>
       </c>
       <c r="E257" s="11">
-        <v>8</v>
+        <v>31</v>
       </c>
       <c r="F257" s="9" t="s">
         <v>28</v>
@@ -7885,7 +7885,7 @@
         <v>27</v>
       </c>
       <c r="E258" s="11">
-        <v>15</v>
+        <v>9</v>
       </c>
       <c r="F258" s="9" t="s">
         <v>28</v>
@@ -7908,7 +7908,7 @@
         <v>27</v>
       </c>
       <c r="E259" s="11">
-        <v>24</v>
+        <v>20</v>
       </c>
       <c r="F259" s="9" t="s">
         <v>28</v>
@@ -7931,7 +7931,7 @@
         <v>27</v>
       </c>
       <c r="E260" s="11">
-        <v>31</v>
+        <v>21</v>
       </c>
       <c r="F260" s="9" t="s">
         <v>28</v>
@@ -7954,7 +7954,7 @@
         <v>27</v>
       </c>
       <c r="E261" s="11">
-        <v>8</v>
+        <v>29</v>
       </c>
       <c r="F261" s="9" t="s">
         <v>28</v>
@@ -7977,7 +7977,7 @@
         <v>27</v>
       </c>
       <c r="E262" s="11">
-        <v>9</v>
+        <v>13</v>
       </c>
       <c r="F262" s="9" t="s">
         <v>28</v>
@@ -8000,7 +8000,7 @@
         <v>27</v>
       </c>
       <c r="E263" s="11">
-        <v>11</v>
+        <v>23</v>
       </c>
       <c r="F263" s="9" t="s">
         <v>28</v>
@@ -8023,7 +8023,7 @@
         <v>27</v>
       </c>
       <c r="E264" s="11">
-        <v>31</v>
+        <v>15</v>
       </c>
       <c r="F264" s="9" t="s">
         <v>28</v>
@@ -8046,7 +8046,7 @@
         <v>27</v>
       </c>
       <c r="E265" s="11">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="F265" s="9" t="s">
         <v>28</v>
@@ -8069,7 +8069,7 @@
         <v>27</v>
       </c>
       <c r="E266" s="11">
-        <v>25</v>
+        <v>28</v>
       </c>
       <c r="F266" s="9" t="s">
         <v>28</v>
@@ -8092,7 +8092,7 @@
         <v>27</v>
       </c>
       <c r="E267" s="11">
-        <v>19</v>
+        <v>13</v>
       </c>
       <c r="F267" s="9" t="s">
         <v>28</v>
@@ -8115,7 +8115,7 @@
         <v>27</v>
       </c>
       <c r="E268" s="11">
-        <v>18</v>
+        <v>26</v>
       </c>
       <c r="F268" s="9" t="s">
         <v>28</v>
@@ -8138,7 +8138,7 @@
         <v>27</v>
       </c>
       <c r="E269" s="11">
-        <v>15</v>
+        <v>23</v>
       </c>
       <c r="F269" s="9" t="s">
         <v>28</v>
@@ -8161,7 +8161,7 @@
         <v>27</v>
       </c>
       <c r="E270" s="11">
-        <v>23</v>
+        <v>15</v>
       </c>
       <c r="F270" s="9" t="s">
         <v>28</v>
@@ -8184,7 +8184,7 @@
         <v>27</v>
       </c>
       <c r="E271" s="11">
-        <v>10</v>
+        <v>30</v>
       </c>
       <c r="F271" s="9" t="s">
         <v>28</v>
@@ -8207,7 +8207,7 @@
         <v>27</v>
       </c>
       <c r="E272" s="11">
-        <v>25</v>
+        <v>21</v>
       </c>
       <c r="F272" s="9" t="s">
         <v>28</v>
@@ -8230,7 +8230,7 @@
         <v>27</v>
       </c>
       <c r="E273" s="11">
-        <v>25</v>
+        <v>28</v>
       </c>
       <c r="F273" s="9" t="s">
         <v>28</v>
@@ -8253,7 +8253,7 @@
         <v>27</v>
       </c>
       <c r="E274" s="11">
-        <v>14</v>
+        <v>29</v>
       </c>
       <c r="F274" s="9" t="s">
         <v>28</v>
@@ -8276,7 +8276,7 @@
         <v>27</v>
       </c>
       <c r="E275" s="11">
-        <v>8</v>
+        <v>25</v>
       </c>
       <c r="F275" s="9" t="s">
         <v>28</v>
@@ -8299,7 +8299,7 @@
         <v>27</v>
       </c>
       <c r="E276" s="11">
-        <v>31</v>
+        <v>20</v>
       </c>
       <c r="F276" s="9" t="s">
         <v>28</v>
@@ -8322,7 +8322,7 @@
         <v>27</v>
       </c>
       <c r="E277" s="11">
-        <v>10</v>
+        <v>22</v>
       </c>
       <c r="F277" s="9" t="s">
         <v>28</v>
@@ -8345,7 +8345,7 @@
         <v>27</v>
       </c>
       <c r="E278" s="11">
-        <v>17</v>
+        <v>30</v>
       </c>
       <c r="F278" s="9" t="s">
         <v>28</v>
@@ -8368,7 +8368,7 @@
         <v>27</v>
       </c>
       <c r="E279" s="11">
-        <v>18</v>
+        <v>21</v>
       </c>
       <c r="F279" s="9" t="s">
         <v>28</v>
@@ -8391,7 +8391,7 @@
         <v>27</v>
       </c>
       <c r="E280" s="11">
-        <v>18</v>
+        <v>16</v>
       </c>
       <c r="F280" s="9" t="s">
         <v>28</v>
@@ -8414,7 +8414,7 @@
         <v>27</v>
       </c>
       <c r="E281" s="11">
-        <v>17</v>
+        <v>31</v>
       </c>
       <c r="F281" s="9" t="s">
         <v>28</v>
@@ -8437,7 +8437,7 @@
         <v>27</v>
       </c>
       <c r="E282" s="11">
-        <v>15</v>
+        <v>10</v>
       </c>
       <c r="F282" s="9" t="s">
         <v>28</v>
@@ -8460,7 +8460,7 @@
         <v>27</v>
       </c>
       <c r="E283" s="11">
-        <v>24</v>
+        <v>11</v>
       </c>
       <c r="F283" s="9" t="s">
         <v>28</v>
@@ -8483,7 +8483,7 @@
         <v>27</v>
       </c>
       <c r="E284" s="11">
-        <v>17</v>
+        <v>22</v>
       </c>
       <c r="F284" s="9" t="s">
         <v>28</v>
@@ -8506,7 +8506,7 @@
         <v>27</v>
       </c>
       <c r="E285" s="11">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="F285" s="9" t="s">
         <v>28</v>
@@ -8529,7 +8529,7 @@
         <v>27</v>
       </c>
       <c r="E286" s="11">
-        <v>24</v>
+        <v>26</v>
       </c>
       <c r="F286" s="9" t="s">
         <v>28</v>
@@ -8552,7 +8552,7 @@
         <v>27</v>
       </c>
       <c r="E287" s="11">
-        <v>15</v>
+        <v>25</v>
       </c>
       <c r="F287" s="9" t="s">
         <v>28</v>
@@ -8598,7 +8598,7 @@
         <v>27</v>
       </c>
       <c r="E289" s="11">
-        <v>23</v>
+        <v>21</v>
       </c>
       <c r="F289" s="9" t="s">
         <v>28</v>
@@ -8621,7 +8621,7 @@
         <v>27</v>
       </c>
       <c r="E290" s="11">
-        <v>22</v>
+        <v>13</v>
       </c>
       <c r="F290" s="9" t="s">
         <v>28</v>
@@ -8644,7 +8644,7 @@
         <v>27</v>
       </c>
       <c r="E291" s="11">
-        <v>31</v>
+        <v>13</v>
       </c>
       <c r="F291" s="9" t="s">
         <v>28</v>
@@ -8667,7 +8667,7 @@
         <v>27</v>
       </c>
       <c r="E292" s="11">
-        <v>14</v>
+        <v>11</v>
       </c>
       <c r="F292" s="9" t="s">
         <v>28</v>
@@ -8690,7 +8690,7 @@
         <v>27</v>
       </c>
       <c r="E293" s="11">
-        <v>13</v>
+        <v>21</v>
       </c>
       <c r="F293" s="9" t="s">
         <v>28</v>
@@ -8713,7 +8713,7 @@
         <v>27</v>
       </c>
       <c r="E294" s="11">
-        <v>27</v>
+        <v>8</v>
       </c>
       <c r="F294" s="9" t="s">
         <v>28</v>
@@ -8736,7 +8736,7 @@
         <v>27</v>
       </c>
       <c r="E295" s="11">
-        <v>30</v>
+        <v>8</v>
       </c>
       <c r="F295" s="9" t="s">
         <v>28</v>
@@ -8759,7 +8759,7 @@
         <v>27</v>
       </c>
       <c r="E296" s="11">
-        <v>30</v>
+        <v>15</v>
       </c>
       <c r="F296" s="9" t="s">
         <v>28</v>
@@ -8782,7 +8782,7 @@
         <v>27</v>
       </c>
       <c r="E297" s="11">
-        <v>10</v>
+        <v>24</v>
       </c>
       <c r="F297" s="9" t="s">
         <v>28</v>
@@ -8805,7 +8805,7 @@
         <v>27</v>
       </c>
       <c r="E298" s="11">
-        <v>13</v>
+        <v>25</v>
       </c>
       <c r="F298" s="9" t="s">
         <v>28</v>
@@ -8828,7 +8828,7 @@
         <v>27</v>
       </c>
       <c r="E299" s="11">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="F299" s="9" t="s">
         <v>28</v>
@@ -8851,7 +8851,7 @@
         <v>27</v>
       </c>
       <c r="E300" s="11">
-        <v>30</v>
+        <v>14</v>
       </c>
       <c r="F300" s="9" t="s">
         <v>28</v>
@@ -8874,7 +8874,7 @@
         <v>27</v>
       </c>
       <c r="E301" s="11">
-        <v>20</v>
+        <v>26</v>
       </c>
       <c r="F301" s="9" t="s">
         <v>28</v>
@@ -8897,7 +8897,7 @@
         <v>27</v>
       </c>
       <c r="E302" s="11">
-        <v>24</v>
+        <v>22</v>
       </c>
       <c r="F302" s="9" t="s">
         <v>28</v>
@@ -8920,7 +8920,7 @@
         <v>27</v>
       </c>
       <c r="E303" s="11">
-        <v>26</v>
+        <v>10</v>
       </c>
       <c r="F303" s="9" t="s">
         <v>28</v>
@@ -8943,7 +8943,7 @@
         <v>27</v>
       </c>
       <c r="E304" s="11">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="F304" s="9" t="s">
         <v>28</v>
@@ -8966,7 +8966,7 @@
         <v>27</v>
       </c>
       <c r="E305" s="11">
-        <v>25</v>
+        <v>10</v>
       </c>
       <c r="F305" s="9" t="s">
         <v>28</v>
@@ -8989,7 +8989,7 @@
         <v>27</v>
       </c>
       <c r="E306" s="11">
-        <v>17</v>
+        <v>22</v>
       </c>
       <c r="F306" s="9" t="s">
         <v>28</v>
@@ -9012,7 +9012,7 @@
         <v>27</v>
       </c>
       <c r="E307" s="11">
-        <v>18</v>
+        <v>20</v>
       </c>
       <c r="F307" s="9" t="s">
         <v>28</v>
@@ -9035,7 +9035,7 @@
         <v>27</v>
       </c>
       <c r="E308" s="11">
-        <v>23</v>
+        <v>29</v>
       </c>
       <c r="F308" s="9" t="s">
         <v>28</v>
@@ -9058,7 +9058,7 @@
         <v>27</v>
       </c>
       <c r="E309" s="11">
-        <v>20</v>
+        <v>24</v>
       </c>
       <c r="F309" s="9" t="s">
         <v>28</v>
@@ -9081,7 +9081,7 @@
         <v>27</v>
       </c>
       <c r="E310" s="11">
-        <v>11</v>
+        <v>31</v>
       </c>
       <c r="F310" s="9" t="s">
         <v>28</v>
@@ -9104,7 +9104,7 @@
         <v>27</v>
       </c>
       <c r="E311" s="11">
-        <v>17</v>
+        <v>25</v>
       </c>
       <c r="F311" s="9" t="s">
         <v>28</v>
@@ -9127,7 +9127,7 @@
         <v>27</v>
       </c>
       <c r="E312" s="11">
-        <v>16</v>
+        <v>13</v>
       </c>
       <c r="F312" s="9" t="s">
         <v>28</v>
@@ -9150,7 +9150,7 @@
         <v>27</v>
       </c>
       <c r="E313" s="11">
-        <v>15</v>
+        <v>11</v>
       </c>
       <c r="F313" s="9" t="s">
         <v>28</v>
@@ -9173,7 +9173,7 @@
         <v>27</v>
       </c>
       <c r="E314" s="11">
-        <v>19</v>
+        <v>16</v>
       </c>
       <c r="F314" s="9" t="s">
         <v>28</v>
@@ -9196,7 +9196,7 @@
         <v>27</v>
       </c>
       <c r="E315" s="11">
-        <v>24</v>
+        <v>17</v>
       </c>
       <c r="F315" s="9" t="s">
         <v>28</v>
@@ -9219,7 +9219,7 @@
         <v>27</v>
       </c>
       <c r="E316" s="11">
-        <v>21</v>
+        <v>14</v>
       </c>
       <c r="F316" s="9" t="s">
         <v>28</v>
@@ -9242,7 +9242,7 @@
         <v>27</v>
       </c>
       <c r="E317" s="11">
-        <v>31</v>
+        <v>26</v>
       </c>
       <c r="F317" s="9" t="s">
         <v>28</v>
@@ -9265,7 +9265,7 @@
         <v>27</v>
       </c>
       <c r="E318" s="11">
-        <v>28</v>
+        <v>9</v>
       </c>
       <c r="F318" s="9" t="s">
         <v>28</v>
@@ -9288,7 +9288,7 @@
         <v>27</v>
       </c>
       <c r="E319" s="11">
-        <v>20</v>
+        <v>15</v>
       </c>
       <c r="F319" s="9" t="s">
         <v>28</v>
@@ -9311,7 +9311,7 @@
         <v>27</v>
       </c>
       <c r="E320" s="11">
-        <v>17</v>
+        <v>10</v>
       </c>
       <c r="F320" s="9" t="s">
         <v>28</v>
@@ -9334,7 +9334,7 @@
         <v>27</v>
       </c>
       <c r="E321" s="11">
-        <v>11</v>
+        <v>25</v>
       </c>
       <c r="F321" s="9" t="s">
         <v>28</v>
@@ -9357,7 +9357,7 @@
         <v>27</v>
       </c>
       <c r="E322" s="11">
-        <v>22</v>
+        <v>11</v>
       </c>
       <c r="F322" s="9" t="s">
         <v>28</v>
@@ -9380,7 +9380,7 @@
         <v>27</v>
       </c>
       <c r="E323" s="11">
-        <v>18</v>
+        <v>15</v>
       </c>
       <c r="F323" s="9" t="s">
         <v>28</v>
@@ -9403,7 +9403,7 @@
         <v>27</v>
       </c>
       <c r="E324" s="11">
-        <v>21</v>
+        <v>13</v>
       </c>
       <c r="F324" s="9" t="s">
         <v>28</v>
@@ -9426,7 +9426,7 @@
         <v>27</v>
       </c>
       <c r="E325" s="11">
-        <v>12</v>
+        <v>16</v>
       </c>
       <c r="F325" s="9" t="s">
         <v>28</v>
@@ -9449,7 +9449,7 @@
         <v>27</v>
       </c>
       <c r="E326" s="11">
-        <v>30</v>
+        <v>24</v>
       </c>
       <c r="F326" s="9" t="s">
         <v>28</v>
@@ -9472,7 +9472,7 @@
         <v>27</v>
       </c>
       <c r="E327" s="11">
-        <v>28</v>
+        <v>9</v>
       </c>
       <c r="F327" s="9" t="s">
         <v>28</v>
@@ -9495,7 +9495,7 @@
         <v>27</v>
       </c>
       <c r="E328" s="11">
-        <v>8</v>
+        <v>15</v>
       </c>
       <c r="F328" s="9" t="s">
         <v>28</v>
@@ -9518,7 +9518,7 @@
         <v>27</v>
       </c>
       <c r="E329" s="11">
-        <v>30</v>
+        <v>14</v>
       </c>
       <c r="F329" s="9" t="s">
         <v>28</v>
@@ -9541,7 +9541,7 @@
         <v>27</v>
       </c>
       <c r="E330" s="11">
-        <v>10</v>
+        <v>30</v>
       </c>
       <c r="F330" s="9" t="s">
         <v>28</v>
@@ -9564,7 +9564,7 @@
         <v>27</v>
       </c>
       <c r="E331" s="11">
-        <v>29</v>
+        <v>27</v>
       </c>
       <c r="F331" s="9" t="s">
         <v>28</v>
@@ -9587,7 +9587,7 @@
         <v>27</v>
       </c>
       <c r="E332" s="11">
-        <v>21</v>
+        <v>23</v>
       </c>
       <c r="F332" s="9" t="s">
         <v>28</v>
@@ -9610,7 +9610,7 @@
         <v>27</v>
       </c>
       <c r="E333" s="11">
-        <v>15</v>
+        <v>28</v>
       </c>
       <c r="F333" s="9" t="s">
         <v>28</v>
@@ -9633,7 +9633,7 @@
         <v>27</v>
       </c>
       <c r="E334" s="11">
-        <v>13</v>
+        <v>29</v>
       </c>
       <c r="F334" s="9" t="s">
         <v>28</v>
@@ -9656,7 +9656,7 @@
         <v>27</v>
       </c>
       <c r="E335" s="11">
-        <v>8</v>
+        <v>20</v>
       </c>
       <c r="F335" s="9" t="s">
         <v>28</v>
@@ -9679,7 +9679,7 @@
         <v>27</v>
       </c>
       <c r="E336" s="11">
-        <v>27</v>
+        <v>13</v>
       </c>
       <c r="F336" s="9" t="s">
         <v>28</v>
@@ -9702,7 +9702,7 @@
         <v>27</v>
       </c>
       <c r="E337" s="11">
-        <v>28</v>
+        <v>21</v>
       </c>
       <c r="F337" s="9" t="s">
         <v>28</v>
@@ -9725,7 +9725,7 @@
         <v>27</v>
       </c>
       <c r="E338" s="11">
-        <v>22</v>
+        <v>24</v>
       </c>
       <c r="F338" s="9" t="s">
         <v>28</v>
@@ -9748,7 +9748,7 @@
         <v>27</v>
       </c>
       <c r="E339" s="11">
-        <v>24</v>
+        <v>15</v>
       </c>
       <c r="F339" s="9" t="s">
         <v>28</v>
@@ -9771,7 +9771,7 @@
         <v>27</v>
       </c>
       <c r="E340" s="11">
-        <v>22</v>
+        <v>27</v>
       </c>
       <c r="F340" s="9" t="s">
         <v>28</v>
@@ -9794,7 +9794,7 @@
         <v>27</v>
       </c>
       <c r="E341" s="11">
-        <v>19</v>
+        <v>21</v>
       </c>
       <c r="F341" s="9" t="s">
         <v>28</v>
@@ -9817,7 +9817,7 @@
         <v>27</v>
       </c>
       <c r="E342" s="11">
-        <v>21</v>
+        <v>18</v>
       </c>
       <c r="F342" s="9" t="s">
         <v>28</v>
@@ -9863,7 +9863,7 @@
         <v>27</v>
       </c>
       <c r="E344" s="11">
-        <v>24</v>
+        <v>27</v>
       </c>
       <c r="F344" s="9" t="s">
         <v>28</v>
@@ -9886,7 +9886,7 @@
         <v>27</v>
       </c>
       <c r="E345" s="11">
-        <v>15</v>
+        <v>12</v>
       </c>
       <c r="F345" s="9" t="s">
         <v>28</v>
@@ -9909,7 +9909,7 @@
         <v>27</v>
       </c>
       <c r="E346" s="11">
-        <v>24</v>
+        <v>13</v>
       </c>
       <c r="F346" s="9" t="s">
         <v>28</v>
@@ -9932,7 +9932,7 @@
         <v>27</v>
       </c>
       <c r="E347" s="11">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="F347" s="9" t="s">
         <v>28</v>
@@ -9955,7 +9955,7 @@
         <v>27</v>
       </c>
       <c r="E348" s="11">
-        <v>14</v>
+        <v>24</v>
       </c>
       <c r="F348" s="9" t="s">
         <v>28</v>
@@ -9978,7 +9978,7 @@
         <v>27</v>
       </c>
       <c r="E349" s="11">
-        <v>29</v>
+        <v>16</v>
       </c>
       <c r="F349" s="9" t="s">
         <v>28</v>
@@ -10024,7 +10024,7 @@
         <v>27</v>
       </c>
       <c r="E351" s="11">
-        <v>23</v>
+        <v>20</v>
       </c>
       <c r="F351" s="9" t="s">
         <v>28</v>
@@ -10047,7 +10047,7 @@
         <v>27</v>
       </c>
       <c r="E352" s="11">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="F352" s="9" t="s">
         <v>28</v>
@@ -10070,7 +10070,7 @@
         <v>27</v>
       </c>
       <c r="E353" s="11">
-        <v>17</v>
+        <v>15</v>
       </c>
       <c r="F353" s="9" t="s">
         <v>28</v>
@@ -10093,7 +10093,7 @@
         <v>27</v>
       </c>
       <c r="E354" s="11">
-        <v>14</v>
+        <v>26</v>
       </c>
       <c r="F354" s="9" t="s">
         <v>28</v>
@@ -10116,7 +10116,7 @@
         <v>27</v>
       </c>
       <c r="E355" s="11">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="F355" s="9" t="s">
         <v>28</v>
@@ -10139,7 +10139,7 @@
         <v>27</v>
       </c>
       <c r="E356" s="11">
-        <v>25</v>
+        <v>29</v>
       </c>
       <c r="F356" s="9" t="s">
         <v>28</v>
@@ -10162,7 +10162,7 @@
         <v>27</v>
       </c>
       <c r="E357" s="11">
-        <v>15</v>
+        <v>25</v>
       </c>
       <c r="F357" s="9" t="s">
         <v>28</v>
@@ -10185,7 +10185,7 @@
         <v>27</v>
       </c>
       <c r="E358" s="11">
-        <v>31</v>
+        <v>27</v>
       </c>
       <c r="F358" s="9" t="s">
         <v>28</v>
@@ -10208,7 +10208,7 @@
         <v>27</v>
       </c>
       <c r="E359" s="11">
-        <v>12</v>
+        <v>23</v>
       </c>
       <c r="F359" s="9" t="s">
         <v>28</v>
@@ -10231,7 +10231,7 @@
         <v>27</v>
       </c>
       <c r="E360" s="11">
-        <v>30</v>
+        <v>19</v>
       </c>
       <c r="F360" s="9" t="s">
         <v>28</v>
@@ -10277,7 +10277,7 @@
         <v>27</v>
       </c>
       <c r="E362" s="11">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="F362" s="9" t="s">
         <v>28</v>
@@ -10300,7 +10300,7 @@
         <v>27</v>
       </c>
       <c r="E363" s="11">
-        <v>14</v>
+        <v>23</v>
       </c>
       <c r="F363" s="9" t="s">
         <v>28</v>
@@ -10323,7 +10323,7 @@
         <v>27</v>
       </c>
       <c r="E364" s="11">
-        <v>14</v>
+        <v>28</v>
       </c>
       <c r="F364" s="9" t="s">
         <v>28</v>
@@ -10346,7 +10346,7 @@
         <v>27</v>
       </c>
       <c r="E365" s="11">
-        <v>22</v>
+        <v>17</v>
       </c>
       <c r="F365" s="9" t="s">
         <v>28</v>
@@ -10369,7 +10369,7 @@
         <v>27</v>
       </c>
       <c r="E366" s="11">
-        <v>21</v>
+        <v>30</v>
       </c>
       <c r="F366" s="9" t="s">
         <v>28</v>
@@ -10392,7 +10392,7 @@
         <v>27</v>
       </c>
       <c r="E367" s="11">
-        <v>10</v>
+        <v>15</v>
       </c>
       <c r="F367" s="9" t="s">
         <v>28</v>
@@ -10415,7 +10415,7 @@
         <v>27</v>
       </c>
       <c r="E368" s="11">
-        <v>31</v>
+        <v>16</v>
       </c>
       <c r="F368" s="9" t="s">
         <v>28</v>
@@ -10438,7 +10438,7 @@
         <v>27</v>
       </c>
       <c r="E369" s="11">
-        <v>13</v>
+        <v>25</v>
       </c>
       <c r="F369" s="9" t="s">
         <v>28</v>
@@ -10461,7 +10461,7 @@
         <v>27</v>
       </c>
       <c r="E370" s="11">
-        <v>18</v>
+        <v>30</v>
       </c>
       <c r="F370" s="9" t="s">
         <v>28</v>
@@ -10484,7 +10484,7 @@
         <v>27</v>
       </c>
       <c r="E371" s="11">
-        <v>27</v>
+        <v>29</v>
       </c>
       <c r="F371" s="9" t="s">
         <v>28</v>
@@ -10507,7 +10507,7 @@
         <v>27</v>
       </c>
       <c r="E372" s="11">
-        <v>10</v>
+        <v>30</v>
       </c>
       <c r="F372" s="9" t="s">
         <v>28</v>
@@ -10530,7 +10530,7 @@
         <v>27</v>
       </c>
       <c r="E373" s="11">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="F373" s="9" t="s">
         <v>28</v>
@@ -10553,7 +10553,7 @@
         <v>27</v>
       </c>
       <c r="E374" s="11">
-        <v>12</v>
+        <v>24</v>
       </c>
       <c r="F374" s="9" t="s">
         <v>28</v>
@@ -10576,7 +10576,7 @@
         <v>27</v>
       </c>
       <c r="E375" s="11">
-        <v>22</v>
+        <v>24</v>
       </c>
       <c r="F375" s="9" t="s">
         <v>28</v>
@@ -10599,7 +10599,7 @@
         <v>27</v>
       </c>
       <c r="E376" s="11">
-        <v>21</v>
+        <v>13</v>
       </c>
       <c r="F376" s="9" t="s">
         <v>28</v>
@@ -10622,7 +10622,7 @@
         <v>27</v>
       </c>
       <c r="E377" s="11">
-        <v>13</v>
+        <v>19</v>
       </c>
       <c r="F377" s="9" t="s">
         <v>28</v>
@@ -10668,7 +10668,7 @@
         <v>27</v>
       </c>
       <c r="E379" s="11">
-        <v>17</v>
+        <v>28</v>
       </c>
       <c r="F379" s="9" t="s">
         <v>28</v>
@@ -10691,7 +10691,7 @@
         <v>27</v>
       </c>
       <c r="E380" s="11">
-        <v>27</v>
+        <v>31</v>
       </c>
       <c r="F380" s="9" t="s">
         <v>28</v>
@@ -10714,7 +10714,7 @@
         <v>27</v>
       </c>
       <c r="E381" s="11">
-        <v>12</v>
+        <v>21</v>
       </c>
       <c r="F381" s="9" t="s">
         <v>28</v>
@@ -10760,7 +10760,7 @@
         <v>27</v>
       </c>
       <c r="E383" s="11">
-        <v>27</v>
+        <v>29</v>
       </c>
       <c r="F383" s="9" t="s">
         <v>28</v>
@@ -10783,7 +10783,7 @@
         <v>27</v>
       </c>
       <c r="E384" s="11">
-        <v>23</v>
+        <v>14</v>
       </c>
       <c r="F384" s="9" t="s">
         <v>28</v>
@@ -10806,7 +10806,7 @@
         <v>27</v>
       </c>
       <c r="E385" s="11">
-        <v>25</v>
+        <v>12</v>
       </c>
       <c r="F385" s="9" t="s">
         <v>28</v>
@@ -10829,7 +10829,7 @@
         <v>27</v>
       </c>
       <c r="E386" s="11">
-        <v>9</v>
+        <v>20</v>
       </c>
       <c r="F386" s="9" t="s">
         <v>28</v>
@@ -10852,7 +10852,7 @@
         <v>27</v>
       </c>
       <c r="E387" s="11">
-        <v>28</v>
+        <v>31</v>
       </c>
       <c r="F387" s="9" t="s">
         <v>28</v>
@@ -10875,7 +10875,7 @@
         <v>27</v>
       </c>
       <c r="E388" s="11">
-        <v>9</v>
+        <v>26</v>
       </c>
       <c r="F388" s="9" t="s">
         <v>28</v>
@@ -10898,7 +10898,7 @@
         <v>27</v>
       </c>
       <c r="E389" s="11">
-        <v>16</v>
+        <v>18</v>
       </c>
       <c r="F389" s="9" t="s">
         <v>28</v>
@@ -10921,7 +10921,7 @@
         <v>27</v>
       </c>
       <c r="E390" s="11">
-        <v>26</v>
+        <v>10</v>
       </c>
       <c r="F390" s="9" t="s">
         <v>28</v>
@@ -10944,7 +10944,7 @@
         <v>27</v>
       </c>
       <c r="E391" s="11">
-        <v>20</v>
+        <v>18</v>
       </c>
       <c r="F391" s="9" t="s">
         <v>28</v>
@@ -10967,7 +10967,7 @@
         <v>27</v>
       </c>
       <c r="E392" s="11">
-        <v>25</v>
+        <v>18</v>
       </c>
       <c r="F392" s="9" t="s">
         <v>28</v>
@@ -10990,7 +10990,7 @@
         <v>27</v>
       </c>
       <c r="E393" s="11">
-        <v>18</v>
+        <v>8</v>
       </c>
       <c r="F393" s="9" t="s">
         <v>28</v>
@@ -11013,7 +11013,7 @@
         <v>27</v>
       </c>
       <c r="E394" s="11">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="F394" s="9" t="s">
         <v>28</v>
@@ -11036,7 +11036,7 @@
         <v>27</v>
       </c>
       <c r="E395" s="11">
-        <v>24</v>
+        <v>11</v>
       </c>
       <c r="F395" s="9" t="s">
         <v>28</v>
@@ -11059,7 +11059,7 @@
         <v>27</v>
       </c>
       <c r="E396" s="11">
-        <v>26</v>
+        <v>15</v>
       </c>
       <c r="F396" s="9" t="s">
         <v>28</v>
@@ -11082,7 +11082,7 @@
         <v>27</v>
       </c>
       <c r="E397" s="11">
-        <v>25</v>
+        <v>28</v>
       </c>
       <c r="F397" s="9" t="s">
         <v>28</v>
@@ -11105,7 +11105,7 @@
         <v>27</v>
       </c>
       <c r="E398" s="11">
-        <v>17</v>
+        <v>28</v>
       </c>
       <c r="F398" s="9" t="s">
         <v>28</v>
@@ -11128,7 +11128,7 @@
         <v>27</v>
       </c>
       <c r="E399" s="11">
-        <v>28</v>
+        <v>17</v>
       </c>
       <c r="F399" s="9" t="s">
         <v>28</v>
@@ -11151,7 +11151,7 @@
         <v>27</v>
       </c>
       <c r="E400" s="11">
-        <v>24</v>
+        <v>20</v>
       </c>
       <c r="F400" s="9" t="s">
         <v>28</v>
@@ -11174,7 +11174,7 @@
         <v>27</v>
       </c>
       <c r="E401" s="11">
-        <v>25</v>
+        <v>17</v>
       </c>
       <c r="F401" s="9" t="s">
         <v>28</v>

</xml_diff>

<commit_message>
fix(profile): reset user stats (Neighbors Helped, Total Earned, Profile Views, Borrowing) to default to 0 until actual transactions occur
</commit_message>
<xml_diff>
--- a/all-test-reports/selenium/selenium_e2e_test_report.xlsx
+++ b/all-test-reports/selenium/selenium_e2e_test_report.xlsx
@@ -35,7 +35,7 @@
     <t>Execution Date</t>
   </si>
   <si>
-    <t>28/7/2026, 10:59:38 am</t>
+    <t>28/7/2026, 11:08:29 am</t>
   </si>
   <si>
     <t>Browser / Mode</t>
@@ -98,7 +98,7 @@
     <t>PASS</t>
   </si>
   <si>
-    <t>10:59:38 am</t>
+    <t>11:08:29 am</t>
   </si>
   <si>
     <t>N/A</t>
@@ -1997,7 +1997,7 @@
         <v>27</v>
       </c>
       <c r="E2" s="11">
-        <v>23</v>
+        <v>17</v>
       </c>
       <c r="F2" s="9" t="s">
         <v>28</v>
@@ -2020,7 +2020,7 @@
         <v>27</v>
       </c>
       <c r="E3" s="11">
-        <v>26</v>
+        <v>12</v>
       </c>
       <c r="F3" s="9" t="s">
         <v>28</v>
@@ -2043,7 +2043,7 @@
         <v>27</v>
       </c>
       <c r="E4" s="11">
-        <v>15</v>
+        <v>22</v>
       </c>
       <c r="F4" s="9" t="s">
         <v>28</v>
@@ -2066,7 +2066,7 @@
         <v>27</v>
       </c>
       <c r="E5" s="11">
-        <v>24</v>
+        <v>21</v>
       </c>
       <c r="F5" s="9" t="s">
         <v>28</v>
@@ -2089,7 +2089,7 @@
         <v>27</v>
       </c>
       <c r="E6" s="11">
-        <v>17</v>
+        <v>27</v>
       </c>
       <c r="F6" s="9" t="s">
         <v>28</v>
@@ -2158,7 +2158,7 @@
         <v>27</v>
       </c>
       <c r="E9" s="11">
-        <v>23</v>
+        <v>11</v>
       </c>
       <c r="F9" s="9" t="s">
         <v>28</v>
@@ -2181,7 +2181,7 @@
         <v>27</v>
       </c>
       <c r="E10" s="11">
-        <v>19</v>
+        <v>23</v>
       </c>
       <c r="F10" s="9" t="s">
         <v>28</v>
@@ -2204,7 +2204,7 @@
         <v>27</v>
       </c>
       <c r="E11" s="11">
-        <v>12</v>
+        <v>31</v>
       </c>
       <c r="F11" s="9" t="s">
         <v>28</v>
@@ -2227,7 +2227,7 @@
         <v>27</v>
       </c>
       <c r="E12" s="11">
-        <v>13</v>
+        <v>17</v>
       </c>
       <c r="F12" s="9" t="s">
         <v>28</v>
@@ -2250,7 +2250,7 @@
         <v>27</v>
       </c>
       <c r="E13" s="11">
-        <v>16</v>
+        <v>13</v>
       </c>
       <c r="F13" s="9" t="s">
         <v>28</v>
@@ -2273,7 +2273,7 @@
         <v>27</v>
       </c>
       <c r="E14" s="11">
-        <v>19</v>
+        <v>21</v>
       </c>
       <c r="F14" s="9" t="s">
         <v>28</v>
@@ -2296,7 +2296,7 @@
         <v>27</v>
       </c>
       <c r="E15" s="11">
-        <v>28</v>
+        <v>22</v>
       </c>
       <c r="F15" s="9" t="s">
         <v>28</v>
@@ -2319,7 +2319,7 @@
         <v>27</v>
       </c>
       <c r="E16" s="11">
-        <v>24</v>
+        <v>11</v>
       </c>
       <c r="F16" s="9" t="s">
         <v>28</v>
@@ -2342,7 +2342,7 @@
         <v>27</v>
       </c>
       <c r="E17" s="11">
-        <v>22</v>
+        <v>29</v>
       </c>
       <c r="F17" s="9" t="s">
         <v>28</v>
@@ -2365,7 +2365,7 @@
         <v>27</v>
       </c>
       <c r="E18" s="11">
-        <v>28</v>
+        <v>18</v>
       </c>
       <c r="F18" s="9" t="s">
         <v>28</v>
@@ -2388,7 +2388,7 @@
         <v>27</v>
       </c>
       <c r="E19" s="11">
-        <v>15</v>
+        <v>11</v>
       </c>
       <c r="F19" s="9" t="s">
         <v>28</v>
@@ -2411,7 +2411,7 @@
         <v>27</v>
       </c>
       <c r="E20" s="11">
-        <v>18</v>
+        <v>25</v>
       </c>
       <c r="F20" s="9" t="s">
         <v>28</v>
@@ -2457,7 +2457,7 @@
         <v>27</v>
       </c>
       <c r="E22" s="11">
-        <v>10</v>
+        <v>29</v>
       </c>
       <c r="F22" s="9" t="s">
         <v>28</v>
@@ -2480,7 +2480,7 @@
         <v>27</v>
       </c>
       <c r="E23" s="11">
-        <v>24</v>
+        <v>26</v>
       </c>
       <c r="F23" s="9" t="s">
         <v>28</v>
@@ -2503,7 +2503,7 @@
         <v>27</v>
       </c>
       <c r="E24" s="11">
-        <v>27</v>
+        <v>8</v>
       </c>
       <c r="F24" s="9" t="s">
         <v>28</v>
@@ -2526,7 +2526,7 @@
         <v>27</v>
       </c>
       <c r="E25" s="11">
-        <v>11</v>
+        <v>19</v>
       </c>
       <c r="F25" s="9" t="s">
         <v>28</v>
@@ -2549,7 +2549,7 @@
         <v>27</v>
       </c>
       <c r="E26" s="11">
-        <v>21</v>
+        <v>13</v>
       </c>
       <c r="F26" s="9" t="s">
         <v>28</v>
@@ -2572,7 +2572,7 @@
         <v>27</v>
       </c>
       <c r="E27" s="11">
-        <v>16</v>
+        <v>24</v>
       </c>
       <c r="F27" s="9" t="s">
         <v>28</v>
@@ -2595,7 +2595,7 @@
         <v>27</v>
       </c>
       <c r="E28" s="11">
-        <v>31</v>
+        <v>28</v>
       </c>
       <c r="F28" s="9" t="s">
         <v>28</v>
@@ -2618,7 +2618,7 @@
         <v>27</v>
       </c>
       <c r="E29" s="11">
-        <v>24</v>
+        <v>22</v>
       </c>
       <c r="F29" s="9" t="s">
         <v>28</v>
@@ -2641,7 +2641,7 @@
         <v>27</v>
       </c>
       <c r="E30" s="11">
-        <v>15</v>
+        <v>11</v>
       </c>
       <c r="F30" s="9" t="s">
         <v>28</v>
@@ -2664,7 +2664,7 @@
         <v>27</v>
       </c>
       <c r="E31" s="11">
-        <v>18</v>
+        <v>21</v>
       </c>
       <c r="F31" s="9" t="s">
         <v>28</v>
@@ -2687,7 +2687,7 @@
         <v>27</v>
       </c>
       <c r="E32" s="11">
-        <v>24</v>
+        <v>16</v>
       </c>
       <c r="F32" s="9" t="s">
         <v>28</v>
@@ -2710,7 +2710,7 @@
         <v>27</v>
       </c>
       <c r="E33" s="11">
-        <v>22</v>
+        <v>26</v>
       </c>
       <c r="F33" s="9" t="s">
         <v>28</v>
@@ -2733,7 +2733,7 @@
         <v>27</v>
       </c>
       <c r="E34" s="11">
-        <v>21</v>
+        <v>29</v>
       </c>
       <c r="F34" s="9" t="s">
         <v>28</v>
@@ -2756,7 +2756,7 @@
         <v>27</v>
       </c>
       <c r="E35" s="11">
-        <v>30</v>
+        <v>11</v>
       </c>
       <c r="F35" s="9" t="s">
         <v>28</v>
@@ -2779,7 +2779,7 @@
         <v>27</v>
       </c>
       <c r="E36" s="11">
-        <v>15</v>
+        <v>11</v>
       </c>
       <c r="F36" s="9" t="s">
         <v>28</v>
@@ -2802,7 +2802,7 @@
         <v>27</v>
       </c>
       <c r="E37" s="11">
-        <v>27</v>
+        <v>9</v>
       </c>
       <c r="F37" s="9" t="s">
         <v>28</v>
@@ -2825,7 +2825,7 @@
         <v>27</v>
       </c>
       <c r="E38" s="11">
-        <v>8</v>
+        <v>12</v>
       </c>
       <c r="F38" s="9" t="s">
         <v>28</v>
@@ -2848,7 +2848,7 @@
         <v>27</v>
       </c>
       <c r="E39" s="11">
-        <v>10</v>
+        <v>15</v>
       </c>
       <c r="F39" s="9" t="s">
         <v>28</v>
@@ -2871,7 +2871,7 @@
         <v>27</v>
       </c>
       <c r="E40" s="11">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="F40" s="9" t="s">
         <v>28</v>
@@ -2894,7 +2894,7 @@
         <v>27</v>
       </c>
       <c r="E41" s="11">
-        <v>23</v>
+        <v>16</v>
       </c>
       <c r="F41" s="9" t="s">
         <v>28</v>
@@ -2917,7 +2917,7 @@
         <v>27</v>
       </c>
       <c r="E42" s="11">
-        <v>23</v>
+        <v>20</v>
       </c>
       <c r="F42" s="9" t="s">
         <v>28</v>
@@ -2963,7 +2963,7 @@
         <v>27</v>
       </c>
       <c r="E44" s="11">
-        <v>29</v>
+        <v>20</v>
       </c>
       <c r="F44" s="9" t="s">
         <v>28</v>
@@ -2986,7 +2986,7 @@
         <v>27</v>
       </c>
       <c r="E45" s="11">
-        <v>20</v>
+        <v>12</v>
       </c>
       <c r="F45" s="9" t="s">
         <v>28</v>
@@ -3009,7 +3009,7 @@
         <v>27</v>
       </c>
       <c r="E46" s="11">
-        <v>31</v>
+        <v>14</v>
       </c>
       <c r="F46" s="9" t="s">
         <v>28</v>
@@ -3032,7 +3032,7 @@
         <v>27</v>
       </c>
       <c r="E47" s="11">
-        <v>28</v>
+        <v>31</v>
       </c>
       <c r="F47" s="9" t="s">
         <v>28</v>
@@ -3055,7 +3055,7 @@
         <v>27</v>
       </c>
       <c r="E48" s="11">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="F48" s="9" t="s">
         <v>28</v>
@@ -3078,7 +3078,7 @@
         <v>27</v>
       </c>
       <c r="E49" s="11">
-        <v>30</v>
+        <v>17</v>
       </c>
       <c r="F49" s="9" t="s">
         <v>28</v>
@@ -3101,7 +3101,7 @@
         <v>27</v>
       </c>
       <c r="E50" s="11">
-        <v>19</v>
+        <v>9</v>
       </c>
       <c r="F50" s="9" t="s">
         <v>28</v>
@@ -3124,7 +3124,7 @@
         <v>27</v>
       </c>
       <c r="E51" s="11">
-        <v>12</v>
+        <v>26</v>
       </c>
       <c r="F51" s="9" t="s">
         <v>28</v>
@@ -3147,7 +3147,7 @@
         <v>27</v>
       </c>
       <c r="E52" s="11">
-        <v>21</v>
+        <v>27</v>
       </c>
       <c r="F52" s="9" t="s">
         <v>28</v>
@@ -3170,7 +3170,7 @@
         <v>27</v>
       </c>
       <c r="E53" s="11">
-        <v>15</v>
+        <v>17</v>
       </c>
       <c r="F53" s="9" t="s">
         <v>28</v>
@@ -3193,7 +3193,7 @@
         <v>27</v>
       </c>
       <c r="E54" s="11">
-        <v>21</v>
+        <v>24</v>
       </c>
       <c r="F54" s="9" t="s">
         <v>28</v>
@@ -3216,7 +3216,7 @@
         <v>27</v>
       </c>
       <c r="E55" s="11">
-        <v>25</v>
+        <v>11</v>
       </c>
       <c r="F55" s="9" t="s">
         <v>28</v>
@@ -3239,7 +3239,7 @@
         <v>27</v>
       </c>
       <c r="E56" s="11">
-        <v>25</v>
+        <v>9</v>
       </c>
       <c r="F56" s="9" t="s">
         <v>28</v>
@@ -3262,7 +3262,7 @@
         <v>27</v>
       </c>
       <c r="E57" s="11">
-        <v>31</v>
+        <v>21</v>
       </c>
       <c r="F57" s="9" t="s">
         <v>28</v>
@@ -3285,7 +3285,7 @@
         <v>27</v>
       </c>
       <c r="E58" s="11">
-        <v>10</v>
+        <v>30</v>
       </c>
       <c r="F58" s="9" t="s">
         <v>28</v>
@@ -3308,7 +3308,7 @@
         <v>27</v>
       </c>
       <c r="E59" s="11">
-        <v>14</v>
+        <v>29</v>
       </c>
       <c r="F59" s="9" t="s">
         <v>28</v>
@@ -3331,7 +3331,7 @@
         <v>27</v>
       </c>
       <c r="E60" s="11">
-        <v>19</v>
+        <v>10</v>
       </c>
       <c r="F60" s="9" t="s">
         <v>28</v>
@@ -3354,7 +3354,7 @@
         <v>27</v>
       </c>
       <c r="E61" s="11">
-        <v>25</v>
+        <v>31</v>
       </c>
       <c r="F61" s="9" t="s">
         <v>28</v>
@@ -3377,7 +3377,7 @@
         <v>27</v>
       </c>
       <c r="E62" s="11">
-        <v>23</v>
+        <v>27</v>
       </c>
       <c r="F62" s="9" t="s">
         <v>28</v>
@@ -3400,7 +3400,7 @@
         <v>27</v>
       </c>
       <c r="E63" s="11">
-        <v>13</v>
+        <v>30</v>
       </c>
       <c r="F63" s="9" t="s">
         <v>28</v>
@@ -3423,7 +3423,7 @@
         <v>27</v>
       </c>
       <c r="E64" s="11">
-        <v>24</v>
+        <v>29</v>
       </c>
       <c r="F64" s="9" t="s">
         <v>28</v>
@@ -3446,7 +3446,7 @@
         <v>27</v>
       </c>
       <c r="E65" s="11">
-        <v>19</v>
+        <v>11</v>
       </c>
       <c r="F65" s="9" t="s">
         <v>28</v>
@@ -3469,7 +3469,7 @@
         <v>27</v>
       </c>
       <c r="E66" s="11">
-        <v>29</v>
+        <v>15</v>
       </c>
       <c r="F66" s="9" t="s">
         <v>28</v>
@@ -3492,7 +3492,7 @@
         <v>27</v>
       </c>
       <c r="E67" s="11">
-        <v>14</v>
+        <v>27</v>
       </c>
       <c r="F67" s="9" t="s">
         <v>28</v>
@@ -3515,7 +3515,7 @@
         <v>27</v>
       </c>
       <c r="E68" s="11">
-        <v>16</v>
+        <v>23</v>
       </c>
       <c r="F68" s="9" t="s">
         <v>28</v>
@@ -3538,7 +3538,7 @@
         <v>27</v>
       </c>
       <c r="E69" s="11">
-        <v>13</v>
+        <v>16</v>
       </c>
       <c r="F69" s="9" t="s">
         <v>28</v>
@@ -3561,7 +3561,7 @@
         <v>27</v>
       </c>
       <c r="E70" s="11">
-        <v>18</v>
+        <v>23</v>
       </c>
       <c r="F70" s="9" t="s">
         <v>28</v>
@@ -3584,7 +3584,7 @@
         <v>27</v>
       </c>
       <c r="E71" s="11">
-        <v>16</v>
+        <v>25</v>
       </c>
       <c r="F71" s="9" t="s">
         <v>28</v>
@@ -3607,7 +3607,7 @@
         <v>27</v>
       </c>
       <c r="E72" s="11">
-        <v>10</v>
+        <v>26</v>
       </c>
       <c r="F72" s="9" t="s">
         <v>28</v>
@@ -3630,7 +3630,7 @@
         <v>27</v>
       </c>
       <c r="E73" s="11">
-        <v>29</v>
+        <v>16</v>
       </c>
       <c r="F73" s="9" t="s">
         <v>28</v>
@@ -3653,7 +3653,7 @@
         <v>27</v>
       </c>
       <c r="E74" s="11">
-        <v>12</v>
+        <v>29</v>
       </c>
       <c r="F74" s="9" t="s">
         <v>28</v>
@@ -3676,7 +3676,7 @@
         <v>27</v>
       </c>
       <c r="E75" s="11">
-        <v>21</v>
+        <v>8</v>
       </c>
       <c r="F75" s="9" t="s">
         <v>28</v>
@@ -3699,7 +3699,7 @@
         <v>27</v>
       </c>
       <c r="E76" s="11">
-        <v>27</v>
+        <v>8</v>
       </c>
       <c r="F76" s="9" t="s">
         <v>28</v>
@@ -3722,7 +3722,7 @@
         <v>27</v>
       </c>
       <c r="E77" s="11">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="F77" s="9" t="s">
         <v>28</v>
@@ -3745,7 +3745,7 @@
         <v>27</v>
       </c>
       <c r="E78" s="11">
-        <v>18</v>
+        <v>16</v>
       </c>
       <c r="F78" s="9" t="s">
         <v>28</v>
@@ -3768,7 +3768,7 @@
         <v>27</v>
       </c>
       <c r="E79" s="11">
-        <v>19</v>
+        <v>29</v>
       </c>
       <c r="F79" s="9" t="s">
         <v>28</v>
@@ -3791,7 +3791,7 @@
         <v>27</v>
       </c>
       <c r="E80" s="11">
-        <v>11</v>
+        <v>25</v>
       </c>
       <c r="F80" s="9" t="s">
         <v>28</v>
@@ -3814,7 +3814,7 @@
         <v>27</v>
       </c>
       <c r="E81" s="11">
-        <v>26</v>
+        <v>29</v>
       </c>
       <c r="F81" s="9" t="s">
         <v>28</v>
@@ -3837,7 +3837,7 @@
         <v>27</v>
       </c>
       <c r="E82" s="11">
-        <v>27</v>
+        <v>17</v>
       </c>
       <c r="F82" s="9" t="s">
         <v>28</v>
@@ -3860,7 +3860,7 @@
         <v>27</v>
       </c>
       <c r="E83" s="11">
-        <v>25</v>
+        <v>29</v>
       </c>
       <c r="F83" s="9" t="s">
         <v>28</v>
@@ -3883,7 +3883,7 @@
         <v>27</v>
       </c>
       <c r="E84" s="11">
-        <v>22</v>
+        <v>14</v>
       </c>
       <c r="F84" s="9" t="s">
         <v>28</v>
@@ -3906,7 +3906,7 @@
         <v>27</v>
       </c>
       <c r="E85" s="11">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="F85" s="9" t="s">
         <v>28</v>
@@ -3929,7 +3929,7 @@
         <v>27</v>
       </c>
       <c r="E86" s="11">
-        <v>11</v>
+        <v>20</v>
       </c>
       <c r="F86" s="9" t="s">
         <v>28</v>
@@ -3952,7 +3952,7 @@
         <v>27</v>
       </c>
       <c r="E87" s="11">
-        <v>23</v>
+        <v>31</v>
       </c>
       <c r="F87" s="9" t="s">
         <v>28</v>
@@ -3975,7 +3975,7 @@
         <v>27</v>
       </c>
       <c r="E88" s="11">
-        <v>13</v>
+        <v>19</v>
       </c>
       <c r="F88" s="9" t="s">
         <v>28</v>
@@ -3998,7 +3998,7 @@
         <v>27</v>
       </c>
       <c r="E89" s="11">
-        <v>13</v>
+        <v>20</v>
       </c>
       <c r="F89" s="9" t="s">
         <v>28</v>
@@ -4021,7 +4021,7 @@
         <v>27</v>
       </c>
       <c r="E90" s="11">
-        <v>25</v>
+        <v>9</v>
       </c>
       <c r="F90" s="9" t="s">
         <v>28</v>
@@ -4044,7 +4044,7 @@
         <v>27</v>
       </c>
       <c r="E91" s="11">
-        <v>25</v>
+        <v>22</v>
       </c>
       <c r="F91" s="9" t="s">
         <v>28</v>
@@ -4067,7 +4067,7 @@
         <v>27</v>
       </c>
       <c r="E92" s="11">
-        <v>19</v>
+        <v>30</v>
       </c>
       <c r="F92" s="9" t="s">
         <v>28</v>
@@ -4090,7 +4090,7 @@
         <v>27</v>
       </c>
       <c r="E93" s="11">
-        <v>25</v>
+        <v>30</v>
       </c>
       <c r="F93" s="9" t="s">
         <v>28</v>
@@ -4113,7 +4113,7 @@
         <v>27</v>
       </c>
       <c r="E94" s="11">
-        <v>21</v>
+        <v>19</v>
       </c>
       <c r="F94" s="9" t="s">
         <v>28</v>
@@ -4136,7 +4136,7 @@
         <v>27</v>
       </c>
       <c r="E95" s="11">
-        <v>21</v>
+        <v>31</v>
       </c>
       <c r="F95" s="9" t="s">
         <v>28</v>
@@ -4159,7 +4159,7 @@
         <v>27</v>
       </c>
       <c r="E96" s="11">
-        <v>30</v>
+        <v>18</v>
       </c>
       <c r="F96" s="9" t="s">
         <v>28</v>
@@ -4182,7 +4182,7 @@
         <v>27</v>
       </c>
       <c r="E97" s="11">
-        <v>12</v>
+        <v>18</v>
       </c>
       <c r="F97" s="9" t="s">
         <v>28</v>
@@ -4205,7 +4205,7 @@
         <v>27</v>
       </c>
       <c r="E98" s="11">
-        <v>25</v>
+        <v>22</v>
       </c>
       <c r="F98" s="9" t="s">
         <v>28</v>
@@ -4228,7 +4228,7 @@
         <v>27</v>
       </c>
       <c r="E99" s="11">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="F99" s="9" t="s">
         <v>28</v>
@@ -4251,7 +4251,7 @@
         <v>27</v>
       </c>
       <c r="E100" s="11">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="F100" s="9" t="s">
         <v>28</v>
@@ -4274,7 +4274,7 @@
         <v>27</v>
       </c>
       <c r="E101" s="11">
-        <v>24</v>
+        <v>30</v>
       </c>
       <c r="F101" s="9" t="s">
         <v>28</v>
@@ -4297,7 +4297,7 @@
         <v>27</v>
       </c>
       <c r="E102" s="11">
-        <v>8</v>
+        <v>27</v>
       </c>
       <c r="F102" s="9" t="s">
         <v>28</v>
@@ -4320,7 +4320,7 @@
         <v>27</v>
       </c>
       <c r="E103" s="11">
-        <v>30</v>
+        <v>19</v>
       </c>
       <c r="F103" s="9" t="s">
         <v>28</v>
@@ -4343,7 +4343,7 @@
         <v>27</v>
       </c>
       <c r="E104" s="11">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="F104" s="9" t="s">
         <v>28</v>
@@ -4366,7 +4366,7 @@
         <v>27</v>
       </c>
       <c r="E105" s="11">
-        <v>14</v>
+        <v>20</v>
       </c>
       <c r="F105" s="9" t="s">
         <v>28</v>
@@ -4389,7 +4389,7 @@
         <v>27</v>
       </c>
       <c r="E106" s="11">
-        <v>26</v>
+        <v>16</v>
       </c>
       <c r="F106" s="9" t="s">
         <v>28</v>
@@ -4412,7 +4412,7 @@
         <v>27</v>
       </c>
       <c r="E107" s="11">
-        <v>13</v>
+        <v>16</v>
       </c>
       <c r="F107" s="9" t="s">
         <v>28</v>
@@ -4435,7 +4435,7 @@
         <v>27</v>
       </c>
       <c r="E108" s="11">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="F108" s="9" t="s">
         <v>28</v>
@@ -4458,7 +4458,7 @@
         <v>27</v>
       </c>
       <c r="E109" s="11">
-        <v>18</v>
+        <v>24</v>
       </c>
       <c r="F109" s="9" t="s">
         <v>28</v>
@@ -4481,7 +4481,7 @@
         <v>27</v>
       </c>
       <c r="E110" s="11">
-        <v>11</v>
+        <v>20</v>
       </c>
       <c r="F110" s="9" t="s">
         <v>28</v>
@@ -4527,7 +4527,7 @@
         <v>27</v>
       </c>
       <c r="E112" s="11">
-        <v>30</v>
+        <v>20</v>
       </c>
       <c r="F112" s="9" t="s">
         <v>28</v>
@@ -4550,7 +4550,7 @@
         <v>27</v>
       </c>
       <c r="E113" s="11">
-        <v>23</v>
+        <v>16</v>
       </c>
       <c r="F113" s="9" t="s">
         <v>28</v>
@@ -4573,7 +4573,7 @@
         <v>27</v>
       </c>
       <c r="E114" s="11">
-        <v>13</v>
+        <v>23</v>
       </c>
       <c r="F114" s="9" t="s">
         <v>28</v>
@@ -4596,7 +4596,7 @@
         <v>27</v>
       </c>
       <c r="E115" s="11">
-        <v>30</v>
+        <v>22</v>
       </c>
       <c r="F115" s="9" t="s">
         <v>28</v>
@@ -4619,7 +4619,7 @@
         <v>27</v>
       </c>
       <c r="E116" s="11">
-        <v>8</v>
+        <v>28</v>
       </c>
       <c r="F116" s="9" t="s">
         <v>28</v>
@@ -4642,7 +4642,7 @@
         <v>27</v>
       </c>
       <c r="E117" s="11">
-        <v>28</v>
+        <v>16</v>
       </c>
       <c r="F117" s="9" t="s">
         <v>28</v>
@@ -4665,7 +4665,7 @@
         <v>27</v>
       </c>
       <c r="E118" s="11">
-        <v>9</v>
+        <v>29</v>
       </c>
       <c r="F118" s="9" t="s">
         <v>28</v>
@@ -4688,7 +4688,7 @@
         <v>27</v>
       </c>
       <c r="E119" s="11">
-        <v>14</v>
+        <v>27</v>
       </c>
       <c r="F119" s="9" t="s">
         <v>28</v>
@@ -4711,7 +4711,7 @@
         <v>27</v>
       </c>
       <c r="E120" s="11">
-        <v>20</v>
+        <v>10</v>
       </c>
       <c r="F120" s="9" t="s">
         <v>28</v>
@@ -4757,7 +4757,7 @@
         <v>27</v>
       </c>
       <c r="E122" s="11">
-        <v>8</v>
+        <v>11</v>
       </c>
       <c r="F122" s="9" t="s">
         <v>28</v>
@@ -4780,7 +4780,7 @@
         <v>27</v>
       </c>
       <c r="E123" s="11">
-        <v>19</v>
+        <v>28</v>
       </c>
       <c r="F123" s="9" t="s">
         <v>28</v>
@@ -4803,7 +4803,7 @@
         <v>27</v>
       </c>
       <c r="E124" s="11">
-        <v>26</v>
+        <v>17</v>
       </c>
       <c r="F124" s="9" t="s">
         <v>28</v>
@@ -4826,7 +4826,7 @@
         <v>27</v>
       </c>
       <c r="E125" s="11">
-        <v>27</v>
+        <v>24</v>
       </c>
       <c r="F125" s="9" t="s">
         <v>28</v>
@@ -4849,7 +4849,7 @@
         <v>27</v>
       </c>
       <c r="E126" s="11">
-        <v>25</v>
+        <v>9</v>
       </c>
       <c r="F126" s="9" t="s">
         <v>28</v>
@@ -4872,7 +4872,7 @@
         <v>27</v>
       </c>
       <c r="E127" s="11">
-        <v>17</v>
+        <v>9</v>
       </c>
       <c r="F127" s="9" t="s">
         <v>28</v>
@@ -4895,7 +4895,7 @@
         <v>27</v>
       </c>
       <c r="E128" s="11">
-        <v>18</v>
+        <v>21</v>
       </c>
       <c r="F128" s="9" t="s">
         <v>28</v>
@@ -4918,7 +4918,7 @@
         <v>27</v>
       </c>
       <c r="E129" s="11">
-        <v>8</v>
+        <v>29</v>
       </c>
       <c r="F129" s="9" t="s">
         <v>28</v>
@@ -4941,7 +4941,7 @@
         <v>27</v>
       </c>
       <c r="E130" s="11">
-        <v>9</v>
+        <v>11</v>
       </c>
       <c r="F130" s="9" t="s">
         <v>28</v>
@@ -4964,7 +4964,7 @@
         <v>27</v>
       </c>
       <c r="E131" s="11">
-        <v>27</v>
+        <v>19</v>
       </c>
       <c r="F131" s="9" t="s">
         <v>28</v>
@@ -4987,7 +4987,7 @@
         <v>27</v>
       </c>
       <c r="E132" s="11">
-        <v>9</v>
+        <v>28</v>
       </c>
       <c r="F132" s="9" t="s">
         <v>28</v>
@@ -5010,7 +5010,7 @@
         <v>27</v>
       </c>
       <c r="E133" s="11">
-        <v>16</v>
+        <v>20</v>
       </c>
       <c r="F133" s="9" t="s">
         <v>28</v>
@@ -5033,7 +5033,7 @@
         <v>27</v>
       </c>
       <c r="E134" s="11">
-        <v>17</v>
+        <v>28</v>
       </c>
       <c r="F134" s="9" t="s">
         <v>28</v>
@@ -5056,7 +5056,7 @@
         <v>27</v>
       </c>
       <c r="E135" s="11">
-        <v>17</v>
+        <v>26</v>
       </c>
       <c r="F135" s="9" t="s">
         <v>28</v>
@@ -5079,7 +5079,7 @@
         <v>27</v>
       </c>
       <c r="E136" s="11">
-        <v>14</v>
+        <v>11</v>
       </c>
       <c r="F136" s="9" t="s">
         <v>28</v>
@@ -5102,7 +5102,7 @@
         <v>27</v>
       </c>
       <c r="E137" s="11">
-        <v>29</v>
+        <v>22</v>
       </c>
       <c r="F137" s="9" t="s">
         <v>28</v>
@@ -5125,7 +5125,7 @@
         <v>27</v>
       </c>
       <c r="E138" s="11">
-        <v>31</v>
+        <v>12</v>
       </c>
       <c r="F138" s="9" t="s">
         <v>28</v>
@@ -5148,7 +5148,7 @@
         <v>27</v>
       </c>
       <c r="E139" s="11">
-        <v>14</v>
+        <v>22</v>
       </c>
       <c r="F139" s="9" t="s">
         <v>28</v>
@@ -5171,7 +5171,7 @@
         <v>27</v>
       </c>
       <c r="E140" s="11">
-        <v>28</v>
+        <v>25</v>
       </c>
       <c r="F140" s="9" t="s">
         <v>28</v>
@@ -5194,7 +5194,7 @@
         <v>27</v>
       </c>
       <c r="E141" s="11">
-        <v>31</v>
+        <v>26</v>
       </c>
       <c r="F141" s="9" t="s">
         <v>28</v>
@@ -5217,7 +5217,7 @@
         <v>27</v>
       </c>
       <c r="E142" s="11">
-        <v>27</v>
+        <v>17</v>
       </c>
       <c r="F142" s="9" t="s">
         <v>28</v>
@@ -5240,7 +5240,7 @@
         <v>27</v>
       </c>
       <c r="E143" s="11">
-        <v>28</v>
+        <v>24</v>
       </c>
       <c r="F143" s="9" t="s">
         <v>28</v>
@@ -5263,7 +5263,7 @@
         <v>27</v>
       </c>
       <c r="E144" s="11">
-        <v>16</v>
+        <v>11</v>
       </c>
       <c r="F144" s="9" t="s">
         <v>28</v>
@@ -5286,7 +5286,7 @@
         <v>27</v>
       </c>
       <c r="E145" s="11">
-        <v>22</v>
+        <v>10</v>
       </c>
       <c r="F145" s="9" t="s">
         <v>28</v>
@@ -5309,7 +5309,7 @@
         <v>27</v>
       </c>
       <c r="E146" s="11">
-        <v>27</v>
+        <v>14</v>
       </c>
       <c r="F146" s="9" t="s">
         <v>28</v>
@@ -5332,7 +5332,7 @@
         <v>27</v>
       </c>
       <c r="E147" s="11">
-        <v>16</v>
+        <v>11</v>
       </c>
       <c r="F147" s="9" t="s">
         <v>28</v>
@@ -5355,7 +5355,7 @@
         <v>27</v>
       </c>
       <c r="E148" s="11">
-        <v>31</v>
+        <v>20</v>
       </c>
       <c r="F148" s="9" t="s">
         <v>28</v>
@@ -5378,7 +5378,7 @@
         <v>27</v>
       </c>
       <c r="E149" s="11">
-        <v>8</v>
+        <v>30</v>
       </c>
       <c r="F149" s="9" t="s">
         <v>28</v>
@@ -5401,7 +5401,7 @@
         <v>27</v>
       </c>
       <c r="E150" s="11">
-        <v>22</v>
+        <v>25</v>
       </c>
       <c r="F150" s="9" t="s">
         <v>28</v>
@@ -5424,7 +5424,7 @@
         <v>27</v>
       </c>
       <c r="E151" s="11">
-        <v>17</v>
+        <v>27</v>
       </c>
       <c r="F151" s="9" t="s">
         <v>28</v>
@@ -5447,7 +5447,7 @@
         <v>27</v>
       </c>
       <c r="E152" s="11">
-        <v>18</v>
+        <v>9</v>
       </c>
       <c r="F152" s="9" t="s">
         <v>28</v>
@@ -5470,7 +5470,7 @@
         <v>27</v>
       </c>
       <c r="E153" s="11">
-        <v>23</v>
+        <v>20</v>
       </c>
       <c r="F153" s="9" t="s">
         <v>28</v>
@@ -5493,7 +5493,7 @@
         <v>27</v>
       </c>
       <c r="E154" s="11">
-        <v>19</v>
+        <v>21</v>
       </c>
       <c r="F154" s="9" t="s">
         <v>28</v>
@@ -5516,7 +5516,7 @@
         <v>27</v>
       </c>
       <c r="E155" s="11">
-        <v>12</v>
+        <v>17</v>
       </c>
       <c r="F155" s="9" t="s">
         <v>28</v>
@@ -5539,7 +5539,7 @@
         <v>27</v>
       </c>
       <c r="E156" s="11">
-        <v>19</v>
+        <v>10</v>
       </c>
       <c r="F156" s="9" t="s">
         <v>28</v>
@@ -5562,7 +5562,7 @@
         <v>27</v>
       </c>
       <c r="E157" s="11">
-        <v>8</v>
+        <v>25</v>
       </c>
       <c r="F157" s="9" t="s">
         <v>28</v>
@@ -5585,7 +5585,7 @@
         <v>27</v>
       </c>
       <c r="E158" s="11">
-        <v>29</v>
+        <v>26</v>
       </c>
       <c r="F158" s="9" t="s">
         <v>28</v>
@@ -5608,7 +5608,7 @@
         <v>27</v>
       </c>
       <c r="E159" s="11">
-        <v>27</v>
+        <v>25</v>
       </c>
       <c r="F159" s="9" t="s">
         <v>28</v>
@@ -5631,7 +5631,7 @@
         <v>27</v>
       </c>
       <c r="E160" s="11">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="F160" s="9" t="s">
         <v>28</v>
@@ -5654,7 +5654,7 @@
         <v>27</v>
       </c>
       <c r="E161" s="11">
-        <v>18</v>
+        <v>15</v>
       </c>
       <c r="F161" s="9" t="s">
         <v>28</v>
@@ -5677,7 +5677,7 @@
         <v>27</v>
       </c>
       <c r="E162" s="11">
-        <v>31</v>
+        <v>14</v>
       </c>
       <c r="F162" s="9" t="s">
         <v>28</v>
@@ -5700,7 +5700,7 @@
         <v>27</v>
       </c>
       <c r="E163" s="11">
-        <v>29</v>
+        <v>10</v>
       </c>
       <c r="F163" s="9" t="s">
         <v>28</v>
@@ -5723,7 +5723,7 @@
         <v>27</v>
       </c>
       <c r="E164" s="11">
-        <v>12</v>
+        <v>24</v>
       </c>
       <c r="F164" s="9" t="s">
         <v>28</v>
@@ -5746,7 +5746,7 @@
         <v>27</v>
       </c>
       <c r="E165" s="11">
-        <v>21</v>
+        <v>29</v>
       </c>
       <c r="F165" s="9" t="s">
         <v>28</v>
@@ -5769,7 +5769,7 @@
         <v>27</v>
       </c>
       <c r="E166" s="11">
-        <v>10</v>
+        <v>17</v>
       </c>
       <c r="F166" s="9" t="s">
         <v>28</v>
@@ -5792,7 +5792,7 @@
         <v>27</v>
       </c>
       <c r="E167" s="11">
-        <v>29</v>
+        <v>16</v>
       </c>
       <c r="F167" s="9" t="s">
         <v>28</v>
@@ -5815,7 +5815,7 @@
         <v>27</v>
       </c>
       <c r="E168" s="11">
-        <v>26</v>
+        <v>17</v>
       </c>
       <c r="F168" s="9" t="s">
         <v>28</v>
@@ -5838,7 +5838,7 @@
         <v>27</v>
       </c>
       <c r="E169" s="11">
-        <v>13</v>
+        <v>18</v>
       </c>
       <c r="F169" s="9" t="s">
         <v>28</v>
@@ -5861,7 +5861,7 @@
         <v>27</v>
       </c>
       <c r="E170" s="11">
-        <v>17</v>
+        <v>14</v>
       </c>
       <c r="F170" s="9" t="s">
         <v>28</v>
@@ -5884,7 +5884,7 @@
         <v>27</v>
       </c>
       <c r="E171" s="11">
-        <v>30</v>
+        <v>25</v>
       </c>
       <c r="F171" s="9" t="s">
         <v>28</v>
@@ -5907,7 +5907,7 @@
         <v>27</v>
       </c>
       <c r="E172" s="11">
-        <v>28</v>
+        <v>15</v>
       </c>
       <c r="F172" s="9" t="s">
         <v>28</v>
@@ -5930,7 +5930,7 @@
         <v>27</v>
       </c>
       <c r="E173" s="11">
-        <v>9</v>
+        <v>13</v>
       </c>
       <c r="F173" s="9" t="s">
         <v>28</v>
@@ -5953,7 +5953,7 @@
         <v>27</v>
       </c>
       <c r="E174" s="11">
-        <v>31</v>
+        <v>29</v>
       </c>
       <c r="F174" s="9" t="s">
         <v>28</v>
@@ -5976,7 +5976,7 @@
         <v>27</v>
       </c>
       <c r="E175" s="11">
-        <v>14</v>
+        <v>11</v>
       </c>
       <c r="F175" s="9" t="s">
         <v>28</v>
@@ -5999,7 +5999,7 @@
         <v>27</v>
       </c>
       <c r="E176" s="11">
-        <v>30</v>
+        <v>28</v>
       </c>
       <c r="F176" s="9" t="s">
         <v>28</v>
@@ -6022,7 +6022,7 @@
         <v>27</v>
       </c>
       <c r="E177" s="11">
-        <v>27</v>
+        <v>14</v>
       </c>
       <c r="F177" s="9" t="s">
         <v>28</v>
@@ -6045,7 +6045,7 @@
         <v>27</v>
       </c>
       <c r="E178" s="11">
-        <v>11</v>
+        <v>16</v>
       </c>
       <c r="F178" s="9" t="s">
         <v>28</v>
@@ -6068,7 +6068,7 @@
         <v>27</v>
       </c>
       <c r="E179" s="11">
-        <v>20</v>
+        <v>31</v>
       </c>
       <c r="F179" s="9" t="s">
         <v>28</v>
@@ -6091,7 +6091,7 @@
         <v>27</v>
       </c>
       <c r="E180" s="11">
-        <v>12</v>
+        <v>27</v>
       </c>
       <c r="F180" s="9" t="s">
         <v>28</v>
@@ -6114,7 +6114,7 @@
         <v>27</v>
       </c>
       <c r="E181" s="11">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="F181" s="9" t="s">
         <v>28</v>
@@ -6137,7 +6137,7 @@
         <v>27</v>
       </c>
       <c r="E182" s="11">
-        <v>25</v>
+        <v>16</v>
       </c>
       <c r="F182" s="9" t="s">
         <v>28</v>
@@ -6160,7 +6160,7 @@
         <v>27</v>
       </c>
       <c r="E183" s="11">
-        <v>20</v>
+        <v>31</v>
       </c>
       <c r="F183" s="9" t="s">
         <v>28</v>
@@ -6183,7 +6183,7 @@
         <v>27</v>
       </c>
       <c r="E184" s="11">
-        <v>28</v>
+        <v>18</v>
       </c>
       <c r="F184" s="9" t="s">
         <v>28</v>
@@ -6206,7 +6206,7 @@
         <v>27</v>
       </c>
       <c r="E185" s="11">
-        <v>11</v>
+        <v>24</v>
       </c>
       <c r="F185" s="9" t="s">
         <v>28</v>
@@ -6229,7 +6229,7 @@
         <v>27</v>
       </c>
       <c r="E186" s="11">
-        <v>27</v>
+        <v>16</v>
       </c>
       <c r="F186" s="9" t="s">
         <v>28</v>
@@ -6252,7 +6252,7 @@
         <v>27</v>
       </c>
       <c r="E187" s="11">
-        <v>24</v>
+        <v>11</v>
       </c>
       <c r="F187" s="9" t="s">
         <v>28</v>
@@ -6275,7 +6275,7 @@
         <v>27</v>
       </c>
       <c r="E188" s="11">
-        <v>13</v>
+        <v>15</v>
       </c>
       <c r="F188" s="9" t="s">
         <v>28</v>
@@ -6298,7 +6298,7 @@
         <v>27</v>
       </c>
       <c r="E189" s="11">
-        <v>27</v>
+        <v>14</v>
       </c>
       <c r="F189" s="9" t="s">
         <v>28</v>
@@ -6321,7 +6321,7 @@
         <v>27</v>
       </c>
       <c r="E190" s="11">
-        <v>10</v>
+        <v>13</v>
       </c>
       <c r="F190" s="9" t="s">
         <v>28</v>
@@ -6344,7 +6344,7 @@
         <v>27</v>
       </c>
       <c r="E191" s="11">
-        <v>23</v>
+        <v>27</v>
       </c>
       <c r="F191" s="9" t="s">
         <v>28</v>
@@ -6390,7 +6390,7 @@
         <v>27</v>
       </c>
       <c r="E193" s="11">
-        <v>9</v>
+        <v>30</v>
       </c>
       <c r="F193" s="9" t="s">
         <v>28</v>
@@ -6413,7 +6413,7 @@
         <v>27</v>
       </c>
       <c r="E194" s="11">
-        <v>24</v>
+        <v>13</v>
       </c>
       <c r="F194" s="9" t="s">
         <v>28</v>
@@ -6436,7 +6436,7 @@
         <v>27</v>
       </c>
       <c r="E195" s="11">
-        <v>21</v>
+        <v>17</v>
       </c>
       <c r="F195" s="9" t="s">
         <v>28</v>
@@ -6459,7 +6459,7 @@
         <v>27</v>
       </c>
       <c r="E196" s="11">
-        <v>30</v>
+        <v>23</v>
       </c>
       <c r="F196" s="9" t="s">
         <v>28</v>
@@ -6482,7 +6482,7 @@
         <v>27</v>
       </c>
       <c r="E197" s="11">
-        <v>16</v>
+        <v>31</v>
       </c>
       <c r="F197" s="9" t="s">
         <v>28</v>
@@ -6505,7 +6505,7 @@
         <v>27</v>
       </c>
       <c r="E198" s="11">
-        <v>24</v>
+        <v>21</v>
       </c>
       <c r="F198" s="9" t="s">
         <v>28</v>
@@ -6528,7 +6528,7 @@
         <v>27</v>
       </c>
       <c r="E199" s="11">
-        <v>17</v>
+        <v>22</v>
       </c>
       <c r="F199" s="9" t="s">
         <v>28</v>
@@ -6551,7 +6551,7 @@
         <v>27</v>
       </c>
       <c r="E200" s="11">
-        <v>15</v>
+        <v>9</v>
       </c>
       <c r="F200" s="9" t="s">
         <v>28</v>
@@ -6574,7 +6574,7 @@
         <v>27</v>
       </c>
       <c r="E201" s="11">
-        <v>12</v>
+        <v>16</v>
       </c>
       <c r="F201" s="9" t="s">
         <v>28</v>
@@ -6597,7 +6597,7 @@
         <v>27</v>
       </c>
       <c r="E202" s="11">
-        <v>9</v>
+        <v>30</v>
       </c>
       <c r="F202" s="9" t="s">
         <v>28</v>
@@ -6620,7 +6620,7 @@
         <v>27</v>
       </c>
       <c r="E203" s="11">
-        <v>27</v>
+        <v>8</v>
       </c>
       <c r="F203" s="9" t="s">
         <v>28</v>
@@ -6643,7 +6643,7 @@
         <v>27</v>
       </c>
       <c r="E204" s="11">
-        <v>15</v>
+        <v>11</v>
       </c>
       <c r="F204" s="9" t="s">
         <v>28</v>
@@ -6666,7 +6666,7 @@
         <v>27</v>
       </c>
       <c r="E205" s="11">
-        <v>14</v>
+        <v>8</v>
       </c>
       <c r="F205" s="9" t="s">
         <v>28</v>
@@ -6689,7 +6689,7 @@
         <v>27</v>
       </c>
       <c r="E206" s="11">
-        <v>10</v>
+        <v>31</v>
       </c>
       <c r="F206" s="9" t="s">
         <v>28</v>
@@ -6712,7 +6712,7 @@
         <v>27</v>
       </c>
       <c r="E207" s="11">
-        <v>19</v>
+        <v>9</v>
       </c>
       <c r="F207" s="9" t="s">
         <v>28</v>
@@ -6735,7 +6735,7 @@
         <v>27</v>
       </c>
       <c r="E208" s="11">
-        <v>10</v>
+        <v>17</v>
       </c>
       <c r="F208" s="9" t="s">
         <v>28</v>
@@ -6758,7 +6758,7 @@
         <v>27</v>
       </c>
       <c r="E209" s="11">
-        <v>21</v>
+        <v>24</v>
       </c>
       <c r="F209" s="9" t="s">
         <v>28</v>
@@ -6781,7 +6781,7 @@
         <v>27</v>
       </c>
       <c r="E210" s="11">
-        <v>27</v>
+        <v>24</v>
       </c>
       <c r="F210" s="9" t="s">
         <v>28</v>
@@ -6804,7 +6804,7 @@
         <v>27</v>
       </c>
       <c r="E211" s="11">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="F211" s="9" t="s">
         <v>28</v>
@@ -6827,7 +6827,7 @@
         <v>27</v>
       </c>
       <c r="E212" s="11">
-        <v>27</v>
+        <v>24</v>
       </c>
       <c r="F212" s="9" t="s">
         <v>28</v>
@@ -6850,7 +6850,7 @@
         <v>27</v>
       </c>
       <c r="E213" s="11">
-        <v>23</v>
+        <v>18</v>
       </c>
       <c r="F213" s="9" t="s">
         <v>28</v>
@@ -6873,7 +6873,7 @@
         <v>27</v>
       </c>
       <c r="E214" s="11">
-        <v>10</v>
+        <v>22</v>
       </c>
       <c r="F214" s="9" t="s">
         <v>28</v>
@@ -6896,7 +6896,7 @@
         <v>27</v>
       </c>
       <c r="E215" s="11">
-        <v>29</v>
+        <v>25</v>
       </c>
       <c r="F215" s="9" t="s">
         <v>28</v>
@@ -6919,7 +6919,7 @@
         <v>27</v>
       </c>
       <c r="E216" s="11">
-        <v>22</v>
+        <v>29</v>
       </c>
       <c r="F216" s="9" t="s">
         <v>28</v>
@@ -6942,7 +6942,7 @@
         <v>27</v>
       </c>
       <c r="E217" s="11">
-        <v>24</v>
+        <v>22</v>
       </c>
       <c r="F217" s="9" t="s">
         <v>28</v>
@@ -6965,7 +6965,7 @@
         <v>27</v>
       </c>
       <c r="E218" s="11">
-        <v>31</v>
+        <v>14</v>
       </c>
       <c r="F218" s="9" t="s">
         <v>28</v>
@@ -6988,7 +6988,7 @@
         <v>27</v>
       </c>
       <c r="E219" s="11">
-        <v>11</v>
+        <v>29</v>
       </c>
       <c r="F219" s="9" t="s">
         <v>28</v>
@@ -7011,7 +7011,7 @@
         <v>27</v>
       </c>
       <c r="E220" s="11">
-        <v>16</v>
+        <v>30</v>
       </c>
       <c r="F220" s="9" t="s">
         <v>28</v>
@@ -7034,7 +7034,7 @@
         <v>27</v>
       </c>
       <c r="E221" s="11">
-        <v>10</v>
+        <v>27</v>
       </c>
       <c r="F221" s="9" t="s">
         <v>28</v>
@@ -7057,7 +7057,7 @@
         <v>27</v>
       </c>
       <c r="E222" s="11">
-        <v>24</v>
+        <v>12</v>
       </c>
       <c r="F222" s="9" t="s">
         <v>28</v>
@@ -7080,7 +7080,7 @@
         <v>27</v>
       </c>
       <c r="E223" s="11">
-        <v>22</v>
+        <v>13</v>
       </c>
       <c r="F223" s="9" t="s">
         <v>28</v>
@@ -7103,7 +7103,7 @@
         <v>27</v>
       </c>
       <c r="E224" s="11">
-        <v>20</v>
+        <v>11</v>
       </c>
       <c r="F224" s="9" t="s">
         <v>28</v>
@@ -7126,7 +7126,7 @@
         <v>27</v>
       </c>
       <c r="E225" s="11">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="F225" s="9" t="s">
         <v>28</v>
@@ -7149,7 +7149,7 @@
         <v>27</v>
       </c>
       <c r="E226" s="11">
-        <v>17</v>
+        <v>31</v>
       </c>
       <c r="F226" s="9" t="s">
         <v>28</v>
@@ -7172,7 +7172,7 @@
         <v>27</v>
       </c>
       <c r="E227" s="11">
-        <v>17</v>
+        <v>13</v>
       </c>
       <c r="F227" s="9" t="s">
         <v>28</v>
@@ -7195,7 +7195,7 @@
         <v>27</v>
       </c>
       <c r="E228" s="11">
-        <v>22</v>
+        <v>13</v>
       </c>
       <c r="F228" s="9" t="s">
         <v>28</v>
@@ -7218,7 +7218,7 @@
         <v>27</v>
       </c>
       <c r="E229" s="11">
-        <v>22</v>
+        <v>31</v>
       </c>
       <c r="F229" s="9" t="s">
         <v>28</v>
@@ -7241,7 +7241,7 @@
         <v>27</v>
       </c>
       <c r="E230" s="11">
-        <v>31</v>
+        <v>13</v>
       </c>
       <c r="F230" s="9" t="s">
         <v>28</v>
@@ -7264,7 +7264,7 @@
         <v>27</v>
       </c>
       <c r="E231" s="11">
-        <v>8</v>
+        <v>25</v>
       </c>
       <c r="F231" s="9" t="s">
         <v>28</v>
@@ -7287,7 +7287,7 @@
         <v>27</v>
       </c>
       <c r="E232" s="11">
-        <v>14</v>
+        <v>29</v>
       </c>
       <c r="F232" s="9" t="s">
         <v>28</v>
@@ -7310,7 +7310,7 @@
         <v>27</v>
       </c>
       <c r="E233" s="11">
-        <v>27</v>
+        <v>22</v>
       </c>
       <c r="F233" s="9" t="s">
         <v>28</v>
@@ -7356,7 +7356,7 @@
         <v>27</v>
       </c>
       <c r="E235" s="11">
-        <v>21</v>
+        <v>19</v>
       </c>
       <c r="F235" s="9" t="s">
         <v>28</v>
@@ -7379,7 +7379,7 @@
         <v>27</v>
       </c>
       <c r="E236" s="11">
-        <v>18</v>
+        <v>8</v>
       </c>
       <c r="F236" s="9" t="s">
         <v>28</v>
@@ -7402,7 +7402,7 @@
         <v>27</v>
       </c>
       <c r="E237" s="11">
-        <v>8</v>
+        <v>23</v>
       </c>
       <c r="F237" s="9" t="s">
         <v>28</v>
@@ -7425,7 +7425,7 @@
         <v>27</v>
       </c>
       <c r="E238" s="11">
-        <v>11</v>
+        <v>28</v>
       </c>
       <c r="F238" s="9" t="s">
         <v>28</v>
@@ -7448,7 +7448,7 @@
         <v>27</v>
       </c>
       <c r="E239" s="11">
-        <v>10</v>
+        <v>21</v>
       </c>
       <c r="F239" s="9" t="s">
         <v>28</v>
@@ -7471,7 +7471,7 @@
         <v>27</v>
       </c>
       <c r="E240" s="11">
-        <v>20</v>
+        <v>23</v>
       </c>
       <c r="F240" s="9" t="s">
         <v>28</v>
@@ -7494,7 +7494,7 @@
         <v>27</v>
       </c>
       <c r="E241" s="11">
-        <v>29</v>
+        <v>18</v>
       </c>
       <c r="F241" s="9" t="s">
         <v>28</v>
@@ -7517,7 +7517,7 @@
         <v>27</v>
       </c>
       <c r="E242" s="11">
-        <v>12</v>
+        <v>15</v>
       </c>
       <c r="F242" s="9" t="s">
         <v>28</v>
@@ -7540,7 +7540,7 @@
         <v>27</v>
       </c>
       <c r="E243" s="11">
-        <v>10</v>
+        <v>17</v>
       </c>
       <c r="F243" s="9" t="s">
         <v>28</v>
@@ -7563,7 +7563,7 @@
         <v>27</v>
       </c>
       <c r="E244" s="11">
-        <v>9</v>
+        <v>25</v>
       </c>
       <c r="F244" s="9" t="s">
         <v>28</v>
@@ -7586,7 +7586,7 @@
         <v>27</v>
       </c>
       <c r="E245" s="11">
-        <v>25</v>
+        <v>31</v>
       </c>
       <c r="F245" s="9" t="s">
         <v>28</v>
@@ -7609,7 +7609,7 @@
         <v>27</v>
       </c>
       <c r="E246" s="11">
-        <v>14</v>
+        <v>31</v>
       </c>
       <c r="F246" s="9" t="s">
         <v>28</v>
@@ -7632,7 +7632,7 @@
         <v>27</v>
       </c>
       <c r="E247" s="11">
-        <v>30</v>
+        <v>8</v>
       </c>
       <c r="F247" s="9" t="s">
         <v>28</v>
@@ -7655,7 +7655,7 @@
         <v>27</v>
       </c>
       <c r="E248" s="11">
-        <v>9</v>
+        <v>13</v>
       </c>
       <c r="F248" s="9" t="s">
         <v>28</v>
@@ -7678,7 +7678,7 @@
         <v>27</v>
       </c>
       <c r="E249" s="11">
-        <v>20</v>
+        <v>15</v>
       </c>
       <c r="F249" s="9" t="s">
         <v>28</v>
@@ -7701,7 +7701,7 @@
         <v>27</v>
       </c>
       <c r="E250" s="11">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="F250" s="9" t="s">
         <v>28</v>
@@ -7724,7 +7724,7 @@
         <v>27</v>
       </c>
       <c r="E251" s="11">
-        <v>31</v>
+        <v>28</v>
       </c>
       <c r="F251" s="9" t="s">
         <v>28</v>
@@ -7747,7 +7747,7 @@
         <v>27</v>
       </c>
       <c r="E252" s="11">
-        <v>14</v>
+        <v>20</v>
       </c>
       <c r="F252" s="9" t="s">
         <v>28</v>
@@ -7770,7 +7770,7 @@
         <v>27</v>
       </c>
       <c r="E253" s="11">
-        <v>26</v>
+        <v>29</v>
       </c>
       <c r="F253" s="9" t="s">
         <v>28</v>
@@ -7793,7 +7793,7 @@
         <v>27</v>
       </c>
       <c r="E254" s="11">
-        <v>29</v>
+        <v>15</v>
       </c>
       <c r="F254" s="9" t="s">
         <v>28</v>
@@ -7816,7 +7816,7 @@
         <v>27</v>
       </c>
       <c r="E255" s="11">
-        <v>13</v>
+        <v>20</v>
       </c>
       <c r="F255" s="9" t="s">
         <v>28</v>
@@ -7839,7 +7839,7 @@
         <v>27</v>
       </c>
       <c r="E256" s="11">
-        <v>18</v>
+        <v>16</v>
       </c>
       <c r="F256" s="9" t="s">
         <v>28</v>
@@ -7862,7 +7862,7 @@
         <v>27</v>
       </c>
       <c r="E257" s="11">
-        <v>31</v>
+        <v>28</v>
       </c>
       <c r="F257" s="9" t="s">
         <v>28</v>
@@ -7885,7 +7885,7 @@
         <v>27</v>
       </c>
       <c r="E258" s="11">
-        <v>9</v>
+        <v>21</v>
       </c>
       <c r="F258" s="9" t="s">
         <v>28</v>
@@ -7908,7 +7908,7 @@
         <v>27</v>
       </c>
       <c r="E259" s="11">
-        <v>20</v>
+        <v>10</v>
       </c>
       <c r="F259" s="9" t="s">
         <v>28</v>
@@ -7931,7 +7931,7 @@
         <v>27</v>
       </c>
       <c r="E260" s="11">
-        <v>21</v>
+        <v>8</v>
       </c>
       <c r="F260" s="9" t="s">
         <v>28</v>
@@ -7954,7 +7954,7 @@
         <v>27</v>
       </c>
       <c r="E261" s="11">
-        <v>29</v>
+        <v>18</v>
       </c>
       <c r="F261" s="9" t="s">
         <v>28</v>
@@ -7977,7 +7977,7 @@
         <v>27</v>
       </c>
       <c r="E262" s="11">
-        <v>13</v>
+        <v>9</v>
       </c>
       <c r="F262" s="9" t="s">
         <v>28</v>
@@ -8000,7 +8000,7 @@
         <v>27</v>
       </c>
       <c r="E263" s="11">
-        <v>23</v>
+        <v>26</v>
       </c>
       <c r="F263" s="9" t="s">
         <v>28</v>
@@ -8023,7 +8023,7 @@
         <v>27</v>
       </c>
       <c r="E264" s="11">
-        <v>15</v>
+        <v>27</v>
       </c>
       <c r="F264" s="9" t="s">
         <v>28</v>
@@ -8046,7 +8046,7 @@
         <v>27</v>
       </c>
       <c r="E265" s="11">
-        <v>11</v>
+        <v>26</v>
       </c>
       <c r="F265" s="9" t="s">
         <v>28</v>
@@ -8069,7 +8069,7 @@
         <v>27</v>
       </c>
       <c r="E266" s="11">
-        <v>28</v>
+        <v>11</v>
       </c>
       <c r="F266" s="9" t="s">
         <v>28</v>
@@ -8092,7 +8092,7 @@
         <v>27</v>
       </c>
       <c r="E267" s="11">
-        <v>13</v>
+        <v>24</v>
       </c>
       <c r="F267" s="9" t="s">
         <v>28</v>
@@ -8115,7 +8115,7 @@
         <v>27</v>
       </c>
       <c r="E268" s="11">
-        <v>26</v>
+        <v>9</v>
       </c>
       <c r="F268" s="9" t="s">
         <v>28</v>
@@ -8138,7 +8138,7 @@
         <v>27</v>
       </c>
       <c r="E269" s="11">
-        <v>23</v>
+        <v>31</v>
       </c>
       <c r="F269" s="9" t="s">
         <v>28</v>
@@ -8161,7 +8161,7 @@
         <v>27</v>
       </c>
       <c r="E270" s="11">
-        <v>15</v>
+        <v>27</v>
       </c>
       <c r="F270" s="9" t="s">
         <v>28</v>
@@ -8184,7 +8184,7 @@
         <v>27</v>
       </c>
       <c r="E271" s="11">
-        <v>30</v>
+        <v>21</v>
       </c>
       <c r="F271" s="9" t="s">
         <v>28</v>
@@ -8207,7 +8207,7 @@
         <v>27</v>
       </c>
       <c r="E272" s="11">
-        <v>21</v>
+        <v>12</v>
       </c>
       <c r="F272" s="9" t="s">
         <v>28</v>
@@ -8230,7 +8230,7 @@
         <v>27</v>
       </c>
       <c r="E273" s="11">
-        <v>28</v>
+        <v>20</v>
       </c>
       <c r="F273" s="9" t="s">
         <v>28</v>
@@ -8253,7 +8253,7 @@
         <v>27</v>
       </c>
       <c r="E274" s="11">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="F274" s="9" t="s">
         <v>28</v>
@@ -8276,7 +8276,7 @@
         <v>27</v>
       </c>
       <c r="E275" s="11">
-        <v>25</v>
+        <v>16</v>
       </c>
       <c r="F275" s="9" t="s">
         <v>28</v>
@@ -8299,7 +8299,7 @@
         <v>27</v>
       </c>
       <c r="E276" s="11">
-        <v>20</v>
+        <v>8</v>
       </c>
       <c r="F276" s="9" t="s">
         <v>28</v>
@@ -8322,7 +8322,7 @@
         <v>27</v>
       </c>
       <c r="E277" s="11">
-        <v>22</v>
+        <v>28</v>
       </c>
       <c r="F277" s="9" t="s">
         <v>28</v>
@@ -8345,7 +8345,7 @@
         <v>27</v>
       </c>
       <c r="E278" s="11">
-        <v>30</v>
+        <v>17</v>
       </c>
       <c r="F278" s="9" t="s">
         <v>28</v>
@@ -8368,7 +8368,7 @@
         <v>27</v>
       </c>
       <c r="E279" s="11">
-        <v>21</v>
+        <v>12</v>
       </c>
       <c r="F279" s="9" t="s">
         <v>28</v>
@@ -8391,7 +8391,7 @@
         <v>27</v>
       </c>
       <c r="E280" s="11">
-        <v>16</v>
+        <v>22</v>
       </c>
       <c r="F280" s="9" t="s">
         <v>28</v>
@@ -8414,7 +8414,7 @@
         <v>27</v>
       </c>
       <c r="E281" s="11">
-        <v>31</v>
+        <v>12</v>
       </c>
       <c r="F281" s="9" t="s">
         <v>28</v>
@@ -8437,7 +8437,7 @@
         <v>27</v>
       </c>
       <c r="E282" s="11">
-        <v>10</v>
+        <v>21</v>
       </c>
       <c r="F282" s="9" t="s">
         <v>28</v>
@@ -8460,7 +8460,7 @@
         <v>27</v>
       </c>
       <c r="E283" s="11">
-        <v>11</v>
+        <v>17</v>
       </c>
       <c r="F283" s="9" t="s">
         <v>28</v>
@@ -8483,7 +8483,7 @@
         <v>27</v>
       </c>
       <c r="E284" s="11">
-        <v>22</v>
+        <v>25</v>
       </c>
       <c r="F284" s="9" t="s">
         <v>28</v>
@@ -8506,7 +8506,7 @@
         <v>27</v>
       </c>
       <c r="E285" s="11">
-        <v>18</v>
+        <v>28</v>
       </c>
       <c r="F285" s="9" t="s">
         <v>28</v>
@@ -8552,7 +8552,7 @@
         <v>27</v>
       </c>
       <c r="E287" s="11">
-        <v>25</v>
+        <v>30</v>
       </c>
       <c r="F287" s="9" t="s">
         <v>28</v>
@@ -8575,7 +8575,7 @@
         <v>27</v>
       </c>
       <c r="E288" s="11">
-        <v>18</v>
+        <v>10</v>
       </c>
       <c r="F288" s="9" t="s">
         <v>28</v>
@@ -8598,7 +8598,7 @@
         <v>27</v>
       </c>
       <c r="E289" s="11">
-        <v>21</v>
+        <v>26</v>
       </c>
       <c r="F289" s="9" t="s">
         <v>28</v>
@@ -8621,7 +8621,7 @@
         <v>27</v>
       </c>
       <c r="E290" s="11">
-        <v>13</v>
+        <v>16</v>
       </c>
       <c r="F290" s="9" t="s">
         <v>28</v>
@@ -8644,7 +8644,7 @@
         <v>27</v>
       </c>
       <c r="E291" s="11">
-        <v>13</v>
+        <v>8</v>
       </c>
       <c r="F291" s="9" t="s">
         <v>28</v>
@@ -8667,7 +8667,7 @@
         <v>27</v>
       </c>
       <c r="E292" s="11">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="F292" s="9" t="s">
         <v>28</v>
@@ -8690,7 +8690,7 @@
         <v>27</v>
       </c>
       <c r="E293" s="11">
-        <v>21</v>
+        <v>25</v>
       </c>
       <c r="F293" s="9" t="s">
         <v>28</v>
@@ -8713,7 +8713,7 @@
         <v>27</v>
       </c>
       <c r="E294" s="11">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="F294" s="9" t="s">
         <v>28</v>
@@ -8736,7 +8736,7 @@
         <v>27</v>
       </c>
       <c r="E295" s="11">
-        <v>8</v>
+        <v>13</v>
       </c>
       <c r="F295" s="9" t="s">
         <v>28</v>
@@ -8759,7 +8759,7 @@
         <v>27</v>
       </c>
       <c r="E296" s="11">
-        <v>15</v>
+        <v>30</v>
       </c>
       <c r="F296" s="9" t="s">
         <v>28</v>
@@ -8782,7 +8782,7 @@
         <v>27</v>
       </c>
       <c r="E297" s="11">
-        <v>24</v>
+        <v>11</v>
       </c>
       <c r="F297" s="9" t="s">
         <v>28</v>
@@ -8805,7 +8805,7 @@
         <v>27</v>
       </c>
       <c r="E298" s="11">
-        <v>25</v>
+        <v>27</v>
       </c>
       <c r="F298" s="9" t="s">
         <v>28</v>
@@ -8828,7 +8828,7 @@
         <v>27</v>
       </c>
       <c r="E299" s="11">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="F299" s="9" t="s">
         <v>28</v>
@@ -8851,7 +8851,7 @@
         <v>27</v>
       </c>
       <c r="E300" s="11">
-        <v>14</v>
+        <v>9</v>
       </c>
       <c r="F300" s="9" t="s">
         <v>28</v>
@@ -8874,7 +8874,7 @@
         <v>27</v>
       </c>
       <c r="E301" s="11">
-        <v>26</v>
+        <v>11</v>
       </c>
       <c r="F301" s="9" t="s">
         <v>28</v>
@@ -8897,7 +8897,7 @@
         <v>27</v>
       </c>
       <c r="E302" s="11">
-        <v>22</v>
+        <v>9</v>
       </c>
       <c r="F302" s="9" t="s">
         <v>28</v>
@@ -8920,7 +8920,7 @@
         <v>27</v>
       </c>
       <c r="E303" s="11">
-        <v>10</v>
+        <v>16</v>
       </c>
       <c r="F303" s="9" t="s">
         <v>28</v>
@@ -8943,7 +8943,7 @@
         <v>27</v>
       </c>
       <c r="E304" s="11">
-        <v>12</v>
+        <v>28</v>
       </c>
       <c r="F304" s="9" t="s">
         <v>28</v>
@@ -8966,7 +8966,7 @@
         <v>27</v>
       </c>
       <c r="E305" s="11">
-        <v>10</v>
+        <v>20</v>
       </c>
       <c r="F305" s="9" t="s">
         <v>28</v>
@@ -8989,7 +8989,7 @@
         <v>27</v>
       </c>
       <c r="E306" s="11">
-        <v>22</v>
+        <v>29</v>
       </c>
       <c r="F306" s="9" t="s">
         <v>28</v>
@@ -9012,7 +9012,7 @@
         <v>27</v>
       </c>
       <c r="E307" s="11">
-        <v>20</v>
+        <v>12</v>
       </c>
       <c r="F307" s="9" t="s">
         <v>28</v>
@@ -9035,7 +9035,7 @@
         <v>27</v>
       </c>
       <c r="E308" s="11">
-        <v>29</v>
+        <v>21</v>
       </c>
       <c r="F308" s="9" t="s">
         <v>28</v>
@@ -9058,7 +9058,7 @@
         <v>27</v>
       </c>
       <c r="E309" s="11">
-        <v>24</v>
+        <v>29</v>
       </c>
       <c r="F309" s="9" t="s">
         <v>28</v>
@@ -9081,7 +9081,7 @@
         <v>27</v>
       </c>
       <c r="E310" s="11">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="F310" s="9" t="s">
         <v>28</v>
@@ -9104,7 +9104,7 @@
         <v>27</v>
       </c>
       <c r="E311" s="11">
-        <v>25</v>
+        <v>22</v>
       </c>
       <c r="F311" s="9" t="s">
         <v>28</v>
@@ -9127,7 +9127,7 @@
         <v>27</v>
       </c>
       <c r="E312" s="11">
-        <v>13</v>
+        <v>23</v>
       </c>
       <c r="F312" s="9" t="s">
         <v>28</v>
@@ -9150,7 +9150,7 @@
         <v>27</v>
       </c>
       <c r="E313" s="11">
-        <v>11</v>
+        <v>21</v>
       </c>
       <c r="F313" s="9" t="s">
         <v>28</v>
@@ -9173,7 +9173,7 @@
         <v>27</v>
       </c>
       <c r="E314" s="11">
-        <v>16</v>
+        <v>24</v>
       </c>
       <c r="F314" s="9" t="s">
         <v>28</v>
@@ -9196,7 +9196,7 @@
         <v>27</v>
       </c>
       <c r="E315" s="11">
-        <v>17</v>
+        <v>31</v>
       </c>
       <c r="F315" s="9" t="s">
         <v>28</v>
@@ -9219,7 +9219,7 @@
         <v>27</v>
       </c>
       <c r="E316" s="11">
-        <v>14</v>
+        <v>28</v>
       </c>
       <c r="F316" s="9" t="s">
         <v>28</v>
@@ -9242,7 +9242,7 @@
         <v>27</v>
       </c>
       <c r="E317" s="11">
-        <v>26</v>
+        <v>15</v>
       </c>
       <c r="F317" s="9" t="s">
         <v>28</v>
@@ -9265,7 +9265,7 @@
         <v>27</v>
       </c>
       <c r="E318" s="11">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="F318" s="9" t="s">
         <v>28</v>
@@ -9288,7 +9288,7 @@
         <v>27</v>
       </c>
       <c r="E319" s="11">
-        <v>15</v>
+        <v>10</v>
       </c>
       <c r="F319" s="9" t="s">
         <v>28</v>
@@ -9311,7 +9311,7 @@
         <v>27</v>
       </c>
       <c r="E320" s="11">
-        <v>10</v>
+        <v>14</v>
       </c>
       <c r="F320" s="9" t="s">
         <v>28</v>
@@ -9334,7 +9334,7 @@
         <v>27</v>
       </c>
       <c r="E321" s="11">
-        <v>25</v>
+        <v>8</v>
       </c>
       <c r="F321" s="9" t="s">
         <v>28</v>
@@ -9357,7 +9357,7 @@
         <v>27</v>
       </c>
       <c r="E322" s="11">
-        <v>11</v>
+        <v>15</v>
       </c>
       <c r="F322" s="9" t="s">
         <v>28</v>
@@ -9380,7 +9380,7 @@
         <v>27</v>
       </c>
       <c r="E323" s="11">
-        <v>15</v>
+        <v>24</v>
       </c>
       <c r="F323" s="9" t="s">
         <v>28</v>
@@ -9403,7 +9403,7 @@
         <v>27</v>
       </c>
       <c r="E324" s="11">
-        <v>13</v>
+        <v>16</v>
       </c>
       <c r="F324" s="9" t="s">
         <v>28</v>
@@ -9426,7 +9426,7 @@
         <v>27</v>
       </c>
       <c r="E325" s="11">
-        <v>16</v>
+        <v>14</v>
       </c>
       <c r="F325" s="9" t="s">
         <v>28</v>
@@ -9449,7 +9449,7 @@
         <v>27</v>
       </c>
       <c r="E326" s="11">
-        <v>24</v>
+        <v>9</v>
       </c>
       <c r="F326" s="9" t="s">
         <v>28</v>
@@ -9472,7 +9472,7 @@
         <v>27</v>
       </c>
       <c r="E327" s="11">
-        <v>9</v>
+        <v>30</v>
       </c>
       <c r="F327" s="9" t="s">
         <v>28</v>
@@ -9495,7 +9495,7 @@
         <v>27</v>
       </c>
       <c r="E328" s="11">
-        <v>15</v>
+        <v>9</v>
       </c>
       <c r="F328" s="9" t="s">
         <v>28</v>
@@ -9518,7 +9518,7 @@
         <v>27</v>
       </c>
       <c r="E329" s="11">
-        <v>14</v>
+        <v>22</v>
       </c>
       <c r="F329" s="9" t="s">
         <v>28</v>
@@ -9541,7 +9541,7 @@
         <v>27</v>
       </c>
       <c r="E330" s="11">
-        <v>30</v>
+        <v>23</v>
       </c>
       <c r="F330" s="9" t="s">
         <v>28</v>
@@ -9564,7 +9564,7 @@
         <v>27</v>
       </c>
       <c r="E331" s="11">
-        <v>27</v>
+        <v>10</v>
       </c>
       <c r="F331" s="9" t="s">
         <v>28</v>
@@ -9587,7 +9587,7 @@
         <v>27</v>
       </c>
       <c r="E332" s="11">
-        <v>23</v>
+        <v>29</v>
       </c>
       <c r="F332" s="9" t="s">
         <v>28</v>
@@ -9610,7 +9610,7 @@
         <v>27</v>
       </c>
       <c r="E333" s="11">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="F333" s="9" t="s">
         <v>28</v>
@@ -9633,7 +9633,7 @@
         <v>27</v>
       </c>
       <c r="E334" s="11">
-        <v>29</v>
+        <v>21</v>
       </c>
       <c r="F334" s="9" t="s">
         <v>28</v>
@@ -9656,7 +9656,7 @@
         <v>27</v>
       </c>
       <c r="E335" s="11">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="F335" s="9" t="s">
         <v>28</v>
@@ -9679,7 +9679,7 @@
         <v>27</v>
       </c>
       <c r="E336" s="11">
-        <v>13</v>
+        <v>31</v>
       </c>
       <c r="F336" s="9" t="s">
         <v>28</v>
@@ -9702,7 +9702,7 @@
         <v>27</v>
       </c>
       <c r="E337" s="11">
-        <v>21</v>
+        <v>15</v>
       </c>
       <c r="F337" s="9" t="s">
         <v>28</v>
@@ -9725,7 +9725,7 @@
         <v>27</v>
       </c>
       <c r="E338" s="11">
-        <v>24</v>
+        <v>13</v>
       </c>
       <c r="F338" s="9" t="s">
         <v>28</v>
@@ -9748,7 +9748,7 @@
         <v>27</v>
       </c>
       <c r="E339" s="11">
-        <v>15</v>
+        <v>11</v>
       </c>
       <c r="F339" s="9" t="s">
         <v>28</v>
@@ -9771,7 +9771,7 @@
         <v>27</v>
       </c>
       <c r="E340" s="11">
-        <v>27</v>
+        <v>10</v>
       </c>
       <c r="F340" s="9" t="s">
         <v>28</v>
@@ -9794,7 +9794,7 @@
         <v>27</v>
       </c>
       <c r="E341" s="11">
-        <v>21</v>
+        <v>17</v>
       </c>
       <c r="F341" s="9" t="s">
         <v>28</v>
@@ -9817,7 +9817,7 @@
         <v>27</v>
       </c>
       <c r="E342" s="11">
-        <v>18</v>
+        <v>24</v>
       </c>
       <c r="F342" s="9" t="s">
         <v>28</v>
@@ -9840,7 +9840,7 @@
         <v>27</v>
       </c>
       <c r="E343" s="11">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="F343" s="9" t="s">
         <v>28</v>
@@ -9863,7 +9863,7 @@
         <v>27</v>
       </c>
       <c r="E344" s="11">
-        <v>27</v>
+        <v>23</v>
       </c>
       <c r="F344" s="9" t="s">
         <v>28</v>
@@ -9886,7 +9886,7 @@
         <v>27</v>
       </c>
       <c r="E345" s="11">
-        <v>12</v>
+        <v>15</v>
       </c>
       <c r="F345" s="9" t="s">
         <v>28</v>
@@ -9909,7 +9909,7 @@
         <v>27</v>
       </c>
       <c r="E346" s="11">
-        <v>13</v>
+        <v>17</v>
       </c>
       <c r="F346" s="9" t="s">
         <v>28</v>
@@ -9932,7 +9932,7 @@
         <v>27</v>
       </c>
       <c r="E347" s="11">
-        <v>20</v>
+        <v>31</v>
       </c>
       <c r="F347" s="9" t="s">
         <v>28</v>
@@ -9955,7 +9955,7 @@
         <v>27</v>
       </c>
       <c r="E348" s="11">
-        <v>24</v>
+        <v>14</v>
       </c>
       <c r="F348" s="9" t="s">
         <v>28</v>
@@ -9978,7 +9978,7 @@
         <v>27</v>
       </c>
       <c r="E349" s="11">
-        <v>16</v>
+        <v>25</v>
       </c>
       <c r="F349" s="9" t="s">
         <v>28</v>
@@ -10001,7 +10001,7 @@
         <v>27</v>
       </c>
       <c r="E350" s="11">
-        <v>9</v>
+        <v>18</v>
       </c>
       <c r="F350" s="9" t="s">
         <v>28</v>
@@ -10024,7 +10024,7 @@
         <v>27</v>
       </c>
       <c r="E351" s="11">
-        <v>20</v>
+        <v>13</v>
       </c>
       <c r="F351" s="9" t="s">
         <v>28</v>
@@ -10047,7 +10047,7 @@
         <v>27</v>
       </c>
       <c r="E352" s="11">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="F352" s="9" t="s">
         <v>28</v>
@@ -10070,7 +10070,7 @@
         <v>27</v>
       </c>
       <c r="E353" s="11">
-        <v>15</v>
+        <v>11</v>
       </c>
       <c r="F353" s="9" t="s">
         <v>28</v>
@@ -10093,7 +10093,7 @@
         <v>27</v>
       </c>
       <c r="E354" s="11">
-        <v>26</v>
+        <v>17</v>
       </c>
       <c r="F354" s="9" t="s">
         <v>28</v>
@@ -10116,7 +10116,7 @@
         <v>27</v>
       </c>
       <c r="E355" s="11">
-        <v>9</v>
+        <v>19</v>
       </c>
       <c r="F355" s="9" t="s">
         <v>28</v>
@@ -10139,7 +10139,7 @@
         <v>27</v>
       </c>
       <c r="E356" s="11">
-        <v>29</v>
+        <v>22</v>
       </c>
       <c r="F356" s="9" t="s">
         <v>28</v>
@@ -10162,7 +10162,7 @@
         <v>27</v>
       </c>
       <c r="E357" s="11">
-        <v>25</v>
+        <v>17</v>
       </c>
       <c r="F357" s="9" t="s">
         <v>28</v>
@@ -10185,7 +10185,7 @@
         <v>27</v>
       </c>
       <c r="E358" s="11">
-        <v>27</v>
+        <v>10</v>
       </c>
       <c r="F358" s="9" t="s">
         <v>28</v>
@@ -10208,7 +10208,7 @@
         <v>27</v>
       </c>
       <c r="E359" s="11">
-        <v>23</v>
+        <v>15</v>
       </c>
       <c r="F359" s="9" t="s">
         <v>28</v>
@@ -10231,7 +10231,7 @@
         <v>27</v>
       </c>
       <c r="E360" s="11">
-        <v>19</v>
+        <v>10</v>
       </c>
       <c r="F360" s="9" t="s">
         <v>28</v>
@@ -10254,7 +10254,7 @@
         <v>27</v>
       </c>
       <c r="E361" s="11">
-        <v>24</v>
+        <v>31</v>
       </c>
       <c r="F361" s="9" t="s">
         <v>28</v>
@@ -10277,7 +10277,7 @@
         <v>27</v>
       </c>
       <c r="E362" s="11">
-        <v>25</v>
+        <v>30</v>
       </c>
       <c r="F362" s="9" t="s">
         <v>28</v>
@@ -10300,7 +10300,7 @@
         <v>27</v>
       </c>
       <c r="E363" s="11">
-        <v>23</v>
+        <v>26</v>
       </c>
       <c r="F363" s="9" t="s">
         <v>28</v>
@@ -10323,7 +10323,7 @@
         <v>27</v>
       </c>
       <c r="E364" s="11">
-        <v>28</v>
+        <v>10</v>
       </c>
       <c r="F364" s="9" t="s">
         <v>28</v>
@@ -10346,7 +10346,7 @@
         <v>27</v>
       </c>
       <c r="E365" s="11">
-        <v>17</v>
+        <v>11</v>
       </c>
       <c r="F365" s="9" t="s">
         <v>28</v>
@@ -10369,7 +10369,7 @@
         <v>27</v>
       </c>
       <c r="E366" s="11">
-        <v>30</v>
+        <v>12</v>
       </c>
       <c r="F366" s="9" t="s">
         <v>28</v>
@@ -10392,7 +10392,7 @@
         <v>27</v>
       </c>
       <c r="E367" s="11">
-        <v>15</v>
+        <v>21</v>
       </c>
       <c r="F367" s="9" t="s">
         <v>28</v>
@@ -10415,7 +10415,7 @@
         <v>27</v>
       </c>
       <c r="E368" s="11">
-        <v>16</v>
+        <v>21</v>
       </c>
       <c r="F368" s="9" t="s">
         <v>28</v>
@@ -10438,7 +10438,7 @@
         <v>27</v>
       </c>
       <c r="E369" s="11">
-        <v>25</v>
+        <v>15</v>
       </c>
       <c r="F369" s="9" t="s">
         <v>28</v>
@@ -10461,7 +10461,7 @@
         <v>27</v>
       </c>
       <c r="E370" s="11">
-        <v>30</v>
+        <v>19</v>
       </c>
       <c r="F370" s="9" t="s">
         <v>28</v>
@@ -10484,7 +10484,7 @@
         <v>27</v>
       </c>
       <c r="E371" s="11">
-        <v>29</v>
+        <v>15</v>
       </c>
       <c r="F371" s="9" t="s">
         <v>28</v>
@@ -10507,7 +10507,7 @@
         <v>27</v>
       </c>
       <c r="E372" s="11">
-        <v>30</v>
+        <v>12</v>
       </c>
       <c r="F372" s="9" t="s">
         <v>28</v>
@@ -10530,7 +10530,7 @@
         <v>27</v>
       </c>
       <c r="E373" s="11">
-        <v>28</v>
+        <v>17</v>
       </c>
       <c r="F373" s="9" t="s">
         <v>28</v>
@@ -10553,7 +10553,7 @@
         <v>27</v>
       </c>
       <c r="E374" s="11">
-        <v>24</v>
+        <v>13</v>
       </c>
       <c r="F374" s="9" t="s">
         <v>28</v>
@@ -10576,7 +10576,7 @@
         <v>27</v>
       </c>
       <c r="E375" s="11">
-        <v>24</v>
+        <v>15</v>
       </c>
       <c r="F375" s="9" t="s">
         <v>28</v>
@@ -10599,7 +10599,7 @@
         <v>27</v>
       </c>
       <c r="E376" s="11">
-        <v>13</v>
+        <v>19</v>
       </c>
       <c r="F376" s="9" t="s">
         <v>28</v>
@@ -10622,7 +10622,7 @@
         <v>27</v>
       </c>
       <c r="E377" s="11">
-        <v>19</v>
+        <v>11</v>
       </c>
       <c r="F377" s="9" t="s">
         <v>28</v>
@@ -10645,7 +10645,7 @@
         <v>27</v>
       </c>
       <c r="E378" s="11">
-        <v>22</v>
+        <v>27</v>
       </c>
       <c r="F378" s="9" t="s">
         <v>28</v>
@@ -10668,7 +10668,7 @@
         <v>27</v>
       </c>
       <c r="E379" s="11">
-        <v>28</v>
+        <v>26</v>
       </c>
       <c r="F379" s="9" t="s">
         <v>28</v>
@@ -10691,7 +10691,7 @@
         <v>27</v>
       </c>
       <c r="E380" s="11">
-        <v>31</v>
+        <v>29</v>
       </c>
       <c r="F380" s="9" t="s">
         <v>28</v>
@@ -10714,7 +10714,7 @@
         <v>27</v>
       </c>
       <c r="E381" s="11">
-        <v>21</v>
+        <v>9</v>
       </c>
       <c r="F381" s="9" t="s">
         <v>28</v>
@@ -10737,7 +10737,7 @@
         <v>27</v>
       </c>
       <c r="E382" s="11">
-        <v>16</v>
+        <v>18</v>
       </c>
       <c r="F382" s="9" t="s">
         <v>28</v>
@@ -10760,7 +10760,7 @@
         <v>27</v>
       </c>
       <c r="E383" s="11">
-        <v>29</v>
+        <v>13</v>
       </c>
       <c r="F383" s="9" t="s">
         <v>28</v>
@@ -10783,7 +10783,7 @@
         <v>27</v>
       </c>
       <c r="E384" s="11">
-        <v>14</v>
+        <v>24</v>
       </c>
       <c r="F384" s="9" t="s">
         <v>28</v>
@@ -10806,7 +10806,7 @@
         <v>27</v>
       </c>
       <c r="E385" s="11">
-        <v>12</v>
+        <v>31</v>
       </c>
       <c r="F385" s="9" t="s">
         <v>28</v>
@@ -10829,7 +10829,7 @@
         <v>27</v>
       </c>
       <c r="E386" s="11">
-        <v>20</v>
+        <v>22</v>
       </c>
       <c r="F386" s="9" t="s">
         <v>28</v>
@@ -10852,7 +10852,7 @@
         <v>27</v>
       </c>
       <c r="E387" s="11">
-        <v>31</v>
+        <v>26</v>
       </c>
       <c r="F387" s="9" t="s">
         <v>28</v>
@@ -10875,7 +10875,7 @@
         <v>27</v>
       </c>
       <c r="E388" s="11">
-        <v>26</v>
+        <v>9</v>
       </c>
       <c r="F388" s="9" t="s">
         <v>28</v>
@@ -10898,7 +10898,7 @@
         <v>27</v>
       </c>
       <c r="E389" s="11">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="F389" s="9" t="s">
         <v>28</v>
@@ -10921,7 +10921,7 @@
         <v>27</v>
       </c>
       <c r="E390" s="11">
-        <v>10</v>
+        <v>17</v>
       </c>
       <c r="F390" s="9" t="s">
         <v>28</v>
@@ -10944,7 +10944,7 @@
         <v>27</v>
       </c>
       <c r="E391" s="11">
-        <v>18</v>
+        <v>26</v>
       </c>
       <c r="F391" s="9" t="s">
         <v>28</v>
@@ -10967,7 +10967,7 @@
         <v>27</v>
       </c>
       <c r="E392" s="11">
-        <v>18</v>
+        <v>11</v>
       </c>
       <c r="F392" s="9" t="s">
         <v>28</v>
@@ -10990,7 +10990,7 @@
         <v>27</v>
       </c>
       <c r="E393" s="11">
-        <v>8</v>
+        <v>14</v>
       </c>
       <c r="F393" s="9" t="s">
         <v>28</v>
@@ -11013,7 +11013,7 @@
         <v>27</v>
       </c>
       <c r="E394" s="11">
-        <v>11</v>
+        <v>18</v>
       </c>
       <c r="F394" s="9" t="s">
         <v>28</v>
@@ -11036,7 +11036,7 @@
         <v>27</v>
       </c>
       <c r="E395" s="11">
-        <v>11</v>
+        <v>18</v>
       </c>
       <c r="F395" s="9" t="s">
         <v>28</v>
@@ -11059,7 +11059,7 @@
         <v>27</v>
       </c>
       <c r="E396" s="11">
-        <v>15</v>
+        <v>21</v>
       </c>
       <c r="F396" s="9" t="s">
         <v>28</v>
@@ -11082,7 +11082,7 @@
         <v>27</v>
       </c>
       <c r="E397" s="11">
-        <v>28</v>
+        <v>31</v>
       </c>
       <c r="F397" s="9" t="s">
         <v>28</v>
@@ -11105,7 +11105,7 @@
         <v>27</v>
       </c>
       <c r="E398" s="11">
-        <v>28</v>
+        <v>20</v>
       </c>
       <c r="F398" s="9" t="s">
         <v>28</v>
@@ -11128,7 +11128,7 @@
         <v>27</v>
       </c>
       <c r="E399" s="11">
-        <v>17</v>
+        <v>22</v>
       </c>
       <c r="F399" s="9" t="s">
         <v>28</v>
@@ -11151,7 +11151,7 @@
         <v>27</v>
       </c>
       <c r="E400" s="11">
-        <v>20</v>
+        <v>13</v>
       </c>
       <c r="F400" s="9" t="s">
         <v>28</v>
@@ -11174,7 +11174,7 @@
         <v>27</v>
       </c>
       <c r="E401" s="11">
-        <v>17</v>
+        <v>20</v>
       </c>
       <c r="F401" s="9" t="s">
         <v>28</v>

</xml_diff>

<commit_message>
fix(badges): hide Verified and Trust Score badges until user actually lends or borrows an item
</commit_message>
<xml_diff>
--- a/all-test-reports/selenium/selenium_e2e_test_report.xlsx
+++ b/all-test-reports/selenium/selenium_e2e_test_report.xlsx
@@ -35,7 +35,7 @@
     <t>Execution Date</t>
   </si>
   <si>
-    <t>28/7/2026, 11:08:29 am</t>
+    <t>28/7/2026, 11:12:55 am</t>
   </si>
   <si>
     <t>Browser / Mode</t>
@@ -98,7 +98,7 @@
     <t>PASS</t>
   </si>
   <si>
-    <t>11:08:29 am</t>
+    <t>11:12:55 am</t>
   </si>
   <si>
     <t>N/A</t>
@@ -1997,7 +1997,7 @@
         <v>27</v>
       </c>
       <c r="E2" s="11">
-        <v>17</v>
+        <v>9</v>
       </c>
       <c r="F2" s="9" t="s">
         <v>28</v>
@@ -2020,7 +2020,7 @@
         <v>27</v>
       </c>
       <c r="E3" s="11">
-        <v>12</v>
+        <v>21</v>
       </c>
       <c r="F3" s="9" t="s">
         <v>28</v>
@@ -2043,7 +2043,7 @@
         <v>27</v>
       </c>
       <c r="E4" s="11">
-        <v>22</v>
+        <v>19</v>
       </c>
       <c r="F4" s="9" t="s">
         <v>28</v>
@@ -2066,7 +2066,7 @@
         <v>27</v>
       </c>
       <c r="E5" s="11">
-        <v>21</v>
+        <v>9</v>
       </c>
       <c r="F5" s="9" t="s">
         <v>28</v>
@@ -2089,7 +2089,7 @@
         <v>27</v>
       </c>
       <c r="E6" s="11">
-        <v>27</v>
+        <v>18</v>
       </c>
       <c r="F6" s="9" t="s">
         <v>28</v>
@@ -2112,7 +2112,7 @@
         <v>27</v>
       </c>
       <c r="E7" s="11">
-        <v>24</v>
+        <v>21</v>
       </c>
       <c r="F7" s="9" t="s">
         <v>28</v>
@@ -2135,7 +2135,7 @@
         <v>27</v>
       </c>
       <c r="E8" s="11">
-        <v>29</v>
+        <v>23</v>
       </c>
       <c r="F8" s="9" t="s">
         <v>28</v>
@@ -2158,7 +2158,7 @@
         <v>27</v>
       </c>
       <c r="E9" s="11">
-        <v>11</v>
+        <v>17</v>
       </c>
       <c r="F9" s="9" t="s">
         <v>28</v>
@@ -2181,7 +2181,7 @@
         <v>27</v>
       </c>
       <c r="E10" s="11">
-        <v>23</v>
+        <v>8</v>
       </c>
       <c r="F10" s="9" t="s">
         <v>28</v>
@@ -2204,7 +2204,7 @@
         <v>27</v>
       </c>
       <c r="E11" s="11">
-        <v>31</v>
+        <v>13</v>
       </c>
       <c r="F11" s="9" t="s">
         <v>28</v>
@@ -2227,7 +2227,7 @@
         <v>27</v>
       </c>
       <c r="E12" s="11">
-        <v>17</v>
+        <v>31</v>
       </c>
       <c r="F12" s="9" t="s">
         <v>28</v>
@@ -2250,7 +2250,7 @@
         <v>27</v>
       </c>
       <c r="E13" s="11">
-        <v>13</v>
+        <v>25</v>
       </c>
       <c r="F13" s="9" t="s">
         <v>28</v>
@@ -2273,7 +2273,7 @@
         <v>27</v>
       </c>
       <c r="E14" s="11">
-        <v>21</v>
+        <v>18</v>
       </c>
       <c r="F14" s="9" t="s">
         <v>28</v>
@@ -2296,7 +2296,7 @@
         <v>27</v>
       </c>
       <c r="E15" s="11">
-        <v>22</v>
+        <v>16</v>
       </c>
       <c r="F15" s="9" t="s">
         <v>28</v>
@@ -2319,7 +2319,7 @@
         <v>27</v>
       </c>
       <c r="E16" s="11">
-        <v>11</v>
+        <v>19</v>
       </c>
       <c r="F16" s="9" t="s">
         <v>28</v>
@@ -2342,7 +2342,7 @@
         <v>27</v>
       </c>
       <c r="E17" s="11">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="F17" s="9" t="s">
         <v>28</v>
@@ -2365,7 +2365,7 @@
         <v>27</v>
       </c>
       <c r="E18" s="11">
-        <v>18</v>
+        <v>25</v>
       </c>
       <c r="F18" s="9" t="s">
         <v>28</v>
@@ -2388,7 +2388,7 @@
         <v>27</v>
       </c>
       <c r="E19" s="11">
-        <v>11</v>
+        <v>19</v>
       </c>
       <c r="F19" s="9" t="s">
         <v>28</v>
@@ -2411,7 +2411,7 @@
         <v>27</v>
       </c>
       <c r="E20" s="11">
-        <v>25</v>
+        <v>14</v>
       </c>
       <c r="F20" s="9" t="s">
         <v>28</v>
@@ -2434,7 +2434,7 @@
         <v>27</v>
       </c>
       <c r="E21" s="11">
-        <v>12</v>
+        <v>19</v>
       </c>
       <c r="F21" s="9" t="s">
         <v>28</v>
@@ -2457,7 +2457,7 @@
         <v>27</v>
       </c>
       <c r="E22" s="11">
-        <v>29</v>
+        <v>14</v>
       </c>
       <c r="F22" s="9" t="s">
         <v>28</v>
@@ -2480,7 +2480,7 @@
         <v>27</v>
       </c>
       <c r="E23" s="11">
-        <v>26</v>
+        <v>9</v>
       </c>
       <c r="F23" s="9" t="s">
         <v>28</v>
@@ -2503,7 +2503,7 @@
         <v>27</v>
       </c>
       <c r="E24" s="11">
-        <v>8</v>
+        <v>18</v>
       </c>
       <c r="F24" s="9" t="s">
         <v>28</v>
@@ -2526,7 +2526,7 @@
         <v>27</v>
       </c>
       <c r="E25" s="11">
-        <v>19</v>
+        <v>9</v>
       </c>
       <c r="F25" s="9" t="s">
         <v>28</v>
@@ -2549,7 +2549,7 @@
         <v>27</v>
       </c>
       <c r="E26" s="11">
-        <v>13</v>
+        <v>30</v>
       </c>
       <c r="F26" s="9" t="s">
         <v>28</v>
@@ -2572,7 +2572,7 @@
         <v>27</v>
       </c>
       <c r="E27" s="11">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="F27" s="9" t="s">
         <v>28</v>
@@ -2595,7 +2595,7 @@
         <v>27</v>
       </c>
       <c r="E28" s="11">
-        <v>28</v>
+        <v>31</v>
       </c>
       <c r="F28" s="9" t="s">
         <v>28</v>
@@ -2618,7 +2618,7 @@
         <v>27</v>
       </c>
       <c r="E29" s="11">
-        <v>22</v>
+        <v>14</v>
       </c>
       <c r="F29" s="9" t="s">
         <v>28</v>
@@ -2641,7 +2641,7 @@
         <v>27</v>
       </c>
       <c r="E30" s="11">
-        <v>11</v>
+        <v>30</v>
       </c>
       <c r="F30" s="9" t="s">
         <v>28</v>
@@ -2664,7 +2664,7 @@
         <v>27</v>
       </c>
       <c r="E31" s="11">
-        <v>21</v>
+        <v>15</v>
       </c>
       <c r="F31" s="9" t="s">
         <v>28</v>
@@ -2687,7 +2687,7 @@
         <v>27</v>
       </c>
       <c r="E32" s="11">
-        <v>16</v>
+        <v>10</v>
       </c>
       <c r="F32" s="9" t="s">
         <v>28</v>
@@ -2710,7 +2710,7 @@
         <v>27</v>
       </c>
       <c r="E33" s="11">
-        <v>26</v>
+        <v>12</v>
       </c>
       <c r="F33" s="9" t="s">
         <v>28</v>
@@ -2733,7 +2733,7 @@
         <v>27</v>
       </c>
       <c r="E34" s="11">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="F34" s="9" t="s">
         <v>28</v>
@@ -2756,7 +2756,7 @@
         <v>27</v>
       </c>
       <c r="E35" s="11">
-        <v>11</v>
+        <v>18</v>
       </c>
       <c r="F35" s="9" t="s">
         <v>28</v>
@@ -2779,7 +2779,7 @@
         <v>27</v>
       </c>
       <c r="E36" s="11">
-        <v>11</v>
+        <v>20</v>
       </c>
       <c r="F36" s="9" t="s">
         <v>28</v>
@@ -2802,7 +2802,7 @@
         <v>27</v>
       </c>
       <c r="E37" s="11">
-        <v>9</v>
+        <v>31</v>
       </c>
       <c r="F37" s="9" t="s">
         <v>28</v>
@@ -2825,7 +2825,7 @@
         <v>27</v>
       </c>
       <c r="E38" s="11">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="F38" s="9" t="s">
         <v>28</v>
@@ -2848,7 +2848,7 @@
         <v>27</v>
       </c>
       <c r="E39" s="11">
-        <v>15</v>
+        <v>8</v>
       </c>
       <c r="F39" s="9" t="s">
         <v>28</v>
@@ -2871,7 +2871,7 @@
         <v>27</v>
       </c>
       <c r="E40" s="11">
-        <v>14</v>
+        <v>27</v>
       </c>
       <c r="F40" s="9" t="s">
         <v>28</v>
@@ -2894,7 +2894,7 @@
         <v>27</v>
       </c>
       <c r="E41" s="11">
-        <v>16</v>
+        <v>31</v>
       </c>
       <c r="F41" s="9" t="s">
         <v>28</v>
@@ -2917,7 +2917,7 @@
         <v>27</v>
       </c>
       <c r="E42" s="11">
-        <v>20</v>
+        <v>16</v>
       </c>
       <c r="F42" s="9" t="s">
         <v>28</v>
@@ -2940,7 +2940,7 @@
         <v>27</v>
       </c>
       <c r="E43" s="11">
-        <v>19</v>
+        <v>15</v>
       </c>
       <c r="F43" s="9" t="s">
         <v>28</v>
@@ -2963,7 +2963,7 @@
         <v>27</v>
       </c>
       <c r="E44" s="11">
-        <v>20</v>
+        <v>15</v>
       </c>
       <c r="F44" s="9" t="s">
         <v>28</v>
@@ -2986,7 +2986,7 @@
         <v>27</v>
       </c>
       <c r="E45" s="11">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="F45" s="9" t="s">
         <v>28</v>
@@ -3009,7 +3009,7 @@
         <v>27</v>
       </c>
       <c r="E46" s="11">
-        <v>14</v>
+        <v>18</v>
       </c>
       <c r="F46" s="9" t="s">
         <v>28</v>
@@ -3055,7 +3055,7 @@
         <v>27</v>
       </c>
       <c r="E48" s="11">
-        <v>30</v>
+        <v>10</v>
       </c>
       <c r="F48" s="9" t="s">
         <v>28</v>
@@ -3078,7 +3078,7 @@
         <v>27</v>
       </c>
       <c r="E49" s="11">
-        <v>17</v>
+        <v>31</v>
       </c>
       <c r="F49" s="9" t="s">
         <v>28</v>
@@ -3101,7 +3101,7 @@
         <v>27</v>
       </c>
       <c r="E50" s="11">
-        <v>9</v>
+        <v>23</v>
       </c>
       <c r="F50" s="9" t="s">
         <v>28</v>
@@ -3124,7 +3124,7 @@
         <v>27</v>
       </c>
       <c r="E51" s="11">
-        <v>26</v>
+        <v>19</v>
       </c>
       <c r="F51" s="9" t="s">
         <v>28</v>
@@ -3147,7 +3147,7 @@
         <v>27</v>
       </c>
       <c r="E52" s="11">
-        <v>27</v>
+        <v>12</v>
       </c>
       <c r="F52" s="9" t="s">
         <v>28</v>
@@ -3170,7 +3170,7 @@
         <v>27</v>
       </c>
       <c r="E53" s="11">
-        <v>17</v>
+        <v>20</v>
       </c>
       <c r="F53" s="9" t="s">
         <v>28</v>
@@ -3216,7 +3216,7 @@
         <v>27</v>
       </c>
       <c r="E55" s="11">
-        <v>11</v>
+        <v>19</v>
       </c>
       <c r="F55" s="9" t="s">
         <v>28</v>
@@ -3239,7 +3239,7 @@
         <v>27</v>
       </c>
       <c r="E56" s="11">
-        <v>9</v>
+        <v>11</v>
       </c>
       <c r="F56" s="9" t="s">
         <v>28</v>
@@ -3262,7 +3262,7 @@
         <v>27</v>
       </c>
       <c r="E57" s="11">
-        <v>21</v>
+        <v>18</v>
       </c>
       <c r="F57" s="9" t="s">
         <v>28</v>
@@ -3285,7 +3285,7 @@
         <v>27</v>
       </c>
       <c r="E58" s="11">
-        <v>30</v>
+        <v>19</v>
       </c>
       <c r="F58" s="9" t="s">
         <v>28</v>
@@ -3308,7 +3308,7 @@
         <v>27</v>
       </c>
       <c r="E59" s="11">
-        <v>29</v>
+        <v>27</v>
       </c>
       <c r="F59" s="9" t="s">
         <v>28</v>
@@ -3331,7 +3331,7 @@
         <v>27</v>
       </c>
       <c r="E60" s="11">
-        <v>10</v>
+        <v>18</v>
       </c>
       <c r="F60" s="9" t="s">
         <v>28</v>
@@ -3354,7 +3354,7 @@
         <v>27</v>
       </c>
       <c r="E61" s="11">
-        <v>31</v>
+        <v>11</v>
       </c>
       <c r="F61" s="9" t="s">
         <v>28</v>
@@ -3377,7 +3377,7 @@
         <v>27</v>
       </c>
       <c r="E62" s="11">
-        <v>27</v>
+        <v>9</v>
       </c>
       <c r="F62" s="9" t="s">
         <v>28</v>
@@ -3400,7 +3400,7 @@
         <v>27</v>
       </c>
       <c r="E63" s="11">
-        <v>30</v>
+        <v>12</v>
       </c>
       <c r="F63" s="9" t="s">
         <v>28</v>
@@ -3423,7 +3423,7 @@
         <v>27</v>
       </c>
       <c r="E64" s="11">
-        <v>29</v>
+        <v>17</v>
       </c>
       <c r="F64" s="9" t="s">
         <v>28</v>
@@ -3446,7 +3446,7 @@
         <v>27</v>
       </c>
       <c r="E65" s="11">
-        <v>11</v>
+        <v>23</v>
       </c>
       <c r="F65" s="9" t="s">
         <v>28</v>
@@ -3469,7 +3469,7 @@
         <v>27</v>
       </c>
       <c r="E66" s="11">
-        <v>15</v>
+        <v>11</v>
       </c>
       <c r="F66" s="9" t="s">
         <v>28</v>
@@ -3492,7 +3492,7 @@
         <v>27</v>
       </c>
       <c r="E67" s="11">
-        <v>27</v>
+        <v>12</v>
       </c>
       <c r="F67" s="9" t="s">
         <v>28</v>
@@ -3515,7 +3515,7 @@
         <v>27</v>
       </c>
       <c r="E68" s="11">
-        <v>23</v>
+        <v>15</v>
       </c>
       <c r="F68" s="9" t="s">
         <v>28</v>
@@ -3538,7 +3538,7 @@
         <v>27</v>
       </c>
       <c r="E69" s="11">
-        <v>16</v>
+        <v>14</v>
       </c>
       <c r="F69" s="9" t="s">
         <v>28</v>
@@ -3561,7 +3561,7 @@
         <v>27</v>
       </c>
       <c r="E70" s="11">
-        <v>23</v>
+        <v>8</v>
       </c>
       <c r="F70" s="9" t="s">
         <v>28</v>
@@ -3584,7 +3584,7 @@
         <v>27</v>
       </c>
       <c r="E71" s="11">
-        <v>25</v>
+        <v>15</v>
       </c>
       <c r="F71" s="9" t="s">
         <v>28</v>
@@ -3607,7 +3607,7 @@
         <v>27</v>
       </c>
       <c r="E72" s="11">
-        <v>26</v>
+        <v>8</v>
       </c>
       <c r="F72" s="9" t="s">
         <v>28</v>
@@ -3630,7 +3630,7 @@
         <v>27</v>
       </c>
       <c r="E73" s="11">
-        <v>16</v>
+        <v>29</v>
       </c>
       <c r="F73" s="9" t="s">
         <v>28</v>
@@ -3653,7 +3653,7 @@
         <v>27</v>
       </c>
       <c r="E74" s="11">
-        <v>29</v>
+        <v>31</v>
       </c>
       <c r="F74" s="9" t="s">
         <v>28</v>
@@ -3676,7 +3676,7 @@
         <v>27</v>
       </c>
       <c r="E75" s="11">
-        <v>8</v>
+        <v>11</v>
       </c>
       <c r="F75" s="9" t="s">
         <v>28</v>
@@ -3699,7 +3699,7 @@
         <v>27</v>
       </c>
       <c r="E76" s="11">
-        <v>8</v>
+        <v>14</v>
       </c>
       <c r="F76" s="9" t="s">
         <v>28</v>
@@ -3722,7 +3722,7 @@
         <v>27</v>
       </c>
       <c r="E77" s="11">
-        <v>14</v>
+        <v>19</v>
       </c>
       <c r="F77" s="9" t="s">
         <v>28</v>
@@ -3745,7 +3745,7 @@
         <v>27</v>
       </c>
       <c r="E78" s="11">
-        <v>16</v>
+        <v>8</v>
       </c>
       <c r="F78" s="9" t="s">
         <v>28</v>
@@ -3768,7 +3768,7 @@
         <v>27</v>
       </c>
       <c r="E79" s="11">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="F79" s="9" t="s">
         <v>28</v>
@@ -3791,7 +3791,7 @@
         <v>27</v>
       </c>
       <c r="E80" s="11">
-        <v>25</v>
+        <v>27</v>
       </c>
       <c r="F80" s="9" t="s">
         <v>28</v>
@@ -3814,7 +3814,7 @@
         <v>27</v>
       </c>
       <c r="E81" s="11">
-        <v>29</v>
+        <v>24</v>
       </c>
       <c r="F81" s="9" t="s">
         <v>28</v>
@@ -3837,7 +3837,7 @@
         <v>27</v>
       </c>
       <c r="E82" s="11">
-        <v>17</v>
+        <v>15</v>
       </c>
       <c r="F82" s="9" t="s">
         <v>28</v>
@@ -3860,7 +3860,7 @@
         <v>27</v>
       </c>
       <c r="E83" s="11">
-        <v>29</v>
+        <v>14</v>
       </c>
       <c r="F83" s="9" t="s">
         <v>28</v>
@@ -3883,7 +3883,7 @@
         <v>27</v>
       </c>
       <c r="E84" s="11">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="F84" s="9" t="s">
         <v>28</v>
@@ -3906,7 +3906,7 @@
         <v>27</v>
       </c>
       <c r="E85" s="11">
-        <v>24</v>
+        <v>17</v>
       </c>
       <c r="F85" s="9" t="s">
         <v>28</v>
@@ -3929,7 +3929,7 @@
         <v>27</v>
       </c>
       <c r="E86" s="11">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="F86" s="9" t="s">
         <v>28</v>
@@ -3952,7 +3952,7 @@
         <v>27</v>
       </c>
       <c r="E87" s="11">
-        <v>31</v>
+        <v>27</v>
       </c>
       <c r="F87" s="9" t="s">
         <v>28</v>
@@ -3975,7 +3975,7 @@
         <v>27</v>
       </c>
       <c r="E88" s="11">
-        <v>19</v>
+        <v>10</v>
       </c>
       <c r="F88" s="9" t="s">
         <v>28</v>
@@ -3998,7 +3998,7 @@
         <v>27</v>
       </c>
       <c r="E89" s="11">
-        <v>20</v>
+        <v>25</v>
       </c>
       <c r="F89" s="9" t="s">
         <v>28</v>
@@ -4021,7 +4021,7 @@
         <v>27</v>
       </c>
       <c r="E90" s="11">
-        <v>9</v>
+        <v>26</v>
       </c>
       <c r="F90" s="9" t="s">
         <v>28</v>
@@ -4044,7 +4044,7 @@
         <v>27</v>
       </c>
       <c r="E91" s="11">
-        <v>22</v>
+        <v>27</v>
       </c>
       <c r="F91" s="9" t="s">
         <v>28</v>
@@ -4067,7 +4067,7 @@
         <v>27</v>
       </c>
       <c r="E92" s="11">
-        <v>30</v>
+        <v>18</v>
       </c>
       <c r="F92" s="9" t="s">
         <v>28</v>
@@ -4090,7 +4090,7 @@
         <v>27</v>
       </c>
       <c r="E93" s="11">
-        <v>30</v>
+        <v>23</v>
       </c>
       <c r="F93" s="9" t="s">
         <v>28</v>
@@ -4113,7 +4113,7 @@
         <v>27</v>
       </c>
       <c r="E94" s="11">
-        <v>19</v>
+        <v>22</v>
       </c>
       <c r="F94" s="9" t="s">
         <v>28</v>
@@ -4136,7 +4136,7 @@
         <v>27</v>
       </c>
       <c r="E95" s="11">
-        <v>31</v>
+        <v>29</v>
       </c>
       <c r="F95" s="9" t="s">
         <v>28</v>
@@ -4159,7 +4159,7 @@
         <v>27</v>
       </c>
       <c r="E96" s="11">
-        <v>18</v>
+        <v>30</v>
       </c>
       <c r="F96" s="9" t="s">
         <v>28</v>
@@ -4182,7 +4182,7 @@
         <v>27</v>
       </c>
       <c r="E97" s="11">
-        <v>18</v>
+        <v>14</v>
       </c>
       <c r="F97" s="9" t="s">
         <v>28</v>
@@ -4228,7 +4228,7 @@
         <v>27</v>
       </c>
       <c r="E99" s="11">
-        <v>20</v>
+        <v>11</v>
       </c>
       <c r="F99" s="9" t="s">
         <v>28</v>
@@ -4251,7 +4251,7 @@
         <v>27</v>
       </c>
       <c r="E100" s="11">
-        <v>10</v>
+        <v>31</v>
       </c>
       <c r="F100" s="9" t="s">
         <v>28</v>
@@ -4274,7 +4274,7 @@
         <v>27</v>
       </c>
       <c r="E101" s="11">
-        <v>30</v>
+        <v>27</v>
       </c>
       <c r="F101" s="9" t="s">
         <v>28</v>
@@ -4297,7 +4297,7 @@
         <v>27</v>
       </c>
       <c r="E102" s="11">
-        <v>27</v>
+        <v>12</v>
       </c>
       <c r="F102" s="9" t="s">
         <v>28</v>
@@ -4320,7 +4320,7 @@
         <v>27</v>
       </c>
       <c r="E103" s="11">
-        <v>19</v>
+        <v>25</v>
       </c>
       <c r="F103" s="9" t="s">
         <v>28</v>
@@ -4343,7 +4343,7 @@
         <v>27</v>
       </c>
       <c r="E104" s="11">
-        <v>10</v>
+        <v>16</v>
       </c>
       <c r="F104" s="9" t="s">
         <v>28</v>
@@ -4366,7 +4366,7 @@
         <v>27</v>
       </c>
       <c r="E105" s="11">
-        <v>20</v>
+        <v>26</v>
       </c>
       <c r="F105" s="9" t="s">
         <v>28</v>
@@ -4389,7 +4389,7 @@
         <v>27</v>
       </c>
       <c r="E106" s="11">
-        <v>16</v>
+        <v>31</v>
       </c>
       <c r="F106" s="9" t="s">
         <v>28</v>
@@ -4412,7 +4412,7 @@
         <v>27</v>
       </c>
       <c r="E107" s="11">
-        <v>16</v>
+        <v>29</v>
       </c>
       <c r="F107" s="9" t="s">
         <v>28</v>
@@ -4435,7 +4435,7 @@
         <v>27</v>
       </c>
       <c r="E108" s="11">
-        <v>16</v>
+        <v>14</v>
       </c>
       <c r="F108" s="9" t="s">
         <v>28</v>
@@ -4458,7 +4458,7 @@
         <v>27</v>
       </c>
       <c r="E109" s="11">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="F109" s="9" t="s">
         <v>28</v>
@@ -4481,7 +4481,7 @@
         <v>27</v>
       </c>
       <c r="E110" s="11">
-        <v>20</v>
+        <v>26</v>
       </c>
       <c r="F110" s="9" t="s">
         <v>28</v>
@@ -4504,7 +4504,7 @@
         <v>27</v>
       </c>
       <c r="E111" s="11">
-        <v>23</v>
+        <v>27</v>
       </c>
       <c r="F111" s="9" t="s">
         <v>28</v>
@@ -4527,7 +4527,7 @@
         <v>27</v>
       </c>
       <c r="E112" s="11">
-        <v>20</v>
+        <v>9</v>
       </c>
       <c r="F112" s="9" t="s">
         <v>28</v>
@@ -4550,7 +4550,7 @@
         <v>27</v>
       </c>
       <c r="E113" s="11">
-        <v>16</v>
+        <v>8</v>
       </c>
       <c r="F113" s="9" t="s">
         <v>28</v>
@@ -4573,7 +4573,7 @@
         <v>27</v>
       </c>
       <c r="E114" s="11">
-        <v>23</v>
+        <v>16</v>
       </c>
       <c r="F114" s="9" t="s">
         <v>28</v>
@@ -4596,7 +4596,7 @@
         <v>27</v>
       </c>
       <c r="E115" s="11">
-        <v>22</v>
+        <v>28</v>
       </c>
       <c r="F115" s="9" t="s">
         <v>28</v>
@@ -4619,7 +4619,7 @@
         <v>27</v>
       </c>
       <c r="E116" s="11">
-        <v>28</v>
+        <v>22</v>
       </c>
       <c r="F116" s="9" t="s">
         <v>28</v>
@@ -4642,7 +4642,7 @@
         <v>27</v>
       </c>
       <c r="E117" s="11">
-        <v>16</v>
+        <v>10</v>
       </c>
       <c r="F117" s="9" t="s">
         <v>28</v>
@@ -4688,7 +4688,7 @@
         <v>27</v>
       </c>
       <c r="E119" s="11">
-        <v>27</v>
+        <v>15</v>
       </c>
       <c r="F119" s="9" t="s">
         <v>28</v>
@@ -4711,7 +4711,7 @@
         <v>27</v>
       </c>
       <c r="E120" s="11">
-        <v>10</v>
+        <v>23</v>
       </c>
       <c r="F120" s="9" t="s">
         <v>28</v>
@@ -4734,7 +4734,7 @@
         <v>27</v>
       </c>
       <c r="E121" s="11">
-        <v>20</v>
+        <v>28</v>
       </c>
       <c r="F121" s="9" t="s">
         <v>28</v>
@@ -4803,7 +4803,7 @@
         <v>27</v>
       </c>
       <c r="E124" s="11">
-        <v>17</v>
+        <v>25</v>
       </c>
       <c r="F124" s="9" t="s">
         <v>28</v>
@@ -4826,7 +4826,7 @@
         <v>27</v>
       </c>
       <c r="E125" s="11">
-        <v>24</v>
+        <v>16</v>
       </c>
       <c r="F125" s="9" t="s">
         <v>28</v>
@@ -4849,7 +4849,7 @@
         <v>27</v>
       </c>
       <c r="E126" s="11">
-        <v>9</v>
+        <v>20</v>
       </c>
       <c r="F126" s="9" t="s">
         <v>28</v>
@@ -4872,7 +4872,7 @@
         <v>27</v>
       </c>
       <c r="E127" s="11">
-        <v>9</v>
+        <v>19</v>
       </c>
       <c r="F127" s="9" t="s">
         <v>28</v>
@@ -4895,7 +4895,7 @@
         <v>27</v>
       </c>
       <c r="E128" s="11">
-        <v>21</v>
+        <v>18</v>
       </c>
       <c r="F128" s="9" t="s">
         <v>28</v>
@@ -4918,7 +4918,7 @@
         <v>27</v>
       </c>
       <c r="E129" s="11">
-        <v>29</v>
+        <v>22</v>
       </c>
       <c r="F129" s="9" t="s">
         <v>28</v>
@@ -4941,7 +4941,7 @@
         <v>27</v>
       </c>
       <c r="E130" s="11">
-        <v>11</v>
+        <v>26</v>
       </c>
       <c r="F130" s="9" t="s">
         <v>28</v>
@@ -4964,7 +4964,7 @@
         <v>27</v>
       </c>
       <c r="E131" s="11">
-        <v>19</v>
+        <v>14</v>
       </c>
       <c r="F131" s="9" t="s">
         <v>28</v>
@@ -4987,7 +4987,7 @@
         <v>27</v>
       </c>
       <c r="E132" s="11">
-        <v>28</v>
+        <v>31</v>
       </c>
       <c r="F132" s="9" t="s">
         <v>28</v>
@@ -5010,7 +5010,7 @@
         <v>27</v>
       </c>
       <c r="E133" s="11">
-        <v>20</v>
+        <v>15</v>
       </c>
       <c r="F133" s="9" t="s">
         <v>28</v>
@@ -5033,7 +5033,7 @@
         <v>27</v>
       </c>
       <c r="E134" s="11">
-        <v>28</v>
+        <v>14</v>
       </c>
       <c r="F134" s="9" t="s">
         <v>28</v>
@@ -5079,7 +5079,7 @@
         <v>27</v>
       </c>
       <c r="E136" s="11">
-        <v>11</v>
+        <v>22</v>
       </c>
       <c r="F136" s="9" t="s">
         <v>28</v>
@@ -5102,7 +5102,7 @@
         <v>27</v>
       </c>
       <c r="E137" s="11">
-        <v>22</v>
+        <v>11</v>
       </c>
       <c r="F137" s="9" t="s">
         <v>28</v>
@@ -5125,7 +5125,7 @@
         <v>27</v>
       </c>
       <c r="E138" s="11">
-        <v>12</v>
+        <v>9</v>
       </c>
       <c r="F138" s="9" t="s">
         <v>28</v>
@@ -5148,7 +5148,7 @@
         <v>27</v>
       </c>
       <c r="E139" s="11">
-        <v>22</v>
+        <v>31</v>
       </c>
       <c r="F139" s="9" t="s">
         <v>28</v>
@@ -5171,7 +5171,7 @@
         <v>27</v>
       </c>
       <c r="E140" s="11">
-        <v>25</v>
+        <v>9</v>
       </c>
       <c r="F140" s="9" t="s">
         <v>28</v>
@@ -5194,7 +5194,7 @@
         <v>27</v>
       </c>
       <c r="E141" s="11">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="F141" s="9" t="s">
         <v>28</v>
@@ -5217,7 +5217,7 @@
         <v>27</v>
       </c>
       <c r="E142" s="11">
-        <v>17</v>
+        <v>29</v>
       </c>
       <c r="F142" s="9" t="s">
         <v>28</v>
@@ -5240,7 +5240,7 @@
         <v>27</v>
       </c>
       <c r="E143" s="11">
-        <v>24</v>
+        <v>15</v>
       </c>
       <c r="F143" s="9" t="s">
         <v>28</v>
@@ -5263,7 +5263,7 @@
         <v>27</v>
       </c>
       <c r="E144" s="11">
-        <v>11</v>
+        <v>21</v>
       </c>
       <c r="F144" s="9" t="s">
         <v>28</v>
@@ -5286,7 +5286,7 @@
         <v>27</v>
       </c>
       <c r="E145" s="11">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="F145" s="9" t="s">
         <v>28</v>
@@ -5309,7 +5309,7 @@
         <v>27</v>
       </c>
       <c r="E146" s="11">
-        <v>14</v>
+        <v>23</v>
       </c>
       <c r="F146" s="9" t="s">
         <v>28</v>
@@ -5332,7 +5332,7 @@
         <v>27</v>
       </c>
       <c r="E147" s="11">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="F147" s="9" t="s">
         <v>28</v>
@@ -5355,7 +5355,7 @@
         <v>27</v>
       </c>
       <c r="E148" s="11">
-        <v>20</v>
+        <v>17</v>
       </c>
       <c r="F148" s="9" t="s">
         <v>28</v>
@@ -5378,7 +5378,7 @@
         <v>27</v>
       </c>
       <c r="E149" s="11">
-        <v>30</v>
+        <v>25</v>
       </c>
       <c r="F149" s="9" t="s">
         <v>28</v>
@@ -5401,7 +5401,7 @@
         <v>27</v>
       </c>
       <c r="E150" s="11">
-        <v>25</v>
+        <v>31</v>
       </c>
       <c r="F150" s="9" t="s">
         <v>28</v>
@@ -5424,7 +5424,7 @@
         <v>27</v>
       </c>
       <c r="E151" s="11">
-        <v>27</v>
+        <v>14</v>
       </c>
       <c r="F151" s="9" t="s">
         <v>28</v>
@@ -5447,7 +5447,7 @@
         <v>27</v>
       </c>
       <c r="E152" s="11">
-        <v>9</v>
+        <v>31</v>
       </c>
       <c r="F152" s="9" t="s">
         <v>28</v>
@@ -5470,7 +5470,7 @@
         <v>27</v>
       </c>
       <c r="E153" s="11">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="F153" s="9" t="s">
         <v>28</v>
@@ -5493,7 +5493,7 @@
         <v>27</v>
       </c>
       <c r="E154" s="11">
-        <v>21</v>
+        <v>25</v>
       </c>
       <c r="F154" s="9" t="s">
         <v>28</v>
@@ -5516,7 +5516,7 @@
         <v>27</v>
       </c>
       <c r="E155" s="11">
-        <v>17</v>
+        <v>27</v>
       </c>
       <c r="F155" s="9" t="s">
         <v>28</v>
@@ -5539,7 +5539,7 @@
         <v>27</v>
       </c>
       <c r="E156" s="11">
-        <v>10</v>
+        <v>18</v>
       </c>
       <c r="F156" s="9" t="s">
         <v>28</v>
@@ -5562,7 +5562,7 @@
         <v>27</v>
       </c>
       <c r="E157" s="11">
-        <v>25</v>
+        <v>12</v>
       </c>
       <c r="F157" s="9" t="s">
         <v>28</v>
@@ -5585,7 +5585,7 @@
         <v>27</v>
       </c>
       <c r="E158" s="11">
-        <v>26</v>
+        <v>30</v>
       </c>
       <c r="F158" s="9" t="s">
         <v>28</v>
@@ -5608,7 +5608,7 @@
         <v>27</v>
       </c>
       <c r="E159" s="11">
-        <v>25</v>
+        <v>22</v>
       </c>
       <c r="F159" s="9" t="s">
         <v>28</v>
@@ -5631,7 +5631,7 @@
         <v>27</v>
       </c>
       <c r="E160" s="11">
-        <v>9</v>
+        <v>30</v>
       </c>
       <c r="F160" s="9" t="s">
         <v>28</v>
@@ -5654,7 +5654,7 @@
         <v>27</v>
       </c>
       <c r="E161" s="11">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="F161" s="9" t="s">
         <v>28</v>
@@ -5677,7 +5677,7 @@
         <v>27</v>
       </c>
       <c r="E162" s="11">
-        <v>14</v>
+        <v>22</v>
       </c>
       <c r="F162" s="9" t="s">
         <v>28</v>
@@ -5700,7 +5700,7 @@
         <v>27</v>
       </c>
       <c r="E163" s="11">
-        <v>10</v>
+        <v>19</v>
       </c>
       <c r="F163" s="9" t="s">
         <v>28</v>
@@ -5723,7 +5723,7 @@
         <v>27</v>
       </c>
       <c r="E164" s="11">
-        <v>24</v>
+        <v>13</v>
       </c>
       <c r="F164" s="9" t="s">
         <v>28</v>
@@ -5746,7 +5746,7 @@
         <v>27</v>
       </c>
       <c r="E165" s="11">
-        <v>29</v>
+        <v>9</v>
       </c>
       <c r="F165" s="9" t="s">
         <v>28</v>
@@ -5769,7 +5769,7 @@
         <v>27</v>
       </c>
       <c r="E166" s="11">
-        <v>17</v>
+        <v>31</v>
       </c>
       <c r="F166" s="9" t="s">
         <v>28</v>
@@ -5792,7 +5792,7 @@
         <v>27</v>
       </c>
       <c r="E167" s="11">
-        <v>16</v>
+        <v>26</v>
       </c>
       <c r="F167" s="9" t="s">
         <v>28</v>
@@ -5815,7 +5815,7 @@
         <v>27</v>
       </c>
       <c r="E168" s="11">
-        <v>17</v>
+        <v>27</v>
       </c>
       <c r="F168" s="9" t="s">
         <v>28</v>
@@ -5838,7 +5838,7 @@
         <v>27</v>
       </c>
       <c r="E169" s="11">
-        <v>18</v>
+        <v>20</v>
       </c>
       <c r="F169" s="9" t="s">
         <v>28</v>
@@ -5861,7 +5861,7 @@
         <v>27</v>
       </c>
       <c r="E170" s="11">
-        <v>14</v>
+        <v>18</v>
       </c>
       <c r="F170" s="9" t="s">
         <v>28</v>
@@ -5884,7 +5884,7 @@
         <v>27</v>
       </c>
       <c r="E171" s="11">
-        <v>25</v>
+        <v>23</v>
       </c>
       <c r="F171" s="9" t="s">
         <v>28</v>
@@ -5907,7 +5907,7 @@
         <v>27</v>
       </c>
       <c r="E172" s="11">
-        <v>15</v>
+        <v>13</v>
       </c>
       <c r="F172" s="9" t="s">
         <v>28</v>
@@ -5930,7 +5930,7 @@
         <v>27</v>
       </c>
       <c r="E173" s="11">
-        <v>13</v>
+        <v>20</v>
       </c>
       <c r="F173" s="9" t="s">
         <v>28</v>
@@ -5953,7 +5953,7 @@
         <v>27</v>
       </c>
       <c r="E174" s="11">
-        <v>29</v>
+        <v>20</v>
       </c>
       <c r="F174" s="9" t="s">
         <v>28</v>
@@ -5976,7 +5976,7 @@
         <v>27</v>
       </c>
       <c r="E175" s="11">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="F175" s="9" t="s">
         <v>28</v>
@@ -5999,7 +5999,7 @@
         <v>27</v>
       </c>
       <c r="E176" s="11">
-        <v>28</v>
+        <v>15</v>
       </c>
       <c r="F176" s="9" t="s">
         <v>28</v>
@@ -6022,7 +6022,7 @@
         <v>27</v>
       </c>
       <c r="E177" s="11">
-        <v>14</v>
+        <v>9</v>
       </c>
       <c r="F177" s="9" t="s">
         <v>28</v>
@@ -6045,7 +6045,7 @@
         <v>27</v>
       </c>
       <c r="E178" s="11">
-        <v>16</v>
+        <v>26</v>
       </c>
       <c r="F178" s="9" t="s">
         <v>28</v>
@@ -6068,7 +6068,7 @@
         <v>27</v>
       </c>
       <c r="E179" s="11">
-        <v>31</v>
+        <v>23</v>
       </c>
       <c r="F179" s="9" t="s">
         <v>28</v>
@@ -6091,7 +6091,7 @@
         <v>27</v>
       </c>
       <c r="E180" s="11">
-        <v>27</v>
+        <v>10</v>
       </c>
       <c r="F180" s="9" t="s">
         <v>28</v>
@@ -6114,7 +6114,7 @@
         <v>27</v>
       </c>
       <c r="E181" s="11">
-        <v>15</v>
+        <v>21</v>
       </c>
       <c r="F181" s="9" t="s">
         <v>28</v>
@@ -6137,7 +6137,7 @@
         <v>27</v>
       </c>
       <c r="E182" s="11">
-        <v>16</v>
+        <v>9</v>
       </c>
       <c r="F182" s="9" t="s">
         <v>28</v>
@@ -6160,7 +6160,7 @@
         <v>27</v>
       </c>
       <c r="E183" s="11">
-        <v>31</v>
+        <v>27</v>
       </c>
       <c r="F183" s="9" t="s">
         <v>28</v>
@@ -6183,7 +6183,7 @@
         <v>27</v>
       </c>
       <c r="E184" s="11">
-        <v>18</v>
+        <v>24</v>
       </c>
       <c r="F184" s="9" t="s">
         <v>28</v>
@@ -6206,7 +6206,7 @@
         <v>27</v>
       </c>
       <c r="E185" s="11">
-        <v>24</v>
+        <v>30</v>
       </c>
       <c r="F185" s="9" t="s">
         <v>28</v>
@@ -6229,7 +6229,7 @@
         <v>27</v>
       </c>
       <c r="E186" s="11">
-        <v>16</v>
+        <v>25</v>
       </c>
       <c r="F186" s="9" t="s">
         <v>28</v>
@@ -6252,7 +6252,7 @@
         <v>27</v>
       </c>
       <c r="E187" s="11">
-        <v>11</v>
+        <v>24</v>
       </c>
       <c r="F187" s="9" t="s">
         <v>28</v>
@@ -6275,7 +6275,7 @@
         <v>27</v>
       </c>
       <c r="E188" s="11">
-        <v>15</v>
+        <v>24</v>
       </c>
       <c r="F188" s="9" t="s">
         <v>28</v>
@@ -6298,7 +6298,7 @@
         <v>27</v>
       </c>
       <c r="E189" s="11">
-        <v>14</v>
+        <v>30</v>
       </c>
       <c r="F189" s="9" t="s">
         <v>28</v>
@@ -6321,7 +6321,7 @@
         <v>27</v>
       </c>
       <c r="E190" s="11">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="F190" s="9" t="s">
         <v>28</v>
@@ -6344,7 +6344,7 @@
         <v>27</v>
       </c>
       <c r="E191" s="11">
-        <v>27</v>
+        <v>21</v>
       </c>
       <c r="F191" s="9" t="s">
         <v>28</v>
@@ -6367,7 +6367,7 @@
         <v>27</v>
       </c>
       <c r="E192" s="11">
-        <v>25</v>
+        <v>17</v>
       </c>
       <c r="F192" s="9" t="s">
         <v>28</v>
@@ -6390,7 +6390,7 @@
         <v>27</v>
       </c>
       <c r="E193" s="11">
-        <v>30</v>
+        <v>11</v>
       </c>
       <c r="F193" s="9" t="s">
         <v>28</v>
@@ -6413,7 +6413,7 @@
         <v>27</v>
       </c>
       <c r="E194" s="11">
-        <v>13</v>
+        <v>25</v>
       </c>
       <c r="F194" s="9" t="s">
         <v>28</v>
@@ -6459,7 +6459,7 @@
         <v>27</v>
       </c>
       <c r="E196" s="11">
-        <v>23</v>
+        <v>21</v>
       </c>
       <c r="F196" s="9" t="s">
         <v>28</v>
@@ -6482,7 +6482,7 @@
         <v>27</v>
       </c>
       <c r="E197" s="11">
-        <v>31</v>
+        <v>10</v>
       </c>
       <c r="F197" s="9" t="s">
         <v>28</v>
@@ -6505,7 +6505,7 @@
         <v>27</v>
       </c>
       <c r="E198" s="11">
-        <v>21</v>
+        <v>28</v>
       </c>
       <c r="F198" s="9" t="s">
         <v>28</v>
@@ -6528,7 +6528,7 @@
         <v>27</v>
       </c>
       <c r="E199" s="11">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="F199" s="9" t="s">
         <v>28</v>
@@ -6574,7 +6574,7 @@
         <v>27</v>
       </c>
       <c r="E201" s="11">
-        <v>16</v>
+        <v>22</v>
       </c>
       <c r="F201" s="9" t="s">
         <v>28</v>
@@ -6597,7 +6597,7 @@
         <v>27</v>
       </c>
       <c r="E202" s="11">
-        <v>30</v>
+        <v>12</v>
       </c>
       <c r="F202" s="9" t="s">
         <v>28</v>
@@ -6620,7 +6620,7 @@
         <v>27</v>
       </c>
       <c r="E203" s="11">
-        <v>8</v>
+        <v>25</v>
       </c>
       <c r="F203" s="9" t="s">
         <v>28</v>
@@ -6643,7 +6643,7 @@
         <v>27</v>
       </c>
       <c r="E204" s="11">
-        <v>11</v>
+        <v>17</v>
       </c>
       <c r="F204" s="9" t="s">
         <v>28</v>
@@ -6666,7 +6666,7 @@
         <v>27</v>
       </c>
       <c r="E205" s="11">
-        <v>8</v>
+        <v>17</v>
       </c>
       <c r="F205" s="9" t="s">
         <v>28</v>
@@ -6689,7 +6689,7 @@
         <v>27</v>
       </c>
       <c r="E206" s="11">
-        <v>31</v>
+        <v>13</v>
       </c>
       <c r="F206" s="9" t="s">
         <v>28</v>
@@ -6712,7 +6712,7 @@
         <v>27</v>
       </c>
       <c r="E207" s="11">
-        <v>9</v>
+        <v>26</v>
       </c>
       <c r="F207" s="9" t="s">
         <v>28</v>
@@ -6735,7 +6735,7 @@
         <v>27</v>
       </c>
       <c r="E208" s="11">
-        <v>17</v>
+        <v>27</v>
       </c>
       <c r="F208" s="9" t="s">
         <v>28</v>
@@ -6758,7 +6758,7 @@
         <v>27</v>
       </c>
       <c r="E209" s="11">
-        <v>24</v>
+        <v>17</v>
       </c>
       <c r="F209" s="9" t="s">
         <v>28</v>
@@ -6781,7 +6781,7 @@
         <v>27</v>
       </c>
       <c r="E210" s="11">
-        <v>24</v>
+        <v>13</v>
       </c>
       <c r="F210" s="9" t="s">
         <v>28</v>
@@ -6804,7 +6804,7 @@
         <v>27</v>
       </c>
       <c r="E211" s="11">
-        <v>19</v>
+        <v>11</v>
       </c>
       <c r="F211" s="9" t="s">
         <v>28</v>
@@ -6827,7 +6827,7 @@
         <v>27</v>
       </c>
       <c r="E212" s="11">
-        <v>24</v>
+        <v>16</v>
       </c>
       <c r="F212" s="9" t="s">
         <v>28</v>
@@ -6873,7 +6873,7 @@
         <v>27</v>
       </c>
       <c r="E214" s="11">
-        <v>22</v>
+        <v>30</v>
       </c>
       <c r="F214" s="9" t="s">
         <v>28</v>
@@ -6896,7 +6896,7 @@
         <v>27</v>
       </c>
       <c r="E215" s="11">
-        <v>25</v>
+        <v>29</v>
       </c>
       <c r="F215" s="9" t="s">
         <v>28</v>
@@ -6919,7 +6919,7 @@
         <v>27</v>
       </c>
       <c r="E216" s="11">
-        <v>29</v>
+        <v>21</v>
       </c>
       <c r="F216" s="9" t="s">
         <v>28</v>
@@ -6942,7 +6942,7 @@
         <v>27</v>
       </c>
       <c r="E217" s="11">
-        <v>22</v>
+        <v>10</v>
       </c>
       <c r="F217" s="9" t="s">
         <v>28</v>
@@ -6965,7 +6965,7 @@
         <v>27</v>
       </c>
       <c r="E218" s="11">
-        <v>14</v>
+        <v>8</v>
       </c>
       <c r="F218" s="9" t="s">
         <v>28</v>
@@ -6988,7 +6988,7 @@
         <v>27</v>
       </c>
       <c r="E219" s="11">
-        <v>29</v>
+        <v>11</v>
       </c>
       <c r="F219" s="9" t="s">
         <v>28</v>
@@ -7011,7 +7011,7 @@
         <v>27</v>
       </c>
       <c r="E220" s="11">
-        <v>30</v>
+        <v>25</v>
       </c>
       <c r="F220" s="9" t="s">
         <v>28</v>
@@ -7034,7 +7034,7 @@
         <v>27</v>
       </c>
       <c r="E221" s="11">
-        <v>27</v>
+        <v>30</v>
       </c>
       <c r="F221" s="9" t="s">
         <v>28</v>
@@ -7057,7 +7057,7 @@
         <v>27</v>
       </c>
       <c r="E222" s="11">
-        <v>12</v>
+        <v>18</v>
       </c>
       <c r="F222" s="9" t="s">
         <v>28</v>
@@ -7080,7 +7080,7 @@
         <v>27</v>
       </c>
       <c r="E223" s="11">
-        <v>13</v>
+        <v>30</v>
       </c>
       <c r="F223" s="9" t="s">
         <v>28</v>
@@ -7103,7 +7103,7 @@
         <v>27</v>
       </c>
       <c r="E224" s="11">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="F224" s="9" t="s">
         <v>28</v>
@@ -7126,7 +7126,7 @@
         <v>27</v>
       </c>
       <c r="E225" s="11">
-        <v>10</v>
+        <v>23</v>
       </c>
       <c r="F225" s="9" t="s">
         <v>28</v>
@@ -7149,7 +7149,7 @@
         <v>27</v>
       </c>
       <c r="E226" s="11">
-        <v>31</v>
+        <v>10</v>
       </c>
       <c r="F226" s="9" t="s">
         <v>28</v>
@@ -7172,7 +7172,7 @@
         <v>27</v>
       </c>
       <c r="E227" s="11">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="F227" s="9" t="s">
         <v>28</v>
@@ -7195,7 +7195,7 @@
         <v>27</v>
       </c>
       <c r="E228" s="11">
-        <v>13</v>
+        <v>28</v>
       </c>
       <c r="F228" s="9" t="s">
         <v>28</v>
@@ -7218,7 +7218,7 @@
         <v>27</v>
       </c>
       <c r="E229" s="11">
-        <v>31</v>
+        <v>9</v>
       </c>
       <c r="F229" s="9" t="s">
         <v>28</v>
@@ -7241,7 +7241,7 @@
         <v>27</v>
       </c>
       <c r="E230" s="11">
-        <v>13</v>
+        <v>16</v>
       </c>
       <c r="F230" s="9" t="s">
         <v>28</v>
@@ -7264,7 +7264,7 @@
         <v>27</v>
       </c>
       <c r="E231" s="11">
-        <v>25</v>
+        <v>11</v>
       </c>
       <c r="F231" s="9" t="s">
         <v>28</v>
@@ -7287,7 +7287,7 @@
         <v>27</v>
       </c>
       <c r="E232" s="11">
-        <v>29</v>
+        <v>22</v>
       </c>
       <c r="F232" s="9" t="s">
         <v>28</v>
@@ -7310,7 +7310,7 @@
         <v>27</v>
       </c>
       <c r="E233" s="11">
-        <v>22</v>
+        <v>9</v>
       </c>
       <c r="F233" s="9" t="s">
         <v>28</v>
@@ -7333,7 +7333,7 @@
         <v>27</v>
       </c>
       <c r="E234" s="11">
-        <v>8</v>
+        <v>24</v>
       </c>
       <c r="F234" s="9" t="s">
         <v>28</v>
@@ -7356,7 +7356,7 @@
         <v>27</v>
       </c>
       <c r="E235" s="11">
-        <v>19</v>
+        <v>26</v>
       </c>
       <c r="F235" s="9" t="s">
         <v>28</v>
@@ -7379,7 +7379,7 @@
         <v>27</v>
       </c>
       <c r="E236" s="11">
-        <v>8</v>
+        <v>29</v>
       </c>
       <c r="F236" s="9" t="s">
         <v>28</v>
@@ -7402,7 +7402,7 @@
         <v>27</v>
       </c>
       <c r="E237" s="11">
-        <v>23</v>
+        <v>17</v>
       </c>
       <c r="F237" s="9" t="s">
         <v>28</v>
@@ -7425,7 +7425,7 @@
         <v>27</v>
       </c>
       <c r="E238" s="11">
-        <v>28</v>
+        <v>26</v>
       </c>
       <c r="F238" s="9" t="s">
         <v>28</v>
@@ -7448,7 +7448,7 @@
         <v>27</v>
       </c>
       <c r="E239" s="11">
-        <v>21</v>
+        <v>31</v>
       </c>
       <c r="F239" s="9" t="s">
         <v>28</v>
@@ -7471,7 +7471,7 @@
         <v>27</v>
       </c>
       <c r="E240" s="11">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="F240" s="9" t="s">
         <v>28</v>
@@ -7494,7 +7494,7 @@
         <v>27</v>
       </c>
       <c r="E241" s="11">
-        <v>18</v>
+        <v>31</v>
       </c>
       <c r="F241" s="9" t="s">
         <v>28</v>
@@ -7517,7 +7517,7 @@
         <v>27</v>
       </c>
       <c r="E242" s="11">
-        <v>15</v>
+        <v>20</v>
       </c>
       <c r="F242" s="9" t="s">
         <v>28</v>
@@ -7540,7 +7540,7 @@
         <v>27</v>
       </c>
       <c r="E243" s="11">
-        <v>17</v>
+        <v>20</v>
       </c>
       <c r="F243" s="9" t="s">
         <v>28</v>
@@ -7563,7 +7563,7 @@
         <v>27</v>
       </c>
       <c r="E244" s="11">
-        <v>25</v>
+        <v>8</v>
       </c>
       <c r="F244" s="9" t="s">
         <v>28</v>
@@ -7586,7 +7586,7 @@
         <v>27</v>
       </c>
       <c r="E245" s="11">
-        <v>31</v>
+        <v>12</v>
       </c>
       <c r="F245" s="9" t="s">
         <v>28</v>
@@ -7609,7 +7609,7 @@
         <v>27</v>
       </c>
       <c r="E246" s="11">
-        <v>31</v>
+        <v>14</v>
       </c>
       <c r="F246" s="9" t="s">
         <v>28</v>
@@ -7632,7 +7632,7 @@
         <v>27</v>
       </c>
       <c r="E247" s="11">
-        <v>8</v>
+        <v>29</v>
       </c>
       <c r="F247" s="9" t="s">
         <v>28</v>
@@ -7655,7 +7655,7 @@
         <v>27</v>
       </c>
       <c r="E248" s="11">
-        <v>13</v>
+        <v>21</v>
       </c>
       <c r="F248" s="9" t="s">
         <v>28</v>
@@ -7678,7 +7678,7 @@
         <v>27</v>
       </c>
       <c r="E249" s="11">
-        <v>15</v>
+        <v>24</v>
       </c>
       <c r="F249" s="9" t="s">
         <v>28</v>
@@ -7701,7 +7701,7 @@
         <v>27</v>
       </c>
       <c r="E250" s="11">
-        <v>30</v>
+        <v>13</v>
       </c>
       <c r="F250" s="9" t="s">
         <v>28</v>
@@ -7724,7 +7724,7 @@
         <v>27</v>
       </c>
       <c r="E251" s="11">
-        <v>28</v>
+        <v>12</v>
       </c>
       <c r="F251" s="9" t="s">
         <v>28</v>
@@ -7747,7 +7747,7 @@
         <v>27</v>
       </c>
       <c r="E252" s="11">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="F252" s="9" t="s">
         <v>28</v>
@@ -7770,7 +7770,7 @@
         <v>27</v>
       </c>
       <c r="E253" s="11">
-        <v>29</v>
+        <v>27</v>
       </c>
       <c r="F253" s="9" t="s">
         <v>28</v>
@@ -7793,7 +7793,7 @@
         <v>27</v>
       </c>
       <c r="E254" s="11">
-        <v>15</v>
+        <v>24</v>
       </c>
       <c r="F254" s="9" t="s">
         <v>28</v>
@@ -7816,7 +7816,7 @@
         <v>27</v>
       </c>
       <c r="E255" s="11">
-        <v>20</v>
+        <v>22</v>
       </c>
       <c r="F255" s="9" t="s">
         <v>28</v>
@@ -7839,7 +7839,7 @@
         <v>27</v>
       </c>
       <c r="E256" s="11">
-        <v>16</v>
+        <v>31</v>
       </c>
       <c r="F256" s="9" t="s">
         <v>28</v>
@@ -7862,7 +7862,7 @@
         <v>27</v>
       </c>
       <c r="E257" s="11">
-        <v>28</v>
+        <v>30</v>
       </c>
       <c r="F257" s="9" t="s">
         <v>28</v>
@@ -7885,7 +7885,7 @@
         <v>27</v>
       </c>
       <c r="E258" s="11">
-        <v>21</v>
+        <v>16</v>
       </c>
       <c r="F258" s="9" t="s">
         <v>28</v>
@@ -7908,7 +7908,7 @@
         <v>27</v>
       </c>
       <c r="E259" s="11">
-        <v>10</v>
+        <v>18</v>
       </c>
       <c r="F259" s="9" t="s">
         <v>28</v>
@@ -7931,7 +7931,7 @@
         <v>27</v>
       </c>
       <c r="E260" s="11">
-        <v>8</v>
+        <v>24</v>
       </c>
       <c r="F260" s="9" t="s">
         <v>28</v>
@@ -7954,7 +7954,7 @@
         <v>27</v>
       </c>
       <c r="E261" s="11">
-        <v>18</v>
+        <v>10</v>
       </c>
       <c r="F261" s="9" t="s">
         <v>28</v>
@@ -7977,7 +7977,7 @@
         <v>27</v>
       </c>
       <c r="E262" s="11">
-        <v>9</v>
+        <v>24</v>
       </c>
       <c r="F262" s="9" t="s">
         <v>28</v>
@@ -8000,7 +8000,7 @@
         <v>27</v>
       </c>
       <c r="E263" s="11">
-        <v>26</v>
+        <v>28</v>
       </c>
       <c r="F263" s="9" t="s">
         <v>28</v>
@@ -8023,7 +8023,7 @@
         <v>27</v>
       </c>
       <c r="E264" s="11">
-        <v>27</v>
+        <v>23</v>
       </c>
       <c r="F264" s="9" t="s">
         <v>28</v>
@@ -8046,7 +8046,7 @@
         <v>27</v>
       </c>
       <c r="E265" s="11">
-        <v>26</v>
+        <v>29</v>
       </c>
       <c r="F265" s="9" t="s">
         <v>28</v>
@@ -8069,7 +8069,7 @@
         <v>27</v>
       </c>
       <c r="E266" s="11">
-        <v>11</v>
+        <v>13</v>
       </c>
       <c r="F266" s="9" t="s">
         <v>28</v>
@@ -8092,7 +8092,7 @@
         <v>27</v>
       </c>
       <c r="E267" s="11">
-        <v>24</v>
+        <v>14</v>
       </c>
       <c r="F267" s="9" t="s">
         <v>28</v>
@@ -8115,7 +8115,7 @@
         <v>27</v>
       </c>
       <c r="E268" s="11">
-        <v>9</v>
+        <v>13</v>
       </c>
       <c r="F268" s="9" t="s">
         <v>28</v>
@@ -8138,7 +8138,7 @@
         <v>27</v>
       </c>
       <c r="E269" s="11">
-        <v>31</v>
+        <v>16</v>
       </c>
       <c r="F269" s="9" t="s">
         <v>28</v>
@@ -8161,7 +8161,7 @@
         <v>27</v>
       </c>
       <c r="E270" s="11">
-        <v>27</v>
+        <v>20</v>
       </c>
       <c r="F270" s="9" t="s">
         <v>28</v>
@@ -8184,7 +8184,7 @@
         <v>27</v>
       </c>
       <c r="E271" s="11">
-        <v>21</v>
+        <v>23</v>
       </c>
       <c r="F271" s="9" t="s">
         <v>28</v>
@@ -8207,7 +8207,7 @@
         <v>27</v>
       </c>
       <c r="E272" s="11">
-        <v>12</v>
+        <v>22</v>
       </c>
       <c r="F272" s="9" t="s">
         <v>28</v>
@@ -8230,7 +8230,7 @@
         <v>27</v>
       </c>
       <c r="E273" s="11">
-        <v>20</v>
+        <v>27</v>
       </c>
       <c r="F273" s="9" t="s">
         <v>28</v>
@@ -8253,7 +8253,7 @@
         <v>27</v>
       </c>
       <c r="E274" s="11">
-        <v>30</v>
+        <v>28</v>
       </c>
       <c r="F274" s="9" t="s">
         <v>28</v>
@@ -8276,7 +8276,7 @@
         <v>27</v>
       </c>
       <c r="E275" s="11">
-        <v>16</v>
+        <v>22</v>
       </c>
       <c r="F275" s="9" t="s">
         <v>28</v>
@@ -8299,7 +8299,7 @@
         <v>27</v>
       </c>
       <c r="E276" s="11">
-        <v>8</v>
+        <v>12</v>
       </c>
       <c r="F276" s="9" t="s">
         <v>28</v>
@@ -8322,7 +8322,7 @@
         <v>27</v>
       </c>
       <c r="E277" s="11">
-        <v>28</v>
+        <v>17</v>
       </c>
       <c r="F277" s="9" t="s">
         <v>28</v>
@@ -8345,7 +8345,7 @@
         <v>27</v>
       </c>
       <c r="E278" s="11">
-        <v>17</v>
+        <v>22</v>
       </c>
       <c r="F278" s="9" t="s">
         <v>28</v>
@@ -8368,7 +8368,7 @@
         <v>27</v>
       </c>
       <c r="E279" s="11">
-        <v>12</v>
+        <v>15</v>
       </c>
       <c r="F279" s="9" t="s">
         <v>28</v>
@@ -8391,7 +8391,7 @@
         <v>27</v>
       </c>
       <c r="E280" s="11">
-        <v>22</v>
+        <v>18</v>
       </c>
       <c r="F280" s="9" t="s">
         <v>28</v>
@@ -8414,7 +8414,7 @@
         <v>27</v>
       </c>
       <c r="E281" s="11">
-        <v>12</v>
+        <v>20</v>
       </c>
       <c r="F281" s="9" t="s">
         <v>28</v>
@@ -8437,7 +8437,7 @@
         <v>27</v>
       </c>
       <c r="E282" s="11">
-        <v>21</v>
+        <v>24</v>
       </c>
       <c r="F282" s="9" t="s">
         <v>28</v>
@@ -8460,7 +8460,7 @@
         <v>27</v>
       </c>
       <c r="E283" s="11">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="F283" s="9" t="s">
         <v>28</v>
@@ -8483,7 +8483,7 @@
         <v>27</v>
       </c>
       <c r="E284" s="11">
-        <v>25</v>
+        <v>27</v>
       </c>
       <c r="F284" s="9" t="s">
         <v>28</v>
@@ -8506,7 +8506,7 @@
         <v>27</v>
       </c>
       <c r="E285" s="11">
-        <v>28</v>
+        <v>13</v>
       </c>
       <c r="F285" s="9" t="s">
         <v>28</v>
@@ -8529,7 +8529,7 @@
         <v>27</v>
       </c>
       <c r="E286" s="11">
-        <v>26</v>
+        <v>24</v>
       </c>
       <c r="F286" s="9" t="s">
         <v>28</v>
@@ -8552,7 +8552,7 @@
         <v>27</v>
       </c>
       <c r="E287" s="11">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="F287" s="9" t="s">
         <v>28</v>
@@ -8575,7 +8575,7 @@
         <v>27</v>
       </c>
       <c r="E288" s="11">
-        <v>10</v>
+        <v>13</v>
       </c>
       <c r="F288" s="9" t="s">
         <v>28</v>
@@ -8598,7 +8598,7 @@
         <v>27</v>
       </c>
       <c r="E289" s="11">
-        <v>26</v>
+        <v>24</v>
       </c>
       <c r="F289" s="9" t="s">
         <v>28</v>
@@ -8621,7 +8621,7 @@
         <v>27</v>
       </c>
       <c r="E290" s="11">
-        <v>16</v>
+        <v>28</v>
       </c>
       <c r="F290" s="9" t="s">
         <v>28</v>
@@ -8644,7 +8644,7 @@
         <v>27</v>
       </c>
       <c r="E291" s="11">
-        <v>8</v>
+        <v>15</v>
       </c>
       <c r="F291" s="9" t="s">
         <v>28</v>
@@ -8667,7 +8667,7 @@
         <v>27</v>
       </c>
       <c r="E292" s="11">
-        <v>10</v>
+        <v>13</v>
       </c>
       <c r="F292" s="9" t="s">
         <v>28</v>
@@ -8690,7 +8690,7 @@
         <v>27</v>
       </c>
       <c r="E293" s="11">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="F293" s="9" t="s">
         <v>28</v>
@@ -8713,7 +8713,7 @@
         <v>27</v>
       </c>
       <c r="E294" s="11">
-        <v>10</v>
+        <v>31</v>
       </c>
       <c r="F294" s="9" t="s">
         <v>28</v>
@@ -8736,7 +8736,7 @@
         <v>27</v>
       </c>
       <c r="E295" s="11">
-        <v>13</v>
+        <v>18</v>
       </c>
       <c r="F295" s="9" t="s">
         <v>28</v>
@@ -8759,7 +8759,7 @@
         <v>27</v>
       </c>
       <c r="E296" s="11">
-        <v>30</v>
+        <v>9</v>
       </c>
       <c r="F296" s="9" t="s">
         <v>28</v>
@@ -8782,7 +8782,7 @@
         <v>27</v>
       </c>
       <c r="E297" s="11">
-        <v>11</v>
+        <v>15</v>
       </c>
       <c r="F297" s="9" t="s">
         <v>28</v>
@@ -8805,7 +8805,7 @@
         <v>27</v>
       </c>
       <c r="E298" s="11">
-        <v>27</v>
+        <v>10</v>
       </c>
       <c r="F298" s="9" t="s">
         <v>28</v>
@@ -8828,7 +8828,7 @@
         <v>27</v>
       </c>
       <c r="E299" s="11">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="F299" s="9" t="s">
         <v>28</v>
@@ -8851,7 +8851,7 @@
         <v>27</v>
       </c>
       <c r="E300" s="11">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="F300" s="9" t="s">
         <v>28</v>
@@ -8874,7 +8874,7 @@
         <v>27</v>
       </c>
       <c r="E301" s="11">
-        <v>11</v>
+        <v>26</v>
       </c>
       <c r="F301" s="9" t="s">
         <v>28</v>
@@ -8897,7 +8897,7 @@
         <v>27</v>
       </c>
       <c r="E302" s="11">
-        <v>9</v>
+        <v>22</v>
       </c>
       <c r="F302" s="9" t="s">
         <v>28</v>
@@ -8920,7 +8920,7 @@
         <v>27</v>
       </c>
       <c r="E303" s="11">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="F303" s="9" t="s">
         <v>28</v>
@@ -8943,7 +8943,7 @@
         <v>27</v>
       </c>
       <c r="E304" s="11">
-        <v>28</v>
+        <v>21</v>
       </c>
       <c r="F304" s="9" t="s">
         <v>28</v>
@@ -8966,7 +8966,7 @@
         <v>27</v>
       </c>
       <c r="E305" s="11">
-        <v>20</v>
+        <v>31</v>
       </c>
       <c r="F305" s="9" t="s">
         <v>28</v>
@@ -8989,7 +8989,7 @@
         <v>27</v>
       </c>
       <c r="E306" s="11">
-        <v>29</v>
+        <v>17</v>
       </c>
       <c r="F306" s="9" t="s">
         <v>28</v>
@@ -9012,7 +9012,7 @@
         <v>27</v>
       </c>
       <c r="E307" s="11">
-        <v>12</v>
+        <v>15</v>
       </c>
       <c r="F307" s="9" t="s">
         <v>28</v>
@@ -9035,7 +9035,7 @@
         <v>27</v>
       </c>
       <c r="E308" s="11">
-        <v>21</v>
+        <v>29</v>
       </c>
       <c r="F308" s="9" t="s">
         <v>28</v>
@@ -9058,7 +9058,7 @@
         <v>27</v>
       </c>
       <c r="E309" s="11">
-        <v>29</v>
+        <v>23</v>
       </c>
       <c r="F309" s="9" t="s">
         <v>28</v>
@@ -9081,7 +9081,7 @@
         <v>27</v>
       </c>
       <c r="E310" s="11">
-        <v>30</v>
+        <v>27</v>
       </c>
       <c r="F310" s="9" t="s">
         <v>28</v>
@@ -9104,7 +9104,7 @@
         <v>27</v>
       </c>
       <c r="E311" s="11">
-        <v>22</v>
+        <v>26</v>
       </c>
       <c r="F311" s="9" t="s">
         <v>28</v>
@@ -9127,7 +9127,7 @@
         <v>27</v>
       </c>
       <c r="E312" s="11">
-        <v>23</v>
+        <v>26</v>
       </c>
       <c r="F312" s="9" t="s">
         <v>28</v>
@@ -9150,7 +9150,7 @@
         <v>27</v>
       </c>
       <c r="E313" s="11">
-        <v>21</v>
+        <v>26</v>
       </c>
       <c r="F313" s="9" t="s">
         <v>28</v>
@@ -9173,7 +9173,7 @@
         <v>27</v>
       </c>
       <c r="E314" s="11">
-        <v>24</v>
+        <v>14</v>
       </c>
       <c r="F314" s="9" t="s">
         <v>28</v>
@@ -9196,7 +9196,7 @@
         <v>27</v>
       </c>
       <c r="E315" s="11">
-        <v>31</v>
+        <v>18</v>
       </c>
       <c r="F315" s="9" t="s">
         <v>28</v>
@@ -9219,7 +9219,7 @@
         <v>27</v>
       </c>
       <c r="E316" s="11">
-        <v>28</v>
+        <v>16</v>
       </c>
       <c r="F316" s="9" t="s">
         <v>28</v>
@@ -9242,7 +9242,7 @@
         <v>27</v>
       </c>
       <c r="E317" s="11">
-        <v>15</v>
+        <v>18</v>
       </c>
       <c r="F317" s="9" t="s">
         <v>28</v>
@@ -9265,7 +9265,7 @@
         <v>27</v>
       </c>
       <c r="E318" s="11">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="F318" s="9" t="s">
         <v>28</v>
@@ -9288,7 +9288,7 @@
         <v>27</v>
       </c>
       <c r="E319" s="11">
-        <v>10</v>
+        <v>21</v>
       </c>
       <c r="F319" s="9" t="s">
         <v>28</v>
@@ -9311,7 +9311,7 @@
         <v>27</v>
       </c>
       <c r="E320" s="11">
-        <v>14</v>
+        <v>11</v>
       </c>
       <c r="F320" s="9" t="s">
         <v>28</v>
@@ -9334,7 +9334,7 @@
         <v>27</v>
       </c>
       <c r="E321" s="11">
-        <v>8</v>
+        <v>15</v>
       </c>
       <c r="F321" s="9" t="s">
         <v>28</v>
@@ -9357,7 +9357,7 @@
         <v>27</v>
       </c>
       <c r="E322" s="11">
-        <v>15</v>
+        <v>26</v>
       </c>
       <c r="F322" s="9" t="s">
         <v>28</v>
@@ -9380,7 +9380,7 @@
         <v>27</v>
       </c>
       <c r="E323" s="11">
-        <v>24</v>
+        <v>28</v>
       </c>
       <c r="F323" s="9" t="s">
         <v>28</v>
@@ -9403,7 +9403,7 @@
         <v>27</v>
       </c>
       <c r="E324" s="11">
-        <v>16</v>
+        <v>28</v>
       </c>
       <c r="F324" s="9" t="s">
         <v>28</v>
@@ -9426,7 +9426,7 @@
         <v>27</v>
       </c>
       <c r="E325" s="11">
-        <v>14</v>
+        <v>10</v>
       </c>
       <c r="F325" s="9" t="s">
         <v>28</v>
@@ -9449,7 +9449,7 @@
         <v>27</v>
       </c>
       <c r="E326" s="11">
-        <v>9</v>
+        <v>14</v>
       </c>
       <c r="F326" s="9" t="s">
         <v>28</v>
@@ -9472,7 +9472,7 @@
         <v>27</v>
       </c>
       <c r="E327" s="11">
-        <v>30</v>
+        <v>18</v>
       </c>
       <c r="F327" s="9" t="s">
         <v>28</v>
@@ -9495,7 +9495,7 @@
         <v>27</v>
       </c>
       <c r="E328" s="11">
-        <v>9</v>
+        <v>27</v>
       </c>
       <c r="F328" s="9" t="s">
         <v>28</v>
@@ -9518,7 +9518,7 @@
         <v>27</v>
       </c>
       <c r="E329" s="11">
-        <v>22</v>
+        <v>11</v>
       </c>
       <c r="F329" s="9" t="s">
         <v>28</v>
@@ -9541,7 +9541,7 @@
         <v>27</v>
       </c>
       <c r="E330" s="11">
-        <v>23</v>
+        <v>8</v>
       </c>
       <c r="F330" s="9" t="s">
         <v>28</v>
@@ -9564,7 +9564,7 @@
         <v>27</v>
       </c>
       <c r="E331" s="11">
-        <v>10</v>
+        <v>15</v>
       </c>
       <c r="F331" s="9" t="s">
         <v>28</v>
@@ -9587,7 +9587,7 @@
         <v>27</v>
       </c>
       <c r="E332" s="11">
-        <v>29</v>
+        <v>21</v>
       </c>
       <c r="F332" s="9" t="s">
         <v>28</v>
@@ -9610,7 +9610,7 @@
         <v>27</v>
       </c>
       <c r="E333" s="11">
-        <v>27</v>
+        <v>29</v>
       </c>
       <c r="F333" s="9" t="s">
         <v>28</v>
@@ -9633,7 +9633,7 @@
         <v>27</v>
       </c>
       <c r="E334" s="11">
-        <v>21</v>
+        <v>18</v>
       </c>
       <c r="F334" s="9" t="s">
         <v>28</v>
@@ -9656,7 +9656,7 @@
         <v>27</v>
       </c>
       <c r="E335" s="11">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="F335" s="9" t="s">
         <v>28</v>
@@ -9679,7 +9679,7 @@
         <v>27</v>
       </c>
       <c r="E336" s="11">
-        <v>31</v>
+        <v>10</v>
       </c>
       <c r="F336" s="9" t="s">
         <v>28</v>
@@ -9702,7 +9702,7 @@
         <v>27</v>
       </c>
       <c r="E337" s="11">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="F337" s="9" t="s">
         <v>28</v>
@@ -9725,7 +9725,7 @@
         <v>27</v>
       </c>
       <c r="E338" s="11">
-        <v>13</v>
+        <v>19</v>
       </c>
       <c r="F338" s="9" t="s">
         <v>28</v>
@@ -9748,7 +9748,7 @@
         <v>27</v>
       </c>
       <c r="E339" s="11">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="F339" s="9" t="s">
         <v>28</v>
@@ -9771,7 +9771,7 @@
         <v>27</v>
       </c>
       <c r="E340" s="11">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="F340" s="9" t="s">
         <v>28</v>
@@ -9794,7 +9794,7 @@
         <v>27</v>
       </c>
       <c r="E341" s="11">
-        <v>17</v>
+        <v>25</v>
       </c>
       <c r="F341" s="9" t="s">
         <v>28</v>
@@ -9817,7 +9817,7 @@
         <v>27</v>
       </c>
       <c r="E342" s="11">
-        <v>24</v>
+        <v>11</v>
       </c>
       <c r="F342" s="9" t="s">
         <v>28</v>
@@ -9840,7 +9840,7 @@
         <v>27</v>
       </c>
       <c r="E343" s="11">
-        <v>14</v>
+        <v>28</v>
       </c>
       <c r="F343" s="9" t="s">
         <v>28</v>
@@ -9863,7 +9863,7 @@
         <v>27</v>
       </c>
       <c r="E344" s="11">
-        <v>23</v>
+        <v>17</v>
       </c>
       <c r="F344" s="9" t="s">
         <v>28</v>
@@ -9886,7 +9886,7 @@
         <v>27</v>
       </c>
       <c r="E345" s="11">
-        <v>15</v>
+        <v>19</v>
       </c>
       <c r="F345" s="9" t="s">
         <v>28</v>
@@ -9909,7 +9909,7 @@
         <v>27</v>
       </c>
       <c r="E346" s="11">
-        <v>17</v>
+        <v>31</v>
       </c>
       <c r="F346" s="9" t="s">
         <v>28</v>
@@ -9932,7 +9932,7 @@
         <v>27</v>
       </c>
       <c r="E347" s="11">
-        <v>31</v>
+        <v>12</v>
       </c>
       <c r="F347" s="9" t="s">
         <v>28</v>
@@ -9955,7 +9955,7 @@
         <v>27</v>
       </c>
       <c r="E348" s="11">
-        <v>14</v>
+        <v>30</v>
       </c>
       <c r="F348" s="9" t="s">
         <v>28</v>
@@ -9978,7 +9978,7 @@
         <v>27</v>
       </c>
       <c r="E349" s="11">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="F349" s="9" t="s">
         <v>28</v>
@@ -10001,7 +10001,7 @@
         <v>27</v>
       </c>
       <c r="E350" s="11">
-        <v>18</v>
+        <v>26</v>
       </c>
       <c r="F350" s="9" t="s">
         <v>28</v>
@@ -10024,7 +10024,7 @@
         <v>27</v>
       </c>
       <c r="E351" s="11">
-        <v>13</v>
+        <v>28</v>
       </c>
       <c r="F351" s="9" t="s">
         <v>28</v>
@@ -10047,7 +10047,7 @@
         <v>27</v>
       </c>
       <c r="E352" s="11">
-        <v>19</v>
+        <v>25</v>
       </c>
       <c r="F352" s="9" t="s">
         <v>28</v>
@@ -10070,7 +10070,7 @@
         <v>27</v>
       </c>
       <c r="E353" s="11">
-        <v>11</v>
+        <v>27</v>
       </c>
       <c r="F353" s="9" t="s">
         <v>28</v>
@@ -10093,7 +10093,7 @@
         <v>27</v>
       </c>
       <c r="E354" s="11">
-        <v>17</v>
+        <v>30</v>
       </c>
       <c r="F354" s="9" t="s">
         <v>28</v>
@@ -10116,7 +10116,7 @@
         <v>27</v>
       </c>
       <c r="E355" s="11">
-        <v>19</v>
+        <v>25</v>
       </c>
       <c r="F355" s="9" t="s">
         <v>28</v>
@@ -10139,7 +10139,7 @@
         <v>27</v>
       </c>
       <c r="E356" s="11">
-        <v>22</v>
+        <v>29</v>
       </c>
       <c r="F356" s="9" t="s">
         <v>28</v>
@@ -10162,7 +10162,7 @@
         <v>27</v>
       </c>
       <c r="E357" s="11">
-        <v>17</v>
+        <v>26</v>
       </c>
       <c r="F357" s="9" t="s">
         <v>28</v>
@@ -10208,7 +10208,7 @@
         <v>27</v>
       </c>
       <c r="E359" s="11">
-        <v>15</v>
+        <v>18</v>
       </c>
       <c r="F359" s="9" t="s">
         <v>28</v>
@@ -10231,7 +10231,7 @@
         <v>27</v>
       </c>
       <c r="E360" s="11">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="F360" s="9" t="s">
         <v>28</v>
@@ -10254,7 +10254,7 @@
         <v>27</v>
       </c>
       <c r="E361" s="11">
-        <v>31</v>
+        <v>18</v>
       </c>
       <c r="F361" s="9" t="s">
         <v>28</v>
@@ -10277,7 +10277,7 @@
         <v>27</v>
       </c>
       <c r="E362" s="11">
-        <v>30</v>
+        <v>22</v>
       </c>
       <c r="F362" s="9" t="s">
         <v>28</v>
@@ -10323,7 +10323,7 @@
         <v>27</v>
       </c>
       <c r="E364" s="11">
-        <v>10</v>
+        <v>27</v>
       </c>
       <c r="F364" s="9" t="s">
         <v>28</v>
@@ -10369,7 +10369,7 @@
         <v>27</v>
       </c>
       <c r="E366" s="11">
-        <v>12</v>
+        <v>17</v>
       </c>
       <c r="F366" s="9" t="s">
         <v>28</v>
@@ -10392,7 +10392,7 @@
         <v>27</v>
       </c>
       <c r="E367" s="11">
-        <v>21</v>
+        <v>29</v>
       </c>
       <c r="F367" s="9" t="s">
         <v>28</v>
@@ -10415,7 +10415,7 @@
         <v>27</v>
       </c>
       <c r="E368" s="11">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="F368" s="9" t="s">
         <v>28</v>
@@ -10438,7 +10438,7 @@
         <v>27</v>
       </c>
       <c r="E369" s="11">
-        <v>15</v>
+        <v>27</v>
       </c>
       <c r="F369" s="9" t="s">
         <v>28</v>
@@ -10461,7 +10461,7 @@
         <v>27</v>
       </c>
       <c r="E370" s="11">
-        <v>19</v>
+        <v>24</v>
       </c>
       <c r="F370" s="9" t="s">
         <v>28</v>
@@ -10484,7 +10484,7 @@
         <v>27</v>
       </c>
       <c r="E371" s="11">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="F371" s="9" t="s">
         <v>28</v>
@@ -10507,7 +10507,7 @@
         <v>27</v>
       </c>
       <c r="E372" s="11">
-        <v>12</v>
+        <v>27</v>
       </c>
       <c r="F372" s="9" t="s">
         <v>28</v>
@@ -10530,7 +10530,7 @@
         <v>27</v>
       </c>
       <c r="E373" s="11">
-        <v>17</v>
+        <v>10</v>
       </c>
       <c r="F373" s="9" t="s">
         <v>28</v>
@@ -10553,7 +10553,7 @@
         <v>27</v>
       </c>
       <c r="E374" s="11">
-        <v>13</v>
+        <v>23</v>
       </c>
       <c r="F374" s="9" t="s">
         <v>28</v>
@@ -10576,7 +10576,7 @@
         <v>27</v>
       </c>
       <c r="E375" s="11">
-        <v>15</v>
+        <v>28</v>
       </c>
       <c r="F375" s="9" t="s">
         <v>28</v>
@@ -10599,7 +10599,7 @@
         <v>27</v>
       </c>
       <c r="E376" s="11">
-        <v>19</v>
+        <v>24</v>
       </c>
       <c r="F376" s="9" t="s">
         <v>28</v>
@@ -10622,7 +10622,7 @@
         <v>27</v>
       </c>
       <c r="E377" s="11">
-        <v>11</v>
+        <v>24</v>
       </c>
       <c r="F377" s="9" t="s">
         <v>28</v>
@@ -10645,7 +10645,7 @@
         <v>27</v>
       </c>
       <c r="E378" s="11">
-        <v>27</v>
+        <v>31</v>
       </c>
       <c r="F378" s="9" t="s">
         <v>28</v>
@@ -10668,7 +10668,7 @@
         <v>27</v>
       </c>
       <c r="E379" s="11">
-        <v>26</v>
+        <v>21</v>
       </c>
       <c r="F379" s="9" t="s">
         <v>28</v>
@@ -10691,7 +10691,7 @@
         <v>27</v>
       </c>
       <c r="E380" s="11">
-        <v>29</v>
+        <v>20</v>
       </c>
       <c r="F380" s="9" t="s">
         <v>28</v>
@@ -10714,7 +10714,7 @@
         <v>27</v>
       </c>
       <c r="E381" s="11">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="F381" s="9" t="s">
         <v>28</v>
@@ -10737,7 +10737,7 @@
         <v>27</v>
       </c>
       <c r="E382" s="11">
-        <v>18</v>
+        <v>26</v>
       </c>
       <c r="F382" s="9" t="s">
         <v>28</v>
@@ -10760,7 +10760,7 @@
         <v>27</v>
       </c>
       <c r="E383" s="11">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="F383" s="9" t="s">
         <v>28</v>
@@ -10783,7 +10783,7 @@
         <v>27</v>
       </c>
       <c r="E384" s="11">
-        <v>24</v>
+        <v>17</v>
       </c>
       <c r="F384" s="9" t="s">
         <v>28</v>
@@ -10806,7 +10806,7 @@
         <v>27</v>
       </c>
       <c r="E385" s="11">
-        <v>31</v>
+        <v>10</v>
       </c>
       <c r="F385" s="9" t="s">
         <v>28</v>
@@ -10829,7 +10829,7 @@
         <v>27</v>
       </c>
       <c r="E386" s="11">
-        <v>22</v>
+        <v>19</v>
       </c>
       <c r="F386" s="9" t="s">
         <v>28</v>
@@ -10852,7 +10852,7 @@
         <v>27</v>
       </c>
       <c r="E387" s="11">
-        <v>26</v>
+        <v>8</v>
       </c>
       <c r="F387" s="9" t="s">
         <v>28</v>
@@ -10875,7 +10875,7 @@
         <v>27</v>
       </c>
       <c r="E388" s="11">
-        <v>9</v>
+        <v>19</v>
       </c>
       <c r="F388" s="9" t="s">
         <v>28</v>
@@ -10898,7 +10898,7 @@
         <v>27</v>
       </c>
       <c r="E389" s="11">
-        <v>19</v>
+        <v>17</v>
       </c>
       <c r="F389" s="9" t="s">
         <v>28</v>
@@ -10921,7 +10921,7 @@
         <v>27</v>
       </c>
       <c r="E390" s="11">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="F390" s="9" t="s">
         <v>28</v>
@@ -10944,7 +10944,7 @@
         <v>27</v>
       </c>
       <c r="E391" s="11">
-        <v>26</v>
+        <v>12</v>
       </c>
       <c r="F391" s="9" t="s">
         <v>28</v>
@@ -10967,7 +10967,7 @@
         <v>27</v>
       </c>
       <c r="E392" s="11">
-        <v>11</v>
+        <v>24</v>
       </c>
       <c r="F392" s="9" t="s">
         <v>28</v>
@@ -10990,7 +10990,7 @@
         <v>27</v>
       </c>
       <c r="E393" s="11">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="F393" s="9" t="s">
         <v>28</v>
@@ -11013,7 +11013,7 @@
         <v>27</v>
       </c>
       <c r="E394" s="11">
-        <v>18</v>
+        <v>13</v>
       </c>
       <c r="F394" s="9" t="s">
         <v>28</v>
@@ -11036,7 +11036,7 @@
         <v>27</v>
       </c>
       <c r="E395" s="11">
-        <v>18</v>
+        <v>24</v>
       </c>
       <c r="F395" s="9" t="s">
         <v>28</v>
@@ -11059,7 +11059,7 @@
         <v>27</v>
       </c>
       <c r="E396" s="11">
-        <v>21</v>
+        <v>26</v>
       </c>
       <c r="F396" s="9" t="s">
         <v>28</v>
@@ -11082,7 +11082,7 @@
         <v>27</v>
       </c>
       <c r="E397" s="11">
-        <v>31</v>
+        <v>24</v>
       </c>
       <c r="F397" s="9" t="s">
         <v>28</v>
@@ -11105,7 +11105,7 @@
         <v>27</v>
       </c>
       <c r="E398" s="11">
-        <v>20</v>
+        <v>24</v>
       </c>
       <c r="F398" s="9" t="s">
         <v>28</v>
@@ -11151,7 +11151,7 @@
         <v>27</v>
       </c>
       <c r="E400" s="11">
-        <v>13</v>
+        <v>9</v>
       </c>
       <c r="F400" s="9" t="s">
         <v>28</v>
@@ -11174,7 +11174,7 @@
         <v>27</v>
       </c>
       <c r="E401" s="11">
-        <v>20</v>
+        <v>25</v>
       </c>
       <c r="F401" s="9" t="s">
         <v>28</v>

</xml_diff>

<commit_message>
feat(my-items): add Items Published section with publisher edit and delete modal functionality
</commit_message>
<xml_diff>
--- a/all-test-reports/selenium/selenium_e2e_test_report.xlsx
+++ b/all-test-reports/selenium/selenium_e2e_test_report.xlsx
@@ -35,7 +35,7 @@
     <t>Execution Date</t>
   </si>
   <si>
-    <t>28/7/2026, 11:12:55 am</t>
+    <t>28/7/2026, 11:17:39 am</t>
   </si>
   <si>
     <t>Browser / Mode</t>
@@ -98,7 +98,7 @@
     <t>PASS</t>
   </si>
   <si>
-    <t>11:12:55 am</t>
+    <t>11:17:39 am</t>
   </si>
   <si>
     <t>N/A</t>
@@ -1997,7 +1997,7 @@
         <v>27</v>
       </c>
       <c r="E2" s="11">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="F2" s="9" t="s">
         <v>28</v>
@@ -2020,7 +2020,7 @@
         <v>27</v>
       </c>
       <c r="E3" s="11">
-        <v>21</v>
+        <v>30</v>
       </c>
       <c r="F3" s="9" t="s">
         <v>28</v>
@@ -2043,7 +2043,7 @@
         <v>27</v>
       </c>
       <c r="E4" s="11">
-        <v>19</v>
+        <v>8</v>
       </c>
       <c r="F4" s="9" t="s">
         <v>28</v>
@@ -2066,7 +2066,7 @@
         <v>27</v>
       </c>
       <c r="E5" s="11">
-        <v>9</v>
+        <v>14</v>
       </c>
       <c r="F5" s="9" t="s">
         <v>28</v>
@@ -2089,7 +2089,7 @@
         <v>27</v>
       </c>
       <c r="E6" s="11">
-        <v>18</v>
+        <v>11</v>
       </c>
       <c r="F6" s="9" t="s">
         <v>28</v>
@@ -2112,7 +2112,7 @@
         <v>27</v>
       </c>
       <c r="E7" s="11">
-        <v>21</v>
+        <v>23</v>
       </c>
       <c r="F7" s="9" t="s">
         <v>28</v>
@@ -2135,7 +2135,7 @@
         <v>27</v>
       </c>
       <c r="E8" s="11">
-        <v>23</v>
+        <v>28</v>
       </c>
       <c r="F8" s="9" t="s">
         <v>28</v>
@@ -2158,7 +2158,7 @@
         <v>27</v>
       </c>
       <c r="E9" s="11">
-        <v>17</v>
+        <v>25</v>
       </c>
       <c r="F9" s="9" t="s">
         <v>28</v>
@@ -2181,7 +2181,7 @@
         <v>27</v>
       </c>
       <c r="E10" s="11">
-        <v>8</v>
+        <v>11</v>
       </c>
       <c r="F10" s="9" t="s">
         <v>28</v>
@@ -2204,7 +2204,7 @@
         <v>27</v>
       </c>
       <c r="E11" s="11">
-        <v>13</v>
+        <v>29</v>
       </c>
       <c r="F11" s="9" t="s">
         <v>28</v>
@@ -2227,7 +2227,7 @@
         <v>27</v>
       </c>
       <c r="E12" s="11">
-        <v>31</v>
+        <v>8</v>
       </c>
       <c r="F12" s="9" t="s">
         <v>28</v>
@@ -2250,7 +2250,7 @@
         <v>27</v>
       </c>
       <c r="E13" s="11">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="F13" s="9" t="s">
         <v>28</v>
@@ -2273,7 +2273,7 @@
         <v>27</v>
       </c>
       <c r="E14" s="11">
-        <v>18</v>
+        <v>22</v>
       </c>
       <c r="F14" s="9" t="s">
         <v>28</v>
@@ -2296,7 +2296,7 @@
         <v>27</v>
       </c>
       <c r="E15" s="11">
-        <v>16</v>
+        <v>25</v>
       </c>
       <c r="F15" s="9" t="s">
         <v>28</v>
@@ -2319,7 +2319,7 @@
         <v>27</v>
       </c>
       <c r="E16" s="11">
-        <v>19</v>
+        <v>25</v>
       </c>
       <c r="F16" s="9" t="s">
         <v>28</v>
@@ -2342,7 +2342,7 @@
         <v>27</v>
       </c>
       <c r="E17" s="11">
-        <v>28</v>
+        <v>17</v>
       </c>
       <c r="F17" s="9" t="s">
         <v>28</v>
@@ -2365,7 +2365,7 @@
         <v>27</v>
       </c>
       <c r="E18" s="11">
-        <v>25</v>
+        <v>21</v>
       </c>
       <c r="F18" s="9" t="s">
         <v>28</v>
@@ -2388,7 +2388,7 @@
         <v>27</v>
       </c>
       <c r="E19" s="11">
-        <v>19</v>
+        <v>16</v>
       </c>
       <c r="F19" s="9" t="s">
         <v>28</v>
@@ -2411,7 +2411,7 @@
         <v>27</v>
       </c>
       <c r="E20" s="11">
-        <v>14</v>
+        <v>10</v>
       </c>
       <c r="F20" s="9" t="s">
         <v>28</v>
@@ -2434,7 +2434,7 @@
         <v>27</v>
       </c>
       <c r="E21" s="11">
-        <v>19</v>
+        <v>24</v>
       </c>
       <c r="F21" s="9" t="s">
         <v>28</v>
@@ -2457,7 +2457,7 @@
         <v>27</v>
       </c>
       <c r="E22" s="11">
-        <v>14</v>
+        <v>10</v>
       </c>
       <c r="F22" s="9" t="s">
         <v>28</v>
@@ -2480,7 +2480,7 @@
         <v>27</v>
       </c>
       <c r="E23" s="11">
-        <v>9</v>
+        <v>20</v>
       </c>
       <c r="F23" s="9" t="s">
         <v>28</v>
@@ -2503,7 +2503,7 @@
         <v>27</v>
       </c>
       <c r="E24" s="11">
-        <v>18</v>
+        <v>13</v>
       </c>
       <c r="F24" s="9" t="s">
         <v>28</v>
@@ -2526,7 +2526,7 @@
         <v>27</v>
       </c>
       <c r="E25" s="11">
-        <v>9</v>
+        <v>12</v>
       </c>
       <c r="F25" s="9" t="s">
         <v>28</v>
@@ -2549,7 +2549,7 @@
         <v>27</v>
       </c>
       <c r="E26" s="11">
-        <v>30</v>
+        <v>18</v>
       </c>
       <c r="F26" s="9" t="s">
         <v>28</v>
@@ -2572,7 +2572,7 @@
         <v>27</v>
       </c>
       <c r="E27" s="11">
-        <v>23</v>
+        <v>21</v>
       </c>
       <c r="F27" s="9" t="s">
         <v>28</v>
@@ -2595,7 +2595,7 @@
         <v>27</v>
       </c>
       <c r="E28" s="11">
-        <v>31</v>
+        <v>14</v>
       </c>
       <c r="F28" s="9" t="s">
         <v>28</v>
@@ -2618,7 +2618,7 @@
         <v>27</v>
       </c>
       <c r="E29" s="11">
-        <v>14</v>
+        <v>24</v>
       </c>
       <c r="F29" s="9" t="s">
         <v>28</v>
@@ -2641,7 +2641,7 @@
         <v>27</v>
       </c>
       <c r="E30" s="11">
-        <v>30</v>
+        <v>13</v>
       </c>
       <c r="F30" s="9" t="s">
         <v>28</v>
@@ -2664,7 +2664,7 @@
         <v>27</v>
       </c>
       <c r="E31" s="11">
-        <v>15</v>
+        <v>26</v>
       </c>
       <c r="F31" s="9" t="s">
         <v>28</v>
@@ -2687,7 +2687,7 @@
         <v>27</v>
       </c>
       <c r="E32" s="11">
-        <v>10</v>
+        <v>30</v>
       </c>
       <c r="F32" s="9" t="s">
         <v>28</v>
@@ -2710,7 +2710,7 @@
         <v>27</v>
       </c>
       <c r="E33" s="11">
-        <v>12</v>
+        <v>9</v>
       </c>
       <c r="F33" s="9" t="s">
         <v>28</v>
@@ -2733,7 +2733,7 @@
         <v>27</v>
       </c>
       <c r="E34" s="11">
-        <v>28</v>
+        <v>25</v>
       </c>
       <c r="F34" s="9" t="s">
         <v>28</v>
@@ -2756,7 +2756,7 @@
         <v>27</v>
       </c>
       <c r="E35" s="11">
-        <v>18</v>
+        <v>26</v>
       </c>
       <c r="F35" s="9" t="s">
         <v>28</v>
@@ -2779,7 +2779,7 @@
         <v>27</v>
       </c>
       <c r="E36" s="11">
-        <v>20</v>
+        <v>28</v>
       </c>
       <c r="F36" s="9" t="s">
         <v>28</v>
@@ -2802,7 +2802,7 @@
         <v>27</v>
       </c>
       <c r="E37" s="11">
-        <v>31</v>
+        <v>22</v>
       </c>
       <c r="F37" s="9" t="s">
         <v>28</v>
@@ -2825,7 +2825,7 @@
         <v>27</v>
       </c>
       <c r="E38" s="11">
-        <v>14</v>
+        <v>16</v>
       </c>
       <c r="F38" s="9" t="s">
         <v>28</v>
@@ -2848,7 +2848,7 @@
         <v>27</v>
       </c>
       <c r="E39" s="11">
-        <v>8</v>
+        <v>19</v>
       </c>
       <c r="F39" s="9" t="s">
         <v>28</v>
@@ -2871,7 +2871,7 @@
         <v>27</v>
       </c>
       <c r="E40" s="11">
-        <v>27</v>
+        <v>19</v>
       </c>
       <c r="F40" s="9" t="s">
         <v>28</v>
@@ -2894,7 +2894,7 @@
         <v>27</v>
       </c>
       <c r="E41" s="11">
-        <v>31</v>
+        <v>29</v>
       </c>
       <c r="F41" s="9" t="s">
         <v>28</v>
@@ -2917,7 +2917,7 @@
         <v>27</v>
       </c>
       <c r="E42" s="11">
-        <v>16</v>
+        <v>10</v>
       </c>
       <c r="F42" s="9" t="s">
         <v>28</v>
@@ -2940,7 +2940,7 @@
         <v>27</v>
       </c>
       <c r="E43" s="11">
-        <v>15</v>
+        <v>10</v>
       </c>
       <c r="F43" s="9" t="s">
         <v>28</v>
@@ -2963,7 +2963,7 @@
         <v>27</v>
       </c>
       <c r="E44" s="11">
-        <v>15</v>
+        <v>10</v>
       </c>
       <c r="F44" s="9" t="s">
         <v>28</v>
@@ -2986,7 +2986,7 @@
         <v>27</v>
       </c>
       <c r="E45" s="11">
-        <v>13</v>
+        <v>20</v>
       </c>
       <c r="F45" s="9" t="s">
         <v>28</v>
@@ -3009,7 +3009,7 @@
         <v>27</v>
       </c>
       <c r="E46" s="11">
-        <v>18</v>
+        <v>9</v>
       </c>
       <c r="F46" s="9" t="s">
         <v>28</v>
@@ -3032,7 +3032,7 @@
         <v>27</v>
       </c>
       <c r="E47" s="11">
-        <v>31</v>
+        <v>15</v>
       </c>
       <c r="F47" s="9" t="s">
         <v>28</v>
@@ -3055,7 +3055,7 @@
         <v>27</v>
       </c>
       <c r="E48" s="11">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="F48" s="9" t="s">
         <v>28</v>
@@ -3078,7 +3078,7 @@
         <v>27</v>
       </c>
       <c r="E49" s="11">
-        <v>31</v>
+        <v>23</v>
       </c>
       <c r="F49" s="9" t="s">
         <v>28</v>
@@ -3101,7 +3101,7 @@
         <v>27</v>
       </c>
       <c r="E50" s="11">
-        <v>23</v>
+        <v>9</v>
       </c>
       <c r="F50" s="9" t="s">
         <v>28</v>
@@ -3124,7 +3124,7 @@
         <v>27</v>
       </c>
       <c r="E51" s="11">
-        <v>19</v>
+        <v>14</v>
       </c>
       <c r="F51" s="9" t="s">
         <v>28</v>
@@ -3147,7 +3147,7 @@
         <v>27</v>
       </c>
       <c r="E52" s="11">
-        <v>12</v>
+        <v>9</v>
       </c>
       <c r="F52" s="9" t="s">
         <v>28</v>
@@ -3170,7 +3170,7 @@
         <v>27</v>
       </c>
       <c r="E53" s="11">
-        <v>20</v>
+        <v>14</v>
       </c>
       <c r="F53" s="9" t="s">
         <v>28</v>
@@ -3193,7 +3193,7 @@
         <v>27</v>
       </c>
       <c r="E54" s="11">
-        <v>24</v>
+        <v>10</v>
       </c>
       <c r="F54" s="9" t="s">
         <v>28</v>
@@ -3216,7 +3216,7 @@
         <v>27</v>
       </c>
       <c r="E55" s="11">
-        <v>19</v>
+        <v>24</v>
       </c>
       <c r="F55" s="9" t="s">
         <v>28</v>
@@ -3262,7 +3262,7 @@
         <v>27</v>
       </c>
       <c r="E57" s="11">
-        <v>18</v>
+        <v>30</v>
       </c>
       <c r="F57" s="9" t="s">
         <v>28</v>
@@ -3285,7 +3285,7 @@
         <v>27</v>
       </c>
       <c r="E58" s="11">
-        <v>19</v>
+        <v>11</v>
       </c>
       <c r="F58" s="9" t="s">
         <v>28</v>
@@ -3308,7 +3308,7 @@
         <v>27</v>
       </c>
       <c r="E59" s="11">
-        <v>27</v>
+        <v>11</v>
       </c>
       <c r="F59" s="9" t="s">
         <v>28</v>
@@ -3331,7 +3331,7 @@
         <v>27</v>
       </c>
       <c r="E60" s="11">
-        <v>18</v>
+        <v>9</v>
       </c>
       <c r="F60" s="9" t="s">
         <v>28</v>
@@ -3354,7 +3354,7 @@
         <v>27</v>
       </c>
       <c r="E61" s="11">
-        <v>11</v>
+        <v>25</v>
       </c>
       <c r="F61" s="9" t="s">
         <v>28</v>
@@ -3377,7 +3377,7 @@
         <v>27</v>
       </c>
       <c r="E62" s="11">
-        <v>9</v>
+        <v>28</v>
       </c>
       <c r="F62" s="9" t="s">
         <v>28</v>
@@ -3400,7 +3400,7 @@
         <v>27</v>
       </c>
       <c r="E63" s="11">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="F63" s="9" t="s">
         <v>28</v>
@@ -3423,7 +3423,7 @@
         <v>27</v>
       </c>
       <c r="E64" s="11">
-        <v>17</v>
+        <v>10</v>
       </c>
       <c r="F64" s="9" t="s">
         <v>28</v>
@@ -3446,7 +3446,7 @@
         <v>27</v>
       </c>
       <c r="E65" s="11">
-        <v>23</v>
+        <v>19</v>
       </c>
       <c r="F65" s="9" t="s">
         <v>28</v>
@@ -3469,7 +3469,7 @@
         <v>27</v>
       </c>
       <c r="E66" s="11">
-        <v>11</v>
+        <v>8</v>
       </c>
       <c r="F66" s="9" t="s">
         <v>28</v>
@@ -3515,7 +3515,7 @@
         <v>27</v>
       </c>
       <c r="E68" s="11">
-        <v>15</v>
+        <v>22</v>
       </c>
       <c r="F68" s="9" t="s">
         <v>28</v>
@@ -3538,7 +3538,7 @@
         <v>27</v>
       </c>
       <c r="E69" s="11">
-        <v>14</v>
+        <v>16</v>
       </c>
       <c r="F69" s="9" t="s">
         <v>28</v>
@@ -3561,7 +3561,7 @@
         <v>27</v>
       </c>
       <c r="E70" s="11">
-        <v>8</v>
+        <v>12</v>
       </c>
       <c r="F70" s="9" t="s">
         <v>28</v>
@@ -3584,7 +3584,7 @@
         <v>27</v>
       </c>
       <c r="E71" s="11">
-        <v>15</v>
+        <v>17</v>
       </c>
       <c r="F71" s="9" t="s">
         <v>28</v>
@@ -3607,7 +3607,7 @@
         <v>27</v>
       </c>
       <c r="E72" s="11">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="F72" s="9" t="s">
         <v>28</v>
@@ -3630,7 +3630,7 @@
         <v>27</v>
       </c>
       <c r="E73" s="11">
-        <v>29</v>
+        <v>25</v>
       </c>
       <c r="F73" s="9" t="s">
         <v>28</v>
@@ -3653,7 +3653,7 @@
         <v>27</v>
       </c>
       <c r="E74" s="11">
-        <v>31</v>
+        <v>15</v>
       </c>
       <c r="F74" s="9" t="s">
         <v>28</v>
@@ -3676,7 +3676,7 @@
         <v>27</v>
       </c>
       <c r="E75" s="11">
-        <v>11</v>
+        <v>24</v>
       </c>
       <c r="F75" s="9" t="s">
         <v>28</v>
@@ -3699,7 +3699,7 @@
         <v>27</v>
       </c>
       <c r="E76" s="11">
-        <v>14</v>
+        <v>16</v>
       </c>
       <c r="F76" s="9" t="s">
         <v>28</v>
@@ -3745,7 +3745,7 @@
         <v>27</v>
       </c>
       <c r="E78" s="11">
-        <v>8</v>
+        <v>14</v>
       </c>
       <c r="F78" s="9" t="s">
         <v>28</v>
@@ -3768,7 +3768,7 @@
         <v>27</v>
       </c>
       <c r="E79" s="11">
-        <v>28</v>
+        <v>19</v>
       </c>
       <c r="F79" s="9" t="s">
         <v>28</v>
@@ -3791,7 +3791,7 @@
         <v>27</v>
       </c>
       <c r="E80" s="11">
-        <v>27</v>
+        <v>10</v>
       </c>
       <c r="F80" s="9" t="s">
         <v>28</v>
@@ -3814,7 +3814,7 @@
         <v>27</v>
       </c>
       <c r="E81" s="11">
-        <v>24</v>
+        <v>11</v>
       </c>
       <c r="F81" s="9" t="s">
         <v>28</v>
@@ -3837,7 +3837,7 @@
         <v>27</v>
       </c>
       <c r="E82" s="11">
-        <v>15</v>
+        <v>24</v>
       </c>
       <c r="F82" s="9" t="s">
         <v>28</v>
@@ -3860,7 +3860,7 @@
         <v>27</v>
       </c>
       <c r="E83" s="11">
-        <v>14</v>
+        <v>19</v>
       </c>
       <c r="F83" s="9" t="s">
         <v>28</v>
@@ -3883,7 +3883,7 @@
         <v>27</v>
       </c>
       <c r="E84" s="11">
-        <v>15</v>
+        <v>29</v>
       </c>
       <c r="F84" s="9" t="s">
         <v>28</v>
@@ -3906,7 +3906,7 @@
         <v>27</v>
       </c>
       <c r="E85" s="11">
-        <v>17</v>
+        <v>30</v>
       </c>
       <c r="F85" s="9" t="s">
         <v>28</v>
@@ -3929,7 +3929,7 @@
         <v>27</v>
       </c>
       <c r="E86" s="11">
-        <v>21</v>
+        <v>30</v>
       </c>
       <c r="F86" s="9" t="s">
         <v>28</v>
@@ -3952,7 +3952,7 @@
         <v>27</v>
       </c>
       <c r="E87" s="11">
-        <v>27</v>
+        <v>23</v>
       </c>
       <c r="F87" s="9" t="s">
         <v>28</v>
@@ -3975,7 +3975,7 @@
         <v>27</v>
       </c>
       <c r="E88" s="11">
-        <v>10</v>
+        <v>19</v>
       </c>
       <c r="F88" s="9" t="s">
         <v>28</v>
@@ -3998,7 +3998,7 @@
         <v>27</v>
       </c>
       <c r="E89" s="11">
-        <v>25</v>
+        <v>18</v>
       </c>
       <c r="F89" s="9" t="s">
         <v>28</v>
@@ -4021,7 +4021,7 @@
         <v>27</v>
       </c>
       <c r="E90" s="11">
-        <v>26</v>
+        <v>24</v>
       </c>
       <c r="F90" s="9" t="s">
         <v>28</v>
@@ -4044,7 +4044,7 @@
         <v>27</v>
       </c>
       <c r="E91" s="11">
-        <v>27</v>
+        <v>30</v>
       </c>
       <c r="F91" s="9" t="s">
         <v>28</v>
@@ -4067,7 +4067,7 @@
         <v>27</v>
       </c>
       <c r="E92" s="11">
-        <v>18</v>
+        <v>8</v>
       </c>
       <c r="F92" s="9" t="s">
         <v>28</v>
@@ -4090,7 +4090,7 @@
         <v>27</v>
       </c>
       <c r="E93" s="11">
-        <v>23</v>
+        <v>15</v>
       </c>
       <c r="F93" s="9" t="s">
         <v>28</v>
@@ -4113,7 +4113,7 @@
         <v>27</v>
       </c>
       <c r="E94" s="11">
-        <v>22</v>
+        <v>24</v>
       </c>
       <c r="F94" s="9" t="s">
         <v>28</v>
@@ -4136,7 +4136,7 @@
         <v>27</v>
       </c>
       <c r="E95" s="11">
-        <v>29</v>
+        <v>21</v>
       </c>
       <c r="F95" s="9" t="s">
         <v>28</v>
@@ -4159,7 +4159,7 @@
         <v>27</v>
       </c>
       <c r="E96" s="11">
-        <v>30</v>
+        <v>18</v>
       </c>
       <c r="F96" s="9" t="s">
         <v>28</v>
@@ -4182,7 +4182,7 @@
         <v>27</v>
       </c>
       <c r="E97" s="11">
-        <v>14</v>
+        <v>25</v>
       </c>
       <c r="F97" s="9" t="s">
         <v>28</v>
@@ -4228,7 +4228,7 @@
         <v>27</v>
       </c>
       <c r="E99" s="11">
-        <v>11</v>
+        <v>13</v>
       </c>
       <c r="F99" s="9" t="s">
         <v>28</v>
@@ -4251,7 +4251,7 @@
         <v>27</v>
       </c>
       <c r="E100" s="11">
-        <v>31</v>
+        <v>28</v>
       </c>
       <c r="F100" s="9" t="s">
         <v>28</v>
@@ -4274,7 +4274,7 @@
         <v>27</v>
       </c>
       <c r="E101" s="11">
-        <v>27</v>
+        <v>21</v>
       </c>
       <c r="F101" s="9" t="s">
         <v>28</v>
@@ -4297,7 +4297,7 @@
         <v>27</v>
       </c>
       <c r="E102" s="11">
-        <v>12</v>
+        <v>29</v>
       </c>
       <c r="F102" s="9" t="s">
         <v>28</v>
@@ -4320,7 +4320,7 @@
         <v>27</v>
       </c>
       <c r="E103" s="11">
-        <v>25</v>
+        <v>18</v>
       </c>
       <c r="F103" s="9" t="s">
         <v>28</v>
@@ -4343,7 +4343,7 @@
         <v>27</v>
       </c>
       <c r="E104" s="11">
-        <v>16</v>
+        <v>13</v>
       </c>
       <c r="F104" s="9" t="s">
         <v>28</v>
@@ -4366,7 +4366,7 @@
         <v>27</v>
       </c>
       <c r="E105" s="11">
-        <v>26</v>
+        <v>10</v>
       </c>
       <c r="F105" s="9" t="s">
         <v>28</v>
@@ -4389,7 +4389,7 @@
         <v>27</v>
       </c>
       <c r="E106" s="11">
-        <v>31</v>
+        <v>9</v>
       </c>
       <c r="F106" s="9" t="s">
         <v>28</v>
@@ -4412,7 +4412,7 @@
         <v>27</v>
       </c>
       <c r="E107" s="11">
-        <v>29</v>
+        <v>23</v>
       </c>
       <c r="F107" s="9" t="s">
         <v>28</v>
@@ -4458,7 +4458,7 @@
         <v>27</v>
       </c>
       <c r="E109" s="11">
-        <v>25</v>
+        <v>21</v>
       </c>
       <c r="F109" s="9" t="s">
         <v>28</v>
@@ -4481,7 +4481,7 @@
         <v>27</v>
       </c>
       <c r="E110" s="11">
-        <v>26</v>
+        <v>17</v>
       </c>
       <c r="F110" s="9" t="s">
         <v>28</v>
@@ -4504,7 +4504,7 @@
         <v>27</v>
       </c>
       <c r="E111" s="11">
-        <v>27</v>
+        <v>17</v>
       </c>
       <c r="F111" s="9" t="s">
         <v>28</v>
@@ -4527,7 +4527,7 @@
         <v>27</v>
       </c>
       <c r="E112" s="11">
-        <v>9</v>
+        <v>26</v>
       </c>
       <c r="F112" s="9" t="s">
         <v>28</v>
@@ -4550,7 +4550,7 @@
         <v>27</v>
       </c>
       <c r="E113" s="11">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="F113" s="9" t="s">
         <v>28</v>
@@ -4573,7 +4573,7 @@
         <v>27</v>
       </c>
       <c r="E114" s="11">
-        <v>16</v>
+        <v>10</v>
       </c>
       <c r="F114" s="9" t="s">
         <v>28</v>
@@ -4596,7 +4596,7 @@
         <v>27</v>
       </c>
       <c r="E115" s="11">
-        <v>28</v>
+        <v>17</v>
       </c>
       <c r="F115" s="9" t="s">
         <v>28</v>
@@ -4619,7 +4619,7 @@
         <v>27</v>
       </c>
       <c r="E116" s="11">
-        <v>22</v>
+        <v>31</v>
       </c>
       <c r="F116" s="9" t="s">
         <v>28</v>
@@ -4642,7 +4642,7 @@
         <v>27</v>
       </c>
       <c r="E117" s="11">
-        <v>10</v>
+        <v>17</v>
       </c>
       <c r="F117" s="9" t="s">
         <v>28</v>
@@ -4665,7 +4665,7 @@
         <v>27</v>
       </c>
       <c r="E118" s="11">
-        <v>29</v>
+        <v>17</v>
       </c>
       <c r="F118" s="9" t="s">
         <v>28</v>
@@ -4688,7 +4688,7 @@
         <v>27</v>
       </c>
       <c r="E119" s="11">
-        <v>15</v>
+        <v>26</v>
       </c>
       <c r="F119" s="9" t="s">
         <v>28</v>
@@ -4711,7 +4711,7 @@
         <v>27</v>
       </c>
       <c r="E120" s="11">
-        <v>23</v>
+        <v>9</v>
       </c>
       <c r="F120" s="9" t="s">
         <v>28</v>
@@ -4734,7 +4734,7 @@
         <v>27</v>
       </c>
       <c r="E121" s="11">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="F121" s="9" t="s">
         <v>28</v>
@@ -4780,7 +4780,7 @@
         <v>27</v>
       </c>
       <c r="E123" s="11">
-        <v>28</v>
+        <v>24</v>
       </c>
       <c r="F123" s="9" t="s">
         <v>28</v>
@@ -4803,7 +4803,7 @@
         <v>27</v>
       </c>
       <c r="E124" s="11">
-        <v>25</v>
+        <v>17</v>
       </c>
       <c r="F124" s="9" t="s">
         <v>28</v>
@@ -4826,7 +4826,7 @@
         <v>27</v>
       </c>
       <c r="E125" s="11">
-        <v>16</v>
+        <v>30</v>
       </c>
       <c r="F125" s="9" t="s">
         <v>28</v>
@@ -4849,7 +4849,7 @@
         <v>27</v>
       </c>
       <c r="E126" s="11">
-        <v>20</v>
+        <v>13</v>
       </c>
       <c r="F126" s="9" t="s">
         <v>28</v>
@@ -4872,7 +4872,7 @@
         <v>27</v>
       </c>
       <c r="E127" s="11">
-        <v>19</v>
+        <v>11</v>
       </c>
       <c r="F127" s="9" t="s">
         <v>28</v>
@@ -4895,7 +4895,7 @@
         <v>27</v>
       </c>
       <c r="E128" s="11">
-        <v>18</v>
+        <v>10</v>
       </c>
       <c r="F128" s="9" t="s">
         <v>28</v>
@@ -4918,7 +4918,7 @@
         <v>27</v>
       </c>
       <c r="E129" s="11">
-        <v>22</v>
+        <v>30</v>
       </c>
       <c r="F129" s="9" t="s">
         <v>28</v>
@@ -4941,7 +4941,7 @@
         <v>27</v>
       </c>
       <c r="E130" s="11">
-        <v>26</v>
+        <v>19</v>
       </c>
       <c r="F130" s="9" t="s">
         <v>28</v>
@@ -4964,7 +4964,7 @@
         <v>27</v>
       </c>
       <c r="E131" s="11">
-        <v>14</v>
+        <v>19</v>
       </c>
       <c r="F131" s="9" t="s">
         <v>28</v>
@@ -4987,7 +4987,7 @@
         <v>27</v>
       </c>
       <c r="E132" s="11">
-        <v>31</v>
+        <v>24</v>
       </c>
       <c r="F132" s="9" t="s">
         <v>28</v>
@@ -5010,7 +5010,7 @@
         <v>27</v>
       </c>
       <c r="E133" s="11">
-        <v>15</v>
+        <v>19</v>
       </c>
       <c r="F133" s="9" t="s">
         <v>28</v>
@@ -5033,7 +5033,7 @@
         <v>27</v>
       </c>
       <c r="E134" s="11">
-        <v>14</v>
+        <v>22</v>
       </c>
       <c r="F134" s="9" t="s">
         <v>28</v>
@@ -5056,7 +5056,7 @@
         <v>27</v>
       </c>
       <c r="E135" s="11">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="F135" s="9" t="s">
         <v>28</v>
@@ -5079,7 +5079,7 @@
         <v>27</v>
       </c>
       <c r="E136" s="11">
-        <v>22</v>
+        <v>30</v>
       </c>
       <c r="F136" s="9" t="s">
         <v>28</v>
@@ -5102,7 +5102,7 @@
         <v>27</v>
       </c>
       <c r="E137" s="11">
-        <v>11</v>
+        <v>23</v>
       </c>
       <c r="F137" s="9" t="s">
         <v>28</v>
@@ -5125,7 +5125,7 @@
         <v>27</v>
       </c>
       <c r="E138" s="11">
-        <v>9</v>
+        <v>28</v>
       </c>
       <c r="F138" s="9" t="s">
         <v>28</v>
@@ -5148,7 +5148,7 @@
         <v>27</v>
       </c>
       <c r="E139" s="11">
-        <v>31</v>
+        <v>26</v>
       </c>
       <c r="F139" s="9" t="s">
         <v>28</v>
@@ -5171,7 +5171,7 @@
         <v>27</v>
       </c>
       <c r="E140" s="11">
-        <v>9</v>
+        <v>22</v>
       </c>
       <c r="F140" s="9" t="s">
         <v>28</v>
@@ -5194,7 +5194,7 @@
         <v>27</v>
       </c>
       <c r="E141" s="11">
-        <v>27</v>
+        <v>23</v>
       </c>
       <c r="F141" s="9" t="s">
         <v>28</v>
@@ -5217,7 +5217,7 @@
         <v>27</v>
       </c>
       <c r="E142" s="11">
-        <v>29</v>
+        <v>20</v>
       </c>
       <c r="F142" s="9" t="s">
         <v>28</v>
@@ -5240,7 +5240,7 @@
         <v>27</v>
       </c>
       <c r="E143" s="11">
-        <v>15</v>
+        <v>11</v>
       </c>
       <c r="F143" s="9" t="s">
         <v>28</v>
@@ -5263,7 +5263,7 @@
         <v>27</v>
       </c>
       <c r="E144" s="11">
-        <v>21</v>
+        <v>27</v>
       </c>
       <c r="F144" s="9" t="s">
         <v>28</v>
@@ -5309,7 +5309,7 @@
         <v>27</v>
       </c>
       <c r="E146" s="11">
-        <v>23</v>
+        <v>18</v>
       </c>
       <c r="F146" s="9" t="s">
         <v>28</v>
@@ -5332,7 +5332,7 @@
         <v>27</v>
       </c>
       <c r="E147" s="11">
-        <v>12</v>
+        <v>9</v>
       </c>
       <c r="F147" s="9" t="s">
         <v>28</v>
@@ -5355,7 +5355,7 @@
         <v>27</v>
       </c>
       <c r="E148" s="11">
-        <v>17</v>
+        <v>11</v>
       </c>
       <c r="F148" s="9" t="s">
         <v>28</v>
@@ -5378,7 +5378,7 @@
         <v>27</v>
       </c>
       <c r="E149" s="11">
-        <v>25</v>
+        <v>12</v>
       </c>
       <c r="F149" s="9" t="s">
         <v>28</v>
@@ -5401,7 +5401,7 @@
         <v>27</v>
       </c>
       <c r="E150" s="11">
-        <v>31</v>
+        <v>14</v>
       </c>
       <c r="F150" s="9" t="s">
         <v>28</v>
@@ -5424,7 +5424,7 @@
         <v>27</v>
       </c>
       <c r="E151" s="11">
-        <v>14</v>
+        <v>29</v>
       </c>
       <c r="F151" s="9" t="s">
         <v>28</v>
@@ -5447,7 +5447,7 @@
         <v>27</v>
       </c>
       <c r="E152" s="11">
-        <v>31</v>
+        <v>16</v>
       </c>
       <c r="F152" s="9" t="s">
         <v>28</v>
@@ -5470,7 +5470,7 @@
         <v>27</v>
       </c>
       <c r="E153" s="11">
-        <v>19</v>
+        <v>13</v>
       </c>
       <c r="F153" s="9" t="s">
         <v>28</v>
@@ -5493,7 +5493,7 @@
         <v>27</v>
       </c>
       <c r="E154" s="11">
-        <v>25</v>
+        <v>27</v>
       </c>
       <c r="F154" s="9" t="s">
         <v>28</v>
@@ -5516,7 +5516,7 @@
         <v>27</v>
       </c>
       <c r="E155" s="11">
-        <v>27</v>
+        <v>15</v>
       </c>
       <c r="F155" s="9" t="s">
         <v>28</v>
@@ -5539,7 +5539,7 @@
         <v>27</v>
       </c>
       <c r="E156" s="11">
-        <v>18</v>
+        <v>9</v>
       </c>
       <c r="F156" s="9" t="s">
         <v>28</v>
@@ -5562,7 +5562,7 @@
         <v>27</v>
       </c>
       <c r="E157" s="11">
-        <v>12</v>
+        <v>20</v>
       </c>
       <c r="F157" s="9" t="s">
         <v>28</v>
@@ -5585,7 +5585,7 @@
         <v>27</v>
       </c>
       <c r="E158" s="11">
-        <v>30</v>
+        <v>13</v>
       </c>
       <c r="F158" s="9" t="s">
         <v>28</v>
@@ -5608,7 +5608,7 @@
         <v>27</v>
       </c>
       <c r="E159" s="11">
-        <v>22</v>
+        <v>15</v>
       </c>
       <c r="F159" s="9" t="s">
         <v>28</v>
@@ -5631,7 +5631,7 @@
         <v>27</v>
       </c>
       <c r="E160" s="11">
-        <v>30</v>
+        <v>8</v>
       </c>
       <c r="F160" s="9" t="s">
         <v>28</v>
@@ -5654,7 +5654,7 @@
         <v>27</v>
       </c>
       <c r="E161" s="11">
-        <v>16</v>
+        <v>18</v>
       </c>
       <c r="F161" s="9" t="s">
         <v>28</v>
@@ -5677,7 +5677,7 @@
         <v>27</v>
       </c>
       <c r="E162" s="11">
-        <v>22</v>
+        <v>19</v>
       </c>
       <c r="F162" s="9" t="s">
         <v>28</v>
@@ -5700,7 +5700,7 @@
         <v>27</v>
       </c>
       <c r="E163" s="11">
-        <v>19</v>
+        <v>9</v>
       </c>
       <c r="F163" s="9" t="s">
         <v>28</v>
@@ -5723,7 +5723,7 @@
         <v>27</v>
       </c>
       <c r="E164" s="11">
-        <v>13</v>
+        <v>19</v>
       </c>
       <c r="F164" s="9" t="s">
         <v>28</v>
@@ -5746,7 +5746,7 @@
         <v>27</v>
       </c>
       <c r="E165" s="11">
-        <v>9</v>
+        <v>28</v>
       </c>
       <c r="F165" s="9" t="s">
         <v>28</v>
@@ -5769,7 +5769,7 @@
         <v>27</v>
       </c>
       <c r="E166" s="11">
-        <v>31</v>
+        <v>22</v>
       </c>
       <c r="F166" s="9" t="s">
         <v>28</v>
@@ -5792,7 +5792,7 @@
         <v>27</v>
       </c>
       <c r="E167" s="11">
-        <v>26</v>
+        <v>31</v>
       </c>
       <c r="F167" s="9" t="s">
         <v>28</v>
@@ -5815,7 +5815,7 @@
         <v>27</v>
       </c>
       <c r="E168" s="11">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="F168" s="9" t="s">
         <v>28</v>
@@ -5838,7 +5838,7 @@
         <v>27</v>
       </c>
       <c r="E169" s="11">
-        <v>20</v>
+        <v>22</v>
       </c>
       <c r="F169" s="9" t="s">
         <v>28</v>
@@ -5861,7 +5861,7 @@
         <v>27</v>
       </c>
       <c r="E170" s="11">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="F170" s="9" t="s">
         <v>28</v>
@@ -5884,7 +5884,7 @@
         <v>27</v>
       </c>
       <c r="E171" s="11">
-        <v>23</v>
+        <v>28</v>
       </c>
       <c r="F171" s="9" t="s">
         <v>28</v>
@@ -5907,7 +5907,7 @@
         <v>27</v>
       </c>
       <c r="E172" s="11">
-        <v>13</v>
+        <v>27</v>
       </c>
       <c r="F172" s="9" t="s">
         <v>28</v>
@@ -5930,7 +5930,7 @@
         <v>27</v>
       </c>
       <c r="E173" s="11">
-        <v>20</v>
+        <v>25</v>
       </c>
       <c r="F173" s="9" t="s">
         <v>28</v>
@@ -5953,7 +5953,7 @@
         <v>27</v>
       </c>
       <c r="E174" s="11">
-        <v>20</v>
+        <v>23</v>
       </c>
       <c r="F174" s="9" t="s">
         <v>28</v>
@@ -5976,7 +5976,7 @@
         <v>27</v>
       </c>
       <c r="E175" s="11">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="F175" s="9" t="s">
         <v>28</v>
@@ -5999,7 +5999,7 @@
         <v>27</v>
       </c>
       <c r="E176" s="11">
-        <v>15</v>
+        <v>10</v>
       </c>
       <c r="F176" s="9" t="s">
         <v>28</v>
@@ -6045,7 +6045,7 @@
         <v>27</v>
       </c>
       <c r="E178" s="11">
-        <v>26</v>
+        <v>10</v>
       </c>
       <c r="F178" s="9" t="s">
         <v>28</v>
@@ -6068,7 +6068,7 @@
         <v>27</v>
       </c>
       <c r="E179" s="11">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="F179" s="9" t="s">
         <v>28</v>
@@ -6091,7 +6091,7 @@
         <v>27</v>
       </c>
       <c r="E180" s="11">
-        <v>10</v>
+        <v>22</v>
       </c>
       <c r="F180" s="9" t="s">
         <v>28</v>
@@ -6114,7 +6114,7 @@
         <v>27</v>
       </c>
       <c r="E181" s="11">
-        <v>21</v>
+        <v>17</v>
       </c>
       <c r="F181" s="9" t="s">
         <v>28</v>
@@ -6137,7 +6137,7 @@
         <v>27</v>
       </c>
       <c r="E182" s="11">
-        <v>9</v>
+        <v>25</v>
       </c>
       <c r="F182" s="9" t="s">
         <v>28</v>
@@ -6160,7 +6160,7 @@
         <v>27</v>
       </c>
       <c r="E183" s="11">
-        <v>27</v>
+        <v>21</v>
       </c>
       <c r="F183" s="9" t="s">
         <v>28</v>
@@ -6183,7 +6183,7 @@
         <v>27</v>
       </c>
       <c r="E184" s="11">
-        <v>24</v>
+        <v>12</v>
       </c>
       <c r="F184" s="9" t="s">
         <v>28</v>
@@ -6206,7 +6206,7 @@
         <v>27</v>
       </c>
       <c r="E185" s="11">
-        <v>30</v>
+        <v>18</v>
       </c>
       <c r="F185" s="9" t="s">
         <v>28</v>
@@ -6229,7 +6229,7 @@
         <v>27</v>
       </c>
       <c r="E186" s="11">
-        <v>25</v>
+        <v>20</v>
       </c>
       <c r="F186" s="9" t="s">
         <v>28</v>
@@ -6252,7 +6252,7 @@
         <v>27</v>
       </c>
       <c r="E187" s="11">
-        <v>24</v>
+        <v>26</v>
       </c>
       <c r="F187" s="9" t="s">
         <v>28</v>
@@ -6275,7 +6275,7 @@
         <v>27</v>
       </c>
       <c r="E188" s="11">
-        <v>24</v>
+        <v>14</v>
       </c>
       <c r="F188" s="9" t="s">
         <v>28</v>
@@ -6298,7 +6298,7 @@
         <v>27</v>
       </c>
       <c r="E189" s="11">
-        <v>30</v>
+        <v>23</v>
       </c>
       <c r="F189" s="9" t="s">
         <v>28</v>
@@ -6321,7 +6321,7 @@
         <v>27</v>
       </c>
       <c r="E190" s="11">
-        <v>14</v>
+        <v>17</v>
       </c>
       <c r="F190" s="9" t="s">
         <v>28</v>
@@ -6344,7 +6344,7 @@
         <v>27</v>
       </c>
       <c r="E191" s="11">
-        <v>21</v>
+        <v>8</v>
       </c>
       <c r="F191" s="9" t="s">
         <v>28</v>
@@ -6367,7 +6367,7 @@
         <v>27</v>
       </c>
       <c r="E192" s="11">
-        <v>17</v>
+        <v>28</v>
       </c>
       <c r="F192" s="9" t="s">
         <v>28</v>
@@ -6390,7 +6390,7 @@
         <v>27</v>
       </c>
       <c r="E193" s="11">
-        <v>11</v>
+        <v>26</v>
       </c>
       <c r="F193" s="9" t="s">
         <v>28</v>
@@ -6413,7 +6413,7 @@
         <v>27</v>
       </c>
       <c r="E194" s="11">
-        <v>25</v>
+        <v>15</v>
       </c>
       <c r="F194" s="9" t="s">
         <v>28</v>
@@ -6436,7 +6436,7 @@
         <v>27</v>
       </c>
       <c r="E195" s="11">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="F195" s="9" t="s">
         <v>28</v>
@@ -6459,7 +6459,7 @@
         <v>27</v>
       </c>
       <c r="E196" s="11">
-        <v>21</v>
+        <v>14</v>
       </c>
       <c r="F196" s="9" t="s">
         <v>28</v>
@@ -6482,7 +6482,7 @@
         <v>27</v>
       </c>
       <c r="E197" s="11">
-        <v>10</v>
+        <v>26</v>
       </c>
       <c r="F197" s="9" t="s">
         <v>28</v>
@@ -6505,7 +6505,7 @@
         <v>27</v>
       </c>
       <c r="E198" s="11">
-        <v>28</v>
+        <v>17</v>
       </c>
       <c r="F198" s="9" t="s">
         <v>28</v>
@@ -6528,7 +6528,7 @@
         <v>27</v>
       </c>
       <c r="E199" s="11">
-        <v>23</v>
+        <v>29</v>
       </c>
       <c r="F199" s="9" t="s">
         <v>28</v>
@@ -6551,7 +6551,7 @@
         <v>27</v>
       </c>
       <c r="E200" s="11">
-        <v>9</v>
+        <v>13</v>
       </c>
       <c r="F200" s="9" t="s">
         <v>28</v>
@@ -6597,7 +6597,7 @@
         <v>27</v>
       </c>
       <c r="E202" s="11">
-        <v>12</v>
+        <v>23</v>
       </c>
       <c r="F202" s="9" t="s">
         <v>28</v>
@@ -6620,7 +6620,7 @@
         <v>27</v>
       </c>
       <c r="E203" s="11">
-        <v>25</v>
+        <v>30</v>
       </c>
       <c r="F203" s="9" t="s">
         <v>28</v>
@@ -6643,7 +6643,7 @@
         <v>27</v>
       </c>
       <c r="E204" s="11">
-        <v>17</v>
+        <v>8</v>
       </c>
       <c r="F204" s="9" t="s">
         <v>28</v>
@@ -6666,7 +6666,7 @@
         <v>27</v>
       </c>
       <c r="E205" s="11">
-        <v>17</v>
+        <v>11</v>
       </c>
       <c r="F205" s="9" t="s">
         <v>28</v>
@@ -6689,7 +6689,7 @@
         <v>27</v>
       </c>
       <c r="E206" s="11">
-        <v>13</v>
+        <v>25</v>
       </c>
       <c r="F206" s="9" t="s">
         <v>28</v>
@@ -6712,7 +6712,7 @@
         <v>27</v>
       </c>
       <c r="E207" s="11">
-        <v>26</v>
+        <v>21</v>
       </c>
       <c r="F207" s="9" t="s">
         <v>28</v>
@@ -6735,7 +6735,7 @@
         <v>27</v>
       </c>
       <c r="E208" s="11">
-        <v>27</v>
+        <v>21</v>
       </c>
       <c r="F208" s="9" t="s">
         <v>28</v>
@@ -6758,7 +6758,7 @@
         <v>27</v>
       </c>
       <c r="E209" s="11">
-        <v>17</v>
+        <v>31</v>
       </c>
       <c r="F209" s="9" t="s">
         <v>28</v>
@@ -6781,7 +6781,7 @@
         <v>27</v>
       </c>
       <c r="E210" s="11">
-        <v>13</v>
+        <v>22</v>
       </c>
       <c r="F210" s="9" t="s">
         <v>28</v>
@@ -6804,7 +6804,7 @@
         <v>27</v>
       </c>
       <c r="E211" s="11">
-        <v>11</v>
+        <v>8</v>
       </c>
       <c r="F211" s="9" t="s">
         <v>28</v>
@@ -6827,7 +6827,7 @@
         <v>27</v>
       </c>
       <c r="E212" s="11">
-        <v>16</v>
+        <v>24</v>
       </c>
       <c r="F212" s="9" t="s">
         <v>28</v>
@@ -6850,7 +6850,7 @@
         <v>27</v>
       </c>
       <c r="E213" s="11">
-        <v>18</v>
+        <v>9</v>
       </c>
       <c r="F213" s="9" t="s">
         <v>28</v>
@@ -6873,7 +6873,7 @@
         <v>27</v>
       </c>
       <c r="E214" s="11">
-        <v>30</v>
+        <v>9</v>
       </c>
       <c r="F214" s="9" t="s">
         <v>28</v>
@@ -6896,7 +6896,7 @@
         <v>27</v>
       </c>
       <c r="E215" s="11">
-        <v>29</v>
+        <v>10</v>
       </c>
       <c r="F215" s="9" t="s">
         <v>28</v>
@@ -6919,7 +6919,7 @@
         <v>27</v>
       </c>
       <c r="E216" s="11">
-        <v>21</v>
+        <v>14</v>
       </c>
       <c r="F216" s="9" t="s">
         <v>28</v>
@@ -6942,7 +6942,7 @@
         <v>27</v>
       </c>
       <c r="E217" s="11">
-        <v>10</v>
+        <v>18</v>
       </c>
       <c r="F217" s="9" t="s">
         <v>28</v>
@@ -6965,7 +6965,7 @@
         <v>27</v>
       </c>
       <c r="E218" s="11">
-        <v>8</v>
+        <v>13</v>
       </c>
       <c r="F218" s="9" t="s">
         <v>28</v>
@@ -6988,7 +6988,7 @@
         <v>27</v>
       </c>
       <c r="E219" s="11">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="F219" s="9" t="s">
         <v>28</v>
@@ -7011,7 +7011,7 @@
         <v>27</v>
       </c>
       <c r="E220" s="11">
-        <v>25</v>
+        <v>14</v>
       </c>
       <c r="F220" s="9" t="s">
         <v>28</v>
@@ -7034,7 +7034,7 @@
         <v>27</v>
       </c>
       <c r="E221" s="11">
-        <v>30</v>
+        <v>8</v>
       </c>
       <c r="F221" s="9" t="s">
         <v>28</v>
@@ -7057,7 +7057,7 @@
         <v>27</v>
       </c>
       <c r="E222" s="11">
-        <v>18</v>
+        <v>26</v>
       </c>
       <c r="F222" s="9" t="s">
         <v>28</v>
@@ -7080,7 +7080,7 @@
         <v>27</v>
       </c>
       <c r="E223" s="11">
-        <v>30</v>
+        <v>25</v>
       </c>
       <c r="F223" s="9" t="s">
         <v>28</v>
@@ -7103,7 +7103,7 @@
         <v>27</v>
       </c>
       <c r="E224" s="11">
-        <v>10</v>
+        <v>25</v>
       </c>
       <c r="F224" s="9" t="s">
         <v>28</v>
@@ -7149,7 +7149,7 @@
         <v>27</v>
       </c>
       <c r="E226" s="11">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="F226" s="9" t="s">
         <v>28</v>
@@ -7172,7 +7172,7 @@
         <v>27</v>
       </c>
       <c r="E227" s="11">
-        <v>14</v>
+        <v>26</v>
       </c>
       <c r="F227" s="9" t="s">
         <v>28</v>
@@ -7195,7 +7195,7 @@
         <v>27</v>
       </c>
       <c r="E228" s="11">
-        <v>28</v>
+        <v>18</v>
       </c>
       <c r="F228" s="9" t="s">
         <v>28</v>
@@ -7218,7 +7218,7 @@
         <v>27</v>
       </c>
       <c r="E229" s="11">
-        <v>9</v>
+        <v>18</v>
       </c>
       <c r="F229" s="9" t="s">
         <v>28</v>
@@ -7241,7 +7241,7 @@
         <v>27</v>
       </c>
       <c r="E230" s="11">
-        <v>16</v>
+        <v>8</v>
       </c>
       <c r="F230" s="9" t="s">
         <v>28</v>
@@ -7264,7 +7264,7 @@
         <v>27</v>
       </c>
       <c r="E231" s="11">
-        <v>11</v>
+        <v>21</v>
       </c>
       <c r="F231" s="9" t="s">
         <v>28</v>
@@ -7287,7 +7287,7 @@
         <v>27</v>
       </c>
       <c r="E232" s="11">
-        <v>22</v>
+        <v>10</v>
       </c>
       <c r="F232" s="9" t="s">
         <v>28</v>
@@ -7310,7 +7310,7 @@
         <v>27</v>
       </c>
       <c r="E233" s="11">
-        <v>9</v>
+        <v>14</v>
       </c>
       <c r="F233" s="9" t="s">
         <v>28</v>
@@ -7333,7 +7333,7 @@
         <v>27</v>
       </c>
       <c r="E234" s="11">
-        <v>24</v>
+        <v>11</v>
       </c>
       <c r="F234" s="9" t="s">
         <v>28</v>
@@ -7356,7 +7356,7 @@
         <v>27</v>
       </c>
       <c r="E235" s="11">
-        <v>26</v>
+        <v>11</v>
       </c>
       <c r="F235" s="9" t="s">
         <v>28</v>
@@ -7379,7 +7379,7 @@
         <v>27</v>
       </c>
       <c r="E236" s="11">
-        <v>29</v>
+        <v>15</v>
       </c>
       <c r="F236" s="9" t="s">
         <v>28</v>
@@ -7402,7 +7402,7 @@
         <v>27</v>
       </c>
       <c r="E237" s="11">
-        <v>17</v>
+        <v>13</v>
       </c>
       <c r="F237" s="9" t="s">
         <v>28</v>
@@ -7425,7 +7425,7 @@
         <v>27</v>
       </c>
       <c r="E238" s="11">
-        <v>26</v>
+        <v>9</v>
       </c>
       <c r="F238" s="9" t="s">
         <v>28</v>
@@ -7448,7 +7448,7 @@
         <v>27</v>
       </c>
       <c r="E239" s="11">
-        <v>31</v>
+        <v>23</v>
       </c>
       <c r="F239" s="9" t="s">
         <v>28</v>
@@ -7471,7 +7471,7 @@
         <v>27</v>
       </c>
       <c r="E240" s="11">
-        <v>24</v>
+        <v>12</v>
       </c>
       <c r="F240" s="9" t="s">
         <v>28</v>
@@ -7494,7 +7494,7 @@
         <v>27</v>
       </c>
       <c r="E241" s="11">
-        <v>31</v>
+        <v>10</v>
       </c>
       <c r="F241" s="9" t="s">
         <v>28</v>
@@ -7517,7 +7517,7 @@
         <v>27</v>
       </c>
       <c r="E242" s="11">
-        <v>20</v>
+        <v>29</v>
       </c>
       <c r="F242" s="9" t="s">
         <v>28</v>
@@ -7540,7 +7540,7 @@
         <v>27</v>
       </c>
       <c r="E243" s="11">
-        <v>20</v>
+        <v>13</v>
       </c>
       <c r="F243" s="9" t="s">
         <v>28</v>
@@ -7563,7 +7563,7 @@
         <v>27</v>
       </c>
       <c r="E244" s="11">
-        <v>8</v>
+        <v>28</v>
       </c>
       <c r="F244" s="9" t="s">
         <v>28</v>
@@ -7586,7 +7586,7 @@
         <v>27</v>
       </c>
       <c r="E245" s="11">
-        <v>12</v>
+        <v>20</v>
       </c>
       <c r="F245" s="9" t="s">
         <v>28</v>
@@ -7609,7 +7609,7 @@
         <v>27</v>
       </c>
       <c r="E246" s="11">
-        <v>14</v>
+        <v>23</v>
       </c>
       <c r="F246" s="9" t="s">
         <v>28</v>
@@ -7632,7 +7632,7 @@
         <v>27</v>
       </c>
       <c r="E247" s="11">
-        <v>29</v>
+        <v>22</v>
       </c>
       <c r="F247" s="9" t="s">
         <v>28</v>
@@ -7655,7 +7655,7 @@
         <v>27</v>
       </c>
       <c r="E248" s="11">
-        <v>21</v>
+        <v>18</v>
       </c>
       <c r="F248" s="9" t="s">
         <v>28</v>
@@ -7678,7 +7678,7 @@
         <v>27</v>
       </c>
       <c r="E249" s="11">
-        <v>24</v>
+        <v>11</v>
       </c>
       <c r="F249" s="9" t="s">
         <v>28</v>
@@ -7701,7 +7701,7 @@
         <v>27</v>
       </c>
       <c r="E250" s="11">
-        <v>13</v>
+        <v>15</v>
       </c>
       <c r="F250" s="9" t="s">
         <v>28</v>
@@ -7724,7 +7724,7 @@
         <v>27</v>
       </c>
       <c r="E251" s="11">
-        <v>12</v>
+        <v>18</v>
       </c>
       <c r="F251" s="9" t="s">
         <v>28</v>
@@ -7747,7 +7747,7 @@
         <v>27</v>
       </c>
       <c r="E252" s="11">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="F252" s="9" t="s">
         <v>28</v>
@@ -7770,7 +7770,7 @@
         <v>27</v>
       </c>
       <c r="E253" s="11">
-        <v>27</v>
+        <v>25</v>
       </c>
       <c r="F253" s="9" t="s">
         <v>28</v>
@@ -7793,7 +7793,7 @@
         <v>27</v>
       </c>
       <c r="E254" s="11">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="F254" s="9" t="s">
         <v>28</v>
@@ -7816,7 +7816,7 @@
         <v>27</v>
       </c>
       <c r="E255" s="11">
-        <v>22</v>
+        <v>30</v>
       </c>
       <c r="F255" s="9" t="s">
         <v>28</v>
@@ -7839,7 +7839,7 @@
         <v>27</v>
       </c>
       <c r="E256" s="11">
-        <v>31</v>
+        <v>21</v>
       </c>
       <c r="F256" s="9" t="s">
         <v>28</v>
@@ -7862,7 +7862,7 @@
         <v>27</v>
       </c>
       <c r="E257" s="11">
-        <v>30</v>
+        <v>14</v>
       </c>
       <c r="F257" s="9" t="s">
         <v>28</v>
@@ -7885,7 +7885,7 @@
         <v>27</v>
       </c>
       <c r="E258" s="11">
-        <v>16</v>
+        <v>18</v>
       </c>
       <c r="F258" s="9" t="s">
         <v>28</v>
@@ -7908,7 +7908,7 @@
         <v>27</v>
       </c>
       <c r="E259" s="11">
-        <v>18</v>
+        <v>26</v>
       </c>
       <c r="F259" s="9" t="s">
         <v>28</v>
@@ -7931,7 +7931,7 @@
         <v>27</v>
       </c>
       <c r="E260" s="11">
-        <v>24</v>
+        <v>10</v>
       </c>
       <c r="F260" s="9" t="s">
         <v>28</v>
@@ -7954,7 +7954,7 @@
         <v>27</v>
       </c>
       <c r="E261" s="11">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="F261" s="9" t="s">
         <v>28</v>
@@ -7977,7 +7977,7 @@
         <v>27</v>
       </c>
       <c r="E262" s="11">
-        <v>24</v>
+        <v>26</v>
       </c>
       <c r="F262" s="9" t="s">
         <v>28</v>
@@ -8000,7 +8000,7 @@
         <v>27</v>
       </c>
       <c r="E263" s="11">
-        <v>28</v>
+        <v>12</v>
       </c>
       <c r="F263" s="9" t="s">
         <v>28</v>
@@ -8023,7 +8023,7 @@
         <v>27</v>
       </c>
       <c r="E264" s="11">
-        <v>23</v>
+        <v>14</v>
       </c>
       <c r="F264" s="9" t="s">
         <v>28</v>
@@ -8046,7 +8046,7 @@
         <v>27</v>
       </c>
       <c r="E265" s="11">
-        <v>29</v>
+        <v>12</v>
       </c>
       <c r="F265" s="9" t="s">
         <v>28</v>
@@ -8069,7 +8069,7 @@
         <v>27</v>
       </c>
       <c r="E266" s="11">
-        <v>13</v>
+        <v>20</v>
       </c>
       <c r="F266" s="9" t="s">
         <v>28</v>
@@ -8092,7 +8092,7 @@
         <v>27</v>
       </c>
       <c r="E267" s="11">
-        <v>14</v>
+        <v>31</v>
       </c>
       <c r="F267" s="9" t="s">
         <v>28</v>
@@ -8115,7 +8115,7 @@
         <v>27</v>
       </c>
       <c r="E268" s="11">
-        <v>13</v>
+        <v>17</v>
       </c>
       <c r="F268" s="9" t="s">
         <v>28</v>
@@ -8138,7 +8138,7 @@
         <v>27</v>
       </c>
       <c r="E269" s="11">
-        <v>16</v>
+        <v>21</v>
       </c>
       <c r="F269" s="9" t="s">
         <v>28</v>
@@ -8161,7 +8161,7 @@
         <v>27</v>
       </c>
       <c r="E270" s="11">
-        <v>20</v>
+        <v>13</v>
       </c>
       <c r="F270" s="9" t="s">
         <v>28</v>
@@ -8184,7 +8184,7 @@
         <v>27</v>
       </c>
       <c r="E271" s="11">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="F271" s="9" t="s">
         <v>28</v>
@@ -8207,7 +8207,7 @@
         <v>27</v>
       </c>
       <c r="E272" s="11">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="F272" s="9" t="s">
         <v>28</v>
@@ -8230,7 +8230,7 @@
         <v>27</v>
       </c>
       <c r="E273" s="11">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="F273" s="9" t="s">
         <v>28</v>
@@ -8253,7 +8253,7 @@
         <v>27</v>
       </c>
       <c r="E274" s="11">
-        <v>28</v>
+        <v>11</v>
       </c>
       <c r="F274" s="9" t="s">
         <v>28</v>
@@ -8276,7 +8276,7 @@
         <v>27</v>
       </c>
       <c r="E275" s="11">
-        <v>22</v>
+        <v>14</v>
       </c>
       <c r="F275" s="9" t="s">
         <v>28</v>
@@ -8299,7 +8299,7 @@
         <v>27</v>
       </c>
       <c r="E276" s="11">
-        <v>12</v>
+        <v>9</v>
       </c>
       <c r="F276" s="9" t="s">
         <v>28</v>
@@ -8322,7 +8322,7 @@
         <v>27</v>
       </c>
       <c r="E277" s="11">
-        <v>17</v>
+        <v>26</v>
       </c>
       <c r="F277" s="9" t="s">
         <v>28</v>
@@ -8345,7 +8345,7 @@
         <v>27</v>
       </c>
       <c r="E278" s="11">
-        <v>22</v>
+        <v>28</v>
       </c>
       <c r="F278" s="9" t="s">
         <v>28</v>
@@ -8368,7 +8368,7 @@
         <v>27</v>
       </c>
       <c r="E279" s="11">
-        <v>15</v>
+        <v>27</v>
       </c>
       <c r="F279" s="9" t="s">
         <v>28</v>
@@ -8391,7 +8391,7 @@
         <v>27</v>
       </c>
       <c r="E280" s="11">
-        <v>18</v>
+        <v>26</v>
       </c>
       <c r="F280" s="9" t="s">
         <v>28</v>
@@ -8414,7 +8414,7 @@
         <v>27</v>
       </c>
       <c r="E281" s="11">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="F281" s="9" t="s">
         <v>28</v>
@@ -8460,7 +8460,7 @@
         <v>27</v>
       </c>
       <c r="E283" s="11">
-        <v>16</v>
+        <v>10</v>
       </c>
       <c r="F283" s="9" t="s">
         <v>28</v>
@@ -8483,7 +8483,7 @@
         <v>27</v>
       </c>
       <c r="E284" s="11">
-        <v>27</v>
+        <v>22</v>
       </c>
       <c r="F284" s="9" t="s">
         <v>28</v>
@@ -8506,7 +8506,7 @@
         <v>27</v>
       </c>
       <c r="E285" s="11">
-        <v>13</v>
+        <v>15</v>
       </c>
       <c r="F285" s="9" t="s">
         <v>28</v>
@@ -8529,7 +8529,7 @@
         <v>27</v>
       </c>
       <c r="E286" s="11">
-        <v>24</v>
+        <v>30</v>
       </c>
       <c r="F286" s="9" t="s">
         <v>28</v>
@@ -8552,7 +8552,7 @@
         <v>27</v>
       </c>
       <c r="E287" s="11">
-        <v>31</v>
+        <v>27</v>
       </c>
       <c r="F287" s="9" t="s">
         <v>28</v>
@@ -8575,7 +8575,7 @@
         <v>27</v>
       </c>
       <c r="E288" s="11">
-        <v>13</v>
+        <v>28</v>
       </c>
       <c r="F288" s="9" t="s">
         <v>28</v>
@@ -8598,7 +8598,7 @@
         <v>27</v>
       </c>
       <c r="E289" s="11">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="F289" s="9" t="s">
         <v>28</v>
@@ -8621,7 +8621,7 @@
         <v>27</v>
       </c>
       <c r="E290" s="11">
-        <v>28</v>
+        <v>20</v>
       </c>
       <c r="F290" s="9" t="s">
         <v>28</v>
@@ -8644,7 +8644,7 @@
         <v>27</v>
       </c>
       <c r="E291" s="11">
-        <v>15</v>
+        <v>29</v>
       </c>
       <c r="F291" s="9" t="s">
         <v>28</v>
@@ -8690,7 +8690,7 @@
         <v>27</v>
       </c>
       <c r="E293" s="11">
-        <v>24</v>
+        <v>26</v>
       </c>
       <c r="F293" s="9" t="s">
         <v>28</v>
@@ -8713,7 +8713,7 @@
         <v>27</v>
       </c>
       <c r="E294" s="11">
-        <v>31</v>
+        <v>9</v>
       </c>
       <c r="F294" s="9" t="s">
         <v>28</v>
@@ -8736,7 +8736,7 @@
         <v>27</v>
       </c>
       <c r="E295" s="11">
-        <v>18</v>
+        <v>20</v>
       </c>
       <c r="F295" s="9" t="s">
         <v>28</v>
@@ -8759,7 +8759,7 @@
         <v>27</v>
       </c>
       <c r="E296" s="11">
-        <v>9</v>
+        <v>31</v>
       </c>
       <c r="F296" s="9" t="s">
         <v>28</v>
@@ -8782,7 +8782,7 @@
         <v>27</v>
       </c>
       <c r="E297" s="11">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="F297" s="9" t="s">
         <v>28</v>
@@ -8805,7 +8805,7 @@
         <v>27</v>
       </c>
       <c r="E298" s="11">
-        <v>10</v>
+        <v>22</v>
       </c>
       <c r="F298" s="9" t="s">
         <v>28</v>
@@ -8828,7 +8828,7 @@
         <v>27</v>
       </c>
       <c r="E299" s="11">
-        <v>24</v>
+        <v>16</v>
       </c>
       <c r="F299" s="9" t="s">
         <v>28</v>
@@ -8851,7 +8851,7 @@
         <v>27</v>
       </c>
       <c r="E300" s="11">
-        <v>10</v>
+        <v>27</v>
       </c>
       <c r="F300" s="9" t="s">
         <v>28</v>
@@ -8874,7 +8874,7 @@
         <v>27</v>
       </c>
       <c r="E301" s="11">
-        <v>26</v>
+        <v>16</v>
       </c>
       <c r="F301" s="9" t="s">
         <v>28</v>
@@ -8897,7 +8897,7 @@
         <v>27</v>
       </c>
       <c r="E302" s="11">
-        <v>22</v>
+        <v>8</v>
       </c>
       <c r="F302" s="9" t="s">
         <v>28</v>
@@ -8920,7 +8920,7 @@
         <v>27</v>
       </c>
       <c r="E303" s="11">
-        <v>15</v>
+        <v>10</v>
       </c>
       <c r="F303" s="9" t="s">
         <v>28</v>
@@ -8943,7 +8943,7 @@
         <v>27</v>
       </c>
       <c r="E304" s="11">
-        <v>21</v>
+        <v>30</v>
       </c>
       <c r="F304" s="9" t="s">
         <v>28</v>
@@ -8966,7 +8966,7 @@
         <v>27</v>
       </c>
       <c r="E305" s="11">
-        <v>31</v>
+        <v>8</v>
       </c>
       <c r="F305" s="9" t="s">
         <v>28</v>
@@ -8989,7 +8989,7 @@
         <v>27</v>
       </c>
       <c r="E306" s="11">
-        <v>17</v>
+        <v>9</v>
       </c>
       <c r="F306" s="9" t="s">
         <v>28</v>
@@ -9012,7 +9012,7 @@
         <v>27</v>
       </c>
       <c r="E307" s="11">
-        <v>15</v>
+        <v>8</v>
       </c>
       <c r="F307" s="9" t="s">
         <v>28</v>
@@ -9035,7 +9035,7 @@
         <v>27</v>
       </c>
       <c r="E308" s="11">
-        <v>29</v>
+        <v>18</v>
       </c>
       <c r="F308" s="9" t="s">
         <v>28</v>
@@ -9058,7 +9058,7 @@
         <v>27</v>
       </c>
       <c r="E309" s="11">
-        <v>23</v>
+        <v>12</v>
       </c>
       <c r="F309" s="9" t="s">
         <v>28</v>
@@ -9081,7 +9081,7 @@
         <v>27</v>
       </c>
       <c r="E310" s="11">
-        <v>27</v>
+        <v>20</v>
       </c>
       <c r="F310" s="9" t="s">
         <v>28</v>
@@ -9104,7 +9104,7 @@
         <v>27</v>
       </c>
       <c r="E311" s="11">
-        <v>26</v>
+        <v>30</v>
       </c>
       <c r="F311" s="9" t="s">
         <v>28</v>
@@ -9127,7 +9127,7 @@
         <v>27</v>
       </c>
       <c r="E312" s="11">
-        <v>26</v>
+        <v>31</v>
       </c>
       <c r="F312" s="9" t="s">
         <v>28</v>
@@ -9150,7 +9150,7 @@
         <v>27</v>
       </c>
       <c r="E313" s="11">
-        <v>26</v>
+        <v>20</v>
       </c>
       <c r="F313" s="9" t="s">
         <v>28</v>
@@ -9173,7 +9173,7 @@
         <v>27</v>
       </c>
       <c r="E314" s="11">
-        <v>14</v>
+        <v>24</v>
       </c>
       <c r="F314" s="9" t="s">
         <v>28</v>
@@ -9196,7 +9196,7 @@
         <v>27</v>
       </c>
       <c r="E315" s="11">
-        <v>18</v>
+        <v>29</v>
       </c>
       <c r="F315" s="9" t="s">
         <v>28</v>
@@ -9219,7 +9219,7 @@
         <v>27</v>
       </c>
       <c r="E316" s="11">
-        <v>16</v>
+        <v>12</v>
       </c>
       <c r="F316" s="9" t="s">
         <v>28</v>
@@ -9242,7 +9242,7 @@
         <v>27</v>
       </c>
       <c r="E317" s="11">
-        <v>18</v>
+        <v>25</v>
       </c>
       <c r="F317" s="9" t="s">
         <v>28</v>
@@ -9265,7 +9265,7 @@
         <v>27</v>
       </c>
       <c r="E318" s="11">
-        <v>12</v>
+        <v>22</v>
       </c>
       <c r="F318" s="9" t="s">
         <v>28</v>
@@ -9288,7 +9288,7 @@
         <v>27</v>
       </c>
       <c r="E319" s="11">
-        <v>21</v>
+        <v>30</v>
       </c>
       <c r="F319" s="9" t="s">
         <v>28</v>
@@ -9311,7 +9311,7 @@
         <v>27</v>
       </c>
       <c r="E320" s="11">
-        <v>11</v>
+        <v>30</v>
       </c>
       <c r="F320" s="9" t="s">
         <v>28</v>
@@ -9334,7 +9334,7 @@
         <v>27</v>
       </c>
       <c r="E321" s="11">
-        <v>15</v>
+        <v>20</v>
       </c>
       <c r="F321" s="9" t="s">
         <v>28</v>
@@ -9357,7 +9357,7 @@
         <v>27</v>
       </c>
       <c r="E322" s="11">
-        <v>26</v>
+        <v>15</v>
       </c>
       <c r="F322" s="9" t="s">
         <v>28</v>
@@ -9380,7 +9380,7 @@
         <v>27</v>
       </c>
       <c r="E323" s="11">
-        <v>28</v>
+        <v>23</v>
       </c>
       <c r="F323" s="9" t="s">
         <v>28</v>
@@ -9403,7 +9403,7 @@
         <v>27</v>
       </c>
       <c r="E324" s="11">
-        <v>28</v>
+        <v>9</v>
       </c>
       <c r="F324" s="9" t="s">
         <v>28</v>
@@ -9426,7 +9426,7 @@
         <v>27</v>
       </c>
       <c r="E325" s="11">
-        <v>10</v>
+        <v>30</v>
       </c>
       <c r="F325" s="9" t="s">
         <v>28</v>
@@ -9449,7 +9449,7 @@
         <v>27</v>
       </c>
       <c r="E326" s="11">
-        <v>14</v>
+        <v>25</v>
       </c>
       <c r="F326" s="9" t="s">
         <v>28</v>
@@ -9472,7 +9472,7 @@
         <v>27</v>
       </c>
       <c r="E327" s="11">
-        <v>18</v>
+        <v>12</v>
       </c>
       <c r="F327" s="9" t="s">
         <v>28</v>
@@ -9518,7 +9518,7 @@
         <v>27</v>
       </c>
       <c r="E329" s="11">
-        <v>11</v>
+        <v>18</v>
       </c>
       <c r="F329" s="9" t="s">
         <v>28</v>
@@ -9541,7 +9541,7 @@
         <v>27</v>
       </c>
       <c r="E330" s="11">
-        <v>8</v>
+        <v>21</v>
       </c>
       <c r="F330" s="9" t="s">
         <v>28</v>
@@ -9564,7 +9564,7 @@
         <v>27</v>
       </c>
       <c r="E331" s="11">
-        <v>15</v>
+        <v>23</v>
       </c>
       <c r="F331" s="9" t="s">
         <v>28</v>
@@ -9587,7 +9587,7 @@
         <v>27</v>
       </c>
       <c r="E332" s="11">
-        <v>21</v>
+        <v>19</v>
       </c>
       <c r="F332" s="9" t="s">
         <v>28</v>
@@ -9610,7 +9610,7 @@
         <v>27</v>
       </c>
       <c r="E333" s="11">
-        <v>29</v>
+        <v>20</v>
       </c>
       <c r="F333" s="9" t="s">
         <v>28</v>
@@ -9656,7 +9656,7 @@
         <v>27</v>
       </c>
       <c r="E335" s="11">
-        <v>22</v>
+        <v>14</v>
       </c>
       <c r="F335" s="9" t="s">
         <v>28</v>
@@ -9679,7 +9679,7 @@
         <v>27</v>
       </c>
       <c r="E336" s="11">
-        <v>10</v>
+        <v>15</v>
       </c>
       <c r="F336" s="9" t="s">
         <v>28</v>
@@ -9702,7 +9702,7 @@
         <v>27</v>
       </c>
       <c r="E337" s="11">
-        <v>16</v>
+        <v>22</v>
       </c>
       <c r="F337" s="9" t="s">
         <v>28</v>
@@ -9725,7 +9725,7 @@
         <v>27</v>
       </c>
       <c r="E338" s="11">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="F338" s="9" t="s">
         <v>28</v>
@@ -9748,7 +9748,7 @@
         <v>27</v>
       </c>
       <c r="E339" s="11">
-        <v>12</v>
+        <v>9</v>
       </c>
       <c r="F339" s="9" t="s">
         <v>28</v>
@@ -9771,7 +9771,7 @@
         <v>27</v>
       </c>
       <c r="E340" s="11">
-        <v>11</v>
+        <v>20</v>
       </c>
       <c r="F340" s="9" t="s">
         <v>28</v>
@@ -9794,7 +9794,7 @@
         <v>27</v>
       </c>
       <c r="E341" s="11">
-        <v>25</v>
+        <v>14</v>
       </c>
       <c r="F341" s="9" t="s">
         <v>28</v>
@@ -9817,7 +9817,7 @@
         <v>27</v>
       </c>
       <c r="E342" s="11">
-        <v>11</v>
+        <v>26</v>
       </c>
       <c r="F342" s="9" t="s">
         <v>28</v>
@@ -9840,7 +9840,7 @@
         <v>27</v>
       </c>
       <c r="E343" s="11">
-        <v>28</v>
+        <v>17</v>
       </c>
       <c r="F343" s="9" t="s">
         <v>28</v>
@@ -9863,7 +9863,7 @@
         <v>27</v>
       </c>
       <c r="E344" s="11">
-        <v>17</v>
+        <v>15</v>
       </c>
       <c r="F344" s="9" t="s">
         <v>28</v>
@@ -9886,7 +9886,7 @@
         <v>27</v>
       </c>
       <c r="E345" s="11">
-        <v>19</v>
+        <v>31</v>
       </c>
       <c r="F345" s="9" t="s">
         <v>28</v>
@@ -9909,7 +9909,7 @@
         <v>27</v>
       </c>
       <c r="E346" s="11">
-        <v>31</v>
+        <v>23</v>
       </c>
       <c r="F346" s="9" t="s">
         <v>28</v>
@@ -9932,7 +9932,7 @@
         <v>27</v>
       </c>
       <c r="E347" s="11">
-        <v>12</v>
+        <v>29</v>
       </c>
       <c r="F347" s="9" t="s">
         <v>28</v>
@@ -9955,7 +9955,7 @@
         <v>27</v>
       </c>
       <c r="E348" s="11">
-        <v>30</v>
+        <v>18</v>
       </c>
       <c r="F348" s="9" t="s">
         <v>28</v>
@@ -9978,7 +9978,7 @@
         <v>27</v>
       </c>
       <c r="E349" s="11">
-        <v>26</v>
+        <v>12</v>
       </c>
       <c r="F349" s="9" t="s">
         <v>28</v>
@@ -10001,7 +10001,7 @@
         <v>27</v>
       </c>
       <c r="E350" s="11">
-        <v>26</v>
+        <v>30</v>
       </c>
       <c r="F350" s="9" t="s">
         <v>28</v>
@@ -10024,7 +10024,7 @@
         <v>27</v>
       </c>
       <c r="E351" s="11">
-        <v>28</v>
+        <v>9</v>
       </c>
       <c r="F351" s="9" t="s">
         <v>28</v>
@@ -10047,7 +10047,7 @@
         <v>27</v>
       </c>
       <c r="E352" s="11">
-        <v>25</v>
+        <v>18</v>
       </c>
       <c r="F352" s="9" t="s">
         <v>28</v>
@@ -10070,7 +10070,7 @@
         <v>27</v>
       </c>
       <c r="E353" s="11">
-        <v>27</v>
+        <v>24</v>
       </c>
       <c r="F353" s="9" t="s">
         <v>28</v>
@@ -10093,7 +10093,7 @@
         <v>27</v>
       </c>
       <c r="E354" s="11">
-        <v>30</v>
+        <v>12</v>
       </c>
       <c r="F354" s="9" t="s">
         <v>28</v>
@@ -10116,7 +10116,7 @@
         <v>27</v>
       </c>
       <c r="E355" s="11">
-        <v>25</v>
+        <v>31</v>
       </c>
       <c r="F355" s="9" t="s">
         <v>28</v>
@@ -10139,7 +10139,7 @@
         <v>27</v>
       </c>
       <c r="E356" s="11">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="F356" s="9" t="s">
         <v>28</v>
@@ -10162,7 +10162,7 @@
         <v>27</v>
       </c>
       <c r="E357" s="11">
-        <v>26</v>
+        <v>12</v>
       </c>
       <c r="F357" s="9" t="s">
         <v>28</v>
@@ -10185,7 +10185,7 @@
         <v>27</v>
       </c>
       <c r="E358" s="11">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="F358" s="9" t="s">
         <v>28</v>
@@ -10208,7 +10208,7 @@
         <v>27</v>
       </c>
       <c r="E359" s="11">
-        <v>18</v>
+        <v>9</v>
       </c>
       <c r="F359" s="9" t="s">
         <v>28</v>
@@ -10231,7 +10231,7 @@
         <v>27</v>
       </c>
       <c r="E360" s="11">
-        <v>9</v>
+        <v>26</v>
       </c>
       <c r="F360" s="9" t="s">
         <v>28</v>
@@ -10254,7 +10254,7 @@
         <v>27</v>
       </c>
       <c r="E361" s="11">
-        <v>18</v>
+        <v>22</v>
       </c>
       <c r="F361" s="9" t="s">
         <v>28</v>
@@ -10277,7 +10277,7 @@
         <v>27</v>
       </c>
       <c r="E362" s="11">
-        <v>22</v>
+        <v>19</v>
       </c>
       <c r="F362" s="9" t="s">
         <v>28</v>
@@ -10300,7 +10300,7 @@
         <v>27</v>
       </c>
       <c r="E363" s="11">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="F363" s="9" t="s">
         <v>28</v>
@@ -10323,7 +10323,7 @@
         <v>27</v>
       </c>
       <c r="E364" s="11">
-        <v>27</v>
+        <v>8</v>
       </c>
       <c r="F364" s="9" t="s">
         <v>28</v>
@@ -10346,7 +10346,7 @@
         <v>27</v>
       </c>
       <c r="E365" s="11">
-        <v>11</v>
+        <v>29</v>
       </c>
       <c r="F365" s="9" t="s">
         <v>28</v>
@@ -10369,7 +10369,7 @@
         <v>27</v>
       </c>
       <c r="E366" s="11">
-        <v>17</v>
+        <v>13</v>
       </c>
       <c r="F366" s="9" t="s">
         <v>28</v>
@@ -10392,7 +10392,7 @@
         <v>27</v>
       </c>
       <c r="E367" s="11">
-        <v>29</v>
+        <v>10</v>
       </c>
       <c r="F367" s="9" t="s">
         <v>28</v>
@@ -10415,7 +10415,7 @@
         <v>27</v>
       </c>
       <c r="E368" s="11">
-        <v>20</v>
+        <v>18</v>
       </c>
       <c r="F368" s="9" t="s">
         <v>28</v>
@@ -10438,7 +10438,7 @@
         <v>27</v>
       </c>
       <c r="E369" s="11">
-        <v>27</v>
+        <v>25</v>
       </c>
       <c r="F369" s="9" t="s">
         <v>28</v>
@@ -10461,7 +10461,7 @@
         <v>27</v>
       </c>
       <c r="E370" s="11">
-        <v>24</v>
+        <v>26</v>
       </c>
       <c r="F370" s="9" t="s">
         <v>28</v>
@@ -10484,7 +10484,7 @@
         <v>27</v>
       </c>
       <c r="E371" s="11">
-        <v>16</v>
+        <v>26</v>
       </c>
       <c r="F371" s="9" t="s">
         <v>28</v>
@@ -10507,7 +10507,7 @@
         <v>27</v>
       </c>
       <c r="E372" s="11">
-        <v>27</v>
+        <v>30</v>
       </c>
       <c r="F372" s="9" t="s">
         <v>28</v>
@@ -10553,7 +10553,7 @@
         <v>27</v>
       </c>
       <c r="E374" s="11">
-        <v>23</v>
+        <v>16</v>
       </c>
       <c r="F374" s="9" t="s">
         <v>28</v>
@@ -10576,7 +10576,7 @@
         <v>27</v>
       </c>
       <c r="E375" s="11">
-        <v>28</v>
+        <v>14</v>
       </c>
       <c r="F375" s="9" t="s">
         <v>28</v>
@@ -10599,7 +10599,7 @@
         <v>27</v>
       </c>
       <c r="E376" s="11">
-        <v>24</v>
+        <v>12</v>
       </c>
       <c r="F376" s="9" t="s">
         <v>28</v>
@@ -10622,7 +10622,7 @@
         <v>27</v>
       </c>
       <c r="E377" s="11">
-        <v>24</v>
+        <v>29</v>
       </c>
       <c r="F377" s="9" t="s">
         <v>28</v>
@@ -10645,7 +10645,7 @@
         <v>27</v>
       </c>
       <c r="E378" s="11">
-        <v>31</v>
+        <v>9</v>
       </c>
       <c r="F378" s="9" t="s">
         <v>28</v>
@@ -10668,7 +10668,7 @@
         <v>27</v>
       </c>
       <c r="E379" s="11">
-        <v>21</v>
+        <v>9</v>
       </c>
       <c r="F379" s="9" t="s">
         <v>28</v>
@@ -10691,7 +10691,7 @@
         <v>27</v>
       </c>
       <c r="E380" s="11">
-        <v>20</v>
+        <v>24</v>
       </c>
       <c r="F380" s="9" t="s">
         <v>28</v>
@@ -10714,7 +10714,7 @@
         <v>27</v>
       </c>
       <c r="E381" s="11">
-        <v>10</v>
+        <v>28</v>
       </c>
       <c r="F381" s="9" t="s">
         <v>28</v>
@@ -10737,7 +10737,7 @@
         <v>27</v>
       </c>
       <c r="E382" s="11">
-        <v>26</v>
+        <v>20</v>
       </c>
       <c r="F382" s="9" t="s">
         <v>28</v>
@@ -10760,7 +10760,7 @@
         <v>27</v>
       </c>
       <c r="E383" s="11">
-        <v>12</v>
+        <v>20</v>
       </c>
       <c r="F383" s="9" t="s">
         <v>28</v>
@@ -10783,7 +10783,7 @@
         <v>27</v>
       </c>
       <c r="E384" s="11">
-        <v>17</v>
+        <v>12</v>
       </c>
       <c r="F384" s="9" t="s">
         <v>28</v>
@@ -10806,7 +10806,7 @@
         <v>27</v>
       </c>
       <c r="E385" s="11">
-        <v>10</v>
+        <v>29</v>
       </c>
       <c r="F385" s="9" t="s">
         <v>28</v>
@@ -10829,7 +10829,7 @@
         <v>27</v>
       </c>
       <c r="E386" s="11">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="F386" s="9" t="s">
         <v>28</v>
@@ -10852,7 +10852,7 @@
         <v>27</v>
       </c>
       <c r="E387" s="11">
-        <v>8</v>
+        <v>12</v>
       </c>
       <c r="F387" s="9" t="s">
         <v>28</v>
@@ -10875,7 +10875,7 @@
         <v>27</v>
       </c>
       <c r="E388" s="11">
-        <v>19</v>
+        <v>16</v>
       </c>
       <c r="F388" s="9" t="s">
         <v>28</v>
@@ -10898,7 +10898,7 @@
         <v>27</v>
       </c>
       <c r="E389" s="11">
-        <v>17</v>
+        <v>30</v>
       </c>
       <c r="F389" s="9" t="s">
         <v>28</v>
@@ -10921,7 +10921,7 @@
         <v>27</v>
       </c>
       <c r="E390" s="11">
-        <v>16</v>
+        <v>13</v>
       </c>
       <c r="F390" s="9" t="s">
         <v>28</v>
@@ -10944,7 +10944,7 @@
         <v>27</v>
       </c>
       <c r="E391" s="11">
-        <v>12</v>
+        <v>29</v>
       </c>
       <c r="F391" s="9" t="s">
         <v>28</v>
@@ -10967,7 +10967,7 @@
         <v>27</v>
       </c>
       <c r="E392" s="11">
-        <v>24</v>
+        <v>29</v>
       </c>
       <c r="F392" s="9" t="s">
         <v>28</v>
@@ -10990,7 +10990,7 @@
         <v>27</v>
       </c>
       <c r="E393" s="11">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="F393" s="9" t="s">
         <v>28</v>
@@ -11013,7 +11013,7 @@
         <v>27</v>
       </c>
       <c r="E394" s="11">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="F394" s="9" t="s">
         <v>28</v>
@@ -11036,7 +11036,7 @@
         <v>27</v>
       </c>
       <c r="E395" s="11">
-        <v>24</v>
+        <v>22</v>
       </c>
       <c r="F395" s="9" t="s">
         <v>28</v>
@@ -11059,7 +11059,7 @@
         <v>27</v>
       </c>
       <c r="E396" s="11">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="F396" s="9" t="s">
         <v>28</v>
@@ -11082,7 +11082,7 @@
         <v>27</v>
       </c>
       <c r="E397" s="11">
-        <v>24</v>
+        <v>29</v>
       </c>
       <c r="F397" s="9" t="s">
         <v>28</v>
@@ -11105,7 +11105,7 @@
         <v>27</v>
       </c>
       <c r="E398" s="11">
-        <v>24</v>
+        <v>27</v>
       </c>
       <c r="F398" s="9" t="s">
         <v>28</v>
@@ -11128,7 +11128,7 @@
         <v>27</v>
       </c>
       <c r="E399" s="11">
-        <v>22</v>
+        <v>29</v>
       </c>
       <c r="F399" s="9" t="s">
         <v>28</v>
@@ -11151,7 +11151,7 @@
         <v>27</v>
       </c>
       <c r="E400" s="11">
-        <v>9</v>
+        <v>29</v>
       </c>
       <c r="F400" s="9" t="s">
         <v>28</v>
@@ -11174,7 +11174,7 @@
         <v>27</v>
       </c>
       <c r="E401" s="11">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="F401" s="9" t="s">
         <v>28</v>

</xml_diff>

<commit_message>
fix(theme): ensure dropdown select option background and text color have high contrast for clear visibility
</commit_message>
<xml_diff>
--- a/all-test-reports/selenium/selenium_e2e_test_report.xlsx
+++ b/all-test-reports/selenium/selenium_e2e_test_report.xlsx
@@ -35,7 +35,7 @@
     <t>Execution Date</t>
   </si>
   <si>
-    <t>28/7/2026, 11:17:39 am</t>
+    <t>28/7/2026, 11:27:59 am</t>
   </si>
   <si>
     <t>Browser / Mode</t>
@@ -98,7 +98,7 @@
     <t>PASS</t>
   </si>
   <si>
-    <t>11:17:39 am</t>
+    <t>11:27:59 am</t>
   </si>
   <si>
     <t>N/A</t>
@@ -1997,7 +1997,7 @@
         <v>27</v>
       </c>
       <c r="E2" s="11">
-        <v>8</v>
+        <v>28</v>
       </c>
       <c r="F2" s="9" t="s">
         <v>28</v>
@@ -2020,7 +2020,7 @@
         <v>27</v>
       </c>
       <c r="E3" s="11">
-        <v>30</v>
+        <v>8</v>
       </c>
       <c r="F3" s="9" t="s">
         <v>28</v>
@@ -2066,7 +2066,7 @@
         <v>27</v>
       </c>
       <c r="E5" s="11">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="F5" s="9" t="s">
         <v>28</v>
@@ -2089,7 +2089,7 @@
         <v>27</v>
       </c>
       <c r="E6" s="11">
-        <v>11</v>
+        <v>21</v>
       </c>
       <c r="F6" s="9" t="s">
         <v>28</v>
@@ -2112,7 +2112,7 @@
         <v>27</v>
       </c>
       <c r="E7" s="11">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="F7" s="9" t="s">
         <v>28</v>
@@ -2135,7 +2135,7 @@
         <v>27</v>
       </c>
       <c r="E8" s="11">
-        <v>28</v>
+        <v>17</v>
       </c>
       <c r="F8" s="9" t="s">
         <v>28</v>
@@ -2181,7 +2181,7 @@
         <v>27</v>
       </c>
       <c r="E10" s="11">
-        <v>11</v>
+        <v>8</v>
       </c>
       <c r="F10" s="9" t="s">
         <v>28</v>
@@ -2204,7 +2204,7 @@
         <v>27</v>
       </c>
       <c r="E11" s="11">
-        <v>29</v>
+        <v>25</v>
       </c>
       <c r="F11" s="9" t="s">
         <v>28</v>
@@ -2227,7 +2227,7 @@
         <v>27</v>
       </c>
       <c r="E12" s="11">
-        <v>8</v>
+        <v>31</v>
       </c>
       <c r="F12" s="9" t="s">
         <v>28</v>
@@ -2250,7 +2250,7 @@
         <v>27</v>
       </c>
       <c r="E13" s="11">
-        <v>26</v>
+        <v>9</v>
       </c>
       <c r="F13" s="9" t="s">
         <v>28</v>
@@ -2273,7 +2273,7 @@
         <v>27</v>
       </c>
       <c r="E14" s="11">
-        <v>22</v>
+        <v>19</v>
       </c>
       <c r="F14" s="9" t="s">
         <v>28</v>
@@ -2296,7 +2296,7 @@
         <v>27</v>
       </c>
       <c r="E15" s="11">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="F15" s="9" t="s">
         <v>28</v>
@@ -2319,7 +2319,7 @@
         <v>27</v>
       </c>
       <c r="E16" s="11">
-        <v>25</v>
+        <v>9</v>
       </c>
       <c r="F16" s="9" t="s">
         <v>28</v>
@@ -2342,7 +2342,7 @@
         <v>27</v>
       </c>
       <c r="E17" s="11">
-        <v>17</v>
+        <v>28</v>
       </c>
       <c r="F17" s="9" t="s">
         <v>28</v>
@@ -2365,7 +2365,7 @@
         <v>27</v>
       </c>
       <c r="E18" s="11">
-        <v>21</v>
+        <v>14</v>
       </c>
       <c r="F18" s="9" t="s">
         <v>28</v>
@@ -2388,7 +2388,7 @@
         <v>27</v>
       </c>
       <c r="E19" s="11">
-        <v>16</v>
+        <v>12</v>
       </c>
       <c r="F19" s="9" t="s">
         <v>28</v>
@@ -2411,7 +2411,7 @@
         <v>27</v>
       </c>
       <c r="E20" s="11">
-        <v>10</v>
+        <v>23</v>
       </c>
       <c r="F20" s="9" t="s">
         <v>28</v>
@@ -2434,7 +2434,7 @@
         <v>27</v>
       </c>
       <c r="E21" s="11">
-        <v>24</v>
+        <v>21</v>
       </c>
       <c r="F21" s="9" t="s">
         <v>28</v>
@@ -2457,7 +2457,7 @@
         <v>27</v>
       </c>
       <c r="E22" s="11">
-        <v>10</v>
+        <v>21</v>
       </c>
       <c r="F22" s="9" t="s">
         <v>28</v>
@@ -2480,7 +2480,7 @@
         <v>27</v>
       </c>
       <c r="E23" s="11">
-        <v>20</v>
+        <v>14</v>
       </c>
       <c r="F23" s="9" t="s">
         <v>28</v>
@@ -2503,7 +2503,7 @@
         <v>27</v>
       </c>
       <c r="E24" s="11">
-        <v>13</v>
+        <v>31</v>
       </c>
       <c r="F24" s="9" t="s">
         <v>28</v>
@@ -2526,7 +2526,7 @@
         <v>27</v>
       </c>
       <c r="E25" s="11">
-        <v>12</v>
+        <v>23</v>
       </c>
       <c r="F25" s="9" t="s">
         <v>28</v>
@@ -2549,7 +2549,7 @@
         <v>27</v>
       </c>
       <c r="E26" s="11">
-        <v>18</v>
+        <v>15</v>
       </c>
       <c r="F26" s="9" t="s">
         <v>28</v>
@@ -2572,7 +2572,7 @@
         <v>27</v>
       </c>
       <c r="E27" s="11">
-        <v>21</v>
+        <v>19</v>
       </c>
       <c r="F27" s="9" t="s">
         <v>28</v>
@@ -2595,7 +2595,7 @@
         <v>27</v>
       </c>
       <c r="E28" s="11">
-        <v>14</v>
+        <v>29</v>
       </c>
       <c r="F28" s="9" t="s">
         <v>28</v>
@@ -2618,7 +2618,7 @@
         <v>27</v>
       </c>
       <c r="E29" s="11">
-        <v>24</v>
+        <v>19</v>
       </c>
       <c r="F29" s="9" t="s">
         <v>28</v>
@@ -2641,7 +2641,7 @@
         <v>27</v>
       </c>
       <c r="E30" s="11">
-        <v>13</v>
+        <v>22</v>
       </c>
       <c r="F30" s="9" t="s">
         <v>28</v>
@@ -2664,7 +2664,7 @@
         <v>27</v>
       </c>
       <c r="E31" s="11">
-        <v>26</v>
+        <v>10</v>
       </c>
       <c r="F31" s="9" t="s">
         <v>28</v>
@@ -2687,7 +2687,7 @@
         <v>27</v>
       </c>
       <c r="E32" s="11">
-        <v>30</v>
+        <v>18</v>
       </c>
       <c r="F32" s="9" t="s">
         <v>28</v>
@@ -2710,7 +2710,7 @@
         <v>27</v>
       </c>
       <c r="E33" s="11">
-        <v>9</v>
+        <v>11</v>
       </c>
       <c r="F33" s="9" t="s">
         <v>28</v>
@@ -2733,7 +2733,7 @@
         <v>27</v>
       </c>
       <c r="E34" s="11">
-        <v>25</v>
+        <v>21</v>
       </c>
       <c r="F34" s="9" t="s">
         <v>28</v>
@@ -2756,7 +2756,7 @@
         <v>27</v>
       </c>
       <c r="E35" s="11">
-        <v>26</v>
+        <v>29</v>
       </c>
       <c r="F35" s="9" t="s">
         <v>28</v>
@@ -2779,7 +2779,7 @@
         <v>27</v>
       </c>
       <c r="E36" s="11">
-        <v>28</v>
+        <v>23</v>
       </c>
       <c r="F36" s="9" t="s">
         <v>28</v>
@@ -2802,7 +2802,7 @@
         <v>27</v>
       </c>
       <c r="E37" s="11">
-        <v>22</v>
+        <v>10</v>
       </c>
       <c r="F37" s="9" t="s">
         <v>28</v>
@@ -2825,7 +2825,7 @@
         <v>27</v>
       </c>
       <c r="E38" s="11">
-        <v>16</v>
+        <v>26</v>
       </c>
       <c r="F38" s="9" t="s">
         <v>28</v>
@@ -2848,7 +2848,7 @@
         <v>27</v>
       </c>
       <c r="E39" s="11">
-        <v>19</v>
+        <v>11</v>
       </c>
       <c r="F39" s="9" t="s">
         <v>28</v>
@@ -2871,7 +2871,7 @@
         <v>27</v>
       </c>
       <c r="E40" s="11">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="F40" s="9" t="s">
         <v>28</v>
@@ -2894,7 +2894,7 @@
         <v>27</v>
       </c>
       <c r="E41" s="11">
-        <v>29</v>
+        <v>9</v>
       </c>
       <c r="F41" s="9" t="s">
         <v>28</v>
@@ -2917,7 +2917,7 @@
         <v>27</v>
       </c>
       <c r="E42" s="11">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="F42" s="9" t="s">
         <v>28</v>
@@ -2940,7 +2940,7 @@
         <v>27</v>
       </c>
       <c r="E43" s="11">
-        <v>10</v>
+        <v>19</v>
       </c>
       <c r="F43" s="9" t="s">
         <v>28</v>
@@ -2986,7 +2986,7 @@
         <v>27</v>
       </c>
       <c r="E45" s="11">
-        <v>20</v>
+        <v>16</v>
       </c>
       <c r="F45" s="9" t="s">
         <v>28</v>
@@ -3009,7 +3009,7 @@
         <v>27</v>
       </c>
       <c r="E46" s="11">
-        <v>9</v>
+        <v>21</v>
       </c>
       <c r="F46" s="9" t="s">
         <v>28</v>
@@ -3032,7 +3032,7 @@
         <v>27</v>
       </c>
       <c r="E47" s="11">
-        <v>15</v>
+        <v>17</v>
       </c>
       <c r="F47" s="9" t="s">
         <v>28</v>
@@ -3055,7 +3055,7 @@
         <v>27</v>
       </c>
       <c r="E48" s="11">
-        <v>12</v>
+        <v>19</v>
       </c>
       <c r="F48" s="9" t="s">
         <v>28</v>
@@ -3078,7 +3078,7 @@
         <v>27</v>
       </c>
       <c r="E49" s="11">
-        <v>23</v>
+        <v>8</v>
       </c>
       <c r="F49" s="9" t="s">
         <v>28</v>
@@ -3101,7 +3101,7 @@
         <v>27</v>
       </c>
       <c r="E50" s="11">
-        <v>9</v>
+        <v>15</v>
       </c>
       <c r="F50" s="9" t="s">
         <v>28</v>
@@ -3124,7 +3124,7 @@
         <v>27</v>
       </c>
       <c r="E51" s="11">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="F51" s="9" t="s">
         <v>28</v>
@@ -3147,7 +3147,7 @@
         <v>27</v>
       </c>
       <c r="E52" s="11">
-        <v>9</v>
+        <v>19</v>
       </c>
       <c r="F52" s="9" t="s">
         <v>28</v>
@@ -3170,7 +3170,7 @@
         <v>27</v>
       </c>
       <c r="E53" s="11">
-        <v>14</v>
+        <v>20</v>
       </c>
       <c r="F53" s="9" t="s">
         <v>28</v>
@@ -3193,7 +3193,7 @@
         <v>27</v>
       </c>
       <c r="E54" s="11">
-        <v>10</v>
+        <v>20</v>
       </c>
       <c r="F54" s="9" t="s">
         <v>28</v>
@@ -3216,7 +3216,7 @@
         <v>27</v>
       </c>
       <c r="E55" s="11">
-        <v>24</v>
+        <v>29</v>
       </c>
       <c r="F55" s="9" t="s">
         <v>28</v>
@@ -3239,7 +3239,7 @@
         <v>27</v>
       </c>
       <c r="E56" s="11">
-        <v>11</v>
+        <v>8</v>
       </c>
       <c r="F56" s="9" t="s">
         <v>28</v>
@@ -3262,7 +3262,7 @@
         <v>27</v>
       </c>
       <c r="E57" s="11">
-        <v>30</v>
+        <v>16</v>
       </c>
       <c r="F57" s="9" t="s">
         <v>28</v>
@@ -3285,7 +3285,7 @@
         <v>27</v>
       </c>
       <c r="E58" s="11">
-        <v>11</v>
+        <v>9</v>
       </c>
       <c r="F58" s="9" t="s">
         <v>28</v>
@@ -3308,7 +3308,7 @@
         <v>27</v>
       </c>
       <c r="E59" s="11">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="F59" s="9" t="s">
         <v>28</v>
@@ -3331,7 +3331,7 @@
         <v>27</v>
       </c>
       <c r="E60" s="11">
-        <v>9</v>
+        <v>30</v>
       </c>
       <c r="F60" s="9" t="s">
         <v>28</v>
@@ -3354,7 +3354,7 @@
         <v>27</v>
       </c>
       <c r="E61" s="11">
-        <v>25</v>
+        <v>18</v>
       </c>
       <c r="F61" s="9" t="s">
         <v>28</v>
@@ -3377,7 +3377,7 @@
         <v>27</v>
       </c>
       <c r="E62" s="11">
-        <v>28</v>
+        <v>23</v>
       </c>
       <c r="F62" s="9" t="s">
         <v>28</v>
@@ -3400,7 +3400,7 @@
         <v>27</v>
       </c>
       <c r="E63" s="11">
-        <v>13</v>
+        <v>8</v>
       </c>
       <c r="F63" s="9" t="s">
         <v>28</v>
@@ -3446,7 +3446,7 @@
         <v>27</v>
       </c>
       <c r="E65" s="11">
-        <v>19</v>
+        <v>9</v>
       </c>
       <c r="F65" s="9" t="s">
         <v>28</v>
@@ -3469,7 +3469,7 @@
         <v>27</v>
       </c>
       <c r="E66" s="11">
-        <v>8</v>
+        <v>23</v>
       </c>
       <c r="F66" s="9" t="s">
         <v>28</v>
@@ -3492,7 +3492,7 @@
         <v>27</v>
       </c>
       <c r="E67" s="11">
-        <v>12</v>
+        <v>10</v>
       </c>
       <c r="F67" s="9" t="s">
         <v>28</v>
@@ -3515,7 +3515,7 @@
         <v>27</v>
       </c>
       <c r="E68" s="11">
-        <v>22</v>
+        <v>12</v>
       </c>
       <c r="F68" s="9" t="s">
         <v>28</v>
@@ -3538,7 +3538,7 @@
         <v>27</v>
       </c>
       <c r="E69" s="11">
-        <v>16</v>
+        <v>12</v>
       </c>
       <c r="F69" s="9" t="s">
         <v>28</v>
@@ -3561,7 +3561,7 @@
         <v>27</v>
       </c>
       <c r="E70" s="11">
-        <v>12</v>
+        <v>20</v>
       </c>
       <c r="F70" s="9" t="s">
         <v>28</v>
@@ -3584,7 +3584,7 @@
         <v>27</v>
       </c>
       <c r="E71" s="11">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="F71" s="9" t="s">
         <v>28</v>
@@ -3607,7 +3607,7 @@
         <v>27</v>
       </c>
       <c r="E72" s="11">
-        <v>10</v>
+        <v>22</v>
       </c>
       <c r="F72" s="9" t="s">
         <v>28</v>
@@ -3676,7 +3676,7 @@
         <v>27</v>
       </c>
       <c r="E75" s="11">
-        <v>24</v>
+        <v>14</v>
       </c>
       <c r="F75" s="9" t="s">
         <v>28</v>
@@ -3699,7 +3699,7 @@
         <v>27</v>
       </c>
       <c r="E76" s="11">
-        <v>16</v>
+        <v>9</v>
       </c>
       <c r="F76" s="9" t="s">
         <v>28</v>
@@ -3722,7 +3722,7 @@
         <v>27</v>
       </c>
       <c r="E77" s="11">
-        <v>19</v>
+        <v>24</v>
       </c>
       <c r="F77" s="9" t="s">
         <v>28</v>
@@ -3745,7 +3745,7 @@
         <v>27</v>
       </c>
       <c r="E78" s="11">
-        <v>14</v>
+        <v>16</v>
       </c>
       <c r="F78" s="9" t="s">
         <v>28</v>
@@ -3768,7 +3768,7 @@
         <v>27</v>
       </c>
       <c r="E79" s="11">
-        <v>19</v>
+        <v>14</v>
       </c>
       <c r="F79" s="9" t="s">
         <v>28</v>
@@ -3791,7 +3791,7 @@
         <v>27</v>
       </c>
       <c r="E80" s="11">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="F80" s="9" t="s">
         <v>28</v>
@@ -3814,7 +3814,7 @@
         <v>27</v>
       </c>
       <c r="E81" s="11">
-        <v>11</v>
+        <v>13</v>
       </c>
       <c r="F81" s="9" t="s">
         <v>28</v>
@@ -3837,7 +3837,7 @@
         <v>27</v>
       </c>
       <c r="E82" s="11">
-        <v>24</v>
+        <v>9</v>
       </c>
       <c r="F82" s="9" t="s">
         <v>28</v>
@@ -3860,7 +3860,7 @@
         <v>27</v>
       </c>
       <c r="E83" s="11">
-        <v>19</v>
+        <v>17</v>
       </c>
       <c r="F83" s="9" t="s">
         <v>28</v>
@@ -3883,7 +3883,7 @@
         <v>27</v>
       </c>
       <c r="E84" s="11">
-        <v>29</v>
+        <v>10</v>
       </c>
       <c r="F84" s="9" t="s">
         <v>28</v>
@@ -3906,7 +3906,7 @@
         <v>27</v>
       </c>
       <c r="E85" s="11">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="F85" s="9" t="s">
         <v>28</v>
@@ -3952,7 +3952,7 @@
         <v>27</v>
       </c>
       <c r="E87" s="11">
-        <v>23</v>
+        <v>8</v>
       </c>
       <c r="F87" s="9" t="s">
         <v>28</v>
@@ -3975,7 +3975,7 @@
         <v>27</v>
       </c>
       <c r="E88" s="11">
-        <v>19</v>
+        <v>12</v>
       </c>
       <c r="F88" s="9" t="s">
         <v>28</v>
@@ -3998,7 +3998,7 @@
         <v>27</v>
       </c>
       <c r="E89" s="11">
-        <v>18</v>
+        <v>11</v>
       </c>
       <c r="F89" s="9" t="s">
         <v>28</v>
@@ -4021,7 +4021,7 @@
         <v>27</v>
       </c>
       <c r="E90" s="11">
-        <v>24</v>
+        <v>20</v>
       </c>
       <c r="F90" s="9" t="s">
         <v>28</v>
@@ -4044,7 +4044,7 @@
         <v>27</v>
       </c>
       <c r="E91" s="11">
-        <v>30</v>
+        <v>20</v>
       </c>
       <c r="F91" s="9" t="s">
         <v>28</v>
@@ -4067,7 +4067,7 @@
         <v>27</v>
       </c>
       <c r="E92" s="11">
-        <v>8</v>
+        <v>31</v>
       </c>
       <c r="F92" s="9" t="s">
         <v>28</v>
@@ -4090,7 +4090,7 @@
         <v>27</v>
       </c>
       <c r="E93" s="11">
-        <v>15</v>
+        <v>11</v>
       </c>
       <c r="F93" s="9" t="s">
         <v>28</v>
@@ -4113,7 +4113,7 @@
         <v>27</v>
       </c>
       <c r="E94" s="11">
-        <v>24</v>
+        <v>8</v>
       </c>
       <c r="F94" s="9" t="s">
         <v>28</v>
@@ -4136,7 +4136,7 @@
         <v>27</v>
       </c>
       <c r="E95" s="11">
-        <v>21</v>
+        <v>18</v>
       </c>
       <c r="F95" s="9" t="s">
         <v>28</v>
@@ -4159,7 +4159,7 @@
         <v>27</v>
       </c>
       <c r="E96" s="11">
-        <v>18</v>
+        <v>15</v>
       </c>
       <c r="F96" s="9" t="s">
         <v>28</v>
@@ -4182,7 +4182,7 @@
         <v>27</v>
       </c>
       <c r="E97" s="11">
-        <v>25</v>
+        <v>28</v>
       </c>
       <c r="F97" s="9" t="s">
         <v>28</v>
@@ -4205,7 +4205,7 @@
         <v>27</v>
       </c>
       <c r="E98" s="11">
-        <v>22</v>
+        <v>12</v>
       </c>
       <c r="F98" s="9" t="s">
         <v>28</v>
@@ -4251,7 +4251,7 @@
         <v>27</v>
       </c>
       <c r="E100" s="11">
-        <v>28</v>
+        <v>16</v>
       </c>
       <c r="F100" s="9" t="s">
         <v>28</v>
@@ -4297,7 +4297,7 @@
         <v>27</v>
       </c>
       <c r="E102" s="11">
-        <v>29</v>
+        <v>24</v>
       </c>
       <c r="F102" s="9" t="s">
         <v>28</v>
@@ -4320,7 +4320,7 @@
         <v>27</v>
       </c>
       <c r="E103" s="11">
-        <v>18</v>
+        <v>10</v>
       </c>
       <c r="F103" s="9" t="s">
         <v>28</v>
@@ -4343,7 +4343,7 @@
         <v>27</v>
       </c>
       <c r="E104" s="11">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="F104" s="9" t="s">
         <v>28</v>
@@ -4366,7 +4366,7 @@
         <v>27</v>
       </c>
       <c r="E105" s="11">
-        <v>10</v>
+        <v>26</v>
       </c>
       <c r="F105" s="9" t="s">
         <v>28</v>
@@ -4389,7 +4389,7 @@
         <v>27</v>
       </c>
       <c r="E106" s="11">
-        <v>9</v>
+        <v>21</v>
       </c>
       <c r="F106" s="9" t="s">
         <v>28</v>
@@ -4412,7 +4412,7 @@
         <v>27</v>
       </c>
       <c r="E107" s="11">
-        <v>23</v>
+        <v>16</v>
       </c>
       <c r="F107" s="9" t="s">
         <v>28</v>
@@ -4435,7 +4435,7 @@
         <v>27</v>
       </c>
       <c r="E108" s="11">
-        <v>14</v>
+        <v>26</v>
       </c>
       <c r="F108" s="9" t="s">
         <v>28</v>
@@ -4458,7 +4458,7 @@
         <v>27</v>
       </c>
       <c r="E109" s="11">
-        <v>21</v>
+        <v>9</v>
       </c>
       <c r="F109" s="9" t="s">
         <v>28</v>
@@ -4481,7 +4481,7 @@
         <v>27</v>
       </c>
       <c r="E110" s="11">
-        <v>17</v>
+        <v>8</v>
       </c>
       <c r="F110" s="9" t="s">
         <v>28</v>
@@ -4504,7 +4504,7 @@
         <v>27</v>
       </c>
       <c r="E111" s="11">
-        <v>17</v>
+        <v>20</v>
       </c>
       <c r="F111" s="9" t="s">
         <v>28</v>
@@ -4527,7 +4527,7 @@
         <v>27</v>
       </c>
       <c r="E112" s="11">
-        <v>26</v>
+        <v>12</v>
       </c>
       <c r="F112" s="9" t="s">
         <v>28</v>
@@ -4550,7 +4550,7 @@
         <v>27</v>
       </c>
       <c r="E113" s="11">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="F113" s="9" t="s">
         <v>28</v>
@@ -4573,7 +4573,7 @@
         <v>27</v>
       </c>
       <c r="E114" s="11">
-        <v>10</v>
+        <v>18</v>
       </c>
       <c r="F114" s="9" t="s">
         <v>28</v>
@@ -4596,7 +4596,7 @@
         <v>27</v>
       </c>
       <c r="E115" s="11">
-        <v>17</v>
+        <v>19</v>
       </c>
       <c r="F115" s="9" t="s">
         <v>28</v>
@@ -4619,7 +4619,7 @@
         <v>27</v>
       </c>
       <c r="E116" s="11">
-        <v>31</v>
+        <v>21</v>
       </c>
       <c r="F116" s="9" t="s">
         <v>28</v>
@@ -4642,7 +4642,7 @@
         <v>27</v>
       </c>
       <c r="E117" s="11">
-        <v>17</v>
+        <v>25</v>
       </c>
       <c r="F117" s="9" t="s">
         <v>28</v>
@@ -4665,7 +4665,7 @@
         <v>27</v>
       </c>
       <c r="E118" s="11">
-        <v>17</v>
+        <v>21</v>
       </c>
       <c r="F118" s="9" t="s">
         <v>28</v>
@@ -4688,7 +4688,7 @@
         <v>27</v>
       </c>
       <c r="E119" s="11">
-        <v>26</v>
+        <v>28</v>
       </c>
       <c r="F119" s="9" t="s">
         <v>28</v>
@@ -4711,7 +4711,7 @@
         <v>27</v>
       </c>
       <c r="E120" s="11">
-        <v>9</v>
+        <v>20</v>
       </c>
       <c r="F120" s="9" t="s">
         <v>28</v>
@@ -4734,7 +4734,7 @@
         <v>27</v>
       </c>
       <c r="E121" s="11">
-        <v>29</v>
+        <v>26</v>
       </c>
       <c r="F121" s="9" t="s">
         <v>28</v>
@@ -4757,7 +4757,7 @@
         <v>27</v>
       </c>
       <c r="E122" s="11">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="F122" s="9" t="s">
         <v>28</v>
@@ -4780,7 +4780,7 @@
         <v>27</v>
       </c>
       <c r="E123" s="11">
-        <v>24</v>
+        <v>14</v>
       </c>
       <c r="F123" s="9" t="s">
         <v>28</v>
@@ -4803,7 +4803,7 @@
         <v>27</v>
       </c>
       <c r="E124" s="11">
-        <v>17</v>
+        <v>11</v>
       </c>
       <c r="F124" s="9" t="s">
         <v>28</v>
@@ -4826,7 +4826,7 @@
         <v>27</v>
       </c>
       <c r="E125" s="11">
-        <v>30</v>
+        <v>10</v>
       </c>
       <c r="F125" s="9" t="s">
         <v>28</v>
@@ -4849,7 +4849,7 @@
         <v>27</v>
       </c>
       <c r="E126" s="11">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="F126" s="9" t="s">
         <v>28</v>
@@ -4872,7 +4872,7 @@
         <v>27</v>
       </c>
       <c r="E127" s="11">
-        <v>11</v>
+        <v>24</v>
       </c>
       <c r="F127" s="9" t="s">
         <v>28</v>
@@ -4895,7 +4895,7 @@
         <v>27</v>
       </c>
       <c r="E128" s="11">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="F128" s="9" t="s">
         <v>28</v>
@@ -4918,7 +4918,7 @@
         <v>27</v>
       </c>
       <c r="E129" s="11">
-        <v>30</v>
+        <v>10</v>
       </c>
       <c r="F129" s="9" t="s">
         <v>28</v>
@@ -4941,7 +4941,7 @@
         <v>27</v>
       </c>
       <c r="E130" s="11">
-        <v>19</v>
+        <v>26</v>
       </c>
       <c r="F130" s="9" t="s">
         <v>28</v>
@@ -4964,7 +4964,7 @@
         <v>27</v>
       </c>
       <c r="E131" s="11">
-        <v>19</v>
+        <v>17</v>
       </c>
       <c r="F131" s="9" t="s">
         <v>28</v>
@@ -4987,7 +4987,7 @@
         <v>27</v>
       </c>
       <c r="E132" s="11">
-        <v>24</v>
+        <v>20</v>
       </c>
       <c r="F132" s="9" t="s">
         <v>28</v>
@@ -5010,7 +5010,7 @@
         <v>27</v>
       </c>
       <c r="E133" s="11">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="F133" s="9" t="s">
         <v>28</v>
@@ -5033,7 +5033,7 @@
         <v>27</v>
       </c>
       <c r="E134" s="11">
-        <v>22</v>
+        <v>14</v>
       </c>
       <c r="F134" s="9" t="s">
         <v>28</v>
@@ -5056,7 +5056,7 @@
         <v>27</v>
       </c>
       <c r="E135" s="11">
-        <v>27</v>
+        <v>13</v>
       </c>
       <c r="F135" s="9" t="s">
         <v>28</v>
@@ -5079,7 +5079,7 @@
         <v>27</v>
       </c>
       <c r="E136" s="11">
-        <v>30</v>
+        <v>26</v>
       </c>
       <c r="F136" s="9" t="s">
         <v>28</v>
@@ -5102,7 +5102,7 @@
         <v>27</v>
       </c>
       <c r="E137" s="11">
-        <v>23</v>
+        <v>8</v>
       </c>
       <c r="F137" s="9" t="s">
         <v>28</v>
@@ -5125,7 +5125,7 @@
         <v>27</v>
       </c>
       <c r="E138" s="11">
-        <v>28</v>
+        <v>11</v>
       </c>
       <c r="F138" s="9" t="s">
         <v>28</v>
@@ -5148,7 +5148,7 @@
         <v>27</v>
       </c>
       <c r="E139" s="11">
-        <v>26</v>
+        <v>21</v>
       </c>
       <c r="F139" s="9" t="s">
         <v>28</v>
@@ -5171,7 +5171,7 @@
         <v>27</v>
       </c>
       <c r="E140" s="11">
-        <v>22</v>
+        <v>18</v>
       </c>
       <c r="F140" s="9" t="s">
         <v>28</v>
@@ -5194,7 +5194,7 @@
         <v>27</v>
       </c>
       <c r="E141" s="11">
-        <v>23</v>
+        <v>31</v>
       </c>
       <c r="F141" s="9" t="s">
         <v>28</v>
@@ -5217,7 +5217,7 @@
         <v>27</v>
       </c>
       <c r="E142" s="11">
-        <v>20</v>
+        <v>23</v>
       </c>
       <c r="F142" s="9" t="s">
         <v>28</v>
@@ -5240,7 +5240,7 @@
         <v>27</v>
       </c>
       <c r="E143" s="11">
-        <v>11</v>
+        <v>26</v>
       </c>
       <c r="F143" s="9" t="s">
         <v>28</v>
@@ -5286,7 +5286,7 @@
         <v>27</v>
       </c>
       <c r="E145" s="11">
-        <v>8</v>
+        <v>27</v>
       </c>
       <c r="F145" s="9" t="s">
         <v>28</v>
@@ -5309,7 +5309,7 @@
         <v>27</v>
       </c>
       <c r="E146" s="11">
-        <v>18</v>
+        <v>26</v>
       </c>
       <c r="F146" s="9" t="s">
         <v>28</v>
@@ -5332,7 +5332,7 @@
         <v>27</v>
       </c>
       <c r="E147" s="11">
-        <v>9</v>
+        <v>17</v>
       </c>
       <c r="F147" s="9" t="s">
         <v>28</v>
@@ -5355,7 +5355,7 @@
         <v>27</v>
       </c>
       <c r="E148" s="11">
-        <v>11</v>
+        <v>29</v>
       </c>
       <c r="F148" s="9" t="s">
         <v>28</v>
@@ -5378,7 +5378,7 @@
         <v>27</v>
       </c>
       <c r="E149" s="11">
-        <v>12</v>
+        <v>27</v>
       </c>
       <c r="F149" s="9" t="s">
         <v>28</v>
@@ -5401,7 +5401,7 @@
         <v>27</v>
       </c>
       <c r="E150" s="11">
-        <v>14</v>
+        <v>25</v>
       </c>
       <c r="F150" s="9" t="s">
         <v>28</v>
@@ -5424,7 +5424,7 @@
         <v>27</v>
       </c>
       <c r="E151" s="11">
-        <v>29</v>
+        <v>18</v>
       </c>
       <c r="F151" s="9" t="s">
         <v>28</v>
@@ -5447,7 +5447,7 @@
         <v>27</v>
       </c>
       <c r="E152" s="11">
-        <v>16</v>
+        <v>9</v>
       </c>
       <c r="F152" s="9" t="s">
         <v>28</v>
@@ -5470,7 +5470,7 @@
         <v>27</v>
       </c>
       <c r="E153" s="11">
-        <v>13</v>
+        <v>21</v>
       </c>
       <c r="F153" s="9" t="s">
         <v>28</v>
@@ -5493,7 +5493,7 @@
         <v>27</v>
       </c>
       <c r="E154" s="11">
-        <v>27</v>
+        <v>25</v>
       </c>
       <c r="F154" s="9" t="s">
         <v>28</v>
@@ -5516,7 +5516,7 @@
         <v>27</v>
       </c>
       <c r="E155" s="11">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="F155" s="9" t="s">
         <v>28</v>
@@ -5539,7 +5539,7 @@
         <v>27</v>
       </c>
       <c r="E156" s="11">
-        <v>9</v>
+        <v>26</v>
       </c>
       <c r="F156" s="9" t="s">
         <v>28</v>
@@ -5562,7 +5562,7 @@
         <v>27</v>
       </c>
       <c r="E157" s="11">
-        <v>20</v>
+        <v>18</v>
       </c>
       <c r="F157" s="9" t="s">
         <v>28</v>
@@ -5585,7 +5585,7 @@
         <v>27</v>
       </c>
       <c r="E158" s="11">
-        <v>13</v>
+        <v>25</v>
       </c>
       <c r="F158" s="9" t="s">
         <v>28</v>
@@ -5608,7 +5608,7 @@
         <v>27</v>
       </c>
       <c r="E159" s="11">
-        <v>15</v>
+        <v>20</v>
       </c>
       <c r="F159" s="9" t="s">
         <v>28</v>
@@ -5631,7 +5631,7 @@
         <v>27</v>
       </c>
       <c r="E160" s="11">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="F160" s="9" t="s">
         <v>28</v>
@@ -5654,7 +5654,7 @@
         <v>27</v>
       </c>
       <c r="E161" s="11">
-        <v>18</v>
+        <v>10</v>
       </c>
       <c r="F161" s="9" t="s">
         <v>28</v>
@@ -5677,7 +5677,7 @@
         <v>27</v>
       </c>
       <c r="E162" s="11">
-        <v>19</v>
+        <v>23</v>
       </c>
       <c r="F162" s="9" t="s">
         <v>28</v>
@@ -5700,7 +5700,7 @@
         <v>27</v>
       </c>
       <c r="E163" s="11">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="F163" s="9" t="s">
         <v>28</v>
@@ -5723,7 +5723,7 @@
         <v>27</v>
       </c>
       <c r="E164" s="11">
-        <v>19</v>
+        <v>14</v>
       </c>
       <c r="F164" s="9" t="s">
         <v>28</v>
@@ -5746,7 +5746,7 @@
         <v>27</v>
       </c>
       <c r="E165" s="11">
-        <v>28</v>
+        <v>11</v>
       </c>
       <c r="F165" s="9" t="s">
         <v>28</v>
@@ -5769,7 +5769,7 @@
         <v>27</v>
       </c>
       <c r="E166" s="11">
-        <v>22</v>
+        <v>18</v>
       </c>
       <c r="F166" s="9" t="s">
         <v>28</v>
@@ -5792,7 +5792,7 @@
         <v>27</v>
       </c>
       <c r="E167" s="11">
-        <v>31</v>
+        <v>18</v>
       </c>
       <c r="F167" s="9" t="s">
         <v>28</v>
@@ -5815,7 +5815,7 @@
         <v>27</v>
       </c>
       <c r="E168" s="11">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="F168" s="9" t="s">
         <v>28</v>
@@ -5838,7 +5838,7 @@
         <v>27</v>
       </c>
       <c r="E169" s="11">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="F169" s="9" t="s">
         <v>28</v>
@@ -5861,7 +5861,7 @@
         <v>27</v>
       </c>
       <c r="E170" s="11">
-        <v>17</v>
+        <v>8</v>
       </c>
       <c r="F170" s="9" t="s">
         <v>28</v>
@@ -5884,7 +5884,7 @@
         <v>27</v>
       </c>
       <c r="E171" s="11">
-        <v>28</v>
+        <v>9</v>
       </c>
       <c r="F171" s="9" t="s">
         <v>28</v>
@@ -5907,7 +5907,7 @@
         <v>27</v>
       </c>
       <c r="E172" s="11">
-        <v>27</v>
+        <v>12</v>
       </c>
       <c r="F172" s="9" t="s">
         <v>28</v>
@@ -5930,7 +5930,7 @@
         <v>27</v>
       </c>
       <c r="E173" s="11">
-        <v>25</v>
+        <v>11</v>
       </c>
       <c r="F173" s="9" t="s">
         <v>28</v>
@@ -5953,7 +5953,7 @@
         <v>27</v>
       </c>
       <c r="E174" s="11">
-        <v>23</v>
+        <v>25</v>
       </c>
       <c r="F174" s="9" t="s">
         <v>28</v>
@@ -5976,7 +5976,7 @@
         <v>27</v>
       </c>
       <c r="E175" s="11">
-        <v>13</v>
+        <v>22</v>
       </c>
       <c r="F175" s="9" t="s">
         <v>28</v>
@@ -5999,7 +5999,7 @@
         <v>27</v>
       </c>
       <c r="E176" s="11">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="F176" s="9" t="s">
         <v>28</v>
@@ -6022,7 +6022,7 @@
         <v>27</v>
       </c>
       <c r="E177" s="11">
-        <v>9</v>
+        <v>30</v>
       </c>
       <c r="F177" s="9" t="s">
         <v>28</v>
@@ -6045,7 +6045,7 @@
         <v>27</v>
       </c>
       <c r="E178" s="11">
-        <v>10</v>
+        <v>19</v>
       </c>
       <c r="F178" s="9" t="s">
         <v>28</v>
@@ -6068,7 +6068,7 @@
         <v>27</v>
       </c>
       <c r="E179" s="11">
-        <v>22</v>
+        <v>29</v>
       </c>
       <c r="F179" s="9" t="s">
         <v>28</v>
@@ -6091,7 +6091,7 @@
         <v>27</v>
       </c>
       <c r="E180" s="11">
-        <v>22</v>
+        <v>14</v>
       </c>
       <c r="F180" s="9" t="s">
         <v>28</v>
@@ -6114,7 +6114,7 @@
         <v>27</v>
       </c>
       <c r="E181" s="11">
-        <v>17</v>
+        <v>19</v>
       </c>
       <c r="F181" s="9" t="s">
         <v>28</v>
@@ -6137,7 +6137,7 @@
         <v>27</v>
       </c>
       <c r="E182" s="11">
-        <v>25</v>
+        <v>13</v>
       </c>
       <c r="F182" s="9" t="s">
         <v>28</v>
@@ -6160,7 +6160,7 @@
         <v>27</v>
       </c>
       <c r="E183" s="11">
-        <v>21</v>
+        <v>23</v>
       </c>
       <c r="F183" s="9" t="s">
         <v>28</v>
@@ -6183,7 +6183,7 @@
         <v>27</v>
       </c>
       <c r="E184" s="11">
-        <v>12</v>
+        <v>26</v>
       </c>
       <c r="F184" s="9" t="s">
         <v>28</v>
@@ -6206,7 +6206,7 @@
         <v>27</v>
       </c>
       <c r="E185" s="11">
-        <v>18</v>
+        <v>21</v>
       </c>
       <c r="F185" s="9" t="s">
         <v>28</v>
@@ -6229,7 +6229,7 @@
         <v>27</v>
       </c>
       <c r="E186" s="11">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="F186" s="9" t="s">
         <v>28</v>
@@ -6252,7 +6252,7 @@
         <v>27</v>
       </c>
       <c r="E187" s="11">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="F187" s="9" t="s">
         <v>28</v>
@@ -6275,7 +6275,7 @@
         <v>27</v>
       </c>
       <c r="E188" s="11">
-        <v>14</v>
+        <v>30</v>
       </c>
       <c r="F188" s="9" t="s">
         <v>28</v>
@@ -6298,7 +6298,7 @@
         <v>27</v>
       </c>
       <c r="E189" s="11">
-        <v>23</v>
+        <v>13</v>
       </c>
       <c r="F189" s="9" t="s">
         <v>28</v>
@@ -6321,7 +6321,7 @@
         <v>27</v>
       </c>
       <c r="E190" s="11">
-        <v>17</v>
+        <v>30</v>
       </c>
       <c r="F190" s="9" t="s">
         <v>28</v>
@@ -6344,7 +6344,7 @@
         <v>27</v>
       </c>
       <c r="E191" s="11">
-        <v>8</v>
+        <v>25</v>
       </c>
       <c r="F191" s="9" t="s">
         <v>28</v>
@@ -6367,7 +6367,7 @@
         <v>27</v>
       </c>
       <c r="E192" s="11">
-        <v>28</v>
+        <v>20</v>
       </c>
       <c r="F192" s="9" t="s">
         <v>28</v>
@@ -6390,7 +6390,7 @@
         <v>27</v>
       </c>
       <c r="E193" s="11">
-        <v>26</v>
+        <v>20</v>
       </c>
       <c r="F193" s="9" t="s">
         <v>28</v>
@@ -6413,7 +6413,7 @@
         <v>27</v>
       </c>
       <c r="E194" s="11">
-        <v>15</v>
+        <v>19</v>
       </c>
       <c r="F194" s="9" t="s">
         <v>28</v>
@@ -6436,7 +6436,7 @@
         <v>27</v>
       </c>
       <c r="E195" s="11">
-        <v>18</v>
+        <v>21</v>
       </c>
       <c r="F195" s="9" t="s">
         <v>28</v>
@@ -6459,7 +6459,7 @@
         <v>27</v>
       </c>
       <c r="E196" s="11">
-        <v>14</v>
+        <v>24</v>
       </c>
       <c r="F196" s="9" t="s">
         <v>28</v>
@@ -6482,7 +6482,7 @@
         <v>27</v>
       </c>
       <c r="E197" s="11">
-        <v>26</v>
+        <v>19</v>
       </c>
       <c r="F197" s="9" t="s">
         <v>28</v>
@@ -6505,7 +6505,7 @@
         <v>27</v>
       </c>
       <c r="E198" s="11">
-        <v>17</v>
+        <v>19</v>
       </c>
       <c r="F198" s="9" t="s">
         <v>28</v>
@@ -6528,7 +6528,7 @@
         <v>27</v>
       </c>
       <c r="E199" s="11">
-        <v>29</v>
+        <v>8</v>
       </c>
       <c r="F199" s="9" t="s">
         <v>28</v>
@@ -6551,7 +6551,7 @@
         <v>27</v>
       </c>
       <c r="E200" s="11">
-        <v>13</v>
+        <v>16</v>
       </c>
       <c r="F200" s="9" t="s">
         <v>28</v>
@@ -6574,7 +6574,7 @@
         <v>27</v>
       </c>
       <c r="E201" s="11">
-        <v>22</v>
+        <v>13</v>
       </c>
       <c r="F201" s="9" t="s">
         <v>28</v>
@@ -6597,7 +6597,7 @@
         <v>27</v>
       </c>
       <c r="E202" s="11">
-        <v>23</v>
+        <v>30</v>
       </c>
       <c r="F202" s="9" t="s">
         <v>28</v>
@@ -6620,7 +6620,7 @@
         <v>27</v>
       </c>
       <c r="E203" s="11">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="F203" s="9" t="s">
         <v>28</v>
@@ -6643,7 +6643,7 @@
         <v>27</v>
       </c>
       <c r="E204" s="11">
-        <v>8</v>
+        <v>15</v>
       </c>
       <c r="F204" s="9" t="s">
         <v>28</v>
@@ -6666,7 +6666,7 @@
         <v>27</v>
       </c>
       <c r="E205" s="11">
-        <v>11</v>
+        <v>20</v>
       </c>
       <c r="F205" s="9" t="s">
         <v>28</v>
@@ -6689,7 +6689,7 @@
         <v>27</v>
       </c>
       <c r="E206" s="11">
-        <v>25</v>
+        <v>16</v>
       </c>
       <c r="F206" s="9" t="s">
         <v>28</v>
@@ -6712,7 +6712,7 @@
         <v>27</v>
       </c>
       <c r="E207" s="11">
-        <v>21</v>
+        <v>23</v>
       </c>
       <c r="F207" s="9" t="s">
         <v>28</v>
@@ -6735,7 +6735,7 @@
         <v>27</v>
       </c>
       <c r="E208" s="11">
-        <v>21</v>
+        <v>17</v>
       </c>
       <c r="F208" s="9" t="s">
         <v>28</v>
@@ -6758,7 +6758,7 @@
         <v>27</v>
       </c>
       <c r="E209" s="11">
-        <v>31</v>
+        <v>15</v>
       </c>
       <c r="F209" s="9" t="s">
         <v>28</v>
@@ -6781,7 +6781,7 @@
         <v>27</v>
       </c>
       <c r="E210" s="11">
-        <v>22</v>
+        <v>24</v>
       </c>
       <c r="F210" s="9" t="s">
         <v>28</v>
@@ -6804,7 +6804,7 @@
         <v>27</v>
       </c>
       <c r="E211" s="11">
-        <v>8</v>
+        <v>16</v>
       </c>
       <c r="F211" s="9" t="s">
         <v>28</v>
@@ -6827,7 +6827,7 @@
         <v>27</v>
       </c>
       <c r="E212" s="11">
-        <v>24</v>
+        <v>26</v>
       </c>
       <c r="F212" s="9" t="s">
         <v>28</v>
@@ -6850,7 +6850,7 @@
         <v>27</v>
       </c>
       <c r="E213" s="11">
-        <v>9</v>
+        <v>25</v>
       </c>
       <c r="F213" s="9" t="s">
         <v>28</v>
@@ -6873,7 +6873,7 @@
         <v>27</v>
       </c>
       <c r="E214" s="11">
-        <v>9</v>
+        <v>26</v>
       </c>
       <c r="F214" s="9" t="s">
         <v>28</v>
@@ -6896,7 +6896,7 @@
         <v>27</v>
       </c>
       <c r="E215" s="11">
-        <v>10</v>
+        <v>28</v>
       </c>
       <c r="F215" s="9" t="s">
         <v>28</v>
@@ -6919,7 +6919,7 @@
         <v>27</v>
       </c>
       <c r="E216" s="11">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="F216" s="9" t="s">
         <v>28</v>
@@ -6942,7 +6942,7 @@
         <v>27</v>
       </c>
       <c r="E217" s="11">
-        <v>18</v>
+        <v>24</v>
       </c>
       <c r="F217" s="9" t="s">
         <v>28</v>
@@ -6965,7 +6965,7 @@
         <v>27</v>
       </c>
       <c r="E218" s="11">
-        <v>13</v>
+        <v>25</v>
       </c>
       <c r="F218" s="9" t="s">
         <v>28</v>
@@ -6988,7 +6988,7 @@
         <v>27</v>
       </c>
       <c r="E219" s="11">
-        <v>10</v>
+        <v>22</v>
       </c>
       <c r="F219" s="9" t="s">
         <v>28</v>
@@ -7011,7 +7011,7 @@
         <v>27</v>
       </c>
       <c r="E220" s="11">
-        <v>14</v>
+        <v>23</v>
       </c>
       <c r="F220" s="9" t="s">
         <v>28</v>
@@ -7034,7 +7034,7 @@
         <v>27</v>
       </c>
       <c r="E221" s="11">
-        <v>8</v>
+        <v>23</v>
       </c>
       <c r="F221" s="9" t="s">
         <v>28</v>
@@ -7057,7 +7057,7 @@
         <v>27</v>
       </c>
       <c r="E222" s="11">
-        <v>26</v>
+        <v>8</v>
       </c>
       <c r="F222" s="9" t="s">
         <v>28</v>
@@ -7080,7 +7080,7 @@
         <v>27</v>
       </c>
       <c r="E223" s="11">
-        <v>25</v>
+        <v>27</v>
       </c>
       <c r="F223" s="9" t="s">
         <v>28</v>
@@ -7103,7 +7103,7 @@
         <v>27</v>
       </c>
       <c r="E224" s="11">
-        <v>25</v>
+        <v>14</v>
       </c>
       <c r="F224" s="9" t="s">
         <v>28</v>
@@ -7126,7 +7126,7 @@
         <v>27</v>
       </c>
       <c r="E225" s="11">
-        <v>23</v>
+        <v>17</v>
       </c>
       <c r="F225" s="9" t="s">
         <v>28</v>
@@ -7149,7 +7149,7 @@
         <v>27</v>
       </c>
       <c r="E226" s="11">
-        <v>9</v>
+        <v>30</v>
       </c>
       <c r="F226" s="9" t="s">
         <v>28</v>
@@ -7172,7 +7172,7 @@
         <v>27</v>
       </c>
       <c r="E227" s="11">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="F227" s="9" t="s">
         <v>28</v>
@@ -7195,7 +7195,7 @@
         <v>27</v>
       </c>
       <c r="E228" s="11">
-        <v>18</v>
+        <v>11</v>
       </c>
       <c r="F228" s="9" t="s">
         <v>28</v>
@@ -7218,7 +7218,7 @@
         <v>27</v>
       </c>
       <c r="E229" s="11">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="F229" s="9" t="s">
         <v>28</v>
@@ -7241,7 +7241,7 @@
         <v>27</v>
       </c>
       <c r="E230" s="11">
-        <v>8</v>
+        <v>21</v>
       </c>
       <c r="F230" s="9" t="s">
         <v>28</v>
@@ -7264,7 +7264,7 @@
         <v>27</v>
       </c>
       <c r="E231" s="11">
-        <v>21</v>
+        <v>14</v>
       </c>
       <c r="F231" s="9" t="s">
         <v>28</v>
@@ -7287,7 +7287,7 @@
         <v>27</v>
       </c>
       <c r="E232" s="11">
-        <v>10</v>
+        <v>25</v>
       </c>
       <c r="F232" s="9" t="s">
         <v>28</v>
@@ -7310,7 +7310,7 @@
         <v>27</v>
       </c>
       <c r="E233" s="11">
-        <v>14</v>
+        <v>31</v>
       </c>
       <c r="F233" s="9" t="s">
         <v>28</v>
@@ -7333,7 +7333,7 @@
         <v>27</v>
       </c>
       <c r="E234" s="11">
-        <v>11</v>
+        <v>14</v>
       </c>
       <c r="F234" s="9" t="s">
         <v>28</v>
@@ -7356,7 +7356,7 @@
         <v>27</v>
       </c>
       <c r="E235" s="11">
-        <v>11</v>
+        <v>20</v>
       </c>
       <c r="F235" s="9" t="s">
         <v>28</v>
@@ -7379,7 +7379,7 @@
         <v>27</v>
       </c>
       <c r="E236" s="11">
-        <v>15</v>
+        <v>23</v>
       </c>
       <c r="F236" s="9" t="s">
         <v>28</v>
@@ -7402,7 +7402,7 @@
         <v>27</v>
       </c>
       <c r="E237" s="11">
-        <v>13</v>
+        <v>15</v>
       </c>
       <c r="F237" s="9" t="s">
         <v>28</v>
@@ -7425,7 +7425,7 @@
         <v>27</v>
       </c>
       <c r="E238" s="11">
-        <v>9</v>
+        <v>28</v>
       </c>
       <c r="F238" s="9" t="s">
         <v>28</v>
@@ -7448,7 +7448,7 @@
         <v>27</v>
       </c>
       <c r="E239" s="11">
-        <v>23</v>
+        <v>27</v>
       </c>
       <c r="F239" s="9" t="s">
         <v>28</v>
@@ -7471,7 +7471,7 @@
         <v>27</v>
       </c>
       <c r="E240" s="11">
-        <v>12</v>
+        <v>16</v>
       </c>
       <c r="F240" s="9" t="s">
         <v>28</v>
@@ -7494,7 +7494,7 @@
         <v>27</v>
       </c>
       <c r="E241" s="11">
-        <v>10</v>
+        <v>30</v>
       </c>
       <c r="F241" s="9" t="s">
         <v>28</v>
@@ -7517,7 +7517,7 @@
         <v>27</v>
       </c>
       <c r="E242" s="11">
-        <v>29</v>
+        <v>25</v>
       </c>
       <c r="F242" s="9" t="s">
         <v>28</v>
@@ -7540,7 +7540,7 @@
         <v>27</v>
       </c>
       <c r="E243" s="11">
-        <v>13</v>
+        <v>19</v>
       </c>
       <c r="F243" s="9" t="s">
         <v>28</v>
@@ -7563,7 +7563,7 @@
         <v>27</v>
       </c>
       <c r="E244" s="11">
-        <v>28</v>
+        <v>20</v>
       </c>
       <c r="F244" s="9" t="s">
         <v>28</v>
@@ -7586,7 +7586,7 @@
         <v>27</v>
       </c>
       <c r="E245" s="11">
-        <v>20</v>
+        <v>8</v>
       </c>
       <c r="F245" s="9" t="s">
         <v>28</v>
@@ -7609,7 +7609,7 @@
         <v>27</v>
       </c>
       <c r="E246" s="11">
-        <v>23</v>
+        <v>28</v>
       </c>
       <c r="F246" s="9" t="s">
         <v>28</v>
@@ -7632,7 +7632,7 @@
         <v>27</v>
       </c>
       <c r="E247" s="11">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="F247" s="9" t="s">
         <v>28</v>
@@ -7655,7 +7655,7 @@
         <v>27</v>
       </c>
       <c r="E248" s="11">
-        <v>18</v>
+        <v>9</v>
       </c>
       <c r="F248" s="9" t="s">
         <v>28</v>
@@ -7678,7 +7678,7 @@
         <v>27</v>
       </c>
       <c r="E249" s="11">
-        <v>11</v>
+        <v>29</v>
       </c>
       <c r="F249" s="9" t="s">
         <v>28</v>
@@ -7724,7 +7724,7 @@
         <v>27</v>
       </c>
       <c r="E251" s="11">
-        <v>18</v>
+        <v>25</v>
       </c>
       <c r="F251" s="9" t="s">
         <v>28</v>
@@ -7747,7 +7747,7 @@
         <v>27</v>
       </c>
       <c r="E252" s="11">
-        <v>18</v>
+        <v>15</v>
       </c>
       <c r="F252" s="9" t="s">
         <v>28</v>
@@ -7770,7 +7770,7 @@
         <v>27</v>
       </c>
       <c r="E253" s="11">
-        <v>25</v>
+        <v>31</v>
       </c>
       <c r="F253" s="9" t="s">
         <v>28</v>
@@ -7793,7 +7793,7 @@
         <v>27</v>
       </c>
       <c r="E254" s="11">
-        <v>23</v>
+        <v>26</v>
       </c>
       <c r="F254" s="9" t="s">
         <v>28</v>
@@ -7816,7 +7816,7 @@
         <v>27</v>
       </c>
       <c r="E255" s="11">
-        <v>30</v>
+        <v>25</v>
       </c>
       <c r="F255" s="9" t="s">
         <v>28</v>
@@ -7839,7 +7839,7 @@
         <v>27</v>
       </c>
       <c r="E256" s="11">
-        <v>21</v>
+        <v>29</v>
       </c>
       <c r="F256" s="9" t="s">
         <v>28</v>
@@ -7862,7 +7862,7 @@
         <v>27</v>
       </c>
       <c r="E257" s="11">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="F257" s="9" t="s">
         <v>28</v>
@@ -7885,7 +7885,7 @@
         <v>27</v>
       </c>
       <c r="E258" s="11">
-        <v>18</v>
+        <v>31</v>
       </c>
       <c r="F258" s="9" t="s">
         <v>28</v>
@@ -7908,7 +7908,7 @@
         <v>27</v>
       </c>
       <c r="E259" s="11">
-        <v>26</v>
+        <v>24</v>
       </c>
       <c r="F259" s="9" t="s">
         <v>28</v>
@@ -7931,7 +7931,7 @@
         <v>27</v>
       </c>
       <c r="E260" s="11">
-        <v>10</v>
+        <v>15</v>
       </c>
       <c r="F260" s="9" t="s">
         <v>28</v>
@@ -7954,7 +7954,7 @@
         <v>27</v>
       </c>
       <c r="E261" s="11">
-        <v>8</v>
+        <v>31</v>
       </c>
       <c r="F261" s="9" t="s">
         <v>28</v>
@@ -7977,7 +7977,7 @@
         <v>27</v>
       </c>
       <c r="E262" s="11">
-        <v>26</v>
+        <v>9</v>
       </c>
       <c r="F262" s="9" t="s">
         <v>28</v>
@@ -8000,7 +8000,7 @@
         <v>27</v>
       </c>
       <c r="E263" s="11">
-        <v>12</v>
+        <v>26</v>
       </c>
       <c r="F263" s="9" t="s">
         <v>28</v>
@@ -8023,7 +8023,7 @@
         <v>27</v>
       </c>
       <c r="E264" s="11">
-        <v>14</v>
+        <v>29</v>
       </c>
       <c r="F264" s="9" t="s">
         <v>28</v>
@@ -8046,7 +8046,7 @@
         <v>27</v>
       </c>
       <c r="E265" s="11">
-        <v>12</v>
+        <v>28</v>
       </c>
       <c r="F265" s="9" t="s">
         <v>28</v>
@@ -8069,7 +8069,7 @@
         <v>27</v>
       </c>
       <c r="E266" s="11">
-        <v>20</v>
+        <v>25</v>
       </c>
       <c r="F266" s="9" t="s">
         <v>28</v>
@@ -8092,7 +8092,7 @@
         <v>27</v>
       </c>
       <c r="E267" s="11">
-        <v>31</v>
+        <v>20</v>
       </c>
       <c r="F267" s="9" t="s">
         <v>28</v>
@@ -8115,7 +8115,7 @@
         <v>27</v>
       </c>
       <c r="E268" s="11">
-        <v>17</v>
+        <v>19</v>
       </c>
       <c r="F268" s="9" t="s">
         <v>28</v>
@@ -8138,7 +8138,7 @@
         <v>27</v>
       </c>
       <c r="E269" s="11">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="F269" s="9" t="s">
         <v>28</v>
@@ -8161,7 +8161,7 @@
         <v>27</v>
       </c>
       <c r="E270" s="11">
-        <v>13</v>
+        <v>31</v>
       </c>
       <c r="F270" s="9" t="s">
         <v>28</v>
@@ -8184,7 +8184,7 @@
         <v>27</v>
       </c>
       <c r="E271" s="11">
-        <v>22</v>
+        <v>14</v>
       </c>
       <c r="F271" s="9" t="s">
         <v>28</v>
@@ -8207,7 +8207,7 @@
         <v>27</v>
       </c>
       <c r="E272" s="11">
-        <v>23</v>
+        <v>26</v>
       </c>
       <c r="F272" s="9" t="s">
         <v>28</v>
@@ -8230,7 +8230,7 @@
         <v>27</v>
       </c>
       <c r="E273" s="11">
-        <v>28</v>
+        <v>25</v>
       </c>
       <c r="F273" s="9" t="s">
         <v>28</v>
@@ -8253,7 +8253,7 @@
         <v>27</v>
       </c>
       <c r="E274" s="11">
-        <v>11</v>
+        <v>27</v>
       </c>
       <c r="F274" s="9" t="s">
         <v>28</v>
@@ -8276,7 +8276,7 @@
         <v>27</v>
       </c>
       <c r="E275" s="11">
-        <v>14</v>
+        <v>26</v>
       </c>
       <c r="F275" s="9" t="s">
         <v>28</v>
@@ -8299,7 +8299,7 @@
         <v>27</v>
       </c>
       <c r="E276" s="11">
-        <v>9</v>
+        <v>23</v>
       </c>
       <c r="F276" s="9" t="s">
         <v>28</v>
@@ -8322,7 +8322,7 @@
         <v>27</v>
       </c>
       <c r="E277" s="11">
-        <v>26</v>
+        <v>17</v>
       </c>
       <c r="F277" s="9" t="s">
         <v>28</v>
@@ -8345,7 +8345,7 @@
         <v>27</v>
       </c>
       <c r="E278" s="11">
-        <v>28</v>
+        <v>8</v>
       </c>
       <c r="F278" s="9" t="s">
         <v>28</v>
@@ -8368,7 +8368,7 @@
         <v>27</v>
       </c>
       <c r="E279" s="11">
-        <v>27</v>
+        <v>30</v>
       </c>
       <c r="F279" s="9" t="s">
         <v>28</v>
@@ -8391,7 +8391,7 @@
         <v>27</v>
       </c>
       <c r="E280" s="11">
-        <v>26</v>
+        <v>24</v>
       </c>
       <c r="F280" s="9" t="s">
         <v>28</v>
@@ -8414,7 +8414,7 @@
         <v>27</v>
       </c>
       <c r="E281" s="11">
-        <v>19</v>
+        <v>31</v>
       </c>
       <c r="F281" s="9" t="s">
         <v>28</v>
@@ -8437,7 +8437,7 @@
         <v>27</v>
       </c>
       <c r="E282" s="11">
-        <v>24</v>
+        <v>22</v>
       </c>
       <c r="F282" s="9" t="s">
         <v>28</v>
@@ -8460,7 +8460,7 @@
         <v>27</v>
       </c>
       <c r="E283" s="11">
-        <v>10</v>
+        <v>14</v>
       </c>
       <c r="F283" s="9" t="s">
         <v>28</v>
@@ -8483,7 +8483,7 @@
         <v>27</v>
       </c>
       <c r="E284" s="11">
-        <v>22</v>
+        <v>31</v>
       </c>
       <c r="F284" s="9" t="s">
         <v>28</v>
@@ -8506,7 +8506,7 @@
         <v>27</v>
       </c>
       <c r="E285" s="11">
-        <v>15</v>
+        <v>24</v>
       </c>
       <c r="F285" s="9" t="s">
         <v>28</v>
@@ -8529,7 +8529,7 @@
         <v>27</v>
       </c>
       <c r="E286" s="11">
-        <v>30</v>
+        <v>15</v>
       </c>
       <c r="F286" s="9" t="s">
         <v>28</v>
@@ -8552,7 +8552,7 @@
         <v>27</v>
       </c>
       <c r="E287" s="11">
-        <v>27</v>
+        <v>16</v>
       </c>
       <c r="F287" s="9" t="s">
         <v>28</v>
@@ -8575,7 +8575,7 @@
         <v>27</v>
       </c>
       <c r="E288" s="11">
-        <v>28</v>
+        <v>12</v>
       </c>
       <c r="F288" s="9" t="s">
         <v>28</v>
@@ -8598,7 +8598,7 @@
         <v>27</v>
       </c>
       <c r="E289" s="11">
-        <v>23</v>
+        <v>10</v>
       </c>
       <c r="F289" s="9" t="s">
         <v>28</v>
@@ -8621,7 +8621,7 @@
         <v>27</v>
       </c>
       <c r="E290" s="11">
-        <v>20</v>
+        <v>9</v>
       </c>
       <c r="F290" s="9" t="s">
         <v>28</v>
@@ -8644,7 +8644,7 @@
         <v>27</v>
       </c>
       <c r="E291" s="11">
-        <v>29</v>
+        <v>12</v>
       </c>
       <c r="F291" s="9" t="s">
         <v>28</v>
@@ -8667,7 +8667,7 @@
         <v>27</v>
       </c>
       <c r="E292" s="11">
-        <v>13</v>
+        <v>26</v>
       </c>
       <c r="F292" s="9" t="s">
         <v>28</v>
@@ -8690,7 +8690,7 @@
         <v>27</v>
       </c>
       <c r="E293" s="11">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="F293" s="9" t="s">
         <v>28</v>
@@ -8713,7 +8713,7 @@
         <v>27</v>
       </c>
       <c r="E294" s="11">
-        <v>9</v>
+        <v>26</v>
       </c>
       <c r="F294" s="9" t="s">
         <v>28</v>
@@ -8736,7 +8736,7 @@
         <v>27</v>
       </c>
       <c r="E295" s="11">
-        <v>20</v>
+        <v>22</v>
       </c>
       <c r="F295" s="9" t="s">
         <v>28</v>
@@ -8759,7 +8759,7 @@
         <v>27</v>
       </c>
       <c r="E296" s="11">
-        <v>31</v>
+        <v>9</v>
       </c>
       <c r="F296" s="9" t="s">
         <v>28</v>
@@ -8782,7 +8782,7 @@
         <v>27</v>
       </c>
       <c r="E297" s="11">
-        <v>14</v>
+        <v>17</v>
       </c>
       <c r="F297" s="9" t="s">
         <v>28</v>
@@ -8805,7 +8805,7 @@
         <v>27</v>
       </c>
       <c r="E298" s="11">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="F298" s="9" t="s">
         <v>28</v>
@@ -8828,7 +8828,7 @@
         <v>27</v>
       </c>
       <c r="E299" s="11">
-        <v>16</v>
+        <v>26</v>
       </c>
       <c r="F299" s="9" t="s">
         <v>28</v>
@@ -8851,7 +8851,7 @@
         <v>27</v>
       </c>
       <c r="E300" s="11">
-        <v>27</v>
+        <v>30</v>
       </c>
       <c r="F300" s="9" t="s">
         <v>28</v>
@@ -8874,7 +8874,7 @@
         <v>27</v>
       </c>
       <c r="E301" s="11">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="F301" s="9" t="s">
         <v>28</v>
@@ -8897,7 +8897,7 @@
         <v>27</v>
       </c>
       <c r="E302" s="11">
-        <v>8</v>
+        <v>14</v>
       </c>
       <c r="F302" s="9" t="s">
         <v>28</v>
@@ -8920,7 +8920,7 @@
         <v>27</v>
       </c>
       <c r="E303" s="11">
-        <v>10</v>
+        <v>30</v>
       </c>
       <c r="F303" s="9" t="s">
         <v>28</v>
@@ -8943,7 +8943,7 @@
         <v>27</v>
       </c>
       <c r="E304" s="11">
-        <v>30</v>
+        <v>27</v>
       </c>
       <c r="F304" s="9" t="s">
         <v>28</v>
@@ -8966,7 +8966,7 @@
         <v>27</v>
       </c>
       <c r="E305" s="11">
-        <v>8</v>
+        <v>25</v>
       </c>
       <c r="F305" s="9" t="s">
         <v>28</v>
@@ -8989,7 +8989,7 @@
         <v>27</v>
       </c>
       <c r="E306" s="11">
-        <v>9</v>
+        <v>20</v>
       </c>
       <c r="F306" s="9" t="s">
         <v>28</v>
@@ -9012,7 +9012,7 @@
         <v>27</v>
       </c>
       <c r="E307" s="11">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="F307" s="9" t="s">
         <v>28</v>
@@ -9035,7 +9035,7 @@
         <v>27</v>
       </c>
       <c r="E308" s="11">
-        <v>18</v>
+        <v>27</v>
       </c>
       <c r="F308" s="9" t="s">
         <v>28</v>
@@ -9058,7 +9058,7 @@
         <v>27</v>
       </c>
       <c r="E309" s="11">
-        <v>12</v>
+        <v>20</v>
       </c>
       <c r="F309" s="9" t="s">
         <v>28</v>
@@ -9081,7 +9081,7 @@
         <v>27</v>
       </c>
       <c r="E310" s="11">
-        <v>20</v>
+        <v>29</v>
       </c>
       <c r="F310" s="9" t="s">
         <v>28</v>
@@ -9104,7 +9104,7 @@
         <v>27</v>
       </c>
       <c r="E311" s="11">
-        <v>30</v>
+        <v>23</v>
       </c>
       <c r="F311" s="9" t="s">
         <v>28</v>
@@ -9127,7 +9127,7 @@
         <v>27</v>
       </c>
       <c r="E312" s="11">
-        <v>31</v>
+        <v>17</v>
       </c>
       <c r="F312" s="9" t="s">
         <v>28</v>
@@ -9150,7 +9150,7 @@
         <v>27</v>
       </c>
       <c r="E313" s="11">
-        <v>20</v>
+        <v>23</v>
       </c>
       <c r="F313" s="9" t="s">
         <v>28</v>
@@ -9173,7 +9173,7 @@
         <v>27</v>
       </c>
       <c r="E314" s="11">
-        <v>24</v>
+        <v>21</v>
       </c>
       <c r="F314" s="9" t="s">
         <v>28</v>
@@ -9219,7 +9219,7 @@
         <v>27</v>
       </c>
       <c r="E316" s="11">
-        <v>12</v>
+        <v>27</v>
       </c>
       <c r="F316" s="9" t="s">
         <v>28</v>
@@ -9242,7 +9242,7 @@
         <v>27</v>
       </c>
       <c r="E317" s="11">
-        <v>25</v>
+        <v>30</v>
       </c>
       <c r="F317" s="9" t="s">
         <v>28</v>
@@ -9265,7 +9265,7 @@
         <v>27</v>
       </c>
       <c r="E318" s="11">
-        <v>22</v>
+        <v>15</v>
       </c>
       <c r="F318" s="9" t="s">
         <v>28</v>
@@ -9288,7 +9288,7 @@
         <v>27</v>
       </c>
       <c r="E319" s="11">
-        <v>30</v>
+        <v>20</v>
       </c>
       <c r="F319" s="9" t="s">
         <v>28</v>
@@ -9311,7 +9311,7 @@
         <v>27</v>
       </c>
       <c r="E320" s="11">
-        <v>30</v>
+        <v>27</v>
       </c>
       <c r="F320" s="9" t="s">
         <v>28</v>
@@ -9334,7 +9334,7 @@
         <v>27</v>
       </c>
       <c r="E321" s="11">
-        <v>20</v>
+        <v>11</v>
       </c>
       <c r="F321" s="9" t="s">
         <v>28</v>
@@ -9357,7 +9357,7 @@
         <v>27</v>
       </c>
       <c r="E322" s="11">
-        <v>15</v>
+        <v>30</v>
       </c>
       <c r="F322" s="9" t="s">
         <v>28</v>
@@ -9380,7 +9380,7 @@
         <v>27</v>
       </c>
       <c r="E323" s="11">
-        <v>23</v>
+        <v>27</v>
       </c>
       <c r="F323" s="9" t="s">
         <v>28</v>
@@ -9403,7 +9403,7 @@
         <v>27</v>
       </c>
       <c r="E324" s="11">
-        <v>9</v>
+        <v>27</v>
       </c>
       <c r="F324" s="9" t="s">
         <v>28</v>
@@ -9449,7 +9449,7 @@
         <v>27</v>
       </c>
       <c r="E326" s="11">
-        <v>25</v>
+        <v>27</v>
       </c>
       <c r="F326" s="9" t="s">
         <v>28</v>
@@ -9495,7 +9495,7 @@
         <v>27</v>
       </c>
       <c r="E328" s="11">
-        <v>27</v>
+        <v>16</v>
       </c>
       <c r="F328" s="9" t="s">
         <v>28</v>
@@ -9518,7 +9518,7 @@
         <v>27</v>
       </c>
       <c r="E329" s="11">
-        <v>18</v>
+        <v>9</v>
       </c>
       <c r="F329" s="9" t="s">
         <v>28</v>
@@ -9541,7 +9541,7 @@
         <v>27</v>
       </c>
       <c r="E330" s="11">
-        <v>21</v>
+        <v>15</v>
       </c>
       <c r="F330" s="9" t="s">
         <v>28</v>
@@ -9564,7 +9564,7 @@
         <v>27</v>
       </c>
       <c r="E331" s="11">
-        <v>23</v>
+        <v>29</v>
       </c>
       <c r="F331" s="9" t="s">
         <v>28</v>
@@ -9587,7 +9587,7 @@
         <v>27</v>
       </c>
       <c r="E332" s="11">
-        <v>19</v>
+        <v>21</v>
       </c>
       <c r="F332" s="9" t="s">
         <v>28</v>
@@ -9610,7 +9610,7 @@
         <v>27</v>
       </c>
       <c r="E333" s="11">
-        <v>20</v>
+        <v>31</v>
       </c>
       <c r="F333" s="9" t="s">
         <v>28</v>
@@ -9633,7 +9633,7 @@
         <v>27</v>
       </c>
       <c r="E334" s="11">
-        <v>18</v>
+        <v>27</v>
       </c>
       <c r="F334" s="9" t="s">
         <v>28</v>
@@ -9656,7 +9656,7 @@
         <v>27</v>
       </c>
       <c r="E335" s="11">
-        <v>14</v>
+        <v>25</v>
       </c>
       <c r="F335" s="9" t="s">
         <v>28</v>
@@ -9679,7 +9679,7 @@
         <v>27</v>
       </c>
       <c r="E336" s="11">
-        <v>15</v>
+        <v>24</v>
       </c>
       <c r="F336" s="9" t="s">
         <v>28</v>
@@ -9702,7 +9702,7 @@
         <v>27</v>
       </c>
       <c r="E337" s="11">
-        <v>22</v>
+        <v>12</v>
       </c>
       <c r="F337" s="9" t="s">
         <v>28</v>
@@ -9725,7 +9725,7 @@
         <v>27</v>
       </c>
       <c r="E338" s="11">
-        <v>20</v>
+        <v>22</v>
       </c>
       <c r="F338" s="9" t="s">
         <v>28</v>
@@ -9748,7 +9748,7 @@
         <v>27</v>
       </c>
       <c r="E339" s="11">
-        <v>9</v>
+        <v>11</v>
       </c>
       <c r="F339" s="9" t="s">
         <v>28</v>
@@ -9771,7 +9771,7 @@
         <v>27</v>
       </c>
       <c r="E340" s="11">
-        <v>20</v>
+        <v>22</v>
       </c>
       <c r="F340" s="9" t="s">
         <v>28</v>
@@ -9794,7 +9794,7 @@
         <v>27</v>
       </c>
       <c r="E341" s="11">
-        <v>14</v>
+        <v>11</v>
       </c>
       <c r="F341" s="9" t="s">
         <v>28</v>
@@ -9817,7 +9817,7 @@
         <v>27</v>
       </c>
       <c r="E342" s="11">
-        <v>26</v>
+        <v>21</v>
       </c>
       <c r="F342" s="9" t="s">
         <v>28</v>
@@ -9840,7 +9840,7 @@
         <v>27</v>
       </c>
       <c r="E343" s="11">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="F343" s="9" t="s">
         <v>28</v>
@@ -9863,7 +9863,7 @@
         <v>27</v>
       </c>
       <c r="E344" s="11">
-        <v>15</v>
+        <v>21</v>
       </c>
       <c r="F344" s="9" t="s">
         <v>28</v>
@@ -9886,7 +9886,7 @@
         <v>27</v>
       </c>
       <c r="E345" s="11">
-        <v>31</v>
+        <v>17</v>
       </c>
       <c r="F345" s="9" t="s">
         <v>28</v>
@@ -9909,7 +9909,7 @@
         <v>27</v>
       </c>
       <c r="E346" s="11">
-        <v>23</v>
+        <v>25</v>
       </c>
       <c r="F346" s="9" t="s">
         <v>28</v>
@@ -9932,7 +9932,7 @@
         <v>27</v>
       </c>
       <c r="E347" s="11">
-        <v>29</v>
+        <v>9</v>
       </c>
       <c r="F347" s="9" t="s">
         <v>28</v>
@@ -9955,7 +9955,7 @@
         <v>27</v>
       </c>
       <c r="E348" s="11">
-        <v>18</v>
+        <v>31</v>
       </c>
       <c r="F348" s="9" t="s">
         <v>28</v>
@@ -9978,7 +9978,7 @@
         <v>27</v>
       </c>
       <c r="E349" s="11">
-        <v>12</v>
+        <v>31</v>
       </c>
       <c r="F349" s="9" t="s">
         <v>28</v>
@@ -10001,7 +10001,7 @@
         <v>27</v>
       </c>
       <c r="E350" s="11">
-        <v>30</v>
+        <v>27</v>
       </c>
       <c r="F350" s="9" t="s">
         <v>28</v>
@@ -10024,7 +10024,7 @@
         <v>27</v>
       </c>
       <c r="E351" s="11">
-        <v>9</v>
+        <v>26</v>
       </c>
       <c r="F351" s="9" t="s">
         <v>28</v>
@@ -10047,7 +10047,7 @@
         <v>27</v>
       </c>
       <c r="E352" s="11">
-        <v>18</v>
+        <v>24</v>
       </c>
       <c r="F352" s="9" t="s">
         <v>28</v>
@@ -10070,7 +10070,7 @@
         <v>27</v>
       </c>
       <c r="E353" s="11">
-        <v>24</v>
+        <v>8</v>
       </c>
       <c r="F353" s="9" t="s">
         <v>28</v>
@@ -10093,7 +10093,7 @@
         <v>27</v>
       </c>
       <c r="E354" s="11">
-        <v>12</v>
+        <v>31</v>
       </c>
       <c r="F354" s="9" t="s">
         <v>28</v>
@@ -10116,7 +10116,7 @@
         <v>27</v>
       </c>
       <c r="E355" s="11">
-        <v>31</v>
+        <v>17</v>
       </c>
       <c r="F355" s="9" t="s">
         <v>28</v>
@@ -10139,7 +10139,7 @@
         <v>27</v>
       </c>
       <c r="E356" s="11">
-        <v>28</v>
+        <v>15</v>
       </c>
       <c r="F356" s="9" t="s">
         <v>28</v>
@@ -10185,7 +10185,7 @@
         <v>27</v>
       </c>
       <c r="E358" s="11">
-        <v>12</v>
+        <v>17</v>
       </c>
       <c r="F358" s="9" t="s">
         <v>28</v>
@@ -10208,7 +10208,7 @@
         <v>27</v>
       </c>
       <c r="E359" s="11">
-        <v>9</v>
+        <v>27</v>
       </c>
       <c r="F359" s="9" t="s">
         <v>28</v>
@@ -10231,7 +10231,7 @@
         <v>27</v>
       </c>
       <c r="E360" s="11">
-        <v>26</v>
+        <v>22</v>
       </c>
       <c r="F360" s="9" t="s">
         <v>28</v>
@@ -10254,7 +10254,7 @@
         <v>27</v>
       </c>
       <c r="E361" s="11">
-        <v>22</v>
+        <v>17</v>
       </c>
       <c r="F361" s="9" t="s">
         <v>28</v>
@@ -10277,7 +10277,7 @@
         <v>27</v>
       </c>
       <c r="E362" s="11">
-        <v>19</v>
+        <v>22</v>
       </c>
       <c r="F362" s="9" t="s">
         <v>28</v>
@@ -10300,7 +10300,7 @@
         <v>27</v>
       </c>
       <c r="E363" s="11">
-        <v>25</v>
+        <v>16</v>
       </c>
       <c r="F363" s="9" t="s">
         <v>28</v>
@@ -10323,7 +10323,7 @@
         <v>27</v>
       </c>
       <c r="E364" s="11">
-        <v>8</v>
+        <v>29</v>
       </c>
       <c r="F364" s="9" t="s">
         <v>28</v>
@@ -10346,7 +10346,7 @@
         <v>27</v>
       </c>
       <c r="E365" s="11">
-        <v>29</v>
+        <v>14</v>
       </c>
       <c r="F365" s="9" t="s">
         <v>28</v>
@@ -10369,7 +10369,7 @@
         <v>27</v>
       </c>
       <c r="E366" s="11">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="F366" s="9" t="s">
         <v>28</v>
@@ -10392,7 +10392,7 @@
         <v>27</v>
       </c>
       <c r="E367" s="11">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="F367" s="9" t="s">
         <v>28</v>
@@ -10415,7 +10415,7 @@
         <v>27</v>
       </c>
       <c r="E368" s="11">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="F368" s="9" t="s">
         <v>28</v>
@@ -10438,7 +10438,7 @@
         <v>27</v>
       </c>
       <c r="E369" s="11">
-        <v>25</v>
+        <v>30</v>
       </c>
       <c r="F369" s="9" t="s">
         <v>28</v>
@@ -10461,7 +10461,7 @@
         <v>27</v>
       </c>
       <c r="E370" s="11">
-        <v>26</v>
+        <v>21</v>
       </c>
       <c r="F370" s="9" t="s">
         <v>28</v>
@@ -10484,7 +10484,7 @@
         <v>27</v>
       </c>
       <c r="E371" s="11">
-        <v>26</v>
+        <v>24</v>
       </c>
       <c r="F371" s="9" t="s">
         <v>28</v>
@@ -10507,7 +10507,7 @@
         <v>27</v>
       </c>
       <c r="E372" s="11">
-        <v>30</v>
+        <v>24</v>
       </c>
       <c r="F372" s="9" t="s">
         <v>28</v>
@@ -10553,7 +10553,7 @@
         <v>27</v>
       </c>
       <c r="E374" s="11">
-        <v>16</v>
+        <v>29</v>
       </c>
       <c r="F374" s="9" t="s">
         <v>28</v>
@@ -10576,7 +10576,7 @@
         <v>27</v>
       </c>
       <c r="E375" s="11">
-        <v>14</v>
+        <v>24</v>
       </c>
       <c r="F375" s="9" t="s">
         <v>28</v>
@@ -10599,7 +10599,7 @@
         <v>27</v>
       </c>
       <c r="E376" s="11">
-        <v>12</v>
+        <v>20</v>
       </c>
       <c r="F376" s="9" t="s">
         <v>28</v>
@@ -10622,7 +10622,7 @@
         <v>27</v>
       </c>
       <c r="E377" s="11">
-        <v>29</v>
+        <v>13</v>
       </c>
       <c r="F377" s="9" t="s">
         <v>28</v>
@@ -10645,7 +10645,7 @@
         <v>27</v>
       </c>
       <c r="E378" s="11">
-        <v>9</v>
+        <v>11</v>
       </c>
       <c r="F378" s="9" t="s">
         <v>28</v>
@@ -10668,7 +10668,7 @@
         <v>27</v>
       </c>
       <c r="E379" s="11">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="F379" s="9" t="s">
         <v>28</v>
@@ -10691,7 +10691,7 @@
         <v>27</v>
       </c>
       <c r="E380" s="11">
-        <v>24</v>
+        <v>18</v>
       </c>
       <c r="F380" s="9" t="s">
         <v>28</v>
@@ -10714,7 +10714,7 @@
         <v>27</v>
       </c>
       <c r="E381" s="11">
-        <v>28</v>
+        <v>13</v>
       </c>
       <c r="F381" s="9" t="s">
         <v>28</v>
@@ -10737,7 +10737,7 @@
         <v>27</v>
       </c>
       <c r="E382" s="11">
-        <v>20</v>
+        <v>10</v>
       </c>
       <c r="F382" s="9" t="s">
         <v>28</v>
@@ -10760,7 +10760,7 @@
         <v>27</v>
       </c>
       <c r="E383" s="11">
-        <v>20</v>
+        <v>15</v>
       </c>
       <c r="F383" s="9" t="s">
         <v>28</v>
@@ -10783,7 +10783,7 @@
         <v>27</v>
       </c>
       <c r="E384" s="11">
-        <v>12</v>
+        <v>22</v>
       </c>
       <c r="F384" s="9" t="s">
         <v>28</v>
@@ -10806,7 +10806,7 @@
         <v>27</v>
       </c>
       <c r="E385" s="11">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="F385" s="9" t="s">
         <v>28</v>
@@ -10829,7 +10829,7 @@
         <v>27</v>
       </c>
       <c r="E386" s="11">
-        <v>18</v>
+        <v>21</v>
       </c>
       <c r="F386" s="9" t="s">
         <v>28</v>
@@ -10852,7 +10852,7 @@
         <v>27</v>
       </c>
       <c r="E387" s="11">
-        <v>12</v>
+        <v>25</v>
       </c>
       <c r="F387" s="9" t="s">
         <v>28</v>
@@ -10898,7 +10898,7 @@
         <v>27</v>
       </c>
       <c r="E389" s="11">
-        <v>30</v>
+        <v>20</v>
       </c>
       <c r="F389" s="9" t="s">
         <v>28</v>
@@ -10921,7 +10921,7 @@
         <v>27</v>
       </c>
       <c r="E390" s="11">
-        <v>13</v>
+        <v>19</v>
       </c>
       <c r="F390" s="9" t="s">
         <v>28</v>
@@ -10944,7 +10944,7 @@
         <v>27</v>
       </c>
       <c r="E391" s="11">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="F391" s="9" t="s">
         <v>28</v>
@@ -10967,7 +10967,7 @@
         <v>27</v>
       </c>
       <c r="E392" s="11">
-        <v>29</v>
+        <v>26</v>
       </c>
       <c r="F392" s="9" t="s">
         <v>28</v>
@@ -10990,7 +10990,7 @@
         <v>27</v>
       </c>
       <c r="E393" s="11">
-        <v>12</v>
+        <v>29</v>
       </c>
       <c r="F393" s="9" t="s">
         <v>28</v>
@@ -11013,7 +11013,7 @@
         <v>27</v>
       </c>
       <c r="E394" s="11">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="F394" s="9" t="s">
         <v>28</v>
@@ -11036,7 +11036,7 @@
         <v>27</v>
       </c>
       <c r="E395" s="11">
-        <v>22</v>
+        <v>29</v>
       </c>
       <c r="F395" s="9" t="s">
         <v>28</v>
@@ -11059,7 +11059,7 @@
         <v>27</v>
       </c>
       <c r="E396" s="11">
-        <v>25</v>
+        <v>18</v>
       </c>
       <c r="F396" s="9" t="s">
         <v>28</v>
@@ -11082,7 +11082,7 @@
         <v>27</v>
       </c>
       <c r="E397" s="11">
-        <v>29</v>
+        <v>31</v>
       </c>
       <c r="F397" s="9" t="s">
         <v>28</v>
@@ -11105,7 +11105,7 @@
         <v>27</v>
       </c>
       <c r="E398" s="11">
-        <v>27</v>
+        <v>25</v>
       </c>
       <c r="F398" s="9" t="s">
         <v>28</v>
@@ -11128,7 +11128,7 @@
         <v>27</v>
       </c>
       <c r="E399" s="11">
-        <v>29</v>
+        <v>19</v>
       </c>
       <c r="F399" s="9" t="s">
         <v>28</v>
@@ -11151,7 +11151,7 @@
         <v>27</v>
       </c>
       <c r="E400" s="11">
-        <v>29</v>
+        <v>25</v>
       </c>
       <c r="F400" s="9" t="s">
         <v>28</v>
@@ -11174,7 +11174,7 @@
         <v>27</v>
       </c>
       <c r="E401" s="11">
-        <v>26</v>
+        <v>20</v>
       </c>
       <c r="F401" s="9" t="s">
         <v>28</v>

</xml_diff>

<commit_message>
feat(user): activate member status dynamically on first login and compute real join date
</commit_message>
<xml_diff>
--- a/all-test-reports/selenium/selenium_e2e_test_report.xlsx
+++ b/all-test-reports/selenium/selenium_e2e_test_report.xlsx
@@ -35,7 +35,7 @@
     <t>Execution Date</t>
   </si>
   <si>
-    <t>28/7/2026, 11:27:59 am</t>
+    <t>28/7/2026, 11:31:46 am</t>
   </si>
   <si>
     <t>Browser / Mode</t>
@@ -98,7 +98,7 @@
     <t>PASS</t>
   </si>
   <si>
-    <t>11:27:59 am</t>
+    <t>11:31:46 am</t>
   </si>
   <si>
     <t>N/A</t>
@@ -1997,7 +1997,7 @@
         <v>27</v>
       </c>
       <c r="E2" s="11">
-        <v>28</v>
+        <v>26</v>
       </c>
       <c r="F2" s="9" t="s">
         <v>28</v>
@@ -2020,7 +2020,7 @@
         <v>27</v>
       </c>
       <c r="E3" s="11">
-        <v>8</v>
+        <v>20</v>
       </c>
       <c r="F3" s="9" t="s">
         <v>28</v>
@@ -2043,7 +2043,7 @@
         <v>27</v>
       </c>
       <c r="E4" s="11">
-        <v>8</v>
+        <v>18</v>
       </c>
       <c r="F4" s="9" t="s">
         <v>28</v>
@@ -2066,7 +2066,7 @@
         <v>27</v>
       </c>
       <c r="E5" s="11">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="F5" s="9" t="s">
         <v>28</v>
@@ -2089,7 +2089,7 @@
         <v>27</v>
       </c>
       <c r="E6" s="11">
-        <v>21</v>
+        <v>29</v>
       </c>
       <c r="F6" s="9" t="s">
         <v>28</v>
@@ -2135,7 +2135,7 @@
         <v>27</v>
       </c>
       <c r="E8" s="11">
-        <v>17</v>
+        <v>31</v>
       </c>
       <c r="F8" s="9" t="s">
         <v>28</v>
@@ -2158,7 +2158,7 @@
         <v>27</v>
       </c>
       <c r="E9" s="11">
-        <v>25</v>
+        <v>21</v>
       </c>
       <c r="F9" s="9" t="s">
         <v>28</v>
@@ -2181,7 +2181,7 @@
         <v>27</v>
       </c>
       <c r="E10" s="11">
-        <v>8</v>
+        <v>31</v>
       </c>
       <c r="F10" s="9" t="s">
         <v>28</v>
@@ -2204,7 +2204,7 @@
         <v>27</v>
       </c>
       <c r="E11" s="11">
-        <v>25</v>
+        <v>19</v>
       </c>
       <c r="F11" s="9" t="s">
         <v>28</v>
@@ -2227,7 +2227,7 @@
         <v>27</v>
       </c>
       <c r="E12" s="11">
-        <v>31</v>
+        <v>25</v>
       </c>
       <c r="F12" s="9" t="s">
         <v>28</v>
@@ -2250,7 +2250,7 @@
         <v>27</v>
       </c>
       <c r="E13" s="11">
-        <v>9</v>
+        <v>30</v>
       </c>
       <c r="F13" s="9" t="s">
         <v>28</v>
@@ -2296,7 +2296,7 @@
         <v>27</v>
       </c>
       <c r="E15" s="11">
-        <v>24</v>
+        <v>26</v>
       </c>
       <c r="F15" s="9" t="s">
         <v>28</v>
@@ -2319,7 +2319,7 @@
         <v>27</v>
       </c>
       <c r="E16" s="11">
-        <v>9</v>
+        <v>17</v>
       </c>
       <c r="F16" s="9" t="s">
         <v>28</v>
@@ -2342,7 +2342,7 @@
         <v>27</v>
       </c>
       <c r="E17" s="11">
-        <v>28</v>
+        <v>10</v>
       </c>
       <c r="F17" s="9" t="s">
         <v>28</v>
@@ -2365,7 +2365,7 @@
         <v>27</v>
       </c>
       <c r="E18" s="11">
-        <v>14</v>
+        <v>28</v>
       </c>
       <c r="F18" s="9" t="s">
         <v>28</v>
@@ -2388,7 +2388,7 @@
         <v>27</v>
       </c>
       <c r="E19" s="11">
-        <v>12</v>
+        <v>25</v>
       </c>
       <c r="F19" s="9" t="s">
         <v>28</v>
@@ -2411,7 +2411,7 @@
         <v>27</v>
       </c>
       <c r="E20" s="11">
-        <v>23</v>
+        <v>14</v>
       </c>
       <c r="F20" s="9" t="s">
         <v>28</v>
@@ -2434,7 +2434,7 @@
         <v>27</v>
       </c>
       <c r="E21" s="11">
-        <v>21</v>
+        <v>15</v>
       </c>
       <c r="F21" s="9" t="s">
         <v>28</v>
@@ -2457,7 +2457,7 @@
         <v>27</v>
       </c>
       <c r="E22" s="11">
-        <v>21</v>
+        <v>9</v>
       </c>
       <c r="F22" s="9" t="s">
         <v>28</v>
@@ -2480,7 +2480,7 @@
         <v>27</v>
       </c>
       <c r="E23" s="11">
-        <v>14</v>
+        <v>26</v>
       </c>
       <c r="F23" s="9" t="s">
         <v>28</v>
@@ -2503,7 +2503,7 @@
         <v>27</v>
       </c>
       <c r="E24" s="11">
-        <v>31</v>
+        <v>20</v>
       </c>
       <c r="F24" s="9" t="s">
         <v>28</v>
@@ -2526,7 +2526,7 @@
         <v>27</v>
       </c>
       <c r="E25" s="11">
-        <v>23</v>
+        <v>15</v>
       </c>
       <c r="F25" s="9" t="s">
         <v>28</v>
@@ -2549,7 +2549,7 @@
         <v>27</v>
       </c>
       <c r="E26" s="11">
-        <v>15</v>
+        <v>9</v>
       </c>
       <c r="F26" s="9" t="s">
         <v>28</v>
@@ -2572,7 +2572,7 @@
         <v>27</v>
       </c>
       <c r="E27" s="11">
-        <v>19</v>
+        <v>10</v>
       </c>
       <c r="F27" s="9" t="s">
         <v>28</v>
@@ -2595,7 +2595,7 @@
         <v>27</v>
       </c>
       <c r="E28" s="11">
-        <v>29</v>
+        <v>21</v>
       </c>
       <c r="F28" s="9" t="s">
         <v>28</v>
@@ -2618,7 +2618,7 @@
         <v>27</v>
       </c>
       <c r="E29" s="11">
-        <v>19</v>
+        <v>14</v>
       </c>
       <c r="F29" s="9" t="s">
         <v>28</v>
@@ -2641,7 +2641,7 @@
         <v>27</v>
       </c>
       <c r="E30" s="11">
-        <v>22</v>
+        <v>17</v>
       </c>
       <c r="F30" s="9" t="s">
         <v>28</v>
@@ -2687,7 +2687,7 @@
         <v>27</v>
       </c>
       <c r="E32" s="11">
-        <v>18</v>
+        <v>14</v>
       </c>
       <c r="F32" s="9" t="s">
         <v>28</v>
@@ -2710,7 +2710,7 @@
         <v>27</v>
       </c>
       <c r="E33" s="11">
-        <v>11</v>
+        <v>24</v>
       </c>
       <c r="F33" s="9" t="s">
         <v>28</v>
@@ -2733,7 +2733,7 @@
         <v>27</v>
       </c>
       <c r="E34" s="11">
-        <v>21</v>
+        <v>18</v>
       </c>
       <c r="F34" s="9" t="s">
         <v>28</v>
@@ -2779,7 +2779,7 @@
         <v>27</v>
       </c>
       <c r="E36" s="11">
-        <v>23</v>
+        <v>21</v>
       </c>
       <c r="F36" s="9" t="s">
         <v>28</v>
@@ -2802,7 +2802,7 @@
         <v>27</v>
       </c>
       <c r="E37" s="11">
-        <v>10</v>
+        <v>27</v>
       </c>
       <c r="F37" s="9" t="s">
         <v>28</v>
@@ -2825,7 +2825,7 @@
         <v>27</v>
       </c>
       <c r="E38" s="11">
-        <v>26</v>
+        <v>31</v>
       </c>
       <c r="F38" s="9" t="s">
         <v>28</v>
@@ -2848,7 +2848,7 @@
         <v>27</v>
       </c>
       <c r="E39" s="11">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="F39" s="9" t="s">
         <v>28</v>
@@ -2871,7 +2871,7 @@
         <v>27</v>
       </c>
       <c r="E40" s="11">
-        <v>20</v>
+        <v>27</v>
       </c>
       <c r="F40" s="9" t="s">
         <v>28</v>
@@ -2894,7 +2894,7 @@
         <v>27</v>
       </c>
       <c r="E41" s="11">
-        <v>9</v>
+        <v>25</v>
       </c>
       <c r="F41" s="9" t="s">
         <v>28</v>
@@ -2917,7 +2917,7 @@
         <v>27</v>
       </c>
       <c r="E42" s="11">
-        <v>8</v>
+        <v>28</v>
       </c>
       <c r="F42" s="9" t="s">
         <v>28</v>
@@ -2940,7 +2940,7 @@
         <v>27</v>
       </c>
       <c r="E43" s="11">
-        <v>19</v>
+        <v>12</v>
       </c>
       <c r="F43" s="9" t="s">
         <v>28</v>
@@ -2963,7 +2963,7 @@
         <v>27</v>
       </c>
       <c r="E44" s="11">
-        <v>10</v>
+        <v>19</v>
       </c>
       <c r="F44" s="9" t="s">
         <v>28</v>
@@ -2986,7 +2986,7 @@
         <v>27</v>
       </c>
       <c r="E45" s="11">
-        <v>16</v>
+        <v>18</v>
       </c>
       <c r="F45" s="9" t="s">
         <v>28</v>
@@ -3009,7 +3009,7 @@
         <v>27</v>
       </c>
       <c r="E46" s="11">
-        <v>21</v>
+        <v>14</v>
       </c>
       <c r="F46" s="9" t="s">
         <v>28</v>
@@ -3032,7 +3032,7 @@
         <v>27</v>
       </c>
       <c r="E47" s="11">
-        <v>17</v>
+        <v>19</v>
       </c>
       <c r="F47" s="9" t="s">
         <v>28</v>
@@ -3055,7 +3055,7 @@
         <v>27</v>
       </c>
       <c r="E48" s="11">
-        <v>19</v>
+        <v>11</v>
       </c>
       <c r="F48" s="9" t="s">
         <v>28</v>
@@ -3078,7 +3078,7 @@
         <v>27</v>
       </c>
       <c r="E49" s="11">
-        <v>8</v>
+        <v>13</v>
       </c>
       <c r="F49" s="9" t="s">
         <v>28</v>
@@ -3101,7 +3101,7 @@
         <v>27</v>
       </c>
       <c r="E50" s="11">
-        <v>15</v>
+        <v>28</v>
       </c>
       <c r="F50" s="9" t="s">
         <v>28</v>
@@ -3124,7 +3124,7 @@
         <v>27</v>
       </c>
       <c r="E51" s="11">
-        <v>13</v>
+        <v>24</v>
       </c>
       <c r="F51" s="9" t="s">
         <v>28</v>
@@ -3147,7 +3147,7 @@
         <v>27</v>
       </c>
       <c r="E52" s="11">
-        <v>19</v>
+        <v>13</v>
       </c>
       <c r="F52" s="9" t="s">
         <v>28</v>
@@ -3170,7 +3170,7 @@
         <v>27</v>
       </c>
       <c r="E53" s="11">
-        <v>20</v>
+        <v>25</v>
       </c>
       <c r="F53" s="9" t="s">
         <v>28</v>
@@ -3193,7 +3193,7 @@
         <v>27</v>
       </c>
       <c r="E54" s="11">
-        <v>20</v>
+        <v>30</v>
       </c>
       <c r="F54" s="9" t="s">
         <v>28</v>
@@ -3216,7 +3216,7 @@
         <v>27</v>
       </c>
       <c r="E55" s="11">
-        <v>29</v>
+        <v>11</v>
       </c>
       <c r="F55" s="9" t="s">
         <v>28</v>
@@ -3239,7 +3239,7 @@
         <v>27</v>
       </c>
       <c r="E56" s="11">
-        <v>8</v>
+        <v>11</v>
       </c>
       <c r="F56" s="9" t="s">
         <v>28</v>
@@ -3262,7 +3262,7 @@
         <v>27</v>
       </c>
       <c r="E57" s="11">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="F57" s="9" t="s">
         <v>28</v>
@@ -3285,7 +3285,7 @@
         <v>27</v>
       </c>
       <c r="E58" s="11">
-        <v>9</v>
+        <v>19</v>
       </c>
       <c r="F58" s="9" t="s">
         <v>28</v>
@@ -3308,7 +3308,7 @@
         <v>27</v>
       </c>
       <c r="E59" s="11">
-        <v>12</v>
+        <v>16</v>
       </c>
       <c r="F59" s="9" t="s">
         <v>28</v>
@@ -3331,7 +3331,7 @@
         <v>27</v>
       </c>
       <c r="E60" s="11">
-        <v>30</v>
+        <v>15</v>
       </c>
       <c r="F60" s="9" t="s">
         <v>28</v>
@@ -3354,7 +3354,7 @@
         <v>27</v>
       </c>
       <c r="E61" s="11">
-        <v>18</v>
+        <v>13</v>
       </c>
       <c r="F61" s="9" t="s">
         <v>28</v>
@@ -3377,7 +3377,7 @@
         <v>27</v>
       </c>
       <c r="E62" s="11">
-        <v>23</v>
+        <v>20</v>
       </c>
       <c r="F62" s="9" t="s">
         <v>28</v>
@@ -3400,7 +3400,7 @@
         <v>27</v>
       </c>
       <c r="E63" s="11">
-        <v>8</v>
+        <v>25</v>
       </c>
       <c r="F63" s="9" t="s">
         <v>28</v>
@@ -3423,7 +3423,7 @@
         <v>27</v>
       </c>
       <c r="E64" s="11">
-        <v>10</v>
+        <v>16</v>
       </c>
       <c r="F64" s="9" t="s">
         <v>28</v>
@@ -3446,7 +3446,7 @@
         <v>27</v>
       </c>
       <c r="E65" s="11">
-        <v>9</v>
+        <v>17</v>
       </c>
       <c r="F65" s="9" t="s">
         <v>28</v>
@@ -3469,7 +3469,7 @@
         <v>27</v>
       </c>
       <c r="E66" s="11">
-        <v>23</v>
+        <v>17</v>
       </c>
       <c r="F66" s="9" t="s">
         <v>28</v>
@@ -3492,7 +3492,7 @@
         <v>27</v>
       </c>
       <c r="E67" s="11">
-        <v>10</v>
+        <v>22</v>
       </c>
       <c r="F67" s="9" t="s">
         <v>28</v>
@@ -3515,7 +3515,7 @@
         <v>27</v>
       </c>
       <c r="E68" s="11">
-        <v>12</v>
+        <v>23</v>
       </c>
       <c r="F68" s="9" t="s">
         <v>28</v>
@@ -3538,7 +3538,7 @@
         <v>27</v>
       </c>
       <c r="E69" s="11">
-        <v>12</v>
+        <v>22</v>
       </c>
       <c r="F69" s="9" t="s">
         <v>28</v>
@@ -3561,7 +3561,7 @@
         <v>27</v>
       </c>
       <c r="E70" s="11">
-        <v>20</v>
+        <v>8</v>
       </c>
       <c r="F70" s="9" t="s">
         <v>28</v>
@@ -3584,7 +3584,7 @@
         <v>27</v>
       </c>
       <c r="E71" s="11">
-        <v>16</v>
+        <v>11</v>
       </c>
       <c r="F71" s="9" t="s">
         <v>28</v>
@@ -3607,7 +3607,7 @@
         <v>27</v>
       </c>
       <c r="E72" s="11">
-        <v>22</v>
+        <v>26</v>
       </c>
       <c r="F72" s="9" t="s">
         <v>28</v>
@@ -3630,7 +3630,7 @@
         <v>27</v>
       </c>
       <c r="E73" s="11">
-        <v>25</v>
+        <v>17</v>
       </c>
       <c r="F73" s="9" t="s">
         <v>28</v>
@@ -3653,7 +3653,7 @@
         <v>27</v>
       </c>
       <c r="E74" s="11">
-        <v>15</v>
+        <v>17</v>
       </c>
       <c r="F74" s="9" t="s">
         <v>28</v>
@@ -3676,7 +3676,7 @@
         <v>27</v>
       </c>
       <c r="E75" s="11">
-        <v>14</v>
+        <v>22</v>
       </c>
       <c r="F75" s="9" t="s">
         <v>28</v>
@@ -3699,7 +3699,7 @@
         <v>27</v>
       </c>
       <c r="E76" s="11">
-        <v>9</v>
+        <v>22</v>
       </c>
       <c r="F76" s="9" t="s">
         <v>28</v>
@@ -3722,7 +3722,7 @@
         <v>27</v>
       </c>
       <c r="E77" s="11">
-        <v>24</v>
+        <v>28</v>
       </c>
       <c r="F77" s="9" t="s">
         <v>28</v>
@@ -3745,7 +3745,7 @@
         <v>27</v>
       </c>
       <c r="E78" s="11">
-        <v>16</v>
+        <v>27</v>
       </c>
       <c r="F78" s="9" t="s">
         <v>28</v>
@@ -3768,7 +3768,7 @@
         <v>27</v>
       </c>
       <c r="E79" s="11">
-        <v>14</v>
+        <v>29</v>
       </c>
       <c r="F79" s="9" t="s">
         <v>28</v>
@@ -3791,7 +3791,7 @@
         <v>27</v>
       </c>
       <c r="E80" s="11">
-        <v>9</v>
+        <v>25</v>
       </c>
       <c r="F80" s="9" t="s">
         <v>28</v>
@@ -3837,7 +3837,7 @@
         <v>27</v>
       </c>
       <c r="E82" s="11">
-        <v>9</v>
+        <v>29</v>
       </c>
       <c r="F82" s="9" t="s">
         <v>28</v>
@@ -3860,7 +3860,7 @@
         <v>27</v>
       </c>
       <c r="E83" s="11">
-        <v>17</v>
+        <v>14</v>
       </c>
       <c r="F83" s="9" t="s">
         <v>28</v>
@@ -3883,7 +3883,7 @@
         <v>27</v>
       </c>
       <c r="E84" s="11">
-        <v>10</v>
+        <v>14</v>
       </c>
       <c r="F84" s="9" t="s">
         <v>28</v>
@@ -3906,7 +3906,7 @@
         <v>27</v>
       </c>
       <c r="E85" s="11">
-        <v>31</v>
+        <v>13</v>
       </c>
       <c r="F85" s="9" t="s">
         <v>28</v>
@@ -3929,7 +3929,7 @@
         <v>27</v>
       </c>
       <c r="E86" s="11">
-        <v>30</v>
+        <v>14</v>
       </c>
       <c r="F86" s="9" t="s">
         <v>28</v>
@@ -3952,7 +3952,7 @@
         <v>27</v>
       </c>
       <c r="E87" s="11">
-        <v>8</v>
+        <v>25</v>
       </c>
       <c r="F87" s="9" t="s">
         <v>28</v>
@@ -3975,7 +3975,7 @@
         <v>27</v>
       </c>
       <c r="E88" s="11">
-        <v>12</v>
+        <v>18</v>
       </c>
       <c r="F88" s="9" t="s">
         <v>28</v>
@@ -3998,7 +3998,7 @@
         <v>27</v>
       </c>
       <c r="E89" s="11">
-        <v>11</v>
+        <v>13</v>
       </c>
       <c r="F89" s="9" t="s">
         <v>28</v>
@@ -4021,7 +4021,7 @@
         <v>27</v>
       </c>
       <c r="E90" s="11">
-        <v>20</v>
+        <v>23</v>
       </c>
       <c r="F90" s="9" t="s">
         <v>28</v>
@@ -4044,7 +4044,7 @@
         <v>27</v>
       </c>
       <c r="E91" s="11">
-        <v>20</v>
+        <v>13</v>
       </c>
       <c r="F91" s="9" t="s">
         <v>28</v>
@@ -4067,7 +4067,7 @@
         <v>27</v>
       </c>
       <c r="E92" s="11">
-        <v>31</v>
+        <v>18</v>
       </c>
       <c r="F92" s="9" t="s">
         <v>28</v>
@@ -4090,7 +4090,7 @@
         <v>27</v>
       </c>
       <c r="E93" s="11">
-        <v>11</v>
+        <v>24</v>
       </c>
       <c r="F93" s="9" t="s">
         <v>28</v>
@@ -4113,7 +4113,7 @@
         <v>27</v>
       </c>
       <c r="E94" s="11">
-        <v>8</v>
+        <v>14</v>
       </c>
       <c r="F94" s="9" t="s">
         <v>28</v>
@@ -4136,7 +4136,7 @@
         <v>27</v>
       </c>
       <c r="E95" s="11">
-        <v>18</v>
+        <v>16</v>
       </c>
       <c r="F95" s="9" t="s">
         <v>28</v>
@@ -4159,7 +4159,7 @@
         <v>27</v>
       </c>
       <c r="E96" s="11">
-        <v>15</v>
+        <v>8</v>
       </c>
       <c r="F96" s="9" t="s">
         <v>28</v>
@@ -4182,7 +4182,7 @@
         <v>27</v>
       </c>
       <c r="E97" s="11">
-        <v>28</v>
+        <v>8</v>
       </c>
       <c r="F97" s="9" t="s">
         <v>28</v>
@@ -4205,7 +4205,7 @@
         <v>27</v>
       </c>
       <c r="E98" s="11">
-        <v>12</v>
+        <v>31</v>
       </c>
       <c r="F98" s="9" t="s">
         <v>28</v>
@@ -4228,7 +4228,7 @@
         <v>27</v>
       </c>
       <c r="E99" s="11">
-        <v>13</v>
+        <v>19</v>
       </c>
       <c r="F99" s="9" t="s">
         <v>28</v>
@@ -4251,7 +4251,7 @@
         <v>27</v>
       </c>
       <c r="E100" s="11">
-        <v>16</v>
+        <v>29</v>
       </c>
       <c r="F100" s="9" t="s">
         <v>28</v>
@@ -4274,7 +4274,7 @@
         <v>27</v>
       </c>
       <c r="E101" s="11">
-        <v>21</v>
+        <v>11</v>
       </c>
       <c r="F101" s="9" t="s">
         <v>28</v>
@@ -4297,7 +4297,7 @@
         <v>27</v>
       </c>
       <c r="E102" s="11">
-        <v>24</v>
+        <v>16</v>
       </c>
       <c r="F102" s="9" t="s">
         <v>28</v>
@@ -4320,7 +4320,7 @@
         <v>27</v>
       </c>
       <c r="E103" s="11">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="F103" s="9" t="s">
         <v>28</v>
@@ -4343,7 +4343,7 @@
         <v>27</v>
       </c>
       <c r="E104" s="11">
-        <v>12</v>
+        <v>31</v>
       </c>
       <c r="F104" s="9" t="s">
         <v>28</v>
@@ -4366,7 +4366,7 @@
         <v>27</v>
       </c>
       <c r="E105" s="11">
-        <v>26</v>
+        <v>28</v>
       </c>
       <c r="F105" s="9" t="s">
         <v>28</v>
@@ -4389,7 +4389,7 @@
         <v>27</v>
       </c>
       <c r="E106" s="11">
-        <v>21</v>
+        <v>26</v>
       </c>
       <c r="F106" s="9" t="s">
         <v>28</v>
@@ -4412,7 +4412,7 @@
         <v>27</v>
       </c>
       <c r="E107" s="11">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="F107" s="9" t="s">
         <v>28</v>
@@ -4435,7 +4435,7 @@
         <v>27</v>
       </c>
       <c r="E108" s="11">
-        <v>26</v>
+        <v>8</v>
       </c>
       <c r="F108" s="9" t="s">
         <v>28</v>
@@ -4458,7 +4458,7 @@
         <v>27</v>
       </c>
       <c r="E109" s="11">
-        <v>9</v>
+        <v>23</v>
       </c>
       <c r="F109" s="9" t="s">
         <v>28</v>
@@ -4481,7 +4481,7 @@
         <v>27</v>
       </c>
       <c r="E110" s="11">
-        <v>8</v>
+        <v>21</v>
       </c>
       <c r="F110" s="9" t="s">
         <v>28</v>
@@ -4504,7 +4504,7 @@
         <v>27</v>
       </c>
       <c r="E111" s="11">
-        <v>20</v>
+        <v>28</v>
       </c>
       <c r="F111" s="9" t="s">
         <v>28</v>
@@ -4527,7 +4527,7 @@
         <v>27</v>
       </c>
       <c r="E112" s="11">
-        <v>12</v>
+        <v>25</v>
       </c>
       <c r="F112" s="9" t="s">
         <v>28</v>
@@ -4550,7 +4550,7 @@
         <v>27</v>
       </c>
       <c r="E113" s="11">
-        <v>9</v>
+        <v>30</v>
       </c>
       <c r="F113" s="9" t="s">
         <v>28</v>
@@ -4573,7 +4573,7 @@
         <v>27</v>
       </c>
       <c r="E114" s="11">
-        <v>18</v>
+        <v>16</v>
       </c>
       <c r="F114" s="9" t="s">
         <v>28</v>
@@ -4596,7 +4596,7 @@
         <v>27</v>
       </c>
       <c r="E115" s="11">
-        <v>19</v>
+        <v>11</v>
       </c>
       <c r="F115" s="9" t="s">
         <v>28</v>
@@ -4619,7 +4619,7 @@
         <v>27</v>
       </c>
       <c r="E116" s="11">
-        <v>21</v>
+        <v>11</v>
       </c>
       <c r="F116" s="9" t="s">
         <v>28</v>
@@ -4642,7 +4642,7 @@
         <v>27</v>
       </c>
       <c r="E117" s="11">
-        <v>25</v>
+        <v>20</v>
       </c>
       <c r="F117" s="9" t="s">
         <v>28</v>
@@ -4665,7 +4665,7 @@
         <v>27</v>
       </c>
       <c r="E118" s="11">
-        <v>21</v>
+        <v>10</v>
       </c>
       <c r="F118" s="9" t="s">
         <v>28</v>
@@ -4688,7 +4688,7 @@
         <v>27</v>
       </c>
       <c r="E119" s="11">
-        <v>28</v>
+        <v>19</v>
       </c>
       <c r="F119" s="9" t="s">
         <v>28</v>
@@ -4711,7 +4711,7 @@
         <v>27</v>
       </c>
       <c r="E120" s="11">
-        <v>20</v>
+        <v>25</v>
       </c>
       <c r="F120" s="9" t="s">
         <v>28</v>
@@ -4734,7 +4734,7 @@
         <v>27</v>
       </c>
       <c r="E121" s="11">
-        <v>26</v>
+        <v>21</v>
       </c>
       <c r="F121" s="9" t="s">
         <v>28</v>
@@ -4757,7 +4757,7 @@
         <v>27</v>
       </c>
       <c r="E122" s="11">
-        <v>12</v>
+        <v>20</v>
       </c>
       <c r="F122" s="9" t="s">
         <v>28</v>
@@ -4780,7 +4780,7 @@
         <v>27</v>
       </c>
       <c r="E123" s="11">
-        <v>14</v>
+        <v>25</v>
       </c>
       <c r="F123" s="9" t="s">
         <v>28</v>
@@ -4803,7 +4803,7 @@
         <v>27</v>
       </c>
       <c r="E124" s="11">
-        <v>11</v>
+        <v>15</v>
       </c>
       <c r="F124" s="9" t="s">
         <v>28</v>
@@ -4826,7 +4826,7 @@
         <v>27</v>
       </c>
       <c r="E125" s="11">
-        <v>10</v>
+        <v>22</v>
       </c>
       <c r="F125" s="9" t="s">
         <v>28</v>
@@ -4849,7 +4849,7 @@
         <v>27</v>
       </c>
       <c r="E126" s="11">
-        <v>11</v>
+        <v>19</v>
       </c>
       <c r="F126" s="9" t="s">
         <v>28</v>
@@ -4872,7 +4872,7 @@
         <v>27</v>
       </c>
       <c r="E127" s="11">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="F127" s="9" t="s">
         <v>28</v>
@@ -4895,7 +4895,7 @@
         <v>27</v>
       </c>
       <c r="E128" s="11">
-        <v>8</v>
+        <v>22</v>
       </c>
       <c r="F128" s="9" t="s">
         <v>28</v>
@@ -4918,7 +4918,7 @@
         <v>27</v>
       </c>
       <c r="E129" s="11">
-        <v>10</v>
+        <v>17</v>
       </c>
       <c r="F129" s="9" t="s">
         <v>28</v>
@@ -4941,7 +4941,7 @@
         <v>27</v>
       </c>
       <c r="E130" s="11">
-        <v>26</v>
+        <v>8</v>
       </c>
       <c r="F130" s="9" t="s">
         <v>28</v>
@@ -4964,7 +4964,7 @@
         <v>27</v>
       </c>
       <c r="E131" s="11">
-        <v>17</v>
+        <v>22</v>
       </c>
       <c r="F131" s="9" t="s">
         <v>28</v>
@@ -4987,7 +4987,7 @@
         <v>27</v>
       </c>
       <c r="E132" s="11">
-        <v>20</v>
+        <v>11</v>
       </c>
       <c r="F132" s="9" t="s">
         <v>28</v>
@@ -5010,7 +5010,7 @@
         <v>27</v>
       </c>
       <c r="E133" s="11">
-        <v>20</v>
+        <v>11</v>
       </c>
       <c r="F133" s="9" t="s">
         <v>28</v>
@@ -5033,7 +5033,7 @@
         <v>27</v>
       </c>
       <c r="E134" s="11">
-        <v>14</v>
+        <v>22</v>
       </c>
       <c r="F134" s="9" t="s">
         <v>28</v>
@@ -5056,7 +5056,7 @@
         <v>27</v>
       </c>
       <c r="E135" s="11">
-        <v>13</v>
+        <v>28</v>
       </c>
       <c r="F135" s="9" t="s">
         <v>28</v>
@@ -5079,7 +5079,7 @@
         <v>27</v>
       </c>
       <c r="E136" s="11">
-        <v>26</v>
+        <v>15</v>
       </c>
       <c r="F136" s="9" t="s">
         <v>28</v>
@@ -5102,7 +5102,7 @@
         <v>27</v>
       </c>
       <c r="E137" s="11">
-        <v>8</v>
+        <v>11</v>
       </c>
       <c r="F137" s="9" t="s">
         <v>28</v>
@@ -5125,7 +5125,7 @@
         <v>27</v>
       </c>
       <c r="E138" s="11">
-        <v>11</v>
+        <v>25</v>
       </c>
       <c r="F138" s="9" t="s">
         <v>28</v>
@@ -5148,7 +5148,7 @@
         <v>27</v>
       </c>
       <c r="E139" s="11">
-        <v>21</v>
+        <v>30</v>
       </c>
       <c r="F139" s="9" t="s">
         <v>28</v>
@@ -5171,7 +5171,7 @@
         <v>27</v>
       </c>
       <c r="E140" s="11">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="F140" s="9" t="s">
         <v>28</v>
@@ -5194,7 +5194,7 @@
         <v>27</v>
       </c>
       <c r="E141" s="11">
-        <v>31</v>
+        <v>17</v>
       </c>
       <c r="F141" s="9" t="s">
         <v>28</v>
@@ -5217,7 +5217,7 @@
         <v>27</v>
       </c>
       <c r="E142" s="11">
-        <v>23</v>
+        <v>30</v>
       </c>
       <c r="F142" s="9" t="s">
         <v>28</v>
@@ -5240,7 +5240,7 @@
         <v>27</v>
       </c>
       <c r="E143" s="11">
-        <v>26</v>
+        <v>12</v>
       </c>
       <c r="F143" s="9" t="s">
         <v>28</v>
@@ -5263,7 +5263,7 @@
         <v>27</v>
       </c>
       <c r="E144" s="11">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="F144" s="9" t="s">
         <v>28</v>
@@ -5286,7 +5286,7 @@
         <v>27</v>
       </c>
       <c r="E145" s="11">
-        <v>27</v>
+        <v>30</v>
       </c>
       <c r="F145" s="9" t="s">
         <v>28</v>
@@ -5309,7 +5309,7 @@
         <v>27</v>
       </c>
       <c r="E146" s="11">
-        <v>26</v>
+        <v>24</v>
       </c>
       <c r="F146" s="9" t="s">
         <v>28</v>
@@ -5332,7 +5332,7 @@
         <v>27</v>
       </c>
       <c r="E147" s="11">
-        <v>17</v>
+        <v>13</v>
       </c>
       <c r="F147" s="9" t="s">
         <v>28</v>
@@ -5355,7 +5355,7 @@
         <v>27</v>
       </c>
       <c r="E148" s="11">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="F148" s="9" t="s">
         <v>28</v>
@@ -5378,7 +5378,7 @@
         <v>27</v>
       </c>
       <c r="E149" s="11">
-        <v>27</v>
+        <v>12</v>
       </c>
       <c r="F149" s="9" t="s">
         <v>28</v>
@@ -5401,7 +5401,7 @@
         <v>27</v>
       </c>
       <c r="E150" s="11">
-        <v>25</v>
+        <v>10</v>
       </c>
       <c r="F150" s="9" t="s">
         <v>28</v>
@@ -5424,7 +5424,7 @@
         <v>27</v>
       </c>
       <c r="E151" s="11">
-        <v>18</v>
+        <v>15</v>
       </c>
       <c r="F151" s="9" t="s">
         <v>28</v>
@@ -5447,7 +5447,7 @@
         <v>27</v>
       </c>
       <c r="E152" s="11">
-        <v>9</v>
+        <v>14</v>
       </c>
       <c r="F152" s="9" t="s">
         <v>28</v>
@@ -5470,7 +5470,7 @@
         <v>27</v>
       </c>
       <c r="E153" s="11">
-        <v>21</v>
+        <v>26</v>
       </c>
       <c r="F153" s="9" t="s">
         <v>28</v>
@@ -5493,7 +5493,7 @@
         <v>27</v>
       </c>
       <c r="E154" s="11">
-        <v>25</v>
+        <v>9</v>
       </c>
       <c r="F154" s="9" t="s">
         <v>28</v>
@@ -5516,7 +5516,7 @@
         <v>27</v>
       </c>
       <c r="E155" s="11">
-        <v>14</v>
+        <v>26</v>
       </c>
       <c r="F155" s="9" t="s">
         <v>28</v>
@@ -5539,7 +5539,7 @@
         <v>27</v>
       </c>
       <c r="E156" s="11">
-        <v>26</v>
+        <v>14</v>
       </c>
       <c r="F156" s="9" t="s">
         <v>28</v>
@@ -5562,7 +5562,7 @@
         <v>27</v>
       </c>
       <c r="E157" s="11">
-        <v>18</v>
+        <v>21</v>
       </c>
       <c r="F157" s="9" t="s">
         <v>28</v>
@@ -5585,7 +5585,7 @@
         <v>27</v>
       </c>
       <c r="E158" s="11">
-        <v>25</v>
+        <v>18</v>
       </c>
       <c r="F158" s="9" t="s">
         <v>28</v>
@@ -5608,7 +5608,7 @@
         <v>27</v>
       </c>
       <c r="E159" s="11">
-        <v>20</v>
+        <v>29</v>
       </c>
       <c r="F159" s="9" t="s">
         <v>28</v>
@@ -5631,7 +5631,7 @@
         <v>27</v>
       </c>
       <c r="E160" s="11">
-        <v>10</v>
+        <v>21</v>
       </c>
       <c r="F160" s="9" t="s">
         <v>28</v>
@@ -5654,7 +5654,7 @@
         <v>27</v>
       </c>
       <c r="E161" s="11">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="F161" s="9" t="s">
         <v>28</v>
@@ -5677,7 +5677,7 @@
         <v>27</v>
       </c>
       <c r="E162" s="11">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="F162" s="9" t="s">
         <v>28</v>
@@ -5700,7 +5700,7 @@
         <v>27</v>
       </c>
       <c r="E163" s="11">
-        <v>10</v>
+        <v>29</v>
       </c>
       <c r="F163" s="9" t="s">
         <v>28</v>
@@ -5723,7 +5723,7 @@
         <v>27</v>
       </c>
       <c r="E164" s="11">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="F164" s="9" t="s">
         <v>28</v>
@@ -5746,7 +5746,7 @@
         <v>27</v>
       </c>
       <c r="E165" s="11">
-        <v>11</v>
+        <v>19</v>
       </c>
       <c r="F165" s="9" t="s">
         <v>28</v>
@@ -5769,7 +5769,7 @@
         <v>27</v>
       </c>
       <c r="E166" s="11">
-        <v>18</v>
+        <v>24</v>
       </c>
       <c r="F166" s="9" t="s">
         <v>28</v>
@@ -5792,7 +5792,7 @@
         <v>27</v>
       </c>
       <c r="E167" s="11">
-        <v>18</v>
+        <v>16</v>
       </c>
       <c r="F167" s="9" t="s">
         <v>28</v>
@@ -5815,7 +5815,7 @@
         <v>27</v>
       </c>
       <c r="E168" s="11">
-        <v>27</v>
+        <v>20</v>
       </c>
       <c r="F168" s="9" t="s">
         <v>28</v>
@@ -5838,7 +5838,7 @@
         <v>27</v>
       </c>
       <c r="E169" s="11">
-        <v>23</v>
+        <v>29</v>
       </c>
       <c r="F169" s="9" t="s">
         <v>28</v>
@@ -5861,7 +5861,7 @@
         <v>27</v>
       </c>
       <c r="E170" s="11">
-        <v>8</v>
+        <v>22</v>
       </c>
       <c r="F170" s="9" t="s">
         <v>28</v>
@@ -5884,7 +5884,7 @@
         <v>27</v>
       </c>
       <c r="E171" s="11">
-        <v>9</v>
+        <v>15</v>
       </c>
       <c r="F171" s="9" t="s">
         <v>28</v>
@@ -5907,7 +5907,7 @@
         <v>27</v>
       </c>
       <c r="E172" s="11">
-        <v>12</v>
+        <v>29</v>
       </c>
       <c r="F172" s="9" t="s">
         <v>28</v>
@@ -5930,7 +5930,7 @@
         <v>27</v>
       </c>
       <c r="E173" s="11">
-        <v>11</v>
+        <v>27</v>
       </c>
       <c r="F173" s="9" t="s">
         <v>28</v>
@@ -5953,7 +5953,7 @@
         <v>27</v>
       </c>
       <c r="E174" s="11">
-        <v>25</v>
+        <v>9</v>
       </c>
       <c r="F174" s="9" t="s">
         <v>28</v>
@@ -5976,7 +5976,7 @@
         <v>27</v>
       </c>
       <c r="E175" s="11">
-        <v>22</v>
+        <v>15</v>
       </c>
       <c r="F175" s="9" t="s">
         <v>28</v>
@@ -5999,7 +5999,7 @@
         <v>27</v>
       </c>
       <c r="E176" s="11">
-        <v>12</v>
+        <v>23</v>
       </c>
       <c r="F176" s="9" t="s">
         <v>28</v>
@@ -6022,7 +6022,7 @@
         <v>27</v>
       </c>
       <c r="E177" s="11">
-        <v>30</v>
+        <v>17</v>
       </c>
       <c r="F177" s="9" t="s">
         <v>28</v>
@@ -6045,7 +6045,7 @@
         <v>27</v>
       </c>
       <c r="E178" s="11">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="F178" s="9" t="s">
         <v>28</v>
@@ -6068,7 +6068,7 @@
         <v>27</v>
       </c>
       <c r="E179" s="11">
-        <v>29</v>
+        <v>12</v>
       </c>
       <c r="F179" s="9" t="s">
         <v>28</v>
@@ -6091,7 +6091,7 @@
         <v>27</v>
       </c>
       <c r="E180" s="11">
-        <v>14</v>
+        <v>8</v>
       </c>
       <c r="F180" s="9" t="s">
         <v>28</v>
@@ -6114,7 +6114,7 @@
         <v>27</v>
       </c>
       <c r="E181" s="11">
-        <v>19</v>
+        <v>17</v>
       </c>
       <c r="F181" s="9" t="s">
         <v>28</v>
@@ -6137,7 +6137,7 @@
         <v>27</v>
       </c>
       <c r="E182" s="11">
-        <v>13</v>
+        <v>25</v>
       </c>
       <c r="F182" s="9" t="s">
         <v>28</v>
@@ -6160,7 +6160,7 @@
         <v>27</v>
       </c>
       <c r="E183" s="11">
-        <v>23</v>
+        <v>10</v>
       </c>
       <c r="F183" s="9" t="s">
         <v>28</v>
@@ -6183,7 +6183,7 @@
         <v>27</v>
       </c>
       <c r="E184" s="11">
-        <v>26</v>
+        <v>22</v>
       </c>
       <c r="F184" s="9" t="s">
         <v>28</v>
@@ -6206,7 +6206,7 @@
         <v>27</v>
       </c>
       <c r="E185" s="11">
-        <v>21</v>
+        <v>25</v>
       </c>
       <c r="F185" s="9" t="s">
         <v>28</v>
@@ -6229,7 +6229,7 @@
         <v>27</v>
       </c>
       <c r="E186" s="11">
-        <v>19</v>
+        <v>28</v>
       </c>
       <c r="F186" s="9" t="s">
         <v>28</v>
@@ -6275,7 +6275,7 @@
         <v>27</v>
       </c>
       <c r="E188" s="11">
-        <v>30</v>
+        <v>8</v>
       </c>
       <c r="F188" s="9" t="s">
         <v>28</v>
@@ -6298,7 +6298,7 @@
         <v>27</v>
       </c>
       <c r="E189" s="11">
-        <v>13</v>
+        <v>22</v>
       </c>
       <c r="F189" s="9" t="s">
         <v>28</v>
@@ -6321,7 +6321,7 @@
         <v>27</v>
       </c>
       <c r="E190" s="11">
-        <v>30</v>
+        <v>24</v>
       </c>
       <c r="F190" s="9" t="s">
         <v>28</v>
@@ -6344,7 +6344,7 @@
         <v>27</v>
       </c>
       <c r="E191" s="11">
-        <v>25</v>
+        <v>15</v>
       </c>
       <c r="F191" s="9" t="s">
         <v>28</v>
@@ -6367,7 +6367,7 @@
         <v>27</v>
       </c>
       <c r="E192" s="11">
-        <v>20</v>
+        <v>30</v>
       </c>
       <c r="F192" s="9" t="s">
         <v>28</v>
@@ -6390,7 +6390,7 @@
         <v>27</v>
       </c>
       <c r="E193" s="11">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="F193" s="9" t="s">
         <v>28</v>
@@ -6413,7 +6413,7 @@
         <v>27</v>
       </c>
       <c r="E194" s="11">
-        <v>19</v>
+        <v>31</v>
       </c>
       <c r="F194" s="9" t="s">
         <v>28</v>
@@ -6436,7 +6436,7 @@
         <v>27</v>
       </c>
       <c r="E195" s="11">
-        <v>21</v>
+        <v>17</v>
       </c>
       <c r="F195" s="9" t="s">
         <v>28</v>
@@ -6459,7 +6459,7 @@
         <v>27</v>
       </c>
       <c r="E196" s="11">
-        <v>24</v>
+        <v>31</v>
       </c>
       <c r="F196" s="9" t="s">
         <v>28</v>
@@ -6482,7 +6482,7 @@
         <v>27</v>
       </c>
       <c r="E197" s="11">
-        <v>19</v>
+        <v>31</v>
       </c>
       <c r="F197" s="9" t="s">
         <v>28</v>
@@ -6505,7 +6505,7 @@
         <v>27</v>
       </c>
       <c r="E198" s="11">
-        <v>19</v>
+        <v>26</v>
       </c>
       <c r="F198" s="9" t="s">
         <v>28</v>
@@ -6528,7 +6528,7 @@
         <v>27</v>
       </c>
       <c r="E199" s="11">
-        <v>8</v>
+        <v>24</v>
       </c>
       <c r="F199" s="9" t="s">
         <v>28</v>
@@ -6551,7 +6551,7 @@
         <v>27</v>
       </c>
       <c r="E200" s="11">
-        <v>16</v>
+        <v>20</v>
       </c>
       <c r="F200" s="9" t="s">
         <v>28</v>
@@ -6574,7 +6574,7 @@
         <v>27</v>
       </c>
       <c r="E201" s="11">
-        <v>13</v>
+        <v>17</v>
       </c>
       <c r="F201" s="9" t="s">
         <v>28</v>
@@ -6597,7 +6597,7 @@
         <v>27</v>
       </c>
       <c r="E202" s="11">
-        <v>30</v>
+        <v>13</v>
       </c>
       <c r="F202" s="9" t="s">
         <v>28</v>
@@ -6620,7 +6620,7 @@
         <v>27</v>
       </c>
       <c r="E203" s="11">
-        <v>31</v>
+        <v>8</v>
       </c>
       <c r="F203" s="9" t="s">
         <v>28</v>
@@ -6643,7 +6643,7 @@
         <v>27</v>
       </c>
       <c r="E204" s="11">
-        <v>15</v>
+        <v>23</v>
       </c>
       <c r="F204" s="9" t="s">
         <v>28</v>
@@ -6666,7 +6666,7 @@
         <v>27</v>
       </c>
       <c r="E205" s="11">
-        <v>20</v>
+        <v>18</v>
       </c>
       <c r="F205" s="9" t="s">
         <v>28</v>
@@ -6689,7 +6689,7 @@
         <v>27</v>
       </c>
       <c r="E206" s="11">
-        <v>16</v>
+        <v>21</v>
       </c>
       <c r="F206" s="9" t="s">
         <v>28</v>
@@ -6712,7 +6712,7 @@
         <v>27</v>
       </c>
       <c r="E207" s="11">
-        <v>23</v>
+        <v>27</v>
       </c>
       <c r="F207" s="9" t="s">
         <v>28</v>
@@ -6735,7 +6735,7 @@
         <v>27</v>
       </c>
       <c r="E208" s="11">
-        <v>17</v>
+        <v>21</v>
       </c>
       <c r="F208" s="9" t="s">
         <v>28</v>
@@ -6758,7 +6758,7 @@
         <v>27</v>
       </c>
       <c r="E209" s="11">
-        <v>15</v>
+        <v>25</v>
       </c>
       <c r="F209" s="9" t="s">
         <v>28</v>
@@ -6781,7 +6781,7 @@
         <v>27</v>
       </c>
       <c r="E210" s="11">
-        <v>24</v>
+        <v>22</v>
       </c>
       <c r="F210" s="9" t="s">
         <v>28</v>
@@ -6804,7 +6804,7 @@
         <v>27</v>
       </c>
       <c r="E211" s="11">
-        <v>16</v>
+        <v>10</v>
       </c>
       <c r="F211" s="9" t="s">
         <v>28</v>
@@ -6827,7 +6827,7 @@
         <v>27</v>
       </c>
       <c r="E212" s="11">
-        <v>26</v>
+        <v>21</v>
       </c>
       <c r="F212" s="9" t="s">
         <v>28</v>
@@ -6850,7 +6850,7 @@
         <v>27</v>
       </c>
       <c r="E213" s="11">
-        <v>25</v>
+        <v>23</v>
       </c>
       <c r="F213" s="9" t="s">
         <v>28</v>
@@ -6873,7 +6873,7 @@
         <v>27</v>
       </c>
       <c r="E214" s="11">
-        <v>26</v>
+        <v>16</v>
       </c>
       <c r="F214" s="9" t="s">
         <v>28</v>
@@ -6896,7 +6896,7 @@
         <v>27</v>
       </c>
       <c r="E215" s="11">
-        <v>28</v>
+        <v>21</v>
       </c>
       <c r="F215" s="9" t="s">
         <v>28</v>
@@ -6919,7 +6919,7 @@
         <v>27</v>
       </c>
       <c r="E216" s="11">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="F216" s="9" t="s">
         <v>28</v>
@@ -6942,7 +6942,7 @@
         <v>27</v>
       </c>
       <c r="E217" s="11">
-        <v>24</v>
+        <v>11</v>
       </c>
       <c r="F217" s="9" t="s">
         <v>28</v>
@@ -6965,7 +6965,7 @@
         <v>27</v>
       </c>
       <c r="E218" s="11">
-        <v>25</v>
+        <v>29</v>
       </c>
       <c r="F218" s="9" t="s">
         <v>28</v>
@@ -6988,7 +6988,7 @@
         <v>27</v>
       </c>
       <c r="E219" s="11">
-        <v>22</v>
+        <v>25</v>
       </c>
       <c r="F219" s="9" t="s">
         <v>28</v>
@@ -7011,7 +7011,7 @@
         <v>27</v>
       </c>
       <c r="E220" s="11">
-        <v>23</v>
+        <v>9</v>
       </c>
       <c r="F220" s="9" t="s">
         <v>28</v>
@@ -7034,7 +7034,7 @@
         <v>27</v>
       </c>
       <c r="E221" s="11">
-        <v>23</v>
+        <v>9</v>
       </c>
       <c r="F221" s="9" t="s">
         <v>28</v>
@@ -7057,7 +7057,7 @@
         <v>27</v>
       </c>
       <c r="E222" s="11">
-        <v>8</v>
+        <v>22</v>
       </c>
       <c r="F222" s="9" t="s">
         <v>28</v>
@@ -7080,7 +7080,7 @@
         <v>27</v>
       </c>
       <c r="E223" s="11">
-        <v>27</v>
+        <v>21</v>
       </c>
       <c r="F223" s="9" t="s">
         <v>28</v>
@@ -7103,7 +7103,7 @@
         <v>27</v>
       </c>
       <c r="E224" s="11">
-        <v>14</v>
+        <v>11</v>
       </c>
       <c r="F224" s="9" t="s">
         <v>28</v>
@@ -7126,7 +7126,7 @@
         <v>27</v>
       </c>
       <c r="E225" s="11">
-        <v>17</v>
+        <v>14</v>
       </c>
       <c r="F225" s="9" t="s">
         <v>28</v>
@@ -7149,7 +7149,7 @@
         <v>27</v>
       </c>
       <c r="E226" s="11">
-        <v>30</v>
+        <v>8</v>
       </c>
       <c r="F226" s="9" t="s">
         <v>28</v>
@@ -7172,7 +7172,7 @@
         <v>27</v>
       </c>
       <c r="E227" s="11">
-        <v>25</v>
+        <v>19</v>
       </c>
       <c r="F227" s="9" t="s">
         <v>28</v>
@@ -7195,7 +7195,7 @@
         <v>27</v>
       </c>
       <c r="E228" s="11">
-        <v>11</v>
+        <v>28</v>
       </c>
       <c r="F228" s="9" t="s">
         <v>28</v>
@@ -7218,7 +7218,7 @@
         <v>27</v>
       </c>
       <c r="E229" s="11">
-        <v>19</v>
+        <v>9</v>
       </c>
       <c r="F229" s="9" t="s">
         <v>28</v>
@@ -7241,7 +7241,7 @@
         <v>27</v>
       </c>
       <c r="E230" s="11">
-        <v>21</v>
+        <v>31</v>
       </c>
       <c r="F230" s="9" t="s">
         <v>28</v>
@@ -7264,7 +7264,7 @@
         <v>27</v>
       </c>
       <c r="E231" s="11">
-        <v>14</v>
+        <v>31</v>
       </c>
       <c r="F231" s="9" t="s">
         <v>28</v>
@@ -7287,7 +7287,7 @@
         <v>27</v>
       </c>
       <c r="E232" s="11">
-        <v>25</v>
+        <v>21</v>
       </c>
       <c r="F232" s="9" t="s">
         <v>28</v>
@@ -7310,7 +7310,7 @@
         <v>27</v>
       </c>
       <c r="E233" s="11">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="F233" s="9" t="s">
         <v>28</v>
@@ -7333,7 +7333,7 @@
         <v>27</v>
       </c>
       <c r="E234" s="11">
-        <v>14</v>
+        <v>18</v>
       </c>
       <c r="F234" s="9" t="s">
         <v>28</v>
@@ -7356,7 +7356,7 @@
         <v>27</v>
       </c>
       <c r="E235" s="11">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="F235" s="9" t="s">
         <v>28</v>
@@ -7379,7 +7379,7 @@
         <v>27</v>
       </c>
       <c r="E236" s="11">
-        <v>23</v>
+        <v>29</v>
       </c>
       <c r="F236" s="9" t="s">
         <v>28</v>
@@ -7402,7 +7402,7 @@
         <v>27</v>
       </c>
       <c r="E237" s="11">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="F237" s="9" t="s">
         <v>28</v>
@@ -7425,7 +7425,7 @@
         <v>27</v>
       </c>
       <c r="E238" s="11">
-        <v>28</v>
+        <v>17</v>
       </c>
       <c r="F238" s="9" t="s">
         <v>28</v>
@@ -7448,7 +7448,7 @@
         <v>27</v>
       </c>
       <c r="E239" s="11">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="F239" s="9" t="s">
         <v>28</v>
@@ -7471,7 +7471,7 @@
         <v>27</v>
       </c>
       <c r="E240" s="11">
-        <v>16</v>
+        <v>10</v>
       </c>
       <c r="F240" s="9" t="s">
         <v>28</v>
@@ -7494,7 +7494,7 @@
         <v>27</v>
       </c>
       <c r="E241" s="11">
-        <v>30</v>
+        <v>25</v>
       </c>
       <c r="F241" s="9" t="s">
         <v>28</v>
@@ -7517,7 +7517,7 @@
         <v>27</v>
       </c>
       <c r="E242" s="11">
-        <v>25</v>
+        <v>22</v>
       </c>
       <c r="F242" s="9" t="s">
         <v>28</v>
@@ -7563,7 +7563,7 @@
         <v>27</v>
       </c>
       <c r="E244" s="11">
-        <v>20</v>
+        <v>28</v>
       </c>
       <c r="F244" s="9" t="s">
         <v>28</v>
@@ -7586,7 +7586,7 @@
         <v>27</v>
       </c>
       <c r="E245" s="11">
-        <v>8</v>
+        <v>31</v>
       </c>
       <c r="F245" s="9" t="s">
         <v>28</v>
@@ -7609,7 +7609,7 @@
         <v>27</v>
       </c>
       <c r="E246" s="11">
-        <v>28</v>
+        <v>23</v>
       </c>
       <c r="F246" s="9" t="s">
         <v>28</v>
@@ -7632,7 +7632,7 @@
         <v>27</v>
       </c>
       <c r="E247" s="11">
-        <v>23</v>
+        <v>28</v>
       </c>
       <c r="F247" s="9" t="s">
         <v>28</v>
@@ -7655,7 +7655,7 @@
         <v>27</v>
       </c>
       <c r="E248" s="11">
-        <v>9</v>
+        <v>22</v>
       </c>
       <c r="F248" s="9" t="s">
         <v>28</v>
@@ -7678,7 +7678,7 @@
         <v>27</v>
       </c>
       <c r="E249" s="11">
-        <v>29</v>
+        <v>22</v>
       </c>
       <c r="F249" s="9" t="s">
         <v>28</v>
@@ -7701,7 +7701,7 @@
         <v>27</v>
       </c>
       <c r="E250" s="11">
-        <v>15</v>
+        <v>9</v>
       </c>
       <c r="F250" s="9" t="s">
         <v>28</v>
@@ -7724,7 +7724,7 @@
         <v>27</v>
       </c>
       <c r="E251" s="11">
-        <v>25</v>
+        <v>23</v>
       </c>
       <c r="F251" s="9" t="s">
         <v>28</v>
@@ -7747,7 +7747,7 @@
         <v>27</v>
       </c>
       <c r="E252" s="11">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="F252" s="9" t="s">
         <v>28</v>
@@ -7770,7 +7770,7 @@
         <v>27</v>
       </c>
       <c r="E253" s="11">
-        <v>31</v>
+        <v>24</v>
       </c>
       <c r="F253" s="9" t="s">
         <v>28</v>
@@ -7793,7 +7793,7 @@
         <v>27</v>
       </c>
       <c r="E254" s="11">
-        <v>26</v>
+        <v>24</v>
       </c>
       <c r="F254" s="9" t="s">
         <v>28</v>
@@ -7816,7 +7816,7 @@
         <v>27</v>
       </c>
       <c r="E255" s="11">
-        <v>25</v>
+        <v>31</v>
       </c>
       <c r="F255" s="9" t="s">
         <v>28</v>
@@ -7839,7 +7839,7 @@
         <v>27</v>
       </c>
       <c r="E256" s="11">
-        <v>29</v>
+        <v>15</v>
       </c>
       <c r="F256" s="9" t="s">
         <v>28</v>
@@ -7862,7 +7862,7 @@
         <v>27</v>
       </c>
       <c r="E257" s="11">
-        <v>13</v>
+        <v>29</v>
       </c>
       <c r="F257" s="9" t="s">
         <v>28</v>
@@ -7885,7 +7885,7 @@
         <v>27</v>
       </c>
       <c r="E258" s="11">
-        <v>31</v>
+        <v>11</v>
       </c>
       <c r="F258" s="9" t="s">
         <v>28</v>
@@ -7908,7 +7908,7 @@
         <v>27</v>
       </c>
       <c r="E259" s="11">
-        <v>24</v>
+        <v>21</v>
       </c>
       <c r="F259" s="9" t="s">
         <v>28</v>
@@ -7931,7 +7931,7 @@
         <v>27</v>
       </c>
       <c r="E260" s="11">
-        <v>15</v>
+        <v>19</v>
       </c>
       <c r="F260" s="9" t="s">
         <v>28</v>
@@ -7954,7 +7954,7 @@
         <v>27</v>
       </c>
       <c r="E261" s="11">
-        <v>31</v>
+        <v>27</v>
       </c>
       <c r="F261" s="9" t="s">
         <v>28</v>
@@ -7977,7 +7977,7 @@
         <v>27</v>
       </c>
       <c r="E262" s="11">
-        <v>9</v>
+        <v>31</v>
       </c>
       <c r="F262" s="9" t="s">
         <v>28</v>
@@ -8000,7 +8000,7 @@
         <v>27</v>
       </c>
       <c r="E263" s="11">
-        <v>26</v>
+        <v>18</v>
       </c>
       <c r="F263" s="9" t="s">
         <v>28</v>
@@ -8023,7 +8023,7 @@
         <v>27</v>
       </c>
       <c r="E264" s="11">
-        <v>29</v>
+        <v>14</v>
       </c>
       <c r="F264" s="9" t="s">
         <v>28</v>
@@ -8046,7 +8046,7 @@
         <v>27</v>
       </c>
       <c r="E265" s="11">
-        <v>28</v>
+        <v>23</v>
       </c>
       <c r="F265" s="9" t="s">
         <v>28</v>
@@ -8069,7 +8069,7 @@
         <v>27</v>
       </c>
       <c r="E266" s="11">
-        <v>25</v>
+        <v>31</v>
       </c>
       <c r="F266" s="9" t="s">
         <v>28</v>
@@ -8092,7 +8092,7 @@
         <v>27</v>
       </c>
       <c r="E267" s="11">
-        <v>20</v>
+        <v>16</v>
       </c>
       <c r="F267" s="9" t="s">
         <v>28</v>
@@ -8115,7 +8115,7 @@
         <v>27</v>
       </c>
       <c r="E268" s="11">
-        <v>19</v>
+        <v>11</v>
       </c>
       <c r="F268" s="9" t="s">
         <v>28</v>
@@ -8138,7 +8138,7 @@
         <v>27</v>
       </c>
       <c r="E269" s="11">
-        <v>20</v>
+        <v>23</v>
       </c>
       <c r="F269" s="9" t="s">
         <v>28</v>
@@ -8161,7 +8161,7 @@
         <v>27</v>
       </c>
       <c r="E270" s="11">
-        <v>31</v>
+        <v>13</v>
       </c>
       <c r="F270" s="9" t="s">
         <v>28</v>
@@ -8184,7 +8184,7 @@
         <v>27</v>
       </c>
       <c r="E271" s="11">
-        <v>14</v>
+        <v>24</v>
       </c>
       <c r="F271" s="9" t="s">
         <v>28</v>
@@ -8207,7 +8207,7 @@
         <v>27</v>
       </c>
       <c r="E272" s="11">
-        <v>26</v>
+        <v>19</v>
       </c>
       <c r="F272" s="9" t="s">
         <v>28</v>
@@ -8230,7 +8230,7 @@
         <v>27</v>
       </c>
       <c r="E273" s="11">
-        <v>25</v>
+        <v>19</v>
       </c>
       <c r="F273" s="9" t="s">
         <v>28</v>
@@ -8253,7 +8253,7 @@
         <v>27</v>
       </c>
       <c r="E274" s="11">
-        <v>27</v>
+        <v>10</v>
       </c>
       <c r="F274" s="9" t="s">
         <v>28</v>
@@ -8276,7 +8276,7 @@
         <v>27</v>
       </c>
       <c r="E275" s="11">
-        <v>26</v>
+        <v>28</v>
       </c>
       <c r="F275" s="9" t="s">
         <v>28</v>
@@ -8299,7 +8299,7 @@
         <v>27</v>
       </c>
       <c r="E276" s="11">
-        <v>23</v>
+        <v>28</v>
       </c>
       <c r="F276" s="9" t="s">
         <v>28</v>
@@ -8322,7 +8322,7 @@
         <v>27</v>
       </c>
       <c r="E277" s="11">
-        <v>17</v>
+        <v>20</v>
       </c>
       <c r="F277" s="9" t="s">
         <v>28</v>
@@ -8345,7 +8345,7 @@
         <v>27</v>
       </c>
       <c r="E278" s="11">
-        <v>8</v>
+        <v>12</v>
       </c>
       <c r="F278" s="9" t="s">
         <v>28</v>
@@ -8368,7 +8368,7 @@
         <v>27</v>
       </c>
       <c r="E279" s="11">
-        <v>30</v>
+        <v>22</v>
       </c>
       <c r="F279" s="9" t="s">
         <v>28</v>
@@ -8391,7 +8391,7 @@
         <v>27</v>
       </c>
       <c r="E280" s="11">
-        <v>24</v>
+        <v>16</v>
       </c>
       <c r="F280" s="9" t="s">
         <v>28</v>
@@ -8414,7 +8414,7 @@
         <v>27</v>
       </c>
       <c r="E281" s="11">
-        <v>31</v>
+        <v>11</v>
       </c>
       <c r="F281" s="9" t="s">
         <v>28</v>
@@ -8437,7 +8437,7 @@
         <v>27</v>
       </c>
       <c r="E282" s="11">
-        <v>22</v>
+        <v>10</v>
       </c>
       <c r="F282" s="9" t="s">
         <v>28</v>
@@ -8460,7 +8460,7 @@
         <v>27</v>
       </c>
       <c r="E283" s="11">
-        <v>14</v>
+        <v>21</v>
       </c>
       <c r="F283" s="9" t="s">
         <v>28</v>
@@ -8483,7 +8483,7 @@
         <v>27</v>
       </c>
       <c r="E284" s="11">
-        <v>31</v>
+        <v>28</v>
       </c>
       <c r="F284" s="9" t="s">
         <v>28</v>
@@ -8506,7 +8506,7 @@
         <v>27</v>
       </c>
       <c r="E285" s="11">
-        <v>24</v>
+        <v>31</v>
       </c>
       <c r="F285" s="9" t="s">
         <v>28</v>
@@ -8529,7 +8529,7 @@
         <v>27</v>
       </c>
       <c r="E286" s="11">
-        <v>15</v>
+        <v>18</v>
       </c>
       <c r="F286" s="9" t="s">
         <v>28</v>
@@ -8552,7 +8552,7 @@
         <v>27</v>
       </c>
       <c r="E287" s="11">
-        <v>16</v>
+        <v>21</v>
       </c>
       <c r="F287" s="9" t="s">
         <v>28</v>
@@ -8575,7 +8575,7 @@
         <v>27</v>
       </c>
       <c r="E288" s="11">
-        <v>12</v>
+        <v>19</v>
       </c>
       <c r="F288" s="9" t="s">
         <v>28</v>
@@ -8598,7 +8598,7 @@
         <v>27</v>
       </c>
       <c r="E289" s="11">
-        <v>10</v>
+        <v>15</v>
       </c>
       <c r="F289" s="9" t="s">
         <v>28</v>
@@ -8621,7 +8621,7 @@
         <v>27</v>
       </c>
       <c r="E290" s="11">
-        <v>9</v>
+        <v>29</v>
       </c>
       <c r="F290" s="9" t="s">
         <v>28</v>
@@ -8644,7 +8644,7 @@
         <v>27</v>
       </c>
       <c r="E291" s="11">
-        <v>12</v>
+        <v>21</v>
       </c>
       <c r="F291" s="9" t="s">
         <v>28</v>
@@ -8667,7 +8667,7 @@
         <v>27</v>
       </c>
       <c r="E292" s="11">
-        <v>26</v>
+        <v>19</v>
       </c>
       <c r="F292" s="9" t="s">
         <v>28</v>
@@ -8690,7 +8690,7 @@
         <v>27</v>
       </c>
       <c r="E293" s="11">
-        <v>27</v>
+        <v>8</v>
       </c>
       <c r="F293" s="9" t="s">
         <v>28</v>
@@ -8713,7 +8713,7 @@
         <v>27</v>
       </c>
       <c r="E294" s="11">
-        <v>26</v>
+        <v>17</v>
       </c>
       <c r="F294" s="9" t="s">
         <v>28</v>
@@ -8736,7 +8736,7 @@
         <v>27</v>
       </c>
       <c r="E295" s="11">
-        <v>22</v>
+        <v>10</v>
       </c>
       <c r="F295" s="9" t="s">
         <v>28</v>
@@ -8759,7 +8759,7 @@
         <v>27</v>
       </c>
       <c r="E296" s="11">
-        <v>9</v>
+        <v>11</v>
       </c>
       <c r="F296" s="9" t="s">
         <v>28</v>
@@ -8782,7 +8782,7 @@
         <v>27</v>
       </c>
       <c r="E297" s="11">
-        <v>17</v>
+        <v>21</v>
       </c>
       <c r="F297" s="9" t="s">
         <v>28</v>
@@ -8805,7 +8805,7 @@
         <v>27</v>
       </c>
       <c r="E298" s="11">
-        <v>23</v>
+        <v>11</v>
       </c>
       <c r="F298" s="9" t="s">
         <v>28</v>
@@ -8828,7 +8828,7 @@
         <v>27</v>
       </c>
       <c r="E299" s="11">
-        <v>26</v>
+        <v>11</v>
       </c>
       <c r="F299" s="9" t="s">
         <v>28</v>
@@ -8851,7 +8851,7 @@
         <v>27</v>
       </c>
       <c r="E300" s="11">
-        <v>30</v>
+        <v>12</v>
       </c>
       <c r="F300" s="9" t="s">
         <v>28</v>
@@ -8874,7 +8874,7 @@
         <v>27</v>
       </c>
       <c r="E301" s="11">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="F301" s="9" t="s">
         <v>28</v>
@@ -8897,7 +8897,7 @@
         <v>27</v>
       </c>
       <c r="E302" s="11">
-        <v>14</v>
+        <v>18</v>
       </c>
       <c r="F302" s="9" t="s">
         <v>28</v>
@@ -8920,7 +8920,7 @@
         <v>27</v>
       </c>
       <c r="E303" s="11">
-        <v>30</v>
+        <v>9</v>
       </c>
       <c r="F303" s="9" t="s">
         <v>28</v>
@@ -8943,7 +8943,7 @@
         <v>27</v>
       </c>
       <c r="E304" s="11">
-        <v>27</v>
+        <v>13</v>
       </c>
       <c r="F304" s="9" t="s">
         <v>28</v>
@@ -8966,7 +8966,7 @@
         <v>27</v>
       </c>
       <c r="E305" s="11">
-        <v>25</v>
+        <v>31</v>
       </c>
       <c r="F305" s="9" t="s">
         <v>28</v>
@@ -8989,7 +8989,7 @@
         <v>27</v>
       </c>
       <c r="E306" s="11">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="F306" s="9" t="s">
         <v>28</v>
@@ -9012,7 +9012,7 @@
         <v>27</v>
       </c>
       <c r="E307" s="11">
-        <v>9</v>
+        <v>13</v>
       </c>
       <c r="F307" s="9" t="s">
         <v>28</v>
@@ -9035,7 +9035,7 @@
         <v>27</v>
       </c>
       <c r="E308" s="11">
-        <v>27</v>
+        <v>23</v>
       </c>
       <c r="F308" s="9" t="s">
         <v>28</v>
@@ -9058,7 +9058,7 @@
         <v>27</v>
       </c>
       <c r="E309" s="11">
-        <v>20</v>
+        <v>30</v>
       </c>
       <c r="F309" s="9" t="s">
         <v>28</v>
@@ -9081,7 +9081,7 @@
         <v>27</v>
       </c>
       <c r="E310" s="11">
-        <v>29</v>
+        <v>8</v>
       </c>
       <c r="F310" s="9" t="s">
         <v>28</v>
@@ -9104,7 +9104,7 @@
         <v>27</v>
       </c>
       <c r="E311" s="11">
-        <v>23</v>
+        <v>19</v>
       </c>
       <c r="F311" s="9" t="s">
         <v>28</v>
@@ -9127,7 +9127,7 @@
         <v>27</v>
       </c>
       <c r="E312" s="11">
-        <v>17</v>
+        <v>15</v>
       </c>
       <c r="F312" s="9" t="s">
         <v>28</v>
@@ -9150,7 +9150,7 @@
         <v>27</v>
       </c>
       <c r="E313" s="11">
-        <v>23</v>
+        <v>10</v>
       </c>
       <c r="F313" s="9" t="s">
         <v>28</v>
@@ -9173,7 +9173,7 @@
         <v>27</v>
       </c>
       <c r="E314" s="11">
-        <v>21</v>
+        <v>24</v>
       </c>
       <c r="F314" s="9" t="s">
         <v>28</v>
@@ -9196,7 +9196,7 @@
         <v>27</v>
       </c>
       <c r="E315" s="11">
-        <v>29</v>
+        <v>18</v>
       </c>
       <c r="F315" s="9" t="s">
         <v>28</v>
@@ -9242,7 +9242,7 @@
         <v>27</v>
       </c>
       <c r="E317" s="11">
-        <v>30</v>
+        <v>22</v>
       </c>
       <c r="F317" s="9" t="s">
         <v>28</v>
@@ -9265,7 +9265,7 @@
         <v>27</v>
       </c>
       <c r="E318" s="11">
-        <v>15</v>
+        <v>17</v>
       </c>
       <c r="F318" s="9" t="s">
         <v>28</v>
@@ -9288,7 +9288,7 @@
         <v>27</v>
       </c>
       <c r="E319" s="11">
-        <v>20</v>
+        <v>24</v>
       </c>
       <c r="F319" s="9" t="s">
         <v>28</v>
@@ -9311,7 +9311,7 @@
         <v>27</v>
       </c>
       <c r="E320" s="11">
-        <v>27</v>
+        <v>20</v>
       </c>
       <c r="F320" s="9" t="s">
         <v>28</v>
@@ -9334,7 +9334,7 @@
         <v>27</v>
       </c>
       <c r="E321" s="11">
-        <v>11</v>
+        <v>17</v>
       </c>
       <c r="F321" s="9" t="s">
         <v>28</v>
@@ -9357,7 +9357,7 @@
         <v>27</v>
       </c>
       <c r="E322" s="11">
-        <v>30</v>
+        <v>20</v>
       </c>
       <c r="F322" s="9" t="s">
         <v>28</v>
@@ -9403,7 +9403,7 @@
         <v>27</v>
       </c>
       <c r="E324" s="11">
-        <v>27</v>
+        <v>18</v>
       </c>
       <c r="F324" s="9" t="s">
         <v>28</v>
@@ -9426,7 +9426,7 @@
         <v>27</v>
       </c>
       <c r="E325" s="11">
-        <v>30</v>
+        <v>24</v>
       </c>
       <c r="F325" s="9" t="s">
         <v>28</v>
@@ -9449,7 +9449,7 @@
         <v>27</v>
       </c>
       <c r="E326" s="11">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="F326" s="9" t="s">
         <v>28</v>
@@ -9472,7 +9472,7 @@
         <v>27</v>
       </c>
       <c r="E327" s="11">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="F327" s="9" t="s">
         <v>28</v>
@@ -9495,7 +9495,7 @@
         <v>27</v>
       </c>
       <c r="E328" s="11">
-        <v>16</v>
+        <v>28</v>
       </c>
       <c r="F328" s="9" t="s">
         <v>28</v>
@@ -9518,7 +9518,7 @@
         <v>27</v>
       </c>
       <c r="E329" s="11">
-        <v>9</v>
+        <v>24</v>
       </c>
       <c r="F329" s="9" t="s">
         <v>28</v>
@@ -9541,7 +9541,7 @@
         <v>27</v>
       </c>
       <c r="E330" s="11">
-        <v>15</v>
+        <v>13</v>
       </c>
       <c r="F330" s="9" t="s">
         <v>28</v>
@@ -9564,7 +9564,7 @@
         <v>27</v>
       </c>
       <c r="E331" s="11">
-        <v>29</v>
+        <v>8</v>
       </c>
       <c r="F331" s="9" t="s">
         <v>28</v>
@@ -9587,7 +9587,7 @@
         <v>27</v>
       </c>
       <c r="E332" s="11">
-        <v>21</v>
+        <v>15</v>
       </c>
       <c r="F332" s="9" t="s">
         <v>28</v>
@@ -9610,7 +9610,7 @@
         <v>27</v>
       </c>
       <c r="E333" s="11">
-        <v>31</v>
+        <v>24</v>
       </c>
       <c r="F333" s="9" t="s">
         <v>28</v>
@@ -9633,7 +9633,7 @@
         <v>27</v>
       </c>
       <c r="E334" s="11">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="F334" s="9" t="s">
         <v>28</v>
@@ -9656,7 +9656,7 @@
         <v>27</v>
       </c>
       <c r="E335" s="11">
-        <v>25</v>
+        <v>18</v>
       </c>
       <c r="F335" s="9" t="s">
         <v>28</v>
@@ -9679,7 +9679,7 @@
         <v>27</v>
       </c>
       <c r="E336" s="11">
-        <v>24</v>
+        <v>22</v>
       </c>
       <c r="F336" s="9" t="s">
         <v>28</v>
@@ -9702,7 +9702,7 @@
         <v>27</v>
       </c>
       <c r="E337" s="11">
-        <v>12</v>
+        <v>19</v>
       </c>
       <c r="F337" s="9" t="s">
         <v>28</v>
@@ -9725,7 +9725,7 @@
         <v>27</v>
       </c>
       <c r="E338" s="11">
-        <v>22</v>
+        <v>28</v>
       </c>
       <c r="F338" s="9" t="s">
         <v>28</v>
@@ -9748,7 +9748,7 @@
         <v>27</v>
       </c>
       <c r="E339" s="11">
-        <v>11</v>
+        <v>30</v>
       </c>
       <c r="F339" s="9" t="s">
         <v>28</v>
@@ -9771,7 +9771,7 @@
         <v>27</v>
       </c>
       <c r="E340" s="11">
-        <v>22</v>
+        <v>20</v>
       </c>
       <c r="F340" s="9" t="s">
         <v>28</v>
@@ -9794,7 +9794,7 @@
         <v>27</v>
       </c>
       <c r="E341" s="11">
-        <v>11</v>
+        <v>28</v>
       </c>
       <c r="F341" s="9" t="s">
         <v>28</v>
@@ -9817,7 +9817,7 @@
         <v>27</v>
       </c>
       <c r="E342" s="11">
-        <v>21</v>
+        <v>13</v>
       </c>
       <c r="F342" s="9" t="s">
         <v>28</v>
@@ -9840,7 +9840,7 @@
         <v>27</v>
       </c>
       <c r="E343" s="11">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="F343" s="9" t="s">
         <v>28</v>
@@ -9863,7 +9863,7 @@
         <v>27</v>
       </c>
       <c r="E344" s="11">
-        <v>21</v>
+        <v>23</v>
       </c>
       <c r="F344" s="9" t="s">
         <v>28</v>
@@ -9886,7 +9886,7 @@
         <v>27</v>
       </c>
       <c r="E345" s="11">
-        <v>17</v>
+        <v>27</v>
       </c>
       <c r="F345" s="9" t="s">
         <v>28</v>
@@ -9909,7 +9909,7 @@
         <v>27</v>
       </c>
       <c r="E346" s="11">
-        <v>25</v>
+        <v>10</v>
       </c>
       <c r="F346" s="9" t="s">
         <v>28</v>
@@ -9932,7 +9932,7 @@
         <v>27</v>
       </c>
       <c r="E347" s="11">
-        <v>9</v>
+        <v>27</v>
       </c>
       <c r="F347" s="9" t="s">
         <v>28</v>
@@ -9955,7 +9955,7 @@
         <v>27</v>
       </c>
       <c r="E348" s="11">
-        <v>31</v>
+        <v>20</v>
       </c>
       <c r="F348" s="9" t="s">
         <v>28</v>
@@ -9978,7 +9978,7 @@
         <v>27</v>
       </c>
       <c r="E349" s="11">
-        <v>31</v>
+        <v>8</v>
       </c>
       <c r="F349" s="9" t="s">
         <v>28</v>
@@ -10001,7 +10001,7 @@
         <v>27</v>
       </c>
       <c r="E350" s="11">
-        <v>27</v>
+        <v>23</v>
       </c>
       <c r="F350" s="9" t="s">
         <v>28</v>
@@ -10024,7 +10024,7 @@
         <v>27</v>
       </c>
       <c r="E351" s="11">
-        <v>26</v>
+        <v>28</v>
       </c>
       <c r="F351" s="9" t="s">
         <v>28</v>
@@ -10047,7 +10047,7 @@
         <v>27</v>
       </c>
       <c r="E352" s="11">
-        <v>24</v>
+        <v>13</v>
       </c>
       <c r="F352" s="9" t="s">
         <v>28</v>
@@ -10070,7 +10070,7 @@
         <v>27</v>
       </c>
       <c r="E353" s="11">
-        <v>8</v>
+        <v>11</v>
       </c>
       <c r="F353" s="9" t="s">
         <v>28</v>
@@ -10093,7 +10093,7 @@
         <v>27</v>
       </c>
       <c r="E354" s="11">
-        <v>31</v>
+        <v>12</v>
       </c>
       <c r="F354" s="9" t="s">
         <v>28</v>
@@ -10116,7 +10116,7 @@
         <v>27</v>
       </c>
       <c r="E355" s="11">
-        <v>17</v>
+        <v>29</v>
       </c>
       <c r="F355" s="9" t="s">
         <v>28</v>
@@ -10139,7 +10139,7 @@
         <v>27</v>
       </c>
       <c r="E356" s="11">
-        <v>15</v>
+        <v>30</v>
       </c>
       <c r="F356" s="9" t="s">
         <v>28</v>
@@ -10162,7 +10162,7 @@
         <v>27</v>
       </c>
       <c r="E357" s="11">
-        <v>12</v>
+        <v>15</v>
       </c>
       <c r="F357" s="9" t="s">
         <v>28</v>
@@ -10185,7 +10185,7 @@
         <v>27</v>
       </c>
       <c r="E358" s="11">
-        <v>17</v>
+        <v>12</v>
       </c>
       <c r="F358" s="9" t="s">
         <v>28</v>
@@ -10208,7 +10208,7 @@
         <v>27</v>
       </c>
       <c r="E359" s="11">
-        <v>27</v>
+        <v>8</v>
       </c>
       <c r="F359" s="9" t="s">
         <v>28</v>
@@ -10231,7 +10231,7 @@
         <v>27</v>
       </c>
       <c r="E360" s="11">
-        <v>22</v>
+        <v>13</v>
       </c>
       <c r="F360" s="9" t="s">
         <v>28</v>
@@ -10254,7 +10254,7 @@
         <v>27</v>
       </c>
       <c r="E361" s="11">
-        <v>17</v>
+        <v>30</v>
       </c>
       <c r="F361" s="9" t="s">
         <v>28</v>
@@ -10277,7 +10277,7 @@
         <v>27</v>
       </c>
       <c r="E362" s="11">
-        <v>22</v>
+        <v>14</v>
       </c>
       <c r="F362" s="9" t="s">
         <v>28</v>
@@ -10300,7 +10300,7 @@
         <v>27</v>
       </c>
       <c r="E363" s="11">
-        <v>16</v>
+        <v>13</v>
       </c>
       <c r="F363" s="9" t="s">
         <v>28</v>
@@ -10323,7 +10323,7 @@
         <v>27</v>
       </c>
       <c r="E364" s="11">
-        <v>29</v>
+        <v>27</v>
       </c>
       <c r="F364" s="9" t="s">
         <v>28</v>
@@ -10346,7 +10346,7 @@
         <v>27</v>
       </c>
       <c r="E365" s="11">
-        <v>14</v>
+        <v>23</v>
       </c>
       <c r="F365" s="9" t="s">
         <v>28</v>
@@ -10369,7 +10369,7 @@
         <v>27</v>
       </c>
       <c r="E366" s="11">
-        <v>14</v>
+        <v>31</v>
       </c>
       <c r="F366" s="9" t="s">
         <v>28</v>
@@ -10392,7 +10392,7 @@
         <v>27</v>
       </c>
       <c r="E367" s="11">
-        <v>12</v>
+        <v>18</v>
       </c>
       <c r="F367" s="9" t="s">
         <v>28</v>
@@ -10415,7 +10415,7 @@
         <v>27</v>
       </c>
       <c r="E368" s="11">
-        <v>17</v>
+        <v>15</v>
       </c>
       <c r="F368" s="9" t="s">
         <v>28</v>
@@ -10438,7 +10438,7 @@
         <v>27</v>
       </c>
       <c r="E369" s="11">
-        <v>30</v>
+        <v>24</v>
       </c>
       <c r="F369" s="9" t="s">
         <v>28</v>
@@ -10461,7 +10461,7 @@
         <v>27</v>
       </c>
       <c r="E370" s="11">
-        <v>21</v>
+        <v>28</v>
       </c>
       <c r="F370" s="9" t="s">
         <v>28</v>
@@ -10484,7 +10484,7 @@
         <v>27</v>
       </c>
       <c r="E371" s="11">
-        <v>24</v>
+        <v>13</v>
       </c>
       <c r="F371" s="9" t="s">
         <v>28</v>
@@ -10507,7 +10507,7 @@
         <v>27</v>
       </c>
       <c r="E372" s="11">
-        <v>24</v>
+        <v>13</v>
       </c>
       <c r="F372" s="9" t="s">
         <v>28</v>
@@ -10530,7 +10530,7 @@
         <v>27</v>
       </c>
       <c r="E373" s="11">
-        <v>10</v>
+        <v>19</v>
       </c>
       <c r="F373" s="9" t="s">
         <v>28</v>
@@ -10553,7 +10553,7 @@
         <v>27</v>
       </c>
       <c r="E374" s="11">
-        <v>29</v>
+        <v>9</v>
       </c>
       <c r="F374" s="9" t="s">
         <v>28</v>
@@ -10576,7 +10576,7 @@
         <v>27</v>
       </c>
       <c r="E375" s="11">
-        <v>24</v>
+        <v>11</v>
       </c>
       <c r="F375" s="9" t="s">
         <v>28</v>
@@ -10599,7 +10599,7 @@
         <v>27</v>
       </c>
       <c r="E376" s="11">
-        <v>20</v>
+        <v>29</v>
       </c>
       <c r="F376" s="9" t="s">
         <v>28</v>
@@ -10622,7 +10622,7 @@
         <v>27</v>
       </c>
       <c r="E377" s="11">
-        <v>13</v>
+        <v>8</v>
       </c>
       <c r="F377" s="9" t="s">
         <v>28</v>
@@ -10645,7 +10645,7 @@
         <v>27</v>
       </c>
       <c r="E378" s="11">
-        <v>11</v>
+        <v>26</v>
       </c>
       <c r="F378" s="9" t="s">
         <v>28</v>
@@ -10668,7 +10668,7 @@
         <v>27</v>
       </c>
       <c r="E379" s="11">
-        <v>10</v>
+        <v>23</v>
       </c>
       <c r="F379" s="9" t="s">
         <v>28</v>
@@ -10691,7 +10691,7 @@
         <v>27</v>
       </c>
       <c r="E380" s="11">
-        <v>18</v>
+        <v>16</v>
       </c>
       <c r="F380" s="9" t="s">
         <v>28</v>
@@ -10714,7 +10714,7 @@
         <v>27</v>
       </c>
       <c r="E381" s="11">
-        <v>13</v>
+        <v>27</v>
       </c>
       <c r="F381" s="9" t="s">
         <v>28</v>
@@ -10737,7 +10737,7 @@
         <v>27</v>
       </c>
       <c r="E382" s="11">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="F382" s="9" t="s">
         <v>28</v>
@@ -10760,7 +10760,7 @@
         <v>27</v>
       </c>
       <c r="E383" s="11">
-        <v>15</v>
+        <v>20</v>
       </c>
       <c r="F383" s="9" t="s">
         <v>28</v>
@@ -10783,7 +10783,7 @@
         <v>27</v>
       </c>
       <c r="E384" s="11">
-        <v>22</v>
+        <v>15</v>
       </c>
       <c r="F384" s="9" t="s">
         <v>28</v>
@@ -10806,7 +10806,7 @@
         <v>27</v>
       </c>
       <c r="E385" s="11">
-        <v>28</v>
+        <v>14</v>
       </c>
       <c r="F385" s="9" t="s">
         <v>28</v>
@@ -10829,7 +10829,7 @@
         <v>27</v>
       </c>
       <c r="E386" s="11">
-        <v>21</v>
+        <v>23</v>
       </c>
       <c r="F386" s="9" t="s">
         <v>28</v>
@@ -10852,7 +10852,7 @@
         <v>27</v>
       </c>
       <c r="E387" s="11">
-        <v>25</v>
+        <v>31</v>
       </c>
       <c r="F387" s="9" t="s">
         <v>28</v>
@@ -10875,7 +10875,7 @@
         <v>27</v>
       </c>
       <c r="E388" s="11">
-        <v>16</v>
+        <v>18</v>
       </c>
       <c r="F388" s="9" t="s">
         <v>28</v>
@@ -10898,7 +10898,7 @@
         <v>27</v>
       </c>
       <c r="E389" s="11">
-        <v>20</v>
+        <v>26</v>
       </c>
       <c r="F389" s="9" t="s">
         <v>28</v>
@@ -10921,7 +10921,7 @@
         <v>27</v>
       </c>
       <c r="E390" s="11">
-        <v>19</v>
+        <v>13</v>
       </c>
       <c r="F390" s="9" t="s">
         <v>28</v>
@@ -10944,7 +10944,7 @@
         <v>27</v>
       </c>
       <c r="E391" s="11">
-        <v>30</v>
+        <v>17</v>
       </c>
       <c r="F391" s="9" t="s">
         <v>28</v>
@@ -10967,7 +10967,7 @@
         <v>27</v>
       </c>
       <c r="E392" s="11">
-        <v>26</v>
+        <v>18</v>
       </c>
       <c r="F392" s="9" t="s">
         <v>28</v>
@@ -11013,7 +11013,7 @@
         <v>27</v>
       </c>
       <c r="E394" s="11">
-        <v>14</v>
+        <v>25</v>
       </c>
       <c r="F394" s="9" t="s">
         <v>28</v>
@@ -11036,7 +11036,7 @@
         <v>27</v>
       </c>
       <c r="E395" s="11">
-        <v>29</v>
+        <v>20</v>
       </c>
       <c r="F395" s="9" t="s">
         <v>28</v>
@@ -11059,7 +11059,7 @@
         <v>27</v>
       </c>
       <c r="E396" s="11">
-        <v>18</v>
+        <v>31</v>
       </c>
       <c r="F396" s="9" t="s">
         <v>28</v>
@@ -11082,7 +11082,7 @@
         <v>27</v>
       </c>
       <c r="E397" s="11">
-        <v>31</v>
+        <v>22</v>
       </c>
       <c r="F397" s="9" t="s">
         <v>28</v>
@@ -11105,7 +11105,7 @@
         <v>27</v>
       </c>
       <c r="E398" s="11">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="F398" s="9" t="s">
         <v>28</v>
@@ -11128,7 +11128,7 @@
         <v>27</v>
       </c>
       <c r="E399" s="11">
-        <v>19</v>
+        <v>8</v>
       </c>
       <c r="F399" s="9" t="s">
         <v>28</v>
@@ -11151,7 +11151,7 @@
         <v>27</v>
       </c>
       <c r="E400" s="11">
-        <v>25</v>
+        <v>20</v>
       </c>
       <c r="F400" s="9" t="s">
         <v>28</v>
@@ -11174,7 +11174,7 @@
         <v>27</v>
       </c>
       <c r="E401" s="11">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="F401" s="9" t="s">
         <v>28</v>

</xml_diff>

<commit_message>
fix(profile): fix missing hasActivity variable and add fallback guest profile data to resolve blank Profile page issue
</commit_message>
<xml_diff>
--- a/all-test-reports/selenium/selenium_e2e_test_report.xlsx
+++ b/all-test-reports/selenium/selenium_e2e_test_report.xlsx
@@ -35,7 +35,7 @@
     <t>Execution Date</t>
   </si>
   <si>
-    <t>28/7/2026, 11:31:46 am</t>
+    <t>28/7/2026, 11:37:58 am</t>
   </si>
   <si>
     <t>Browser / Mode</t>
@@ -98,7 +98,7 @@
     <t>PASS</t>
   </si>
   <si>
-    <t>11:31:46 am</t>
+    <t>11:37:58 am</t>
   </si>
   <si>
     <t>N/A</t>
@@ -1997,7 +1997,7 @@
         <v>27</v>
       </c>
       <c r="E2" s="11">
-        <v>26</v>
+        <v>23</v>
       </c>
       <c r="F2" s="9" t="s">
         <v>28</v>
@@ -2020,7 +2020,7 @@
         <v>27</v>
       </c>
       <c r="E3" s="11">
-        <v>20</v>
+        <v>17</v>
       </c>
       <c r="F3" s="9" t="s">
         <v>28</v>
@@ -2043,7 +2043,7 @@
         <v>27</v>
       </c>
       <c r="E4" s="11">
-        <v>18</v>
+        <v>26</v>
       </c>
       <c r="F4" s="9" t="s">
         <v>28</v>
@@ -2066,7 +2066,7 @@
         <v>27</v>
       </c>
       <c r="E5" s="11">
-        <v>14</v>
+        <v>22</v>
       </c>
       <c r="F5" s="9" t="s">
         <v>28</v>
@@ -2089,7 +2089,7 @@
         <v>27</v>
       </c>
       <c r="E6" s="11">
-        <v>29</v>
+        <v>26</v>
       </c>
       <c r="F6" s="9" t="s">
         <v>28</v>
@@ -2112,7 +2112,7 @@
         <v>27</v>
       </c>
       <c r="E7" s="11">
-        <v>24</v>
+        <v>31</v>
       </c>
       <c r="F7" s="9" t="s">
         <v>28</v>
@@ -2135,7 +2135,7 @@
         <v>27</v>
       </c>
       <c r="E8" s="11">
-        <v>31</v>
+        <v>22</v>
       </c>
       <c r="F8" s="9" t="s">
         <v>28</v>
@@ -2158,7 +2158,7 @@
         <v>27</v>
       </c>
       <c r="E9" s="11">
-        <v>21</v>
+        <v>9</v>
       </c>
       <c r="F9" s="9" t="s">
         <v>28</v>
@@ -2181,7 +2181,7 @@
         <v>27</v>
       </c>
       <c r="E10" s="11">
-        <v>31</v>
+        <v>12</v>
       </c>
       <c r="F10" s="9" t="s">
         <v>28</v>
@@ -2204,7 +2204,7 @@
         <v>27</v>
       </c>
       <c r="E11" s="11">
-        <v>19</v>
+        <v>11</v>
       </c>
       <c r="F11" s="9" t="s">
         <v>28</v>
@@ -2227,7 +2227,7 @@
         <v>27</v>
       </c>
       <c r="E12" s="11">
-        <v>25</v>
+        <v>13</v>
       </c>
       <c r="F12" s="9" t="s">
         <v>28</v>
@@ -2250,7 +2250,7 @@
         <v>27</v>
       </c>
       <c r="E13" s="11">
-        <v>30</v>
+        <v>17</v>
       </c>
       <c r="F13" s="9" t="s">
         <v>28</v>
@@ -2273,7 +2273,7 @@
         <v>27</v>
       </c>
       <c r="E14" s="11">
-        <v>19</v>
+        <v>16</v>
       </c>
       <c r="F14" s="9" t="s">
         <v>28</v>
@@ -2296,7 +2296,7 @@
         <v>27</v>
       </c>
       <c r="E15" s="11">
-        <v>26</v>
+        <v>20</v>
       </c>
       <c r="F15" s="9" t="s">
         <v>28</v>
@@ -2319,7 +2319,7 @@
         <v>27</v>
       </c>
       <c r="E16" s="11">
-        <v>17</v>
+        <v>19</v>
       </c>
       <c r="F16" s="9" t="s">
         <v>28</v>
@@ -2342,7 +2342,7 @@
         <v>27</v>
       </c>
       <c r="E17" s="11">
-        <v>10</v>
+        <v>26</v>
       </c>
       <c r="F17" s="9" t="s">
         <v>28</v>
@@ -2365,7 +2365,7 @@
         <v>27</v>
       </c>
       <c r="E18" s="11">
-        <v>28</v>
+        <v>20</v>
       </c>
       <c r="F18" s="9" t="s">
         <v>28</v>
@@ -2388,7 +2388,7 @@
         <v>27</v>
       </c>
       <c r="E19" s="11">
-        <v>25</v>
+        <v>10</v>
       </c>
       <c r="F19" s="9" t="s">
         <v>28</v>
@@ -2434,7 +2434,7 @@
         <v>27</v>
       </c>
       <c r="E21" s="11">
-        <v>15</v>
+        <v>11</v>
       </c>
       <c r="F21" s="9" t="s">
         <v>28</v>
@@ -2457,7 +2457,7 @@
         <v>27</v>
       </c>
       <c r="E22" s="11">
-        <v>9</v>
+        <v>25</v>
       </c>
       <c r="F22" s="9" t="s">
         <v>28</v>
@@ -2480,7 +2480,7 @@
         <v>27</v>
       </c>
       <c r="E23" s="11">
-        <v>26</v>
+        <v>29</v>
       </c>
       <c r="F23" s="9" t="s">
         <v>28</v>
@@ -2503,7 +2503,7 @@
         <v>27</v>
       </c>
       <c r="E24" s="11">
-        <v>20</v>
+        <v>16</v>
       </c>
       <c r="F24" s="9" t="s">
         <v>28</v>
@@ -2549,7 +2549,7 @@
         <v>27</v>
       </c>
       <c r="E26" s="11">
-        <v>9</v>
+        <v>28</v>
       </c>
       <c r="F26" s="9" t="s">
         <v>28</v>
@@ -2572,7 +2572,7 @@
         <v>27</v>
       </c>
       <c r="E27" s="11">
-        <v>10</v>
+        <v>17</v>
       </c>
       <c r="F27" s="9" t="s">
         <v>28</v>
@@ -2595,7 +2595,7 @@
         <v>27</v>
       </c>
       <c r="E28" s="11">
-        <v>21</v>
+        <v>16</v>
       </c>
       <c r="F28" s="9" t="s">
         <v>28</v>
@@ -2618,7 +2618,7 @@
         <v>27</v>
       </c>
       <c r="E29" s="11">
-        <v>14</v>
+        <v>29</v>
       </c>
       <c r="F29" s="9" t="s">
         <v>28</v>
@@ -2641,7 +2641,7 @@
         <v>27</v>
       </c>
       <c r="E30" s="11">
-        <v>17</v>
+        <v>12</v>
       </c>
       <c r="F30" s="9" t="s">
         <v>28</v>
@@ -2664,7 +2664,7 @@
         <v>27</v>
       </c>
       <c r="E31" s="11">
-        <v>10</v>
+        <v>20</v>
       </c>
       <c r="F31" s="9" t="s">
         <v>28</v>
@@ -2687,7 +2687,7 @@
         <v>27</v>
       </c>
       <c r="E32" s="11">
-        <v>14</v>
+        <v>16</v>
       </c>
       <c r="F32" s="9" t="s">
         <v>28</v>
@@ -2710,7 +2710,7 @@
         <v>27</v>
       </c>
       <c r="E33" s="11">
-        <v>24</v>
+        <v>12</v>
       </c>
       <c r="F33" s="9" t="s">
         <v>28</v>
@@ -2733,7 +2733,7 @@
         <v>27</v>
       </c>
       <c r="E34" s="11">
-        <v>18</v>
+        <v>12</v>
       </c>
       <c r="F34" s="9" t="s">
         <v>28</v>
@@ -2756,7 +2756,7 @@
         <v>27</v>
       </c>
       <c r="E35" s="11">
-        <v>29</v>
+        <v>20</v>
       </c>
       <c r="F35" s="9" t="s">
         <v>28</v>
@@ -2779,7 +2779,7 @@
         <v>27</v>
       </c>
       <c r="E36" s="11">
-        <v>21</v>
+        <v>24</v>
       </c>
       <c r="F36" s="9" t="s">
         <v>28</v>
@@ -2802,7 +2802,7 @@
         <v>27</v>
       </c>
       <c r="E37" s="11">
-        <v>27</v>
+        <v>23</v>
       </c>
       <c r="F37" s="9" t="s">
         <v>28</v>
@@ -2825,7 +2825,7 @@
         <v>27</v>
       </c>
       <c r="E38" s="11">
-        <v>31</v>
+        <v>29</v>
       </c>
       <c r="F38" s="9" t="s">
         <v>28</v>
@@ -2848,7 +2848,7 @@
         <v>27</v>
       </c>
       <c r="E39" s="11">
-        <v>12</v>
+        <v>26</v>
       </c>
       <c r="F39" s="9" t="s">
         <v>28</v>
@@ -2871,7 +2871,7 @@
         <v>27</v>
       </c>
       <c r="E40" s="11">
-        <v>27</v>
+        <v>25</v>
       </c>
       <c r="F40" s="9" t="s">
         <v>28</v>
@@ -2894,7 +2894,7 @@
         <v>27</v>
       </c>
       <c r="E41" s="11">
-        <v>25</v>
+        <v>11</v>
       </c>
       <c r="F41" s="9" t="s">
         <v>28</v>
@@ -2917,7 +2917,7 @@
         <v>27</v>
       </c>
       <c r="E42" s="11">
-        <v>28</v>
+        <v>14</v>
       </c>
       <c r="F42" s="9" t="s">
         <v>28</v>
@@ -2940,7 +2940,7 @@
         <v>27</v>
       </c>
       <c r="E43" s="11">
-        <v>12</v>
+        <v>21</v>
       </c>
       <c r="F43" s="9" t="s">
         <v>28</v>
@@ -2986,7 +2986,7 @@
         <v>27</v>
       </c>
       <c r="E45" s="11">
-        <v>18</v>
+        <v>10</v>
       </c>
       <c r="F45" s="9" t="s">
         <v>28</v>
@@ -3009,7 +3009,7 @@
         <v>27</v>
       </c>
       <c r="E46" s="11">
-        <v>14</v>
+        <v>23</v>
       </c>
       <c r="F46" s="9" t="s">
         <v>28</v>
@@ -3032,7 +3032,7 @@
         <v>27</v>
       </c>
       <c r="E47" s="11">
-        <v>19</v>
+        <v>27</v>
       </c>
       <c r="F47" s="9" t="s">
         <v>28</v>
@@ -3055,7 +3055,7 @@
         <v>27</v>
       </c>
       <c r="E48" s="11">
-        <v>11</v>
+        <v>30</v>
       </c>
       <c r="F48" s="9" t="s">
         <v>28</v>
@@ -3078,7 +3078,7 @@
         <v>27</v>
       </c>
       <c r="E49" s="11">
-        <v>13</v>
+        <v>16</v>
       </c>
       <c r="F49" s="9" t="s">
         <v>28</v>
@@ -3101,7 +3101,7 @@
         <v>27</v>
       </c>
       <c r="E50" s="11">
-        <v>28</v>
+        <v>31</v>
       </c>
       <c r="F50" s="9" t="s">
         <v>28</v>
@@ -3124,7 +3124,7 @@
         <v>27</v>
       </c>
       <c r="E51" s="11">
-        <v>24</v>
+        <v>16</v>
       </c>
       <c r="F51" s="9" t="s">
         <v>28</v>
@@ -3147,7 +3147,7 @@
         <v>27</v>
       </c>
       <c r="E52" s="11">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="F52" s="9" t="s">
         <v>28</v>
@@ -3170,7 +3170,7 @@
         <v>27</v>
       </c>
       <c r="E53" s="11">
-        <v>25</v>
+        <v>27</v>
       </c>
       <c r="F53" s="9" t="s">
         <v>28</v>
@@ -3193,7 +3193,7 @@
         <v>27</v>
       </c>
       <c r="E54" s="11">
-        <v>30</v>
+        <v>15</v>
       </c>
       <c r="F54" s="9" t="s">
         <v>28</v>
@@ -3216,7 +3216,7 @@
         <v>27</v>
       </c>
       <c r="E55" s="11">
-        <v>11</v>
+        <v>8</v>
       </c>
       <c r="F55" s="9" t="s">
         <v>28</v>
@@ -3239,7 +3239,7 @@
         <v>27</v>
       </c>
       <c r="E56" s="11">
-        <v>11</v>
+        <v>8</v>
       </c>
       <c r="F56" s="9" t="s">
         <v>28</v>
@@ -3262,7 +3262,7 @@
         <v>27</v>
       </c>
       <c r="E57" s="11">
-        <v>15</v>
+        <v>22</v>
       </c>
       <c r="F57" s="9" t="s">
         <v>28</v>
@@ -3285,7 +3285,7 @@
         <v>27</v>
       </c>
       <c r="E58" s="11">
-        <v>19</v>
+        <v>15</v>
       </c>
       <c r="F58" s="9" t="s">
         <v>28</v>
@@ -3308,7 +3308,7 @@
         <v>27</v>
       </c>
       <c r="E59" s="11">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="F59" s="9" t="s">
         <v>28</v>
@@ -3331,7 +3331,7 @@
         <v>27</v>
       </c>
       <c r="E60" s="11">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="F60" s="9" t="s">
         <v>28</v>
@@ -3354,7 +3354,7 @@
         <v>27</v>
       </c>
       <c r="E61" s="11">
-        <v>13</v>
+        <v>29</v>
       </c>
       <c r="F61" s="9" t="s">
         <v>28</v>
@@ -3377,7 +3377,7 @@
         <v>27</v>
       </c>
       <c r="E62" s="11">
-        <v>20</v>
+        <v>10</v>
       </c>
       <c r="F62" s="9" t="s">
         <v>28</v>
@@ -3400,7 +3400,7 @@
         <v>27</v>
       </c>
       <c r="E63" s="11">
-        <v>25</v>
+        <v>15</v>
       </c>
       <c r="F63" s="9" t="s">
         <v>28</v>
@@ -3423,7 +3423,7 @@
         <v>27</v>
       </c>
       <c r="E64" s="11">
-        <v>16</v>
+        <v>23</v>
       </c>
       <c r="F64" s="9" t="s">
         <v>28</v>
@@ -3446,7 +3446,7 @@
         <v>27</v>
       </c>
       <c r="E65" s="11">
-        <v>17</v>
+        <v>10</v>
       </c>
       <c r="F65" s="9" t="s">
         <v>28</v>
@@ -3469,7 +3469,7 @@
         <v>27</v>
       </c>
       <c r="E66" s="11">
-        <v>17</v>
+        <v>24</v>
       </c>
       <c r="F66" s="9" t="s">
         <v>28</v>
@@ -3492,7 +3492,7 @@
         <v>27</v>
       </c>
       <c r="E67" s="11">
-        <v>22</v>
+        <v>11</v>
       </c>
       <c r="F67" s="9" t="s">
         <v>28</v>
@@ -3515,7 +3515,7 @@
         <v>27</v>
       </c>
       <c r="E68" s="11">
-        <v>23</v>
+        <v>12</v>
       </c>
       <c r="F68" s="9" t="s">
         <v>28</v>
@@ -3538,7 +3538,7 @@
         <v>27</v>
       </c>
       <c r="E69" s="11">
-        <v>22</v>
+        <v>19</v>
       </c>
       <c r="F69" s="9" t="s">
         <v>28</v>
@@ -3561,7 +3561,7 @@
         <v>27</v>
       </c>
       <c r="E70" s="11">
-        <v>8</v>
+        <v>11</v>
       </c>
       <c r="F70" s="9" t="s">
         <v>28</v>
@@ -3584,7 +3584,7 @@
         <v>27</v>
       </c>
       <c r="E71" s="11">
-        <v>11</v>
+        <v>25</v>
       </c>
       <c r="F71" s="9" t="s">
         <v>28</v>
@@ -3607,7 +3607,7 @@
         <v>27</v>
       </c>
       <c r="E72" s="11">
-        <v>26</v>
+        <v>16</v>
       </c>
       <c r="F72" s="9" t="s">
         <v>28</v>
@@ -3630,7 +3630,7 @@
         <v>27</v>
       </c>
       <c r="E73" s="11">
-        <v>17</v>
+        <v>31</v>
       </c>
       <c r="F73" s="9" t="s">
         <v>28</v>
@@ -3653,7 +3653,7 @@
         <v>27</v>
       </c>
       <c r="E74" s="11">
-        <v>17</v>
+        <v>21</v>
       </c>
       <c r="F74" s="9" t="s">
         <v>28</v>
@@ -3676,7 +3676,7 @@
         <v>27</v>
       </c>
       <c r="E75" s="11">
-        <v>22</v>
+        <v>13</v>
       </c>
       <c r="F75" s="9" t="s">
         <v>28</v>
@@ -3699,7 +3699,7 @@
         <v>27</v>
       </c>
       <c r="E76" s="11">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="F76" s="9" t="s">
         <v>28</v>
@@ -3722,7 +3722,7 @@
         <v>27</v>
       </c>
       <c r="E77" s="11">
-        <v>28</v>
+        <v>13</v>
       </c>
       <c r="F77" s="9" t="s">
         <v>28</v>
@@ -3745,7 +3745,7 @@
         <v>27</v>
       </c>
       <c r="E78" s="11">
-        <v>27</v>
+        <v>19</v>
       </c>
       <c r="F78" s="9" t="s">
         <v>28</v>
@@ -3768,7 +3768,7 @@
         <v>27</v>
       </c>
       <c r="E79" s="11">
-        <v>29</v>
+        <v>9</v>
       </c>
       <c r="F79" s="9" t="s">
         <v>28</v>
@@ -3791,7 +3791,7 @@
         <v>27</v>
       </c>
       <c r="E80" s="11">
-        <v>25</v>
+        <v>9</v>
       </c>
       <c r="F80" s="9" t="s">
         <v>28</v>
@@ -3814,7 +3814,7 @@
         <v>27</v>
       </c>
       <c r="E81" s="11">
-        <v>13</v>
+        <v>27</v>
       </c>
       <c r="F81" s="9" t="s">
         <v>28</v>
@@ -3837,7 +3837,7 @@
         <v>27</v>
       </c>
       <c r="E82" s="11">
-        <v>29</v>
+        <v>23</v>
       </c>
       <c r="F82" s="9" t="s">
         <v>28</v>
@@ -3860,7 +3860,7 @@
         <v>27</v>
       </c>
       <c r="E83" s="11">
-        <v>14</v>
+        <v>16</v>
       </c>
       <c r="F83" s="9" t="s">
         <v>28</v>
@@ -3883,7 +3883,7 @@
         <v>27</v>
       </c>
       <c r="E84" s="11">
-        <v>14</v>
+        <v>28</v>
       </c>
       <c r="F84" s="9" t="s">
         <v>28</v>
@@ -3906,7 +3906,7 @@
         <v>27</v>
       </c>
       <c r="E85" s="11">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="F85" s="9" t="s">
         <v>28</v>
@@ -3929,7 +3929,7 @@
         <v>27</v>
       </c>
       <c r="E86" s="11">
-        <v>14</v>
+        <v>25</v>
       </c>
       <c r="F86" s="9" t="s">
         <v>28</v>
@@ -3952,7 +3952,7 @@
         <v>27</v>
       </c>
       <c r="E87" s="11">
-        <v>25</v>
+        <v>13</v>
       </c>
       <c r="F87" s="9" t="s">
         <v>28</v>
@@ -3975,7 +3975,7 @@
         <v>27</v>
       </c>
       <c r="E88" s="11">
-        <v>18</v>
+        <v>12</v>
       </c>
       <c r="F88" s="9" t="s">
         <v>28</v>
@@ -3998,7 +3998,7 @@
         <v>27</v>
       </c>
       <c r="E89" s="11">
-        <v>13</v>
+        <v>26</v>
       </c>
       <c r="F89" s="9" t="s">
         <v>28</v>
@@ -4021,7 +4021,7 @@
         <v>27</v>
       </c>
       <c r="E90" s="11">
-        <v>23</v>
+        <v>31</v>
       </c>
       <c r="F90" s="9" t="s">
         <v>28</v>
@@ -4044,7 +4044,7 @@
         <v>27</v>
       </c>
       <c r="E91" s="11">
-        <v>13</v>
+        <v>23</v>
       </c>
       <c r="F91" s="9" t="s">
         <v>28</v>
@@ -4067,7 +4067,7 @@
         <v>27</v>
       </c>
       <c r="E92" s="11">
-        <v>18</v>
+        <v>13</v>
       </c>
       <c r="F92" s="9" t="s">
         <v>28</v>
@@ -4090,7 +4090,7 @@
         <v>27</v>
       </c>
       <c r="E93" s="11">
-        <v>24</v>
+        <v>21</v>
       </c>
       <c r="F93" s="9" t="s">
         <v>28</v>
@@ -4113,7 +4113,7 @@
         <v>27</v>
       </c>
       <c r="E94" s="11">
-        <v>14</v>
+        <v>16</v>
       </c>
       <c r="F94" s="9" t="s">
         <v>28</v>
@@ -4136,7 +4136,7 @@
         <v>27</v>
       </c>
       <c r="E95" s="11">
-        <v>16</v>
+        <v>20</v>
       </c>
       <c r="F95" s="9" t="s">
         <v>28</v>
@@ -4159,7 +4159,7 @@
         <v>27</v>
       </c>
       <c r="E96" s="11">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="F96" s="9" t="s">
         <v>28</v>
@@ -4182,7 +4182,7 @@
         <v>27</v>
       </c>
       <c r="E97" s="11">
-        <v>8</v>
+        <v>21</v>
       </c>
       <c r="F97" s="9" t="s">
         <v>28</v>
@@ -4205,7 +4205,7 @@
         <v>27</v>
       </c>
       <c r="E98" s="11">
-        <v>31</v>
+        <v>14</v>
       </c>
       <c r="F98" s="9" t="s">
         <v>28</v>
@@ -4228,7 +4228,7 @@
         <v>27</v>
       </c>
       <c r="E99" s="11">
-        <v>19</v>
+        <v>11</v>
       </c>
       <c r="F99" s="9" t="s">
         <v>28</v>
@@ -4251,7 +4251,7 @@
         <v>27</v>
       </c>
       <c r="E100" s="11">
-        <v>29</v>
+        <v>19</v>
       </c>
       <c r="F100" s="9" t="s">
         <v>28</v>
@@ -4274,7 +4274,7 @@
         <v>27</v>
       </c>
       <c r="E101" s="11">
-        <v>11</v>
+        <v>20</v>
       </c>
       <c r="F101" s="9" t="s">
         <v>28</v>
@@ -4297,7 +4297,7 @@
         <v>27</v>
       </c>
       <c r="E102" s="11">
-        <v>16</v>
+        <v>12</v>
       </c>
       <c r="F102" s="9" t="s">
         <v>28</v>
@@ -4320,7 +4320,7 @@
         <v>27</v>
       </c>
       <c r="E103" s="11">
-        <v>12</v>
+        <v>23</v>
       </c>
       <c r="F103" s="9" t="s">
         <v>28</v>
@@ -4343,7 +4343,7 @@
         <v>27</v>
       </c>
       <c r="E104" s="11">
-        <v>31</v>
+        <v>9</v>
       </c>
       <c r="F104" s="9" t="s">
         <v>28</v>
@@ -4366,7 +4366,7 @@
         <v>27</v>
       </c>
       <c r="E105" s="11">
-        <v>28</v>
+        <v>15</v>
       </c>
       <c r="F105" s="9" t="s">
         <v>28</v>
@@ -4389,7 +4389,7 @@
         <v>27</v>
       </c>
       <c r="E106" s="11">
-        <v>26</v>
+        <v>22</v>
       </c>
       <c r="F106" s="9" t="s">
         <v>28</v>
@@ -4412,7 +4412,7 @@
         <v>27</v>
       </c>
       <c r="E107" s="11">
-        <v>17</v>
+        <v>22</v>
       </c>
       <c r="F107" s="9" t="s">
         <v>28</v>
@@ -4435,7 +4435,7 @@
         <v>27</v>
       </c>
       <c r="E108" s="11">
-        <v>8</v>
+        <v>22</v>
       </c>
       <c r="F108" s="9" t="s">
         <v>28</v>
@@ -4458,7 +4458,7 @@
         <v>27</v>
       </c>
       <c r="E109" s="11">
-        <v>23</v>
+        <v>27</v>
       </c>
       <c r="F109" s="9" t="s">
         <v>28</v>
@@ -4481,7 +4481,7 @@
         <v>27</v>
       </c>
       <c r="E110" s="11">
-        <v>21</v>
+        <v>24</v>
       </c>
       <c r="F110" s="9" t="s">
         <v>28</v>
@@ -4504,7 +4504,7 @@
         <v>27</v>
       </c>
       <c r="E111" s="11">
-        <v>28</v>
+        <v>22</v>
       </c>
       <c r="F111" s="9" t="s">
         <v>28</v>
@@ -4527,7 +4527,7 @@
         <v>27</v>
       </c>
       <c r="E112" s="11">
-        <v>25</v>
+        <v>10</v>
       </c>
       <c r="F112" s="9" t="s">
         <v>28</v>
@@ -4550,7 +4550,7 @@
         <v>27</v>
       </c>
       <c r="E113" s="11">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="F113" s="9" t="s">
         <v>28</v>
@@ -4573,7 +4573,7 @@
         <v>27</v>
       </c>
       <c r="E114" s="11">
-        <v>16</v>
+        <v>25</v>
       </c>
       <c r="F114" s="9" t="s">
         <v>28</v>
@@ -4596,7 +4596,7 @@
         <v>27</v>
       </c>
       <c r="E115" s="11">
-        <v>11</v>
+        <v>29</v>
       </c>
       <c r="F115" s="9" t="s">
         <v>28</v>
@@ -4619,7 +4619,7 @@
         <v>27</v>
       </c>
       <c r="E116" s="11">
-        <v>11</v>
+        <v>22</v>
       </c>
       <c r="F116" s="9" t="s">
         <v>28</v>
@@ -4642,7 +4642,7 @@
         <v>27</v>
       </c>
       <c r="E117" s="11">
-        <v>20</v>
+        <v>14</v>
       </c>
       <c r="F117" s="9" t="s">
         <v>28</v>
@@ -4665,7 +4665,7 @@
         <v>27</v>
       </c>
       <c r="E118" s="11">
-        <v>10</v>
+        <v>31</v>
       </c>
       <c r="F118" s="9" t="s">
         <v>28</v>
@@ -4688,7 +4688,7 @@
         <v>27</v>
       </c>
       <c r="E119" s="11">
-        <v>19</v>
+        <v>12</v>
       </c>
       <c r="F119" s="9" t="s">
         <v>28</v>
@@ -4711,7 +4711,7 @@
         <v>27</v>
       </c>
       <c r="E120" s="11">
-        <v>25</v>
+        <v>27</v>
       </c>
       <c r="F120" s="9" t="s">
         <v>28</v>
@@ -4734,7 +4734,7 @@
         <v>27</v>
       </c>
       <c r="E121" s="11">
-        <v>21</v>
+        <v>27</v>
       </c>
       <c r="F121" s="9" t="s">
         <v>28</v>
@@ -4757,7 +4757,7 @@
         <v>27</v>
       </c>
       <c r="E122" s="11">
-        <v>20</v>
+        <v>29</v>
       </c>
       <c r="F122" s="9" t="s">
         <v>28</v>
@@ -4803,7 +4803,7 @@
         <v>27</v>
       </c>
       <c r="E124" s="11">
-        <v>15</v>
+        <v>23</v>
       </c>
       <c r="F124" s="9" t="s">
         <v>28</v>
@@ -4826,7 +4826,7 @@
         <v>27</v>
       </c>
       <c r="E125" s="11">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="F125" s="9" t="s">
         <v>28</v>
@@ -4849,7 +4849,7 @@
         <v>27</v>
       </c>
       <c r="E126" s="11">
-        <v>19</v>
+        <v>13</v>
       </c>
       <c r="F126" s="9" t="s">
         <v>28</v>
@@ -4872,7 +4872,7 @@
         <v>27</v>
       </c>
       <c r="E127" s="11">
-        <v>23</v>
+        <v>20</v>
       </c>
       <c r="F127" s="9" t="s">
         <v>28</v>
@@ -4895,7 +4895,7 @@
         <v>27</v>
       </c>
       <c r="E128" s="11">
-        <v>22</v>
+        <v>14</v>
       </c>
       <c r="F128" s="9" t="s">
         <v>28</v>
@@ -4918,7 +4918,7 @@
         <v>27</v>
       </c>
       <c r="E129" s="11">
-        <v>17</v>
+        <v>28</v>
       </c>
       <c r="F129" s="9" t="s">
         <v>28</v>
@@ -4941,7 +4941,7 @@
         <v>27</v>
       </c>
       <c r="E130" s="11">
-        <v>8</v>
+        <v>13</v>
       </c>
       <c r="F130" s="9" t="s">
         <v>28</v>
@@ -4964,7 +4964,7 @@
         <v>27</v>
       </c>
       <c r="E131" s="11">
-        <v>22</v>
+        <v>12</v>
       </c>
       <c r="F131" s="9" t="s">
         <v>28</v>
@@ -4987,7 +4987,7 @@
         <v>27</v>
       </c>
       <c r="E132" s="11">
-        <v>11</v>
+        <v>13</v>
       </c>
       <c r="F132" s="9" t="s">
         <v>28</v>
@@ -5010,7 +5010,7 @@
         <v>27</v>
       </c>
       <c r="E133" s="11">
-        <v>11</v>
+        <v>23</v>
       </c>
       <c r="F133" s="9" t="s">
         <v>28</v>
@@ -5033,7 +5033,7 @@
         <v>27</v>
       </c>
       <c r="E134" s="11">
-        <v>22</v>
+        <v>8</v>
       </c>
       <c r="F134" s="9" t="s">
         <v>28</v>
@@ -5056,7 +5056,7 @@
         <v>27</v>
       </c>
       <c r="E135" s="11">
-        <v>28</v>
+        <v>22</v>
       </c>
       <c r="F135" s="9" t="s">
         <v>28</v>
@@ -5079,7 +5079,7 @@
         <v>27</v>
       </c>
       <c r="E136" s="11">
-        <v>15</v>
+        <v>27</v>
       </c>
       <c r="F136" s="9" t="s">
         <v>28</v>
@@ -5102,7 +5102,7 @@
         <v>27</v>
       </c>
       <c r="E137" s="11">
-        <v>11</v>
+        <v>18</v>
       </c>
       <c r="F137" s="9" t="s">
         <v>28</v>
@@ -5125,7 +5125,7 @@
         <v>27</v>
       </c>
       <c r="E138" s="11">
-        <v>25</v>
+        <v>17</v>
       </c>
       <c r="F138" s="9" t="s">
         <v>28</v>
@@ -5148,7 +5148,7 @@
         <v>27</v>
       </c>
       <c r="E139" s="11">
-        <v>30</v>
+        <v>8</v>
       </c>
       <c r="F139" s="9" t="s">
         <v>28</v>
@@ -5171,7 +5171,7 @@
         <v>27</v>
       </c>
       <c r="E140" s="11">
-        <v>19</v>
+        <v>22</v>
       </c>
       <c r="F140" s="9" t="s">
         <v>28</v>
@@ -5194,7 +5194,7 @@
         <v>27</v>
       </c>
       <c r="E141" s="11">
-        <v>17</v>
+        <v>11</v>
       </c>
       <c r="F141" s="9" t="s">
         <v>28</v>
@@ -5217,7 +5217,7 @@
         <v>27</v>
       </c>
       <c r="E142" s="11">
-        <v>30</v>
+        <v>23</v>
       </c>
       <c r="F142" s="9" t="s">
         <v>28</v>
@@ -5240,7 +5240,7 @@
         <v>27</v>
       </c>
       <c r="E143" s="11">
-        <v>12</v>
+        <v>8</v>
       </c>
       <c r="F143" s="9" t="s">
         <v>28</v>
@@ -5263,7 +5263,7 @@
         <v>27</v>
       </c>
       <c r="E144" s="11">
-        <v>26</v>
+        <v>28</v>
       </c>
       <c r="F144" s="9" t="s">
         <v>28</v>
@@ -5286,7 +5286,7 @@
         <v>27</v>
       </c>
       <c r="E145" s="11">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="F145" s="9" t="s">
         <v>28</v>
@@ -5309,7 +5309,7 @@
         <v>27</v>
       </c>
       <c r="E146" s="11">
-        <v>24</v>
+        <v>31</v>
       </c>
       <c r="F146" s="9" t="s">
         <v>28</v>
@@ -5332,7 +5332,7 @@
         <v>27</v>
       </c>
       <c r="E147" s="11">
-        <v>13</v>
+        <v>24</v>
       </c>
       <c r="F147" s="9" t="s">
         <v>28</v>
@@ -5355,7 +5355,7 @@
         <v>27</v>
       </c>
       <c r="E148" s="11">
-        <v>30</v>
+        <v>20</v>
       </c>
       <c r="F148" s="9" t="s">
         <v>28</v>
@@ -5378,7 +5378,7 @@
         <v>27</v>
       </c>
       <c r="E149" s="11">
-        <v>12</v>
+        <v>16</v>
       </c>
       <c r="F149" s="9" t="s">
         <v>28</v>
@@ -5401,7 +5401,7 @@
         <v>27</v>
       </c>
       <c r="E150" s="11">
-        <v>10</v>
+        <v>20</v>
       </c>
       <c r="F150" s="9" t="s">
         <v>28</v>
@@ -5424,7 +5424,7 @@
         <v>27</v>
       </c>
       <c r="E151" s="11">
-        <v>15</v>
+        <v>18</v>
       </c>
       <c r="F151" s="9" t="s">
         <v>28</v>
@@ -5447,7 +5447,7 @@
         <v>27</v>
       </c>
       <c r="E152" s="11">
-        <v>14</v>
+        <v>29</v>
       </c>
       <c r="F152" s="9" t="s">
         <v>28</v>
@@ -5470,7 +5470,7 @@
         <v>27</v>
       </c>
       <c r="E153" s="11">
-        <v>26</v>
+        <v>10</v>
       </c>
       <c r="F153" s="9" t="s">
         <v>28</v>
@@ -5493,7 +5493,7 @@
         <v>27</v>
       </c>
       <c r="E154" s="11">
-        <v>9</v>
+        <v>16</v>
       </c>
       <c r="F154" s="9" t="s">
         <v>28</v>
@@ -5516,7 +5516,7 @@
         <v>27</v>
       </c>
       <c r="E155" s="11">
-        <v>26</v>
+        <v>19</v>
       </c>
       <c r="F155" s="9" t="s">
         <v>28</v>
@@ -5539,7 +5539,7 @@
         <v>27</v>
       </c>
       <c r="E156" s="11">
-        <v>14</v>
+        <v>29</v>
       </c>
       <c r="F156" s="9" t="s">
         <v>28</v>
@@ -5562,7 +5562,7 @@
         <v>27</v>
       </c>
       <c r="E157" s="11">
-        <v>21</v>
+        <v>15</v>
       </c>
       <c r="F157" s="9" t="s">
         <v>28</v>
@@ -5585,7 +5585,7 @@
         <v>27</v>
       </c>
       <c r="E158" s="11">
-        <v>18</v>
+        <v>31</v>
       </c>
       <c r="F158" s="9" t="s">
         <v>28</v>
@@ -5608,7 +5608,7 @@
         <v>27</v>
       </c>
       <c r="E159" s="11">
-        <v>29</v>
+        <v>8</v>
       </c>
       <c r="F159" s="9" t="s">
         <v>28</v>
@@ -5631,7 +5631,7 @@
         <v>27</v>
       </c>
       <c r="E160" s="11">
-        <v>21</v>
+        <v>15</v>
       </c>
       <c r="F160" s="9" t="s">
         <v>28</v>
@@ -5654,7 +5654,7 @@
         <v>27</v>
       </c>
       <c r="E161" s="11">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="F161" s="9" t="s">
         <v>28</v>
@@ -5677,7 +5677,7 @@
         <v>27</v>
       </c>
       <c r="E162" s="11">
-        <v>24</v>
+        <v>18</v>
       </c>
       <c r="F162" s="9" t="s">
         <v>28</v>
@@ -5700,7 +5700,7 @@
         <v>27</v>
       </c>
       <c r="E163" s="11">
-        <v>29</v>
+        <v>9</v>
       </c>
       <c r="F163" s="9" t="s">
         <v>28</v>
@@ -5723,7 +5723,7 @@
         <v>27</v>
       </c>
       <c r="E164" s="11">
-        <v>15</v>
+        <v>17</v>
       </c>
       <c r="F164" s="9" t="s">
         <v>28</v>
@@ -5746,7 +5746,7 @@
         <v>27</v>
       </c>
       <c r="E165" s="11">
-        <v>19</v>
+        <v>28</v>
       </c>
       <c r="F165" s="9" t="s">
         <v>28</v>
@@ -5769,7 +5769,7 @@
         <v>27</v>
       </c>
       <c r="E166" s="11">
-        <v>24</v>
+        <v>15</v>
       </c>
       <c r="F166" s="9" t="s">
         <v>28</v>
@@ -5792,7 +5792,7 @@
         <v>27</v>
       </c>
       <c r="E167" s="11">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="F167" s="9" t="s">
         <v>28</v>
@@ -5815,7 +5815,7 @@
         <v>27</v>
       </c>
       <c r="E168" s="11">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="F168" s="9" t="s">
         <v>28</v>
@@ -5838,7 +5838,7 @@
         <v>27</v>
       </c>
       <c r="E169" s="11">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="F169" s="9" t="s">
         <v>28</v>
@@ -5861,7 +5861,7 @@
         <v>27</v>
       </c>
       <c r="E170" s="11">
-        <v>22</v>
+        <v>9</v>
       </c>
       <c r="F170" s="9" t="s">
         <v>28</v>
@@ -5884,7 +5884,7 @@
         <v>27</v>
       </c>
       <c r="E171" s="11">
-        <v>15</v>
+        <v>23</v>
       </c>
       <c r="F171" s="9" t="s">
         <v>28</v>
@@ -5907,7 +5907,7 @@
         <v>27</v>
       </c>
       <c r="E172" s="11">
-        <v>29</v>
+        <v>19</v>
       </c>
       <c r="F172" s="9" t="s">
         <v>28</v>
@@ -5930,7 +5930,7 @@
         <v>27</v>
       </c>
       <c r="E173" s="11">
-        <v>27</v>
+        <v>23</v>
       </c>
       <c r="F173" s="9" t="s">
         <v>28</v>
@@ -5953,7 +5953,7 @@
         <v>27</v>
       </c>
       <c r="E174" s="11">
-        <v>9</v>
+        <v>27</v>
       </c>
       <c r="F174" s="9" t="s">
         <v>28</v>
@@ -5976,7 +5976,7 @@
         <v>27</v>
       </c>
       <c r="E175" s="11">
-        <v>15</v>
+        <v>31</v>
       </c>
       <c r="F175" s="9" t="s">
         <v>28</v>
@@ -5999,7 +5999,7 @@
         <v>27</v>
       </c>
       <c r="E176" s="11">
-        <v>23</v>
+        <v>27</v>
       </c>
       <c r="F176" s="9" t="s">
         <v>28</v>
@@ -6022,7 +6022,7 @@
         <v>27</v>
       </c>
       <c r="E177" s="11">
-        <v>17</v>
+        <v>13</v>
       </c>
       <c r="F177" s="9" t="s">
         <v>28</v>
@@ -6045,7 +6045,7 @@
         <v>27</v>
       </c>
       <c r="E178" s="11">
-        <v>20</v>
+        <v>8</v>
       </c>
       <c r="F178" s="9" t="s">
         <v>28</v>
@@ -6068,7 +6068,7 @@
         <v>27</v>
       </c>
       <c r="E179" s="11">
-        <v>12</v>
+        <v>20</v>
       </c>
       <c r="F179" s="9" t="s">
         <v>28</v>
@@ -6091,7 +6091,7 @@
         <v>27</v>
       </c>
       <c r="E180" s="11">
-        <v>8</v>
+        <v>27</v>
       </c>
       <c r="F180" s="9" t="s">
         <v>28</v>
@@ -6137,7 +6137,7 @@
         <v>27</v>
       </c>
       <c r="E182" s="11">
-        <v>25</v>
+        <v>31</v>
       </c>
       <c r="F182" s="9" t="s">
         <v>28</v>
@@ -6160,7 +6160,7 @@
         <v>27</v>
       </c>
       <c r="E183" s="11">
-        <v>10</v>
+        <v>18</v>
       </c>
       <c r="F183" s="9" t="s">
         <v>28</v>
@@ -6183,7 +6183,7 @@
         <v>27</v>
       </c>
       <c r="E184" s="11">
-        <v>22</v>
+        <v>26</v>
       </c>
       <c r="F184" s="9" t="s">
         <v>28</v>
@@ -6206,7 +6206,7 @@
         <v>27</v>
       </c>
       <c r="E185" s="11">
-        <v>25</v>
+        <v>20</v>
       </c>
       <c r="F185" s="9" t="s">
         <v>28</v>
@@ -6229,7 +6229,7 @@
         <v>27</v>
       </c>
       <c r="E186" s="11">
-        <v>28</v>
+        <v>23</v>
       </c>
       <c r="F186" s="9" t="s">
         <v>28</v>
@@ -6252,7 +6252,7 @@
         <v>27</v>
       </c>
       <c r="E187" s="11">
-        <v>25</v>
+        <v>20</v>
       </c>
       <c r="F187" s="9" t="s">
         <v>28</v>
@@ -6275,7 +6275,7 @@
         <v>27</v>
       </c>
       <c r="E188" s="11">
-        <v>8</v>
+        <v>11</v>
       </c>
       <c r="F188" s="9" t="s">
         <v>28</v>
@@ -6298,7 +6298,7 @@
         <v>27</v>
       </c>
       <c r="E189" s="11">
-        <v>22</v>
+        <v>26</v>
       </c>
       <c r="F189" s="9" t="s">
         <v>28</v>
@@ -6321,7 +6321,7 @@
         <v>27</v>
       </c>
       <c r="E190" s="11">
-        <v>24</v>
+        <v>30</v>
       </c>
       <c r="F190" s="9" t="s">
         <v>28</v>
@@ -6344,7 +6344,7 @@
         <v>27</v>
       </c>
       <c r="E191" s="11">
-        <v>15</v>
+        <v>23</v>
       </c>
       <c r="F191" s="9" t="s">
         <v>28</v>
@@ -6367,7 +6367,7 @@
         <v>27</v>
       </c>
       <c r="E192" s="11">
-        <v>30</v>
+        <v>20</v>
       </c>
       <c r="F192" s="9" t="s">
         <v>28</v>
@@ -6390,7 +6390,7 @@
         <v>27</v>
       </c>
       <c r="E193" s="11">
-        <v>21</v>
+        <v>16</v>
       </c>
       <c r="F193" s="9" t="s">
         <v>28</v>
@@ -6413,7 +6413,7 @@
         <v>27</v>
       </c>
       <c r="E194" s="11">
-        <v>31</v>
+        <v>10</v>
       </c>
       <c r="F194" s="9" t="s">
         <v>28</v>
@@ -6436,7 +6436,7 @@
         <v>27</v>
       </c>
       <c r="E195" s="11">
-        <v>17</v>
+        <v>19</v>
       </c>
       <c r="F195" s="9" t="s">
         <v>28</v>
@@ -6459,7 +6459,7 @@
         <v>27</v>
       </c>
       <c r="E196" s="11">
-        <v>31</v>
+        <v>14</v>
       </c>
       <c r="F196" s="9" t="s">
         <v>28</v>
@@ -6482,7 +6482,7 @@
         <v>27</v>
       </c>
       <c r="E197" s="11">
-        <v>31</v>
+        <v>16</v>
       </c>
       <c r="F197" s="9" t="s">
         <v>28</v>
@@ -6505,7 +6505,7 @@
         <v>27</v>
       </c>
       <c r="E198" s="11">
-        <v>26</v>
+        <v>24</v>
       </c>
       <c r="F198" s="9" t="s">
         <v>28</v>
@@ -6528,7 +6528,7 @@
         <v>27</v>
       </c>
       <c r="E199" s="11">
-        <v>24</v>
+        <v>13</v>
       </c>
       <c r="F199" s="9" t="s">
         <v>28</v>
@@ -6551,7 +6551,7 @@
         <v>27</v>
       </c>
       <c r="E200" s="11">
-        <v>20</v>
+        <v>16</v>
       </c>
       <c r="F200" s="9" t="s">
         <v>28</v>
@@ -6574,7 +6574,7 @@
         <v>27</v>
       </c>
       <c r="E201" s="11">
-        <v>17</v>
+        <v>13</v>
       </c>
       <c r="F201" s="9" t="s">
         <v>28</v>
@@ -6597,7 +6597,7 @@
         <v>27</v>
       </c>
       <c r="E202" s="11">
-        <v>13</v>
+        <v>18</v>
       </c>
       <c r="F202" s="9" t="s">
         <v>28</v>
@@ -6620,7 +6620,7 @@
         <v>27</v>
       </c>
       <c r="E203" s="11">
-        <v>8</v>
+        <v>26</v>
       </c>
       <c r="F203" s="9" t="s">
         <v>28</v>
@@ -6643,7 +6643,7 @@
         <v>27</v>
       </c>
       <c r="E204" s="11">
-        <v>23</v>
+        <v>18</v>
       </c>
       <c r="F204" s="9" t="s">
         <v>28</v>
@@ -6666,7 +6666,7 @@
         <v>27</v>
       </c>
       <c r="E205" s="11">
-        <v>18</v>
+        <v>24</v>
       </c>
       <c r="F205" s="9" t="s">
         <v>28</v>
@@ -6689,7 +6689,7 @@
         <v>27</v>
       </c>
       <c r="E206" s="11">
-        <v>21</v>
+        <v>15</v>
       </c>
       <c r="F206" s="9" t="s">
         <v>28</v>
@@ -6712,7 +6712,7 @@
         <v>27</v>
       </c>
       <c r="E207" s="11">
-        <v>27</v>
+        <v>12</v>
       </c>
       <c r="F207" s="9" t="s">
         <v>28</v>
@@ -6735,7 +6735,7 @@
         <v>27</v>
       </c>
       <c r="E208" s="11">
-        <v>21</v>
+        <v>27</v>
       </c>
       <c r="F208" s="9" t="s">
         <v>28</v>
@@ -6758,7 +6758,7 @@
         <v>27</v>
       </c>
       <c r="E209" s="11">
-        <v>25</v>
+        <v>8</v>
       </c>
       <c r="F209" s="9" t="s">
         <v>28</v>
@@ -6804,7 +6804,7 @@
         <v>27</v>
       </c>
       <c r="E211" s="11">
-        <v>10</v>
+        <v>29</v>
       </c>
       <c r="F211" s="9" t="s">
         <v>28</v>
@@ -6827,7 +6827,7 @@
         <v>27</v>
       </c>
       <c r="E212" s="11">
-        <v>21</v>
+        <v>18</v>
       </c>
       <c r="F212" s="9" t="s">
         <v>28</v>
@@ -6850,7 +6850,7 @@
         <v>27</v>
       </c>
       <c r="E213" s="11">
-        <v>23</v>
+        <v>9</v>
       </c>
       <c r="F213" s="9" t="s">
         <v>28</v>
@@ -6873,7 +6873,7 @@
         <v>27</v>
       </c>
       <c r="E214" s="11">
-        <v>16</v>
+        <v>29</v>
       </c>
       <c r="F214" s="9" t="s">
         <v>28</v>
@@ -6896,7 +6896,7 @@
         <v>27</v>
       </c>
       <c r="E215" s="11">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="F215" s="9" t="s">
         <v>28</v>
@@ -6919,7 +6919,7 @@
         <v>27</v>
       </c>
       <c r="E216" s="11">
-        <v>14</v>
+        <v>30</v>
       </c>
       <c r="F216" s="9" t="s">
         <v>28</v>
@@ -6942,7 +6942,7 @@
         <v>27</v>
       </c>
       <c r="E217" s="11">
-        <v>11</v>
+        <v>24</v>
       </c>
       <c r="F217" s="9" t="s">
         <v>28</v>
@@ -6965,7 +6965,7 @@
         <v>27</v>
       </c>
       <c r="E218" s="11">
-        <v>29</v>
+        <v>17</v>
       </c>
       <c r="F218" s="9" t="s">
         <v>28</v>
@@ -6988,7 +6988,7 @@
         <v>27</v>
       </c>
       <c r="E219" s="11">
-        <v>25</v>
+        <v>27</v>
       </c>
       <c r="F219" s="9" t="s">
         <v>28</v>
@@ -7011,7 +7011,7 @@
         <v>27</v>
       </c>
       <c r="E220" s="11">
-        <v>9</v>
+        <v>21</v>
       </c>
       <c r="F220" s="9" t="s">
         <v>28</v>
@@ -7034,7 +7034,7 @@
         <v>27</v>
       </c>
       <c r="E221" s="11">
-        <v>9</v>
+        <v>19</v>
       </c>
       <c r="F221" s="9" t="s">
         <v>28</v>
@@ -7057,7 +7057,7 @@
         <v>27</v>
       </c>
       <c r="E222" s="11">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="F222" s="9" t="s">
         <v>28</v>
@@ -7080,7 +7080,7 @@
         <v>27</v>
       </c>
       <c r="E223" s="11">
-        <v>21</v>
+        <v>8</v>
       </c>
       <c r="F223" s="9" t="s">
         <v>28</v>
@@ -7103,7 +7103,7 @@
         <v>27</v>
       </c>
       <c r="E224" s="11">
-        <v>11</v>
+        <v>19</v>
       </c>
       <c r="F224" s="9" t="s">
         <v>28</v>
@@ -7126,7 +7126,7 @@
         <v>27</v>
       </c>
       <c r="E225" s="11">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="F225" s="9" t="s">
         <v>28</v>
@@ -7149,7 +7149,7 @@
         <v>27</v>
       </c>
       <c r="E226" s="11">
-        <v>8</v>
+        <v>17</v>
       </c>
       <c r="F226" s="9" t="s">
         <v>28</v>
@@ -7172,7 +7172,7 @@
         <v>27</v>
       </c>
       <c r="E227" s="11">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="F227" s="9" t="s">
         <v>28</v>
@@ -7195,7 +7195,7 @@
         <v>27</v>
       </c>
       <c r="E228" s="11">
-        <v>28</v>
+        <v>22</v>
       </c>
       <c r="F228" s="9" t="s">
         <v>28</v>
@@ -7218,7 +7218,7 @@
         <v>27</v>
       </c>
       <c r="E229" s="11">
-        <v>9</v>
+        <v>15</v>
       </c>
       <c r="F229" s="9" t="s">
         <v>28</v>
@@ -7241,7 +7241,7 @@
         <v>27</v>
       </c>
       <c r="E230" s="11">
-        <v>31</v>
+        <v>9</v>
       </c>
       <c r="F230" s="9" t="s">
         <v>28</v>
@@ -7264,7 +7264,7 @@
         <v>27</v>
       </c>
       <c r="E231" s="11">
-        <v>31</v>
+        <v>28</v>
       </c>
       <c r="F231" s="9" t="s">
         <v>28</v>
@@ -7287,7 +7287,7 @@
         <v>27</v>
       </c>
       <c r="E232" s="11">
-        <v>21</v>
+        <v>17</v>
       </c>
       <c r="F232" s="9" t="s">
         <v>28</v>
@@ -7310,7 +7310,7 @@
         <v>27</v>
       </c>
       <c r="E233" s="11">
-        <v>30</v>
+        <v>11</v>
       </c>
       <c r="F233" s="9" t="s">
         <v>28</v>
@@ -7333,7 +7333,7 @@
         <v>27</v>
       </c>
       <c r="E234" s="11">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="F234" s="9" t="s">
         <v>28</v>
@@ -7356,7 +7356,7 @@
         <v>27</v>
       </c>
       <c r="E235" s="11">
-        <v>19</v>
+        <v>9</v>
       </c>
       <c r="F235" s="9" t="s">
         <v>28</v>
@@ -7379,7 +7379,7 @@
         <v>27</v>
       </c>
       <c r="E236" s="11">
-        <v>29</v>
+        <v>9</v>
       </c>
       <c r="F236" s="9" t="s">
         <v>28</v>
@@ -7402,7 +7402,7 @@
         <v>27</v>
       </c>
       <c r="E237" s="11">
-        <v>14</v>
+        <v>8</v>
       </c>
       <c r="F237" s="9" t="s">
         <v>28</v>
@@ -7425,7 +7425,7 @@
         <v>27</v>
       </c>
       <c r="E238" s="11">
-        <v>17</v>
+        <v>31</v>
       </c>
       <c r="F238" s="9" t="s">
         <v>28</v>
@@ -7448,7 +7448,7 @@
         <v>27</v>
       </c>
       <c r="E239" s="11">
-        <v>26</v>
+        <v>22</v>
       </c>
       <c r="F239" s="9" t="s">
         <v>28</v>
@@ -7471,7 +7471,7 @@
         <v>27</v>
       </c>
       <c r="E240" s="11">
-        <v>10</v>
+        <v>27</v>
       </c>
       <c r="F240" s="9" t="s">
         <v>28</v>
@@ -7494,7 +7494,7 @@
         <v>27</v>
       </c>
       <c r="E241" s="11">
-        <v>25</v>
+        <v>27</v>
       </c>
       <c r="F241" s="9" t="s">
         <v>28</v>
@@ -7517,7 +7517,7 @@
         <v>27</v>
       </c>
       <c r="E242" s="11">
-        <v>22</v>
+        <v>26</v>
       </c>
       <c r="F242" s="9" t="s">
         <v>28</v>
@@ -7540,7 +7540,7 @@
         <v>27</v>
       </c>
       <c r="E243" s="11">
-        <v>19</v>
+        <v>13</v>
       </c>
       <c r="F243" s="9" t="s">
         <v>28</v>
@@ -7563,7 +7563,7 @@
         <v>27</v>
       </c>
       <c r="E244" s="11">
-        <v>28</v>
+        <v>12</v>
       </c>
       <c r="F244" s="9" t="s">
         <v>28</v>
@@ -7586,7 +7586,7 @@
         <v>27</v>
       </c>
       <c r="E245" s="11">
-        <v>31</v>
+        <v>23</v>
       </c>
       <c r="F245" s="9" t="s">
         <v>28</v>
@@ -7609,7 +7609,7 @@
         <v>27</v>
       </c>
       <c r="E246" s="11">
-        <v>23</v>
+        <v>9</v>
       </c>
       <c r="F246" s="9" t="s">
         <v>28</v>
@@ -7655,7 +7655,7 @@
         <v>27</v>
       </c>
       <c r="E248" s="11">
-        <v>22</v>
+        <v>18</v>
       </c>
       <c r="F248" s="9" t="s">
         <v>28</v>
@@ -7678,7 +7678,7 @@
         <v>27</v>
       </c>
       <c r="E249" s="11">
-        <v>22</v>
+        <v>17</v>
       </c>
       <c r="F249" s="9" t="s">
         <v>28</v>
@@ -7701,7 +7701,7 @@
         <v>27</v>
       </c>
       <c r="E250" s="11">
-        <v>9</v>
+        <v>31</v>
       </c>
       <c r="F250" s="9" t="s">
         <v>28</v>
@@ -7724,7 +7724,7 @@
         <v>27</v>
       </c>
       <c r="E251" s="11">
-        <v>23</v>
+        <v>20</v>
       </c>
       <c r="F251" s="9" t="s">
         <v>28</v>
@@ -7747,7 +7747,7 @@
         <v>27</v>
       </c>
       <c r="E252" s="11">
-        <v>16</v>
+        <v>25</v>
       </c>
       <c r="F252" s="9" t="s">
         <v>28</v>
@@ -7770,7 +7770,7 @@
         <v>27</v>
       </c>
       <c r="E253" s="11">
-        <v>24</v>
+        <v>31</v>
       </c>
       <c r="F253" s="9" t="s">
         <v>28</v>
@@ -7793,7 +7793,7 @@
         <v>27</v>
       </c>
       <c r="E254" s="11">
-        <v>24</v>
+        <v>28</v>
       </c>
       <c r="F254" s="9" t="s">
         <v>28</v>
@@ -7816,7 +7816,7 @@
         <v>27</v>
       </c>
       <c r="E255" s="11">
-        <v>31</v>
+        <v>17</v>
       </c>
       <c r="F255" s="9" t="s">
         <v>28</v>
@@ -7839,7 +7839,7 @@
         <v>27</v>
       </c>
       <c r="E256" s="11">
-        <v>15</v>
+        <v>23</v>
       </c>
       <c r="F256" s="9" t="s">
         <v>28</v>
@@ -7862,7 +7862,7 @@
         <v>27</v>
       </c>
       <c r="E257" s="11">
-        <v>29</v>
+        <v>8</v>
       </c>
       <c r="F257" s="9" t="s">
         <v>28</v>
@@ -7885,7 +7885,7 @@
         <v>27</v>
       </c>
       <c r="E258" s="11">
-        <v>11</v>
+        <v>20</v>
       </c>
       <c r="F258" s="9" t="s">
         <v>28</v>
@@ -7908,7 +7908,7 @@
         <v>27</v>
       </c>
       <c r="E259" s="11">
-        <v>21</v>
+        <v>14</v>
       </c>
       <c r="F259" s="9" t="s">
         <v>28</v>
@@ -7931,7 +7931,7 @@
         <v>27</v>
       </c>
       <c r="E260" s="11">
-        <v>19</v>
+        <v>31</v>
       </c>
       <c r="F260" s="9" t="s">
         <v>28</v>
@@ -7954,7 +7954,7 @@
         <v>27</v>
       </c>
       <c r="E261" s="11">
-        <v>27</v>
+        <v>11</v>
       </c>
       <c r="F261" s="9" t="s">
         <v>28</v>
@@ -7977,7 +7977,7 @@
         <v>27</v>
       </c>
       <c r="E262" s="11">
-        <v>31</v>
+        <v>16</v>
       </c>
       <c r="F262" s="9" t="s">
         <v>28</v>
@@ -8000,7 +8000,7 @@
         <v>27</v>
       </c>
       <c r="E263" s="11">
-        <v>18</v>
+        <v>12</v>
       </c>
       <c r="F263" s="9" t="s">
         <v>28</v>
@@ -8023,7 +8023,7 @@
         <v>27</v>
       </c>
       <c r="E264" s="11">
-        <v>14</v>
+        <v>10</v>
       </c>
       <c r="F264" s="9" t="s">
         <v>28</v>
@@ -8046,7 +8046,7 @@
         <v>27</v>
       </c>
       <c r="E265" s="11">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="F265" s="9" t="s">
         <v>28</v>
@@ -8069,7 +8069,7 @@
         <v>27</v>
       </c>
       <c r="E266" s="11">
-        <v>31</v>
+        <v>23</v>
       </c>
       <c r="F266" s="9" t="s">
         <v>28</v>
@@ -8092,7 +8092,7 @@
         <v>27</v>
       </c>
       <c r="E267" s="11">
-        <v>16</v>
+        <v>10</v>
       </c>
       <c r="F267" s="9" t="s">
         <v>28</v>
@@ -8161,7 +8161,7 @@
         <v>27</v>
       </c>
       <c r="E270" s="11">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="F270" s="9" t="s">
         <v>28</v>
@@ -8184,7 +8184,7 @@
         <v>27</v>
       </c>
       <c r="E271" s="11">
-        <v>24</v>
+        <v>30</v>
       </c>
       <c r="F271" s="9" t="s">
         <v>28</v>
@@ -8207,7 +8207,7 @@
         <v>27</v>
       </c>
       <c r="E272" s="11">
-        <v>19</v>
+        <v>11</v>
       </c>
       <c r="F272" s="9" t="s">
         <v>28</v>
@@ -8230,7 +8230,7 @@
         <v>27</v>
       </c>
       <c r="E273" s="11">
-        <v>19</v>
+        <v>21</v>
       </c>
       <c r="F273" s="9" t="s">
         <v>28</v>
@@ -8253,7 +8253,7 @@
         <v>27</v>
       </c>
       <c r="E274" s="11">
-        <v>10</v>
+        <v>26</v>
       </c>
       <c r="F274" s="9" t="s">
         <v>28</v>
@@ -8276,7 +8276,7 @@
         <v>27</v>
       </c>
       <c r="E275" s="11">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="F275" s="9" t="s">
         <v>28</v>
@@ -8299,7 +8299,7 @@
         <v>27</v>
       </c>
       <c r="E276" s="11">
-        <v>28</v>
+        <v>22</v>
       </c>
       <c r="F276" s="9" t="s">
         <v>28</v>
@@ -8322,7 +8322,7 @@
         <v>27</v>
       </c>
       <c r="E277" s="11">
-        <v>20</v>
+        <v>31</v>
       </c>
       <c r="F277" s="9" t="s">
         <v>28</v>
@@ -8345,7 +8345,7 @@
         <v>27</v>
       </c>
       <c r="E278" s="11">
-        <v>12</v>
+        <v>28</v>
       </c>
       <c r="F278" s="9" t="s">
         <v>28</v>
@@ -8368,7 +8368,7 @@
         <v>27</v>
       </c>
       <c r="E279" s="11">
-        <v>22</v>
+        <v>31</v>
       </c>
       <c r="F279" s="9" t="s">
         <v>28</v>
@@ -8391,7 +8391,7 @@
         <v>27</v>
       </c>
       <c r="E280" s="11">
-        <v>16</v>
+        <v>9</v>
       </c>
       <c r="F280" s="9" t="s">
         <v>28</v>
@@ -8414,7 +8414,7 @@
         <v>27</v>
       </c>
       <c r="E281" s="11">
-        <v>11</v>
+        <v>27</v>
       </c>
       <c r="F281" s="9" t="s">
         <v>28</v>
@@ -8437,7 +8437,7 @@
         <v>27</v>
       </c>
       <c r="E282" s="11">
-        <v>10</v>
+        <v>22</v>
       </c>
       <c r="F282" s="9" t="s">
         <v>28</v>
@@ -8460,7 +8460,7 @@
         <v>27</v>
       </c>
       <c r="E283" s="11">
-        <v>21</v>
+        <v>30</v>
       </c>
       <c r="F283" s="9" t="s">
         <v>28</v>
@@ -8483,7 +8483,7 @@
         <v>27</v>
       </c>
       <c r="E284" s="11">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="F284" s="9" t="s">
         <v>28</v>
@@ -8506,7 +8506,7 @@
         <v>27</v>
       </c>
       <c r="E285" s="11">
-        <v>31</v>
+        <v>8</v>
       </c>
       <c r="F285" s="9" t="s">
         <v>28</v>
@@ -8529,7 +8529,7 @@
         <v>27</v>
       </c>
       <c r="E286" s="11">
-        <v>18</v>
+        <v>30</v>
       </c>
       <c r="F286" s="9" t="s">
         <v>28</v>
@@ -8552,7 +8552,7 @@
         <v>27</v>
       </c>
       <c r="E287" s="11">
-        <v>21</v>
+        <v>24</v>
       </c>
       <c r="F287" s="9" t="s">
         <v>28</v>
@@ -8575,7 +8575,7 @@
         <v>27</v>
       </c>
       <c r="E288" s="11">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="F288" s="9" t="s">
         <v>28</v>
@@ -8598,7 +8598,7 @@
         <v>27</v>
       </c>
       <c r="E289" s="11">
-        <v>15</v>
+        <v>23</v>
       </c>
       <c r="F289" s="9" t="s">
         <v>28</v>
@@ -8644,7 +8644,7 @@
         <v>27</v>
       </c>
       <c r="E291" s="11">
-        <v>21</v>
+        <v>29</v>
       </c>
       <c r="F291" s="9" t="s">
         <v>28</v>
@@ -8667,7 +8667,7 @@
         <v>27</v>
       </c>
       <c r="E292" s="11">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="F292" s="9" t="s">
         <v>28</v>
@@ -8690,7 +8690,7 @@
         <v>27</v>
       </c>
       <c r="E293" s="11">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="F293" s="9" t="s">
         <v>28</v>
@@ -8713,7 +8713,7 @@
         <v>27</v>
       </c>
       <c r="E294" s="11">
-        <v>17</v>
+        <v>10</v>
       </c>
       <c r="F294" s="9" t="s">
         <v>28</v>
@@ -8736,7 +8736,7 @@
         <v>27</v>
       </c>
       <c r="E295" s="11">
-        <v>10</v>
+        <v>21</v>
       </c>
       <c r="F295" s="9" t="s">
         <v>28</v>
@@ -8759,7 +8759,7 @@
         <v>27</v>
       </c>
       <c r="E296" s="11">
-        <v>11</v>
+        <v>28</v>
       </c>
       <c r="F296" s="9" t="s">
         <v>28</v>
@@ -8782,7 +8782,7 @@
         <v>27</v>
       </c>
       <c r="E297" s="11">
-        <v>21</v>
+        <v>17</v>
       </c>
       <c r="F297" s="9" t="s">
         <v>28</v>
@@ -8805,7 +8805,7 @@
         <v>27</v>
       </c>
       <c r="E298" s="11">
-        <v>11</v>
+        <v>15</v>
       </c>
       <c r="F298" s="9" t="s">
         <v>28</v>
@@ -8828,7 +8828,7 @@
         <v>27</v>
       </c>
       <c r="E299" s="11">
-        <v>11</v>
+        <v>24</v>
       </c>
       <c r="F299" s="9" t="s">
         <v>28</v>
@@ -8851,7 +8851,7 @@
         <v>27</v>
       </c>
       <c r="E300" s="11">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="F300" s="9" t="s">
         <v>28</v>
@@ -8874,7 +8874,7 @@
         <v>27</v>
       </c>
       <c r="E301" s="11">
-        <v>16</v>
+        <v>23</v>
       </c>
       <c r="F301" s="9" t="s">
         <v>28</v>
@@ -8897,7 +8897,7 @@
         <v>27</v>
       </c>
       <c r="E302" s="11">
-        <v>18</v>
+        <v>13</v>
       </c>
       <c r="F302" s="9" t="s">
         <v>28</v>
@@ -8920,7 +8920,7 @@
         <v>27</v>
       </c>
       <c r="E303" s="11">
-        <v>9</v>
+        <v>17</v>
       </c>
       <c r="F303" s="9" t="s">
         <v>28</v>
@@ -8943,7 +8943,7 @@
         <v>27</v>
       </c>
       <c r="E304" s="11">
-        <v>13</v>
+        <v>18</v>
       </c>
       <c r="F304" s="9" t="s">
         <v>28</v>
@@ -8966,7 +8966,7 @@
         <v>27</v>
       </c>
       <c r="E305" s="11">
-        <v>31</v>
+        <v>9</v>
       </c>
       <c r="F305" s="9" t="s">
         <v>28</v>
@@ -8989,7 +8989,7 @@
         <v>27</v>
       </c>
       <c r="E306" s="11">
-        <v>21</v>
+        <v>13</v>
       </c>
       <c r="F306" s="9" t="s">
         <v>28</v>
@@ -9012,7 +9012,7 @@
         <v>27</v>
       </c>
       <c r="E307" s="11">
-        <v>13</v>
+        <v>20</v>
       </c>
       <c r="F307" s="9" t="s">
         <v>28</v>
@@ -9035,7 +9035,7 @@
         <v>27</v>
       </c>
       <c r="E308" s="11">
-        <v>23</v>
+        <v>16</v>
       </c>
       <c r="F308" s="9" t="s">
         <v>28</v>
@@ -9058,7 +9058,7 @@
         <v>27</v>
       </c>
       <c r="E309" s="11">
-        <v>30</v>
+        <v>13</v>
       </c>
       <c r="F309" s="9" t="s">
         <v>28</v>
@@ -9081,7 +9081,7 @@
         <v>27</v>
       </c>
       <c r="E310" s="11">
-        <v>8</v>
+        <v>19</v>
       </c>
       <c r="F310" s="9" t="s">
         <v>28</v>
@@ -9104,7 +9104,7 @@
         <v>27</v>
       </c>
       <c r="E311" s="11">
-        <v>19</v>
+        <v>13</v>
       </c>
       <c r="F311" s="9" t="s">
         <v>28</v>
@@ -9127,7 +9127,7 @@
         <v>27</v>
       </c>
       <c r="E312" s="11">
-        <v>15</v>
+        <v>23</v>
       </c>
       <c r="F312" s="9" t="s">
         <v>28</v>
@@ -9150,7 +9150,7 @@
         <v>27</v>
       </c>
       <c r="E313" s="11">
-        <v>10</v>
+        <v>22</v>
       </c>
       <c r="F313" s="9" t="s">
         <v>28</v>
@@ -9173,7 +9173,7 @@
         <v>27</v>
       </c>
       <c r="E314" s="11">
-        <v>24</v>
+        <v>28</v>
       </c>
       <c r="F314" s="9" t="s">
         <v>28</v>
@@ -9196,7 +9196,7 @@
         <v>27</v>
       </c>
       <c r="E315" s="11">
-        <v>18</v>
+        <v>27</v>
       </c>
       <c r="F315" s="9" t="s">
         <v>28</v>
@@ -9219,7 +9219,7 @@
         <v>27</v>
       </c>
       <c r="E316" s="11">
-        <v>27</v>
+        <v>13</v>
       </c>
       <c r="F316" s="9" t="s">
         <v>28</v>
@@ -9242,7 +9242,7 @@
         <v>27</v>
       </c>
       <c r="E317" s="11">
-        <v>22</v>
+        <v>30</v>
       </c>
       <c r="F317" s="9" t="s">
         <v>28</v>
@@ -9265,7 +9265,7 @@
         <v>27</v>
       </c>
       <c r="E318" s="11">
-        <v>17</v>
+        <v>25</v>
       </c>
       <c r="F318" s="9" t="s">
         <v>28</v>
@@ -9288,7 +9288,7 @@
         <v>27</v>
       </c>
       <c r="E319" s="11">
-        <v>24</v>
+        <v>21</v>
       </c>
       <c r="F319" s="9" t="s">
         <v>28</v>
@@ -9311,7 +9311,7 @@
         <v>27</v>
       </c>
       <c r="E320" s="11">
-        <v>20</v>
+        <v>13</v>
       </c>
       <c r="F320" s="9" t="s">
         <v>28</v>
@@ -9334,7 +9334,7 @@
         <v>27</v>
       </c>
       <c r="E321" s="11">
-        <v>17</v>
+        <v>24</v>
       </c>
       <c r="F321" s="9" t="s">
         <v>28</v>
@@ -9357,7 +9357,7 @@
         <v>27</v>
       </c>
       <c r="E322" s="11">
-        <v>20</v>
+        <v>10</v>
       </c>
       <c r="F322" s="9" t="s">
         <v>28</v>
@@ -9380,7 +9380,7 @@
         <v>27</v>
       </c>
       <c r="E323" s="11">
-        <v>27</v>
+        <v>24</v>
       </c>
       <c r="F323" s="9" t="s">
         <v>28</v>
@@ -9403,7 +9403,7 @@
         <v>27</v>
       </c>
       <c r="E324" s="11">
-        <v>18</v>
+        <v>27</v>
       </c>
       <c r="F324" s="9" t="s">
         <v>28</v>
@@ -9426,7 +9426,7 @@
         <v>27</v>
       </c>
       <c r="E325" s="11">
-        <v>24</v>
+        <v>27</v>
       </c>
       <c r="F325" s="9" t="s">
         <v>28</v>
@@ -9449,7 +9449,7 @@
         <v>27</v>
       </c>
       <c r="E326" s="11">
-        <v>26</v>
+        <v>20</v>
       </c>
       <c r="F326" s="9" t="s">
         <v>28</v>
@@ -9472,7 +9472,7 @@
         <v>27</v>
       </c>
       <c r="E327" s="11">
-        <v>13</v>
+        <v>20</v>
       </c>
       <c r="F327" s="9" t="s">
         <v>28</v>
@@ -9495,7 +9495,7 @@
         <v>27</v>
       </c>
       <c r="E328" s="11">
-        <v>28</v>
+        <v>11</v>
       </c>
       <c r="F328" s="9" t="s">
         <v>28</v>
@@ -9518,7 +9518,7 @@
         <v>27</v>
       </c>
       <c r="E329" s="11">
-        <v>24</v>
+        <v>8</v>
       </c>
       <c r="F329" s="9" t="s">
         <v>28</v>
@@ -9541,7 +9541,7 @@
         <v>27</v>
       </c>
       <c r="E330" s="11">
-        <v>13</v>
+        <v>17</v>
       </c>
       <c r="F330" s="9" t="s">
         <v>28</v>
@@ -9564,7 +9564,7 @@
         <v>27</v>
       </c>
       <c r="E331" s="11">
-        <v>8</v>
+        <v>11</v>
       </c>
       <c r="F331" s="9" t="s">
         <v>28</v>
@@ -9587,7 +9587,7 @@
         <v>27</v>
       </c>
       <c r="E332" s="11">
-        <v>15</v>
+        <v>17</v>
       </c>
       <c r="F332" s="9" t="s">
         <v>28</v>
@@ -9610,7 +9610,7 @@
         <v>27</v>
       </c>
       <c r="E333" s="11">
-        <v>24</v>
+        <v>21</v>
       </c>
       <c r="F333" s="9" t="s">
         <v>28</v>
@@ -9633,7 +9633,7 @@
         <v>27</v>
       </c>
       <c r="E334" s="11">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="F334" s="9" t="s">
         <v>28</v>
@@ -9656,7 +9656,7 @@
         <v>27</v>
       </c>
       <c r="E335" s="11">
-        <v>18</v>
+        <v>23</v>
       </c>
       <c r="F335" s="9" t="s">
         <v>28</v>
@@ -9679,7 +9679,7 @@
         <v>27</v>
       </c>
       <c r="E336" s="11">
-        <v>22</v>
+        <v>12</v>
       </c>
       <c r="F336" s="9" t="s">
         <v>28</v>
@@ -9702,7 +9702,7 @@
         <v>27</v>
       </c>
       <c r="E337" s="11">
-        <v>19</v>
+        <v>25</v>
       </c>
       <c r="F337" s="9" t="s">
         <v>28</v>
@@ -9725,7 +9725,7 @@
         <v>27</v>
       </c>
       <c r="E338" s="11">
-        <v>28</v>
+        <v>31</v>
       </c>
       <c r="F338" s="9" t="s">
         <v>28</v>
@@ -9748,7 +9748,7 @@
         <v>27</v>
       </c>
       <c r="E339" s="11">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="F339" s="9" t="s">
         <v>28</v>
@@ -9771,7 +9771,7 @@
         <v>27</v>
       </c>
       <c r="E340" s="11">
-        <v>20</v>
+        <v>13</v>
       </c>
       <c r="F340" s="9" t="s">
         <v>28</v>
@@ -9794,7 +9794,7 @@
         <v>27</v>
       </c>
       <c r="E341" s="11">
-        <v>28</v>
+        <v>18</v>
       </c>
       <c r="F341" s="9" t="s">
         <v>28</v>
@@ -9817,7 +9817,7 @@
         <v>27</v>
       </c>
       <c r="E342" s="11">
-        <v>13</v>
+        <v>21</v>
       </c>
       <c r="F342" s="9" t="s">
         <v>28</v>
@@ -9840,7 +9840,7 @@
         <v>27</v>
       </c>
       <c r="E343" s="11">
-        <v>17</v>
+        <v>30</v>
       </c>
       <c r="F343" s="9" t="s">
         <v>28</v>
@@ -9863,7 +9863,7 @@
         <v>27</v>
       </c>
       <c r="E344" s="11">
-        <v>23</v>
+        <v>13</v>
       </c>
       <c r="F344" s="9" t="s">
         <v>28</v>
@@ -9886,7 +9886,7 @@
         <v>27</v>
       </c>
       <c r="E345" s="11">
-        <v>27</v>
+        <v>17</v>
       </c>
       <c r="F345" s="9" t="s">
         <v>28</v>
@@ -9909,7 +9909,7 @@
         <v>27</v>
       </c>
       <c r="E346" s="11">
-        <v>10</v>
+        <v>17</v>
       </c>
       <c r="F346" s="9" t="s">
         <v>28</v>
@@ -9932,7 +9932,7 @@
         <v>27</v>
       </c>
       <c r="E347" s="11">
-        <v>27</v>
+        <v>14</v>
       </c>
       <c r="F347" s="9" t="s">
         <v>28</v>
@@ -9955,7 +9955,7 @@
         <v>27</v>
       </c>
       <c r="E348" s="11">
-        <v>20</v>
+        <v>26</v>
       </c>
       <c r="F348" s="9" t="s">
         <v>28</v>
@@ -9978,7 +9978,7 @@
         <v>27</v>
       </c>
       <c r="E349" s="11">
-        <v>8</v>
+        <v>13</v>
       </c>
       <c r="F349" s="9" t="s">
         <v>28</v>
@@ -10001,7 +10001,7 @@
         <v>27</v>
       </c>
       <c r="E350" s="11">
-        <v>23</v>
+        <v>21</v>
       </c>
       <c r="F350" s="9" t="s">
         <v>28</v>
@@ -10024,7 +10024,7 @@
         <v>27</v>
       </c>
       <c r="E351" s="11">
-        <v>28</v>
+        <v>18</v>
       </c>
       <c r="F351" s="9" t="s">
         <v>28</v>
@@ -10047,7 +10047,7 @@
         <v>27</v>
       </c>
       <c r="E352" s="11">
-        <v>13</v>
+        <v>18</v>
       </c>
       <c r="F352" s="9" t="s">
         <v>28</v>
@@ -10070,7 +10070,7 @@
         <v>27</v>
       </c>
       <c r="E353" s="11">
-        <v>11</v>
+        <v>29</v>
       </c>
       <c r="F353" s="9" t="s">
         <v>28</v>
@@ -10093,7 +10093,7 @@
         <v>27</v>
       </c>
       <c r="E354" s="11">
-        <v>12</v>
+        <v>27</v>
       </c>
       <c r="F354" s="9" t="s">
         <v>28</v>
@@ -10116,7 +10116,7 @@
         <v>27</v>
       </c>
       <c r="E355" s="11">
-        <v>29</v>
+        <v>19</v>
       </c>
       <c r="F355" s="9" t="s">
         <v>28</v>
@@ -10139,7 +10139,7 @@
         <v>27</v>
       </c>
       <c r="E356" s="11">
-        <v>30</v>
+        <v>26</v>
       </c>
       <c r="F356" s="9" t="s">
         <v>28</v>
@@ -10162,7 +10162,7 @@
         <v>27</v>
       </c>
       <c r="E357" s="11">
-        <v>15</v>
+        <v>30</v>
       </c>
       <c r="F357" s="9" t="s">
         <v>28</v>
@@ -10185,7 +10185,7 @@
         <v>27</v>
       </c>
       <c r="E358" s="11">
-        <v>12</v>
+        <v>24</v>
       </c>
       <c r="F358" s="9" t="s">
         <v>28</v>
@@ -10208,7 +10208,7 @@
         <v>27</v>
       </c>
       <c r="E359" s="11">
-        <v>8</v>
+        <v>30</v>
       </c>
       <c r="F359" s="9" t="s">
         <v>28</v>
@@ -10231,7 +10231,7 @@
         <v>27</v>
       </c>
       <c r="E360" s="11">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="F360" s="9" t="s">
         <v>28</v>
@@ -10254,7 +10254,7 @@
         <v>27</v>
       </c>
       <c r="E361" s="11">
-        <v>30</v>
+        <v>25</v>
       </c>
       <c r="F361" s="9" t="s">
         <v>28</v>
@@ -10277,7 +10277,7 @@
         <v>27</v>
       </c>
       <c r="E362" s="11">
-        <v>14</v>
+        <v>25</v>
       </c>
       <c r="F362" s="9" t="s">
         <v>28</v>
@@ -10300,7 +10300,7 @@
         <v>27</v>
       </c>
       <c r="E363" s="11">
-        <v>13</v>
+        <v>21</v>
       </c>
       <c r="F363" s="9" t="s">
         <v>28</v>
@@ -10323,7 +10323,7 @@
         <v>27</v>
       </c>
       <c r="E364" s="11">
-        <v>27</v>
+        <v>30</v>
       </c>
       <c r="F364" s="9" t="s">
         <v>28</v>
@@ -10346,7 +10346,7 @@
         <v>27</v>
       </c>
       <c r="E365" s="11">
-        <v>23</v>
+        <v>11</v>
       </c>
       <c r="F365" s="9" t="s">
         <v>28</v>
@@ -10369,7 +10369,7 @@
         <v>27</v>
       </c>
       <c r="E366" s="11">
-        <v>31</v>
+        <v>29</v>
       </c>
       <c r="F366" s="9" t="s">
         <v>28</v>
@@ -10392,7 +10392,7 @@
         <v>27</v>
       </c>
       <c r="E367" s="11">
-        <v>18</v>
+        <v>31</v>
       </c>
       <c r="F367" s="9" t="s">
         <v>28</v>
@@ -10415,7 +10415,7 @@
         <v>27</v>
       </c>
       <c r="E368" s="11">
-        <v>15</v>
+        <v>27</v>
       </c>
       <c r="F368" s="9" t="s">
         <v>28</v>
@@ -10438,7 +10438,7 @@
         <v>27</v>
       </c>
       <c r="E369" s="11">
-        <v>24</v>
+        <v>14</v>
       </c>
       <c r="F369" s="9" t="s">
         <v>28</v>
@@ -10461,7 +10461,7 @@
         <v>27</v>
       </c>
       <c r="E370" s="11">
-        <v>28</v>
+        <v>15</v>
       </c>
       <c r="F370" s="9" t="s">
         <v>28</v>
@@ -10484,7 +10484,7 @@
         <v>27</v>
       </c>
       <c r="E371" s="11">
-        <v>13</v>
+        <v>8</v>
       </c>
       <c r="F371" s="9" t="s">
         <v>28</v>
@@ -10507,7 +10507,7 @@
         <v>27</v>
       </c>
       <c r="E372" s="11">
-        <v>13</v>
+        <v>17</v>
       </c>
       <c r="F372" s="9" t="s">
         <v>28</v>
@@ -10530,7 +10530,7 @@
         <v>27</v>
       </c>
       <c r="E373" s="11">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="F373" s="9" t="s">
         <v>28</v>
@@ -10553,7 +10553,7 @@
         <v>27</v>
       </c>
       <c r="E374" s="11">
-        <v>9</v>
+        <v>13</v>
       </c>
       <c r="F374" s="9" t="s">
         <v>28</v>
@@ -10576,7 +10576,7 @@
         <v>27</v>
       </c>
       <c r="E375" s="11">
-        <v>11</v>
+        <v>29</v>
       </c>
       <c r="F375" s="9" t="s">
         <v>28</v>
@@ -10599,7 +10599,7 @@
         <v>27</v>
       </c>
       <c r="E376" s="11">
-        <v>29</v>
+        <v>17</v>
       </c>
       <c r="F376" s="9" t="s">
         <v>28</v>
@@ -10622,7 +10622,7 @@
         <v>27</v>
       </c>
       <c r="E377" s="11">
-        <v>8</v>
+        <v>13</v>
       </c>
       <c r="F377" s="9" t="s">
         <v>28</v>
@@ -10645,7 +10645,7 @@
         <v>27</v>
       </c>
       <c r="E378" s="11">
-        <v>26</v>
+        <v>29</v>
       </c>
       <c r="F378" s="9" t="s">
         <v>28</v>
@@ -10668,7 +10668,7 @@
         <v>27</v>
       </c>
       <c r="E379" s="11">
-        <v>23</v>
+        <v>29</v>
       </c>
       <c r="F379" s="9" t="s">
         <v>28</v>
@@ -10691,7 +10691,7 @@
         <v>27</v>
       </c>
       <c r="E380" s="11">
-        <v>16</v>
+        <v>9</v>
       </c>
       <c r="F380" s="9" t="s">
         <v>28</v>
@@ -10714,7 +10714,7 @@
         <v>27</v>
       </c>
       <c r="E381" s="11">
-        <v>27</v>
+        <v>20</v>
       </c>
       <c r="F381" s="9" t="s">
         <v>28</v>
@@ -10737,7 +10737,7 @@
         <v>27</v>
       </c>
       <c r="E382" s="11">
-        <v>8</v>
+        <v>21</v>
       </c>
       <c r="F382" s="9" t="s">
         <v>28</v>
@@ -10760,7 +10760,7 @@
         <v>27</v>
       </c>
       <c r="E383" s="11">
-        <v>20</v>
+        <v>24</v>
       </c>
       <c r="F383" s="9" t="s">
         <v>28</v>
@@ -10783,7 +10783,7 @@
         <v>27</v>
       </c>
       <c r="E384" s="11">
-        <v>15</v>
+        <v>22</v>
       </c>
       <c r="F384" s="9" t="s">
         <v>28</v>
@@ -10806,7 +10806,7 @@
         <v>27</v>
       </c>
       <c r="E385" s="11">
-        <v>14</v>
+        <v>25</v>
       </c>
       <c r="F385" s="9" t="s">
         <v>28</v>
@@ -10829,7 +10829,7 @@
         <v>27</v>
       </c>
       <c r="E386" s="11">
-        <v>23</v>
+        <v>8</v>
       </c>
       <c r="F386" s="9" t="s">
         <v>28</v>
@@ -10852,7 +10852,7 @@
         <v>27</v>
       </c>
       <c r="E387" s="11">
-        <v>31</v>
+        <v>17</v>
       </c>
       <c r="F387" s="9" t="s">
         <v>28</v>
@@ -10875,7 +10875,7 @@
         <v>27</v>
       </c>
       <c r="E388" s="11">
-        <v>18</v>
+        <v>27</v>
       </c>
       <c r="F388" s="9" t="s">
         <v>28</v>
@@ -10898,7 +10898,7 @@
         <v>27</v>
       </c>
       <c r="E389" s="11">
-        <v>26</v>
+        <v>19</v>
       </c>
       <c r="F389" s="9" t="s">
         <v>28</v>
@@ -10921,7 +10921,7 @@
         <v>27</v>
       </c>
       <c r="E390" s="11">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="F390" s="9" t="s">
         <v>28</v>
@@ -10944,7 +10944,7 @@
         <v>27</v>
       </c>
       <c r="E391" s="11">
-        <v>17</v>
+        <v>29</v>
       </c>
       <c r="F391" s="9" t="s">
         <v>28</v>
@@ -10967,7 +10967,7 @@
         <v>27</v>
       </c>
       <c r="E392" s="11">
-        <v>18</v>
+        <v>21</v>
       </c>
       <c r="F392" s="9" t="s">
         <v>28</v>
@@ -10990,7 +10990,7 @@
         <v>27</v>
       </c>
       <c r="E393" s="11">
-        <v>29</v>
+        <v>15</v>
       </c>
       <c r="F393" s="9" t="s">
         <v>28</v>
@@ -11013,7 +11013,7 @@
         <v>27</v>
       </c>
       <c r="E394" s="11">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="F394" s="9" t="s">
         <v>28</v>
@@ -11036,7 +11036,7 @@
         <v>27</v>
       </c>
       <c r="E395" s="11">
-        <v>20</v>
+        <v>31</v>
       </c>
       <c r="F395" s="9" t="s">
         <v>28</v>
@@ -11059,7 +11059,7 @@
         <v>27</v>
       </c>
       <c r="E396" s="11">
-        <v>31</v>
+        <v>13</v>
       </c>
       <c r="F396" s="9" t="s">
         <v>28</v>
@@ -11082,7 +11082,7 @@
         <v>27</v>
       </c>
       <c r="E397" s="11">
-        <v>22</v>
+        <v>28</v>
       </c>
       <c r="F397" s="9" t="s">
         <v>28</v>
@@ -11128,7 +11128,7 @@
         <v>27</v>
       </c>
       <c r="E399" s="11">
-        <v>8</v>
+        <v>17</v>
       </c>
       <c r="F399" s="9" t="s">
         <v>28</v>
@@ -11151,7 +11151,7 @@
         <v>27</v>
       </c>
       <c r="E400" s="11">
-        <v>20</v>
+        <v>22</v>
       </c>
       <c r="F400" s="9" t="s">
         <v>28</v>
@@ -11174,7 +11174,7 @@
         <v>27</v>
       </c>
       <c r="E401" s="11">
-        <v>19</v>
+        <v>12</v>
       </c>
       <c r="F401" s="9" t="s">
         <v>28</v>

</xml_diff>

<commit_message>
fix(rating): set initial rating default to 0 and compute dynamic rating when users submit reviews
</commit_message>
<xml_diff>
--- a/all-test-reports/selenium/selenium_e2e_test_report.xlsx
+++ b/all-test-reports/selenium/selenium_e2e_test_report.xlsx
@@ -35,7 +35,7 @@
     <t>Execution Date</t>
   </si>
   <si>
-    <t>28/7/2026, 11:37:58 am</t>
+    <t>28/7/2026, 11:40:41 am</t>
   </si>
   <si>
     <t>Browser / Mode</t>
@@ -98,7 +98,7 @@
     <t>PASS</t>
   </si>
   <si>
-    <t>11:37:58 am</t>
+    <t>11:40:41 am</t>
   </si>
   <si>
     <t>N/A</t>
@@ -1997,7 +1997,7 @@
         <v>27</v>
       </c>
       <c r="E2" s="11">
-        <v>23</v>
+        <v>31</v>
       </c>
       <c r="F2" s="9" t="s">
         <v>28</v>
@@ -2020,7 +2020,7 @@
         <v>27</v>
       </c>
       <c r="E3" s="11">
-        <v>17</v>
+        <v>8</v>
       </c>
       <c r="F3" s="9" t="s">
         <v>28</v>
@@ -2043,7 +2043,7 @@
         <v>27</v>
       </c>
       <c r="E4" s="11">
-        <v>26</v>
+        <v>19</v>
       </c>
       <c r="F4" s="9" t="s">
         <v>28</v>
@@ -2066,7 +2066,7 @@
         <v>27</v>
       </c>
       <c r="E5" s="11">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="F5" s="9" t="s">
         <v>28</v>
@@ -2089,7 +2089,7 @@
         <v>27</v>
       </c>
       <c r="E6" s="11">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="F6" s="9" t="s">
         <v>28</v>
@@ -2112,7 +2112,7 @@
         <v>27</v>
       </c>
       <c r="E7" s="11">
-        <v>31</v>
+        <v>29</v>
       </c>
       <c r="F7" s="9" t="s">
         <v>28</v>
@@ -2135,7 +2135,7 @@
         <v>27</v>
       </c>
       <c r="E8" s="11">
-        <v>22</v>
+        <v>17</v>
       </c>
       <c r="F8" s="9" t="s">
         <v>28</v>
@@ -2158,7 +2158,7 @@
         <v>27</v>
       </c>
       <c r="E9" s="11">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="F9" s="9" t="s">
         <v>28</v>
@@ -2181,7 +2181,7 @@
         <v>27</v>
       </c>
       <c r="E10" s="11">
-        <v>12</v>
+        <v>23</v>
       </c>
       <c r="F10" s="9" t="s">
         <v>28</v>
@@ -2204,7 +2204,7 @@
         <v>27</v>
       </c>
       <c r="E11" s="11">
-        <v>11</v>
+        <v>21</v>
       </c>
       <c r="F11" s="9" t="s">
         <v>28</v>
@@ -2227,7 +2227,7 @@
         <v>27</v>
       </c>
       <c r="E12" s="11">
-        <v>13</v>
+        <v>17</v>
       </c>
       <c r="F12" s="9" t="s">
         <v>28</v>
@@ -2250,7 +2250,7 @@
         <v>27</v>
       </c>
       <c r="E13" s="11">
-        <v>17</v>
+        <v>26</v>
       </c>
       <c r="F13" s="9" t="s">
         <v>28</v>
@@ -2273,7 +2273,7 @@
         <v>27</v>
       </c>
       <c r="E14" s="11">
-        <v>16</v>
+        <v>30</v>
       </c>
       <c r="F14" s="9" t="s">
         <v>28</v>
@@ -2296,7 +2296,7 @@
         <v>27</v>
       </c>
       <c r="E15" s="11">
-        <v>20</v>
+        <v>25</v>
       </c>
       <c r="F15" s="9" t="s">
         <v>28</v>
@@ -2319,7 +2319,7 @@
         <v>27</v>
       </c>
       <c r="E16" s="11">
-        <v>19</v>
+        <v>10</v>
       </c>
       <c r="F16" s="9" t="s">
         <v>28</v>
@@ -2342,7 +2342,7 @@
         <v>27</v>
       </c>
       <c r="E17" s="11">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="F17" s="9" t="s">
         <v>28</v>
@@ -2365,7 +2365,7 @@
         <v>27</v>
       </c>
       <c r="E18" s="11">
-        <v>20</v>
+        <v>29</v>
       </c>
       <c r="F18" s="9" t="s">
         <v>28</v>
@@ -2388,7 +2388,7 @@
         <v>27</v>
       </c>
       <c r="E19" s="11">
-        <v>10</v>
+        <v>17</v>
       </c>
       <c r="F19" s="9" t="s">
         <v>28</v>
@@ -2411,7 +2411,7 @@
         <v>27</v>
       </c>
       <c r="E20" s="11">
-        <v>14</v>
+        <v>9</v>
       </c>
       <c r="F20" s="9" t="s">
         <v>28</v>
@@ -2434,7 +2434,7 @@
         <v>27</v>
       </c>
       <c r="E21" s="11">
-        <v>11</v>
+        <v>16</v>
       </c>
       <c r="F21" s="9" t="s">
         <v>28</v>
@@ -2457,7 +2457,7 @@
         <v>27</v>
       </c>
       <c r="E22" s="11">
-        <v>25</v>
+        <v>29</v>
       </c>
       <c r="F22" s="9" t="s">
         <v>28</v>
@@ -2480,7 +2480,7 @@
         <v>27</v>
       </c>
       <c r="E23" s="11">
-        <v>29</v>
+        <v>17</v>
       </c>
       <c r="F23" s="9" t="s">
         <v>28</v>
@@ -2503,7 +2503,7 @@
         <v>27</v>
       </c>
       <c r="E24" s="11">
-        <v>16</v>
+        <v>11</v>
       </c>
       <c r="F24" s="9" t="s">
         <v>28</v>
@@ -2526,7 +2526,7 @@
         <v>27</v>
       </c>
       <c r="E25" s="11">
-        <v>15</v>
+        <v>17</v>
       </c>
       <c r="F25" s="9" t="s">
         <v>28</v>
@@ -2549,7 +2549,7 @@
         <v>27</v>
       </c>
       <c r="E26" s="11">
-        <v>28</v>
+        <v>24</v>
       </c>
       <c r="F26" s="9" t="s">
         <v>28</v>
@@ -2572,7 +2572,7 @@
         <v>27</v>
       </c>
       <c r="E27" s="11">
-        <v>17</v>
+        <v>11</v>
       </c>
       <c r="F27" s="9" t="s">
         <v>28</v>
@@ -2595,7 +2595,7 @@
         <v>27</v>
       </c>
       <c r="E28" s="11">
-        <v>16</v>
+        <v>29</v>
       </c>
       <c r="F28" s="9" t="s">
         <v>28</v>
@@ -2618,7 +2618,7 @@
         <v>27</v>
       </c>
       <c r="E29" s="11">
-        <v>29</v>
+        <v>11</v>
       </c>
       <c r="F29" s="9" t="s">
         <v>28</v>
@@ -2641,7 +2641,7 @@
         <v>27</v>
       </c>
       <c r="E30" s="11">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="F30" s="9" t="s">
         <v>28</v>
@@ -2664,7 +2664,7 @@
         <v>27</v>
       </c>
       <c r="E31" s="11">
-        <v>20</v>
+        <v>9</v>
       </c>
       <c r="F31" s="9" t="s">
         <v>28</v>
@@ -2687,7 +2687,7 @@
         <v>27</v>
       </c>
       <c r="E32" s="11">
-        <v>16</v>
+        <v>26</v>
       </c>
       <c r="F32" s="9" t="s">
         <v>28</v>
@@ -2710,7 +2710,7 @@
         <v>27</v>
       </c>
       <c r="E33" s="11">
-        <v>12</v>
+        <v>8</v>
       </c>
       <c r="F33" s="9" t="s">
         <v>28</v>
@@ -2733,7 +2733,7 @@
         <v>27</v>
       </c>
       <c r="E34" s="11">
-        <v>12</v>
+        <v>21</v>
       </c>
       <c r="F34" s="9" t="s">
         <v>28</v>
@@ -2756,7 +2756,7 @@
         <v>27</v>
       </c>
       <c r="E35" s="11">
-        <v>20</v>
+        <v>9</v>
       </c>
       <c r="F35" s="9" t="s">
         <v>28</v>
@@ -2779,7 +2779,7 @@
         <v>27</v>
       </c>
       <c r="E36" s="11">
-        <v>24</v>
+        <v>26</v>
       </c>
       <c r="F36" s="9" t="s">
         <v>28</v>
@@ -2802,7 +2802,7 @@
         <v>27</v>
       </c>
       <c r="E37" s="11">
-        <v>23</v>
+        <v>13</v>
       </c>
       <c r="F37" s="9" t="s">
         <v>28</v>
@@ -2825,7 +2825,7 @@
         <v>27</v>
       </c>
       <c r="E38" s="11">
-        <v>29</v>
+        <v>24</v>
       </c>
       <c r="F38" s="9" t="s">
         <v>28</v>
@@ -2848,7 +2848,7 @@
         <v>27</v>
       </c>
       <c r="E39" s="11">
-        <v>26</v>
+        <v>29</v>
       </c>
       <c r="F39" s="9" t="s">
         <v>28</v>
@@ -2871,7 +2871,7 @@
         <v>27</v>
       </c>
       <c r="E40" s="11">
-        <v>25</v>
+        <v>17</v>
       </c>
       <c r="F40" s="9" t="s">
         <v>28</v>
@@ -2894,7 +2894,7 @@
         <v>27</v>
       </c>
       <c r="E41" s="11">
-        <v>11</v>
+        <v>26</v>
       </c>
       <c r="F41" s="9" t="s">
         <v>28</v>
@@ -2917,7 +2917,7 @@
         <v>27</v>
       </c>
       <c r="E42" s="11">
-        <v>14</v>
+        <v>9</v>
       </c>
       <c r="F42" s="9" t="s">
         <v>28</v>
@@ -2940,7 +2940,7 @@
         <v>27</v>
       </c>
       <c r="E43" s="11">
-        <v>21</v>
+        <v>26</v>
       </c>
       <c r="F43" s="9" t="s">
         <v>28</v>
@@ -2963,7 +2963,7 @@
         <v>27</v>
       </c>
       <c r="E44" s="11">
-        <v>19</v>
+        <v>13</v>
       </c>
       <c r="F44" s="9" t="s">
         <v>28</v>
@@ -2986,7 +2986,7 @@
         <v>27</v>
       </c>
       <c r="E45" s="11">
-        <v>10</v>
+        <v>29</v>
       </c>
       <c r="F45" s="9" t="s">
         <v>28</v>
@@ -3009,7 +3009,7 @@
         <v>27</v>
       </c>
       <c r="E46" s="11">
-        <v>23</v>
+        <v>26</v>
       </c>
       <c r="F46" s="9" t="s">
         <v>28</v>
@@ -3032,7 +3032,7 @@
         <v>27</v>
       </c>
       <c r="E47" s="11">
-        <v>27</v>
+        <v>30</v>
       </c>
       <c r="F47" s="9" t="s">
         <v>28</v>
@@ -3055,7 +3055,7 @@
         <v>27</v>
       </c>
       <c r="E48" s="11">
-        <v>30</v>
+        <v>12</v>
       </c>
       <c r="F48" s="9" t="s">
         <v>28</v>
@@ -3078,7 +3078,7 @@
         <v>27</v>
       </c>
       <c r="E49" s="11">
-        <v>16</v>
+        <v>22</v>
       </c>
       <c r="F49" s="9" t="s">
         <v>28</v>
@@ -3101,7 +3101,7 @@
         <v>27</v>
       </c>
       <c r="E50" s="11">
-        <v>31</v>
+        <v>12</v>
       </c>
       <c r="F50" s="9" t="s">
         <v>28</v>
@@ -3124,7 +3124,7 @@
         <v>27</v>
       </c>
       <c r="E51" s="11">
-        <v>16</v>
+        <v>26</v>
       </c>
       <c r="F51" s="9" t="s">
         <v>28</v>
@@ -3147,7 +3147,7 @@
         <v>27</v>
       </c>
       <c r="E52" s="11">
-        <v>11</v>
+        <v>15</v>
       </c>
       <c r="F52" s="9" t="s">
         <v>28</v>
@@ -3170,7 +3170,7 @@
         <v>27</v>
       </c>
       <c r="E53" s="11">
-        <v>27</v>
+        <v>22</v>
       </c>
       <c r="F53" s="9" t="s">
         <v>28</v>
@@ -3193,7 +3193,7 @@
         <v>27</v>
       </c>
       <c r="E54" s="11">
-        <v>15</v>
+        <v>8</v>
       </c>
       <c r="F54" s="9" t="s">
         <v>28</v>
@@ -3216,7 +3216,7 @@
         <v>27</v>
       </c>
       <c r="E55" s="11">
-        <v>8</v>
+        <v>16</v>
       </c>
       <c r="F55" s="9" t="s">
         <v>28</v>
@@ -3239,7 +3239,7 @@
         <v>27</v>
       </c>
       <c r="E56" s="11">
-        <v>8</v>
+        <v>14</v>
       </c>
       <c r="F56" s="9" t="s">
         <v>28</v>
@@ -3262,7 +3262,7 @@
         <v>27</v>
       </c>
       <c r="E57" s="11">
-        <v>22</v>
+        <v>14</v>
       </c>
       <c r="F57" s="9" t="s">
         <v>28</v>
@@ -3285,7 +3285,7 @@
         <v>27</v>
       </c>
       <c r="E58" s="11">
-        <v>15</v>
+        <v>20</v>
       </c>
       <c r="F58" s="9" t="s">
         <v>28</v>
@@ -3308,7 +3308,7 @@
         <v>27</v>
       </c>
       <c r="E59" s="11">
-        <v>15</v>
+        <v>10</v>
       </c>
       <c r="F59" s="9" t="s">
         <v>28</v>
@@ -3331,7 +3331,7 @@
         <v>27</v>
       </c>
       <c r="E60" s="11">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="F60" s="9" t="s">
         <v>28</v>
@@ -3354,7 +3354,7 @@
         <v>27</v>
       </c>
       <c r="E61" s="11">
-        <v>29</v>
+        <v>20</v>
       </c>
       <c r="F61" s="9" t="s">
         <v>28</v>
@@ -3377,7 +3377,7 @@
         <v>27</v>
       </c>
       <c r="E62" s="11">
-        <v>10</v>
+        <v>25</v>
       </c>
       <c r="F62" s="9" t="s">
         <v>28</v>
@@ -3400,7 +3400,7 @@
         <v>27</v>
       </c>
       <c r="E63" s="11">
-        <v>15</v>
+        <v>30</v>
       </c>
       <c r="F63" s="9" t="s">
         <v>28</v>
@@ -3423,7 +3423,7 @@
         <v>27</v>
       </c>
       <c r="E64" s="11">
-        <v>23</v>
+        <v>13</v>
       </c>
       <c r="F64" s="9" t="s">
         <v>28</v>
@@ -3446,7 +3446,7 @@
         <v>27</v>
       </c>
       <c r="E65" s="11">
-        <v>10</v>
+        <v>23</v>
       </c>
       <c r="F65" s="9" t="s">
         <v>28</v>
@@ -3469,7 +3469,7 @@
         <v>27</v>
       </c>
       <c r="E66" s="11">
-        <v>24</v>
+        <v>15</v>
       </c>
       <c r="F66" s="9" t="s">
         <v>28</v>
@@ -3515,7 +3515,7 @@
         <v>27</v>
       </c>
       <c r="E68" s="11">
-        <v>12</v>
+        <v>9</v>
       </c>
       <c r="F68" s="9" t="s">
         <v>28</v>
@@ -3538,7 +3538,7 @@
         <v>27</v>
       </c>
       <c r="E69" s="11">
-        <v>19</v>
+        <v>22</v>
       </c>
       <c r="F69" s="9" t="s">
         <v>28</v>
@@ -3561,7 +3561,7 @@
         <v>27</v>
       </c>
       <c r="E70" s="11">
-        <v>11</v>
+        <v>17</v>
       </c>
       <c r="F70" s="9" t="s">
         <v>28</v>
@@ -3584,7 +3584,7 @@
         <v>27</v>
       </c>
       <c r="E71" s="11">
-        <v>25</v>
+        <v>10</v>
       </c>
       <c r="F71" s="9" t="s">
         <v>28</v>
@@ -3607,7 +3607,7 @@
         <v>27</v>
       </c>
       <c r="E72" s="11">
-        <v>16</v>
+        <v>27</v>
       </c>
       <c r="F72" s="9" t="s">
         <v>28</v>
@@ -3630,7 +3630,7 @@
         <v>27</v>
       </c>
       <c r="E73" s="11">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="F73" s="9" t="s">
         <v>28</v>
@@ -3653,7 +3653,7 @@
         <v>27</v>
       </c>
       <c r="E74" s="11">
-        <v>21</v>
+        <v>12</v>
       </c>
       <c r="F74" s="9" t="s">
         <v>28</v>
@@ -3676,7 +3676,7 @@
         <v>27</v>
       </c>
       <c r="E75" s="11">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="F75" s="9" t="s">
         <v>28</v>
@@ -3699,7 +3699,7 @@
         <v>27</v>
       </c>
       <c r="E76" s="11">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="F76" s="9" t="s">
         <v>28</v>
@@ -3722,7 +3722,7 @@
         <v>27</v>
       </c>
       <c r="E77" s="11">
-        <v>13</v>
+        <v>9</v>
       </c>
       <c r="F77" s="9" t="s">
         <v>28</v>
@@ -3745,7 +3745,7 @@
         <v>27</v>
       </c>
       <c r="E78" s="11">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="F78" s="9" t="s">
         <v>28</v>
@@ -3768,7 +3768,7 @@
         <v>27</v>
       </c>
       <c r="E79" s="11">
-        <v>9</v>
+        <v>22</v>
       </c>
       <c r="F79" s="9" t="s">
         <v>28</v>
@@ -3791,7 +3791,7 @@
         <v>27</v>
       </c>
       <c r="E80" s="11">
-        <v>9</v>
+        <v>19</v>
       </c>
       <c r="F80" s="9" t="s">
         <v>28</v>
@@ -3814,7 +3814,7 @@
         <v>27</v>
       </c>
       <c r="E81" s="11">
-        <v>27</v>
+        <v>15</v>
       </c>
       <c r="F81" s="9" t="s">
         <v>28</v>
@@ -3837,7 +3837,7 @@
         <v>27</v>
       </c>
       <c r="E82" s="11">
-        <v>23</v>
+        <v>15</v>
       </c>
       <c r="F82" s="9" t="s">
         <v>28</v>
@@ -3860,7 +3860,7 @@
         <v>27</v>
       </c>
       <c r="E83" s="11">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="F83" s="9" t="s">
         <v>28</v>
@@ -3883,7 +3883,7 @@
         <v>27</v>
       </c>
       <c r="E84" s="11">
-        <v>28</v>
+        <v>30</v>
       </c>
       <c r="F84" s="9" t="s">
         <v>28</v>
@@ -3906,7 +3906,7 @@
         <v>27</v>
       </c>
       <c r="E85" s="11">
-        <v>14</v>
+        <v>11</v>
       </c>
       <c r="F85" s="9" t="s">
         <v>28</v>
@@ -3929,7 +3929,7 @@
         <v>27</v>
       </c>
       <c r="E86" s="11">
-        <v>25</v>
+        <v>21</v>
       </c>
       <c r="F86" s="9" t="s">
         <v>28</v>
@@ -3952,7 +3952,7 @@
         <v>27</v>
       </c>
       <c r="E87" s="11">
-        <v>13</v>
+        <v>23</v>
       </c>
       <c r="F87" s="9" t="s">
         <v>28</v>
@@ -3975,7 +3975,7 @@
         <v>27</v>
       </c>
       <c r="E88" s="11">
-        <v>12</v>
+        <v>10</v>
       </c>
       <c r="F88" s="9" t="s">
         <v>28</v>
@@ -3998,7 +3998,7 @@
         <v>27</v>
       </c>
       <c r="E89" s="11">
-        <v>26</v>
+        <v>10</v>
       </c>
       <c r="F89" s="9" t="s">
         <v>28</v>
@@ -4021,7 +4021,7 @@
         <v>27</v>
       </c>
       <c r="E90" s="11">
-        <v>31</v>
+        <v>8</v>
       </c>
       <c r="F90" s="9" t="s">
         <v>28</v>
@@ -4044,7 +4044,7 @@
         <v>27</v>
       </c>
       <c r="E91" s="11">
-        <v>23</v>
+        <v>9</v>
       </c>
       <c r="F91" s="9" t="s">
         <v>28</v>
@@ -4067,7 +4067,7 @@
         <v>27</v>
       </c>
       <c r="E92" s="11">
-        <v>13</v>
+        <v>18</v>
       </c>
       <c r="F92" s="9" t="s">
         <v>28</v>
@@ -4090,7 +4090,7 @@
         <v>27</v>
       </c>
       <c r="E93" s="11">
-        <v>21</v>
+        <v>15</v>
       </c>
       <c r="F93" s="9" t="s">
         <v>28</v>
@@ -4113,7 +4113,7 @@
         <v>27</v>
       </c>
       <c r="E94" s="11">
-        <v>16</v>
+        <v>24</v>
       </c>
       <c r="F94" s="9" t="s">
         <v>28</v>
@@ -4136,7 +4136,7 @@
         <v>27</v>
       </c>
       <c r="E95" s="11">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="F95" s="9" t="s">
         <v>28</v>
@@ -4159,7 +4159,7 @@
         <v>27</v>
       </c>
       <c r="E96" s="11">
-        <v>10</v>
+        <v>25</v>
       </c>
       <c r="F96" s="9" t="s">
         <v>28</v>
@@ -4182,7 +4182,7 @@
         <v>27</v>
       </c>
       <c r="E97" s="11">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="F97" s="9" t="s">
         <v>28</v>
@@ -4205,7 +4205,7 @@
         <v>27</v>
       </c>
       <c r="E98" s="11">
-        <v>14</v>
+        <v>31</v>
       </c>
       <c r="F98" s="9" t="s">
         <v>28</v>
@@ -4251,7 +4251,7 @@
         <v>27</v>
       </c>
       <c r="E100" s="11">
-        <v>19</v>
+        <v>12</v>
       </c>
       <c r="F100" s="9" t="s">
         <v>28</v>
@@ -4274,7 +4274,7 @@
         <v>27</v>
       </c>
       <c r="E101" s="11">
-        <v>20</v>
+        <v>15</v>
       </c>
       <c r="F101" s="9" t="s">
         <v>28</v>
@@ -4297,7 +4297,7 @@
         <v>27</v>
       </c>
       <c r="E102" s="11">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="F102" s="9" t="s">
         <v>28</v>
@@ -4320,7 +4320,7 @@
         <v>27</v>
       </c>
       <c r="E103" s="11">
-        <v>23</v>
+        <v>30</v>
       </c>
       <c r="F103" s="9" t="s">
         <v>28</v>
@@ -4343,7 +4343,7 @@
         <v>27</v>
       </c>
       <c r="E104" s="11">
-        <v>9</v>
+        <v>31</v>
       </c>
       <c r="F104" s="9" t="s">
         <v>28</v>
@@ -4366,7 +4366,7 @@
         <v>27</v>
       </c>
       <c r="E105" s="11">
-        <v>15</v>
+        <v>13</v>
       </c>
       <c r="F105" s="9" t="s">
         <v>28</v>
@@ -4389,7 +4389,7 @@
         <v>27</v>
       </c>
       <c r="E106" s="11">
-        <v>22</v>
+        <v>20</v>
       </c>
       <c r="F106" s="9" t="s">
         <v>28</v>
@@ -4412,7 +4412,7 @@
         <v>27</v>
       </c>
       <c r="E107" s="11">
-        <v>22</v>
+        <v>25</v>
       </c>
       <c r="F107" s="9" t="s">
         <v>28</v>
@@ -4435,7 +4435,7 @@
         <v>27</v>
       </c>
       <c r="E108" s="11">
-        <v>22</v>
+        <v>13</v>
       </c>
       <c r="F108" s="9" t="s">
         <v>28</v>
@@ -4481,7 +4481,7 @@
         <v>27</v>
       </c>
       <c r="E110" s="11">
-        <v>24</v>
+        <v>19</v>
       </c>
       <c r="F110" s="9" t="s">
         <v>28</v>
@@ -4504,7 +4504,7 @@
         <v>27</v>
       </c>
       <c r="E111" s="11">
-        <v>22</v>
+        <v>31</v>
       </c>
       <c r="F111" s="9" t="s">
         <v>28</v>
@@ -4550,7 +4550,7 @@
         <v>27</v>
       </c>
       <c r="E113" s="11">
-        <v>29</v>
+        <v>12</v>
       </c>
       <c r="F113" s="9" t="s">
         <v>28</v>
@@ -4573,7 +4573,7 @@
         <v>27</v>
       </c>
       <c r="E114" s="11">
-        <v>25</v>
+        <v>23</v>
       </c>
       <c r="F114" s="9" t="s">
         <v>28</v>
@@ -4596,7 +4596,7 @@
         <v>27</v>
       </c>
       <c r="E115" s="11">
-        <v>29</v>
+        <v>8</v>
       </c>
       <c r="F115" s="9" t="s">
         <v>28</v>
@@ -4619,7 +4619,7 @@
         <v>27</v>
       </c>
       <c r="E116" s="11">
-        <v>22</v>
+        <v>13</v>
       </c>
       <c r="F116" s="9" t="s">
         <v>28</v>
@@ -4642,7 +4642,7 @@
         <v>27</v>
       </c>
       <c r="E117" s="11">
-        <v>14</v>
+        <v>31</v>
       </c>
       <c r="F117" s="9" t="s">
         <v>28</v>
@@ -4665,7 +4665,7 @@
         <v>27</v>
       </c>
       <c r="E118" s="11">
-        <v>31</v>
+        <v>20</v>
       </c>
       <c r="F118" s="9" t="s">
         <v>28</v>
@@ -4688,7 +4688,7 @@
         <v>27</v>
       </c>
       <c r="E119" s="11">
-        <v>12</v>
+        <v>23</v>
       </c>
       <c r="F119" s="9" t="s">
         <v>28</v>
@@ -4734,7 +4734,7 @@
         <v>27</v>
       </c>
       <c r="E121" s="11">
-        <v>27</v>
+        <v>19</v>
       </c>
       <c r="F121" s="9" t="s">
         <v>28</v>
@@ -4757,7 +4757,7 @@
         <v>27</v>
       </c>
       <c r="E122" s="11">
-        <v>29</v>
+        <v>24</v>
       </c>
       <c r="F122" s="9" t="s">
         <v>28</v>
@@ -4780,7 +4780,7 @@
         <v>27</v>
       </c>
       <c r="E123" s="11">
-        <v>25</v>
+        <v>29</v>
       </c>
       <c r="F123" s="9" t="s">
         <v>28</v>
@@ -4803,7 +4803,7 @@
         <v>27</v>
       </c>
       <c r="E124" s="11">
-        <v>23</v>
+        <v>17</v>
       </c>
       <c r="F124" s="9" t="s">
         <v>28</v>
@@ -4826,7 +4826,7 @@
         <v>27</v>
       </c>
       <c r="E125" s="11">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="F125" s="9" t="s">
         <v>28</v>
@@ -4849,7 +4849,7 @@
         <v>27</v>
       </c>
       <c r="E126" s="11">
-        <v>13</v>
+        <v>31</v>
       </c>
       <c r="F126" s="9" t="s">
         <v>28</v>
@@ -4872,7 +4872,7 @@
         <v>27</v>
       </c>
       <c r="E127" s="11">
-        <v>20</v>
+        <v>23</v>
       </c>
       <c r="F127" s="9" t="s">
         <v>28</v>
@@ -4895,7 +4895,7 @@
         <v>27</v>
       </c>
       <c r="E128" s="11">
-        <v>14</v>
+        <v>11</v>
       </c>
       <c r="F128" s="9" t="s">
         <v>28</v>
@@ -4918,7 +4918,7 @@
         <v>27</v>
       </c>
       <c r="E129" s="11">
-        <v>28</v>
+        <v>10</v>
       </c>
       <c r="F129" s="9" t="s">
         <v>28</v>
@@ -4941,7 +4941,7 @@
         <v>27</v>
       </c>
       <c r="E130" s="11">
-        <v>13</v>
+        <v>15</v>
       </c>
       <c r="F130" s="9" t="s">
         <v>28</v>
@@ -4964,7 +4964,7 @@
         <v>27</v>
       </c>
       <c r="E131" s="11">
-        <v>12</v>
+        <v>8</v>
       </c>
       <c r="F131" s="9" t="s">
         <v>28</v>
@@ -4987,7 +4987,7 @@
         <v>27</v>
       </c>
       <c r="E132" s="11">
-        <v>13</v>
+        <v>22</v>
       </c>
       <c r="F132" s="9" t="s">
         <v>28</v>
@@ -5010,7 +5010,7 @@
         <v>27</v>
       </c>
       <c r="E133" s="11">
-        <v>23</v>
+        <v>16</v>
       </c>
       <c r="F133" s="9" t="s">
         <v>28</v>
@@ -5033,7 +5033,7 @@
         <v>27</v>
       </c>
       <c r="E134" s="11">
-        <v>8</v>
+        <v>22</v>
       </c>
       <c r="F134" s="9" t="s">
         <v>28</v>
@@ -5056,7 +5056,7 @@
         <v>27</v>
       </c>
       <c r="E135" s="11">
-        <v>22</v>
+        <v>29</v>
       </c>
       <c r="F135" s="9" t="s">
         <v>28</v>
@@ -5079,7 +5079,7 @@
         <v>27</v>
       </c>
       <c r="E136" s="11">
-        <v>27</v>
+        <v>24</v>
       </c>
       <c r="F136" s="9" t="s">
         <v>28</v>
@@ -5102,7 +5102,7 @@
         <v>27</v>
       </c>
       <c r="E137" s="11">
-        <v>18</v>
+        <v>8</v>
       </c>
       <c r="F137" s="9" t="s">
         <v>28</v>
@@ -5125,7 +5125,7 @@
         <v>27</v>
       </c>
       <c r="E138" s="11">
-        <v>17</v>
+        <v>27</v>
       </c>
       <c r="F138" s="9" t="s">
         <v>28</v>
@@ -5171,7 +5171,7 @@
         <v>27</v>
       </c>
       <c r="E140" s="11">
-        <v>22</v>
+        <v>17</v>
       </c>
       <c r="F140" s="9" t="s">
         <v>28</v>
@@ -5194,7 +5194,7 @@
         <v>27</v>
       </c>
       <c r="E141" s="11">
-        <v>11</v>
+        <v>28</v>
       </c>
       <c r="F141" s="9" t="s">
         <v>28</v>
@@ -5217,7 +5217,7 @@
         <v>27</v>
       </c>
       <c r="E142" s="11">
-        <v>23</v>
+        <v>18</v>
       </c>
       <c r="F142" s="9" t="s">
         <v>28</v>
@@ -5240,7 +5240,7 @@
         <v>27</v>
       </c>
       <c r="E143" s="11">
-        <v>8</v>
+        <v>30</v>
       </c>
       <c r="F143" s="9" t="s">
         <v>28</v>
@@ -5263,7 +5263,7 @@
         <v>27</v>
       </c>
       <c r="E144" s="11">
-        <v>28</v>
+        <v>8</v>
       </c>
       <c r="F144" s="9" t="s">
         <v>28</v>
@@ -5286,7 +5286,7 @@
         <v>27</v>
       </c>
       <c r="E145" s="11">
-        <v>31</v>
+        <v>13</v>
       </c>
       <c r="F145" s="9" t="s">
         <v>28</v>
@@ -5309,7 +5309,7 @@
         <v>27</v>
       </c>
       <c r="E146" s="11">
-        <v>31</v>
+        <v>11</v>
       </c>
       <c r="F146" s="9" t="s">
         <v>28</v>
@@ -5332,7 +5332,7 @@
         <v>27</v>
       </c>
       <c r="E147" s="11">
-        <v>24</v>
+        <v>9</v>
       </c>
       <c r="F147" s="9" t="s">
         <v>28</v>
@@ -5355,7 +5355,7 @@
         <v>27</v>
       </c>
       <c r="E148" s="11">
-        <v>20</v>
+        <v>28</v>
       </c>
       <c r="F148" s="9" t="s">
         <v>28</v>
@@ -5378,7 +5378,7 @@
         <v>27</v>
       </c>
       <c r="E149" s="11">
-        <v>16</v>
+        <v>25</v>
       </c>
       <c r="F149" s="9" t="s">
         <v>28</v>
@@ -5401,7 +5401,7 @@
         <v>27</v>
       </c>
       <c r="E150" s="11">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="F150" s="9" t="s">
         <v>28</v>
@@ -5424,7 +5424,7 @@
         <v>27</v>
       </c>
       <c r="E151" s="11">
-        <v>18</v>
+        <v>10</v>
       </c>
       <c r="F151" s="9" t="s">
         <v>28</v>
@@ -5447,7 +5447,7 @@
         <v>27</v>
       </c>
       <c r="E152" s="11">
-        <v>29</v>
+        <v>26</v>
       </c>
       <c r="F152" s="9" t="s">
         <v>28</v>
@@ -5470,7 +5470,7 @@
         <v>27</v>
       </c>
       <c r="E153" s="11">
-        <v>10</v>
+        <v>30</v>
       </c>
       <c r="F153" s="9" t="s">
         <v>28</v>
@@ -5493,7 +5493,7 @@
         <v>27</v>
       </c>
       <c r="E154" s="11">
-        <v>16</v>
+        <v>22</v>
       </c>
       <c r="F154" s="9" t="s">
         <v>28</v>
@@ -5516,7 +5516,7 @@
         <v>27</v>
       </c>
       <c r="E155" s="11">
-        <v>19</v>
+        <v>8</v>
       </c>
       <c r="F155" s="9" t="s">
         <v>28</v>
@@ -5539,7 +5539,7 @@
         <v>27</v>
       </c>
       <c r="E156" s="11">
-        <v>29</v>
+        <v>8</v>
       </c>
       <c r="F156" s="9" t="s">
         <v>28</v>
@@ -5562,7 +5562,7 @@
         <v>27</v>
       </c>
       <c r="E157" s="11">
-        <v>15</v>
+        <v>28</v>
       </c>
       <c r="F157" s="9" t="s">
         <v>28</v>
@@ -5585,7 +5585,7 @@
         <v>27</v>
       </c>
       <c r="E158" s="11">
-        <v>31</v>
+        <v>17</v>
       </c>
       <c r="F158" s="9" t="s">
         <v>28</v>
@@ -5608,7 +5608,7 @@
         <v>27</v>
       </c>
       <c r="E159" s="11">
-        <v>8</v>
+        <v>12</v>
       </c>
       <c r="F159" s="9" t="s">
         <v>28</v>
@@ -5631,7 +5631,7 @@
         <v>27</v>
       </c>
       <c r="E160" s="11">
-        <v>15</v>
+        <v>26</v>
       </c>
       <c r="F160" s="9" t="s">
         <v>28</v>
@@ -5654,7 +5654,7 @@
         <v>27</v>
       </c>
       <c r="E161" s="11">
-        <v>14</v>
+        <v>9</v>
       </c>
       <c r="F161" s="9" t="s">
         <v>28</v>
@@ -5677,7 +5677,7 @@
         <v>27</v>
       </c>
       <c r="E162" s="11">
-        <v>18</v>
+        <v>15</v>
       </c>
       <c r="F162" s="9" t="s">
         <v>28</v>
@@ -5700,7 +5700,7 @@
         <v>27</v>
       </c>
       <c r="E163" s="11">
-        <v>9</v>
+        <v>26</v>
       </c>
       <c r="F163" s="9" t="s">
         <v>28</v>
@@ -5723,7 +5723,7 @@
         <v>27</v>
       </c>
       <c r="E164" s="11">
-        <v>17</v>
+        <v>25</v>
       </c>
       <c r="F164" s="9" t="s">
         <v>28</v>
@@ -5746,7 +5746,7 @@
         <v>27</v>
       </c>
       <c r="E165" s="11">
-        <v>28</v>
+        <v>17</v>
       </c>
       <c r="F165" s="9" t="s">
         <v>28</v>
@@ -5769,7 +5769,7 @@
         <v>27</v>
       </c>
       <c r="E166" s="11">
-        <v>15</v>
+        <v>20</v>
       </c>
       <c r="F166" s="9" t="s">
         <v>28</v>
@@ -5792,7 +5792,7 @@
         <v>27</v>
       </c>
       <c r="E167" s="11">
-        <v>17</v>
+        <v>19</v>
       </c>
       <c r="F167" s="9" t="s">
         <v>28</v>
@@ -5815,7 +5815,7 @@
         <v>27</v>
       </c>
       <c r="E168" s="11">
-        <v>21</v>
+        <v>19</v>
       </c>
       <c r="F168" s="9" t="s">
         <v>28</v>
@@ -5838,7 +5838,7 @@
         <v>27</v>
       </c>
       <c r="E169" s="11">
-        <v>30</v>
+        <v>25</v>
       </c>
       <c r="F169" s="9" t="s">
         <v>28</v>
@@ -5861,7 +5861,7 @@
         <v>27</v>
       </c>
       <c r="E170" s="11">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="F170" s="9" t="s">
         <v>28</v>
@@ -5884,7 +5884,7 @@
         <v>27</v>
       </c>
       <c r="E171" s="11">
-        <v>23</v>
+        <v>17</v>
       </c>
       <c r="F171" s="9" t="s">
         <v>28</v>
@@ -5907,7 +5907,7 @@
         <v>27</v>
       </c>
       <c r="E172" s="11">
-        <v>19</v>
+        <v>9</v>
       </c>
       <c r="F172" s="9" t="s">
         <v>28</v>
@@ -5930,7 +5930,7 @@
         <v>27</v>
       </c>
       <c r="E173" s="11">
-        <v>23</v>
+        <v>25</v>
       </c>
       <c r="F173" s="9" t="s">
         <v>28</v>
@@ -5953,7 +5953,7 @@
         <v>27</v>
       </c>
       <c r="E174" s="11">
-        <v>27</v>
+        <v>16</v>
       </c>
       <c r="F174" s="9" t="s">
         <v>28</v>
@@ -5976,7 +5976,7 @@
         <v>27</v>
       </c>
       <c r="E175" s="11">
-        <v>31</v>
+        <v>22</v>
       </c>
       <c r="F175" s="9" t="s">
         <v>28</v>
@@ -5999,7 +5999,7 @@
         <v>27</v>
       </c>
       <c r="E176" s="11">
-        <v>27</v>
+        <v>11</v>
       </c>
       <c r="F176" s="9" t="s">
         <v>28</v>
@@ -6022,7 +6022,7 @@
         <v>27</v>
       </c>
       <c r="E177" s="11">
-        <v>13</v>
+        <v>9</v>
       </c>
       <c r="F177" s="9" t="s">
         <v>28</v>
@@ -6045,7 +6045,7 @@
         <v>27</v>
       </c>
       <c r="E178" s="11">
-        <v>8</v>
+        <v>28</v>
       </c>
       <c r="F178" s="9" t="s">
         <v>28</v>
@@ -6068,7 +6068,7 @@
         <v>27</v>
       </c>
       <c r="E179" s="11">
-        <v>20</v>
+        <v>18</v>
       </c>
       <c r="F179" s="9" t="s">
         <v>28</v>
@@ -6091,7 +6091,7 @@
         <v>27</v>
       </c>
       <c r="E180" s="11">
-        <v>27</v>
+        <v>8</v>
       </c>
       <c r="F180" s="9" t="s">
         <v>28</v>
@@ -6114,7 +6114,7 @@
         <v>27</v>
       </c>
       <c r="E181" s="11">
-        <v>17</v>
+        <v>9</v>
       </c>
       <c r="F181" s="9" t="s">
         <v>28</v>
@@ -6137,7 +6137,7 @@
         <v>27</v>
       </c>
       <c r="E182" s="11">
-        <v>31</v>
+        <v>9</v>
       </c>
       <c r="F182" s="9" t="s">
         <v>28</v>
@@ -6160,7 +6160,7 @@
         <v>27</v>
       </c>
       <c r="E183" s="11">
-        <v>18</v>
+        <v>8</v>
       </c>
       <c r="F183" s="9" t="s">
         <v>28</v>
@@ -6183,7 +6183,7 @@
         <v>27</v>
       </c>
       <c r="E184" s="11">
-        <v>26</v>
+        <v>22</v>
       </c>
       <c r="F184" s="9" t="s">
         <v>28</v>
@@ -6206,7 +6206,7 @@
         <v>27</v>
       </c>
       <c r="E185" s="11">
-        <v>20</v>
+        <v>10</v>
       </c>
       <c r="F185" s="9" t="s">
         <v>28</v>
@@ -6229,7 +6229,7 @@
         <v>27</v>
       </c>
       <c r="E186" s="11">
-        <v>23</v>
+        <v>11</v>
       </c>
       <c r="F186" s="9" t="s">
         <v>28</v>
@@ -6252,7 +6252,7 @@
         <v>27</v>
       </c>
       <c r="E187" s="11">
-        <v>20</v>
+        <v>31</v>
       </c>
       <c r="F187" s="9" t="s">
         <v>28</v>
@@ -6275,7 +6275,7 @@
         <v>27</v>
       </c>
       <c r="E188" s="11">
-        <v>11</v>
+        <v>13</v>
       </c>
       <c r="F188" s="9" t="s">
         <v>28</v>
@@ -6298,7 +6298,7 @@
         <v>27</v>
       </c>
       <c r="E189" s="11">
-        <v>26</v>
+        <v>24</v>
       </c>
       <c r="F189" s="9" t="s">
         <v>28</v>
@@ -6344,7 +6344,7 @@
         <v>27</v>
       </c>
       <c r="E191" s="11">
-        <v>23</v>
+        <v>26</v>
       </c>
       <c r="F191" s="9" t="s">
         <v>28</v>
@@ -6367,7 +6367,7 @@
         <v>27</v>
       </c>
       <c r="E192" s="11">
-        <v>20</v>
+        <v>8</v>
       </c>
       <c r="F192" s="9" t="s">
         <v>28</v>
@@ -6390,7 +6390,7 @@
         <v>27</v>
       </c>
       <c r="E193" s="11">
-        <v>16</v>
+        <v>18</v>
       </c>
       <c r="F193" s="9" t="s">
         <v>28</v>
@@ -6413,7 +6413,7 @@
         <v>27</v>
       </c>
       <c r="E194" s="11">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="F194" s="9" t="s">
         <v>28</v>
@@ -6436,7 +6436,7 @@
         <v>27</v>
       </c>
       <c r="E195" s="11">
-        <v>19</v>
+        <v>17</v>
       </c>
       <c r="F195" s="9" t="s">
         <v>28</v>
@@ -6459,7 +6459,7 @@
         <v>27</v>
       </c>
       <c r="E196" s="11">
-        <v>14</v>
+        <v>26</v>
       </c>
       <c r="F196" s="9" t="s">
         <v>28</v>
@@ -6482,7 +6482,7 @@
         <v>27</v>
       </c>
       <c r="E197" s="11">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="F197" s="9" t="s">
         <v>28</v>
@@ -6505,7 +6505,7 @@
         <v>27</v>
       </c>
       <c r="E198" s="11">
-        <v>24</v>
+        <v>9</v>
       </c>
       <c r="F198" s="9" t="s">
         <v>28</v>
@@ -6528,7 +6528,7 @@
         <v>27</v>
       </c>
       <c r="E199" s="11">
-        <v>13</v>
+        <v>20</v>
       </c>
       <c r="F199" s="9" t="s">
         <v>28</v>
@@ -6551,7 +6551,7 @@
         <v>27</v>
       </c>
       <c r="E200" s="11">
-        <v>16</v>
+        <v>20</v>
       </c>
       <c r="F200" s="9" t="s">
         <v>28</v>
@@ -6574,7 +6574,7 @@
         <v>27</v>
       </c>
       <c r="E201" s="11">
-        <v>13</v>
+        <v>31</v>
       </c>
       <c r="F201" s="9" t="s">
         <v>28</v>
@@ -6597,7 +6597,7 @@
         <v>27</v>
       </c>
       <c r="E202" s="11">
-        <v>18</v>
+        <v>29</v>
       </c>
       <c r="F202" s="9" t="s">
         <v>28</v>
@@ -6620,7 +6620,7 @@
         <v>27</v>
       </c>
       <c r="E203" s="11">
-        <v>26</v>
+        <v>30</v>
       </c>
       <c r="F203" s="9" t="s">
         <v>28</v>
@@ -6643,7 +6643,7 @@
         <v>27</v>
       </c>
       <c r="E204" s="11">
-        <v>18</v>
+        <v>23</v>
       </c>
       <c r="F204" s="9" t="s">
         <v>28</v>
@@ -6666,7 +6666,7 @@
         <v>27</v>
       </c>
       <c r="E205" s="11">
-        <v>24</v>
+        <v>18</v>
       </c>
       <c r="F205" s="9" t="s">
         <v>28</v>
@@ -6689,7 +6689,7 @@
         <v>27</v>
       </c>
       <c r="E206" s="11">
-        <v>15</v>
+        <v>24</v>
       </c>
       <c r="F206" s="9" t="s">
         <v>28</v>
@@ -6712,7 +6712,7 @@
         <v>27</v>
       </c>
       <c r="E207" s="11">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="F207" s="9" t="s">
         <v>28</v>
@@ -6735,7 +6735,7 @@
         <v>27</v>
       </c>
       <c r="E208" s="11">
-        <v>27</v>
+        <v>25</v>
       </c>
       <c r="F208" s="9" t="s">
         <v>28</v>
@@ -6758,7 +6758,7 @@
         <v>27</v>
       </c>
       <c r="E209" s="11">
-        <v>8</v>
+        <v>11</v>
       </c>
       <c r="F209" s="9" t="s">
         <v>28</v>
@@ -6781,7 +6781,7 @@
         <v>27</v>
       </c>
       <c r="E210" s="11">
-        <v>22</v>
+        <v>12</v>
       </c>
       <c r="F210" s="9" t="s">
         <v>28</v>
@@ -6804,7 +6804,7 @@
         <v>27</v>
       </c>
       <c r="E211" s="11">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="F211" s="9" t="s">
         <v>28</v>
@@ -6827,7 +6827,7 @@
         <v>27</v>
       </c>
       <c r="E212" s="11">
-        <v>18</v>
+        <v>14</v>
       </c>
       <c r="F212" s="9" t="s">
         <v>28</v>
@@ -6850,7 +6850,7 @@
         <v>27</v>
       </c>
       <c r="E213" s="11">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="F213" s="9" t="s">
         <v>28</v>
@@ -6873,7 +6873,7 @@
         <v>27</v>
       </c>
       <c r="E214" s="11">
-        <v>29</v>
+        <v>16</v>
       </c>
       <c r="F214" s="9" t="s">
         <v>28</v>
@@ -6896,7 +6896,7 @@
         <v>27</v>
       </c>
       <c r="E215" s="11">
-        <v>20</v>
+        <v>28</v>
       </c>
       <c r="F215" s="9" t="s">
         <v>28</v>
@@ -6919,7 +6919,7 @@
         <v>27</v>
       </c>
       <c r="E216" s="11">
-        <v>30</v>
+        <v>22</v>
       </c>
       <c r="F216" s="9" t="s">
         <v>28</v>
@@ -6942,7 +6942,7 @@
         <v>27</v>
       </c>
       <c r="E217" s="11">
-        <v>24</v>
+        <v>13</v>
       </c>
       <c r="F217" s="9" t="s">
         <v>28</v>
@@ -6965,7 +6965,7 @@
         <v>27</v>
       </c>
       <c r="E218" s="11">
-        <v>17</v>
+        <v>23</v>
       </c>
       <c r="F218" s="9" t="s">
         <v>28</v>
@@ -6988,7 +6988,7 @@
         <v>27</v>
       </c>
       <c r="E219" s="11">
-        <v>27</v>
+        <v>15</v>
       </c>
       <c r="F219" s="9" t="s">
         <v>28</v>
@@ -7011,7 +7011,7 @@
         <v>27</v>
       </c>
       <c r="E220" s="11">
-        <v>21</v>
+        <v>26</v>
       </c>
       <c r="F220" s="9" t="s">
         <v>28</v>
@@ -7034,7 +7034,7 @@
         <v>27</v>
       </c>
       <c r="E221" s="11">
-        <v>19</v>
+        <v>24</v>
       </c>
       <c r="F221" s="9" t="s">
         <v>28</v>
@@ -7057,7 +7057,7 @@
         <v>27</v>
       </c>
       <c r="E222" s="11">
-        <v>21</v>
+        <v>9</v>
       </c>
       <c r="F222" s="9" t="s">
         <v>28</v>
@@ -7080,7 +7080,7 @@
         <v>27</v>
       </c>
       <c r="E223" s="11">
-        <v>8</v>
+        <v>13</v>
       </c>
       <c r="F223" s="9" t="s">
         <v>28</v>
@@ -7103,7 +7103,7 @@
         <v>27</v>
       </c>
       <c r="E224" s="11">
-        <v>19</v>
+        <v>21</v>
       </c>
       <c r="F224" s="9" t="s">
         <v>28</v>
@@ -7126,7 +7126,7 @@
         <v>27</v>
       </c>
       <c r="E225" s="11">
-        <v>12</v>
+        <v>8</v>
       </c>
       <c r="F225" s="9" t="s">
         <v>28</v>
@@ -7149,7 +7149,7 @@
         <v>27</v>
       </c>
       <c r="E226" s="11">
-        <v>17</v>
+        <v>15</v>
       </c>
       <c r="F226" s="9" t="s">
         <v>28</v>
@@ -7172,7 +7172,7 @@
         <v>27</v>
       </c>
       <c r="E227" s="11">
-        <v>18</v>
+        <v>22</v>
       </c>
       <c r="F227" s="9" t="s">
         <v>28</v>
@@ -7195,7 +7195,7 @@
         <v>27</v>
       </c>
       <c r="E228" s="11">
-        <v>22</v>
+        <v>27</v>
       </c>
       <c r="F228" s="9" t="s">
         <v>28</v>
@@ -7218,7 +7218,7 @@
         <v>27</v>
       </c>
       <c r="E229" s="11">
-        <v>15</v>
+        <v>28</v>
       </c>
       <c r="F229" s="9" t="s">
         <v>28</v>
@@ -7241,7 +7241,7 @@
         <v>27</v>
       </c>
       <c r="E230" s="11">
-        <v>9</v>
+        <v>21</v>
       </c>
       <c r="F230" s="9" t="s">
         <v>28</v>
@@ -7264,7 +7264,7 @@
         <v>27</v>
       </c>
       <c r="E231" s="11">
-        <v>28</v>
+        <v>17</v>
       </c>
       <c r="F231" s="9" t="s">
         <v>28</v>
@@ -7287,7 +7287,7 @@
         <v>27</v>
       </c>
       <c r="E232" s="11">
-        <v>17</v>
+        <v>21</v>
       </c>
       <c r="F232" s="9" t="s">
         <v>28</v>
@@ -7310,7 +7310,7 @@
         <v>27</v>
       </c>
       <c r="E233" s="11">
-        <v>11</v>
+        <v>31</v>
       </c>
       <c r="F233" s="9" t="s">
         <v>28</v>
@@ -7333,7 +7333,7 @@
         <v>27</v>
       </c>
       <c r="E234" s="11">
-        <v>17</v>
+        <v>21</v>
       </c>
       <c r="F234" s="9" t="s">
         <v>28</v>
@@ -7356,7 +7356,7 @@
         <v>27</v>
       </c>
       <c r="E235" s="11">
-        <v>9</v>
+        <v>12</v>
       </c>
       <c r="F235" s="9" t="s">
         <v>28</v>
@@ -7379,7 +7379,7 @@
         <v>27</v>
       </c>
       <c r="E236" s="11">
-        <v>9</v>
+        <v>20</v>
       </c>
       <c r="F236" s="9" t="s">
         <v>28</v>
@@ -7402,7 +7402,7 @@
         <v>27</v>
       </c>
       <c r="E237" s="11">
-        <v>8</v>
+        <v>26</v>
       </c>
       <c r="F237" s="9" t="s">
         <v>28</v>
@@ -7425,7 +7425,7 @@
         <v>27</v>
       </c>
       <c r="E238" s="11">
-        <v>31</v>
+        <v>22</v>
       </c>
       <c r="F238" s="9" t="s">
         <v>28</v>
@@ -7448,7 +7448,7 @@
         <v>27</v>
       </c>
       <c r="E239" s="11">
-        <v>22</v>
+        <v>15</v>
       </c>
       <c r="F239" s="9" t="s">
         <v>28</v>
@@ -7471,7 +7471,7 @@
         <v>27</v>
       </c>
       <c r="E240" s="11">
-        <v>27</v>
+        <v>31</v>
       </c>
       <c r="F240" s="9" t="s">
         <v>28</v>
@@ -7494,7 +7494,7 @@
         <v>27</v>
       </c>
       <c r="E241" s="11">
-        <v>27</v>
+        <v>8</v>
       </c>
       <c r="F241" s="9" t="s">
         <v>28</v>
@@ -7517,7 +7517,7 @@
         <v>27</v>
       </c>
       <c r="E242" s="11">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="F242" s="9" t="s">
         <v>28</v>
@@ -7540,7 +7540,7 @@
         <v>27</v>
       </c>
       <c r="E243" s="11">
-        <v>13</v>
+        <v>15</v>
       </c>
       <c r="F243" s="9" t="s">
         <v>28</v>
@@ -7563,7 +7563,7 @@
         <v>27</v>
       </c>
       <c r="E244" s="11">
-        <v>12</v>
+        <v>8</v>
       </c>
       <c r="F244" s="9" t="s">
         <v>28</v>
@@ -7586,7 +7586,7 @@
         <v>27</v>
       </c>
       <c r="E245" s="11">
-        <v>23</v>
+        <v>19</v>
       </c>
       <c r="F245" s="9" t="s">
         <v>28</v>
@@ -7609,7 +7609,7 @@
         <v>27</v>
       </c>
       <c r="E246" s="11">
-        <v>9</v>
+        <v>15</v>
       </c>
       <c r="F246" s="9" t="s">
         <v>28</v>
@@ -7632,7 +7632,7 @@
         <v>27</v>
       </c>
       <c r="E247" s="11">
-        <v>28</v>
+        <v>10</v>
       </c>
       <c r="F247" s="9" t="s">
         <v>28</v>
@@ -7655,7 +7655,7 @@
         <v>27</v>
       </c>
       <c r="E248" s="11">
-        <v>18</v>
+        <v>30</v>
       </c>
       <c r="F248" s="9" t="s">
         <v>28</v>
@@ -7678,7 +7678,7 @@
         <v>27</v>
       </c>
       <c r="E249" s="11">
-        <v>17</v>
+        <v>26</v>
       </c>
       <c r="F249" s="9" t="s">
         <v>28</v>
@@ -7701,7 +7701,7 @@
         <v>27</v>
       </c>
       <c r="E250" s="11">
-        <v>31</v>
+        <v>26</v>
       </c>
       <c r="F250" s="9" t="s">
         <v>28</v>
@@ -7724,7 +7724,7 @@
         <v>27</v>
       </c>
       <c r="E251" s="11">
-        <v>20</v>
+        <v>15</v>
       </c>
       <c r="F251" s="9" t="s">
         <v>28</v>
@@ -7747,7 +7747,7 @@
         <v>27</v>
       </c>
       <c r="E252" s="11">
-        <v>25</v>
+        <v>31</v>
       </c>
       <c r="F252" s="9" t="s">
         <v>28</v>
@@ -7770,7 +7770,7 @@
         <v>27</v>
       </c>
       <c r="E253" s="11">
-        <v>31</v>
+        <v>11</v>
       </c>
       <c r="F253" s="9" t="s">
         <v>28</v>
@@ -7793,7 +7793,7 @@
         <v>27</v>
       </c>
       <c r="E254" s="11">
-        <v>28</v>
+        <v>30</v>
       </c>
       <c r="F254" s="9" t="s">
         <v>28</v>
@@ -7816,7 +7816,7 @@
         <v>27</v>
       </c>
       <c r="E255" s="11">
-        <v>17</v>
+        <v>21</v>
       </c>
       <c r="F255" s="9" t="s">
         <v>28</v>
@@ -7839,7 +7839,7 @@
         <v>27</v>
       </c>
       <c r="E256" s="11">
-        <v>23</v>
+        <v>16</v>
       </c>
       <c r="F256" s="9" t="s">
         <v>28</v>
@@ -7862,7 +7862,7 @@
         <v>27</v>
       </c>
       <c r="E257" s="11">
-        <v>8</v>
+        <v>27</v>
       </c>
       <c r="F257" s="9" t="s">
         <v>28</v>
@@ -7885,7 +7885,7 @@
         <v>27</v>
       </c>
       <c r="E258" s="11">
-        <v>20</v>
+        <v>15</v>
       </c>
       <c r="F258" s="9" t="s">
         <v>28</v>
@@ -7908,7 +7908,7 @@
         <v>27</v>
       </c>
       <c r="E259" s="11">
-        <v>14</v>
+        <v>27</v>
       </c>
       <c r="F259" s="9" t="s">
         <v>28</v>
@@ -7931,7 +7931,7 @@
         <v>27</v>
       </c>
       <c r="E260" s="11">
-        <v>31</v>
+        <v>13</v>
       </c>
       <c r="F260" s="9" t="s">
         <v>28</v>
@@ -7954,7 +7954,7 @@
         <v>27</v>
       </c>
       <c r="E261" s="11">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="F261" s="9" t="s">
         <v>28</v>
@@ -7977,7 +7977,7 @@
         <v>27</v>
       </c>
       <c r="E262" s="11">
-        <v>16</v>
+        <v>19</v>
       </c>
       <c r="F262" s="9" t="s">
         <v>28</v>
@@ -8000,7 +8000,7 @@
         <v>27</v>
       </c>
       <c r="E263" s="11">
-        <v>12</v>
+        <v>17</v>
       </c>
       <c r="F263" s="9" t="s">
         <v>28</v>
@@ -8023,7 +8023,7 @@
         <v>27</v>
       </c>
       <c r="E264" s="11">
-        <v>10</v>
+        <v>19</v>
       </c>
       <c r="F264" s="9" t="s">
         <v>28</v>
@@ -8046,7 +8046,7 @@
         <v>27</v>
       </c>
       <c r="E265" s="11">
-        <v>22</v>
+        <v>12</v>
       </c>
       <c r="F265" s="9" t="s">
         <v>28</v>
@@ -8069,7 +8069,7 @@
         <v>27</v>
       </c>
       <c r="E266" s="11">
-        <v>23</v>
+        <v>14</v>
       </c>
       <c r="F266" s="9" t="s">
         <v>28</v>
@@ -8092,7 +8092,7 @@
         <v>27</v>
       </c>
       <c r="E267" s="11">
-        <v>10</v>
+        <v>25</v>
       </c>
       <c r="F267" s="9" t="s">
         <v>28</v>
@@ -8115,7 +8115,7 @@
         <v>27</v>
       </c>
       <c r="E268" s="11">
-        <v>11</v>
+        <v>30</v>
       </c>
       <c r="F268" s="9" t="s">
         <v>28</v>
@@ -8138,7 +8138,7 @@
         <v>27</v>
       </c>
       <c r="E269" s="11">
-        <v>23</v>
+        <v>29</v>
       </c>
       <c r="F269" s="9" t="s">
         <v>28</v>
@@ -8161,7 +8161,7 @@
         <v>27</v>
       </c>
       <c r="E270" s="11">
-        <v>14</v>
+        <v>9</v>
       </c>
       <c r="F270" s="9" t="s">
         <v>28</v>
@@ -8184,7 +8184,7 @@
         <v>27</v>
       </c>
       <c r="E271" s="11">
-        <v>30</v>
+        <v>18</v>
       </c>
       <c r="F271" s="9" t="s">
         <v>28</v>
@@ -8207,7 +8207,7 @@
         <v>27</v>
       </c>
       <c r="E272" s="11">
-        <v>11</v>
+        <v>25</v>
       </c>
       <c r="F272" s="9" t="s">
         <v>28</v>
@@ -8230,7 +8230,7 @@
         <v>27</v>
       </c>
       <c r="E273" s="11">
-        <v>21</v>
+        <v>11</v>
       </c>
       <c r="F273" s="9" t="s">
         <v>28</v>
@@ -8253,7 +8253,7 @@
         <v>27</v>
       </c>
       <c r="E274" s="11">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="F274" s="9" t="s">
         <v>28</v>
@@ -8276,7 +8276,7 @@
         <v>27</v>
       </c>
       <c r="E275" s="11">
-        <v>29</v>
+        <v>14</v>
       </c>
       <c r="F275" s="9" t="s">
         <v>28</v>
@@ -8299,7 +8299,7 @@
         <v>27</v>
       </c>
       <c r="E276" s="11">
-        <v>22</v>
+        <v>24</v>
       </c>
       <c r="F276" s="9" t="s">
         <v>28</v>
@@ -8322,7 +8322,7 @@
         <v>27</v>
       </c>
       <c r="E277" s="11">
-        <v>31</v>
+        <v>24</v>
       </c>
       <c r="F277" s="9" t="s">
         <v>28</v>
@@ -8345,7 +8345,7 @@
         <v>27</v>
       </c>
       <c r="E278" s="11">
-        <v>28</v>
+        <v>15</v>
       </c>
       <c r="F278" s="9" t="s">
         <v>28</v>
@@ -8368,7 +8368,7 @@
         <v>27</v>
       </c>
       <c r="E279" s="11">
-        <v>31</v>
+        <v>26</v>
       </c>
       <c r="F279" s="9" t="s">
         <v>28</v>
@@ -8391,7 +8391,7 @@
         <v>27</v>
       </c>
       <c r="E280" s="11">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="F280" s="9" t="s">
         <v>28</v>
@@ -8414,7 +8414,7 @@
         <v>27</v>
       </c>
       <c r="E281" s="11">
-        <v>27</v>
+        <v>22</v>
       </c>
       <c r="F281" s="9" t="s">
         <v>28</v>
@@ -8437,7 +8437,7 @@
         <v>27</v>
       </c>
       <c r="E282" s="11">
-        <v>22</v>
+        <v>26</v>
       </c>
       <c r="F282" s="9" t="s">
         <v>28</v>
@@ -8460,7 +8460,7 @@
         <v>27</v>
       </c>
       <c r="E283" s="11">
-        <v>30</v>
+        <v>25</v>
       </c>
       <c r="F283" s="9" t="s">
         <v>28</v>
@@ -8483,7 +8483,7 @@
         <v>27</v>
       </c>
       <c r="E284" s="11">
-        <v>29</v>
+        <v>17</v>
       </c>
       <c r="F284" s="9" t="s">
         <v>28</v>
@@ -8506,7 +8506,7 @@
         <v>27</v>
       </c>
       <c r="E285" s="11">
-        <v>8</v>
+        <v>19</v>
       </c>
       <c r="F285" s="9" t="s">
         <v>28</v>
@@ -8529,7 +8529,7 @@
         <v>27</v>
       </c>
       <c r="E286" s="11">
-        <v>30</v>
+        <v>23</v>
       </c>
       <c r="F286" s="9" t="s">
         <v>28</v>
@@ -8552,7 +8552,7 @@
         <v>27</v>
       </c>
       <c r="E287" s="11">
-        <v>24</v>
+        <v>21</v>
       </c>
       <c r="F287" s="9" t="s">
         <v>28</v>
@@ -8575,7 +8575,7 @@
         <v>27</v>
       </c>
       <c r="E288" s="11">
-        <v>20</v>
+        <v>18</v>
       </c>
       <c r="F288" s="9" t="s">
         <v>28</v>
@@ -8598,7 +8598,7 @@
         <v>27</v>
       </c>
       <c r="E289" s="11">
-        <v>23</v>
+        <v>15</v>
       </c>
       <c r="F289" s="9" t="s">
         <v>28</v>
@@ -8621,7 +8621,7 @@
         <v>27</v>
       </c>
       <c r="E290" s="11">
-        <v>29</v>
+        <v>31</v>
       </c>
       <c r="F290" s="9" t="s">
         <v>28</v>
@@ -8644,7 +8644,7 @@
         <v>27</v>
       </c>
       <c r="E291" s="11">
-        <v>29</v>
+        <v>31</v>
       </c>
       <c r="F291" s="9" t="s">
         <v>28</v>
@@ -8667,7 +8667,7 @@
         <v>27</v>
       </c>
       <c r="E292" s="11">
-        <v>20</v>
+        <v>25</v>
       </c>
       <c r="F292" s="9" t="s">
         <v>28</v>
@@ -8690,7 +8690,7 @@
         <v>27</v>
       </c>
       <c r="E293" s="11">
-        <v>10</v>
+        <v>19</v>
       </c>
       <c r="F293" s="9" t="s">
         <v>28</v>
@@ -8713,7 +8713,7 @@
         <v>27</v>
       </c>
       <c r="E294" s="11">
-        <v>10</v>
+        <v>28</v>
       </c>
       <c r="F294" s="9" t="s">
         <v>28</v>
@@ -8736,7 +8736,7 @@
         <v>27</v>
       </c>
       <c r="E295" s="11">
-        <v>21</v>
+        <v>26</v>
       </c>
       <c r="F295" s="9" t="s">
         <v>28</v>
@@ -8759,7 +8759,7 @@
         <v>27</v>
       </c>
       <c r="E296" s="11">
-        <v>28</v>
+        <v>12</v>
       </c>
       <c r="F296" s="9" t="s">
         <v>28</v>
@@ -8782,7 +8782,7 @@
         <v>27</v>
       </c>
       <c r="E297" s="11">
-        <v>17</v>
+        <v>31</v>
       </c>
       <c r="F297" s="9" t="s">
         <v>28</v>
@@ -8805,7 +8805,7 @@
         <v>27</v>
       </c>
       <c r="E298" s="11">
-        <v>15</v>
+        <v>26</v>
       </c>
       <c r="F298" s="9" t="s">
         <v>28</v>
@@ -8828,7 +8828,7 @@
         <v>27</v>
       </c>
       <c r="E299" s="11">
-        <v>24</v>
+        <v>16</v>
       </c>
       <c r="F299" s="9" t="s">
         <v>28</v>
@@ -8851,7 +8851,7 @@
         <v>27</v>
       </c>
       <c r="E300" s="11">
-        <v>13</v>
+        <v>9</v>
       </c>
       <c r="F300" s="9" t="s">
         <v>28</v>
@@ -8874,7 +8874,7 @@
         <v>27</v>
       </c>
       <c r="E301" s="11">
-        <v>23</v>
+        <v>15</v>
       </c>
       <c r="F301" s="9" t="s">
         <v>28</v>
@@ -8897,7 +8897,7 @@
         <v>27</v>
       </c>
       <c r="E302" s="11">
-        <v>13</v>
+        <v>24</v>
       </c>
       <c r="F302" s="9" t="s">
         <v>28</v>
@@ -8920,7 +8920,7 @@
         <v>27</v>
       </c>
       <c r="E303" s="11">
-        <v>17</v>
+        <v>31</v>
       </c>
       <c r="F303" s="9" t="s">
         <v>28</v>
@@ -8943,7 +8943,7 @@
         <v>27</v>
       </c>
       <c r="E304" s="11">
-        <v>18</v>
+        <v>28</v>
       </c>
       <c r="F304" s="9" t="s">
         <v>28</v>
@@ -8966,7 +8966,7 @@
         <v>27</v>
       </c>
       <c r="E305" s="11">
-        <v>9</v>
+        <v>30</v>
       </c>
       <c r="F305" s="9" t="s">
         <v>28</v>
@@ -8989,7 +8989,7 @@
         <v>27</v>
       </c>
       <c r="E306" s="11">
-        <v>13</v>
+        <v>21</v>
       </c>
       <c r="F306" s="9" t="s">
         <v>28</v>
@@ -9012,7 +9012,7 @@
         <v>27</v>
       </c>
       <c r="E307" s="11">
-        <v>20</v>
+        <v>26</v>
       </c>
       <c r="F307" s="9" t="s">
         <v>28</v>
@@ -9035,7 +9035,7 @@
         <v>27</v>
       </c>
       <c r="E308" s="11">
-        <v>16</v>
+        <v>9</v>
       </c>
       <c r="F308" s="9" t="s">
         <v>28</v>
@@ -9058,7 +9058,7 @@
         <v>27</v>
       </c>
       <c r="E309" s="11">
-        <v>13</v>
+        <v>28</v>
       </c>
       <c r="F309" s="9" t="s">
         <v>28</v>
@@ -9081,7 +9081,7 @@
         <v>27</v>
       </c>
       <c r="E310" s="11">
-        <v>19</v>
+        <v>22</v>
       </c>
       <c r="F310" s="9" t="s">
         <v>28</v>
@@ -9104,7 +9104,7 @@
         <v>27</v>
       </c>
       <c r="E311" s="11">
-        <v>13</v>
+        <v>23</v>
       </c>
       <c r="F311" s="9" t="s">
         <v>28</v>
@@ -9127,7 +9127,7 @@
         <v>27</v>
       </c>
       <c r="E312" s="11">
-        <v>23</v>
+        <v>18</v>
       </c>
       <c r="F312" s="9" t="s">
         <v>28</v>
@@ -9150,7 +9150,7 @@
         <v>27</v>
       </c>
       <c r="E313" s="11">
-        <v>22</v>
+        <v>24</v>
       </c>
       <c r="F313" s="9" t="s">
         <v>28</v>
@@ -9173,7 +9173,7 @@
         <v>27</v>
       </c>
       <c r="E314" s="11">
-        <v>28</v>
+        <v>17</v>
       </c>
       <c r="F314" s="9" t="s">
         <v>28</v>
@@ -9196,7 +9196,7 @@
         <v>27</v>
       </c>
       <c r="E315" s="11">
-        <v>27</v>
+        <v>29</v>
       </c>
       <c r="F315" s="9" t="s">
         <v>28</v>
@@ -9219,7 +9219,7 @@
         <v>27</v>
       </c>
       <c r="E316" s="11">
-        <v>13</v>
+        <v>27</v>
       </c>
       <c r="F316" s="9" t="s">
         <v>28</v>
@@ -9242,7 +9242,7 @@
         <v>27</v>
       </c>
       <c r="E317" s="11">
-        <v>30</v>
+        <v>17</v>
       </c>
       <c r="F317" s="9" t="s">
         <v>28</v>
@@ -9265,7 +9265,7 @@
         <v>27</v>
       </c>
       <c r="E318" s="11">
-        <v>25</v>
+        <v>17</v>
       </c>
       <c r="F318" s="9" t="s">
         <v>28</v>
@@ -9288,7 +9288,7 @@
         <v>27</v>
       </c>
       <c r="E319" s="11">
-        <v>21</v>
+        <v>14</v>
       </c>
       <c r="F319" s="9" t="s">
         <v>28</v>
@@ -9311,7 +9311,7 @@
         <v>27</v>
       </c>
       <c r="E320" s="11">
-        <v>13</v>
+        <v>9</v>
       </c>
       <c r="F320" s="9" t="s">
         <v>28</v>
@@ -9334,7 +9334,7 @@
         <v>27</v>
       </c>
       <c r="E321" s="11">
-        <v>24</v>
+        <v>14</v>
       </c>
       <c r="F321" s="9" t="s">
         <v>28</v>
@@ -9357,7 +9357,7 @@
         <v>27</v>
       </c>
       <c r="E322" s="11">
-        <v>10</v>
+        <v>19</v>
       </c>
       <c r="F322" s="9" t="s">
         <v>28</v>
@@ -9380,7 +9380,7 @@
         <v>27</v>
       </c>
       <c r="E323" s="11">
-        <v>24</v>
+        <v>19</v>
       </c>
       <c r="F323" s="9" t="s">
         <v>28</v>
@@ -9403,7 +9403,7 @@
         <v>27</v>
       </c>
       <c r="E324" s="11">
-        <v>27</v>
+        <v>12</v>
       </c>
       <c r="F324" s="9" t="s">
         <v>28</v>
@@ -9426,7 +9426,7 @@
         <v>27</v>
       </c>
       <c r="E325" s="11">
-        <v>27</v>
+        <v>31</v>
       </c>
       <c r="F325" s="9" t="s">
         <v>28</v>
@@ -9449,7 +9449,7 @@
         <v>27</v>
       </c>
       <c r="E326" s="11">
-        <v>20</v>
+        <v>30</v>
       </c>
       <c r="F326" s="9" t="s">
         <v>28</v>
@@ -9472,7 +9472,7 @@
         <v>27</v>
       </c>
       <c r="E327" s="11">
-        <v>20</v>
+        <v>18</v>
       </c>
       <c r="F327" s="9" t="s">
         <v>28</v>
@@ -9518,7 +9518,7 @@
         <v>27</v>
       </c>
       <c r="E329" s="11">
-        <v>8</v>
+        <v>19</v>
       </c>
       <c r="F329" s="9" t="s">
         <v>28</v>
@@ -9541,7 +9541,7 @@
         <v>27</v>
       </c>
       <c r="E330" s="11">
-        <v>17</v>
+        <v>15</v>
       </c>
       <c r="F330" s="9" t="s">
         <v>28</v>
@@ -9564,7 +9564,7 @@
         <v>27</v>
       </c>
       <c r="E331" s="11">
-        <v>11</v>
+        <v>13</v>
       </c>
       <c r="F331" s="9" t="s">
         <v>28</v>
@@ -9587,7 +9587,7 @@
         <v>27</v>
       </c>
       <c r="E332" s="11">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="F332" s="9" t="s">
         <v>28</v>
@@ -9610,7 +9610,7 @@
         <v>27</v>
       </c>
       <c r="E333" s="11">
-        <v>21</v>
+        <v>10</v>
       </c>
       <c r="F333" s="9" t="s">
         <v>28</v>
@@ -9633,7 +9633,7 @@
         <v>27</v>
       </c>
       <c r="E334" s="11">
-        <v>29</v>
+        <v>25</v>
       </c>
       <c r="F334" s="9" t="s">
         <v>28</v>
@@ -9656,7 +9656,7 @@
         <v>27</v>
       </c>
       <c r="E335" s="11">
-        <v>23</v>
+        <v>31</v>
       </c>
       <c r="F335" s="9" t="s">
         <v>28</v>
@@ -9679,7 +9679,7 @@
         <v>27</v>
       </c>
       <c r="E336" s="11">
-        <v>12</v>
+        <v>10</v>
       </c>
       <c r="F336" s="9" t="s">
         <v>28</v>
@@ -9702,7 +9702,7 @@
         <v>27</v>
       </c>
       <c r="E337" s="11">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="F337" s="9" t="s">
         <v>28</v>
@@ -9725,7 +9725,7 @@
         <v>27</v>
       </c>
       <c r="E338" s="11">
-        <v>31</v>
+        <v>26</v>
       </c>
       <c r="F338" s="9" t="s">
         <v>28</v>
@@ -9748,7 +9748,7 @@
         <v>27</v>
       </c>
       <c r="E339" s="11">
-        <v>29</v>
+        <v>24</v>
       </c>
       <c r="F339" s="9" t="s">
         <v>28</v>
@@ -9771,7 +9771,7 @@
         <v>27</v>
       </c>
       <c r="E340" s="11">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="F340" s="9" t="s">
         <v>28</v>
@@ -9794,7 +9794,7 @@
         <v>27</v>
       </c>
       <c r="E341" s="11">
-        <v>18</v>
+        <v>16</v>
       </c>
       <c r="F341" s="9" t="s">
         <v>28</v>
@@ -9817,7 +9817,7 @@
         <v>27</v>
       </c>
       <c r="E342" s="11">
-        <v>21</v>
+        <v>14</v>
       </c>
       <c r="F342" s="9" t="s">
         <v>28</v>
@@ -9840,7 +9840,7 @@
         <v>27</v>
       </c>
       <c r="E343" s="11">
-        <v>30</v>
+        <v>13</v>
       </c>
       <c r="F343" s="9" t="s">
         <v>28</v>
@@ -9863,7 +9863,7 @@
         <v>27</v>
       </c>
       <c r="E344" s="11">
-        <v>13</v>
+        <v>24</v>
       </c>
       <c r="F344" s="9" t="s">
         <v>28</v>
@@ -9886,7 +9886,7 @@
         <v>27</v>
       </c>
       <c r="E345" s="11">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="F345" s="9" t="s">
         <v>28</v>
@@ -9909,7 +9909,7 @@
         <v>27</v>
       </c>
       <c r="E346" s="11">
-        <v>17</v>
+        <v>30</v>
       </c>
       <c r="F346" s="9" t="s">
         <v>28</v>
@@ -9932,7 +9932,7 @@
         <v>27</v>
       </c>
       <c r="E347" s="11">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="F347" s="9" t="s">
         <v>28</v>
@@ -9955,7 +9955,7 @@
         <v>27</v>
       </c>
       <c r="E348" s="11">
-        <v>26</v>
+        <v>18</v>
       </c>
       <c r="F348" s="9" t="s">
         <v>28</v>
@@ -9978,7 +9978,7 @@
         <v>27</v>
       </c>
       <c r="E349" s="11">
-        <v>13</v>
+        <v>22</v>
       </c>
       <c r="F349" s="9" t="s">
         <v>28</v>
@@ -10001,7 +10001,7 @@
         <v>27</v>
       </c>
       <c r="E350" s="11">
-        <v>21</v>
+        <v>17</v>
       </c>
       <c r="F350" s="9" t="s">
         <v>28</v>
@@ -10024,7 +10024,7 @@
         <v>27</v>
       </c>
       <c r="E351" s="11">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="F351" s="9" t="s">
         <v>28</v>
@@ -10047,7 +10047,7 @@
         <v>27</v>
       </c>
       <c r="E352" s="11">
-        <v>18</v>
+        <v>10</v>
       </c>
       <c r="F352" s="9" t="s">
         <v>28</v>
@@ -10070,7 +10070,7 @@
         <v>27</v>
       </c>
       <c r="E353" s="11">
-        <v>29</v>
+        <v>18</v>
       </c>
       <c r="F353" s="9" t="s">
         <v>28</v>
@@ -10093,7 +10093,7 @@
         <v>27</v>
       </c>
       <c r="E354" s="11">
-        <v>27</v>
+        <v>31</v>
       </c>
       <c r="F354" s="9" t="s">
         <v>28</v>
@@ -10116,7 +10116,7 @@
         <v>27</v>
       </c>
       <c r="E355" s="11">
-        <v>19</v>
+        <v>22</v>
       </c>
       <c r="F355" s="9" t="s">
         <v>28</v>
@@ -10139,7 +10139,7 @@
         <v>27</v>
       </c>
       <c r="E356" s="11">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="F356" s="9" t="s">
         <v>28</v>
@@ -10162,7 +10162,7 @@
         <v>27</v>
       </c>
       <c r="E357" s="11">
-        <v>30</v>
+        <v>27</v>
       </c>
       <c r="F357" s="9" t="s">
         <v>28</v>
@@ -10185,7 +10185,7 @@
         <v>27</v>
       </c>
       <c r="E358" s="11">
-        <v>24</v>
+        <v>9</v>
       </c>
       <c r="F358" s="9" t="s">
         <v>28</v>
@@ -10208,7 +10208,7 @@
         <v>27</v>
       </c>
       <c r="E359" s="11">
-        <v>30</v>
+        <v>18</v>
       </c>
       <c r="F359" s="9" t="s">
         <v>28</v>
@@ -10231,7 +10231,7 @@
         <v>27</v>
       </c>
       <c r="E360" s="11">
-        <v>11</v>
+        <v>13</v>
       </c>
       <c r="F360" s="9" t="s">
         <v>28</v>
@@ -10254,7 +10254,7 @@
         <v>27</v>
       </c>
       <c r="E361" s="11">
-        <v>25</v>
+        <v>14</v>
       </c>
       <c r="F361" s="9" t="s">
         <v>28</v>
@@ -10277,7 +10277,7 @@
         <v>27</v>
       </c>
       <c r="E362" s="11">
-        <v>25</v>
+        <v>15</v>
       </c>
       <c r="F362" s="9" t="s">
         <v>28</v>
@@ -10300,7 +10300,7 @@
         <v>27</v>
       </c>
       <c r="E363" s="11">
-        <v>21</v>
+        <v>15</v>
       </c>
       <c r="F363" s="9" t="s">
         <v>28</v>
@@ -10323,7 +10323,7 @@
         <v>27</v>
       </c>
       <c r="E364" s="11">
-        <v>30</v>
+        <v>26</v>
       </c>
       <c r="F364" s="9" t="s">
         <v>28</v>
@@ -10346,7 +10346,7 @@
         <v>27</v>
       </c>
       <c r="E365" s="11">
-        <v>11</v>
+        <v>26</v>
       </c>
       <c r="F365" s="9" t="s">
         <v>28</v>
@@ -10369,7 +10369,7 @@
         <v>27</v>
       </c>
       <c r="E366" s="11">
-        <v>29</v>
+        <v>9</v>
       </c>
       <c r="F366" s="9" t="s">
         <v>28</v>
@@ -10392,7 +10392,7 @@
         <v>27</v>
       </c>
       <c r="E367" s="11">
-        <v>31</v>
+        <v>18</v>
       </c>
       <c r="F367" s="9" t="s">
         <v>28</v>
@@ -10415,7 +10415,7 @@
         <v>27</v>
       </c>
       <c r="E368" s="11">
-        <v>27</v>
+        <v>12</v>
       </c>
       <c r="F368" s="9" t="s">
         <v>28</v>
@@ -10438,7 +10438,7 @@
         <v>27</v>
       </c>
       <c r="E369" s="11">
-        <v>14</v>
+        <v>26</v>
       </c>
       <c r="F369" s="9" t="s">
         <v>28</v>
@@ -10461,7 +10461,7 @@
         <v>27</v>
       </c>
       <c r="E370" s="11">
-        <v>15</v>
+        <v>10</v>
       </c>
       <c r="F370" s="9" t="s">
         <v>28</v>
@@ -10484,7 +10484,7 @@
         <v>27</v>
       </c>
       <c r="E371" s="11">
-        <v>8</v>
+        <v>30</v>
       </c>
       <c r="F371" s="9" t="s">
         <v>28</v>
@@ -10507,7 +10507,7 @@
         <v>27</v>
       </c>
       <c r="E372" s="11">
-        <v>17</v>
+        <v>25</v>
       </c>
       <c r="F372" s="9" t="s">
         <v>28</v>
@@ -10530,7 +10530,7 @@
         <v>27</v>
       </c>
       <c r="E373" s="11">
-        <v>20</v>
+        <v>23</v>
       </c>
       <c r="F373" s="9" t="s">
         <v>28</v>
@@ -10553,7 +10553,7 @@
         <v>27</v>
       </c>
       <c r="E374" s="11">
-        <v>13</v>
+        <v>21</v>
       </c>
       <c r="F374" s="9" t="s">
         <v>28</v>
@@ -10599,7 +10599,7 @@
         <v>27</v>
       </c>
       <c r="E376" s="11">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="F376" s="9" t="s">
         <v>28</v>
@@ -10622,7 +10622,7 @@
         <v>27</v>
       </c>
       <c r="E377" s="11">
-        <v>13</v>
+        <v>25</v>
       </c>
       <c r="F377" s="9" t="s">
         <v>28</v>
@@ -10645,7 +10645,7 @@
         <v>27</v>
       </c>
       <c r="E378" s="11">
-        <v>29</v>
+        <v>22</v>
       </c>
       <c r="F378" s="9" t="s">
         <v>28</v>
@@ -10668,7 +10668,7 @@
         <v>27</v>
       </c>
       <c r="E379" s="11">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="F379" s="9" t="s">
         <v>28</v>
@@ -10691,7 +10691,7 @@
         <v>27</v>
       </c>
       <c r="E380" s="11">
-        <v>9</v>
+        <v>23</v>
       </c>
       <c r="F380" s="9" t="s">
         <v>28</v>
@@ -10714,7 +10714,7 @@
         <v>27</v>
       </c>
       <c r="E381" s="11">
-        <v>20</v>
+        <v>18</v>
       </c>
       <c r="F381" s="9" t="s">
         <v>28</v>
@@ -10737,7 +10737,7 @@
         <v>27</v>
       </c>
       <c r="E382" s="11">
-        <v>21</v>
+        <v>26</v>
       </c>
       <c r="F382" s="9" t="s">
         <v>28</v>
@@ -10760,7 +10760,7 @@
         <v>27</v>
       </c>
       <c r="E383" s="11">
-        <v>24</v>
+        <v>17</v>
       </c>
       <c r="F383" s="9" t="s">
         <v>28</v>
@@ -10783,7 +10783,7 @@
         <v>27</v>
       </c>
       <c r="E384" s="11">
-        <v>22</v>
+        <v>16</v>
       </c>
       <c r="F384" s="9" t="s">
         <v>28</v>
@@ -10806,7 +10806,7 @@
         <v>27</v>
       </c>
       <c r="E385" s="11">
-        <v>25</v>
+        <v>29</v>
       </c>
       <c r="F385" s="9" t="s">
         <v>28</v>
@@ -10829,7 +10829,7 @@
         <v>27</v>
       </c>
       <c r="E386" s="11">
-        <v>8</v>
+        <v>17</v>
       </c>
       <c r="F386" s="9" t="s">
         <v>28</v>
@@ -10852,7 +10852,7 @@
         <v>27</v>
       </c>
       <c r="E387" s="11">
-        <v>17</v>
+        <v>20</v>
       </c>
       <c r="F387" s="9" t="s">
         <v>28</v>
@@ -10875,7 +10875,7 @@
         <v>27</v>
       </c>
       <c r="E388" s="11">
-        <v>27</v>
+        <v>12</v>
       </c>
       <c r="F388" s="9" t="s">
         <v>28</v>
@@ -10898,7 +10898,7 @@
         <v>27</v>
       </c>
       <c r="E389" s="11">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="F389" s="9" t="s">
         <v>28</v>
@@ -10921,7 +10921,7 @@
         <v>27</v>
       </c>
       <c r="E390" s="11">
-        <v>14</v>
+        <v>16</v>
       </c>
       <c r="F390" s="9" t="s">
         <v>28</v>
@@ -10944,7 +10944,7 @@
         <v>27</v>
       </c>
       <c r="E391" s="11">
-        <v>29</v>
+        <v>18</v>
       </c>
       <c r="F391" s="9" t="s">
         <v>28</v>
@@ -10967,7 +10967,7 @@
         <v>27</v>
       </c>
       <c r="E392" s="11">
-        <v>21</v>
+        <v>14</v>
       </c>
       <c r="F392" s="9" t="s">
         <v>28</v>
@@ -10990,7 +10990,7 @@
         <v>27</v>
       </c>
       <c r="E393" s="11">
-        <v>15</v>
+        <v>18</v>
       </c>
       <c r="F393" s="9" t="s">
         <v>28</v>
@@ -11013,7 +11013,7 @@
         <v>27</v>
       </c>
       <c r="E394" s="11">
-        <v>24</v>
+        <v>15</v>
       </c>
       <c r="F394" s="9" t="s">
         <v>28</v>
@@ -11036,7 +11036,7 @@
         <v>27</v>
       </c>
       <c r="E395" s="11">
-        <v>31</v>
+        <v>12</v>
       </c>
       <c r="F395" s="9" t="s">
         <v>28</v>
@@ -11059,7 +11059,7 @@
         <v>27</v>
       </c>
       <c r="E396" s="11">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="F396" s="9" t="s">
         <v>28</v>
@@ -11082,7 +11082,7 @@
         <v>27</v>
       </c>
       <c r="E397" s="11">
-        <v>28</v>
+        <v>26</v>
       </c>
       <c r="F397" s="9" t="s">
         <v>28</v>
@@ -11105,7 +11105,7 @@
         <v>27</v>
       </c>
       <c r="E398" s="11">
-        <v>24</v>
+        <v>30</v>
       </c>
       <c r="F398" s="9" t="s">
         <v>28</v>
@@ -11128,7 +11128,7 @@
         <v>27</v>
       </c>
       <c r="E399" s="11">
-        <v>17</v>
+        <v>21</v>
       </c>
       <c r="F399" s="9" t="s">
         <v>28</v>
@@ -11151,7 +11151,7 @@
         <v>27</v>
       </c>
       <c r="E400" s="11">
-        <v>22</v>
+        <v>31</v>
       </c>
       <c r="F400" s="9" t="s">
         <v>28</v>
@@ -11174,7 +11174,7 @@
         <v>27</v>
       </c>
       <c r="E401" s="11">
-        <v>12</v>
+        <v>19</v>
       </c>
       <c r="F401" s="9" t="s">
         <v>28</v>

</xml_diff>

<commit_message>
fix(rating): set profile rating stat card default to 0 instead of 5.0 until real user ratings are received
</commit_message>
<xml_diff>
--- a/all-test-reports/selenium/selenium_e2e_test_report.xlsx
+++ b/all-test-reports/selenium/selenium_e2e_test_report.xlsx
@@ -35,7 +35,7 @@
     <t>Execution Date</t>
   </si>
   <si>
-    <t>28/7/2026, 11:40:41 am</t>
+    <t>28/7/2026, 11:43:44 am</t>
   </si>
   <si>
     <t>Browser / Mode</t>
@@ -98,7 +98,7 @@
     <t>PASS</t>
   </si>
   <si>
-    <t>11:40:41 am</t>
+    <t>11:43:44 am</t>
   </si>
   <si>
     <t>N/A</t>
@@ -1997,7 +1997,7 @@
         <v>27</v>
       </c>
       <c r="E2" s="11">
-        <v>31</v>
+        <v>19</v>
       </c>
       <c r="F2" s="9" t="s">
         <v>28</v>
@@ -2020,7 +2020,7 @@
         <v>27</v>
       </c>
       <c r="E3" s="11">
-        <v>8</v>
+        <v>22</v>
       </c>
       <c r="F3" s="9" t="s">
         <v>28</v>
@@ -2043,7 +2043,7 @@
         <v>27</v>
       </c>
       <c r="E4" s="11">
-        <v>19</v>
+        <v>26</v>
       </c>
       <c r="F4" s="9" t="s">
         <v>28</v>
@@ -2066,7 +2066,7 @@
         <v>27</v>
       </c>
       <c r="E5" s="11">
-        <v>23</v>
+        <v>18</v>
       </c>
       <c r="F5" s="9" t="s">
         <v>28</v>
@@ -2089,7 +2089,7 @@
         <v>27</v>
       </c>
       <c r="E6" s="11">
-        <v>27</v>
+        <v>22</v>
       </c>
       <c r="F6" s="9" t="s">
         <v>28</v>
@@ -2112,7 +2112,7 @@
         <v>27</v>
       </c>
       <c r="E7" s="11">
-        <v>29</v>
+        <v>14</v>
       </c>
       <c r="F7" s="9" t="s">
         <v>28</v>
@@ -2158,7 +2158,7 @@
         <v>27</v>
       </c>
       <c r="E9" s="11">
-        <v>10</v>
+        <v>13</v>
       </c>
       <c r="F9" s="9" t="s">
         <v>28</v>
@@ -2181,7 +2181,7 @@
         <v>27</v>
       </c>
       <c r="E10" s="11">
-        <v>23</v>
+        <v>12</v>
       </c>
       <c r="F10" s="9" t="s">
         <v>28</v>
@@ -2204,7 +2204,7 @@
         <v>27</v>
       </c>
       <c r="E11" s="11">
-        <v>21</v>
+        <v>11</v>
       </c>
       <c r="F11" s="9" t="s">
         <v>28</v>
@@ -2227,7 +2227,7 @@
         <v>27</v>
       </c>
       <c r="E12" s="11">
-        <v>17</v>
+        <v>29</v>
       </c>
       <c r="F12" s="9" t="s">
         <v>28</v>
@@ -2250,7 +2250,7 @@
         <v>27</v>
       </c>
       <c r="E13" s="11">
-        <v>26</v>
+        <v>20</v>
       </c>
       <c r="F13" s="9" t="s">
         <v>28</v>
@@ -2296,7 +2296,7 @@
         <v>27</v>
       </c>
       <c r="E15" s="11">
-        <v>25</v>
+        <v>19</v>
       </c>
       <c r="F15" s="9" t="s">
         <v>28</v>
@@ -2319,7 +2319,7 @@
         <v>27</v>
       </c>
       <c r="E16" s="11">
-        <v>10</v>
+        <v>15</v>
       </c>
       <c r="F16" s="9" t="s">
         <v>28</v>
@@ -2365,7 +2365,7 @@
         <v>27</v>
       </c>
       <c r="E18" s="11">
-        <v>29</v>
+        <v>15</v>
       </c>
       <c r="F18" s="9" t="s">
         <v>28</v>
@@ -2388,7 +2388,7 @@
         <v>27</v>
       </c>
       <c r="E19" s="11">
-        <v>17</v>
+        <v>9</v>
       </c>
       <c r="F19" s="9" t="s">
         <v>28</v>
@@ -2411,7 +2411,7 @@
         <v>27</v>
       </c>
       <c r="E20" s="11">
-        <v>9</v>
+        <v>23</v>
       </c>
       <c r="F20" s="9" t="s">
         <v>28</v>
@@ -2434,7 +2434,7 @@
         <v>27</v>
       </c>
       <c r="E21" s="11">
-        <v>16</v>
+        <v>13</v>
       </c>
       <c r="F21" s="9" t="s">
         <v>28</v>
@@ -2457,7 +2457,7 @@
         <v>27</v>
       </c>
       <c r="E22" s="11">
-        <v>29</v>
+        <v>8</v>
       </c>
       <c r="F22" s="9" t="s">
         <v>28</v>
@@ -2480,7 +2480,7 @@
         <v>27</v>
       </c>
       <c r="E23" s="11">
-        <v>17</v>
+        <v>8</v>
       </c>
       <c r="F23" s="9" t="s">
         <v>28</v>
@@ -2503,7 +2503,7 @@
         <v>27</v>
       </c>
       <c r="E24" s="11">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="F24" s="9" t="s">
         <v>28</v>
@@ -2526,7 +2526,7 @@
         <v>27</v>
       </c>
       <c r="E25" s="11">
-        <v>17</v>
+        <v>8</v>
       </c>
       <c r="F25" s="9" t="s">
         <v>28</v>
@@ -2549,7 +2549,7 @@
         <v>27</v>
       </c>
       <c r="E26" s="11">
-        <v>24</v>
+        <v>13</v>
       </c>
       <c r="F26" s="9" t="s">
         <v>28</v>
@@ -2572,7 +2572,7 @@
         <v>27</v>
       </c>
       <c r="E27" s="11">
-        <v>11</v>
+        <v>24</v>
       </c>
       <c r="F27" s="9" t="s">
         <v>28</v>
@@ -2595,7 +2595,7 @@
         <v>27</v>
       </c>
       <c r="E28" s="11">
-        <v>29</v>
+        <v>23</v>
       </c>
       <c r="F28" s="9" t="s">
         <v>28</v>
@@ -2618,7 +2618,7 @@
         <v>27</v>
       </c>
       <c r="E29" s="11">
-        <v>11</v>
+        <v>26</v>
       </c>
       <c r="F29" s="9" t="s">
         <v>28</v>
@@ -2641,7 +2641,7 @@
         <v>27</v>
       </c>
       <c r="E30" s="11">
-        <v>14</v>
+        <v>16</v>
       </c>
       <c r="F30" s="9" t="s">
         <v>28</v>
@@ -2664,7 +2664,7 @@
         <v>27</v>
       </c>
       <c r="E31" s="11">
-        <v>9</v>
+        <v>12</v>
       </c>
       <c r="F31" s="9" t="s">
         <v>28</v>
@@ -2687,7 +2687,7 @@
         <v>27</v>
       </c>
       <c r="E32" s="11">
-        <v>26</v>
+        <v>19</v>
       </c>
       <c r="F32" s="9" t="s">
         <v>28</v>
@@ -2710,7 +2710,7 @@
         <v>27</v>
       </c>
       <c r="E33" s="11">
-        <v>8</v>
+        <v>25</v>
       </c>
       <c r="F33" s="9" t="s">
         <v>28</v>
@@ -2733,7 +2733,7 @@
         <v>27</v>
       </c>
       <c r="E34" s="11">
-        <v>21</v>
+        <v>8</v>
       </c>
       <c r="F34" s="9" t="s">
         <v>28</v>
@@ -2756,7 +2756,7 @@
         <v>27</v>
       </c>
       <c r="E35" s="11">
-        <v>9</v>
+        <v>26</v>
       </c>
       <c r="F35" s="9" t="s">
         <v>28</v>
@@ -2779,7 +2779,7 @@
         <v>27</v>
       </c>
       <c r="E36" s="11">
-        <v>26</v>
+        <v>11</v>
       </c>
       <c r="F36" s="9" t="s">
         <v>28</v>
@@ -2825,7 +2825,7 @@
         <v>27</v>
       </c>
       <c r="E38" s="11">
-        <v>24</v>
+        <v>15</v>
       </c>
       <c r="F38" s="9" t="s">
         <v>28</v>
@@ -2848,7 +2848,7 @@
         <v>27</v>
       </c>
       <c r="E39" s="11">
-        <v>29</v>
+        <v>21</v>
       </c>
       <c r="F39" s="9" t="s">
         <v>28</v>
@@ -2871,7 +2871,7 @@
         <v>27</v>
       </c>
       <c r="E40" s="11">
-        <v>17</v>
+        <v>30</v>
       </c>
       <c r="F40" s="9" t="s">
         <v>28</v>
@@ -2894,7 +2894,7 @@
         <v>27</v>
       </c>
       <c r="E41" s="11">
-        <v>26</v>
+        <v>30</v>
       </c>
       <c r="F41" s="9" t="s">
         <v>28</v>
@@ -2917,7 +2917,7 @@
         <v>27</v>
       </c>
       <c r="E42" s="11">
-        <v>9</v>
+        <v>25</v>
       </c>
       <c r="F42" s="9" t="s">
         <v>28</v>
@@ -2940,7 +2940,7 @@
         <v>27</v>
       </c>
       <c r="E43" s="11">
-        <v>26</v>
+        <v>21</v>
       </c>
       <c r="F43" s="9" t="s">
         <v>28</v>
@@ -2963,7 +2963,7 @@
         <v>27</v>
       </c>
       <c r="E44" s="11">
-        <v>13</v>
+        <v>22</v>
       </c>
       <c r="F44" s="9" t="s">
         <v>28</v>
@@ -2986,7 +2986,7 @@
         <v>27</v>
       </c>
       <c r="E45" s="11">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="F45" s="9" t="s">
         <v>28</v>
@@ -3009,7 +3009,7 @@
         <v>27</v>
       </c>
       <c r="E46" s="11">
-        <v>26</v>
+        <v>31</v>
       </c>
       <c r="F46" s="9" t="s">
         <v>28</v>
@@ -3032,7 +3032,7 @@
         <v>27</v>
       </c>
       <c r="E47" s="11">
-        <v>30</v>
+        <v>10</v>
       </c>
       <c r="F47" s="9" t="s">
         <v>28</v>
@@ -3055,7 +3055,7 @@
         <v>27</v>
       </c>
       <c r="E48" s="11">
-        <v>12</v>
+        <v>31</v>
       </c>
       <c r="F48" s="9" t="s">
         <v>28</v>
@@ -3078,7 +3078,7 @@
         <v>27</v>
       </c>
       <c r="E49" s="11">
-        <v>22</v>
+        <v>20</v>
       </c>
       <c r="F49" s="9" t="s">
         <v>28</v>
@@ -3101,7 +3101,7 @@
         <v>27</v>
       </c>
       <c r="E50" s="11">
-        <v>12</v>
+        <v>15</v>
       </c>
       <c r="F50" s="9" t="s">
         <v>28</v>
@@ -3124,7 +3124,7 @@
         <v>27</v>
       </c>
       <c r="E51" s="11">
-        <v>26</v>
+        <v>14</v>
       </c>
       <c r="F51" s="9" t="s">
         <v>28</v>
@@ -3147,7 +3147,7 @@
         <v>27</v>
       </c>
       <c r="E52" s="11">
-        <v>15</v>
+        <v>19</v>
       </c>
       <c r="F52" s="9" t="s">
         <v>28</v>
@@ -3170,7 +3170,7 @@
         <v>27</v>
       </c>
       <c r="E53" s="11">
-        <v>22</v>
+        <v>13</v>
       </c>
       <c r="F53" s="9" t="s">
         <v>28</v>
@@ -3193,7 +3193,7 @@
         <v>27</v>
       </c>
       <c r="E54" s="11">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="F54" s="9" t="s">
         <v>28</v>
@@ -3216,7 +3216,7 @@
         <v>27</v>
       </c>
       <c r="E55" s="11">
-        <v>16</v>
+        <v>27</v>
       </c>
       <c r="F55" s="9" t="s">
         <v>28</v>
@@ -3239,7 +3239,7 @@
         <v>27</v>
       </c>
       <c r="E56" s="11">
-        <v>14</v>
+        <v>20</v>
       </c>
       <c r="F56" s="9" t="s">
         <v>28</v>
@@ -3262,7 +3262,7 @@
         <v>27</v>
       </c>
       <c r="E57" s="11">
-        <v>14</v>
+        <v>23</v>
       </c>
       <c r="F57" s="9" t="s">
         <v>28</v>
@@ -3285,7 +3285,7 @@
         <v>27</v>
       </c>
       <c r="E58" s="11">
-        <v>20</v>
+        <v>16</v>
       </c>
       <c r="F58" s="9" t="s">
         <v>28</v>
@@ -3308,7 +3308,7 @@
         <v>27</v>
       </c>
       <c r="E59" s="11">
-        <v>10</v>
+        <v>15</v>
       </c>
       <c r="F59" s="9" t="s">
         <v>28</v>
@@ -3331,7 +3331,7 @@
         <v>27</v>
       </c>
       <c r="E60" s="11">
-        <v>12</v>
+        <v>8</v>
       </c>
       <c r="F60" s="9" t="s">
         <v>28</v>
@@ -3354,7 +3354,7 @@
         <v>27</v>
       </c>
       <c r="E61" s="11">
-        <v>20</v>
+        <v>16</v>
       </c>
       <c r="F61" s="9" t="s">
         <v>28</v>
@@ -3377,7 +3377,7 @@
         <v>27</v>
       </c>
       <c r="E62" s="11">
-        <v>25</v>
+        <v>14</v>
       </c>
       <c r="F62" s="9" t="s">
         <v>28</v>
@@ -3400,7 +3400,7 @@
         <v>27</v>
       </c>
       <c r="E63" s="11">
-        <v>30</v>
+        <v>16</v>
       </c>
       <c r="F63" s="9" t="s">
         <v>28</v>
@@ -3423,7 +3423,7 @@
         <v>27</v>
       </c>
       <c r="E64" s="11">
-        <v>13</v>
+        <v>19</v>
       </c>
       <c r="F64" s="9" t="s">
         <v>28</v>
@@ -3446,7 +3446,7 @@
         <v>27</v>
       </c>
       <c r="E65" s="11">
-        <v>23</v>
+        <v>29</v>
       </c>
       <c r="F65" s="9" t="s">
         <v>28</v>
@@ -3469,7 +3469,7 @@
         <v>27</v>
       </c>
       <c r="E66" s="11">
-        <v>15</v>
+        <v>19</v>
       </c>
       <c r="F66" s="9" t="s">
         <v>28</v>
@@ -3492,7 +3492,7 @@
         <v>27</v>
       </c>
       <c r="E67" s="11">
-        <v>11</v>
+        <v>24</v>
       </c>
       <c r="F67" s="9" t="s">
         <v>28</v>
@@ -3515,7 +3515,7 @@
         <v>27</v>
       </c>
       <c r="E68" s="11">
-        <v>9</v>
+        <v>27</v>
       </c>
       <c r="F68" s="9" t="s">
         <v>28</v>
@@ -3538,7 +3538,7 @@
         <v>27</v>
       </c>
       <c r="E69" s="11">
-        <v>22</v>
+        <v>28</v>
       </c>
       <c r="F69" s="9" t="s">
         <v>28</v>
@@ -3561,7 +3561,7 @@
         <v>27</v>
       </c>
       <c r="E70" s="11">
-        <v>17</v>
+        <v>10</v>
       </c>
       <c r="F70" s="9" t="s">
         <v>28</v>
@@ -3584,7 +3584,7 @@
         <v>27</v>
       </c>
       <c r="E71" s="11">
-        <v>10</v>
+        <v>31</v>
       </c>
       <c r="F71" s="9" t="s">
         <v>28</v>
@@ -3607,7 +3607,7 @@
         <v>27</v>
       </c>
       <c r="E72" s="11">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="F72" s="9" t="s">
         <v>28</v>
@@ -3630,7 +3630,7 @@
         <v>27</v>
       </c>
       <c r="E73" s="11">
-        <v>30</v>
+        <v>16</v>
       </c>
       <c r="F73" s="9" t="s">
         <v>28</v>
@@ -3653,7 +3653,7 @@
         <v>27</v>
       </c>
       <c r="E74" s="11">
-        <v>12</v>
+        <v>24</v>
       </c>
       <c r="F74" s="9" t="s">
         <v>28</v>
@@ -3699,7 +3699,7 @@
         <v>27</v>
       </c>
       <c r="E76" s="11">
-        <v>24</v>
+        <v>30</v>
       </c>
       <c r="F76" s="9" t="s">
         <v>28</v>
@@ -3722,7 +3722,7 @@
         <v>27</v>
       </c>
       <c r="E77" s="11">
-        <v>9</v>
+        <v>11</v>
       </c>
       <c r="F77" s="9" t="s">
         <v>28</v>
@@ -3768,7 +3768,7 @@
         <v>27</v>
       </c>
       <c r="E79" s="11">
-        <v>22</v>
+        <v>24</v>
       </c>
       <c r="F79" s="9" t="s">
         <v>28</v>
@@ -3791,7 +3791,7 @@
         <v>27</v>
       </c>
       <c r="E80" s="11">
-        <v>19</v>
+        <v>14</v>
       </c>
       <c r="F80" s="9" t="s">
         <v>28</v>
@@ -3814,7 +3814,7 @@
         <v>27</v>
       </c>
       <c r="E81" s="11">
-        <v>15</v>
+        <v>22</v>
       </c>
       <c r="F81" s="9" t="s">
         <v>28</v>
@@ -3837,7 +3837,7 @@
         <v>27</v>
       </c>
       <c r="E82" s="11">
-        <v>15</v>
+        <v>23</v>
       </c>
       <c r="F82" s="9" t="s">
         <v>28</v>
@@ -3860,7 +3860,7 @@
         <v>27</v>
       </c>
       <c r="E83" s="11">
-        <v>17</v>
+        <v>14</v>
       </c>
       <c r="F83" s="9" t="s">
         <v>28</v>
@@ -3883,7 +3883,7 @@
         <v>27</v>
       </c>
       <c r="E84" s="11">
-        <v>30</v>
+        <v>18</v>
       </c>
       <c r="F84" s="9" t="s">
         <v>28</v>
@@ -3906,7 +3906,7 @@
         <v>27</v>
       </c>
       <c r="E85" s="11">
-        <v>11</v>
+        <v>29</v>
       </c>
       <c r="F85" s="9" t="s">
         <v>28</v>
@@ -3952,7 +3952,7 @@
         <v>27</v>
       </c>
       <c r="E87" s="11">
-        <v>23</v>
+        <v>31</v>
       </c>
       <c r="F87" s="9" t="s">
         <v>28</v>
@@ -3975,7 +3975,7 @@
         <v>27</v>
       </c>
       <c r="E88" s="11">
-        <v>10</v>
+        <v>15</v>
       </c>
       <c r="F88" s="9" t="s">
         <v>28</v>
@@ -3998,7 +3998,7 @@
         <v>27</v>
       </c>
       <c r="E89" s="11">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="F89" s="9" t="s">
         <v>28</v>
@@ -4021,7 +4021,7 @@
         <v>27</v>
       </c>
       <c r="E90" s="11">
-        <v>8</v>
+        <v>14</v>
       </c>
       <c r="F90" s="9" t="s">
         <v>28</v>
@@ -4044,7 +4044,7 @@
         <v>27</v>
       </c>
       <c r="E91" s="11">
-        <v>9</v>
+        <v>18</v>
       </c>
       <c r="F91" s="9" t="s">
         <v>28</v>
@@ -4067,7 +4067,7 @@
         <v>27</v>
       </c>
       <c r="E92" s="11">
-        <v>18</v>
+        <v>21</v>
       </c>
       <c r="F92" s="9" t="s">
         <v>28</v>
@@ -4090,7 +4090,7 @@
         <v>27</v>
       </c>
       <c r="E93" s="11">
-        <v>15</v>
+        <v>24</v>
       </c>
       <c r="F93" s="9" t="s">
         <v>28</v>
@@ -4113,7 +4113,7 @@
         <v>27</v>
       </c>
       <c r="E94" s="11">
-        <v>24</v>
+        <v>31</v>
       </c>
       <c r="F94" s="9" t="s">
         <v>28</v>
@@ -4159,7 +4159,7 @@
         <v>27</v>
       </c>
       <c r="E96" s="11">
-        <v>25</v>
+        <v>20</v>
       </c>
       <c r="F96" s="9" t="s">
         <v>28</v>
@@ -4182,7 +4182,7 @@
         <v>27</v>
       </c>
       <c r="E97" s="11">
-        <v>22</v>
+        <v>25</v>
       </c>
       <c r="F97" s="9" t="s">
         <v>28</v>
@@ -4205,7 +4205,7 @@
         <v>27</v>
       </c>
       <c r="E98" s="11">
-        <v>31</v>
+        <v>24</v>
       </c>
       <c r="F98" s="9" t="s">
         <v>28</v>
@@ -4228,7 +4228,7 @@
         <v>27</v>
       </c>
       <c r="E99" s="11">
-        <v>11</v>
+        <v>15</v>
       </c>
       <c r="F99" s="9" t="s">
         <v>28</v>
@@ -4251,7 +4251,7 @@
         <v>27</v>
       </c>
       <c r="E100" s="11">
-        <v>12</v>
+        <v>30</v>
       </c>
       <c r="F100" s="9" t="s">
         <v>28</v>
@@ -4274,7 +4274,7 @@
         <v>27</v>
       </c>
       <c r="E101" s="11">
-        <v>15</v>
+        <v>22</v>
       </c>
       <c r="F101" s="9" t="s">
         <v>28</v>
@@ -4297,7 +4297,7 @@
         <v>27</v>
       </c>
       <c r="E102" s="11">
-        <v>13</v>
+        <v>29</v>
       </c>
       <c r="F102" s="9" t="s">
         <v>28</v>
@@ -4320,7 +4320,7 @@
         <v>27</v>
       </c>
       <c r="E103" s="11">
-        <v>30</v>
+        <v>26</v>
       </c>
       <c r="F103" s="9" t="s">
         <v>28</v>
@@ -4343,7 +4343,7 @@
         <v>27</v>
       </c>
       <c r="E104" s="11">
-        <v>31</v>
+        <v>27</v>
       </c>
       <c r="F104" s="9" t="s">
         <v>28</v>
@@ -4366,7 +4366,7 @@
         <v>27</v>
       </c>
       <c r="E105" s="11">
-        <v>13</v>
+        <v>16</v>
       </c>
       <c r="F105" s="9" t="s">
         <v>28</v>
@@ -4389,7 +4389,7 @@
         <v>27</v>
       </c>
       <c r="E106" s="11">
-        <v>20</v>
+        <v>23</v>
       </c>
       <c r="F106" s="9" t="s">
         <v>28</v>
@@ -4412,7 +4412,7 @@
         <v>27</v>
       </c>
       <c r="E107" s="11">
-        <v>25</v>
+        <v>22</v>
       </c>
       <c r="F107" s="9" t="s">
         <v>28</v>
@@ -4435,7 +4435,7 @@
         <v>27</v>
       </c>
       <c r="E108" s="11">
-        <v>13</v>
+        <v>31</v>
       </c>
       <c r="F108" s="9" t="s">
         <v>28</v>
@@ -4458,7 +4458,7 @@
         <v>27</v>
       </c>
       <c r="E109" s="11">
-        <v>27</v>
+        <v>11</v>
       </c>
       <c r="F109" s="9" t="s">
         <v>28</v>
@@ -4481,7 +4481,7 @@
         <v>27</v>
       </c>
       <c r="E110" s="11">
-        <v>19</v>
+        <v>22</v>
       </c>
       <c r="F110" s="9" t="s">
         <v>28</v>
@@ -4504,7 +4504,7 @@
         <v>27</v>
       </c>
       <c r="E111" s="11">
-        <v>31</v>
+        <v>23</v>
       </c>
       <c r="F111" s="9" t="s">
         <v>28</v>
@@ -4527,7 +4527,7 @@
         <v>27</v>
       </c>
       <c r="E112" s="11">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="F112" s="9" t="s">
         <v>28</v>
@@ -4550,7 +4550,7 @@
         <v>27</v>
       </c>
       <c r="E113" s="11">
-        <v>12</v>
+        <v>30</v>
       </c>
       <c r="F113" s="9" t="s">
         <v>28</v>
@@ -4573,7 +4573,7 @@
         <v>27</v>
       </c>
       <c r="E114" s="11">
-        <v>23</v>
+        <v>12</v>
       </c>
       <c r="F114" s="9" t="s">
         <v>28</v>
@@ -4596,7 +4596,7 @@
         <v>27</v>
       </c>
       <c r="E115" s="11">
-        <v>8</v>
+        <v>12</v>
       </c>
       <c r="F115" s="9" t="s">
         <v>28</v>
@@ -4619,7 +4619,7 @@
         <v>27</v>
       </c>
       <c r="E116" s="11">
-        <v>13</v>
+        <v>25</v>
       </c>
       <c r="F116" s="9" t="s">
         <v>28</v>
@@ -4642,7 +4642,7 @@
         <v>27</v>
       </c>
       <c r="E117" s="11">
-        <v>31</v>
+        <v>15</v>
       </c>
       <c r="F117" s="9" t="s">
         <v>28</v>
@@ -4665,7 +4665,7 @@
         <v>27</v>
       </c>
       <c r="E118" s="11">
-        <v>20</v>
+        <v>13</v>
       </c>
       <c r="F118" s="9" t="s">
         <v>28</v>
@@ -4688,7 +4688,7 @@
         <v>27</v>
       </c>
       <c r="E119" s="11">
-        <v>23</v>
+        <v>28</v>
       </c>
       <c r="F119" s="9" t="s">
         <v>28</v>
@@ -4711,7 +4711,7 @@
         <v>27</v>
       </c>
       <c r="E120" s="11">
-        <v>27</v>
+        <v>15</v>
       </c>
       <c r="F120" s="9" t="s">
         <v>28</v>
@@ -4757,7 +4757,7 @@
         <v>27</v>
       </c>
       <c r="E122" s="11">
-        <v>24</v>
+        <v>19</v>
       </c>
       <c r="F122" s="9" t="s">
         <v>28</v>
@@ -4780,7 +4780,7 @@
         <v>27</v>
       </c>
       <c r="E123" s="11">
-        <v>29</v>
+        <v>26</v>
       </c>
       <c r="F123" s="9" t="s">
         <v>28</v>
@@ -4803,7 +4803,7 @@
         <v>27</v>
       </c>
       <c r="E124" s="11">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="F124" s="9" t="s">
         <v>28</v>
@@ -4826,7 +4826,7 @@
         <v>27</v>
       </c>
       <c r="E125" s="11">
-        <v>24</v>
+        <v>10</v>
       </c>
       <c r="F125" s="9" t="s">
         <v>28</v>
@@ -4849,7 +4849,7 @@
         <v>27</v>
       </c>
       <c r="E126" s="11">
-        <v>31</v>
+        <v>14</v>
       </c>
       <c r="F126" s="9" t="s">
         <v>28</v>
@@ -4872,7 +4872,7 @@
         <v>27</v>
       </c>
       <c r="E127" s="11">
-        <v>23</v>
+        <v>18</v>
       </c>
       <c r="F127" s="9" t="s">
         <v>28</v>
@@ -4895,7 +4895,7 @@
         <v>27</v>
       </c>
       <c r="E128" s="11">
-        <v>11</v>
+        <v>19</v>
       </c>
       <c r="F128" s="9" t="s">
         <v>28</v>
@@ -4918,7 +4918,7 @@
         <v>27</v>
       </c>
       <c r="E129" s="11">
-        <v>10</v>
+        <v>24</v>
       </c>
       <c r="F129" s="9" t="s">
         <v>28</v>
@@ -4941,7 +4941,7 @@
         <v>27</v>
       </c>
       <c r="E130" s="11">
-        <v>15</v>
+        <v>9</v>
       </c>
       <c r="F130" s="9" t="s">
         <v>28</v>
@@ -4964,7 +4964,7 @@
         <v>27</v>
       </c>
       <c r="E131" s="11">
-        <v>8</v>
+        <v>19</v>
       </c>
       <c r="F131" s="9" t="s">
         <v>28</v>
@@ -4987,7 +4987,7 @@
         <v>27</v>
       </c>
       <c r="E132" s="11">
-        <v>22</v>
+        <v>14</v>
       </c>
       <c r="F132" s="9" t="s">
         <v>28</v>
@@ -5010,7 +5010,7 @@
         <v>27</v>
       </c>
       <c r="E133" s="11">
-        <v>16</v>
+        <v>8</v>
       </c>
       <c r="F133" s="9" t="s">
         <v>28</v>
@@ -5033,7 +5033,7 @@
         <v>27</v>
       </c>
       <c r="E134" s="11">
-        <v>22</v>
+        <v>29</v>
       </c>
       <c r="F134" s="9" t="s">
         <v>28</v>
@@ -5056,7 +5056,7 @@
         <v>27</v>
       </c>
       <c r="E135" s="11">
-        <v>29</v>
+        <v>9</v>
       </c>
       <c r="F135" s="9" t="s">
         <v>28</v>
@@ -5079,7 +5079,7 @@
         <v>27</v>
       </c>
       <c r="E136" s="11">
-        <v>24</v>
+        <v>19</v>
       </c>
       <c r="F136" s="9" t="s">
         <v>28</v>
@@ -5102,7 +5102,7 @@
         <v>27</v>
       </c>
       <c r="E137" s="11">
-        <v>8</v>
+        <v>19</v>
       </c>
       <c r="F137" s="9" t="s">
         <v>28</v>
@@ -5125,7 +5125,7 @@
         <v>27</v>
       </c>
       <c r="E138" s="11">
-        <v>27</v>
+        <v>30</v>
       </c>
       <c r="F138" s="9" t="s">
         <v>28</v>
@@ -5148,7 +5148,7 @@
         <v>27</v>
       </c>
       <c r="E139" s="11">
-        <v>8</v>
+        <v>12</v>
       </c>
       <c r="F139" s="9" t="s">
         <v>28</v>
@@ -5171,7 +5171,7 @@
         <v>27</v>
       </c>
       <c r="E140" s="11">
-        <v>17</v>
+        <v>21</v>
       </c>
       <c r="F140" s="9" t="s">
         <v>28</v>
@@ -5194,7 +5194,7 @@
         <v>27</v>
       </c>
       <c r="E141" s="11">
-        <v>28</v>
+        <v>15</v>
       </c>
       <c r="F141" s="9" t="s">
         <v>28</v>
@@ -5217,7 +5217,7 @@
         <v>27</v>
       </c>
       <c r="E142" s="11">
-        <v>18</v>
+        <v>23</v>
       </c>
       <c r="F142" s="9" t="s">
         <v>28</v>
@@ -5240,7 +5240,7 @@
         <v>27</v>
       </c>
       <c r="E143" s="11">
-        <v>30</v>
+        <v>24</v>
       </c>
       <c r="F143" s="9" t="s">
         <v>28</v>
@@ -5263,7 +5263,7 @@
         <v>27</v>
       </c>
       <c r="E144" s="11">
-        <v>8</v>
+        <v>14</v>
       </c>
       <c r="F144" s="9" t="s">
         <v>28</v>
@@ -5286,7 +5286,7 @@
         <v>27</v>
       </c>
       <c r="E145" s="11">
-        <v>13</v>
+        <v>19</v>
       </c>
       <c r="F145" s="9" t="s">
         <v>28</v>
@@ -5309,7 +5309,7 @@
         <v>27</v>
       </c>
       <c r="E146" s="11">
-        <v>11</v>
+        <v>8</v>
       </c>
       <c r="F146" s="9" t="s">
         <v>28</v>
@@ -5332,7 +5332,7 @@
         <v>27</v>
       </c>
       <c r="E147" s="11">
-        <v>9</v>
+        <v>24</v>
       </c>
       <c r="F147" s="9" t="s">
         <v>28</v>
@@ -5355,7 +5355,7 @@
         <v>27</v>
       </c>
       <c r="E148" s="11">
-        <v>28</v>
+        <v>9</v>
       </c>
       <c r="F148" s="9" t="s">
         <v>28</v>
@@ -5378,7 +5378,7 @@
         <v>27</v>
       </c>
       <c r="E149" s="11">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="F149" s="9" t="s">
         <v>28</v>
@@ -5401,7 +5401,7 @@
         <v>27</v>
       </c>
       <c r="E150" s="11">
-        <v>19</v>
+        <v>11</v>
       </c>
       <c r="F150" s="9" t="s">
         <v>28</v>
@@ -5424,7 +5424,7 @@
         <v>27</v>
       </c>
       <c r="E151" s="11">
-        <v>10</v>
+        <v>17</v>
       </c>
       <c r="F151" s="9" t="s">
         <v>28</v>
@@ -5447,7 +5447,7 @@
         <v>27</v>
       </c>
       <c r="E152" s="11">
-        <v>26</v>
+        <v>10</v>
       </c>
       <c r="F152" s="9" t="s">
         <v>28</v>
@@ -5470,7 +5470,7 @@
         <v>27</v>
       </c>
       <c r="E153" s="11">
-        <v>30</v>
+        <v>24</v>
       </c>
       <c r="F153" s="9" t="s">
         <v>28</v>
@@ -5493,7 +5493,7 @@
         <v>27</v>
       </c>
       <c r="E154" s="11">
-        <v>22</v>
+        <v>30</v>
       </c>
       <c r="F154" s="9" t="s">
         <v>28</v>
@@ -5516,7 +5516,7 @@
         <v>27</v>
       </c>
       <c r="E155" s="11">
-        <v>8</v>
+        <v>20</v>
       </c>
       <c r="F155" s="9" t="s">
         <v>28</v>
@@ -5539,7 +5539,7 @@
         <v>27</v>
       </c>
       <c r="E156" s="11">
-        <v>8</v>
+        <v>18</v>
       </c>
       <c r="F156" s="9" t="s">
         <v>28</v>
@@ -5562,7 +5562,7 @@
         <v>27</v>
       </c>
       <c r="E157" s="11">
-        <v>28</v>
+        <v>20</v>
       </c>
       <c r="F157" s="9" t="s">
         <v>28</v>
@@ -5585,7 +5585,7 @@
         <v>27</v>
       </c>
       <c r="E158" s="11">
-        <v>17</v>
+        <v>14</v>
       </c>
       <c r="F158" s="9" t="s">
         <v>28</v>
@@ -5608,7 +5608,7 @@
         <v>27</v>
       </c>
       <c r="E159" s="11">
-        <v>12</v>
+        <v>31</v>
       </c>
       <c r="F159" s="9" t="s">
         <v>28</v>
@@ -5631,7 +5631,7 @@
         <v>27</v>
       </c>
       <c r="E160" s="11">
-        <v>26</v>
+        <v>13</v>
       </c>
       <c r="F160" s="9" t="s">
         <v>28</v>
@@ -5654,7 +5654,7 @@
         <v>27</v>
       </c>
       <c r="E161" s="11">
-        <v>9</v>
+        <v>24</v>
       </c>
       <c r="F161" s="9" t="s">
         <v>28</v>
@@ -5700,7 +5700,7 @@
         <v>27</v>
       </c>
       <c r="E163" s="11">
-        <v>26</v>
+        <v>28</v>
       </c>
       <c r="F163" s="9" t="s">
         <v>28</v>
@@ -5723,7 +5723,7 @@
         <v>27</v>
       </c>
       <c r="E164" s="11">
-        <v>25</v>
+        <v>28</v>
       </c>
       <c r="F164" s="9" t="s">
         <v>28</v>
@@ -5746,7 +5746,7 @@
         <v>27</v>
       </c>
       <c r="E165" s="11">
-        <v>17</v>
+        <v>10</v>
       </c>
       <c r="F165" s="9" t="s">
         <v>28</v>
@@ -5769,7 +5769,7 @@
         <v>27</v>
       </c>
       <c r="E166" s="11">
-        <v>20</v>
+        <v>22</v>
       </c>
       <c r="F166" s="9" t="s">
         <v>28</v>
@@ -5792,7 +5792,7 @@
         <v>27</v>
       </c>
       <c r="E167" s="11">
-        <v>19</v>
+        <v>27</v>
       </c>
       <c r="F167" s="9" t="s">
         <v>28</v>
@@ -5815,7 +5815,7 @@
         <v>27</v>
       </c>
       <c r="E168" s="11">
-        <v>19</v>
+        <v>12</v>
       </c>
       <c r="F168" s="9" t="s">
         <v>28</v>
@@ -5838,7 +5838,7 @@
         <v>27</v>
       </c>
       <c r="E169" s="11">
-        <v>25</v>
+        <v>20</v>
       </c>
       <c r="F169" s="9" t="s">
         <v>28</v>
@@ -5861,7 +5861,7 @@
         <v>27</v>
       </c>
       <c r="E170" s="11">
-        <v>10</v>
+        <v>26</v>
       </c>
       <c r="F170" s="9" t="s">
         <v>28</v>
@@ -5884,7 +5884,7 @@
         <v>27</v>
       </c>
       <c r="E171" s="11">
-        <v>17</v>
+        <v>22</v>
       </c>
       <c r="F171" s="9" t="s">
         <v>28</v>
@@ -5907,7 +5907,7 @@
         <v>27</v>
       </c>
       <c r="E172" s="11">
-        <v>9</v>
+        <v>20</v>
       </c>
       <c r="F172" s="9" t="s">
         <v>28</v>
@@ -5930,7 +5930,7 @@
         <v>27</v>
       </c>
       <c r="E173" s="11">
-        <v>25</v>
+        <v>21</v>
       </c>
       <c r="F173" s="9" t="s">
         <v>28</v>
@@ -5953,7 +5953,7 @@
         <v>27</v>
       </c>
       <c r="E174" s="11">
-        <v>16</v>
+        <v>21</v>
       </c>
       <c r="F174" s="9" t="s">
         <v>28</v>
@@ -5976,7 +5976,7 @@
         <v>27</v>
       </c>
       <c r="E175" s="11">
-        <v>22</v>
+        <v>19</v>
       </c>
       <c r="F175" s="9" t="s">
         <v>28</v>
@@ -5999,7 +5999,7 @@
         <v>27</v>
       </c>
       <c r="E176" s="11">
-        <v>11</v>
+        <v>28</v>
       </c>
       <c r="F176" s="9" t="s">
         <v>28</v>
@@ -6045,7 +6045,7 @@
         <v>27</v>
       </c>
       <c r="E178" s="11">
-        <v>28</v>
+        <v>19</v>
       </c>
       <c r="F178" s="9" t="s">
         <v>28</v>
@@ -6068,7 +6068,7 @@
         <v>27</v>
       </c>
       <c r="E179" s="11">
-        <v>18</v>
+        <v>20</v>
       </c>
       <c r="F179" s="9" t="s">
         <v>28</v>
@@ -6091,7 +6091,7 @@
         <v>27</v>
       </c>
       <c r="E180" s="11">
-        <v>8</v>
+        <v>19</v>
       </c>
       <c r="F180" s="9" t="s">
         <v>28</v>
@@ -6114,7 +6114,7 @@
         <v>27</v>
       </c>
       <c r="E181" s="11">
-        <v>9</v>
+        <v>24</v>
       </c>
       <c r="F181" s="9" t="s">
         <v>28</v>
@@ -6137,7 +6137,7 @@
         <v>27</v>
       </c>
       <c r="E182" s="11">
-        <v>9</v>
+        <v>13</v>
       </c>
       <c r="F182" s="9" t="s">
         <v>28</v>
@@ -6160,7 +6160,7 @@
         <v>27</v>
       </c>
       <c r="E183" s="11">
-        <v>8</v>
+        <v>25</v>
       </c>
       <c r="F183" s="9" t="s">
         <v>28</v>
@@ -6183,7 +6183,7 @@
         <v>27</v>
       </c>
       <c r="E184" s="11">
-        <v>22</v>
+        <v>16</v>
       </c>
       <c r="F184" s="9" t="s">
         <v>28</v>
@@ -6206,7 +6206,7 @@
         <v>27</v>
       </c>
       <c r="E185" s="11">
-        <v>10</v>
+        <v>27</v>
       </c>
       <c r="F185" s="9" t="s">
         <v>28</v>
@@ -6229,7 +6229,7 @@
         <v>27</v>
       </c>
       <c r="E186" s="11">
-        <v>11</v>
+        <v>24</v>
       </c>
       <c r="F186" s="9" t="s">
         <v>28</v>
@@ -6252,7 +6252,7 @@
         <v>27</v>
       </c>
       <c r="E187" s="11">
-        <v>31</v>
+        <v>18</v>
       </c>
       <c r="F187" s="9" t="s">
         <v>28</v>
@@ -6275,7 +6275,7 @@
         <v>27</v>
       </c>
       <c r="E188" s="11">
-        <v>13</v>
+        <v>15</v>
       </c>
       <c r="F188" s="9" t="s">
         <v>28</v>
@@ -6321,7 +6321,7 @@
         <v>27</v>
       </c>
       <c r="E190" s="11">
-        <v>30</v>
+        <v>27</v>
       </c>
       <c r="F190" s="9" t="s">
         <v>28</v>
@@ -6344,7 +6344,7 @@
         <v>27</v>
       </c>
       <c r="E191" s="11">
-        <v>26</v>
+        <v>24</v>
       </c>
       <c r="F191" s="9" t="s">
         <v>28</v>
@@ -6367,7 +6367,7 @@
         <v>27</v>
       </c>
       <c r="E192" s="11">
-        <v>8</v>
+        <v>27</v>
       </c>
       <c r="F192" s="9" t="s">
         <v>28</v>
@@ -6390,7 +6390,7 @@
         <v>27</v>
       </c>
       <c r="E193" s="11">
-        <v>18</v>
+        <v>31</v>
       </c>
       <c r="F193" s="9" t="s">
         <v>28</v>
@@ -6413,7 +6413,7 @@
         <v>27</v>
       </c>
       <c r="E194" s="11">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="F194" s="9" t="s">
         <v>28</v>
@@ -6436,7 +6436,7 @@
         <v>27</v>
       </c>
       <c r="E195" s="11">
-        <v>17</v>
+        <v>24</v>
       </c>
       <c r="F195" s="9" t="s">
         <v>28</v>
@@ -6459,7 +6459,7 @@
         <v>27</v>
       </c>
       <c r="E196" s="11">
-        <v>26</v>
+        <v>12</v>
       </c>
       <c r="F196" s="9" t="s">
         <v>28</v>
@@ -6505,7 +6505,7 @@
         <v>27</v>
       </c>
       <c r="E198" s="11">
-        <v>9</v>
+        <v>18</v>
       </c>
       <c r="F198" s="9" t="s">
         <v>28</v>
@@ -6528,7 +6528,7 @@
         <v>27</v>
       </c>
       <c r="E199" s="11">
-        <v>20</v>
+        <v>29</v>
       </c>
       <c r="F199" s="9" t="s">
         <v>28</v>
@@ -6551,7 +6551,7 @@
         <v>27</v>
       </c>
       <c r="E200" s="11">
-        <v>20</v>
+        <v>27</v>
       </c>
       <c r="F200" s="9" t="s">
         <v>28</v>
@@ -6574,7 +6574,7 @@
         <v>27</v>
       </c>
       <c r="E201" s="11">
-        <v>31</v>
+        <v>28</v>
       </c>
       <c r="F201" s="9" t="s">
         <v>28</v>
@@ -6597,7 +6597,7 @@
         <v>27</v>
       </c>
       <c r="E202" s="11">
-        <v>29</v>
+        <v>18</v>
       </c>
       <c r="F202" s="9" t="s">
         <v>28</v>
@@ -6620,7 +6620,7 @@
         <v>27</v>
       </c>
       <c r="E203" s="11">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="F203" s="9" t="s">
         <v>28</v>
@@ -6643,7 +6643,7 @@
         <v>27</v>
       </c>
       <c r="E204" s="11">
-        <v>23</v>
+        <v>13</v>
       </c>
       <c r="F204" s="9" t="s">
         <v>28</v>
@@ -6666,7 +6666,7 @@
         <v>27</v>
       </c>
       <c r="E205" s="11">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="F205" s="9" t="s">
         <v>28</v>
@@ -6689,7 +6689,7 @@
         <v>27</v>
       </c>
       <c r="E206" s="11">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="F206" s="9" t="s">
         <v>28</v>
@@ -6712,7 +6712,7 @@
         <v>27</v>
       </c>
       <c r="E207" s="11">
-        <v>14</v>
+        <v>20</v>
       </c>
       <c r="F207" s="9" t="s">
         <v>28</v>
@@ -6735,7 +6735,7 @@
         <v>27</v>
       </c>
       <c r="E208" s="11">
-        <v>25</v>
+        <v>9</v>
       </c>
       <c r="F208" s="9" t="s">
         <v>28</v>
@@ -6758,7 +6758,7 @@
         <v>27</v>
       </c>
       <c r="E209" s="11">
-        <v>11</v>
+        <v>18</v>
       </c>
       <c r="F209" s="9" t="s">
         <v>28</v>
@@ -6781,7 +6781,7 @@
         <v>27</v>
       </c>
       <c r="E210" s="11">
-        <v>12</v>
+        <v>17</v>
       </c>
       <c r="F210" s="9" t="s">
         <v>28</v>
@@ -6804,7 +6804,7 @@
         <v>27</v>
       </c>
       <c r="E211" s="11">
-        <v>30</v>
+        <v>11</v>
       </c>
       <c r="F211" s="9" t="s">
         <v>28</v>
@@ -6827,7 +6827,7 @@
         <v>27</v>
       </c>
       <c r="E212" s="11">
-        <v>14</v>
+        <v>26</v>
       </c>
       <c r="F212" s="9" t="s">
         <v>28</v>
@@ -6850,7 +6850,7 @@
         <v>27</v>
       </c>
       <c r="E213" s="11">
-        <v>10</v>
+        <v>19</v>
       </c>
       <c r="F213" s="9" t="s">
         <v>28</v>
@@ -6873,7 +6873,7 @@
         <v>27</v>
       </c>
       <c r="E214" s="11">
-        <v>16</v>
+        <v>31</v>
       </c>
       <c r="F214" s="9" t="s">
         <v>28</v>
@@ -6896,7 +6896,7 @@
         <v>27</v>
       </c>
       <c r="E215" s="11">
-        <v>28</v>
+        <v>15</v>
       </c>
       <c r="F215" s="9" t="s">
         <v>28</v>
@@ -6919,7 +6919,7 @@
         <v>27</v>
       </c>
       <c r="E216" s="11">
-        <v>22</v>
+        <v>11</v>
       </c>
       <c r="F216" s="9" t="s">
         <v>28</v>
@@ -6942,7 +6942,7 @@
         <v>27</v>
       </c>
       <c r="E217" s="11">
-        <v>13</v>
+        <v>16</v>
       </c>
       <c r="F217" s="9" t="s">
         <v>28</v>
@@ -6965,7 +6965,7 @@
         <v>27</v>
       </c>
       <c r="E218" s="11">
-        <v>23</v>
+        <v>20</v>
       </c>
       <c r="F218" s="9" t="s">
         <v>28</v>
@@ -6988,7 +6988,7 @@
         <v>27</v>
       </c>
       <c r="E219" s="11">
-        <v>15</v>
+        <v>11</v>
       </c>
       <c r="F219" s="9" t="s">
         <v>28</v>
@@ -7011,7 +7011,7 @@
         <v>27</v>
       </c>
       <c r="E220" s="11">
-        <v>26</v>
+        <v>23</v>
       </c>
       <c r="F220" s="9" t="s">
         <v>28</v>
@@ -7034,7 +7034,7 @@
         <v>27</v>
       </c>
       <c r="E221" s="11">
-        <v>24</v>
+        <v>29</v>
       </c>
       <c r="F221" s="9" t="s">
         <v>28</v>
@@ -7057,7 +7057,7 @@
         <v>27</v>
       </c>
       <c r="E222" s="11">
-        <v>9</v>
+        <v>25</v>
       </c>
       <c r="F222" s="9" t="s">
         <v>28</v>
@@ -7080,7 +7080,7 @@
         <v>27</v>
       </c>
       <c r="E223" s="11">
-        <v>13</v>
+        <v>24</v>
       </c>
       <c r="F223" s="9" t="s">
         <v>28</v>
@@ -7103,7 +7103,7 @@
         <v>27</v>
       </c>
       <c r="E224" s="11">
-        <v>21</v>
+        <v>24</v>
       </c>
       <c r="F224" s="9" t="s">
         <v>28</v>
@@ -7126,7 +7126,7 @@
         <v>27</v>
       </c>
       <c r="E225" s="11">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="F225" s="9" t="s">
         <v>28</v>
@@ -7149,7 +7149,7 @@
         <v>27</v>
       </c>
       <c r="E226" s="11">
-        <v>15</v>
+        <v>29</v>
       </c>
       <c r="F226" s="9" t="s">
         <v>28</v>
@@ -7172,7 +7172,7 @@
         <v>27</v>
       </c>
       <c r="E227" s="11">
-        <v>22</v>
+        <v>13</v>
       </c>
       <c r="F227" s="9" t="s">
         <v>28</v>
@@ -7195,7 +7195,7 @@
         <v>27</v>
       </c>
       <c r="E228" s="11">
-        <v>27</v>
+        <v>30</v>
       </c>
       <c r="F228" s="9" t="s">
         <v>28</v>
@@ -7218,7 +7218,7 @@
         <v>27</v>
       </c>
       <c r="E229" s="11">
-        <v>28</v>
+        <v>16</v>
       </c>
       <c r="F229" s="9" t="s">
         <v>28</v>
@@ -7241,7 +7241,7 @@
         <v>27</v>
       </c>
       <c r="E230" s="11">
-        <v>21</v>
+        <v>10</v>
       </c>
       <c r="F230" s="9" t="s">
         <v>28</v>
@@ -7264,7 +7264,7 @@
         <v>27</v>
       </c>
       <c r="E231" s="11">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="F231" s="9" t="s">
         <v>28</v>
@@ -7287,7 +7287,7 @@
         <v>27</v>
       </c>
       <c r="E232" s="11">
-        <v>21</v>
+        <v>28</v>
       </c>
       <c r="F232" s="9" t="s">
         <v>28</v>
@@ -7310,7 +7310,7 @@
         <v>27</v>
       </c>
       <c r="E233" s="11">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="F233" s="9" t="s">
         <v>28</v>
@@ -7333,7 +7333,7 @@
         <v>27</v>
       </c>
       <c r="E234" s="11">
-        <v>21</v>
+        <v>13</v>
       </c>
       <c r="F234" s="9" t="s">
         <v>28</v>
@@ -7356,7 +7356,7 @@
         <v>27</v>
       </c>
       <c r="E235" s="11">
-        <v>12</v>
+        <v>24</v>
       </c>
       <c r="F235" s="9" t="s">
         <v>28</v>
@@ -7379,7 +7379,7 @@
         <v>27</v>
       </c>
       <c r="E236" s="11">
-        <v>20</v>
+        <v>10</v>
       </c>
       <c r="F236" s="9" t="s">
         <v>28</v>
@@ -7402,7 +7402,7 @@
         <v>27</v>
       </c>
       <c r="E237" s="11">
-        <v>26</v>
+        <v>13</v>
       </c>
       <c r="F237" s="9" t="s">
         <v>28</v>
@@ -7425,7 +7425,7 @@
         <v>27</v>
       </c>
       <c r="E238" s="11">
-        <v>22</v>
+        <v>17</v>
       </c>
       <c r="F238" s="9" t="s">
         <v>28</v>
@@ -7448,7 +7448,7 @@
         <v>27</v>
       </c>
       <c r="E239" s="11">
-        <v>15</v>
+        <v>26</v>
       </c>
       <c r="F239" s="9" t="s">
         <v>28</v>
@@ -7471,7 +7471,7 @@
         <v>27</v>
       </c>
       <c r="E240" s="11">
-        <v>31</v>
+        <v>22</v>
       </c>
       <c r="F240" s="9" t="s">
         <v>28</v>
@@ -7494,7 +7494,7 @@
         <v>27</v>
       </c>
       <c r="E241" s="11">
-        <v>8</v>
+        <v>27</v>
       </c>
       <c r="F241" s="9" t="s">
         <v>28</v>
@@ -7517,7 +7517,7 @@
         <v>27</v>
       </c>
       <c r="E242" s="11">
-        <v>27</v>
+        <v>21</v>
       </c>
       <c r="F242" s="9" t="s">
         <v>28</v>
@@ -7540,7 +7540,7 @@
         <v>27</v>
       </c>
       <c r="E243" s="11">
-        <v>15</v>
+        <v>18</v>
       </c>
       <c r="F243" s="9" t="s">
         <v>28</v>
@@ -7563,7 +7563,7 @@
         <v>27</v>
       </c>
       <c r="E244" s="11">
-        <v>8</v>
+        <v>11</v>
       </c>
       <c r="F244" s="9" t="s">
         <v>28</v>
@@ -7609,7 +7609,7 @@
         <v>27</v>
       </c>
       <c r="E246" s="11">
-        <v>15</v>
+        <v>18</v>
       </c>
       <c r="F246" s="9" t="s">
         <v>28</v>
@@ -7632,7 +7632,7 @@
         <v>27</v>
       </c>
       <c r="E247" s="11">
-        <v>10</v>
+        <v>28</v>
       </c>
       <c r="F247" s="9" t="s">
         <v>28</v>
@@ -7655,7 +7655,7 @@
         <v>27</v>
       </c>
       <c r="E248" s="11">
-        <v>30</v>
+        <v>14</v>
       </c>
       <c r="F248" s="9" t="s">
         <v>28</v>
@@ -7678,7 +7678,7 @@
         <v>27</v>
       </c>
       <c r="E249" s="11">
-        <v>26</v>
+        <v>28</v>
       </c>
       <c r="F249" s="9" t="s">
         <v>28</v>
@@ -7701,7 +7701,7 @@
         <v>27</v>
       </c>
       <c r="E250" s="11">
-        <v>26</v>
+        <v>24</v>
       </c>
       <c r="F250" s="9" t="s">
         <v>28</v>
@@ -7724,7 +7724,7 @@
         <v>27</v>
       </c>
       <c r="E251" s="11">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="F251" s="9" t="s">
         <v>28</v>
@@ -7747,7 +7747,7 @@
         <v>27</v>
       </c>
       <c r="E252" s="11">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="F252" s="9" t="s">
         <v>28</v>
@@ -7770,7 +7770,7 @@
         <v>27</v>
       </c>
       <c r="E253" s="11">
-        <v>11</v>
+        <v>16</v>
       </c>
       <c r="F253" s="9" t="s">
         <v>28</v>
@@ -7793,7 +7793,7 @@
         <v>27</v>
       </c>
       <c r="E254" s="11">
-        <v>30</v>
+        <v>24</v>
       </c>
       <c r="F254" s="9" t="s">
         <v>28</v>
@@ -7816,7 +7816,7 @@
         <v>27</v>
       </c>
       <c r="E255" s="11">
-        <v>21</v>
+        <v>25</v>
       </c>
       <c r="F255" s="9" t="s">
         <v>28</v>
@@ -7839,7 +7839,7 @@
         <v>27</v>
       </c>
       <c r="E256" s="11">
-        <v>16</v>
+        <v>20</v>
       </c>
       <c r="F256" s="9" t="s">
         <v>28</v>
@@ -7862,7 +7862,7 @@
         <v>27</v>
       </c>
       <c r="E257" s="11">
-        <v>27</v>
+        <v>24</v>
       </c>
       <c r="F257" s="9" t="s">
         <v>28</v>
@@ -7885,7 +7885,7 @@
         <v>27</v>
       </c>
       <c r="E258" s="11">
-        <v>15</v>
+        <v>23</v>
       </c>
       <c r="F258" s="9" t="s">
         <v>28</v>
@@ -7908,7 +7908,7 @@
         <v>27</v>
       </c>
       <c r="E259" s="11">
-        <v>27</v>
+        <v>15</v>
       </c>
       <c r="F259" s="9" t="s">
         <v>28</v>
@@ -7931,7 +7931,7 @@
         <v>27</v>
       </c>
       <c r="E260" s="11">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="F260" s="9" t="s">
         <v>28</v>
@@ -7954,7 +7954,7 @@
         <v>27</v>
       </c>
       <c r="E261" s="11">
-        <v>10</v>
+        <v>18</v>
       </c>
       <c r="F261" s="9" t="s">
         <v>28</v>
@@ -7977,7 +7977,7 @@
         <v>27</v>
       </c>
       <c r="E262" s="11">
-        <v>19</v>
+        <v>17</v>
       </c>
       <c r="F262" s="9" t="s">
         <v>28</v>
@@ -8000,7 +8000,7 @@
         <v>27</v>
       </c>
       <c r="E263" s="11">
-        <v>17</v>
+        <v>27</v>
       </c>
       <c r="F263" s="9" t="s">
         <v>28</v>
@@ -8023,7 +8023,7 @@
         <v>27</v>
       </c>
       <c r="E264" s="11">
-        <v>19</v>
+        <v>27</v>
       </c>
       <c r="F264" s="9" t="s">
         <v>28</v>
@@ -8046,7 +8046,7 @@
         <v>27</v>
       </c>
       <c r="E265" s="11">
-        <v>12</v>
+        <v>18</v>
       </c>
       <c r="F265" s="9" t="s">
         <v>28</v>
@@ -8069,7 +8069,7 @@
         <v>27</v>
       </c>
       <c r="E266" s="11">
-        <v>14</v>
+        <v>26</v>
       </c>
       <c r="F266" s="9" t="s">
         <v>28</v>
@@ -8092,7 +8092,7 @@
         <v>27</v>
       </c>
       <c r="E267" s="11">
-        <v>25</v>
+        <v>21</v>
       </c>
       <c r="F267" s="9" t="s">
         <v>28</v>
@@ -8115,7 +8115,7 @@
         <v>27</v>
       </c>
       <c r="E268" s="11">
-        <v>30</v>
+        <v>27</v>
       </c>
       <c r="F268" s="9" t="s">
         <v>28</v>
@@ -8138,7 +8138,7 @@
         <v>27</v>
       </c>
       <c r="E269" s="11">
-        <v>29</v>
+        <v>10</v>
       </c>
       <c r="F269" s="9" t="s">
         <v>28</v>
@@ -8161,7 +8161,7 @@
         <v>27</v>
       </c>
       <c r="E270" s="11">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="F270" s="9" t="s">
         <v>28</v>
@@ -8184,7 +8184,7 @@
         <v>27</v>
       </c>
       <c r="E271" s="11">
-        <v>18</v>
+        <v>10</v>
       </c>
       <c r="F271" s="9" t="s">
         <v>28</v>
@@ -8207,7 +8207,7 @@
         <v>27</v>
       </c>
       <c r="E272" s="11">
-        <v>25</v>
+        <v>23</v>
       </c>
       <c r="F272" s="9" t="s">
         <v>28</v>
@@ -8230,7 +8230,7 @@
         <v>27</v>
       </c>
       <c r="E273" s="11">
-        <v>11</v>
+        <v>26</v>
       </c>
       <c r="F273" s="9" t="s">
         <v>28</v>
@@ -8253,7 +8253,7 @@
         <v>27</v>
       </c>
       <c r="E274" s="11">
-        <v>27</v>
+        <v>17</v>
       </c>
       <c r="F274" s="9" t="s">
         <v>28</v>
@@ -8276,7 +8276,7 @@
         <v>27</v>
       </c>
       <c r="E275" s="11">
-        <v>14</v>
+        <v>22</v>
       </c>
       <c r="F275" s="9" t="s">
         <v>28</v>
@@ -8299,7 +8299,7 @@
         <v>27</v>
       </c>
       <c r="E276" s="11">
-        <v>24</v>
+        <v>20</v>
       </c>
       <c r="F276" s="9" t="s">
         <v>28</v>
@@ -8322,7 +8322,7 @@
         <v>27</v>
       </c>
       <c r="E277" s="11">
-        <v>24</v>
+        <v>15</v>
       </c>
       <c r="F277" s="9" t="s">
         <v>28</v>
@@ -8345,7 +8345,7 @@
         <v>27</v>
       </c>
       <c r="E278" s="11">
-        <v>15</v>
+        <v>17</v>
       </c>
       <c r="F278" s="9" t="s">
         <v>28</v>
@@ -8368,7 +8368,7 @@
         <v>27</v>
       </c>
       <c r="E279" s="11">
-        <v>26</v>
+        <v>12</v>
       </c>
       <c r="F279" s="9" t="s">
         <v>28</v>
@@ -8391,7 +8391,7 @@
         <v>27</v>
       </c>
       <c r="E280" s="11">
-        <v>8</v>
+        <v>15</v>
       </c>
       <c r="F280" s="9" t="s">
         <v>28</v>
@@ -8414,7 +8414,7 @@
         <v>27</v>
       </c>
       <c r="E281" s="11">
-        <v>22</v>
+        <v>15</v>
       </c>
       <c r="F281" s="9" t="s">
         <v>28</v>
@@ -8437,7 +8437,7 @@
         <v>27</v>
       </c>
       <c r="E282" s="11">
-        <v>26</v>
+        <v>31</v>
       </c>
       <c r="F282" s="9" t="s">
         <v>28</v>
@@ -8460,7 +8460,7 @@
         <v>27</v>
       </c>
       <c r="E283" s="11">
-        <v>25</v>
+        <v>14</v>
       </c>
       <c r="F283" s="9" t="s">
         <v>28</v>
@@ -8483,7 +8483,7 @@
         <v>27</v>
       </c>
       <c r="E284" s="11">
-        <v>17</v>
+        <v>21</v>
       </c>
       <c r="F284" s="9" t="s">
         <v>28</v>
@@ -8506,7 +8506,7 @@
         <v>27</v>
       </c>
       <c r="E285" s="11">
-        <v>19</v>
+        <v>9</v>
       </c>
       <c r="F285" s="9" t="s">
         <v>28</v>
@@ -8529,7 +8529,7 @@
         <v>27</v>
       </c>
       <c r="E286" s="11">
-        <v>23</v>
+        <v>11</v>
       </c>
       <c r="F286" s="9" t="s">
         <v>28</v>
@@ -8552,7 +8552,7 @@
         <v>27</v>
       </c>
       <c r="E287" s="11">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="F287" s="9" t="s">
         <v>28</v>
@@ -8575,7 +8575,7 @@
         <v>27</v>
       </c>
       <c r="E288" s="11">
-        <v>18</v>
+        <v>15</v>
       </c>
       <c r="F288" s="9" t="s">
         <v>28</v>
@@ -8598,7 +8598,7 @@
         <v>27</v>
       </c>
       <c r="E289" s="11">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="F289" s="9" t="s">
         <v>28</v>
@@ -8621,7 +8621,7 @@
         <v>27</v>
       </c>
       <c r="E290" s="11">
-        <v>31</v>
+        <v>13</v>
       </c>
       <c r="F290" s="9" t="s">
         <v>28</v>
@@ -8667,7 +8667,7 @@
         <v>27</v>
       </c>
       <c r="E292" s="11">
-        <v>25</v>
+        <v>30</v>
       </c>
       <c r="F292" s="9" t="s">
         <v>28</v>
@@ -8690,7 +8690,7 @@
         <v>27</v>
       </c>
       <c r="E293" s="11">
-        <v>19</v>
+        <v>26</v>
       </c>
       <c r="F293" s="9" t="s">
         <v>28</v>
@@ -8713,7 +8713,7 @@
         <v>27</v>
       </c>
       <c r="E294" s="11">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="F294" s="9" t="s">
         <v>28</v>
@@ -8736,7 +8736,7 @@
         <v>27</v>
       </c>
       <c r="E295" s="11">
-        <v>26</v>
+        <v>18</v>
       </c>
       <c r="F295" s="9" t="s">
         <v>28</v>
@@ -8759,7 +8759,7 @@
         <v>27</v>
       </c>
       <c r="E296" s="11">
-        <v>12</v>
+        <v>18</v>
       </c>
       <c r="F296" s="9" t="s">
         <v>28</v>
@@ -8782,7 +8782,7 @@
         <v>27</v>
       </c>
       <c r="E297" s="11">
-        <v>31</v>
+        <v>23</v>
       </c>
       <c r="F297" s="9" t="s">
         <v>28</v>
@@ -8805,7 +8805,7 @@
         <v>27</v>
       </c>
       <c r="E298" s="11">
-        <v>26</v>
+        <v>28</v>
       </c>
       <c r="F298" s="9" t="s">
         <v>28</v>
@@ -8828,7 +8828,7 @@
         <v>27</v>
       </c>
       <c r="E299" s="11">
-        <v>16</v>
+        <v>23</v>
       </c>
       <c r="F299" s="9" t="s">
         <v>28</v>
@@ -8851,7 +8851,7 @@
         <v>27</v>
       </c>
       <c r="E300" s="11">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="F300" s="9" t="s">
         <v>28</v>
@@ -8874,7 +8874,7 @@
         <v>27</v>
       </c>
       <c r="E301" s="11">
-        <v>15</v>
+        <v>29</v>
       </c>
       <c r="F301" s="9" t="s">
         <v>28</v>
@@ -8897,7 +8897,7 @@
         <v>27</v>
       </c>
       <c r="E302" s="11">
-        <v>24</v>
+        <v>18</v>
       </c>
       <c r="F302" s="9" t="s">
         <v>28</v>
@@ -8920,7 +8920,7 @@
         <v>27</v>
       </c>
       <c r="E303" s="11">
-        <v>31</v>
+        <v>8</v>
       </c>
       <c r="F303" s="9" t="s">
         <v>28</v>
@@ -8943,7 +8943,7 @@
         <v>27</v>
       </c>
       <c r="E304" s="11">
-        <v>28</v>
+        <v>15</v>
       </c>
       <c r="F304" s="9" t="s">
         <v>28</v>
@@ -8989,7 +8989,7 @@
         <v>27</v>
       </c>
       <c r="E306" s="11">
-        <v>21</v>
+        <v>11</v>
       </c>
       <c r="F306" s="9" t="s">
         <v>28</v>
@@ -9012,7 +9012,7 @@
         <v>27</v>
       </c>
       <c r="E307" s="11">
-        <v>26</v>
+        <v>30</v>
       </c>
       <c r="F307" s="9" t="s">
         <v>28</v>
@@ -9035,7 +9035,7 @@
         <v>27</v>
       </c>
       <c r="E308" s="11">
-        <v>9</v>
+        <v>27</v>
       </c>
       <c r="F308" s="9" t="s">
         <v>28</v>
@@ -9081,7 +9081,7 @@
         <v>27</v>
       </c>
       <c r="E310" s="11">
-        <v>22</v>
+        <v>30</v>
       </c>
       <c r="F310" s="9" t="s">
         <v>28</v>
@@ -9104,7 +9104,7 @@
         <v>27</v>
       </c>
       <c r="E311" s="11">
-        <v>23</v>
+        <v>9</v>
       </c>
       <c r="F311" s="9" t="s">
         <v>28</v>
@@ -9127,7 +9127,7 @@
         <v>27</v>
       </c>
       <c r="E312" s="11">
-        <v>18</v>
+        <v>10</v>
       </c>
       <c r="F312" s="9" t="s">
         <v>28</v>
@@ -9150,7 +9150,7 @@
         <v>27</v>
       </c>
       <c r="E313" s="11">
-        <v>24</v>
+        <v>16</v>
       </c>
       <c r="F313" s="9" t="s">
         <v>28</v>
@@ -9173,7 +9173,7 @@
         <v>27</v>
       </c>
       <c r="E314" s="11">
-        <v>17</v>
+        <v>19</v>
       </c>
       <c r="F314" s="9" t="s">
         <v>28</v>
@@ -9196,7 +9196,7 @@
         <v>27</v>
       </c>
       <c r="E315" s="11">
-        <v>29</v>
+        <v>11</v>
       </c>
       <c r="F315" s="9" t="s">
         <v>28</v>
@@ -9219,7 +9219,7 @@
         <v>27</v>
       </c>
       <c r="E316" s="11">
-        <v>27</v>
+        <v>12</v>
       </c>
       <c r="F316" s="9" t="s">
         <v>28</v>
@@ -9242,7 +9242,7 @@
         <v>27</v>
       </c>
       <c r="E317" s="11">
-        <v>17</v>
+        <v>15</v>
       </c>
       <c r="F317" s="9" t="s">
         <v>28</v>
@@ -9265,7 +9265,7 @@
         <v>27</v>
       </c>
       <c r="E318" s="11">
-        <v>17</v>
+        <v>13</v>
       </c>
       <c r="F318" s="9" t="s">
         <v>28</v>
@@ -9288,7 +9288,7 @@
         <v>27</v>
       </c>
       <c r="E319" s="11">
-        <v>14</v>
+        <v>9</v>
       </c>
       <c r="F319" s="9" t="s">
         <v>28</v>
@@ -9311,7 +9311,7 @@
         <v>27</v>
       </c>
       <c r="E320" s="11">
-        <v>9</v>
+        <v>14</v>
       </c>
       <c r="F320" s="9" t="s">
         <v>28</v>
@@ -9334,7 +9334,7 @@
         <v>27</v>
       </c>
       <c r="E321" s="11">
-        <v>14</v>
+        <v>26</v>
       </c>
       <c r="F321" s="9" t="s">
         <v>28</v>
@@ -9357,7 +9357,7 @@
         <v>27</v>
       </c>
       <c r="E322" s="11">
-        <v>19</v>
+        <v>21</v>
       </c>
       <c r="F322" s="9" t="s">
         <v>28</v>
@@ -9380,7 +9380,7 @@
         <v>27</v>
       </c>
       <c r="E323" s="11">
-        <v>19</v>
+        <v>29</v>
       </c>
       <c r="F323" s="9" t="s">
         <v>28</v>
@@ -9403,7 +9403,7 @@
         <v>27</v>
       </c>
       <c r="E324" s="11">
-        <v>12</v>
+        <v>18</v>
       </c>
       <c r="F324" s="9" t="s">
         <v>28</v>
@@ -9426,7 +9426,7 @@
         <v>27</v>
       </c>
       <c r="E325" s="11">
-        <v>31</v>
+        <v>17</v>
       </c>
       <c r="F325" s="9" t="s">
         <v>28</v>
@@ -9449,7 +9449,7 @@
         <v>27</v>
       </c>
       <c r="E326" s="11">
-        <v>30</v>
+        <v>19</v>
       </c>
       <c r="F326" s="9" t="s">
         <v>28</v>
@@ -9472,7 +9472,7 @@
         <v>27</v>
       </c>
       <c r="E327" s="11">
-        <v>18</v>
+        <v>8</v>
       </c>
       <c r="F327" s="9" t="s">
         <v>28</v>
@@ -9495,7 +9495,7 @@
         <v>27</v>
       </c>
       <c r="E328" s="11">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="F328" s="9" t="s">
         <v>28</v>
@@ -9518,7 +9518,7 @@
         <v>27</v>
       </c>
       <c r="E329" s="11">
-        <v>19</v>
+        <v>26</v>
       </c>
       <c r="F329" s="9" t="s">
         <v>28</v>
@@ -9541,7 +9541,7 @@
         <v>27</v>
       </c>
       <c r="E330" s="11">
-        <v>15</v>
+        <v>11</v>
       </c>
       <c r="F330" s="9" t="s">
         <v>28</v>
@@ -9564,7 +9564,7 @@
         <v>27</v>
       </c>
       <c r="E331" s="11">
-        <v>13</v>
+        <v>24</v>
       </c>
       <c r="F331" s="9" t="s">
         <v>28</v>
@@ -9587,7 +9587,7 @@
         <v>27</v>
       </c>
       <c r="E332" s="11">
-        <v>16</v>
+        <v>11</v>
       </c>
       <c r="F332" s="9" t="s">
         <v>28</v>
@@ -9610,7 +9610,7 @@
         <v>27</v>
       </c>
       <c r="E333" s="11">
-        <v>10</v>
+        <v>30</v>
       </c>
       <c r="F333" s="9" t="s">
         <v>28</v>
@@ -9656,7 +9656,7 @@
         <v>27</v>
       </c>
       <c r="E335" s="11">
-        <v>31</v>
+        <v>19</v>
       </c>
       <c r="F335" s="9" t="s">
         <v>28</v>
@@ -9679,7 +9679,7 @@
         <v>27</v>
       </c>
       <c r="E336" s="11">
-        <v>10</v>
+        <v>14</v>
       </c>
       <c r="F336" s="9" t="s">
         <v>28</v>
@@ -9702,7 +9702,7 @@
         <v>27</v>
       </c>
       <c r="E337" s="11">
-        <v>26</v>
+        <v>12</v>
       </c>
       <c r="F337" s="9" t="s">
         <v>28</v>
@@ -9725,7 +9725,7 @@
         <v>27</v>
       </c>
       <c r="E338" s="11">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="F338" s="9" t="s">
         <v>28</v>
@@ -9748,7 +9748,7 @@
         <v>27</v>
       </c>
       <c r="E339" s="11">
-        <v>24</v>
+        <v>30</v>
       </c>
       <c r="F339" s="9" t="s">
         <v>28</v>
@@ -9771,7 +9771,7 @@
         <v>27</v>
       </c>
       <c r="E340" s="11">
-        <v>12</v>
+        <v>20</v>
       </c>
       <c r="F340" s="9" t="s">
         <v>28</v>
@@ -9794,7 +9794,7 @@
         <v>27</v>
       </c>
       <c r="E341" s="11">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="F341" s="9" t="s">
         <v>28</v>
@@ -9817,7 +9817,7 @@
         <v>27</v>
       </c>
       <c r="E342" s="11">
-        <v>14</v>
+        <v>19</v>
       </c>
       <c r="F342" s="9" t="s">
         <v>28</v>
@@ -9840,7 +9840,7 @@
         <v>27</v>
       </c>
       <c r="E343" s="11">
-        <v>13</v>
+        <v>18</v>
       </c>
       <c r="F343" s="9" t="s">
         <v>28</v>
@@ -9863,7 +9863,7 @@
         <v>27</v>
       </c>
       <c r="E344" s="11">
-        <v>24</v>
+        <v>10</v>
       </c>
       <c r="F344" s="9" t="s">
         <v>28</v>
@@ -9886,7 +9886,7 @@
         <v>27</v>
       </c>
       <c r="E345" s="11">
-        <v>16</v>
+        <v>14</v>
       </c>
       <c r="F345" s="9" t="s">
         <v>28</v>
@@ -9909,7 +9909,7 @@
         <v>27</v>
       </c>
       <c r="E346" s="11">
-        <v>30</v>
+        <v>11</v>
       </c>
       <c r="F346" s="9" t="s">
         <v>28</v>
@@ -9932,7 +9932,7 @@
         <v>27</v>
       </c>
       <c r="E347" s="11">
-        <v>15</v>
+        <v>17</v>
       </c>
       <c r="F347" s="9" t="s">
         <v>28</v>
@@ -9955,7 +9955,7 @@
         <v>27</v>
       </c>
       <c r="E348" s="11">
-        <v>18</v>
+        <v>11</v>
       </c>
       <c r="F348" s="9" t="s">
         <v>28</v>
@@ -9978,7 +9978,7 @@
         <v>27</v>
       </c>
       <c r="E349" s="11">
-        <v>22</v>
+        <v>24</v>
       </c>
       <c r="F349" s="9" t="s">
         <v>28</v>
@@ -10001,7 +10001,7 @@
         <v>27</v>
       </c>
       <c r="E350" s="11">
-        <v>17</v>
+        <v>8</v>
       </c>
       <c r="F350" s="9" t="s">
         <v>28</v>
@@ -10024,7 +10024,7 @@
         <v>27</v>
       </c>
       <c r="E351" s="11">
-        <v>19</v>
+        <v>22</v>
       </c>
       <c r="F351" s="9" t="s">
         <v>28</v>
@@ -10070,7 +10070,7 @@
         <v>27</v>
       </c>
       <c r="E353" s="11">
-        <v>18</v>
+        <v>28</v>
       </c>
       <c r="F353" s="9" t="s">
         <v>28</v>
@@ -10093,7 +10093,7 @@
         <v>27</v>
       </c>
       <c r="E354" s="11">
-        <v>31</v>
+        <v>14</v>
       </c>
       <c r="F354" s="9" t="s">
         <v>28</v>
@@ -10116,7 +10116,7 @@
         <v>27</v>
       </c>
       <c r="E355" s="11">
-        <v>22</v>
+        <v>12</v>
       </c>
       <c r="F355" s="9" t="s">
         <v>28</v>
@@ -10139,7 +10139,7 @@
         <v>27</v>
       </c>
       <c r="E356" s="11">
-        <v>25</v>
+        <v>13</v>
       </c>
       <c r="F356" s="9" t="s">
         <v>28</v>
@@ -10162,7 +10162,7 @@
         <v>27</v>
       </c>
       <c r="E357" s="11">
-        <v>27</v>
+        <v>12</v>
       </c>
       <c r="F357" s="9" t="s">
         <v>28</v>
@@ -10185,7 +10185,7 @@
         <v>27</v>
       </c>
       <c r="E358" s="11">
-        <v>9</v>
+        <v>13</v>
       </c>
       <c r="F358" s="9" t="s">
         <v>28</v>
@@ -10208,7 +10208,7 @@
         <v>27</v>
       </c>
       <c r="E359" s="11">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="F359" s="9" t="s">
         <v>28</v>
@@ -10231,7 +10231,7 @@
         <v>27</v>
       </c>
       <c r="E360" s="11">
-        <v>13</v>
+        <v>8</v>
       </c>
       <c r="F360" s="9" t="s">
         <v>28</v>
@@ -10254,7 +10254,7 @@
         <v>27</v>
       </c>
       <c r="E361" s="11">
-        <v>14</v>
+        <v>16</v>
       </c>
       <c r="F361" s="9" t="s">
         <v>28</v>
@@ -10277,7 +10277,7 @@
         <v>27</v>
       </c>
       <c r="E362" s="11">
-        <v>15</v>
+        <v>30</v>
       </c>
       <c r="F362" s="9" t="s">
         <v>28</v>
@@ -10300,7 +10300,7 @@
         <v>27</v>
       </c>
       <c r="E363" s="11">
-        <v>15</v>
+        <v>27</v>
       </c>
       <c r="F363" s="9" t="s">
         <v>28</v>
@@ -10323,7 +10323,7 @@
         <v>27</v>
       </c>
       <c r="E364" s="11">
-        <v>26</v>
+        <v>12</v>
       </c>
       <c r="F364" s="9" t="s">
         <v>28</v>
@@ -10346,7 +10346,7 @@
         <v>27</v>
       </c>
       <c r="E365" s="11">
-        <v>26</v>
+        <v>13</v>
       </c>
       <c r="F365" s="9" t="s">
         <v>28</v>
@@ -10392,7 +10392,7 @@
         <v>27</v>
       </c>
       <c r="E367" s="11">
-        <v>18</v>
+        <v>13</v>
       </c>
       <c r="F367" s="9" t="s">
         <v>28</v>
@@ -10415,7 +10415,7 @@
         <v>27</v>
       </c>
       <c r="E368" s="11">
-        <v>12</v>
+        <v>19</v>
       </c>
       <c r="F368" s="9" t="s">
         <v>28</v>
@@ -10438,7 +10438,7 @@
         <v>27</v>
       </c>
       <c r="E369" s="11">
-        <v>26</v>
+        <v>23</v>
       </c>
       <c r="F369" s="9" t="s">
         <v>28</v>
@@ -10461,7 +10461,7 @@
         <v>27</v>
       </c>
       <c r="E370" s="11">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="F370" s="9" t="s">
         <v>28</v>
@@ -10484,7 +10484,7 @@
         <v>27</v>
       </c>
       <c r="E371" s="11">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="F371" s="9" t="s">
         <v>28</v>
@@ -10507,7 +10507,7 @@
         <v>27</v>
       </c>
       <c r="E372" s="11">
-        <v>25</v>
+        <v>10</v>
       </c>
       <c r="F372" s="9" t="s">
         <v>28</v>
@@ -10530,7 +10530,7 @@
         <v>27</v>
       </c>
       <c r="E373" s="11">
-        <v>23</v>
+        <v>21</v>
       </c>
       <c r="F373" s="9" t="s">
         <v>28</v>
@@ -10553,7 +10553,7 @@
         <v>27</v>
       </c>
       <c r="E374" s="11">
-        <v>21</v>
+        <v>10</v>
       </c>
       <c r="F374" s="9" t="s">
         <v>28</v>
@@ -10576,7 +10576,7 @@
         <v>27</v>
       </c>
       <c r="E375" s="11">
-        <v>29</v>
+        <v>23</v>
       </c>
       <c r="F375" s="9" t="s">
         <v>28</v>
@@ -10622,7 +10622,7 @@
         <v>27</v>
       </c>
       <c r="E377" s="11">
-        <v>25</v>
+        <v>8</v>
       </c>
       <c r="F377" s="9" t="s">
         <v>28</v>
@@ -10645,7 +10645,7 @@
         <v>27</v>
       </c>
       <c r="E378" s="11">
-        <v>22</v>
+        <v>13</v>
       </c>
       <c r="F378" s="9" t="s">
         <v>28</v>
@@ -10668,7 +10668,7 @@
         <v>27</v>
       </c>
       <c r="E379" s="11">
-        <v>30</v>
+        <v>20</v>
       </c>
       <c r="F379" s="9" t="s">
         <v>28</v>
@@ -10691,7 +10691,7 @@
         <v>27</v>
       </c>
       <c r="E380" s="11">
-        <v>23</v>
+        <v>16</v>
       </c>
       <c r="F380" s="9" t="s">
         <v>28</v>
@@ -10714,7 +10714,7 @@
         <v>27</v>
       </c>
       <c r="E381" s="11">
-        <v>18</v>
+        <v>8</v>
       </c>
       <c r="F381" s="9" t="s">
         <v>28</v>
@@ -10737,7 +10737,7 @@
         <v>27</v>
       </c>
       <c r="E382" s="11">
-        <v>26</v>
+        <v>15</v>
       </c>
       <c r="F382" s="9" t="s">
         <v>28</v>
@@ -10760,7 +10760,7 @@
         <v>27</v>
       </c>
       <c r="E383" s="11">
-        <v>17</v>
+        <v>21</v>
       </c>
       <c r="F383" s="9" t="s">
         <v>28</v>
@@ -10783,7 +10783,7 @@
         <v>27</v>
       </c>
       <c r="E384" s="11">
-        <v>16</v>
+        <v>11</v>
       </c>
       <c r="F384" s="9" t="s">
         <v>28</v>
@@ -10806,7 +10806,7 @@
         <v>27</v>
       </c>
       <c r="E385" s="11">
-        <v>29</v>
+        <v>11</v>
       </c>
       <c r="F385" s="9" t="s">
         <v>28</v>
@@ -10829,7 +10829,7 @@
         <v>27</v>
       </c>
       <c r="E386" s="11">
-        <v>17</v>
+        <v>27</v>
       </c>
       <c r="F386" s="9" t="s">
         <v>28</v>
@@ -10852,7 +10852,7 @@
         <v>27</v>
       </c>
       <c r="E387" s="11">
-        <v>20</v>
+        <v>16</v>
       </c>
       <c r="F387" s="9" t="s">
         <v>28</v>
@@ -10875,7 +10875,7 @@
         <v>27</v>
       </c>
       <c r="E388" s="11">
-        <v>12</v>
+        <v>29</v>
       </c>
       <c r="F388" s="9" t="s">
         <v>28</v>
@@ -10898,7 +10898,7 @@
         <v>27</v>
       </c>
       <c r="E389" s="11">
-        <v>18</v>
+        <v>25</v>
       </c>
       <c r="F389" s="9" t="s">
         <v>28</v>
@@ -10921,7 +10921,7 @@
         <v>27</v>
       </c>
       <c r="E390" s="11">
-        <v>16</v>
+        <v>19</v>
       </c>
       <c r="F390" s="9" t="s">
         <v>28</v>
@@ -10944,7 +10944,7 @@
         <v>27</v>
       </c>
       <c r="E391" s="11">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="F391" s="9" t="s">
         <v>28</v>
@@ -10967,7 +10967,7 @@
         <v>27</v>
       </c>
       <c r="E392" s="11">
-        <v>14</v>
+        <v>25</v>
       </c>
       <c r="F392" s="9" t="s">
         <v>28</v>
@@ -10990,7 +10990,7 @@
         <v>27</v>
       </c>
       <c r="E393" s="11">
-        <v>18</v>
+        <v>25</v>
       </c>
       <c r="F393" s="9" t="s">
         <v>28</v>
@@ -11013,7 +11013,7 @@
         <v>27</v>
       </c>
       <c r="E394" s="11">
-        <v>15</v>
+        <v>30</v>
       </c>
       <c r="F394" s="9" t="s">
         <v>28</v>
@@ -11036,7 +11036,7 @@
         <v>27</v>
       </c>
       <c r="E395" s="11">
-        <v>12</v>
+        <v>8</v>
       </c>
       <c r="F395" s="9" t="s">
         <v>28</v>
@@ -11082,7 +11082,7 @@
         <v>27</v>
       </c>
       <c r="E397" s="11">
-        <v>26</v>
+        <v>20</v>
       </c>
       <c r="F397" s="9" t="s">
         <v>28</v>
@@ -11105,7 +11105,7 @@
         <v>27</v>
       </c>
       <c r="E398" s="11">
-        <v>30</v>
+        <v>25</v>
       </c>
       <c r="F398" s="9" t="s">
         <v>28</v>
@@ -11128,7 +11128,7 @@
         <v>27</v>
       </c>
       <c r="E399" s="11">
-        <v>21</v>
+        <v>25</v>
       </c>
       <c r="F399" s="9" t="s">
         <v>28</v>
@@ -11151,7 +11151,7 @@
         <v>27</v>
       </c>
       <c r="E400" s="11">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="F400" s="9" t="s">
         <v>28</v>
@@ -11174,7 +11174,7 @@
         <v>27</v>
       </c>
       <c r="E401" s="11">
-        <v>19</v>
+        <v>27</v>
       </c>
       <c r="F401" s="9" t="s">
         <v>28</v>

</xml_diff>

<commit_message>
feat(admin): configure case-insensitive LK-<USERNAME>-2026 admin secret key verification in admin portal
</commit_message>
<xml_diff>
--- a/all-test-reports/selenium/selenium_e2e_test_report.xlsx
+++ b/all-test-reports/selenium/selenium_e2e_test_report.xlsx
@@ -35,7 +35,7 @@
     <t>Execution Date</t>
   </si>
   <si>
-    <t>28/7/2026, 11:43:44 am</t>
+    <t>28/7/2026, 11:57:28 am</t>
   </si>
   <si>
     <t>Browser / Mode</t>
@@ -98,7 +98,7 @@
     <t>PASS</t>
   </si>
   <si>
-    <t>11:43:44 am</t>
+    <t>11:57:28 am</t>
   </si>
   <si>
     <t>N/A</t>
@@ -1997,7 +1997,7 @@
         <v>27</v>
       </c>
       <c r="E2" s="11">
-        <v>19</v>
+        <v>17</v>
       </c>
       <c r="F2" s="9" t="s">
         <v>28</v>
@@ -2020,7 +2020,7 @@
         <v>27</v>
       </c>
       <c r="E3" s="11">
-        <v>22</v>
+        <v>12</v>
       </c>
       <c r="F3" s="9" t="s">
         <v>28</v>
@@ -2043,7 +2043,7 @@
         <v>27</v>
       </c>
       <c r="E4" s="11">
-        <v>26</v>
+        <v>18</v>
       </c>
       <c r="F4" s="9" t="s">
         <v>28</v>
@@ -2066,7 +2066,7 @@
         <v>27</v>
       </c>
       <c r="E5" s="11">
-        <v>18</v>
+        <v>8</v>
       </c>
       <c r="F5" s="9" t="s">
         <v>28</v>
@@ -2089,7 +2089,7 @@
         <v>27</v>
       </c>
       <c r="E6" s="11">
-        <v>22</v>
+        <v>17</v>
       </c>
       <c r="F6" s="9" t="s">
         <v>28</v>
@@ -2112,7 +2112,7 @@
         <v>27</v>
       </c>
       <c r="E7" s="11">
-        <v>14</v>
+        <v>20</v>
       </c>
       <c r="F7" s="9" t="s">
         <v>28</v>
@@ -2135,7 +2135,7 @@
         <v>27</v>
       </c>
       <c r="E8" s="11">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="F8" s="9" t="s">
         <v>28</v>
@@ -2158,7 +2158,7 @@
         <v>27</v>
       </c>
       <c r="E9" s="11">
-        <v>13</v>
+        <v>21</v>
       </c>
       <c r="F9" s="9" t="s">
         <v>28</v>
@@ -2181,7 +2181,7 @@
         <v>27</v>
       </c>
       <c r="E10" s="11">
-        <v>12</v>
+        <v>16</v>
       </c>
       <c r="F10" s="9" t="s">
         <v>28</v>
@@ -2204,7 +2204,7 @@
         <v>27</v>
       </c>
       <c r="E11" s="11">
-        <v>11</v>
+        <v>28</v>
       </c>
       <c r="F11" s="9" t="s">
         <v>28</v>
@@ -2227,7 +2227,7 @@
         <v>27</v>
       </c>
       <c r="E12" s="11">
-        <v>29</v>
+        <v>10</v>
       </c>
       <c r="F12" s="9" t="s">
         <v>28</v>
@@ -2250,7 +2250,7 @@
         <v>27</v>
       </c>
       <c r="E13" s="11">
-        <v>20</v>
+        <v>8</v>
       </c>
       <c r="F13" s="9" t="s">
         <v>28</v>
@@ -2273,7 +2273,7 @@
         <v>27</v>
       </c>
       <c r="E14" s="11">
-        <v>30</v>
+        <v>21</v>
       </c>
       <c r="F14" s="9" t="s">
         <v>28</v>
@@ -2296,7 +2296,7 @@
         <v>27</v>
       </c>
       <c r="E15" s="11">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="F15" s="9" t="s">
         <v>28</v>
@@ -2319,7 +2319,7 @@
         <v>27</v>
       </c>
       <c r="E16" s="11">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="F16" s="9" t="s">
         <v>28</v>
@@ -2342,7 +2342,7 @@
         <v>27</v>
       </c>
       <c r="E17" s="11">
-        <v>27</v>
+        <v>24</v>
       </c>
       <c r="F17" s="9" t="s">
         <v>28</v>
@@ -2365,7 +2365,7 @@
         <v>27</v>
       </c>
       <c r="E18" s="11">
-        <v>15</v>
+        <v>9</v>
       </c>
       <c r="F18" s="9" t="s">
         <v>28</v>
@@ -2388,7 +2388,7 @@
         <v>27</v>
       </c>
       <c r="E19" s="11">
-        <v>9</v>
+        <v>15</v>
       </c>
       <c r="F19" s="9" t="s">
         <v>28</v>
@@ -2411,7 +2411,7 @@
         <v>27</v>
       </c>
       <c r="E20" s="11">
-        <v>23</v>
+        <v>25</v>
       </c>
       <c r="F20" s="9" t="s">
         <v>28</v>
@@ -2434,7 +2434,7 @@
         <v>27</v>
       </c>
       <c r="E21" s="11">
-        <v>13</v>
+        <v>17</v>
       </c>
       <c r="F21" s="9" t="s">
         <v>28</v>
@@ -2457,7 +2457,7 @@
         <v>27</v>
       </c>
       <c r="E22" s="11">
-        <v>8</v>
+        <v>13</v>
       </c>
       <c r="F22" s="9" t="s">
         <v>28</v>
@@ -2480,7 +2480,7 @@
         <v>27</v>
       </c>
       <c r="E23" s="11">
-        <v>8</v>
+        <v>26</v>
       </c>
       <c r="F23" s="9" t="s">
         <v>28</v>
@@ -2503,7 +2503,7 @@
         <v>27</v>
       </c>
       <c r="E24" s="11">
-        <v>10</v>
+        <v>14</v>
       </c>
       <c r="F24" s="9" t="s">
         <v>28</v>
@@ -2526,7 +2526,7 @@
         <v>27</v>
       </c>
       <c r="E25" s="11">
-        <v>8</v>
+        <v>27</v>
       </c>
       <c r="F25" s="9" t="s">
         <v>28</v>
@@ -2549,7 +2549,7 @@
         <v>27</v>
       </c>
       <c r="E26" s="11">
-        <v>13</v>
+        <v>18</v>
       </c>
       <c r="F26" s="9" t="s">
         <v>28</v>
@@ -2572,7 +2572,7 @@
         <v>27</v>
       </c>
       <c r="E27" s="11">
-        <v>24</v>
+        <v>12</v>
       </c>
       <c r="F27" s="9" t="s">
         <v>28</v>
@@ -2595,7 +2595,7 @@
         <v>27</v>
       </c>
       <c r="E28" s="11">
-        <v>23</v>
+        <v>17</v>
       </c>
       <c r="F28" s="9" t="s">
         <v>28</v>
@@ -2618,7 +2618,7 @@
         <v>27</v>
       </c>
       <c r="E29" s="11">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="F29" s="9" t="s">
         <v>28</v>
@@ -2641,7 +2641,7 @@
         <v>27</v>
       </c>
       <c r="E30" s="11">
-        <v>16</v>
+        <v>9</v>
       </c>
       <c r="F30" s="9" t="s">
         <v>28</v>
@@ -2664,7 +2664,7 @@
         <v>27</v>
       </c>
       <c r="E31" s="11">
-        <v>12</v>
+        <v>28</v>
       </c>
       <c r="F31" s="9" t="s">
         <v>28</v>
@@ -2687,7 +2687,7 @@
         <v>27</v>
       </c>
       <c r="E32" s="11">
-        <v>19</v>
+        <v>11</v>
       </c>
       <c r="F32" s="9" t="s">
         <v>28</v>
@@ -2710,7 +2710,7 @@
         <v>27</v>
       </c>
       <c r="E33" s="11">
-        <v>25</v>
+        <v>8</v>
       </c>
       <c r="F33" s="9" t="s">
         <v>28</v>
@@ -2733,7 +2733,7 @@
         <v>27</v>
       </c>
       <c r="E34" s="11">
-        <v>8</v>
+        <v>23</v>
       </c>
       <c r="F34" s="9" t="s">
         <v>28</v>
@@ -2756,7 +2756,7 @@
         <v>27</v>
       </c>
       <c r="E35" s="11">
-        <v>26</v>
+        <v>31</v>
       </c>
       <c r="F35" s="9" t="s">
         <v>28</v>
@@ -2779,7 +2779,7 @@
         <v>27</v>
       </c>
       <c r="E36" s="11">
-        <v>11</v>
+        <v>20</v>
       </c>
       <c r="F36" s="9" t="s">
         <v>28</v>
@@ -2802,7 +2802,7 @@
         <v>27</v>
       </c>
       <c r="E37" s="11">
-        <v>13</v>
+        <v>23</v>
       </c>
       <c r="F37" s="9" t="s">
         <v>28</v>
@@ -2825,7 +2825,7 @@
         <v>27</v>
       </c>
       <c r="E38" s="11">
-        <v>15</v>
+        <v>8</v>
       </c>
       <c r="F38" s="9" t="s">
         <v>28</v>
@@ -2848,7 +2848,7 @@
         <v>27</v>
       </c>
       <c r="E39" s="11">
-        <v>21</v>
+        <v>31</v>
       </c>
       <c r="F39" s="9" t="s">
         <v>28</v>
@@ -2871,7 +2871,7 @@
         <v>27</v>
       </c>
       <c r="E40" s="11">
-        <v>30</v>
+        <v>10</v>
       </c>
       <c r="F40" s="9" t="s">
         <v>28</v>
@@ -2894,7 +2894,7 @@
         <v>27</v>
       </c>
       <c r="E41" s="11">
-        <v>30</v>
+        <v>14</v>
       </c>
       <c r="F41" s="9" t="s">
         <v>28</v>
@@ -2917,7 +2917,7 @@
         <v>27</v>
       </c>
       <c r="E42" s="11">
-        <v>25</v>
+        <v>10</v>
       </c>
       <c r="F42" s="9" t="s">
         <v>28</v>
@@ -2940,7 +2940,7 @@
         <v>27</v>
       </c>
       <c r="E43" s="11">
-        <v>21</v>
+        <v>23</v>
       </c>
       <c r="F43" s="9" t="s">
         <v>28</v>
@@ -2963,7 +2963,7 @@
         <v>27</v>
       </c>
       <c r="E44" s="11">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="F44" s="9" t="s">
         <v>28</v>
@@ -2986,7 +2986,7 @@
         <v>27</v>
       </c>
       <c r="E45" s="11">
-        <v>30</v>
+        <v>28</v>
       </c>
       <c r="F45" s="9" t="s">
         <v>28</v>
@@ -3009,7 +3009,7 @@
         <v>27</v>
       </c>
       <c r="E46" s="11">
-        <v>31</v>
+        <v>26</v>
       </c>
       <c r="F46" s="9" t="s">
         <v>28</v>
@@ -3032,7 +3032,7 @@
         <v>27</v>
       </c>
       <c r="E47" s="11">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="F47" s="9" t="s">
         <v>28</v>
@@ -3055,7 +3055,7 @@
         <v>27</v>
       </c>
       <c r="E48" s="11">
-        <v>31</v>
+        <v>23</v>
       </c>
       <c r="F48" s="9" t="s">
         <v>28</v>
@@ -3078,7 +3078,7 @@
         <v>27</v>
       </c>
       <c r="E49" s="11">
-        <v>20</v>
+        <v>30</v>
       </c>
       <c r="F49" s="9" t="s">
         <v>28</v>
@@ -3101,7 +3101,7 @@
         <v>27</v>
       </c>
       <c r="E50" s="11">
-        <v>15</v>
+        <v>19</v>
       </c>
       <c r="F50" s="9" t="s">
         <v>28</v>
@@ -3124,7 +3124,7 @@
         <v>27</v>
       </c>
       <c r="E51" s="11">
-        <v>14</v>
+        <v>29</v>
       </c>
       <c r="F51" s="9" t="s">
         <v>28</v>
@@ -3147,7 +3147,7 @@
         <v>27</v>
       </c>
       <c r="E52" s="11">
-        <v>19</v>
+        <v>13</v>
       </c>
       <c r="F52" s="9" t="s">
         <v>28</v>
@@ -3170,7 +3170,7 @@
         <v>27</v>
       </c>
       <c r="E53" s="11">
-        <v>13</v>
+        <v>27</v>
       </c>
       <c r="F53" s="9" t="s">
         <v>28</v>
@@ -3193,7 +3193,7 @@
         <v>27</v>
       </c>
       <c r="E54" s="11">
-        <v>9</v>
+        <v>24</v>
       </c>
       <c r="F54" s="9" t="s">
         <v>28</v>
@@ -3216,7 +3216,7 @@
         <v>27</v>
       </c>
       <c r="E55" s="11">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="F55" s="9" t="s">
         <v>28</v>
@@ -3239,7 +3239,7 @@
         <v>27</v>
       </c>
       <c r="E56" s="11">
-        <v>20</v>
+        <v>9</v>
       </c>
       <c r="F56" s="9" t="s">
         <v>28</v>
@@ -3262,7 +3262,7 @@
         <v>27</v>
       </c>
       <c r="E57" s="11">
-        <v>23</v>
+        <v>30</v>
       </c>
       <c r="F57" s="9" t="s">
         <v>28</v>
@@ -3285,7 +3285,7 @@
         <v>27</v>
       </c>
       <c r="E58" s="11">
-        <v>16</v>
+        <v>10</v>
       </c>
       <c r="F58" s="9" t="s">
         <v>28</v>
@@ -3308,7 +3308,7 @@
         <v>27</v>
       </c>
       <c r="E59" s="11">
-        <v>15</v>
+        <v>24</v>
       </c>
       <c r="F59" s="9" t="s">
         <v>28</v>
@@ -3331,7 +3331,7 @@
         <v>27</v>
       </c>
       <c r="E60" s="11">
-        <v>8</v>
+        <v>18</v>
       </c>
       <c r="F60" s="9" t="s">
         <v>28</v>
@@ -3354,7 +3354,7 @@
         <v>27</v>
       </c>
       <c r="E61" s="11">
-        <v>16</v>
+        <v>18</v>
       </c>
       <c r="F61" s="9" t="s">
         <v>28</v>
@@ -3377,7 +3377,7 @@
         <v>27</v>
       </c>
       <c r="E62" s="11">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="F62" s="9" t="s">
         <v>28</v>
@@ -3400,7 +3400,7 @@
         <v>27</v>
       </c>
       <c r="E63" s="11">
-        <v>16</v>
+        <v>8</v>
       </c>
       <c r="F63" s="9" t="s">
         <v>28</v>
@@ -3423,7 +3423,7 @@
         <v>27</v>
       </c>
       <c r="E64" s="11">
-        <v>19</v>
+        <v>23</v>
       </c>
       <c r="F64" s="9" t="s">
         <v>28</v>
@@ -3446,7 +3446,7 @@
         <v>27</v>
       </c>
       <c r="E65" s="11">
-        <v>29</v>
+        <v>18</v>
       </c>
       <c r="F65" s="9" t="s">
         <v>28</v>
@@ -3469,7 +3469,7 @@
         <v>27</v>
       </c>
       <c r="E66" s="11">
-        <v>19</v>
+        <v>12</v>
       </c>
       <c r="F66" s="9" t="s">
         <v>28</v>
@@ -3492,7 +3492,7 @@
         <v>27</v>
       </c>
       <c r="E67" s="11">
-        <v>24</v>
+        <v>29</v>
       </c>
       <c r="F67" s="9" t="s">
         <v>28</v>
@@ -3515,7 +3515,7 @@
         <v>27</v>
       </c>
       <c r="E68" s="11">
-        <v>27</v>
+        <v>13</v>
       </c>
       <c r="F68" s="9" t="s">
         <v>28</v>
@@ -3538,7 +3538,7 @@
         <v>27</v>
       </c>
       <c r="E69" s="11">
-        <v>28</v>
+        <v>24</v>
       </c>
       <c r="F69" s="9" t="s">
         <v>28</v>
@@ -3561,7 +3561,7 @@
         <v>27</v>
       </c>
       <c r="E70" s="11">
-        <v>10</v>
+        <v>28</v>
       </c>
       <c r="F70" s="9" t="s">
         <v>28</v>
@@ -3584,7 +3584,7 @@
         <v>27</v>
       </c>
       <c r="E71" s="11">
-        <v>31</v>
+        <v>16</v>
       </c>
       <c r="F71" s="9" t="s">
         <v>28</v>
@@ -3607,7 +3607,7 @@
         <v>27</v>
       </c>
       <c r="E72" s="11">
-        <v>28</v>
+        <v>22</v>
       </c>
       <c r="F72" s="9" t="s">
         <v>28</v>
@@ -3630,7 +3630,7 @@
         <v>27</v>
       </c>
       <c r="E73" s="11">
-        <v>16</v>
+        <v>18</v>
       </c>
       <c r="F73" s="9" t="s">
         <v>28</v>
@@ -3653,7 +3653,7 @@
         <v>27</v>
       </c>
       <c r="E74" s="11">
-        <v>24</v>
+        <v>10</v>
       </c>
       <c r="F74" s="9" t="s">
         <v>28</v>
@@ -3676,7 +3676,7 @@
         <v>27</v>
       </c>
       <c r="E75" s="11">
-        <v>12</v>
+        <v>15</v>
       </c>
       <c r="F75" s="9" t="s">
         <v>28</v>
@@ -3699,7 +3699,7 @@
         <v>27</v>
       </c>
       <c r="E76" s="11">
-        <v>30</v>
+        <v>28</v>
       </c>
       <c r="F76" s="9" t="s">
         <v>28</v>
@@ -3745,7 +3745,7 @@
         <v>27</v>
       </c>
       <c r="E78" s="11">
-        <v>20</v>
+        <v>10</v>
       </c>
       <c r="F78" s="9" t="s">
         <v>28</v>
@@ -3768,7 +3768,7 @@
         <v>27</v>
       </c>
       <c r="E79" s="11">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="F79" s="9" t="s">
         <v>28</v>
@@ -3791,7 +3791,7 @@
         <v>27</v>
       </c>
       <c r="E80" s="11">
-        <v>14</v>
+        <v>19</v>
       </c>
       <c r="F80" s="9" t="s">
         <v>28</v>
@@ -3814,7 +3814,7 @@
         <v>27</v>
       </c>
       <c r="E81" s="11">
-        <v>22</v>
+        <v>31</v>
       </c>
       <c r="F81" s="9" t="s">
         <v>28</v>
@@ -3837,7 +3837,7 @@
         <v>27</v>
       </c>
       <c r="E82" s="11">
-        <v>23</v>
+        <v>21</v>
       </c>
       <c r="F82" s="9" t="s">
         <v>28</v>
@@ -3860,7 +3860,7 @@
         <v>27</v>
       </c>
       <c r="E83" s="11">
-        <v>14</v>
+        <v>22</v>
       </c>
       <c r="F83" s="9" t="s">
         <v>28</v>
@@ -3883,7 +3883,7 @@
         <v>27</v>
       </c>
       <c r="E84" s="11">
-        <v>18</v>
+        <v>26</v>
       </c>
       <c r="F84" s="9" t="s">
         <v>28</v>
@@ -3906,7 +3906,7 @@
         <v>27</v>
       </c>
       <c r="E85" s="11">
-        <v>29</v>
+        <v>17</v>
       </c>
       <c r="F85" s="9" t="s">
         <v>28</v>
@@ -3929,7 +3929,7 @@
         <v>27</v>
       </c>
       <c r="E86" s="11">
-        <v>21</v>
+        <v>8</v>
       </c>
       <c r="F86" s="9" t="s">
         <v>28</v>
@@ -3952,7 +3952,7 @@
         <v>27</v>
       </c>
       <c r="E87" s="11">
-        <v>31</v>
+        <v>27</v>
       </c>
       <c r="F87" s="9" t="s">
         <v>28</v>
@@ -3975,7 +3975,7 @@
         <v>27</v>
       </c>
       <c r="E88" s="11">
-        <v>15</v>
+        <v>24</v>
       </c>
       <c r="F88" s="9" t="s">
         <v>28</v>
@@ -3998,7 +3998,7 @@
         <v>27</v>
       </c>
       <c r="E89" s="11">
-        <v>12</v>
+        <v>23</v>
       </c>
       <c r="F89" s="9" t="s">
         <v>28</v>
@@ -4021,7 +4021,7 @@
         <v>27</v>
       </c>
       <c r="E90" s="11">
-        <v>14</v>
+        <v>24</v>
       </c>
       <c r="F90" s="9" t="s">
         <v>28</v>
@@ -4044,7 +4044,7 @@
         <v>27</v>
       </c>
       <c r="E91" s="11">
-        <v>18</v>
+        <v>15</v>
       </c>
       <c r="F91" s="9" t="s">
         <v>28</v>
@@ -4067,7 +4067,7 @@
         <v>27</v>
       </c>
       <c r="E92" s="11">
-        <v>21</v>
+        <v>24</v>
       </c>
       <c r="F92" s="9" t="s">
         <v>28</v>
@@ -4090,7 +4090,7 @@
         <v>27</v>
       </c>
       <c r="E93" s="11">
-        <v>24</v>
+        <v>14</v>
       </c>
       <c r="F93" s="9" t="s">
         <v>28</v>
@@ -4113,7 +4113,7 @@
         <v>27</v>
       </c>
       <c r="E94" s="11">
-        <v>31</v>
+        <v>29</v>
       </c>
       <c r="F94" s="9" t="s">
         <v>28</v>
@@ -4136,7 +4136,7 @@
         <v>27</v>
       </c>
       <c r="E95" s="11">
-        <v>19</v>
+        <v>26</v>
       </c>
       <c r="F95" s="9" t="s">
         <v>28</v>
@@ -4159,7 +4159,7 @@
         <v>27</v>
       </c>
       <c r="E96" s="11">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="F96" s="9" t="s">
         <v>28</v>
@@ -4182,7 +4182,7 @@
         <v>27</v>
       </c>
       <c r="E97" s="11">
-        <v>25</v>
+        <v>16</v>
       </c>
       <c r="F97" s="9" t="s">
         <v>28</v>
@@ -4205,7 +4205,7 @@
         <v>27</v>
       </c>
       <c r="E98" s="11">
-        <v>24</v>
+        <v>27</v>
       </c>
       <c r="F98" s="9" t="s">
         <v>28</v>
@@ -4228,7 +4228,7 @@
         <v>27</v>
       </c>
       <c r="E99" s="11">
-        <v>15</v>
+        <v>26</v>
       </c>
       <c r="F99" s="9" t="s">
         <v>28</v>
@@ -4251,7 +4251,7 @@
         <v>27</v>
       </c>
       <c r="E100" s="11">
-        <v>30</v>
+        <v>16</v>
       </c>
       <c r="F100" s="9" t="s">
         <v>28</v>
@@ -4274,7 +4274,7 @@
         <v>27</v>
       </c>
       <c r="E101" s="11">
-        <v>22</v>
+        <v>31</v>
       </c>
       <c r="F101" s="9" t="s">
         <v>28</v>
@@ -4297,7 +4297,7 @@
         <v>27</v>
       </c>
       <c r="E102" s="11">
-        <v>29</v>
+        <v>14</v>
       </c>
       <c r="F102" s="9" t="s">
         <v>28</v>
@@ -4320,7 +4320,7 @@
         <v>27</v>
       </c>
       <c r="E103" s="11">
-        <v>26</v>
+        <v>10</v>
       </c>
       <c r="F103" s="9" t="s">
         <v>28</v>
@@ -4343,7 +4343,7 @@
         <v>27</v>
       </c>
       <c r="E104" s="11">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="F104" s="9" t="s">
         <v>28</v>
@@ -4366,7 +4366,7 @@
         <v>27</v>
       </c>
       <c r="E105" s="11">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="F105" s="9" t="s">
         <v>28</v>
@@ -4412,7 +4412,7 @@
         <v>27</v>
       </c>
       <c r="E107" s="11">
-        <v>22</v>
+        <v>20</v>
       </c>
       <c r="F107" s="9" t="s">
         <v>28</v>
@@ -4458,7 +4458,7 @@
         <v>27</v>
       </c>
       <c r="E109" s="11">
-        <v>11</v>
+        <v>14</v>
       </c>
       <c r="F109" s="9" t="s">
         <v>28</v>
@@ -4481,7 +4481,7 @@
         <v>27</v>
       </c>
       <c r="E110" s="11">
-        <v>22</v>
+        <v>11</v>
       </c>
       <c r="F110" s="9" t="s">
         <v>28</v>
@@ -4504,7 +4504,7 @@
         <v>27</v>
       </c>
       <c r="E111" s="11">
-        <v>23</v>
+        <v>13</v>
       </c>
       <c r="F111" s="9" t="s">
         <v>28</v>
@@ -4527,7 +4527,7 @@
         <v>27</v>
       </c>
       <c r="E112" s="11">
-        <v>12</v>
+        <v>25</v>
       </c>
       <c r="F112" s="9" t="s">
         <v>28</v>
@@ -4550,7 +4550,7 @@
         <v>27</v>
       </c>
       <c r="E113" s="11">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="F113" s="9" t="s">
         <v>28</v>
@@ -4573,7 +4573,7 @@
         <v>27</v>
       </c>
       <c r="E114" s="11">
-        <v>12</v>
+        <v>9</v>
       </c>
       <c r="F114" s="9" t="s">
         <v>28</v>
@@ -4596,7 +4596,7 @@
         <v>27</v>
       </c>
       <c r="E115" s="11">
-        <v>12</v>
+        <v>31</v>
       </c>
       <c r="F115" s="9" t="s">
         <v>28</v>
@@ -4619,7 +4619,7 @@
         <v>27</v>
       </c>
       <c r="E116" s="11">
-        <v>25</v>
+        <v>19</v>
       </c>
       <c r="F116" s="9" t="s">
         <v>28</v>
@@ -4642,7 +4642,7 @@
         <v>27</v>
       </c>
       <c r="E117" s="11">
-        <v>15</v>
+        <v>30</v>
       </c>
       <c r="F117" s="9" t="s">
         <v>28</v>
@@ -4665,7 +4665,7 @@
         <v>27</v>
       </c>
       <c r="E118" s="11">
-        <v>13</v>
+        <v>10</v>
       </c>
       <c r="F118" s="9" t="s">
         <v>28</v>
@@ -4688,7 +4688,7 @@
         <v>27</v>
       </c>
       <c r="E119" s="11">
-        <v>28</v>
+        <v>19</v>
       </c>
       <c r="F119" s="9" t="s">
         <v>28</v>
@@ -4711,7 +4711,7 @@
         <v>27</v>
       </c>
       <c r="E120" s="11">
-        <v>15</v>
+        <v>13</v>
       </c>
       <c r="F120" s="9" t="s">
         <v>28</v>
@@ -4734,7 +4734,7 @@
         <v>27</v>
       </c>
       <c r="E121" s="11">
-        <v>19</v>
+        <v>22</v>
       </c>
       <c r="F121" s="9" t="s">
         <v>28</v>
@@ -4757,7 +4757,7 @@
         <v>27</v>
       </c>
       <c r="E122" s="11">
-        <v>19</v>
+        <v>13</v>
       </c>
       <c r="F122" s="9" t="s">
         <v>28</v>
@@ -4780,7 +4780,7 @@
         <v>27</v>
       </c>
       <c r="E123" s="11">
-        <v>26</v>
+        <v>24</v>
       </c>
       <c r="F123" s="9" t="s">
         <v>28</v>
@@ -4803,7 +4803,7 @@
         <v>27</v>
       </c>
       <c r="E124" s="11">
-        <v>18</v>
+        <v>9</v>
       </c>
       <c r="F124" s="9" t="s">
         <v>28</v>
@@ -4826,7 +4826,7 @@
         <v>27</v>
       </c>
       <c r="E125" s="11">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="F125" s="9" t="s">
         <v>28</v>
@@ -4849,7 +4849,7 @@
         <v>27</v>
       </c>
       <c r="E126" s="11">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="F126" s="9" t="s">
         <v>28</v>
@@ -4872,7 +4872,7 @@
         <v>27</v>
       </c>
       <c r="E127" s="11">
-        <v>18</v>
+        <v>23</v>
       </c>
       <c r="F127" s="9" t="s">
         <v>28</v>
@@ -4895,7 +4895,7 @@
         <v>27</v>
       </c>
       <c r="E128" s="11">
-        <v>19</v>
+        <v>31</v>
       </c>
       <c r="F128" s="9" t="s">
         <v>28</v>
@@ -4941,7 +4941,7 @@
         <v>27</v>
       </c>
       <c r="E130" s="11">
-        <v>9</v>
+        <v>15</v>
       </c>
       <c r="F130" s="9" t="s">
         <v>28</v>
@@ -4964,7 +4964,7 @@
         <v>27</v>
       </c>
       <c r="E131" s="11">
-        <v>19</v>
+        <v>29</v>
       </c>
       <c r="F131" s="9" t="s">
         <v>28</v>
@@ -4987,7 +4987,7 @@
         <v>27</v>
       </c>
       <c r="E132" s="11">
-        <v>14</v>
+        <v>23</v>
       </c>
       <c r="F132" s="9" t="s">
         <v>28</v>
@@ -5033,7 +5033,7 @@
         <v>27</v>
       </c>
       <c r="E134" s="11">
-        <v>29</v>
+        <v>31</v>
       </c>
       <c r="F134" s="9" t="s">
         <v>28</v>
@@ -5056,7 +5056,7 @@
         <v>27</v>
       </c>
       <c r="E135" s="11">
-        <v>9</v>
+        <v>19</v>
       </c>
       <c r="F135" s="9" t="s">
         <v>28</v>
@@ -5079,7 +5079,7 @@
         <v>27</v>
       </c>
       <c r="E136" s="11">
-        <v>19</v>
+        <v>30</v>
       </c>
       <c r="F136" s="9" t="s">
         <v>28</v>
@@ -5125,7 +5125,7 @@
         <v>27</v>
       </c>
       <c r="E138" s="11">
-        <v>30</v>
+        <v>16</v>
       </c>
       <c r="F138" s="9" t="s">
         <v>28</v>
@@ -5148,7 +5148,7 @@
         <v>27</v>
       </c>
       <c r="E139" s="11">
-        <v>12</v>
+        <v>21</v>
       </c>
       <c r="F139" s="9" t="s">
         <v>28</v>
@@ -5171,7 +5171,7 @@
         <v>27</v>
       </c>
       <c r="E140" s="11">
-        <v>21</v>
+        <v>19</v>
       </c>
       <c r="F140" s="9" t="s">
         <v>28</v>
@@ -5194,7 +5194,7 @@
         <v>27</v>
       </c>
       <c r="E141" s="11">
-        <v>15</v>
+        <v>23</v>
       </c>
       <c r="F141" s="9" t="s">
         <v>28</v>
@@ -5217,7 +5217,7 @@
         <v>27</v>
       </c>
       <c r="E142" s="11">
-        <v>23</v>
+        <v>11</v>
       </c>
       <c r="F142" s="9" t="s">
         <v>28</v>
@@ -5240,7 +5240,7 @@
         <v>27</v>
       </c>
       <c r="E143" s="11">
-        <v>24</v>
+        <v>22</v>
       </c>
       <c r="F143" s="9" t="s">
         <v>28</v>
@@ -5263,7 +5263,7 @@
         <v>27</v>
       </c>
       <c r="E144" s="11">
-        <v>14</v>
+        <v>11</v>
       </c>
       <c r="F144" s="9" t="s">
         <v>28</v>
@@ -5286,7 +5286,7 @@
         <v>27</v>
       </c>
       <c r="E145" s="11">
-        <v>19</v>
+        <v>8</v>
       </c>
       <c r="F145" s="9" t="s">
         <v>28</v>
@@ -5309,7 +5309,7 @@
         <v>27</v>
       </c>
       <c r="E146" s="11">
-        <v>8</v>
+        <v>30</v>
       </c>
       <c r="F146" s="9" t="s">
         <v>28</v>
@@ -5332,7 +5332,7 @@
         <v>27</v>
       </c>
       <c r="E147" s="11">
-        <v>24</v>
+        <v>20</v>
       </c>
       <c r="F147" s="9" t="s">
         <v>28</v>
@@ -5355,7 +5355,7 @@
         <v>27</v>
       </c>
       <c r="E148" s="11">
-        <v>9</v>
+        <v>28</v>
       </c>
       <c r="F148" s="9" t="s">
         <v>28</v>
@@ -5378,7 +5378,7 @@
         <v>27</v>
       </c>
       <c r="E149" s="11">
-        <v>26</v>
+        <v>19</v>
       </c>
       <c r="F149" s="9" t="s">
         <v>28</v>
@@ -5447,7 +5447,7 @@
         <v>27</v>
       </c>
       <c r="E152" s="11">
-        <v>10</v>
+        <v>19</v>
       </c>
       <c r="F152" s="9" t="s">
         <v>28</v>
@@ -5470,7 +5470,7 @@
         <v>27</v>
       </c>
       <c r="E153" s="11">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="F153" s="9" t="s">
         <v>28</v>
@@ -5493,7 +5493,7 @@
         <v>27</v>
       </c>
       <c r="E154" s="11">
-        <v>30</v>
+        <v>13</v>
       </c>
       <c r="F154" s="9" t="s">
         <v>28</v>
@@ -5516,7 +5516,7 @@
         <v>27</v>
       </c>
       <c r="E155" s="11">
-        <v>20</v>
+        <v>8</v>
       </c>
       <c r="F155" s="9" t="s">
         <v>28</v>
@@ -5539,7 +5539,7 @@
         <v>27</v>
       </c>
       <c r="E156" s="11">
-        <v>18</v>
+        <v>9</v>
       </c>
       <c r="F156" s="9" t="s">
         <v>28</v>
@@ -5562,7 +5562,7 @@
         <v>27</v>
       </c>
       <c r="E157" s="11">
-        <v>20</v>
+        <v>12</v>
       </c>
       <c r="F157" s="9" t="s">
         <v>28</v>
@@ -5585,7 +5585,7 @@
         <v>27</v>
       </c>
       <c r="E158" s="11">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="F158" s="9" t="s">
         <v>28</v>
@@ -5608,7 +5608,7 @@
         <v>27</v>
       </c>
       <c r="E159" s="11">
-        <v>31</v>
+        <v>19</v>
       </c>
       <c r="F159" s="9" t="s">
         <v>28</v>
@@ -5631,7 +5631,7 @@
         <v>27</v>
       </c>
       <c r="E160" s="11">
-        <v>13</v>
+        <v>24</v>
       </c>
       <c r="F160" s="9" t="s">
         <v>28</v>
@@ -5654,7 +5654,7 @@
         <v>27</v>
       </c>
       <c r="E161" s="11">
-        <v>24</v>
+        <v>29</v>
       </c>
       <c r="F161" s="9" t="s">
         <v>28</v>
@@ -5677,7 +5677,7 @@
         <v>27</v>
       </c>
       <c r="E162" s="11">
-        <v>15</v>
+        <v>9</v>
       </c>
       <c r="F162" s="9" t="s">
         <v>28</v>
@@ -5700,7 +5700,7 @@
         <v>27</v>
       </c>
       <c r="E163" s="11">
-        <v>28</v>
+        <v>23</v>
       </c>
       <c r="F163" s="9" t="s">
         <v>28</v>
@@ -5723,7 +5723,7 @@
         <v>27</v>
       </c>
       <c r="E164" s="11">
-        <v>28</v>
+        <v>17</v>
       </c>
       <c r="F164" s="9" t="s">
         <v>28</v>
@@ -5746,7 +5746,7 @@
         <v>27</v>
       </c>
       <c r="E165" s="11">
-        <v>10</v>
+        <v>24</v>
       </c>
       <c r="F165" s="9" t="s">
         <v>28</v>
@@ -5769,7 +5769,7 @@
         <v>27</v>
       </c>
       <c r="E166" s="11">
-        <v>22</v>
+        <v>30</v>
       </c>
       <c r="F166" s="9" t="s">
         <v>28</v>
@@ -5792,7 +5792,7 @@
         <v>27</v>
       </c>
       <c r="E167" s="11">
-        <v>27</v>
+        <v>16</v>
       </c>
       <c r="F167" s="9" t="s">
         <v>28</v>
@@ -5815,7 +5815,7 @@
         <v>27</v>
       </c>
       <c r="E168" s="11">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="F168" s="9" t="s">
         <v>28</v>
@@ -5838,7 +5838,7 @@
         <v>27</v>
       </c>
       <c r="E169" s="11">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="F169" s="9" t="s">
         <v>28</v>
@@ -5861,7 +5861,7 @@
         <v>27</v>
       </c>
       <c r="E170" s="11">
-        <v>26</v>
+        <v>21</v>
       </c>
       <c r="F170" s="9" t="s">
         <v>28</v>
@@ -5884,7 +5884,7 @@
         <v>27</v>
       </c>
       <c r="E171" s="11">
-        <v>22</v>
+        <v>11</v>
       </c>
       <c r="F171" s="9" t="s">
         <v>28</v>
@@ -5907,7 +5907,7 @@
         <v>27</v>
       </c>
       <c r="E172" s="11">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="F172" s="9" t="s">
         <v>28</v>
@@ -5930,7 +5930,7 @@
         <v>27</v>
       </c>
       <c r="E173" s="11">
-        <v>21</v>
+        <v>10</v>
       </c>
       <c r="F173" s="9" t="s">
         <v>28</v>
@@ -5953,7 +5953,7 @@
         <v>27</v>
       </c>
       <c r="E174" s="11">
-        <v>21</v>
+        <v>13</v>
       </c>
       <c r="F174" s="9" t="s">
         <v>28</v>
@@ -5976,7 +5976,7 @@
         <v>27</v>
       </c>
       <c r="E175" s="11">
-        <v>19</v>
+        <v>31</v>
       </c>
       <c r="F175" s="9" t="s">
         <v>28</v>
@@ -5999,7 +5999,7 @@
         <v>27</v>
       </c>
       <c r="E176" s="11">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="F176" s="9" t="s">
         <v>28</v>
@@ -6022,7 +6022,7 @@
         <v>27</v>
       </c>
       <c r="E177" s="11">
-        <v>9</v>
+        <v>26</v>
       </c>
       <c r="F177" s="9" t="s">
         <v>28</v>
@@ -6068,7 +6068,7 @@
         <v>27</v>
       </c>
       <c r="E179" s="11">
-        <v>20</v>
+        <v>15</v>
       </c>
       <c r="F179" s="9" t="s">
         <v>28</v>
@@ -6091,7 +6091,7 @@
         <v>27</v>
       </c>
       <c r="E180" s="11">
-        <v>19</v>
+        <v>25</v>
       </c>
       <c r="F180" s="9" t="s">
         <v>28</v>
@@ -6114,7 +6114,7 @@
         <v>27</v>
       </c>
       <c r="E181" s="11">
-        <v>24</v>
+        <v>28</v>
       </c>
       <c r="F181" s="9" t="s">
         <v>28</v>
@@ -6137,7 +6137,7 @@
         <v>27</v>
       </c>
       <c r="E182" s="11">
-        <v>13</v>
+        <v>20</v>
       </c>
       <c r="F182" s="9" t="s">
         <v>28</v>
@@ -6160,7 +6160,7 @@
         <v>27</v>
       </c>
       <c r="E183" s="11">
-        <v>25</v>
+        <v>31</v>
       </c>
       <c r="F183" s="9" t="s">
         <v>28</v>
@@ -6183,7 +6183,7 @@
         <v>27</v>
       </c>
       <c r="E184" s="11">
-        <v>16</v>
+        <v>26</v>
       </c>
       <c r="F184" s="9" t="s">
         <v>28</v>
@@ -6206,7 +6206,7 @@
         <v>27</v>
       </c>
       <c r="E185" s="11">
-        <v>27</v>
+        <v>31</v>
       </c>
       <c r="F185" s="9" t="s">
         <v>28</v>
@@ -6229,7 +6229,7 @@
         <v>27</v>
       </c>
       <c r="E186" s="11">
-        <v>24</v>
+        <v>19</v>
       </c>
       <c r="F186" s="9" t="s">
         <v>28</v>
@@ -6252,7 +6252,7 @@
         <v>27</v>
       </c>
       <c r="E187" s="11">
-        <v>18</v>
+        <v>15</v>
       </c>
       <c r="F187" s="9" t="s">
         <v>28</v>
@@ -6275,7 +6275,7 @@
         <v>27</v>
       </c>
       <c r="E188" s="11">
-        <v>15</v>
+        <v>27</v>
       </c>
       <c r="F188" s="9" t="s">
         <v>28</v>
@@ -6298,7 +6298,7 @@
         <v>27</v>
       </c>
       <c r="E189" s="11">
-        <v>24</v>
+        <v>17</v>
       </c>
       <c r="F189" s="9" t="s">
         <v>28</v>
@@ -6321,7 +6321,7 @@
         <v>27</v>
       </c>
       <c r="E190" s="11">
-        <v>27</v>
+        <v>16</v>
       </c>
       <c r="F190" s="9" t="s">
         <v>28</v>
@@ -6344,7 +6344,7 @@
         <v>27</v>
       </c>
       <c r="E191" s="11">
-        <v>24</v>
+        <v>28</v>
       </c>
       <c r="F191" s="9" t="s">
         <v>28</v>
@@ -6367,7 +6367,7 @@
         <v>27</v>
       </c>
       <c r="E192" s="11">
-        <v>27</v>
+        <v>21</v>
       </c>
       <c r="F192" s="9" t="s">
         <v>28</v>
@@ -6390,7 +6390,7 @@
         <v>27</v>
       </c>
       <c r="E193" s="11">
-        <v>31</v>
+        <v>10</v>
       </c>
       <c r="F193" s="9" t="s">
         <v>28</v>
@@ -6413,7 +6413,7 @@
         <v>27</v>
       </c>
       <c r="E194" s="11">
-        <v>10</v>
+        <v>14</v>
       </c>
       <c r="F194" s="9" t="s">
         <v>28</v>
@@ -6436,7 +6436,7 @@
         <v>27</v>
       </c>
       <c r="E195" s="11">
-        <v>24</v>
+        <v>15</v>
       </c>
       <c r="F195" s="9" t="s">
         <v>28</v>
@@ -6459,7 +6459,7 @@
         <v>27</v>
       </c>
       <c r="E196" s="11">
-        <v>12</v>
+        <v>31</v>
       </c>
       <c r="F196" s="9" t="s">
         <v>28</v>
@@ -6482,7 +6482,7 @@
         <v>27</v>
       </c>
       <c r="E197" s="11">
-        <v>17</v>
+        <v>27</v>
       </c>
       <c r="F197" s="9" t="s">
         <v>28</v>
@@ -6505,7 +6505,7 @@
         <v>27</v>
       </c>
       <c r="E198" s="11">
-        <v>18</v>
+        <v>10</v>
       </c>
       <c r="F198" s="9" t="s">
         <v>28</v>
@@ -6528,7 +6528,7 @@
         <v>27</v>
       </c>
       <c r="E199" s="11">
-        <v>29</v>
+        <v>16</v>
       </c>
       <c r="F199" s="9" t="s">
         <v>28</v>
@@ -6551,7 +6551,7 @@
         <v>27</v>
       </c>
       <c r="E200" s="11">
-        <v>27</v>
+        <v>15</v>
       </c>
       <c r="F200" s="9" t="s">
         <v>28</v>
@@ -6574,7 +6574,7 @@
         <v>27</v>
       </c>
       <c r="E201" s="11">
-        <v>28</v>
+        <v>20</v>
       </c>
       <c r="F201" s="9" t="s">
         <v>28</v>
@@ -6597,7 +6597,7 @@
         <v>27</v>
       </c>
       <c r="E202" s="11">
-        <v>18</v>
+        <v>16</v>
       </c>
       <c r="F202" s="9" t="s">
         <v>28</v>
@@ -6620,7 +6620,7 @@
         <v>27</v>
       </c>
       <c r="E203" s="11">
-        <v>29</v>
+        <v>27</v>
       </c>
       <c r="F203" s="9" t="s">
         <v>28</v>
@@ -6643,7 +6643,7 @@
         <v>27</v>
       </c>
       <c r="E204" s="11">
-        <v>13</v>
+        <v>30</v>
       </c>
       <c r="F204" s="9" t="s">
         <v>28</v>
@@ -6666,7 +6666,7 @@
         <v>27</v>
       </c>
       <c r="E205" s="11">
-        <v>17</v>
+        <v>14</v>
       </c>
       <c r="F205" s="9" t="s">
         <v>28</v>
@@ -6689,7 +6689,7 @@
         <v>27</v>
       </c>
       <c r="E206" s="11">
-        <v>25</v>
+        <v>20</v>
       </c>
       <c r="F206" s="9" t="s">
         <v>28</v>
@@ -6712,7 +6712,7 @@
         <v>27</v>
       </c>
       <c r="E207" s="11">
-        <v>20</v>
+        <v>13</v>
       </c>
       <c r="F207" s="9" t="s">
         <v>28</v>
@@ -6735,7 +6735,7 @@
         <v>27</v>
       </c>
       <c r="E208" s="11">
-        <v>9</v>
+        <v>15</v>
       </c>
       <c r="F208" s="9" t="s">
         <v>28</v>
@@ -6758,7 +6758,7 @@
         <v>27</v>
       </c>
       <c r="E209" s="11">
-        <v>18</v>
+        <v>15</v>
       </c>
       <c r="F209" s="9" t="s">
         <v>28</v>
@@ -6781,7 +6781,7 @@
         <v>27</v>
       </c>
       <c r="E210" s="11">
-        <v>17</v>
+        <v>21</v>
       </c>
       <c r="F210" s="9" t="s">
         <v>28</v>
@@ -6804,7 +6804,7 @@
         <v>27</v>
       </c>
       <c r="E211" s="11">
-        <v>11</v>
+        <v>16</v>
       </c>
       <c r="F211" s="9" t="s">
         <v>28</v>
@@ -6827,7 +6827,7 @@
         <v>27</v>
       </c>
       <c r="E212" s="11">
-        <v>26</v>
+        <v>31</v>
       </c>
       <c r="F212" s="9" t="s">
         <v>28</v>
@@ -6850,7 +6850,7 @@
         <v>27</v>
       </c>
       <c r="E213" s="11">
-        <v>19</v>
+        <v>10</v>
       </c>
       <c r="F213" s="9" t="s">
         <v>28</v>
@@ -6873,7 +6873,7 @@
         <v>27</v>
       </c>
       <c r="E214" s="11">
-        <v>31</v>
+        <v>8</v>
       </c>
       <c r="F214" s="9" t="s">
         <v>28</v>
@@ -6896,7 +6896,7 @@
         <v>27</v>
       </c>
       <c r="E215" s="11">
-        <v>15</v>
+        <v>21</v>
       </c>
       <c r="F215" s="9" t="s">
         <v>28</v>
@@ -6919,7 +6919,7 @@
         <v>27</v>
       </c>
       <c r="E216" s="11">
-        <v>11</v>
+        <v>19</v>
       </c>
       <c r="F216" s="9" t="s">
         <v>28</v>
@@ -6942,7 +6942,7 @@
         <v>27</v>
       </c>
       <c r="E217" s="11">
-        <v>16</v>
+        <v>11</v>
       </c>
       <c r="F217" s="9" t="s">
         <v>28</v>
@@ -6965,7 +6965,7 @@
         <v>27</v>
       </c>
       <c r="E218" s="11">
-        <v>20</v>
+        <v>23</v>
       </c>
       <c r="F218" s="9" t="s">
         <v>28</v>
@@ -6988,7 +6988,7 @@
         <v>27</v>
       </c>
       <c r="E219" s="11">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="F219" s="9" t="s">
         <v>28</v>
@@ -7011,7 +7011,7 @@
         <v>27</v>
       </c>
       <c r="E220" s="11">
-        <v>23</v>
+        <v>30</v>
       </c>
       <c r="F220" s="9" t="s">
         <v>28</v>
@@ -7057,7 +7057,7 @@
         <v>27</v>
       </c>
       <c r="E222" s="11">
-        <v>25</v>
+        <v>14</v>
       </c>
       <c r="F222" s="9" t="s">
         <v>28</v>
@@ -7080,7 +7080,7 @@
         <v>27</v>
       </c>
       <c r="E223" s="11">
-        <v>24</v>
+        <v>30</v>
       </c>
       <c r="F223" s="9" t="s">
         <v>28</v>
@@ -7103,7 +7103,7 @@
         <v>27</v>
       </c>
       <c r="E224" s="11">
-        <v>24</v>
+        <v>13</v>
       </c>
       <c r="F224" s="9" t="s">
         <v>28</v>
@@ -7126,7 +7126,7 @@
         <v>27</v>
       </c>
       <c r="E225" s="11">
-        <v>9</v>
+        <v>25</v>
       </c>
       <c r="F225" s="9" t="s">
         <v>28</v>
@@ -7149,7 +7149,7 @@
         <v>27</v>
       </c>
       <c r="E226" s="11">
-        <v>29</v>
+        <v>15</v>
       </c>
       <c r="F226" s="9" t="s">
         <v>28</v>
@@ -7172,7 +7172,7 @@
         <v>27</v>
       </c>
       <c r="E227" s="11">
-        <v>13</v>
+        <v>20</v>
       </c>
       <c r="F227" s="9" t="s">
         <v>28</v>
@@ -7195,7 +7195,7 @@
         <v>27</v>
       </c>
       <c r="E228" s="11">
-        <v>30</v>
+        <v>16</v>
       </c>
       <c r="F228" s="9" t="s">
         <v>28</v>
@@ -7218,7 +7218,7 @@
         <v>27</v>
       </c>
       <c r="E229" s="11">
-        <v>16</v>
+        <v>12</v>
       </c>
       <c r="F229" s="9" t="s">
         <v>28</v>
@@ -7241,7 +7241,7 @@
         <v>27</v>
       </c>
       <c r="E230" s="11">
-        <v>10</v>
+        <v>16</v>
       </c>
       <c r="F230" s="9" t="s">
         <v>28</v>
@@ -7264,7 +7264,7 @@
         <v>27</v>
       </c>
       <c r="E231" s="11">
-        <v>16</v>
+        <v>29</v>
       </c>
       <c r="F231" s="9" t="s">
         <v>28</v>
@@ -7287,7 +7287,7 @@
         <v>27</v>
       </c>
       <c r="E232" s="11">
-        <v>28</v>
+        <v>10</v>
       </c>
       <c r="F232" s="9" t="s">
         <v>28</v>
@@ -7310,7 +7310,7 @@
         <v>27</v>
       </c>
       <c r="E233" s="11">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="F233" s="9" t="s">
         <v>28</v>
@@ -7333,7 +7333,7 @@
         <v>27</v>
       </c>
       <c r="E234" s="11">
-        <v>13</v>
+        <v>17</v>
       </c>
       <c r="F234" s="9" t="s">
         <v>28</v>
@@ -7356,7 +7356,7 @@
         <v>27</v>
       </c>
       <c r="E235" s="11">
-        <v>24</v>
+        <v>29</v>
       </c>
       <c r="F235" s="9" t="s">
         <v>28</v>
@@ -7379,7 +7379,7 @@
         <v>27</v>
       </c>
       <c r="E236" s="11">
-        <v>10</v>
+        <v>22</v>
       </c>
       <c r="F236" s="9" t="s">
         <v>28</v>
@@ -7402,7 +7402,7 @@
         <v>27</v>
       </c>
       <c r="E237" s="11">
-        <v>13</v>
+        <v>18</v>
       </c>
       <c r="F237" s="9" t="s">
         <v>28</v>
@@ -7425,7 +7425,7 @@
         <v>27</v>
       </c>
       <c r="E238" s="11">
-        <v>17</v>
+        <v>10</v>
       </c>
       <c r="F238" s="9" t="s">
         <v>28</v>
@@ -7448,7 +7448,7 @@
         <v>27</v>
       </c>
       <c r="E239" s="11">
-        <v>26</v>
+        <v>11</v>
       </c>
       <c r="F239" s="9" t="s">
         <v>28</v>
@@ -7471,7 +7471,7 @@
         <v>27</v>
       </c>
       <c r="E240" s="11">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="F240" s="9" t="s">
         <v>28</v>
@@ -7494,7 +7494,7 @@
         <v>27</v>
       </c>
       <c r="E241" s="11">
-        <v>27</v>
+        <v>13</v>
       </c>
       <c r="F241" s="9" t="s">
         <v>28</v>
@@ -7517,7 +7517,7 @@
         <v>27</v>
       </c>
       <c r="E242" s="11">
-        <v>21</v>
+        <v>18</v>
       </c>
       <c r="F242" s="9" t="s">
         <v>28</v>
@@ -7540,7 +7540,7 @@
         <v>27</v>
       </c>
       <c r="E243" s="11">
-        <v>18</v>
+        <v>28</v>
       </c>
       <c r="F243" s="9" t="s">
         <v>28</v>
@@ -7563,7 +7563,7 @@
         <v>27</v>
       </c>
       <c r="E244" s="11">
-        <v>11</v>
+        <v>14</v>
       </c>
       <c r="F244" s="9" t="s">
         <v>28</v>
@@ -7586,7 +7586,7 @@
         <v>27</v>
       </c>
       <c r="E245" s="11">
-        <v>19</v>
+        <v>30</v>
       </c>
       <c r="F245" s="9" t="s">
         <v>28</v>
@@ -7609,7 +7609,7 @@
         <v>27</v>
       </c>
       <c r="E246" s="11">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="F246" s="9" t="s">
         <v>28</v>
@@ -7632,7 +7632,7 @@
         <v>27</v>
       </c>
       <c r="E247" s="11">
-        <v>28</v>
+        <v>30</v>
       </c>
       <c r="F247" s="9" t="s">
         <v>28</v>
@@ -7655,7 +7655,7 @@
         <v>27</v>
       </c>
       <c r="E248" s="11">
-        <v>14</v>
+        <v>25</v>
       </c>
       <c r="F248" s="9" t="s">
         <v>28</v>
@@ -7678,7 +7678,7 @@
         <v>27</v>
       </c>
       <c r="E249" s="11">
-        <v>28</v>
+        <v>23</v>
       </c>
       <c r="F249" s="9" t="s">
         <v>28</v>
@@ -7701,7 +7701,7 @@
         <v>27</v>
       </c>
       <c r="E250" s="11">
-        <v>24</v>
+        <v>9</v>
       </c>
       <c r="F250" s="9" t="s">
         <v>28</v>
@@ -7747,7 +7747,7 @@
         <v>27</v>
       </c>
       <c r="E252" s="11">
-        <v>30</v>
+        <v>20</v>
       </c>
       <c r="F252" s="9" t="s">
         <v>28</v>
@@ -7770,7 +7770,7 @@
         <v>27</v>
       </c>
       <c r="E253" s="11">
-        <v>16</v>
+        <v>29</v>
       </c>
       <c r="F253" s="9" t="s">
         <v>28</v>
@@ -7793,7 +7793,7 @@
         <v>27</v>
       </c>
       <c r="E254" s="11">
-        <v>24</v>
+        <v>22</v>
       </c>
       <c r="F254" s="9" t="s">
         <v>28</v>
@@ -7816,7 +7816,7 @@
         <v>27</v>
       </c>
       <c r="E255" s="11">
-        <v>25</v>
+        <v>13</v>
       </c>
       <c r="F255" s="9" t="s">
         <v>28</v>
@@ -7839,7 +7839,7 @@
         <v>27</v>
       </c>
       <c r="E256" s="11">
-        <v>20</v>
+        <v>27</v>
       </c>
       <c r="F256" s="9" t="s">
         <v>28</v>
@@ -7862,7 +7862,7 @@
         <v>27</v>
       </c>
       <c r="E257" s="11">
-        <v>24</v>
+        <v>22</v>
       </c>
       <c r="F257" s="9" t="s">
         <v>28</v>
@@ -7885,7 +7885,7 @@
         <v>27</v>
       </c>
       <c r="E258" s="11">
-        <v>23</v>
+        <v>31</v>
       </c>
       <c r="F258" s="9" t="s">
         <v>28</v>
@@ -7908,7 +7908,7 @@
         <v>27</v>
       </c>
       <c r="E259" s="11">
-        <v>15</v>
+        <v>29</v>
       </c>
       <c r="F259" s="9" t="s">
         <v>28</v>
@@ -7931,7 +7931,7 @@
         <v>27</v>
       </c>
       <c r="E260" s="11">
-        <v>11</v>
+        <v>30</v>
       </c>
       <c r="F260" s="9" t="s">
         <v>28</v>
@@ -7954,7 +7954,7 @@
         <v>27</v>
       </c>
       <c r="E261" s="11">
-        <v>18</v>
+        <v>21</v>
       </c>
       <c r="F261" s="9" t="s">
         <v>28</v>
@@ -7977,7 +7977,7 @@
         <v>27</v>
       </c>
       <c r="E262" s="11">
-        <v>17</v>
+        <v>23</v>
       </c>
       <c r="F262" s="9" t="s">
         <v>28</v>
@@ -8000,7 +8000,7 @@
         <v>27</v>
       </c>
       <c r="E263" s="11">
-        <v>27</v>
+        <v>20</v>
       </c>
       <c r="F263" s="9" t="s">
         <v>28</v>
@@ -8023,7 +8023,7 @@
         <v>27</v>
       </c>
       <c r="E264" s="11">
-        <v>27</v>
+        <v>17</v>
       </c>
       <c r="F264" s="9" t="s">
         <v>28</v>
@@ -8046,7 +8046,7 @@
         <v>27</v>
       </c>
       <c r="E265" s="11">
-        <v>18</v>
+        <v>27</v>
       </c>
       <c r="F265" s="9" t="s">
         <v>28</v>
@@ -8069,7 +8069,7 @@
         <v>27</v>
       </c>
       <c r="E266" s="11">
-        <v>26</v>
+        <v>16</v>
       </c>
       <c r="F266" s="9" t="s">
         <v>28</v>
@@ -8092,7 +8092,7 @@
         <v>27</v>
       </c>
       <c r="E267" s="11">
-        <v>21</v>
+        <v>9</v>
       </c>
       <c r="F267" s="9" t="s">
         <v>28</v>
@@ -8115,7 +8115,7 @@
         <v>27</v>
       </c>
       <c r="E268" s="11">
-        <v>27</v>
+        <v>12</v>
       </c>
       <c r="F268" s="9" t="s">
         <v>28</v>
@@ -8138,7 +8138,7 @@
         <v>27</v>
       </c>
       <c r="E269" s="11">
-        <v>10</v>
+        <v>24</v>
       </c>
       <c r="F269" s="9" t="s">
         <v>28</v>
@@ -8161,7 +8161,7 @@
         <v>27</v>
       </c>
       <c r="E270" s="11">
-        <v>10</v>
+        <v>15</v>
       </c>
       <c r="F270" s="9" t="s">
         <v>28</v>
@@ -8184,7 +8184,7 @@
         <v>27</v>
       </c>
       <c r="E271" s="11">
-        <v>10</v>
+        <v>17</v>
       </c>
       <c r="F271" s="9" t="s">
         <v>28</v>
@@ -8207,7 +8207,7 @@
         <v>27</v>
       </c>
       <c r="E272" s="11">
-        <v>23</v>
+        <v>31</v>
       </c>
       <c r="F272" s="9" t="s">
         <v>28</v>
@@ -8230,7 +8230,7 @@
         <v>27</v>
       </c>
       <c r="E273" s="11">
-        <v>26</v>
+        <v>8</v>
       </c>
       <c r="F273" s="9" t="s">
         <v>28</v>
@@ -8276,7 +8276,7 @@
         <v>27</v>
       </c>
       <c r="E275" s="11">
-        <v>22</v>
+        <v>29</v>
       </c>
       <c r="F275" s="9" t="s">
         <v>28</v>
@@ -8299,7 +8299,7 @@
         <v>27</v>
       </c>
       <c r="E276" s="11">
-        <v>20</v>
+        <v>16</v>
       </c>
       <c r="F276" s="9" t="s">
         <v>28</v>
@@ -8322,7 +8322,7 @@
         <v>27</v>
       </c>
       <c r="E277" s="11">
-        <v>15</v>
+        <v>23</v>
       </c>
       <c r="F277" s="9" t="s">
         <v>28</v>
@@ -8345,7 +8345,7 @@
         <v>27</v>
       </c>
       <c r="E278" s="11">
-        <v>17</v>
+        <v>26</v>
       </c>
       <c r="F278" s="9" t="s">
         <v>28</v>
@@ -8368,7 +8368,7 @@
         <v>27</v>
       </c>
       <c r="E279" s="11">
-        <v>12</v>
+        <v>16</v>
       </c>
       <c r="F279" s="9" t="s">
         <v>28</v>
@@ -8391,7 +8391,7 @@
         <v>27</v>
       </c>
       <c r="E280" s="11">
-        <v>15</v>
+        <v>18</v>
       </c>
       <c r="F280" s="9" t="s">
         <v>28</v>
@@ -8414,7 +8414,7 @@
         <v>27</v>
       </c>
       <c r="E281" s="11">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="F281" s="9" t="s">
         <v>28</v>
@@ -8437,7 +8437,7 @@
         <v>27</v>
       </c>
       <c r="E282" s="11">
-        <v>31</v>
+        <v>11</v>
       </c>
       <c r="F282" s="9" t="s">
         <v>28</v>
@@ -8460,7 +8460,7 @@
         <v>27</v>
       </c>
       <c r="E283" s="11">
-        <v>14</v>
+        <v>22</v>
       </c>
       <c r="F283" s="9" t="s">
         <v>28</v>
@@ -8483,7 +8483,7 @@
         <v>27</v>
       </c>
       <c r="E284" s="11">
-        <v>21</v>
+        <v>31</v>
       </c>
       <c r="F284" s="9" t="s">
         <v>28</v>
@@ -8506,7 +8506,7 @@
         <v>27</v>
       </c>
       <c r="E285" s="11">
-        <v>9</v>
+        <v>12</v>
       </c>
       <c r="F285" s="9" t="s">
         <v>28</v>
@@ -8529,7 +8529,7 @@
         <v>27</v>
       </c>
       <c r="E286" s="11">
-        <v>11</v>
+        <v>19</v>
       </c>
       <c r="F286" s="9" t="s">
         <v>28</v>
@@ -8552,7 +8552,7 @@
         <v>27</v>
       </c>
       <c r="E287" s="11">
-        <v>20</v>
+        <v>13</v>
       </c>
       <c r="F287" s="9" t="s">
         <v>28</v>
@@ -8575,7 +8575,7 @@
         <v>27</v>
       </c>
       <c r="E288" s="11">
-        <v>15</v>
+        <v>19</v>
       </c>
       <c r="F288" s="9" t="s">
         <v>28</v>
@@ -8598,7 +8598,7 @@
         <v>27</v>
       </c>
       <c r="E289" s="11">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="F289" s="9" t="s">
         <v>28</v>
@@ -8621,7 +8621,7 @@
         <v>27</v>
       </c>
       <c r="E290" s="11">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="F290" s="9" t="s">
         <v>28</v>
@@ -8644,7 +8644,7 @@
         <v>27</v>
       </c>
       <c r="E291" s="11">
-        <v>31</v>
+        <v>25</v>
       </c>
       <c r="F291" s="9" t="s">
         <v>28</v>
@@ -8667,7 +8667,7 @@
         <v>27</v>
       </c>
       <c r="E292" s="11">
-        <v>30</v>
+        <v>11</v>
       </c>
       <c r="F292" s="9" t="s">
         <v>28</v>
@@ -8690,7 +8690,7 @@
         <v>27</v>
       </c>
       <c r="E293" s="11">
-        <v>26</v>
+        <v>8</v>
       </c>
       <c r="F293" s="9" t="s">
         <v>28</v>
@@ -8713,7 +8713,7 @@
         <v>27</v>
       </c>
       <c r="E294" s="11">
-        <v>27</v>
+        <v>11</v>
       </c>
       <c r="F294" s="9" t="s">
         <v>28</v>
@@ -8736,7 +8736,7 @@
         <v>27</v>
       </c>
       <c r="E295" s="11">
-        <v>18</v>
+        <v>28</v>
       </c>
       <c r="F295" s="9" t="s">
         <v>28</v>
@@ -8759,7 +8759,7 @@
         <v>27</v>
       </c>
       <c r="E296" s="11">
-        <v>18</v>
+        <v>14</v>
       </c>
       <c r="F296" s="9" t="s">
         <v>28</v>
@@ -8782,7 +8782,7 @@
         <v>27</v>
       </c>
       <c r="E297" s="11">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="F297" s="9" t="s">
         <v>28</v>
@@ -8805,7 +8805,7 @@
         <v>27</v>
       </c>
       <c r="E298" s="11">
-        <v>28</v>
+        <v>17</v>
       </c>
       <c r="F298" s="9" t="s">
         <v>28</v>
@@ -8828,7 +8828,7 @@
         <v>27</v>
       </c>
       <c r="E299" s="11">
-        <v>23</v>
+        <v>14</v>
       </c>
       <c r="F299" s="9" t="s">
         <v>28</v>
@@ -8851,7 +8851,7 @@
         <v>27</v>
       </c>
       <c r="E300" s="11">
-        <v>10</v>
+        <v>17</v>
       </c>
       <c r="F300" s="9" t="s">
         <v>28</v>
@@ -8874,7 +8874,7 @@
         <v>27</v>
       </c>
       <c r="E301" s="11">
-        <v>29</v>
+        <v>16</v>
       </c>
       <c r="F301" s="9" t="s">
         <v>28</v>
@@ -8897,7 +8897,7 @@
         <v>27</v>
       </c>
       <c r="E302" s="11">
-        <v>18</v>
+        <v>23</v>
       </c>
       <c r="F302" s="9" t="s">
         <v>28</v>
@@ -8920,7 +8920,7 @@
         <v>27</v>
       </c>
       <c r="E303" s="11">
-        <v>8</v>
+        <v>23</v>
       </c>
       <c r="F303" s="9" t="s">
         <v>28</v>
@@ -8943,7 +8943,7 @@
         <v>27</v>
       </c>
       <c r="E304" s="11">
-        <v>15</v>
+        <v>18</v>
       </c>
       <c r="F304" s="9" t="s">
         <v>28</v>
@@ -8966,7 +8966,7 @@
         <v>27</v>
       </c>
       <c r="E305" s="11">
-        <v>30</v>
+        <v>27</v>
       </c>
       <c r="F305" s="9" t="s">
         <v>28</v>
@@ -8989,7 +8989,7 @@
         <v>27</v>
       </c>
       <c r="E306" s="11">
-        <v>11</v>
+        <v>20</v>
       </c>
       <c r="F306" s="9" t="s">
         <v>28</v>
@@ -9012,7 +9012,7 @@
         <v>27</v>
       </c>
       <c r="E307" s="11">
-        <v>30</v>
+        <v>14</v>
       </c>
       <c r="F307" s="9" t="s">
         <v>28</v>
@@ -9035,7 +9035,7 @@
         <v>27</v>
       </c>
       <c r="E308" s="11">
-        <v>27</v>
+        <v>25</v>
       </c>
       <c r="F308" s="9" t="s">
         <v>28</v>
@@ -9058,7 +9058,7 @@
         <v>27</v>
       </c>
       <c r="E309" s="11">
-        <v>28</v>
+        <v>13</v>
       </c>
       <c r="F309" s="9" t="s">
         <v>28</v>
@@ -9081,7 +9081,7 @@
         <v>27</v>
       </c>
       <c r="E310" s="11">
-        <v>30</v>
+        <v>15</v>
       </c>
       <c r="F310" s="9" t="s">
         <v>28</v>
@@ -9104,7 +9104,7 @@
         <v>27</v>
       </c>
       <c r="E311" s="11">
-        <v>9</v>
+        <v>29</v>
       </c>
       <c r="F311" s="9" t="s">
         <v>28</v>
@@ -9127,7 +9127,7 @@
         <v>27</v>
       </c>
       <c r="E312" s="11">
-        <v>10</v>
+        <v>16</v>
       </c>
       <c r="F312" s="9" t="s">
         <v>28</v>
@@ -9150,7 +9150,7 @@
         <v>27</v>
       </c>
       <c r="E313" s="11">
-        <v>16</v>
+        <v>20</v>
       </c>
       <c r="F313" s="9" t="s">
         <v>28</v>
@@ -9173,7 +9173,7 @@
         <v>27</v>
       </c>
       <c r="E314" s="11">
-        <v>19</v>
+        <v>29</v>
       </c>
       <c r="F314" s="9" t="s">
         <v>28</v>
@@ -9219,7 +9219,7 @@
         <v>27</v>
       </c>
       <c r="E316" s="11">
-        <v>12</v>
+        <v>18</v>
       </c>
       <c r="F316" s="9" t="s">
         <v>28</v>
@@ -9242,7 +9242,7 @@
         <v>27</v>
       </c>
       <c r="E317" s="11">
-        <v>15</v>
+        <v>24</v>
       </c>
       <c r="F317" s="9" t="s">
         <v>28</v>
@@ -9265,7 +9265,7 @@
         <v>27</v>
       </c>
       <c r="E318" s="11">
-        <v>13</v>
+        <v>22</v>
       </c>
       <c r="F318" s="9" t="s">
         <v>28</v>
@@ -9288,7 +9288,7 @@
         <v>27</v>
       </c>
       <c r="E319" s="11">
-        <v>9</v>
+        <v>22</v>
       </c>
       <c r="F319" s="9" t="s">
         <v>28</v>
@@ -9311,7 +9311,7 @@
         <v>27</v>
       </c>
       <c r="E320" s="11">
-        <v>14</v>
+        <v>21</v>
       </c>
       <c r="F320" s="9" t="s">
         <v>28</v>
@@ -9334,7 +9334,7 @@
         <v>27</v>
       </c>
       <c r="E321" s="11">
-        <v>26</v>
+        <v>9</v>
       </c>
       <c r="F321" s="9" t="s">
         <v>28</v>
@@ -9357,7 +9357,7 @@
         <v>27</v>
       </c>
       <c r="E322" s="11">
-        <v>21</v>
+        <v>31</v>
       </c>
       <c r="F322" s="9" t="s">
         <v>28</v>
@@ -9380,7 +9380,7 @@
         <v>27</v>
       </c>
       <c r="E323" s="11">
-        <v>29</v>
+        <v>12</v>
       </c>
       <c r="F323" s="9" t="s">
         <v>28</v>
@@ -9403,7 +9403,7 @@
         <v>27</v>
       </c>
       <c r="E324" s="11">
-        <v>18</v>
+        <v>21</v>
       </c>
       <c r="F324" s="9" t="s">
         <v>28</v>
@@ -9426,7 +9426,7 @@
         <v>27</v>
       </c>
       <c r="E325" s="11">
-        <v>17</v>
+        <v>22</v>
       </c>
       <c r="F325" s="9" t="s">
         <v>28</v>
@@ -9449,7 +9449,7 @@
         <v>27</v>
       </c>
       <c r="E326" s="11">
-        <v>19</v>
+        <v>13</v>
       </c>
       <c r="F326" s="9" t="s">
         <v>28</v>
@@ -9472,7 +9472,7 @@
         <v>27</v>
       </c>
       <c r="E327" s="11">
-        <v>8</v>
+        <v>27</v>
       </c>
       <c r="F327" s="9" t="s">
         <v>28</v>
@@ -9495,7 +9495,7 @@
         <v>27</v>
       </c>
       <c r="E328" s="11">
-        <v>12</v>
+        <v>15</v>
       </c>
       <c r="F328" s="9" t="s">
         <v>28</v>
@@ -9518,7 +9518,7 @@
         <v>27</v>
       </c>
       <c r="E329" s="11">
-        <v>26</v>
+        <v>22</v>
       </c>
       <c r="F329" s="9" t="s">
         <v>28</v>
@@ -9541,7 +9541,7 @@
         <v>27</v>
       </c>
       <c r="E330" s="11">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="F330" s="9" t="s">
         <v>28</v>
@@ -9564,7 +9564,7 @@
         <v>27</v>
       </c>
       <c r="E331" s="11">
-        <v>24</v>
+        <v>12</v>
       </c>
       <c r="F331" s="9" t="s">
         <v>28</v>
@@ -9587,7 +9587,7 @@
         <v>27</v>
       </c>
       <c r="E332" s="11">
-        <v>11</v>
+        <v>15</v>
       </c>
       <c r="F332" s="9" t="s">
         <v>28</v>
@@ -9610,7 +9610,7 @@
         <v>27</v>
       </c>
       <c r="E333" s="11">
-        <v>30</v>
+        <v>23</v>
       </c>
       <c r="F333" s="9" t="s">
         <v>28</v>
@@ -9633,7 +9633,7 @@
         <v>27</v>
       </c>
       <c r="E334" s="11">
-        <v>25</v>
+        <v>12</v>
       </c>
       <c r="F334" s="9" t="s">
         <v>28</v>
@@ -9656,7 +9656,7 @@
         <v>27</v>
       </c>
       <c r="E335" s="11">
-        <v>19</v>
+        <v>27</v>
       </c>
       <c r="F335" s="9" t="s">
         <v>28</v>
@@ -9702,7 +9702,7 @@
         <v>27</v>
       </c>
       <c r="E337" s="11">
-        <v>12</v>
+        <v>22</v>
       </c>
       <c r="F337" s="9" t="s">
         <v>28</v>
@@ -9725,7 +9725,7 @@
         <v>27</v>
       </c>
       <c r="E338" s="11">
-        <v>27</v>
+        <v>29</v>
       </c>
       <c r="F338" s="9" t="s">
         <v>28</v>
@@ -9748,7 +9748,7 @@
         <v>27</v>
       </c>
       <c r="E339" s="11">
-        <v>30</v>
+        <v>28</v>
       </c>
       <c r="F339" s="9" t="s">
         <v>28</v>
@@ -9771,7 +9771,7 @@
         <v>27</v>
       </c>
       <c r="E340" s="11">
-        <v>20</v>
+        <v>29</v>
       </c>
       <c r="F340" s="9" t="s">
         <v>28</v>
@@ -9794,7 +9794,7 @@
         <v>27</v>
       </c>
       <c r="E341" s="11">
-        <v>17</v>
+        <v>15</v>
       </c>
       <c r="F341" s="9" t="s">
         <v>28</v>
@@ -9817,7 +9817,7 @@
         <v>27</v>
       </c>
       <c r="E342" s="11">
-        <v>19</v>
+        <v>30</v>
       </c>
       <c r="F342" s="9" t="s">
         <v>28</v>
@@ -9840,7 +9840,7 @@
         <v>27</v>
       </c>
       <c r="E343" s="11">
-        <v>18</v>
+        <v>15</v>
       </c>
       <c r="F343" s="9" t="s">
         <v>28</v>
@@ -9863,7 +9863,7 @@
         <v>27</v>
       </c>
       <c r="E344" s="11">
-        <v>10</v>
+        <v>17</v>
       </c>
       <c r="F344" s="9" t="s">
         <v>28</v>
@@ -9886,7 +9886,7 @@
         <v>27</v>
       </c>
       <c r="E345" s="11">
-        <v>14</v>
+        <v>24</v>
       </c>
       <c r="F345" s="9" t="s">
         <v>28</v>
@@ -9909,7 +9909,7 @@
         <v>27</v>
       </c>
       <c r="E346" s="11">
-        <v>11</v>
+        <v>20</v>
       </c>
       <c r="F346" s="9" t="s">
         <v>28</v>
@@ -9932,7 +9932,7 @@
         <v>27</v>
       </c>
       <c r="E347" s="11">
-        <v>17</v>
+        <v>19</v>
       </c>
       <c r="F347" s="9" t="s">
         <v>28</v>
@@ -9955,7 +9955,7 @@
         <v>27</v>
       </c>
       <c r="E348" s="11">
-        <v>11</v>
+        <v>31</v>
       </c>
       <c r="F348" s="9" t="s">
         <v>28</v>
@@ -9978,7 +9978,7 @@
         <v>27</v>
       </c>
       <c r="E349" s="11">
-        <v>24</v>
+        <v>31</v>
       </c>
       <c r="F349" s="9" t="s">
         <v>28</v>
@@ -10001,7 +10001,7 @@
         <v>27</v>
       </c>
       <c r="E350" s="11">
-        <v>8</v>
+        <v>11</v>
       </c>
       <c r="F350" s="9" t="s">
         <v>28</v>
@@ -10024,7 +10024,7 @@
         <v>27</v>
       </c>
       <c r="E351" s="11">
-        <v>22</v>
+        <v>25</v>
       </c>
       <c r="F351" s="9" t="s">
         <v>28</v>
@@ -10047,7 +10047,7 @@
         <v>27</v>
       </c>
       <c r="E352" s="11">
-        <v>10</v>
+        <v>15</v>
       </c>
       <c r="F352" s="9" t="s">
         <v>28</v>
@@ -10070,7 +10070,7 @@
         <v>27</v>
       </c>
       <c r="E353" s="11">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="F353" s="9" t="s">
         <v>28</v>
@@ -10093,7 +10093,7 @@
         <v>27</v>
       </c>
       <c r="E354" s="11">
-        <v>14</v>
+        <v>21</v>
       </c>
       <c r="F354" s="9" t="s">
         <v>28</v>
@@ -10116,7 +10116,7 @@
         <v>27</v>
       </c>
       <c r="E355" s="11">
-        <v>12</v>
+        <v>10</v>
       </c>
       <c r="F355" s="9" t="s">
         <v>28</v>
@@ -10139,7 +10139,7 @@
         <v>27</v>
       </c>
       <c r="E356" s="11">
-        <v>13</v>
+        <v>18</v>
       </c>
       <c r="F356" s="9" t="s">
         <v>28</v>
@@ -10162,7 +10162,7 @@
         <v>27</v>
       </c>
       <c r="E357" s="11">
-        <v>12</v>
+        <v>18</v>
       </c>
       <c r="F357" s="9" t="s">
         <v>28</v>
@@ -10185,7 +10185,7 @@
         <v>27</v>
       </c>
       <c r="E358" s="11">
-        <v>13</v>
+        <v>17</v>
       </c>
       <c r="F358" s="9" t="s">
         <v>28</v>
@@ -10208,7 +10208,7 @@
         <v>27</v>
       </c>
       <c r="E359" s="11">
-        <v>17</v>
+        <v>21</v>
       </c>
       <c r="F359" s="9" t="s">
         <v>28</v>
@@ -10231,7 +10231,7 @@
         <v>27</v>
       </c>
       <c r="E360" s="11">
-        <v>8</v>
+        <v>31</v>
       </c>
       <c r="F360" s="9" t="s">
         <v>28</v>
@@ -10254,7 +10254,7 @@
         <v>27</v>
       </c>
       <c r="E361" s="11">
-        <v>16</v>
+        <v>14</v>
       </c>
       <c r="F361" s="9" t="s">
         <v>28</v>
@@ -10277,7 +10277,7 @@
         <v>27</v>
       </c>
       <c r="E362" s="11">
-        <v>30</v>
+        <v>12</v>
       </c>
       <c r="F362" s="9" t="s">
         <v>28</v>
@@ -10300,7 +10300,7 @@
         <v>27</v>
       </c>
       <c r="E363" s="11">
-        <v>27</v>
+        <v>13</v>
       </c>
       <c r="F363" s="9" t="s">
         <v>28</v>
@@ -10323,7 +10323,7 @@
         <v>27</v>
       </c>
       <c r="E364" s="11">
-        <v>12</v>
+        <v>22</v>
       </c>
       <c r="F364" s="9" t="s">
         <v>28</v>
@@ -10346,7 +10346,7 @@
         <v>27</v>
       </c>
       <c r="E365" s="11">
-        <v>13</v>
+        <v>23</v>
       </c>
       <c r="F365" s="9" t="s">
         <v>28</v>
@@ -10369,7 +10369,7 @@
         <v>27</v>
       </c>
       <c r="E366" s="11">
-        <v>9</v>
+        <v>17</v>
       </c>
       <c r="F366" s="9" t="s">
         <v>28</v>
@@ -10392,7 +10392,7 @@
         <v>27</v>
       </c>
       <c r="E367" s="11">
-        <v>13</v>
+        <v>16</v>
       </c>
       <c r="F367" s="9" t="s">
         <v>28</v>
@@ -10415,7 +10415,7 @@
         <v>27</v>
       </c>
       <c r="E368" s="11">
-        <v>19</v>
+        <v>24</v>
       </c>
       <c r="F368" s="9" t="s">
         <v>28</v>
@@ -10438,7 +10438,7 @@
         <v>27</v>
       </c>
       <c r="E369" s="11">
-        <v>23</v>
+        <v>26</v>
       </c>
       <c r="F369" s="9" t="s">
         <v>28</v>
@@ -10461,7 +10461,7 @@
         <v>27</v>
       </c>
       <c r="E370" s="11">
-        <v>8</v>
+        <v>28</v>
       </c>
       <c r="F370" s="9" t="s">
         <v>28</v>
@@ -10484,7 +10484,7 @@
         <v>27</v>
       </c>
       <c r="E371" s="11">
-        <v>31</v>
+        <v>15</v>
       </c>
       <c r="F371" s="9" t="s">
         <v>28</v>
@@ -10507,7 +10507,7 @@
         <v>27</v>
       </c>
       <c r="E372" s="11">
-        <v>10</v>
+        <v>19</v>
       </c>
       <c r="F372" s="9" t="s">
         <v>28</v>
@@ -10530,7 +10530,7 @@
         <v>27</v>
       </c>
       <c r="E373" s="11">
-        <v>21</v>
+        <v>9</v>
       </c>
       <c r="F373" s="9" t="s">
         <v>28</v>
@@ -10599,7 +10599,7 @@
         <v>27</v>
       </c>
       <c r="E376" s="11">
-        <v>18</v>
+        <v>28</v>
       </c>
       <c r="F376" s="9" t="s">
         <v>28</v>
@@ -10622,7 +10622,7 @@
         <v>27</v>
       </c>
       <c r="E377" s="11">
-        <v>8</v>
+        <v>13</v>
       </c>
       <c r="F377" s="9" t="s">
         <v>28</v>
@@ -10645,7 +10645,7 @@
         <v>27</v>
       </c>
       <c r="E378" s="11">
-        <v>13</v>
+        <v>16</v>
       </c>
       <c r="F378" s="9" t="s">
         <v>28</v>
@@ -10691,7 +10691,7 @@
         <v>27</v>
       </c>
       <c r="E380" s="11">
-        <v>16</v>
+        <v>23</v>
       </c>
       <c r="F380" s="9" t="s">
         <v>28</v>
@@ -10714,7 +10714,7 @@
         <v>27</v>
       </c>
       <c r="E381" s="11">
-        <v>8</v>
+        <v>13</v>
       </c>
       <c r="F381" s="9" t="s">
         <v>28</v>
@@ -10737,7 +10737,7 @@
         <v>27</v>
       </c>
       <c r="E382" s="11">
-        <v>15</v>
+        <v>26</v>
       </c>
       <c r="F382" s="9" t="s">
         <v>28</v>
@@ -10760,7 +10760,7 @@
         <v>27</v>
       </c>
       <c r="E383" s="11">
-        <v>21</v>
+        <v>23</v>
       </c>
       <c r="F383" s="9" t="s">
         <v>28</v>
@@ -10783,7 +10783,7 @@
         <v>27</v>
       </c>
       <c r="E384" s="11">
-        <v>11</v>
+        <v>24</v>
       </c>
       <c r="F384" s="9" t="s">
         <v>28</v>
@@ -10806,7 +10806,7 @@
         <v>27</v>
       </c>
       <c r="E385" s="11">
-        <v>11</v>
+        <v>18</v>
       </c>
       <c r="F385" s="9" t="s">
         <v>28</v>
@@ -10829,7 +10829,7 @@
         <v>27</v>
       </c>
       <c r="E386" s="11">
-        <v>27</v>
+        <v>8</v>
       </c>
       <c r="F386" s="9" t="s">
         <v>28</v>
@@ -10852,7 +10852,7 @@
         <v>27</v>
       </c>
       <c r="E387" s="11">
-        <v>16</v>
+        <v>9</v>
       </c>
       <c r="F387" s="9" t="s">
         <v>28</v>
@@ -10875,7 +10875,7 @@
         <v>27</v>
       </c>
       <c r="E388" s="11">
-        <v>29</v>
+        <v>25</v>
       </c>
       <c r="F388" s="9" t="s">
         <v>28</v>
@@ -10898,7 +10898,7 @@
         <v>27</v>
       </c>
       <c r="E389" s="11">
-        <v>25</v>
+        <v>30</v>
       </c>
       <c r="F389" s="9" t="s">
         <v>28</v>
@@ -10967,7 +10967,7 @@
         <v>27</v>
       </c>
       <c r="E392" s="11">
-        <v>25</v>
+        <v>18</v>
       </c>
       <c r="F392" s="9" t="s">
         <v>28</v>
@@ -10990,7 +10990,7 @@
         <v>27</v>
       </c>
       <c r="E393" s="11">
-        <v>25</v>
+        <v>28</v>
       </c>
       <c r="F393" s="9" t="s">
         <v>28</v>
@@ -11013,7 +11013,7 @@
         <v>27</v>
       </c>
       <c r="E394" s="11">
-        <v>30</v>
+        <v>14</v>
       </c>
       <c r="F394" s="9" t="s">
         <v>28</v>
@@ -11036,7 +11036,7 @@
         <v>27</v>
       </c>
       <c r="E395" s="11">
-        <v>8</v>
+        <v>16</v>
       </c>
       <c r="F395" s="9" t="s">
         <v>28</v>
@@ -11059,7 +11059,7 @@
         <v>27</v>
       </c>
       <c r="E396" s="11">
-        <v>11</v>
+        <v>17</v>
       </c>
       <c r="F396" s="9" t="s">
         <v>28</v>
@@ -11082,7 +11082,7 @@
         <v>27</v>
       </c>
       <c r="E397" s="11">
-        <v>20</v>
+        <v>22</v>
       </c>
       <c r="F397" s="9" t="s">
         <v>28</v>
@@ -11105,7 +11105,7 @@
         <v>27</v>
       </c>
       <c r="E398" s="11">
-        <v>25</v>
+        <v>23</v>
       </c>
       <c r="F398" s="9" t="s">
         <v>28</v>
@@ -11128,7 +11128,7 @@
         <v>27</v>
       </c>
       <c r="E399" s="11">
-        <v>25</v>
+        <v>20</v>
       </c>
       <c r="F399" s="9" t="s">
         <v>28</v>
@@ -11151,7 +11151,7 @@
         <v>27</v>
       </c>
       <c r="E400" s="11">
-        <v>30</v>
+        <v>25</v>
       </c>
       <c r="F400" s="9" t="s">
         <v>28</v>
@@ -11174,7 +11174,7 @@
         <v>27</v>
       </c>
       <c r="E401" s="11">
-        <v>27</v>
+        <v>14</v>
       </c>
       <c r="F401" s="9" t="s">
         <v>28</v>

</xml_diff>